<commit_message>
Atualizacao automatica 06/04/2026 14:39:35,80
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C6C93FC-5460-4817-B8C9-EF81B5885E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A98B6E4-B4D4-4ABD-8095-86C642610FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34875" yWindow="4665" windowWidth="13830" windowHeight="7110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1304" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1646" uniqueCount="144">
   <si>
     <t>Sel</t>
   </si>
@@ -395,6 +395,63 @@
   </si>
   <si>
     <t>1871400010234</t>
+  </si>
+  <si>
+    <t>1871400010235</t>
+  </si>
+  <si>
+    <t>1871400010236</t>
+  </si>
+  <si>
+    <t>1871400010237</t>
+  </si>
+  <si>
+    <t>1871400010238</t>
+  </si>
+  <si>
+    <t>1871400010239</t>
+  </si>
+  <si>
+    <t>1871400010240</t>
+  </si>
+  <si>
+    <t>1871400010241</t>
+  </si>
+  <si>
+    <t>1871400010242</t>
+  </si>
+  <si>
+    <t>1871400010243</t>
+  </si>
+  <si>
+    <t>1871400010244</t>
+  </si>
+  <si>
+    <t>1871400010245</t>
+  </si>
+  <si>
+    <t>1871400010246</t>
+  </si>
+  <si>
+    <t>1871400010247</t>
+  </si>
+  <si>
+    <t>1871400010248</t>
+  </si>
+  <si>
+    <t>1871400010249</t>
+  </si>
+  <si>
+    <t>1871400010250</t>
+  </si>
+  <si>
+    <t>1871400010251</t>
+  </si>
+  <si>
+    <t>1871400010252</t>
+  </si>
+  <si>
+    <t>1871400010253</t>
   </si>
 </sst>
 </file>
@@ -970,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR71"/>
+  <dimension ref="A1:AR90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -10485,6 +10542,2552 @@
       </c>
       <c r="AR71" s="3" t="s">
         <v>124</v>
+      </c>
+    </row>
+    <row r="72" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
+        <v>1</v>
+      </c>
+      <c r="B72" s="2">
+        <v>2</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F72" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G72" s="5">
+        <v>268</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L72" s="6">
+        <v>246</v>
+      </c>
+      <c r="M72" s="7">
+        <v>100789.67</v>
+      </c>
+      <c r="N72" s="6">
+        <v>1</v>
+      </c>
+      <c r="O72" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P72" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q72" s="6">
+        <v>0</v>
+      </c>
+      <c r="R72" s="7">
+        <v>0</v>
+      </c>
+      <c r="S72" s="9">
+        <v>0</v>
+      </c>
+      <c r="T72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U72" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V72" s="11">
+        <v>11</v>
+      </c>
+      <c r="W72" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X72" s="12">
+        <v>0.54722219999999999</v>
+      </c>
+      <c r="Y72" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB72" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG72" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI72" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK72" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM72" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR72" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
+        <v>1</v>
+      </c>
+      <c r="B73" s="2">
+        <v>2</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F73" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G73" s="5">
+        <v>269</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K73" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L73" s="6">
+        <v>247</v>
+      </c>
+      <c r="M73" s="7">
+        <v>101199.38</v>
+      </c>
+      <c r="N73" s="6">
+        <v>1</v>
+      </c>
+      <c r="O73" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P73" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q73" s="6">
+        <v>0</v>
+      </c>
+      <c r="R73" s="7">
+        <v>0</v>
+      </c>
+      <c r="S73" s="9">
+        <v>0</v>
+      </c>
+      <c r="T73" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U73" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V73" s="11">
+        <v>11</v>
+      </c>
+      <c r="W73" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X73" s="12">
+        <v>0.54722219999999999</v>
+      </c>
+      <c r="Y73" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB73" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG73" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI73" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ73" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK73" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM73" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR73" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
+        <v>1</v>
+      </c>
+      <c r="B74" s="2">
+        <v>2</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F74" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G74" s="5">
+        <v>270</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K74" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L74" s="6">
+        <v>248</v>
+      </c>
+      <c r="M74" s="7">
+        <v>101609.1</v>
+      </c>
+      <c r="N74" s="6">
+        <v>1</v>
+      </c>
+      <c r="O74" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P74" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q74" s="6">
+        <v>0</v>
+      </c>
+      <c r="R74" s="7">
+        <v>0</v>
+      </c>
+      <c r="S74" s="9">
+        <v>0</v>
+      </c>
+      <c r="T74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U74" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V74" s="11">
+        <v>11</v>
+      </c>
+      <c r="W74" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X74" s="12">
+        <v>0.54722219999999999</v>
+      </c>
+      <c r="Y74" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB74" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG74" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI74" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK74" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM74" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR74" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="75" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
+        <v>1</v>
+      </c>
+      <c r="B75" s="2">
+        <v>2</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F75" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G75" s="5">
+        <v>271</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K75" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L75" s="6">
+        <v>249</v>
+      </c>
+      <c r="M75" s="7">
+        <v>102018.81</v>
+      </c>
+      <c r="N75" s="6">
+        <v>1</v>
+      </c>
+      <c r="O75" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P75" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q75" s="6">
+        <v>0</v>
+      </c>
+      <c r="R75" s="7">
+        <v>0</v>
+      </c>
+      <c r="S75" s="9">
+        <v>0</v>
+      </c>
+      <c r="T75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U75" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V75" s="11">
+        <v>11</v>
+      </c>
+      <c r="W75" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X75" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y75" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB75" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG75" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI75" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK75" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM75" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR75" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="76" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
+        <v>1</v>
+      </c>
+      <c r="B76" s="2">
+        <v>2</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F76" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G76" s="5">
+        <v>272</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L76" s="6">
+        <v>250</v>
+      </c>
+      <c r="M76" s="7">
+        <v>102428.52</v>
+      </c>
+      <c r="N76" s="6">
+        <v>1</v>
+      </c>
+      <c r="O76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P76" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q76" s="6">
+        <v>0</v>
+      </c>
+      <c r="R76" s="7">
+        <v>0</v>
+      </c>
+      <c r="S76" s="9">
+        <v>0</v>
+      </c>
+      <c r="T76" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U76" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V76" s="11">
+        <v>11</v>
+      </c>
+      <c r="W76" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X76" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y76" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB76" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG76" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI76" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ76" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK76" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM76" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR76" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="77" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
+        <v>1</v>
+      </c>
+      <c r="B77" s="2">
+        <v>2</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F77" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G77" s="5">
+        <v>273</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K77" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L77" s="6">
+        <v>251</v>
+      </c>
+      <c r="M77" s="7">
+        <v>102838.24</v>
+      </c>
+      <c r="N77" s="6">
+        <v>1</v>
+      </c>
+      <c r="O77" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P77" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q77" s="6">
+        <v>0</v>
+      </c>
+      <c r="R77" s="7">
+        <v>0</v>
+      </c>
+      <c r="S77" s="9">
+        <v>0</v>
+      </c>
+      <c r="T77" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U77" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V77" s="11">
+        <v>11</v>
+      </c>
+      <c r="W77" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X77" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y77" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB77" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG77" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI77" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ77" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK77" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM77" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR77" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
+        <v>1</v>
+      </c>
+      <c r="B78" s="2">
+        <v>2</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F78" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G78" s="5">
+        <v>274</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L78" s="6">
+        <v>252</v>
+      </c>
+      <c r="M78" s="7">
+        <v>103247.95</v>
+      </c>
+      <c r="N78" s="6">
+        <v>1</v>
+      </c>
+      <c r="O78" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P78" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q78" s="6">
+        <v>0</v>
+      </c>
+      <c r="R78" s="7">
+        <v>0</v>
+      </c>
+      <c r="S78" s="9">
+        <v>0</v>
+      </c>
+      <c r="T78" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U78" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V78" s="11">
+        <v>11</v>
+      </c>
+      <c r="W78" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X78" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y78" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB78" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG78" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI78" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ78" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK78" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM78" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR78" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="79" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
+        <v>1</v>
+      </c>
+      <c r="B79" s="2">
+        <v>2</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F79" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G79" s="5">
+        <v>275</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L79" s="6">
+        <v>253</v>
+      </c>
+      <c r="M79" s="7">
+        <v>103657.67</v>
+      </c>
+      <c r="N79" s="6">
+        <v>1</v>
+      </c>
+      <c r="O79" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P79" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q79" s="6">
+        <v>0</v>
+      </c>
+      <c r="R79" s="7">
+        <v>0</v>
+      </c>
+      <c r="S79" s="9">
+        <v>0</v>
+      </c>
+      <c r="T79" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U79" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V79" s="11">
+        <v>11</v>
+      </c>
+      <c r="W79" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X79" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y79" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB79" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG79" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI79" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ79" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK79" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM79" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR79" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="80" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
+        <v>1</v>
+      </c>
+      <c r="B80" s="2">
+        <v>2</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F80" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G80" s="5">
+        <v>276</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I80" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J80" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K80" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L80" s="6">
+        <v>254</v>
+      </c>
+      <c r="M80" s="7">
+        <v>104067.38</v>
+      </c>
+      <c r="N80" s="6">
+        <v>1</v>
+      </c>
+      <c r="O80" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P80" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q80" s="6">
+        <v>0</v>
+      </c>
+      <c r="R80" s="7">
+        <v>0</v>
+      </c>
+      <c r="S80" s="9">
+        <v>0</v>
+      </c>
+      <c r="T80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U80" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V80" s="11">
+        <v>11</v>
+      </c>
+      <c r="W80" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X80" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y80" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB80" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG80" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI80" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK80" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM80" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR80" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
+        <v>1</v>
+      </c>
+      <c r="B81" s="2">
+        <v>2</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F81" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G81" s="5">
+        <v>277</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I81" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K81" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L81" s="6">
+        <v>255</v>
+      </c>
+      <c r="M81" s="7">
+        <v>104477.09</v>
+      </c>
+      <c r="N81" s="6">
+        <v>1</v>
+      </c>
+      <c r="O81" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P81" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q81" s="6">
+        <v>0</v>
+      </c>
+      <c r="R81" s="7">
+        <v>0</v>
+      </c>
+      <c r="S81" s="9">
+        <v>0</v>
+      </c>
+      <c r="T81" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U81" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V81" s="11">
+        <v>11</v>
+      </c>
+      <c r="W81" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X81" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y81" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB81" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG81" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI81" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ81" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK81" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM81" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR81" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="82" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
+        <v>1</v>
+      </c>
+      <c r="B82" s="2">
+        <v>2</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F82" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G82" s="5">
+        <v>278</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L82" s="6">
+        <v>256</v>
+      </c>
+      <c r="M82" s="7">
+        <v>104886.81</v>
+      </c>
+      <c r="N82" s="6">
+        <v>1</v>
+      </c>
+      <c r="O82" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P82" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q82" s="6">
+        <v>0</v>
+      </c>
+      <c r="R82" s="7">
+        <v>0</v>
+      </c>
+      <c r="S82" s="9">
+        <v>0</v>
+      </c>
+      <c r="T82" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U82" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V82" s="11">
+        <v>11</v>
+      </c>
+      <c r="W82" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X82" s="12">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="Y82" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB82" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG82" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI82" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ82" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK82" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM82" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR82" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="83" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
+        <v>1</v>
+      </c>
+      <c r="B83" s="2">
+        <v>2</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F83" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G83" s="5">
+        <v>283</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I83" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J83" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K83" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L83" s="6">
+        <v>257</v>
+      </c>
+      <c r="M83" s="7">
+        <v>105296.52</v>
+      </c>
+      <c r="N83" s="6">
+        <v>1</v>
+      </c>
+      <c r="O83" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P83" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q83" s="6">
+        <v>0</v>
+      </c>
+      <c r="R83" s="7">
+        <v>0</v>
+      </c>
+      <c r="S83" s="9">
+        <v>0</v>
+      </c>
+      <c r="T83" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U83" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V83" s="11">
+        <v>11</v>
+      </c>
+      <c r="W83" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X83" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y83" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB83" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG83" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI83" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ83" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK83" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM83" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR83" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="84" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
+        <v>1</v>
+      </c>
+      <c r="B84" s="2">
+        <v>2</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F84" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G84" s="5">
+        <v>284</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I84" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L84" s="6">
+        <v>258</v>
+      </c>
+      <c r="M84" s="7">
+        <v>105706.24000000001</v>
+      </c>
+      <c r="N84" s="6">
+        <v>1</v>
+      </c>
+      <c r="O84" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P84" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q84" s="6">
+        <v>0</v>
+      </c>
+      <c r="R84" s="7">
+        <v>0</v>
+      </c>
+      <c r="S84" s="9">
+        <v>0</v>
+      </c>
+      <c r="T84" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U84" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V84" s="11">
+        <v>11</v>
+      </c>
+      <c r="W84" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X84" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y84" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB84" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG84" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI84" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ84" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK84" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM84" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR84" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="85" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
+        <v>1</v>
+      </c>
+      <c r="B85" s="2">
+        <v>2</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F85" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G85" s="5">
+        <v>285</v>
+      </c>
+      <c r="H85" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J85" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K85" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L85" s="6">
+        <v>259</v>
+      </c>
+      <c r="M85" s="7">
+        <v>106115.95</v>
+      </c>
+      <c r="N85" s="6">
+        <v>1</v>
+      </c>
+      <c r="O85" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P85" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q85" s="6">
+        <v>0</v>
+      </c>
+      <c r="R85" s="7">
+        <v>0</v>
+      </c>
+      <c r="S85" s="9">
+        <v>0</v>
+      </c>
+      <c r="T85" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U85" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V85" s="11">
+        <v>11</v>
+      </c>
+      <c r="W85" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X85" s="12">
+        <v>0.58958330000000003</v>
+      </c>
+      <c r="Y85" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB85" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG85" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI85" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ85" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK85" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM85" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR85" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="86" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
+        <v>1</v>
+      </c>
+      <c r="B86" s="2">
+        <v>2</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F86" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G86" s="5">
+        <v>286</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J86" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K86" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L86" s="6">
+        <v>260</v>
+      </c>
+      <c r="M86" s="7">
+        <v>106525.67</v>
+      </c>
+      <c r="N86" s="6">
+        <v>1</v>
+      </c>
+      <c r="O86" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P86" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q86" s="6">
+        <v>0</v>
+      </c>
+      <c r="R86" s="7">
+        <v>0</v>
+      </c>
+      <c r="S86" s="9">
+        <v>0</v>
+      </c>
+      <c r="T86" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U86" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V86" s="11">
+        <v>11</v>
+      </c>
+      <c r="W86" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X86" s="12">
+        <v>0.58958330000000003</v>
+      </c>
+      <c r="Y86" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB86" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG86" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI86" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ86" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK86" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM86" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR86" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="87" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
+        <v>1</v>
+      </c>
+      <c r="B87" s="2">
+        <v>2</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F87" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G87" s="5">
+        <v>287</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I87" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J87" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K87" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L87" s="6">
+        <v>261</v>
+      </c>
+      <c r="M87" s="7">
+        <v>106935.38</v>
+      </c>
+      <c r="N87" s="6">
+        <v>1</v>
+      </c>
+      <c r="O87" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P87" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q87" s="6">
+        <v>0</v>
+      </c>
+      <c r="R87" s="7">
+        <v>0</v>
+      </c>
+      <c r="S87" s="9">
+        <v>0</v>
+      </c>
+      <c r="T87" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U87" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V87" s="11">
+        <v>11</v>
+      </c>
+      <c r="W87" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X87" s="12">
+        <v>0.58958330000000003</v>
+      </c>
+      <c r="Y87" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB87" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG87" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI87" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ87" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK87" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM87" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR87" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="88" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
+        <v>1</v>
+      </c>
+      <c r="B88" s="2">
+        <v>2</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F88" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G88" s="5">
+        <v>288</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I88" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L88" s="6">
+        <v>262</v>
+      </c>
+      <c r="M88" s="7">
+        <v>107345.09</v>
+      </c>
+      <c r="N88" s="6">
+        <v>1</v>
+      </c>
+      <c r="O88" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P88" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q88" s="6">
+        <v>0</v>
+      </c>
+      <c r="R88" s="7">
+        <v>0</v>
+      </c>
+      <c r="S88" s="9">
+        <v>0</v>
+      </c>
+      <c r="T88" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U88" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V88" s="11">
+        <v>11</v>
+      </c>
+      <c r="W88" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X88" s="12">
+        <v>0.58958330000000003</v>
+      </c>
+      <c r="Y88" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB88" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG88" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI88" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ88" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK88" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM88" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR88" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="89" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>1</v>
+      </c>
+      <c r="B89" s="2">
+        <v>2</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F89" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G89" s="5">
+        <v>289</v>
+      </c>
+      <c r="H89" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I89" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J89" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K89" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L89" s="6">
+        <v>263</v>
+      </c>
+      <c r="M89" s="7">
+        <v>107754.81</v>
+      </c>
+      <c r="N89" s="6">
+        <v>1</v>
+      </c>
+      <c r="O89" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P89" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q89" s="6">
+        <v>0</v>
+      </c>
+      <c r="R89" s="7">
+        <v>0</v>
+      </c>
+      <c r="S89" s="9">
+        <v>0</v>
+      </c>
+      <c r="T89" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U89" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V89" s="11">
+        <v>11</v>
+      </c>
+      <c r="W89" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X89" s="12">
+        <v>0.58958330000000003</v>
+      </c>
+      <c r="Y89" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB89" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG89" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI89" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ89" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK89" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM89" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR89" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="90" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
+        <v>1</v>
+      </c>
+      <c r="B90" s="2">
+        <v>2</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F90" s="4">
+        <v>46118</v>
+      </c>
+      <c r="G90" s="5">
+        <v>290</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I90" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J90" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K90" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L90" s="6">
+        <v>264</v>
+      </c>
+      <c r="M90" s="7">
+        <v>108164.52</v>
+      </c>
+      <c r="N90" s="6">
+        <v>1</v>
+      </c>
+      <c r="O90" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P90" s="8">
+        <v>409.71</v>
+      </c>
+      <c r="Q90" s="6">
+        <v>0</v>
+      </c>
+      <c r="R90" s="7">
+        <v>0</v>
+      </c>
+      <c r="S90" s="9">
+        <v>0</v>
+      </c>
+      <c r="T90" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U90" s="10">
+        <v>63611</v>
+      </c>
+      <c r="V90" s="11">
+        <v>11</v>
+      </c>
+      <c r="W90" s="4">
+        <v>46118</v>
+      </c>
+      <c r="X90" s="12">
+        <v>0.58958330000000003</v>
+      </c>
+      <c r="Y90" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB90" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG90" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI90" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ90" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK90" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM90" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR90" s="3" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 23/04/2026 14:12:08,93
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCA84CF8-88FC-4079-A973-3A64DF912807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF675933-5CD5-4A37-A40B-ADA27061CE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4076" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4256" uniqueCount="292">
   <si>
     <t>Sel</t>
   </si>
@@ -725,6 +725,36 @@
   </si>
   <si>
     <t>1858700134538</t>
+  </si>
+  <si>
+    <t>1858700134539</t>
+  </si>
+  <si>
+    <t>1858700134540</t>
+  </si>
+  <si>
+    <t>1858700134541</t>
+  </si>
+  <si>
+    <t>1858700134542</t>
+  </si>
+  <si>
+    <t>1858700134543</t>
+  </si>
+  <si>
+    <t>1858700134544</t>
+  </si>
+  <si>
+    <t>1858700134545</t>
+  </si>
+  <si>
+    <t>1858700134546</t>
+  </si>
+  <si>
+    <t>1858700134547</t>
+  </si>
+  <si>
+    <t>1858700134548</t>
   </si>
   <si>
     <t>10016354</t>
@@ -1441,7 +1471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR225"/>
+  <dimension ref="A1:AR235"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -25706,7 +25736,7 @@
         <v>2</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D182" s="3" t="s">
         <v>45</v>
@@ -25718,7 +25748,7 @@
         <v>46135</v>
       </c>
       <c r="G182" s="5">
-        <v>1</v>
+        <v>282</v>
       </c>
       <c r="H182" s="3" t="s">
         <v>47</v>
@@ -25733,19 +25763,19 @@
         <v>50</v>
       </c>
       <c r="L182" s="6">
-        <v>472</v>
+        <v>1206</v>
       </c>
       <c r="M182" s="7">
-        <v>189469.84</v>
+        <v>218361.81</v>
       </c>
       <c r="N182" s="6">
         <v>1</v>
       </c>
       <c r="O182" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P182" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q182" s="6">
         <v>0</v>
@@ -25760,7 +25790,7 @@
         <v>52</v>
       </c>
       <c r="U182" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V182" s="11">
         <v>11</v>
@@ -25769,7 +25799,7 @@
         <v>46135</v>
       </c>
       <c r="X182" s="12">
-        <v>0.29652780000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y182" s="10">
         <v>0</v>
@@ -25802,7 +25832,7 @@
         <v>53</v>
       </c>
       <c r="AI182" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ182" s="3" t="s">
         <v>52</v>
@@ -25829,7 +25859,7 @@
         <v>53</v>
       </c>
       <c r="AR182" s="3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="183" spans="1:44" x14ac:dyDescent="0.3">
@@ -25840,7 +25870,7 @@
         <v>2</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D183" s="3" t="s">
         <v>45</v>
@@ -25852,7 +25882,7 @@
         <v>46135</v>
       </c>
       <c r="G183" s="5">
-        <v>2</v>
+        <v>283</v>
       </c>
       <c r="H183" s="3" t="s">
         <v>47</v>
@@ -25867,19 +25897,19 @@
         <v>50</v>
       </c>
       <c r="L183" s="6">
-        <v>473</v>
+        <v>1207</v>
       </c>
       <c r="M183" s="7">
-        <v>189871.26</v>
+        <v>218542.87</v>
       </c>
       <c r="N183" s="6">
         <v>1</v>
       </c>
       <c r="O183" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P183" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q183" s="6">
         <v>0</v>
@@ -25894,7 +25924,7 @@
         <v>52</v>
       </c>
       <c r="U183" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V183" s="11">
         <v>11</v>
@@ -25903,7 +25933,7 @@
         <v>46135</v>
       </c>
       <c r="X183" s="12">
-        <v>0.29652780000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y183" s="10">
         <v>0</v>
@@ -25936,7 +25966,7 @@
         <v>53</v>
       </c>
       <c r="AI183" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ183" s="3" t="s">
         <v>52</v>
@@ -25963,7 +25993,7 @@
         <v>53</v>
       </c>
       <c r="AR183" s="3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="184" spans="1:44" x14ac:dyDescent="0.3">
@@ -25974,7 +26004,7 @@
         <v>2</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D184" s="3" t="s">
         <v>45</v>
@@ -25986,7 +26016,7 @@
         <v>46135</v>
       </c>
       <c r="G184" s="5">
-        <v>3</v>
+        <v>284</v>
       </c>
       <c r="H184" s="3" t="s">
         <v>47</v>
@@ -26001,19 +26031,19 @@
         <v>50</v>
       </c>
       <c r="L184" s="6">
-        <v>474</v>
+        <v>1208</v>
       </c>
       <c r="M184" s="7">
-        <v>190272.67</v>
+        <v>218723.93</v>
       </c>
       <c r="N184" s="6">
         <v>1</v>
       </c>
       <c r="O184" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P184" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q184" s="6">
         <v>0</v>
@@ -26028,7 +26058,7 @@
         <v>52</v>
       </c>
       <c r="U184" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V184" s="11">
         <v>11</v>
@@ -26037,7 +26067,7 @@
         <v>46135</v>
       </c>
       <c r="X184" s="12">
-        <v>0.29652780000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y184" s="10">
         <v>0</v>
@@ -26070,34 +26100,34 @@
         <v>53</v>
       </c>
       <c r="AI184" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ184" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK184" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL184" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM184" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN184" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO184" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP184" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ184" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR184" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="AJ184" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK184" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL184" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM184" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN184" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO184" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP184" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ184" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR184" s="3" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="185" spans="1:44" x14ac:dyDescent="0.3">
@@ -26108,7 +26138,7 @@
         <v>2</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D185" s="3" t="s">
         <v>45</v>
@@ -26120,7 +26150,7 @@
         <v>46135</v>
       </c>
       <c r="G185" s="5">
-        <v>4</v>
+        <v>285</v>
       </c>
       <c r="H185" s="3" t="s">
         <v>47</v>
@@ -26135,19 +26165,19 @@
         <v>50</v>
       </c>
       <c r="L185" s="6">
-        <v>475</v>
+        <v>1209</v>
       </c>
       <c r="M185" s="7">
-        <v>190674.09</v>
+        <v>218905</v>
       </c>
       <c r="N185" s="6">
         <v>1</v>
       </c>
       <c r="O185" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P185" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q185" s="6">
         <v>0</v>
@@ -26162,7 +26192,7 @@
         <v>52</v>
       </c>
       <c r="U185" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V185" s="11">
         <v>11</v>
@@ -26171,7 +26201,7 @@
         <v>46135</v>
       </c>
       <c r="X185" s="12">
-        <v>0.29652780000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y185" s="10">
         <v>0</v>
@@ -26204,7 +26234,7 @@
         <v>53</v>
       </c>
       <c r="AI185" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ185" s="3" t="s">
         <v>52</v>
@@ -26231,7 +26261,7 @@
         <v>53</v>
       </c>
       <c r="AR185" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="186" spans="1:44" x14ac:dyDescent="0.3">
@@ -26242,7 +26272,7 @@
         <v>2</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D186" s="3" t="s">
         <v>45</v>
@@ -26254,7 +26284,7 @@
         <v>46135</v>
       </c>
       <c r="G186" s="5">
-        <v>49</v>
+        <v>286</v>
       </c>
       <c r="H186" s="3" t="s">
         <v>47</v>
@@ -26269,19 +26299,19 @@
         <v>50</v>
       </c>
       <c r="L186" s="6">
-        <v>476</v>
+        <v>1210</v>
       </c>
       <c r="M186" s="7">
-        <v>191075.51</v>
+        <v>219086.06</v>
       </c>
       <c r="N186" s="6">
         <v>1</v>
       </c>
       <c r="O186" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P186" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q186" s="6">
         <v>0</v>
@@ -26296,7 +26326,7 @@
         <v>52</v>
       </c>
       <c r="U186" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V186" s="11">
         <v>11</v>
@@ -26305,7 +26335,7 @@
         <v>46135</v>
       </c>
       <c r="X186" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y186" s="10">
         <v>0</v>
@@ -26338,7 +26368,7 @@
         <v>53</v>
       </c>
       <c r="AI186" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ186" s="3" t="s">
         <v>52</v>
@@ -26365,7 +26395,7 @@
         <v>53</v>
       </c>
       <c r="AR186" s="3" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="187" spans="1:44" x14ac:dyDescent="0.3">
@@ -26376,7 +26406,7 @@
         <v>2</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D187" s="3" t="s">
         <v>45</v>
@@ -26388,7 +26418,7 @@
         <v>46135</v>
       </c>
       <c r="G187" s="5">
-        <v>50</v>
+        <v>287</v>
       </c>
       <c r="H187" s="3" t="s">
         <v>47</v>
@@ -26403,19 +26433,19 @@
         <v>50</v>
       </c>
       <c r="L187" s="6">
-        <v>477</v>
+        <v>1211</v>
       </c>
       <c r="M187" s="7">
-        <v>191476.93</v>
+        <v>219267.12</v>
       </c>
       <c r="N187" s="6">
         <v>1</v>
       </c>
       <c r="O187" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P187" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q187" s="6">
         <v>0</v>
@@ -26430,7 +26460,7 @@
         <v>52</v>
       </c>
       <c r="U187" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V187" s="11">
         <v>11</v>
@@ -26439,7 +26469,7 @@
         <v>46135</v>
       </c>
       <c r="X187" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y187" s="10">
         <v>0</v>
@@ -26472,7 +26502,7 @@
         <v>53</v>
       </c>
       <c r="AI187" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ187" s="3" t="s">
         <v>52</v>
@@ -26499,7 +26529,7 @@
         <v>53</v>
       </c>
       <c r="AR187" s="3" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="188" spans="1:44" x14ac:dyDescent="0.3">
@@ -26510,7 +26540,7 @@
         <v>2</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D188" s="3" t="s">
         <v>45</v>
@@ -26522,7 +26552,7 @@
         <v>46135</v>
       </c>
       <c r="G188" s="5">
-        <v>51</v>
+        <v>288</v>
       </c>
       <c r="H188" s="3" t="s">
         <v>47</v>
@@ -26537,19 +26567,19 @@
         <v>50</v>
       </c>
       <c r="L188" s="6">
-        <v>478</v>
+        <v>1212</v>
       </c>
       <c r="M188" s="7">
-        <v>191878.35</v>
+        <v>219448.19</v>
       </c>
       <c r="N188" s="6">
         <v>1</v>
       </c>
       <c r="O188" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P188" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q188" s="6">
         <v>0</v>
@@ -26564,7 +26594,7 @@
         <v>52</v>
       </c>
       <c r="U188" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V188" s="11">
         <v>11</v>
@@ -26573,7 +26603,7 @@
         <v>46135</v>
       </c>
       <c r="X188" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y188" s="10">
         <v>0</v>
@@ -26606,7 +26636,7 @@
         <v>53</v>
       </c>
       <c r="AI188" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ188" s="3" t="s">
         <v>52</v>
@@ -26633,7 +26663,7 @@
         <v>53</v>
       </c>
       <c r="AR188" s="3" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="189" spans="1:44" x14ac:dyDescent="0.3">
@@ -26644,7 +26674,7 @@
         <v>2</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D189" s="3" t="s">
         <v>45</v>
@@ -26656,7 +26686,7 @@
         <v>46135</v>
       </c>
       <c r="G189" s="5">
-        <v>52</v>
+        <v>289</v>
       </c>
       <c r="H189" s="3" t="s">
         <v>47</v>
@@ -26671,19 +26701,19 @@
         <v>50</v>
       </c>
       <c r="L189" s="6">
-        <v>479</v>
+        <v>1213</v>
       </c>
       <c r="M189" s="7">
-        <v>192279.77</v>
+        <v>219629.25</v>
       </c>
       <c r="N189" s="6">
         <v>1</v>
       </c>
       <c r="O189" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P189" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q189" s="6">
         <v>0</v>
@@ -26698,7 +26728,7 @@
         <v>52</v>
       </c>
       <c r="U189" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V189" s="11">
         <v>11</v>
@@ -26707,7 +26737,7 @@
         <v>46135</v>
       </c>
       <c r="X189" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y189" s="10">
         <v>0</v>
@@ -26740,7 +26770,7 @@
         <v>53</v>
       </c>
       <c r="AI189" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ189" s="3" t="s">
         <v>52</v>
@@ -26767,7 +26797,7 @@
         <v>53</v>
       </c>
       <c r="AR189" s="3" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="190" spans="1:44" x14ac:dyDescent="0.3">
@@ -26778,7 +26808,7 @@
         <v>2</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D190" s="3" t="s">
         <v>45</v>
@@ -26790,7 +26820,7 @@
         <v>46135</v>
       </c>
       <c r="G190" s="5">
-        <v>53</v>
+        <v>290</v>
       </c>
       <c r="H190" s="3" t="s">
         <v>47</v>
@@ -26805,19 +26835,19 @@
         <v>50</v>
       </c>
       <c r="L190" s="6">
-        <v>480</v>
+        <v>1214</v>
       </c>
       <c r="M190" s="7">
-        <v>192681.19</v>
+        <v>219810.31</v>
       </c>
       <c r="N190" s="6">
         <v>1</v>
       </c>
       <c r="O190" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P190" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q190" s="6">
         <v>0</v>
@@ -26832,7 +26862,7 @@
         <v>52</v>
       </c>
       <c r="U190" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V190" s="11">
         <v>11</v>
@@ -26841,7 +26871,7 @@
         <v>46135</v>
       </c>
       <c r="X190" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y190" s="10">
         <v>0</v>
@@ -26874,7 +26904,7 @@
         <v>53</v>
       </c>
       <c r="AI190" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ190" s="3" t="s">
         <v>52</v>
@@ -26901,7 +26931,7 @@
         <v>53</v>
       </c>
       <c r="AR190" s="3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="191" spans="1:44" x14ac:dyDescent="0.3">
@@ -26912,7 +26942,7 @@
         <v>2</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>235</v>
+        <v>44</v>
       </c>
       <c r="D191" s="3" t="s">
         <v>45</v>
@@ -26924,7 +26954,7 @@
         <v>46135</v>
       </c>
       <c r="G191" s="5">
-        <v>54</v>
+        <v>291</v>
       </c>
       <c r="H191" s="3" t="s">
         <v>47</v>
@@ -26939,19 +26969,19 @@
         <v>50</v>
       </c>
       <c r="L191" s="6">
-        <v>481</v>
+        <v>1215</v>
       </c>
       <c r="M191" s="7">
-        <v>193082.61</v>
+        <v>219991.37</v>
       </c>
       <c r="N191" s="6">
         <v>1</v>
       </c>
       <c r="O191" s="3" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="P191" s="8">
-        <v>401.42</v>
+        <v>181.06</v>
       </c>
       <c r="Q191" s="6">
         <v>0</v>
@@ -26966,7 +26996,7 @@
         <v>52</v>
       </c>
       <c r="U191" s="10">
-        <v>63954</v>
+        <v>63988</v>
       </c>
       <c r="V191" s="11">
         <v>11</v>
@@ -26975,7 +27005,7 @@
         <v>46135</v>
       </c>
       <c r="X191" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.58819440000000001</v>
       </c>
       <c r="Y191" s="10">
         <v>0</v>
@@ -27008,7 +27038,7 @@
         <v>53</v>
       </c>
       <c r="AI191" s="3" t="s">
-        <v>237</v>
+        <v>54</v>
       </c>
       <c r="AJ191" s="3" t="s">
         <v>52</v>
@@ -27035,7 +27065,7 @@
         <v>53</v>
       </c>
       <c r="AR191" s="3" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="192" spans="1:44" x14ac:dyDescent="0.3">
@@ -27046,7 +27076,7 @@
         <v>2</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D192" s="3" t="s">
         <v>45</v>
@@ -27058,7 +27088,7 @@
         <v>46135</v>
       </c>
       <c r="G192" s="5">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="H192" s="3" t="s">
         <v>47</v>
@@ -27073,16 +27103,16 @@
         <v>50</v>
       </c>
       <c r="L192" s="6">
-        <v>482</v>
+        <v>472</v>
       </c>
       <c r="M192" s="7">
-        <v>193484.03</v>
+        <v>189469.84</v>
       </c>
       <c r="N192" s="6">
         <v>1</v>
       </c>
       <c r="O192" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P192" s="8">
         <v>401.42</v>
@@ -27109,7 +27139,7 @@
         <v>46135</v>
       </c>
       <c r="X192" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.29652780000000001</v>
       </c>
       <c r="Y192" s="10">
         <v>0</v>
@@ -27142,7 +27172,7 @@
         <v>53</v>
       </c>
       <c r="AI192" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ192" s="3" t="s">
         <v>52</v>
@@ -27180,7 +27210,7 @@
         <v>2</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D193" s="3" t="s">
         <v>45</v>
@@ -27192,7 +27222,7 @@
         <v>46135</v>
       </c>
       <c r="G193" s="5">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="H193" s="3" t="s">
         <v>47</v>
@@ -27207,16 +27237,16 @@
         <v>50</v>
       </c>
       <c r="L193" s="6">
-        <v>483</v>
+        <v>473</v>
       </c>
       <c r="M193" s="7">
-        <v>193885.45</v>
+        <v>189871.26</v>
       </c>
       <c r="N193" s="6">
         <v>1</v>
       </c>
       <c r="O193" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P193" s="8">
         <v>401.42</v>
@@ -27243,7 +27273,7 @@
         <v>46135</v>
       </c>
       <c r="X193" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.29652780000000001</v>
       </c>
       <c r="Y193" s="10">
         <v>0</v>
@@ -27276,7 +27306,7 @@
         <v>53</v>
       </c>
       <c r="AI193" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ193" s="3" t="s">
         <v>52</v>
@@ -27314,7 +27344,7 @@
         <v>2</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D194" s="3" t="s">
         <v>45</v>
@@ -27326,7 +27356,7 @@
         <v>46135</v>
       </c>
       <c r="G194" s="5">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="H194" s="3" t="s">
         <v>47</v>
@@ -27341,16 +27371,16 @@
         <v>50</v>
       </c>
       <c r="L194" s="6">
-        <v>484</v>
+        <v>474</v>
       </c>
       <c r="M194" s="7">
-        <v>194286.87</v>
+        <v>190272.67</v>
       </c>
       <c r="N194" s="6">
         <v>1</v>
       </c>
       <c r="O194" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P194" s="8">
         <v>401.42</v>
@@ -27377,7 +27407,7 @@
         <v>46135</v>
       </c>
       <c r="X194" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.29652780000000001</v>
       </c>
       <c r="Y194" s="10">
         <v>0</v>
@@ -27410,7 +27440,7 @@
         <v>53</v>
       </c>
       <c r="AI194" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ194" s="3" t="s">
         <v>52</v>
@@ -27448,7 +27478,7 @@
         <v>2</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D195" s="3" t="s">
         <v>45</v>
@@ -27460,7 +27490,7 @@
         <v>46135</v>
       </c>
       <c r="G195" s="5">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="H195" s="3" t="s">
         <v>47</v>
@@ -27475,16 +27505,16 @@
         <v>50</v>
       </c>
       <c r="L195" s="6">
-        <v>485</v>
+        <v>475</v>
       </c>
       <c r="M195" s="7">
-        <v>194688.29</v>
+        <v>190674.09</v>
       </c>
       <c r="N195" s="6">
         <v>1</v>
       </c>
       <c r="O195" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P195" s="8">
         <v>401.42</v>
@@ -27511,7 +27541,7 @@
         <v>46135</v>
       </c>
       <c r="X195" s="12">
-        <v>0.37986110000000001</v>
+        <v>0.29652780000000001</v>
       </c>
       <c r="Y195" s="10">
         <v>0</v>
@@ -27544,7 +27574,7 @@
         <v>53</v>
       </c>
       <c r="AI195" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ195" s="3" t="s">
         <v>52</v>
@@ -27582,7 +27612,7 @@
         <v>2</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D196" s="3" t="s">
         <v>45</v>
@@ -27594,7 +27624,7 @@
         <v>46135</v>
       </c>
       <c r="G196" s="5">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H196" s="3" t="s">
         <v>47</v>
@@ -27609,16 +27639,16 @@
         <v>50</v>
       </c>
       <c r="L196" s="6">
-        <v>486</v>
+        <v>476</v>
       </c>
       <c r="M196" s="7">
-        <v>195089.7</v>
+        <v>191075.51</v>
       </c>
       <c r="N196" s="6">
         <v>1</v>
       </c>
       <c r="O196" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P196" s="8">
         <v>401.42</v>
@@ -27678,7 +27708,7 @@
         <v>53</v>
       </c>
       <c r="AI196" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ196" s="3" t="s">
         <v>52</v>
@@ -27716,7 +27746,7 @@
         <v>2</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D197" s="3" t="s">
         <v>45</v>
@@ -27728,7 +27758,7 @@
         <v>46135</v>
       </c>
       <c r="G197" s="5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H197" s="3" t="s">
         <v>47</v>
@@ -27743,16 +27773,16 @@
         <v>50</v>
       </c>
       <c r="L197" s="6">
-        <v>487</v>
+        <v>477</v>
       </c>
       <c r="M197" s="7">
-        <v>195491.12</v>
+        <v>191476.93</v>
       </c>
       <c r="N197" s="6">
         <v>1</v>
       </c>
       <c r="O197" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P197" s="8">
         <v>401.42</v>
@@ -27812,7 +27842,7 @@
         <v>53</v>
       </c>
       <c r="AI197" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ197" s="3" t="s">
         <v>52</v>
@@ -27850,7 +27880,7 @@
         <v>2</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>45</v>
@@ -27862,7 +27892,7 @@
         <v>46135</v>
       </c>
       <c r="G198" s="5">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H198" s="3" t="s">
         <v>47</v>
@@ -27877,16 +27907,16 @@
         <v>50</v>
       </c>
       <c r="L198" s="6">
-        <v>488</v>
+        <v>478</v>
       </c>
       <c r="M198" s="7">
-        <v>195892.54</v>
+        <v>191878.35</v>
       </c>
       <c r="N198" s="6">
         <v>1</v>
       </c>
       <c r="O198" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P198" s="8">
         <v>401.42</v>
@@ -27946,7 +27976,7 @@
         <v>53</v>
       </c>
       <c r="AI198" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ198" s="3" t="s">
         <v>52</v>
@@ -27984,7 +28014,7 @@
         <v>2</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D199" s="3" t="s">
         <v>45</v>
@@ -27996,7 +28026,7 @@
         <v>46135</v>
       </c>
       <c r="G199" s="5">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="H199" s="3" t="s">
         <v>47</v>
@@ -28011,16 +28041,16 @@
         <v>50</v>
       </c>
       <c r="L199" s="6">
-        <v>489</v>
+        <v>479</v>
       </c>
       <c r="M199" s="7">
-        <v>196293.96</v>
+        <v>192279.77</v>
       </c>
       <c r="N199" s="6">
         <v>1</v>
       </c>
       <c r="O199" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P199" s="8">
         <v>401.42</v>
@@ -28080,7 +28110,7 @@
         <v>53</v>
       </c>
       <c r="AI199" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ199" s="3" t="s">
         <v>52</v>
@@ -28118,7 +28148,7 @@
         <v>2</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D200" s="3" t="s">
         <v>45</v>
@@ -28130,7 +28160,7 @@
         <v>46135</v>
       </c>
       <c r="G200" s="5">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="H200" s="3" t="s">
         <v>47</v>
@@ -28145,16 +28175,16 @@
         <v>50</v>
       </c>
       <c r="L200" s="6">
-        <v>490</v>
+        <v>480</v>
       </c>
       <c r="M200" s="7">
-        <v>196695.38</v>
+        <v>192681.19</v>
       </c>
       <c r="N200" s="6">
         <v>1</v>
       </c>
       <c r="O200" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P200" s="8">
         <v>401.42</v>
@@ -28214,7 +28244,7 @@
         <v>53</v>
       </c>
       <c r="AI200" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ200" s="3" t="s">
         <v>52</v>
@@ -28252,7 +28282,7 @@
         <v>2</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D201" s="3" t="s">
         <v>45</v>
@@ -28264,7 +28294,7 @@
         <v>46135</v>
       </c>
       <c r="G201" s="5">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="H201" s="3" t="s">
         <v>47</v>
@@ -28279,16 +28309,16 @@
         <v>50</v>
       </c>
       <c r="L201" s="6">
-        <v>491</v>
+        <v>481</v>
       </c>
       <c r="M201" s="7">
-        <v>197096.8</v>
+        <v>193082.61</v>
       </c>
       <c r="N201" s="6">
         <v>1</v>
       </c>
       <c r="O201" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P201" s="8">
         <v>401.42</v>
@@ -28348,7 +28378,7 @@
         <v>53</v>
       </c>
       <c r="AI201" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ201" s="3" t="s">
         <v>52</v>
@@ -28386,7 +28416,7 @@
         <v>2</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D202" s="3" t="s">
         <v>45</v>
@@ -28398,7 +28428,7 @@
         <v>46135</v>
       </c>
       <c r="G202" s="5">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H202" s="3" t="s">
         <v>47</v>
@@ -28413,16 +28443,16 @@
         <v>50</v>
       </c>
       <c r="L202" s="6">
-        <v>492</v>
+        <v>482</v>
       </c>
       <c r="M202" s="7">
-        <v>197498.22</v>
+        <v>193484.03</v>
       </c>
       <c r="N202" s="6">
         <v>1</v>
       </c>
       <c r="O202" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P202" s="8">
         <v>401.42</v>
@@ -28482,7 +28512,7 @@
         <v>53</v>
       </c>
       <c r="AI202" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ202" s="3" t="s">
         <v>52</v>
@@ -28520,7 +28550,7 @@
         <v>2</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D203" s="3" t="s">
         <v>45</v>
@@ -28532,7 +28562,7 @@
         <v>46135</v>
       </c>
       <c r="G203" s="5">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="H203" s="3" t="s">
         <v>47</v>
@@ -28547,16 +28577,16 @@
         <v>50</v>
       </c>
       <c r="L203" s="6">
-        <v>493</v>
+        <v>483</v>
       </c>
       <c r="M203" s="7">
-        <v>197899.64</v>
+        <v>193885.45</v>
       </c>
       <c r="N203" s="6">
         <v>1</v>
       </c>
       <c r="O203" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P203" s="8">
         <v>401.42</v>
@@ -28616,7 +28646,7 @@
         <v>53</v>
       </c>
       <c r="AI203" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ203" s="3" t="s">
         <v>52</v>
@@ -28654,7 +28684,7 @@
         <v>2</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D204" s="3" t="s">
         <v>45</v>
@@ -28666,7 +28696,7 @@
         <v>46135</v>
       </c>
       <c r="G204" s="5">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="H204" s="3" t="s">
         <v>47</v>
@@ -28681,16 +28711,16 @@
         <v>50</v>
       </c>
       <c r="L204" s="6">
-        <v>494</v>
+        <v>484</v>
       </c>
       <c r="M204" s="7">
-        <v>198301.06</v>
+        <v>194286.87</v>
       </c>
       <c r="N204" s="6">
         <v>1</v>
       </c>
       <c r="O204" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P204" s="8">
         <v>401.42</v>
@@ -28750,7 +28780,7 @@
         <v>53</v>
       </c>
       <c r="AI204" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ204" s="3" t="s">
         <v>52</v>
@@ -28788,7 +28818,7 @@
         <v>2</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D205" s="3" t="s">
         <v>45</v>
@@ -28800,7 +28830,7 @@
         <v>46135</v>
       </c>
       <c r="G205" s="5">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="H205" s="3" t="s">
         <v>47</v>
@@ -28815,16 +28845,16 @@
         <v>50</v>
       </c>
       <c r="L205" s="6">
-        <v>495</v>
+        <v>485</v>
       </c>
       <c r="M205" s="7">
-        <v>198702.48</v>
+        <v>194688.29</v>
       </c>
       <c r="N205" s="6">
         <v>1</v>
       </c>
       <c r="O205" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P205" s="8">
         <v>401.42</v>
@@ -28884,7 +28914,7 @@
         <v>53</v>
       </c>
       <c r="AI205" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ205" s="3" t="s">
         <v>52</v>
@@ -28922,7 +28952,7 @@
         <v>2</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D206" s="3" t="s">
         <v>45</v>
@@ -28934,7 +28964,7 @@
         <v>46135</v>
       </c>
       <c r="G206" s="5">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H206" s="3" t="s">
         <v>47</v>
@@ -28949,16 +28979,16 @@
         <v>50</v>
       </c>
       <c r="L206" s="6">
-        <v>496</v>
+        <v>486</v>
       </c>
       <c r="M206" s="7">
-        <v>199103.9</v>
+        <v>195089.7</v>
       </c>
       <c r="N206" s="6">
         <v>1</v>
       </c>
       <c r="O206" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P206" s="8">
         <v>401.42</v>
@@ -29018,7 +29048,7 @@
         <v>53</v>
       </c>
       <c r="AI206" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ206" s="3" t="s">
         <v>52</v>
@@ -29056,7 +29086,7 @@
         <v>2</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D207" s="3" t="s">
         <v>45</v>
@@ -29068,7 +29098,7 @@
         <v>46135</v>
       </c>
       <c r="G207" s="5">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H207" s="3" t="s">
         <v>47</v>
@@ -29083,16 +29113,16 @@
         <v>50</v>
       </c>
       <c r="L207" s="6">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="M207" s="7">
-        <v>199505.31</v>
+        <v>195491.12</v>
       </c>
       <c r="N207" s="6">
         <v>1</v>
       </c>
       <c r="O207" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P207" s="8">
         <v>401.42</v>
@@ -29152,7 +29182,7 @@
         <v>53</v>
       </c>
       <c r="AI207" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ207" s="3" t="s">
         <v>52</v>
@@ -29190,7 +29220,7 @@
         <v>2</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D208" s="3" t="s">
         <v>45</v>
@@ -29202,7 +29232,7 @@
         <v>46135</v>
       </c>
       <c r="G208" s="5">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="H208" s="3" t="s">
         <v>47</v>
@@ -29217,16 +29247,16 @@
         <v>50</v>
       </c>
       <c r="L208" s="6">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="M208" s="7">
-        <v>199906.73</v>
+        <v>195892.54</v>
       </c>
       <c r="N208" s="6">
         <v>1</v>
       </c>
       <c r="O208" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P208" s="8">
         <v>401.42</v>
@@ -29286,7 +29316,7 @@
         <v>53</v>
       </c>
       <c r="AI208" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ208" s="3" t="s">
         <v>52</v>
@@ -29324,7 +29354,7 @@
         <v>2</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D209" s="3" t="s">
         <v>45</v>
@@ -29336,7 +29366,7 @@
         <v>46135</v>
       </c>
       <c r="G209" s="5">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="H209" s="3" t="s">
         <v>47</v>
@@ -29351,16 +29381,16 @@
         <v>50</v>
       </c>
       <c r="L209" s="6">
-        <v>499</v>
+        <v>489</v>
       </c>
       <c r="M209" s="7">
-        <v>200308.15</v>
+        <v>196293.96</v>
       </c>
       <c r="N209" s="6">
         <v>1</v>
       </c>
       <c r="O209" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P209" s="8">
         <v>401.42</v>
@@ -29420,7 +29450,7 @@
         <v>53</v>
       </c>
       <c r="AI209" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ209" s="3" t="s">
         <v>52</v>
@@ -29458,7 +29488,7 @@
         <v>2</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D210" s="3" t="s">
         <v>45</v>
@@ -29470,7 +29500,7 @@
         <v>46135</v>
       </c>
       <c r="G210" s="5">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="H210" s="3" t="s">
         <v>47</v>
@@ -29485,16 +29515,16 @@
         <v>50</v>
       </c>
       <c r="L210" s="6">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="M210" s="7">
-        <v>200709.57</v>
+        <v>196695.38</v>
       </c>
       <c r="N210" s="6">
         <v>1</v>
       </c>
       <c r="O210" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P210" s="8">
         <v>401.42</v>
@@ -29554,7 +29584,7 @@
         <v>53</v>
       </c>
       <c r="AI210" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ210" s="3" t="s">
         <v>52</v>
@@ -29592,7 +29622,7 @@
         <v>2</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D211" s="3" t="s">
         <v>45</v>
@@ -29604,7 +29634,7 @@
         <v>46135</v>
       </c>
       <c r="G211" s="5">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="H211" s="3" t="s">
         <v>47</v>
@@ -29619,16 +29649,16 @@
         <v>50</v>
       </c>
       <c r="L211" s="6">
-        <v>501</v>
+        <v>491</v>
       </c>
       <c r="M211" s="7">
-        <v>201110.99</v>
+        <v>197096.8</v>
       </c>
       <c r="N211" s="6">
         <v>1</v>
       </c>
       <c r="O211" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P211" s="8">
         <v>401.42</v>
@@ -29688,7 +29718,7 @@
         <v>53</v>
       </c>
       <c r="AI211" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ211" s="3" t="s">
         <v>52</v>
@@ -29726,7 +29756,7 @@
         <v>2</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D212" s="3" t="s">
         <v>45</v>
@@ -29738,7 +29768,7 @@
         <v>46135</v>
       </c>
       <c r="G212" s="5">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H212" s="3" t="s">
         <v>47</v>
@@ -29753,16 +29783,16 @@
         <v>50</v>
       </c>
       <c r="L212" s="6">
-        <v>502</v>
+        <v>492</v>
       </c>
       <c r="M212" s="7">
-        <v>201512.41</v>
+        <v>197498.22</v>
       </c>
       <c r="N212" s="6">
         <v>1</v>
       </c>
       <c r="O212" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P212" s="8">
         <v>401.42</v>
@@ -29822,7 +29852,7 @@
         <v>53</v>
       </c>
       <c r="AI212" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ212" s="3" t="s">
         <v>52</v>
@@ -29860,7 +29890,7 @@
         <v>2</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D213" s="3" t="s">
         <v>45</v>
@@ -29872,7 +29902,7 @@
         <v>46135</v>
       </c>
       <c r="G213" s="5">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="H213" s="3" t="s">
         <v>47</v>
@@ -29887,16 +29917,16 @@
         <v>50</v>
       </c>
       <c r="L213" s="6">
-        <v>503</v>
+        <v>493</v>
       </c>
       <c r="M213" s="7">
-        <v>201913.83</v>
+        <v>197899.64</v>
       </c>
       <c r="N213" s="6">
         <v>1</v>
       </c>
       <c r="O213" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P213" s="8">
         <v>401.42</v>
@@ -29956,7 +29986,7 @@
         <v>53</v>
       </c>
       <c r="AI213" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ213" s="3" t="s">
         <v>52</v>
@@ -29994,7 +30024,7 @@
         <v>2</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D214" s="3" t="s">
         <v>45</v>
@@ -30006,7 +30036,7 @@
         <v>46135</v>
       </c>
       <c r="G214" s="5">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="H214" s="3" t="s">
         <v>47</v>
@@ -30021,16 +30051,16 @@
         <v>50</v>
       </c>
       <c r="L214" s="6">
-        <v>504</v>
+        <v>494</v>
       </c>
       <c r="M214" s="7">
-        <v>202315.25</v>
+        <v>198301.06</v>
       </c>
       <c r="N214" s="6">
         <v>1</v>
       </c>
       <c r="O214" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P214" s="8">
         <v>401.42</v>
@@ -30057,7 +30087,7 @@
         <v>46135</v>
       </c>
       <c r="X214" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y214" s="10">
         <v>0</v>
@@ -30090,7 +30120,7 @@
         <v>53</v>
       </c>
       <c r="AI214" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ214" s="3" t="s">
         <v>52</v>
@@ -30128,7 +30158,7 @@
         <v>2</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D215" s="3" t="s">
         <v>45</v>
@@ -30140,7 +30170,7 @@
         <v>46135</v>
       </c>
       <c r="G215" s="5">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H215" s="3" t="s">
         <v>47</v>
@@ -30155,16 +30185,16 @@
         <v>50</v>
       </c>
       <c r="L215" s="6">
-        <v>505</v>
+        <v>495</v>
       </c>
       <c r="M215" s="7">
-        <v>202716.67</v>
+        <v>198702.48</v>
       </c>
       <c r="N215" s="6">
         <v>1</v>
       </c>
       <c r="O215" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P215" s="8">
         <v>401.42</v>
@@ -30191,7 +30221,7 @@
         <v>46135</v>
       </c>
       <c r="X215" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y215" s="10">
         <v>0</v>
@@ -30224,7 +30254,7 @@
         <v>53</v>
       </c>
       <c r="AI215" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ215" s="3" t="s">
         <v>52</v>
@@ -30262,7 +30292,7 @@
         <v>2</v>
       </c>
       <c r="C216" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D216" s="3" t="s">
         <v>45</v>
@@ -30274,7 +30304,7 @@
         <v>46135</v>
       </c>
       <c r="G216" s="5">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H216" s="3" t="s">
         <v>47</v>
@@ -30289,16 +30319,16 @@
         <v>50</v>
       </c>
       <c r="L216" s="6">
-        <v>506</v>
+        <v>496</v>
       </c>
       <c r="M216" s="7">
-        <v>203118.09</v>
+        <v>199103.9</v>
       </c>
       <c r="N216" s="6">
         <v>1</v>
       </c>
       <c r="O216" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P216" s="8">
         <v>401.42</v>
@@ -30325,7 +30355,7 @@
         <v>46135</v>
       </c>
       <c r="X216" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y216" s="10">
         <v>0</v>
@@ -30358,7 +30388,7 @@
         <v>53</v>
       </c>
       <c r="AI216" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ216" s="3" t="s">
         <v>52</v>
@@ -30396,7 +30426,7 @@
         <v>2</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D217" s="3" t="s">
         <v>45</v>
@@ -30408,7 +30438,7 @@
         <v>46135</v>
       </c>
       <c r="G217" s="5">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H217" s="3" t="s">
         <v>47</v>
@@ -30423,16 +30453,16 @@
         <v>50</v>
       </c>
       <c r="L217" s="6">
-        <v>507</v>
+        <v>497</v>
       </c>
       <c r="M217" s="7">
-        <v>203519.51</v>
+        <v>199505.31</v>
       </c>
       <c r="N217" s="6">
         <v>1</v>
       </c>
       <c r="O217" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P217" s="8">
         <v>401.42</v>
@@ -30459,7 +30489,7 @@
         <v>46135</v>
       </c>
       <c r="X217" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y217" s="10">
         <v>0</v>
@@ -30492,7 +30522,7 @@
         <v>53</v>
       </c>
       <c r="AI217" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ217" s="3" t="s">
         <v>52</v>
@@ -30530,7 +30560,7 @@
         <v>2</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D218" s="3" t="s">
         <v>45</v>
@@ -30542,7 +30572,7 @@
         <v>46135</v>
       </c>
       <c r="G218" s="5">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="H218" s="3" t="s">
         <v>47</v>
@@ -30557,16 +30587,16 @@
         <v>50</v>
       </c>
       <c r="L218" s="6">
-        <v>508</v>
+        <v>498</v>
       </c>
       <c r="M218" s="7">
-        <v>203920.93</v>
+        <v>199906.73</v>
       </c>
       <c r="N218" s="6">
         <v>1</v>
       </c>
       <c r="O218" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P218" s="8">
         <v>401.42</v>
@@ -30593,7 +30623,7 @@
         <v>46135</v>
       </c>
       <c r="X218" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y218" s="10">
         <v>0</v>
@@ -30626,7 +30656,7 @@
         <v>53</v>
       </c>
       <c r="AI218" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ218" s="3" t="s">
         <v>52</v>
@@ -30664,7 +30694,7 @@
         <v>2</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D219" s="3" t="s">
         <v>45</v>
@@ -30676,7 +30706,7 @@
         <v>46135</v>
       </c>
       <c r="G219" s="5">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="H219" s="3" t="s">
         <v>47</v>
@@ -30691,16 +30721,16 @@
         <v>50</v>
       </c>
       <c r="L219" s="6">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="M219" s="7">
-        <v>204322.34</v>
+        <v>200308.15</v>
       </c>
       <c r="N219" s="6">
         <v>1</v>
       </c>
       <c r="O219" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P219" s="8">
         <v>401.42</v>
@@ -30727,7 +30757,7 @@
         <v>46135</v>
       </c>
       <c r="X219" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y219" s="10">
         <v>0</v>
@@ -30760,7 +30790,7 @@
         <v>53</v>
       </c>
       <c r="AI219" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ219" s="3" t="s">
         <v>52</v>
@@ -30798,7 +30828,7 @@
         <v>2</v>
       </c>
       <c r="C220" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D220" s="3" t="s">
         <v>45</v>
@@ -30810,7 +30840,7 @@
         <v>46135</v>
       </c>
       <c r="G220" s="5">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="H220" s="3" t="s">
         <v>47</v>
@@ -30825,16 +30855,16 @@
         <v>50</v>
       </c>
       <c r="L220" s="6">
-        <v>510</v>
+        <v>500</v>
       </c>
       <c r="M220" s="7">
-        <v>204723.76</v>
+        <v>200709.57</v>
       </c>
       <c r="N220" s="6">
         <v>1</v>
       </c>
       <c r="O220" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P220" s="8">
         <v>401.42</v>
@@ -30861,7 +30891,7 @@
         <v>46135</v>
       </c>
       <c r="X220" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y220" s="10">
         <v>0</v>
@@ -30894,7 +30924,7 @@
         <v>53</v>
       </c>
       <c r="AI220" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ220" s="3" t="s">
         <v>52</v>
@@ -30932,7 +30962,7 @@
         <v>2</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D221" s="3" t="s">
         <v>45</v>
@@ -30944,7 +30974,7 @@
         <v>46135</v>
       </c>
       <c r="G221" s="5">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="H221" s="3" t="s">
         <v>47</v>
@@ -30959,16 +30989,16 @@
         <v>50</v>
       </c>
       <c r="L221" s="6">
-        <v>511</v>
+        <v>501</v>
       </c>
       <c r="M221" s="7">
-        <v>205125.18</v>
+        <v>201110.99</v>
       </c>
       <c r="N221" s="6">
         <v>1</v>
       </c>
       <c r="O221" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P221" s="8">
         <v>401.42</v>
@@ -30995,7 +31025,7 @@
         <v>46135</v>
       </c>
       <c r="X221" s="12">
-        <v>0.4</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y221" s="10">
         <v>0</v>
@@ -31028,7 +31058,7 @@
         <v>53</v>
       </c>
       <c r="AI221" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ221" s="3" t="s">
         <v>52</v>
@@ -31066,7 +31096,7 @@
         <v>2</v>
       </c>
       <c r="C222" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D222" s="3" t="s">
         <v>45</v>
@@ -31078,7 +31108,7 @@
         <v>46135</v>
       </c>
       <c r="G222" s="5">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="H222" s="3" t="s">
         <v>47</v>
@@ -31093,16 +31123,16 @@
         <v>50</v>
       </c>
       <c r="L222" s="6">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="M222" s="7">
-        <v>205526.6</v>
+        <v>201512.41</v>
       </c>
       <c r="N222" s="6">
         <v>1</v>
       </c>
       <c r="O222" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P222" s="8">
         <v>401.42</v>
@@ -31129,7 +31159,7 @@
         <v>46135</v>
       </c>
       <c r="X222" s="12">
-        <v>0.42083330000000002</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y222" s="10">
         <v>0</v>
@@ -31162,7 +31192,7 @@
         <v>53</v>
       </c>
       <c r="AI222" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ222" s="3" t="s">
         <v>52</v>
@@ -31200,7 +31230,7 @@
         <v>2</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D223" s="3" t="s">
         <v>45</v>
@@ -31212,7 +31242,7 @@
         <v>46135</v>
       </c>
       <c r="G223" s="5">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="H223" s="3" t="s">
         <v>47</v>
@@ -31227,16 +31257,16 @@
         <v>50</v>
       </c>
       <c r="L223" s="6">
-        <v>513</v>
+        <v>503</v>
       </c>
       <c r="M223" s="7">
-        <v>205928.02</v>
+        <v>201913.83</v>
       </c>
       <c r="N223" s="6">
         <v>1</v>
       </c>
       <c r="O223" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P223" s="8">
         <v>401.42</v>
@@ -31263,7 +31293,7 @@
         <v>46135</v>
       </c>
       <c r="X223" s="12">
-        <v>0.42083330000000002</v>
+        <v>0.37986110000000001</v>
       </c>
       <c r="Y223" s="10">
         <v>0</v>
@@ -31296,7 +31326,7 @@
         <v>53</v>
       </c>
       <c r="AI223" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ223" s="3" t="s">
         <v>52</v>
@@ -31334,7 +31364,7 @@
         <v>2</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D224" s="3" t="s">
         <v>45</v>
@@ -31346,7 +31376,7 @@
         <v>46135</v>
       </c>
       <c r="G224" s="5">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="H224" s="3" t="s">
         <v>47</v>
@@ -31361,16 +31391,16 @@
         <v>50</v>
       </c>
       <c r="L224" s="6">
-        <v>514</v>
+        <v>504</v>
       </c>
       <c r="M224" s="7">
-        <v>206329.44</v>
+        <v>202315.25</v>
       </c>
       <c r="N224" s="6">
         <v>1</v>
       </c>
       <c r="O224" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P224" s="8">
         <v>401.42</v>
@@ -31397,7 +31427,7 @@
         <v>46135</v>
       </c>
       <c r="X224" s="12">
-        <v>0.42083330000000002</v>
+        <v>0.4</v>
       </c>
       <c r="Y224" s="10">
         <v>0</v>
@@ -31430,7 +31460,7 @@
         <v>53</v>
       </c>
       <c r="AI224" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ224" s="3" t="s">
         <v>52</v>
@@ -31468,7 +31498,7 @@
         <v>2</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="D225" s="3" t="s">
         <v>45</v>
@@ -31480,7 +31510,7 @@
         <v>46135</v>
       </c>
       <c r="G225" s="5">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="H225" s="3" t="s">
         <v>47</v>
@@ -31495,16 +31525,16 @@
         <v>50</v>
       </c>
       <c r="L225" s="6">
-        <v>515</v>
+        <v>505</v>
       </c>
       <c r="M225" s="7">
-        <v>206730.86</v>
+        <v>202716.67</v>
       </c>
       <c r="N225" s="6">
         <v>1</v>
       </c>
       <c r="O225" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="P225" s="8">
         <v>401.42</v>
@@ -31531,7 +31561,7 @@
         <v>46135</v>
       </c>
       <c r="X225" s="12">
-        <v>0.42083330000000002</v>
+        <v>0.4</v>
       </c>
       <c r="Y225" s="10">
         <v>0</v>
@@ -31564,7 +31594,7 @@
         <v>53</v>
       </c>
       <c r="AI225" s="3" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="AJ225" s="3" t="s">
         <v>52</v>
@@ -31592,6 +31622,1346 @@
       </c>
       <c r="AR225" s="3" t="s">
         <v>281</v>
+      </c>
+    </row>
+    <row r="226" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A226" s="1">
+        <v>1</v>
+      </c>
+      <c r="B226" s="2">
+        <v>2</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E226" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F226" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G226" s="5">
+        <v>79</v>
+      </c>
+      <c r="H226" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I226" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J226" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K226" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L226" s="6">
+        <v>506</v>
+      </c>
+      <c r="M226" s="7">
+        <v>203118.09</v>
+      </c>
+      <c r="N226" s="6">
+        <v>1</v>
+      </c>
+      <c r="O226" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P226" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q226" s="6">
+        <v>0</v>
+      </c>
+      <c r="R226" s="7">
+        <v>0</v>
+      </c>
+      <c r="S226" s="9">
+        <v>0</v>
+      </c>
+      <c r="T226" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U226" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V226" s="11">
+        <v>11</v>
+      </c>
+      <c r="W226" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X226" s="12">
+        <v>0.4</v>
+      </c>
+      <c r="Y226" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB226" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG226" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI226" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ226" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK226" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM226" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR226" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="227" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A227" s="1">
+        <v>1</v>
+      </c>
+      <c r="B227" s="2">
+        <v>2</v>
+      </c>
+      <c r="C227" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D227" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E227" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F227" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G227" s="5">
+        <v>80</v>
+      </c>
+      <c r="H227" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I227" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J227" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K227" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L227" s="6">
+        <v>507</v>
+      </c>
+      <c r="M227" s="7">
+        <v>203519.51</v>
+      </c>
+      <c r="N227" s="6">
+        <v>1</v>
+      </c>
+      <c r="O227" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P227" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q227" s="6">
+        <v>0</v>
+      </c>
+      <c r="R227" s="7">
+        <v>0</v>
+      </c>
+      <c r="S227" s="9">
+        <v>0</v>
+      </c>
+      <c r="T227" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U227" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V227" s="11">
+        <v>11</v>
+      </c>
+      <c r="W227" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X227" s="12">
+        <v>0.4</v>
+      </c>
+      <c r="Y227" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB227" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG227" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI227" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ227" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK227" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM227" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR227" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="228" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A228" s="1">
+        <v>1</v>
+      </c>
+      <c r="B228" s="2">
+        <v>2</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D228" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E228" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F228" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G228" s="5">
+        <v>81</v>
+      </c>
+      <c r="H228" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I228" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J228" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K228" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L228" s="6">
+        <v>508</v>
+      </c>
+      <c r="M228" s="7">
+        <v>203920.93</v>
+      </c>
+      <c r="N228" s="6">
+        <v>1</v>
+      </c>
+      <c r="O228" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P228" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q228" s="6">
+        <v>0</v>
+      </c>
+      <c r="R228" s="7">
+        <v>0</v>
+      </c>
+      <c r="S228" s="9">
+        <v>0</v>
+      </c>
+      <c r="T228" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U228" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V228" s="11">
+        <v>11</v>
+      </c>
+      <c r="W228" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X228" s="12">
+        <v>0.4</v>
+      </c>
+      <c r="Y228" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB228" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG228" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI228" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ228" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK228" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM228" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR228" s="3" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="229" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A229" s="1">
+        <v>1</v>
+      </c>
+      <c r="B229" s="2">
+        <v>2</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D229" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E229" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F229" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G229" s="5">
+        <v>82</v>
+      </c>
+      <c r="H229" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I229" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J229" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K229" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L229" s="6">
+        <v>509</v>
+      </c>
+      <c r="M229" s="7">
+        <v>204322.34</v>
+      </c>
+      <c r="N229" s="6">
+        <v>1</v>
+      </c>
+      <c r="O229" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P229" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q229" s="6">
+        <v>0</v>
+      </c>
+      <c r="R229" s="7">
+        <v>0</v>
+      </c>
+      <c r="S229" s="9">
+        <v>0</v>
+      </c>
+      <c r="T229" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U229" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V229" s="11">
+        <v>11</v>
+      </c>
+      <c r="W229" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X229" s="12">
+        <v>0.4</v>
+      </c>
+      <c r="Y229" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB229" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG229" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI229" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ229" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK229" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM229" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR229" s="3" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="230" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A230" s="1">
+        <v>1</v>
+      </c>
+      <c r="B230" s="2">
+        <v>2</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E230" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F230" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G230" s="5">
+        <v>83</v>
+      </c>
+      <c r="H230" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I230" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J230" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K230" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L230" s="6">
+        <v>510</v>
+      </c>
+      <c r="M230" s="7">
+        <v>204723.76</v>
+      </c>
+      <c r="N230" s="6">
+        <v>1</v>
+      </c>
+      <c r="O230" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P230" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q230" s="6">
+        <v>0</v>
+      </c>
+      <c r="R230" s="7">
+        <v>0</v>
+      </c>
+      <c r="S230" s="9">
+        <v>0</v>
+      </c>
+      <c r="T230" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U230" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V230" s="11">
+        <v>11</v>
+      </c>
+      <c r="W230" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X230" s="12">
+        <v>0.4</v>
+      </c>
+      <c r="Y230" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB230" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG230" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI230" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ230" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK230" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM230" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR230" s="3" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="231" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A231" s="1">
+        <v>1</v>
+      </c>
+      <c r="B231" s="2">
+        <v>2</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E231" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F231" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G231" s="5">
+        <v>84</v>
+      </c>
+      <c r="H231" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I231" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J231" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K231" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L231" s="6">
+        <v>511</v>
+      </c>
+      <c r="M231" s="7">
+        <v>205125.18</v>
+      </c>
+      <c r="N231" s="6">
+        <v>1</v>
+      </c>
+      <c r="O231" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P231" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q231" s="6">
+        <v>0</v>
+      </c>
+      <c r="R231" s="7">
+        <v>0</v>
+      </c>
+      <c r="S231" s="9">
+        <v>0</v>
+      </c>
+      <c r="T231" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U231" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V231" s="11">
+        <v>11</v>
+      </c>
+      <c r="W231" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X231" s="12">
+        <v>0.4</v>
+      </c>
+      <c r="Y231" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB231" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG231" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI231" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ231" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK231" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM231" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR231" s="3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="232" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A232" s="1">
+        <v>1</v>
+      </c>
+      <c r="B232" s="2">
+        <v>2</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E232" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F232" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G232" s="5">
+        <v>85</v>
+      </c>
+      <c r="H232" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I232" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J232" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K232" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L232" s="6">
+        <v>512</v>
+      </c>
+      <c r="M232" s="7">
+        <v>205526.6</v>
+      </c>
+      <c r="N232" s="6">
+        <v>1</v>
+      </c>
+      <c r="O232" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P232" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q232" s="6">
+        <v>0</v>
+      </c>
+      <c r="R232" s="7">
+        <v>0</v>
+      </c>
+      <c r="S232" s="9">
+        <v>0</v>
+      </c>
+      <c r="T232" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U232" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V232" s="11">
+        <v>11</v>
+      </c>
+      <c r="W232" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X232" s="12">
+        <v>0.42083330000000002</v>
+      </c>
+      <c r="Y232" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z232" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA232" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB232" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC232" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD232" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE232" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF232" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG232" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH232" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI232" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ232" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK232" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL232" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM232" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN232" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO232" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP232" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ232" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR232" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="233" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A233" s="1">
+        <v>1</v>
+      </c>
+      <c r="B233" s="2">
+        <v>2</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D233" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E233" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F233" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G233" s="5">
+        <v>86</v>
+      </c>
+      <c r="H233" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I233" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J233" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K233" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L233" s="6">
+        <v>513</v>
+      </c>
+      <c r="M233" s="7">
+        <v>205928.02</v>
+      </c>
+      <c r="N233" s="6">
+        <v>1</v>
+      </c>
+      <c r="O233" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P233" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q233" s="6">
+        <v>0</v>
+      </c>
+      <c r="R233" s="7">
+        <v>0</v>
+      </c>
+      <c r="S233" s="9">
+        <v>0</v>
+      </c>
+      <c r="T233" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U233" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V233" s="11">
+        <v>11</v>
+      </c>
+      <c r="W233" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X233" s="12">
+        <v>0.42083330000000002</v>
+      </c>
+      <c r="Y233" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB233" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG233" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI233" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ233" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK233" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM233" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR233" s="3" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="234" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A234" s="1">
+        <v>1</v>
+      </c>
+      <c r="B234" s="2">
+        <v>2</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E234" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F234" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G234" s="5">
+        <v>87</v>
+      </c>
+      <c r="H234" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I234" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J234" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K234" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L234" s="6">
+        <v>514</v>
+      </c>
+      <c r="M234" s="7">
+        <v>206329.44</v>
+      </c>
+      <c r="N234" s="6">
+        <v>1</v>
+      </c>
+      <c r="O234" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P234" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q234" s="6">
+        <v>0</v>
+      </c>
+      <c r="R234" s="7">
+        <v>0</v>
+      </c>
+      <c r="S234" s="9">
+        <v>0</v>
+      </c>
+      <c r="T234" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U234" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V234" s="11">
+        <v>11</v>
+      </c>
+      <c r="W234" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X234" s="12">
+        <v>0.42083330000000002</v>
+      </c>
+      <c r="Y234" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z234" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA234" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB234" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC234" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD234" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE234" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF234" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG234" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH234" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI234" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ234" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK234" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL234" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM234" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN234" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO234" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP234" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ234" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR234" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="235" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A235" s="1">
+        <v>1</v>
+      </c>
+      <c r="B235" s="2">
+        <v>2</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D235" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E235" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F235" s="4">
+        <v>46135</v>
+      </c>
+      <c r="G235" s="5">
+        <v>88</v>
+      </c>
+      <c r="H235" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I235" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J235" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K235" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L235" s="6">
+        <v>515</v>
+      </c>
+      <c r="M235" s="7">
+        <v>206730.86</v>
+      </c>
+      <c r="N235" s="6">
+        <v>1</v>
+      </c>
+      <c r="O235" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="P235" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q235" s="6">
+        <v>0</v>
+      </c>
+      <c r="R235" s="7">
+        <v>0</v>
+      </c>
+      <c r="S235" s="9">
+        <v>0</v>
+      </c>
+      <c r="T235" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U235" s="10">
+        <v>63954</v>
+      </c>
+      <c r="V235" s="11">
+        <v>11</v>
+      </c>
+      <c r="W235" s="4">
+        <v>46135</v>
+      </c>
+      <c r="X235" s="12">
+        <v>0.42083330000000002</v>
+      </c>
+      <c r="Y235" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z235" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA235" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB235" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC235" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD235" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE235" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG235" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI235" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ235" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK235" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL235" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM235" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR235" s="3" t="s">
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 27/04/2026 11:31:09,81
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3A24AE0-0067-4E51-B1EA-6E24A7AEA9EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E135DCE-24EE-4E57-AC75-0780FC6AE9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2472" yWindow="792" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3482" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3680" uniqueCount="260">
   <si>
     <t>Sel</t>
   </si>
@@ -768,6 +768,39 @@
   <si>
     <t>1871600008650</t>
   </si>
+  <si>
+    <t>1871600008651</t>
+  </si>
+  <si>
+    <t>1871600008652</t>
+  </si>
+  <si>
+    <t>1871600008653</t>
+  </si>
+  <si>
+    <t>1871600008654</t>
+  </si>
+  <si>
+    <t>1871600008655</t>
+  </si>
+  <si>
+    <t>1871600008656</t>
+  </si>
+  <si>
+    <t>1871600008657</t>
+  </si>
+  <si>
+    <t>1871600008658</t>
+  </si>
+  <si>
+    <t>1871600008659</t>
+  </si>
+  <si>
+    <t>1871600008660</t>
+  </si>
+  <si>
+    <t>1871600008661</t>
+  </si>
 </sst>
 </file>
 
@@ -1342,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR192"/>
+  <dimension ref="A1:AR203"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -27071,6 +27104,1480 @@
       </c>
       <c r="AR192" s="3" t="s">
         <v>248</v>
+      </c>
+    </row>
+    <row r="193" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A193" s="1">
+        <v>1</v>
+      </c>
+      <c r="B193" s="2">
+        <v>2</v>
+      </c>
+      <c r="C193" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E193" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F193" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G193" s="5">
+        <v>59</v>
+      </c>
+      <c r="H193" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I193" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J193" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K193" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L193" s="6">
+        <v>549</v>
+      </c>
+      <c r="M193" s="7">
+        <v>220379.11</v>
+      </c>
+      <c r="N193" s="6">
+        <v>1</v>
+      </c>
+      <c r="O193" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P193" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q193" s="6">
+        <v>0</v>
+      </c>
+      <c r="R193" s="7">
+        <v>0</v>
+      </c>
+      <c r="S193" s="9">
+        <v>0</v>
+      </c>
+      <c r="T193" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U193" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V193" s="11">
+        <v>11</v>
+      </c>
+      <c r="W193" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X193" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y193" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z193" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA193" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB193" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC193" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD193" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE193" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF193" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG193" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH193" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI193" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ193" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK193" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL193" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM193" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN193" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO193" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP193" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ193" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR193" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="194" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A194" s="1">
+        <v>1</v>
+      </c>
+      <c r="B194" s="2">
+        <v>2</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E194" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F194" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G194" s="5">
+        <v>60</v>
+      </c>
+      <c r="H194" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I194" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J194" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K194" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L194" s="6">
+        <v>550</v>
+      </c>
+      <c r="M194" s="7">
+        <v>220780.53</v>
+      </c>
+      <c r="N194" s="6">
+        <v>1</v>
+      </c>
+      <c r="O194" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P194" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q194" s="6">
+        <v>0</v>
+      </c>
+      <c r="R194" s="7">
+        <v>0</v>
+      </c>
+      <c r="S194" s="9">
+        <v>0</v>
+      </c>
+      <c r="T194" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U194" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V194" s="11">
+        <v>11</v>
+      </c>
+      <c r="W194" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X194" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y194" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z194" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA194" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB194" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC194" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD194" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE194" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG194" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI194" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ194" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK194" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL194" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM194" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR194" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="195" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A195" s="1">
+        <v>1</v>
+      </c>
+      <c r="B195" s="2">
+        <v>2</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D195" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E195" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F195" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G195" s="5">
+        <v>61</v>
+      </c>
+      <c r="H195" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I195" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J195" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K195" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L195" s="6">
+        <v>551</v>
+      </c>
+      <c r="M195" s="7">
+        <v>221181.95</v>
+      </c>
+      <c r="N195" s="6">
+        <v>1</v>
+      </c>
+      <c r="O195" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P195" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q195" s="6">
+        <v>0</v>
+      </c>
+      <c r="R195" s="7">
+        <v>0</v>
+      </c>
+      <c r="S195" s="9">
+        <v>0</v>
+      </c>
+      <c r="T195" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U195" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V195" s="11">
+        <v>11</v>
+      </c>
+      <c r="W195" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X195" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y195" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z195" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA195" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB195" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC195" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD195" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE195" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF195" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG195" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH195" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI195" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ195" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK195" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL195" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM195" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN195" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO195" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP195" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ195" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR195" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="196" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A196" s="1">
+        <v>1</v>
+      </c>
+      <c r="B196" s="2">
+        <v>2</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E196" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F196" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G196" s="5">
+        <v>62</v>
+      </c>
+      <c r="H196" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I196" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J196" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K196" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L196" s="6">
+        <v>552</v>
+      </c>
+      <c r="M196" s="7">
+        <v>221583.37</v>
+      </c>
+      <c r="N196" s="6">
+        <v>1</v>
+      </c>
+      <c r="O196" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P196" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q196" s="6">
+        <v>0</v>
+      </c>
+      <c r="R196" s="7">
+        <v>0</v>
+      </c>
+      <c r="S196" s="9">
+        <v>0</v>
+      </c>
+      <c r="T196" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U196" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V196" s="11">
+        <v>11</v>
+      </c>
+      <c r="W196" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X196" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y196" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z196" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA196" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB196" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC196" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD196" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE196" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG196" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI196" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ196" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK196" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL196" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM196" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR196" s="3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="197" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A197" s="1">
+        <v>1</v>
+      </c>
+      <c r="B197" s="2">
+        <v>2</v>
+      </c>
+      <c r="C197" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D197" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E197" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F197" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G197" s="5">
+        <v>63</v>
+      </c>
+      <c r="H197" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I197" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J197" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K197" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L197" s="6">
+        <v>553</v>
+      </c>
+      <c r="M197" s="7">
+        <v>221984.79</v>
+      </c>
+      <c r="N197" s="6">
+        <v>1</v>
+      </c>
+      <c r="O197" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P197" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q197" s="6">
+        <v>0</v>
+      </c>
+      <c r="R197" s="7">
+        <v>0</v>
+      </c>
+      <c r="S197" s="9">
+        <v>0</v>
+      </c>
+      <c r="T197" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U197" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V197" s="11">
+        <v>11</v>
+      </c>
+      <c r="W197" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X197" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y197" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB197" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG197" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI197" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ197" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK197" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM197" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR197" s="3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="198" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A198" s="1">
+        <v>1</v>
+      </c>
+      <c r="B198" s="2">
+        <v>2</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E198" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F198" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G198" s="5">
+        <v>64</v>
+      </c>
+      <c r="H198" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I198" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J198" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K198" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L198" s="6">
+        <v>554</v>
+      </c>
+      <c r="M198" s="7">
+        <v>222386.21</v>
+      </c>
+      <c r="N198" s="6">
+        <v>1</v>
+      </c>
+      <c r="O198" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P198" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q198" s="6">
+        <v>0</v>
+      </c>
+      <c r="R198" s="7">
+        <v>0</v>
+      </c>
+      <c r="S198" s="9">
+        <v>0</v>
+      </c>
+      <c r="T198" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U198" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V198" s="11">
+        <v>11</v>
+      </c>
+      <c r="W198" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X198" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y198" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB198" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG198" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI198" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ198" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK198" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM198" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR198" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="199" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A199" s="1">
+        <v>1</v>
+      </c>
+      <c r="B199" s="2">
+        <v>2</v>
+      </c>
+      <c r="C199" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E199" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F199" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G199" s="5">
+        <v>65</v>
+      </c>
+      <c r="H199" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I199" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J199" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K199" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L199" s="6">
+        <v>555</v>
+      </c>
+      <c r="M199" s="7">
+        <v>222787.63</v>
+      </c>
+      <c r="N199" s="6">
+        <v>1</v>
+      </c>
+      <c r="O199" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P199" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q199" s="6">
+        <v>0</v>
+      </c>
+      <c r="R199" s="7">
+        <v>0</v>
+      </c>
+      <c r="S199" s="9">
+        <v>0</v>
+      </c>
+      <c r="T199" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U199" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V199" s="11">
+        <v>11</v>
+      </c>
+      <c r="W199" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X199" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y199" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB199" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG199" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI199" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ199" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK199" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM199" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR199" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="200" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A200" s="1">
+        <v>1</v>
+      </c>
+      <c r="B200" s="2">
+        <v>2</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E200" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F200" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G200" s="5">
+        <v>66</v>
+      </c>
+      <c r="H200" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I200" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J200" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K200" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L200" s="6">
+        <v>556</v>
+      </c>
+      <c r="M200" s="7">
+        <v>223189.04</v>
+      </c>
+      <c r="N200" s="6">
+        <v>1</v>
+      </c>
+      <c r="O200" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P200" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q200" s="6">
+        <v>0</v>
+      </c>
+      <c r="R200" s="7">
+        <v>0</v>
+      </c>
+      <c r="S200" s="9">
+        <v>0</v>
+      </c>
+      <c r="T200" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U200" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V200" s="11">
+        <v>11</v>
+      </c>
+      <c r="W200" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X200" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y200" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB200" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG200" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI200" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ200" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK200" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM200" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR200" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="201" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A201" s="1">
+        <v>1</v>
+      </c>
+      <c r="B201" s="2">
+        <v>2</v>
+      </c>
+      <c r="C201" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D201" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E201" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F201" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G201" s="5">
+        <v>67</v>
+      </c>
+      <c r="H201" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I201" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J201" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K201" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L201" s="6">
+        <v>557</v>
+      </c>
+      <c r="M201" s="7">
+        <v>223590.46</v>
+      </c>
+      <c r="N201" s="6">
+        <v>1</v>
+      </c>
+      <c r="O201" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P201" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q201" s="6">
+        <v>0</v>
+      </c>
+      <c r="R201" s="7">
+        <v>0</v>
+      </c>
+      <c r="S201" s="9">
+        <v>0</v>
+      </c>
+      <c r="T201" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U201" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V201" s="11">
+        <v>11</v>
+      </c>
+      <c r="W201" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X201" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y201" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB201" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG201" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI201" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ201" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK201" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM201" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR201" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="202" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A202" s="1">
+        <v>1</v>
+      </c>
+      <c r="B202" s="2">
+        <v>2</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E202" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F202" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G202" s="5">
+        <v>68</v>
+      </c>
+      <c r="H202" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I202" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J202" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K202" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L202" s="6">
+        <v>558</v>
+      </c>
+      <c r="M202" s="7">
+        <v>223991.88</v>
+      </c>
+      <c r="N202" s="6">
+        <v>1</v>
+      </c>
+      <c r="O202" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P202" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q202" s="6">
+        <v>0</v>
+      </c>
+      <c r="R202" s="7">
+        <v>0</v>
+      </c>
+      <c r="S202" s="9">
+        <v>0</v>
+      </c>
+      <c r="T202" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U202" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V202" s="11">
+        <v>11</v>
+      </c>
+      <c r="W202" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X202" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y202" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB202" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG202" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI202" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ202" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK202" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM202" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR202" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="203" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A203" s="1">
+        <v>1</v>
+      </c>
+      <c r="B203" s="2">
+        <v>2</v>
+      </c>
+      <c r="C203" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D203" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E203" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F203" s="4">
+        <v>46139</v>
+      </c>
+      <c r="G203" s="5">
+        <v>69</v>
+      </c>
+      <c r="H203" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I203" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J203" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K203" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L203" s="6">
+        <v>559</v>
+      </c>
+      <c r="M203" s="7">
+        <v>224393.3</v>
+      </c>
+      <c r="N203" s="6">
+        <v>1</v>
+      </c>
+      <c r="O203" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="P203" s="8">
+        <v>401.42</v>
+      </c>
+      <c r="Q203" s="6">
+        <v>0</v>
+      </c>
+      <c r="R203" s="7">
+        <v>0</v>
+      </c>
+      <c r="S203" s="9">
+        <v>0</v>
+      </c>
+      <c r="T203" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U203" s="10">
+        <v>64027</v>
+      </c>
+      <c r="V203" s="11">
+        <v>11</v>
+      </c>
+      <c r="W203" s="4">
+        <v>46139</v>
+      </c>
+      <c r="X203" s="12">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="Y203" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB203" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG203" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI203" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ203" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK203" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM203" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR203" s="3" t="s">
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 04/05/2026 10:44:00,40
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{143FB344-0A84-4CA9-8965-CD5A044F20EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0766802B-C1D3-419F-B3AF-313372BA3650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2384" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2708" uniqueCount="203">
   <si>
     <t>Sel</t>
   </si>
@@ -575,6 +575,60 @@
   </si>
   <si>
     <t>1858700135513</t>
+  </si>
+  <si>
+    <t>1858700135514</t>
+  </si>
+  <si>
+    <t>1858700135515</t>
+  </si>
+  <si>
+    <t>1858700135516</t>
+  </si>
+  <si>
+    <t>1858700135517</t>
+  </si>
+  <si>
+    <t>1858700135518</t>
+  </si>
+  <si>
+    <t>1858700135519</t>
+  </si>
+  <si>
+    <t>1858700135520</t>
+  </si>
+  <si>
+    <t>1858700135521</t>
+  </si>
+  <si>
+    <t>1858700135522</t>
+  </si>
+  <si>
+    <t>1858700135523</t>
+  </si>
+  <si>
+    <t>1858700135524</t>
+  </si>
+  <si>
+    <t>1858700135525</t>
+  </si>
+  <si>
+    <t>1858700135526</t>
+  </si>
+  <si>
+    <t>1858700135527</t>
+  </si>
+  <si>
+    <t>1858700135528</t>
+  </si>
+  <si>
+    <t>1858700135529</t>
+  </si>
+  <si>
+    <t>1858700135530</t>
+  </si>
+  <si>
+    <t>1858700135531</t>
   </si>
 </sst>
 </file>
@@ -1150,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR131"/>
+  <dimension ref="A1:AR149"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -18705,6 +18759,2418 @@
       </c>
       <c r="AR131" s="3" t="s">
         <v>184</v>
+      </c>
+    </row>
+    <row r="132" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A132" s="1">
+        <v>1</v>
+      </c>
+      <c r="B132" s="2">
+        <v>2</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F132" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G132" s="5">
+        <v>132</v>
+      </c>
+      <c r="H132" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I132" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J132" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K132" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L132" s="6">
+        <v>674</v>
+      </c>
+      <c r="M132" s="7">
+        <v>126051.89</v>
+      </c>
+      <c r="N132" s="6">
+        <v>1</v>
+      </c>
+      <c r="O132" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P132" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q132" s="6">
+        <v>0</v>
+      </c>
+      <c r="R132" s="7">
+        <v>0</v>
+      </c>
+      <c r="S132" s="9">
+        <v>0</v>
+      </c>
+      <c r="T132" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U132" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V132" s="11">
+        <v>11</v>
+      </c>
+      <c r="W132" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X132" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y132" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB132" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG132" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI132" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ132" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK132" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM132" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR132" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="133" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A133" s="1">
+        <v>1</v>
+      </c>
+      <c r="B133" s="2">
+        <v>2</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F133" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G133" s="5">
+        <v>133</v>
+      </c>
+      <c r="H133" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I133" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J133" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K133" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L133" s="6">
+        <v>675</v>
+      </c>
+      <c r="M133" s="7">
+        <v>126238.91</v>
+      </c>
+      <c r="N133" s="6">
+        <v>1</v>
+      </c>
+      <c r="O133" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P133" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q133" s="6">
+        <v>0</v>
+      </c>
+      <c r="R133" s="7">
+        <v>0</v>
+      </c>
+      <c r="S133" s="9">
+        <v>0</v>
+      </c>
+      <c r="T133" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U133" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V133" s="11">
+        <v>11</v>
+      </c>
+      <c r="W133" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X133" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y133" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB133" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG133" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI133" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ133" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK133" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM133" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR133" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="134" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A134" s="1">
+        <v>1</v>
+      </c>
+      <c r="B134" s="2">
+        <v>2</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F134" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G134" s="5">
+        <v>134</v>
+      </c>
+      <c r="H134" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I134" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J134" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K134" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L134" s="6">
+        <v>676</v>
+      </c>
+      <c r="M134" s="7">
+        <v>126425.93</v>
+      </c>
+      <c r="N134" s="6">
+        <v>1</v>
+      </c>
+      <c r="O134" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P134" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q134" s="6">
+        <v>0</v>
+      </c>
+      <c r="R134" s="7">
+        <v>0</v>
+      </c>
+      <c r="S134" s="9">
+        <v>0</v>
+      </c>
+      <c r="T134" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U134" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V134" s="11">
+        <v>11</v>
+      </c>
+      <c r="W134" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X134" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y134" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB134" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG134" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI134" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ134" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK134" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM134" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR134" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="135" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A135" s="1">
+        <v>1</v>
+      </c>
+      <c r="B135" s="2">
+        <v>2</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E135" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F135" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G135" s="5">
+        <v>135</v>
+      </c>
+      <c r="H135" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I135" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J135" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K135" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L135" s="6">
+        <v>677</v>
+      </c>
+      <c r="M135" s="7">
+        <v>126612.95</v>
+      </c>
+      <c r="N135" s="6">
+        <v>1</v>
+      </c>
+      <c r="O135" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P135" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q135" s="6">
+        <v>0</v>
+      </c>
+      <c r="R135" s="7">
+        <v>0</v>
+      </c>
+      <c r="S135" s="9">
+        <v>0</v>
+      </c>
+      <c r="T135" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U135" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V135" s="11">
+        <v>11</v>
+      </c>
+      <c r="W135" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X135" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y135" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB135" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG135" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI135" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ135" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK135" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM135" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR135" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="136" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A136" s="1">
+        <v>1</v>
+      </c>
+      <c r="B136" s="2">
+        <v>2</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F136" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G136" s="5">
+        <v>136</v>
+      </c>
+      <c r="H136" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I136" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J136" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K136" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L136" s="6">
+        <v>678</v>
+      </c>
+      <c r="M136" s="7">
+        <v>126799.97</v>
+      </c>
+      <c r="N136" s="6">
+        <v>1</v>
+      </c>
+      <c r="O136" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P136" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q136" s="6">
+        <v>0</v>
+      </c>
+      <c r="R136" s="7">
+        <v>0</v>
+      </c>
+      <c r="S136" s="9">
+        <v>0</v>
+      </c>
+      <c r="T136" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U136" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V136" s="11">
+        <v>11</v>
+      </c>
+      <c r="W136" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X136" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y136" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB136" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG136" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI136" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ136" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK136" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM136" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR136" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="137" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A137" s="1">
+        <v>1</v>
+      </c>
+      <c r="B137" s="2">
+        <v>2</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F137" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G137" s="5">
+        <v>137</v>
+      </c>
+      <c r="H137" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I137" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J137" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K137" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L137" s="6">
+        <v>679</v>
+      </c>
+      <c r="M137" s="7">
+        <v>126986.99</v>
+      </c>
+      <c r="N137" s="6">
+        <v>1</v>
+      </c>
+      <c r="O137" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P137" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q137" s="6">
+        <v>0</v>
+      </c>
+      <c r="R137" s="7">
+        <v>0</v>
+      </c>
+      <c r="S137" s="9">
+        <v>0</v>
+      </c>
+      <c r="T137" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U137" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V137" s="11">
+        <v>11</v>
+      </c>
+      <c r="W137" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X137" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y137" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB137" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG137" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI137" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ137" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK137" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM137" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR137" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="138" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A138" s="1">
+        <v>1</v>
+      </c>
+      <c r="B138" s="2">
+        <v>2</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F138" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G138" s="5">
+        <v>138</v>
+      </c>
+      <c r="H138" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I138" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J138" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K138" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L138" s="6">
+        <v>680</v>
+      </c>
+      <c r="M138" s="7">
+        <v>127174.01</v>
+      </c>
+      <c r="N138" s="6">
+        <v>1</v>
+      </c>
+      <c r="O138" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P138" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q138" s="6">
+        <v>0</v>
+      </c>
+      <c r="R138" s="7">
+        <v>0</v>
+      </c>
+      <c r="S138" s="9">
+        <v>0</v>
+      </c>
+      <c r="T138" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U138" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V138" s="11">
+        <v>11</v>
+      </c>
+      <c r="W138" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X138" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y138" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB138" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG138" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI138" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ138" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK138" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM138" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR138" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="139" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A139" s="1">
+        <v>1</v>
+      </c>
+      <c r="B139" s="2">
+        <v>2</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E139" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F139" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G139" s="5">
+        <v>139</v>
+      </c>
+      <c r="H139" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I139" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J139" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K139" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L139" s="6">
+        <v>681</v>
+      </c>
+      <c r="M139" s="7">
+        <v>127361.03</v>
+      </c>
+      <c r="N139" s="6">
+        <v>1</v>
+      </c>
+      <c r="O139" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P139" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q139" s="6">
+        <v>0</v>
+      </c>
+      <c r="R139" s="7">
+        <v>0</v>
+      </c>
+      <c r="S139" s="9">
+        <v>0</v>
+      </c>
+      <c r="T139" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U139" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V139" s="11">
+        <v>11</v>
+      </c>
+      <c r="W139" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X139" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y139" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB139" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG139" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI139" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ139" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK139" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM139" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR139" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="140" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A140" s="1">
+        <v>1</v>
+      </c>
+      <c r="B140" s="2">
+        <v>2</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F140" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G140" s="5">
+        <v>140</v>
+      </c>
+      <c r="H140" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I140" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J140" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K140" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L140" s="6">
+        <v>682</v>
+      </c>
+      <c r="M140" s="7">
+        <v>127548.05</v>
+      </c>
+      <c r="N140" s="6">
+        <v>1</v>
+      </c>
+      <c r="O140" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P140" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q140" s="6">
+        <v>0</v>
+      </c>
+      <c r="R140" s="7">
+        <v>0</v>
+      </c>
+      <c r="S140" s="9">
+        <v>0</v>
+      </c>
+      <c r="T140" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U140" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V140" s="11">
+        <v>11</v>
+      </c>
+      <c r="W140" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X140" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y140" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB140" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG140" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI140" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ140" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK140" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM140" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR140" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="141" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A141" s="1">
+        <v>1</v>
+      </c>
+      <c r="B141" s="2">
+        <v>2</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E141" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F141" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G141" s="5">
+        <v>141</v>
+      </c>
+      <c r="H141" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I141" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J141" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K141" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L141" s="6">
+        <v>683</v>
+      </c>
+      <c r="M141" s="7">
+        <v>127735.07</v>
+      </c>
+      <c r="N141" s="6">
+        <v>1</v>
+      </c>
+      <c r="O141" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P141" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q141" s="6">
+        <v>0</v>
+      </c>
+      <c r="R141" s="7">
+        <v>0</v>
+      </c>
+      <c r="S141" s="9">
+        <v>0</v>
+      </c>
+      <c r="T141" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U141" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V141" s="11">
+        <v>11</v>
+      </c>
+      <c r="W141" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X141" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y141" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB141" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG141" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI141" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ141" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK141" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM141" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR141" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="142" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A142" s="1">
+        <v>1</v>
+      </c>
+      <c r="B142" s="2">
+        <v>2</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F142" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G142" s="5">
+        <v>142</v>
+      </c>
+      <c r="H142" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I142" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J142" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K142" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L142" s="6">
+        <v>684</v>
+      </c>
+      <c r="M142" s="7">
+        <v>127922.09</v>
+      </c>
+      <c r="N142" s="6">
+        <v>1</v>
+      </c>
+      <c r="O142" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P142" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q142" s="6">
+        <v>0</v>
+      </c>
+      <c r="R142" s="7">
+        <v>0</v>
+      </c>
+      <c r="S142" s="9">
+        <v>0</v>
+      </c>
+      <c r="T142" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U142" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V142" s="11">
+        <v>11</v>
+      </c>
+      <c r="W142" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X142" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y142" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB142" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG142" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI142" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ142" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK142" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM142" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR142" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="143" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A143" s="1">
+        <v>1</v>
+      </c>
+      <c r="B143" s="2">
+        <v>2</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E143" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F143" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G143" s="5">
+        <v>143</v>
+      </c>
+      <c r="H143" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I143" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J143" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K143" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L143" s="6">
+        <v>685</v>
+      </c>
+      <c r="M143" s="7">
+        <v>128109.11</v>
+      </c>
+      <c r="N143" s="6">
+        <v>1</v>
+      </c>
+      <c r="O143" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P143" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q143" s="6">
+        <v>0</v>
+      </c>
+      <c r="R143" s="7">
+        <v>0</v>
+      </c>
+      <c r="S143" s="9">
+        <v>0</v>
+      </c>
+      <c r="T143" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U143" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V143" s="11">
+        <v>11</v>
+      </c>
+      <c r="W143" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X143" s="12">
+        <v>0.44166670000000002</v>
+      </c>
+      <c r="Y143" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z143" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA143" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB143" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC143" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD143" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE143" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF143" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG143" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH143" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI143" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ143" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK143" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL143" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM143" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN143" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO143" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP143" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ143" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR143" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="144" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A144" s="1">
+        <v>1</v>
+      </c>
+      <c r="B144" s="2">
+        <v>2</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F144" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G144" s="5">
+        <v>144</v>
+      </c>
+      <c r="H144" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I144" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J144" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K144" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L144" s="6">
+        <v>686</v>
+      </c>
+      <c r="M144" s="7">
+        <v>128296.13</v>
+      </c>
+      <c r="N144" s="6">
+        <v>1</v>
+      </c>
+      <c r="O144" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P144" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q144" s="6">
+        <v>0</v>
+      </c>
+      <c r="R144" s="7">
+        <v>0</v>
+      </c>
+      <c r="S144" s="9">
+        <v>0</v>
+      </c>
+      <c r="T144" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U144" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V144" s="11">
+        <v>11</v>
+      </c>
+      <c r="W144" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X144" s="12">
+        <v>0.44236110000000001</v>
+      </c>
+      <c r="Y144" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z144" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA144" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB144" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC144" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD144" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE144" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG144" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI144" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ144" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK144" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL144" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM144" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR144" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="145" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A145" s="1">
+        <v>1</v>
+      </c>
+      <c r="B145" s="2">
+        <v>2</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E145" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F145" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G145" s="5">
+        <v>145</v>
+      </c>
+      <c r="H145" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I145" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J145" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K145" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L145" s="6">
+        <v>687</v>
+      </c>
+      <c r="M145" s="7">
+        <v>128483.15</v>
+      </c>
+      <c r="N145" s="6">
+        <v>1</v>
+      </c>
+      <c r="O145" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P145" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q145" s="6">
+        <v>0</v>
+      </c>
+      <c r="R145" s="7">
+        <v>0</v>
+      </c>
+      <c r="S145" s="9">
+        <v>0</v>
+      </c>
+      <c r="T145" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U145" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V145" s="11">
+        <v>11</v>
+      </c>
+      <c r="W145" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X145" s="12">
+        <v>0.44236110000000001</v>
+      </c>
+      <c r="Y145" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z145" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA145" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB145" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC145" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD145" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE145" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG145" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI145" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ145" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK145" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL145" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM145" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR145" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="146" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A146" s="1">
+        <v>1</v>
+      </c>
+      <c r="B146" s="2">
+        <v>2</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F146" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G146" s="5">
+        <v>146</v>
+      </c>
+      <c r="H146" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I146" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J146" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K146" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L146" s="6">
+        <v>688</v>
+      </c>
+      <c r="M146" s="7">
+        <v>128670.17</v>
+      </c>
+      <c r="N146" s="6">
+        <v>1</v>
+      </c>
+      <c r="O146" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P146" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q146" s="6">
+        <v>0</v>
+      </c>
+      <c r="R146" s="7">
+        <v>0</v>
+      </c>
+      <c r="S146" s="9">
+        <v>0</v>
+      </c>
+      <c r="T146" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U146" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V146" s="11">
+        <v>11</v>
+      </c>
+      <c r="W146" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X146" s="12">
+        <v>0.44236110000000001</v>
+      </c>
+      <c r="Y146" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z146" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA146" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB146" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC146" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD146" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE146" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG146" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI146" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ146" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK146" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL146" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM146" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR146" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="147" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A147" s="1">
+        <v>1</v>
+      </c>
+      <c r="B147" s="2">
+        <v>2</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E147" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F147" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G147" s="5">
+        <v>147</v>
+      </c>
+      <c r="H147" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I147" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J147" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K147" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L147" s="6">
+        <v>689</v>
+      </c>
+      <c r="M147" s="7">
+        <v>128857.2</v>
+      </c>
+      <c r="N147" s="6">
+        <v>1</v>
+      </c>
+      <c r="O147" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P147" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q147" s="6">
+        <v>0</v>
+      </c>
+      <c r="R147" s="7">
+        <v>0</v>
+      </c>
+      <c r="S147" s="9">
+        <v>0</v>
+      </c>
+      <c r="T147" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U147" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V147" s="11">
+        <v>11</v>
+      </c>
+      <c r="W147" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X147" s="12">
+        <v>0.44236110000000001</v>
+      </c>
+      <c r="Y147" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z147" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA147" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB147" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC147" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD147" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE147" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG147" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI147" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ147" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK147" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL147" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM147" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR147" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="148" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A148" s="1">
+        <v>1</v>
+      </c>
+      <c r="B148" s="2">
+        <v>2</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F148" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G148" s="5">
+        <v>148</v>
+      </c>
+      <c r="H148" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I148" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J148" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K148" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L148" s="6">
+        <v>690</v>
+      </c>
+      <c r="M148" s="7">
+        <v>129044.22</v>
+      </c>
+      <c r="N148" s="6">
+        <v>1</v>
+      </c>
+      <c r="O148" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P148" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q148" s="6">
+        <v>0</v>
+      </c>
+      <c r="R148" s="7">
+        <v>0</v>
+      </c>
+      <c r="S148" s="9">
+        <v>0</v>
+      </c>
+      <c r="T148" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U148" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V148" s="11">
+        <v>11</v>
+      </c>
+      <c r="W148" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X148" s="12">
+        <v>0.44236110000000001</v>
+      </c>
+      <c r="Y148" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z148" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA148" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB148" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC148" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD148" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE148" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG148" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI148" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ148" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK148" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL148" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM148" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR148" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="149" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A149" s="1">
+        <v>1</v>
+      </c>
+      <c r="B149" s="2">
+        <v>2</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E149" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F149" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G149" s="5">
+        <v>149</v>
+      </c>
+      <c r="H149" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I149" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J149" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K149" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L149" s="6">
+        <v>691</v>
+      </c>
+      <c r="M149" s="7">
+        <v>129231.24</v>
+      </c>
+      <c r="N149" s="6">
+        <v>1</v>
+      </c>
+      <c r="O149" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P149" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q149" s="6">
+        <v>0</v>
+      </c>
+      <c r="R149" s="7">
+        <v>0</v>
+      </c>
+      <c r="S149" s="9">
+        <v>0</v>
+      </c>
+      <c r="T149" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U149" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V149" s="11">
+        <v>11</v>
+      </c>
+      <c r="W149" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X149" s="12">
+        <v>0.44236110000000001</v>
+      </c>
+      <c r="Y149" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z149" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA149" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB149" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC149" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD149" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE149" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF149" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG149" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH149" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI149" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ149" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK149" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL149" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM149" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN149" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO149" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP149" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ149" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR149" s="3" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 04/05/2026 12:19:55,23
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{274A4E76-4709-470D-87A0-52AAA06CAB71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9DED95E2-C241-4B88-AA9D-E3C64A6D9314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3788" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4184" uniqueCount="285">
   <si>
     <t>Sel</t>
   </si>
@@ -810,6 +810,72 @@
   <si>
     <t>1858700135591</t>
   </si>
+  <si>
+    <t>1858700135592</t>
+  </si>
+  <si>
+    <t>1858700135593</t>
+  </si>
+  <si>
+    <t>1858700135594</t>
+  </si>
+  <si>
+    <t>1858700135595</t>
+  </si>
+  <si>
+    <t>1858700135596</t>
+  </si>
+  <si>
+    <t>1858700135597</t>
+  </si>
+  <si>
+    <t>1858700135598</t>
+  </si>
+  <si>
+    <t>1858700135599</t>
+  </si>
+  <si>
+    <t>1858700135600</t>
+  </si>
+  <si>
+    <t>1858700135601</t>
+  </si>
+  <si>
+    <t>1858700135602</t>
+  </si>
+  <si>
+    <t>1858700135603</t>
+  </si>
+  <si>
+    <t>1858700135604</t>
+  </si>
+  <si>
+    <t>1858700135605</t>
+  </si>
+  <si>
+    <t>1858700135606</t>
+  </si>
+  <si>
+    <t>1858700135607</t>
+  </si>
+  <si>
+    <t>1858700135608</t>
+  </si>
+  <si>
+    <t>1858700135609</t>
+  </si>
+  <si>
+    <t>1858700135610</t>
+  </si>
+  <si>
+    <t>1858700135611</t>
+  </si>
+  <si>
+    <t>1858700135612</t>
+  </si>
+  <si>
+    <t>1858700135613</t>
+  </si>
 </sst>
 </file>
 
@@ -1384,7 +1450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR209"/>
+  <dimension ref="A1:AR231"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -29391,6 +29457,2954 @@
       </c>
       <c r="AR209" s="3" t="s">
         <v>262</v>
+      </c>
+    </row>
+    <row r="210" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A210" s="1">
+        <v>1</v>
+      </c>
+      <c r="B210" s="2">
+        <v>2</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D210" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E210" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F210" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G210" s="5">
+        <v>210</v>
+      </c>
+      <c r="H210" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I210" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J210" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K210" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L210" s="6">
+        <v>752</v>
+      </c>
+      <c r="M210" s="7">
+        <v>140639.49</v>
+      </c>
+      <c r="N210" s="6">
+        <v>1</v>
+      </c>
+      <c r="O210" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P210" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q210" s="6">
+        <v>0</v>
+      </c>
+      <c r="R210" s="7">
+        <v>0</v>
+      </c>
+      <c r="S210" s="9">
+        <v>0</v>
+      </c>
+      <c r="T210" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U210" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V210" s="11">
+        <v>11</v>
+      </c>
+      <c r="W210" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X210" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y210" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB210" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG210" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI210" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ210" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK210" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM210" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR210" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="211" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A211" s="1">
+        <v>1</v>
+      </c>
+      <c r="B211" s="2">
+        <v>2</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D211" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E211" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F211" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G211" s="5">
+        <v>211</v>
+      </c>
+      <c r="H211" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I211" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J211" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K211" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L211" s="6">
+        <v>753</v>
+      </c>
+      <c r="M211" s="7">
+        <v>140826.51</v>
+      </c>
+      <c r="N211" s="6">
+        <v>1</v>
+      </c>
+      <c r="O211" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P211" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q211" s="6">
+        <v>0</v>
+      </c>
+      <c r="R211" s="7">
+        <v>0</v>
+      </c>
+      <c r="S211" s="9">
+        <v>0</v>
+      </c>
+      <c r="T211" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U211" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V211" s="11">
+        <v>11</v>
+      </c>
+      <c r="W211" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X211" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y211" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB211" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG211" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI211" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ211" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK211" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM211" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR211" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="212" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A212" s="1">
+        <v>1</v>
+      </c>
+      <c r="B212" s="2">
+        <v>2</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E212" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F212" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G212" s="5">
+        <v>212</v>
+      </c>
+      <c r="H212" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I212" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J212" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K212" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L212" s="6">
+        <v>754</v>
+      </c>
+      <c r="M212" s="7">
+        <v>141013.53</v>
+      </c>
+      <c r="N212" s="6">
+        <v>1</v>
+      </c>
+      <c r="O212" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P212" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q212" s="6">
+        <v>0</v>
+      </c>
+      <c r="R212" s="7">
+        <v>0</v>
+      </c>
+      <c r="S212" s="9">
+        <v>0</v>
+      </c>
+      <c r="T212" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U212" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V212" s="11">
+        <v>11</v>
+      </c>
+      <c r="W212" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X212" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y212" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB212" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG212" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI212" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ212" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK212" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM212" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR212" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="213" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A213" s="1">
+        <v>1</v>
+      </c>
+      <c r="B213" s="2">
+        <v>2</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D213" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E213" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F213" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G213" s="5">
+        <v>213</v>
+      </c>
+      <c r="H213" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I213" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J213" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K213" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L213" s="6">
+        <v>755</v>
+      </c>
+      <c r="M213" s="7">
+        <v>141200.54999999999</v>
+      </c>
+      <c r="N213" s="6">
+        <v>1</v>
+      </c>
+      <c r="O213" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P213" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q213" s="6">
+        <v>0</v>
+      </c>
+      <c r="R213" s="7">
+        <v>0</v>
+      </c>
+      <c r="S213" s="9">
+        <v>0</v>
+      </c>
+      <c r="T213" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U213" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V213" s="11">
+        <v>11</v>
+      </c>
+      <c r="W213" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X213" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y213" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB213" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG213" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI213" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ213" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK213" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM213" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR213" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="214" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A214" s="1">
+        <v>1</v>
+      </c>
+      <c r="B214" s="2">
+        <v>2</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E214" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F214" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G214" s="5">
+        <v>214</v>
+      </c>
+      <c r="H214" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I214" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J214" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K214" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L214" s="6">
+        <v>756</v>
+      </c>
+      <c r="M214" s="7">
+        <v>141387.57999999999</v>
+      </c>
+      <c r="N214" s="6">
+        <v>1</v>
+      </c>
+      <c r="O214" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P214" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q214" s="6">
+        <v>0</v>
+      </c>
+      <c r="R214" s="7">
+        <v>0</v>
+      </c>
+      <c r="S214" s="9">
+        <v>0</v>
+      </c>
+      <c r="T214" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U214" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V214" s="11">
+        <v>11</v>
+      </c>
+      <c r="W214" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X214" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y214" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB214" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG214" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI214" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ214" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK214" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM214" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR214" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="215" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A215" s="1">
+        <v>1</v>
+      </c>
+      <c r="B215" s="2">
+        <v>2</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D215" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E215" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F215" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G215" s="5">
+        <v>215</v>
+      </c>
+      <c r="H215" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I215" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J215" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K215" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L215" s="6">
+        <v>757</v>
+      </c>
+      <c r="M215" s="7">
+        <v>141574.6</v>
+      </c>
+      <c r="N215" s="6">
+        <v>1</v>
+      </c>
+      <c r="O215" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P215" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q215" s="6">
+        <v>0</v>
+      </c>
+      <c r="R215" s="7">
+        <v>0</v>
+      </c>
+      <c r="S215" s="9">
+        <v>0</v>
+      </c>
+      <c r="T215" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U215" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V215" s="11">
+        <v>11</v>
+      </c>
+      <c r="W215" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X215" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y215" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB215" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG215" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI215" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ215" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK215" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM215" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR215" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="216" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A216" s="1">
+        <v>1</v>
+      </c>
+      <c r="B216" s="2">
+        <v>2</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E216" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F216" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G216" s="5">
+        <v>216</v>
+      </c>
+      <c r="H216" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I216" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J216" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K216" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L216" s="6">
+        <v>758</v>
+      </c>
+      <c r="M216" s="7">
+        <v>141761.62</v>
+      </c>
+      <c r="N216" s="6">
+        <v>1</v>
+      </c>
+      <c r="O216" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P216" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q216" s="6">
+        <v>0</v>
+      </c>
+      <c r="R216" s="7">
+        <v>0</v>
+      </c>
+      <c r="S216" s="9">
+        <v>0</v>
+      </c>
+      <c r="T216" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U216" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V216" s="11">
+        <v>11</v>
+      </c>
+      <c r="W216" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X216" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y216" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB216" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG216" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI216" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ216" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK216" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM216" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR216" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="217" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A217" s="1">
+        <v>1</v>
+      </c>
+      <c r="B217" s="2">
+        <v>2</v>
+      </c>
+      <c r="C217" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E217" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F217" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G217" s="5">
+        <v>217</v>
+      </c>
+      <c r="H217" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I217" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J217" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K217" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L217" s="6">
+        <v>759</v>
+      </c>
+      <c r="M217" s="7">
+        <v>141948.64000000001</v>
+      </c>
+      <c r="N217" s="6">
+        <v>1</v>
+      </c>
+      <c r="O217" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P217" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q217" s="6">
+        <v>0</v>
+      </c>
+      <c r="R217" s="7">
+        <v>0</v>
+      </c>
+      <c r="S217" s="9">
+        <v>0</v>
+      </c>
+      <c r="T217" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U217" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V217" s="11">
+        <v>11</v>
+      </c>
+      <c r="W217" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X217" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y217" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB217" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG217" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI217" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ217" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK217" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM217" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR217" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="218" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A218" s="1">
+        <v>1</v>
+      </c>
+      <c r="B218" s="2">
+        <v>2</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D218" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E218" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F218" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G218" s="5">
+        <v>218</v>
+      </c>
+      <c r="H218" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I218" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J218" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K218" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L218" s="6">
+        <v>760</v>
+      </c>
+      <c r="M218" s="7">
+        <v>142135.66</v>
+      </c>
+      <c r="N218" s="6">
+        <v>1</v>
+      </c>
+      <c r="O218" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P218" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q218" s="6">
+        <v>0</v>
+      </c>
+      <c r="R218" s="7">
+        <v>0</v>
+      </c>
+      <c r="S218" s="9">
+        <v>0</v>
+      </c>
+      <c r="T218" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U218" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V218" s="11">
+        <v>11</v>
+      </c>
+      <c r="W218" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X218" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y218" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB218" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG218" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI218" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ218" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK218" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM218" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR218" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="219" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A219" s="1">
+        <v>1</v>
+      </c>
+      <c r="B219" s="2">
+        <v>2</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D219" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E219" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F219" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G219" s="5">
+        <v>219</v>
+      </c>
+      <c r="H219" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I219" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J219" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K219" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L219" s="6">
+        <v>761</v>
+      </c>
+      <c r="M219" s="7">
+        <v>142322.68</v>
+      </c>
+      <c r="N219" s="6">
+        <v>1</v>
+      </c>
+      <c r="O219" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P219" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q219" s="6">
+        <v>0</v>
+      </c>
+      <c r="R219" s="7">
+        <v>0</v>
+      </c>
+      <c r="S219" s="9">
+        <v>0</v>
+      </c>
+      <c r="T219" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U219" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V219" s="11">
+        <v>11</v>
+      </c>
+      <c r="W219" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X219" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y219" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB219" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG219" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI219" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ219" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK219" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM219" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR219" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="220" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A220" s="1">
+        <v>1</v>
+      </c>
+      <c r="B220" s="2">
+        <v>2</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E220" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F220" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G220" s="5">
+        <v>220</v>
+      </c>
+      <c r="H220" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I220" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J220" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K220" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L220" s="6">
+        <v>762</v>
+      </c>
+      <c r="M220" s="7">
+        <v>142509.70000000001</v>
+      </c>
+      <c r="N220" s="6">
+        <v>1</v>
+      </c>
+      <c r="O220" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P220" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q220" s="6">
+        <v>0</v>
+      </c>
+      <c r="R220" s="7">
+        <v>0</v>
+      </c>
+      <c r="S220" s="9">
+        <v>0</v>
+      </c>
+      <c r="T220" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U220" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V220" s="11">
+        <v>11</v>
+      </c>
+      <c r="W220" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X220" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y220" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB220" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG220" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI220" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ220" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK220" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM220" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR220" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="221" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A221" s="1">
+        <v>1</v>
+      </c>
+      <c r="B221" s="2">
+        <v>2</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D221" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E221" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F221" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G221" s="5">
+        <v>221</v>
+      </c>
+      <c r="H221" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I221" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J221" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K221" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L221" s="6">
+        <v>763</v>
+      </c>
+      <c r="M221" s="7">
+        <v>142696.72</v>
+      </c>
+      <c r="N221" s="6">
+        <v>1</v>
+      </c>
+      <c r="O221" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P221" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q221" s="6">
+        <v>0</v>
+      </c>
+      <c r="R221" s="7">
+        <v>0</v>
+      </c>
+      <c r="S221" s="9">
+        <v>0</v>
+      </c>
+      <c r="T221" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U221" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V221" s="11">
+        <v>11</v>
+      </c>
+      <c r="W221" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X221" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y221" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB221" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG221" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI221" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ221" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK221" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM221" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR221" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="222" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A222" s="1">
+        <v>1</v>
+      </c>
+      <c r="B222" s="2">
+        <v>2</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E222" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F222" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G222" s="5">
+        <v>222</v>
+      </c>
+      <c r="H222" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I222" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J222" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K222" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L222" s="6">
+        <v>764</v>
+      </c>
+      <c r="M222" s="7">
+        <v>142883.74</v>
+      </c>
+      <c r="N222" s="6">
+        <v>1</v>
+      </c>
+      <c r="O222" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P222" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q222" s="6">
+        <v>0</v>
+      </c>
+      <c r="R222" s="7">
+        <v>0</v>
+      </c>
+      <c r="S222" s="9">
+        <v>0</v>
+      </c>
+      <c r="T222" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U222" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V222" s="11">
+        <v>11</v>
+      </c>
+      <c r="W222" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X222" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y222" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB222" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG222" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI222" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ222" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK222" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM222" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR222" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="223" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A223" s="1">
+        <v>1</v>
+      </c>
+      <c r="B223" s="2">
+        <v>2</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D223" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E223" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F223" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G223" s="5">
+        <v>223</v>
+      </c>
+      <c r="H223" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I223" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J223" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K223" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L223" s="6">
+        <v>765</v>
+      </c>
+      <c r="M223" s="7">
+        <v>143070.76</v>
+      </c>
+      <c r="N223" s="6">
+        <v>1</v>
+      </c>
+      <c r="O223" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P223" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q223" s="6">
+        <v>0</v>
+      </c>
+      <c r="R223" s="7">
+        <v>0</v>
+      </c>
+      <c r="S223" s="9">
+        <v>0</v>
+      </c>
+      <c r="T223" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U223" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V223" s="11">
+        <v>11</v>
+      </c>
+      <c r="W223" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X223" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y223" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z223" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA223" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB223" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC223" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD223" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE223" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG223" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI223" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ223" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK223" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL223" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM223" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR223" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="224" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A224" s="1">
+        <v>1</v>
+      </c>
+      <c r="B224" s="2">
+        <v>2</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D224" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E224" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F224" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G224" s="5">
+        <v>224</v>
+      </c>
+      <c r="H224" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I224" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J224" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K224" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L224" s="6">
+        <v>766</v>
+      </c>
+      <c r="M224" s="7">
+        <v>143257.78</v>
+      </c>
+      <c r="N224" s="6">
+        <v>1</v>
+      </c>
+      <c r="O224" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P224" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q224" s="6">
+        <v>0</v>
+      </c>
+      <c r="R224" s="7">
+        <v>0</v>
+      </c>
+      <c r="S224" s="9">
+        <v>0</v>
+      </c>
+      <c r="T224" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U224" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V224" s="11">
+        <v>11</v>
+      </c>
+      <c r="W224" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X224" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y224" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z224" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA224" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB224" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC224" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD224" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE224" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF224" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG224" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH224" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI224" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ224" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK224" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL224" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM224" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN224" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO224" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP224" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ224" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR224" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="225" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A225" s="1">
+        <v>1</v>
+      </c>
+      <c r="B225" s="2">
+        <v>2</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D225" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E225" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F225" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G225" s="5">
+        <v>225</v>
+      </c>
+      <c r="H225" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I225" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J225" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K225" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L225" s="6">
+        <v>767</v>
+      </c>
+      <c r="M225" s="7">
+        <v>143444.79999999999</v>
+      </c>
+      <c r="N225" s="6">
+        <v>1</v>
+      </c>
+      <c r="O225" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P225" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q225" s="6">
+        <v>0</v>
+      </c>
+      <c r="R225" s="7">
+        <v>0</v>
+      </c>
+      <c r="S225" s="9">
+        <v>0</v>
+      </c>
+      <c r="T225" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U225" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V225" s="11">
+        <v>11</v>
+      </c>
+      <c r="W225" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X225" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y225" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z225" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA225" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB225" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC225" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD225" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE225" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG225" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI225" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ225" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK225" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL225" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM225" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR225" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="226" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A226" s="1">
+        <v>1</v>
+      </c>
+      <c r="B226" s="2">
+        <v>2</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E226" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F226" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G226" s="5">
+        <v>226</v>
+      </c>
+      <c r="H226" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I226" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J226" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K226" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L226" s="6">
+        <v>768</v>
+      </c>
+      <c r="M226" s="7">
+        <v>143631.82</v>
+      </c>
+      <c r="N226" s="6">
+        <v>1</v>
+      </c>
+      <c r="O226" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P226" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q226" s="6">
+        <v>0</v>
+      </c>
+      <c r="R226" s="7">
+        <v>0</v>
+      </c>
+      <c r="S226" s="9">
+        <v>0</v>
+      </c>
+      <c r="T226" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U226" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V226" s="11">
+        <v>11</v>
+      </c>
+      <c r="W226" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X226" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y226" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB226" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG226" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI226" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ226" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK226" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL226" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM226" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ226" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR226" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="227" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A227" s="1">
+        <v>1</v>
+      </c>
+      <c r="B227" s="2">
+        <v>2</v>
+      </c>
+      <c r="C227" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D227" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E227" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F227" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G227" s="5">
+        <v>227</v>
+      </c>
+      <c r="H227" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I227" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J227" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K227" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L227" s="6">
+        <v>769</v>
+      </c>
+      <c r="M227" s="7">
+        <v>143818.84</v>
+      </c>
+      <c r="N227" s="6">
+        <v>1</v>
+      </c>
+      <c r="O227" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P227" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q227" s="6">
+        <v>0</v>
+      </c>
+      <c r="R227" s="7">
+        <v>0</v>
+      </c>
+      <c r="S227" s="9">
+        <v>0</v>
+      </c>
+      <c r="T227" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U227" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V227" s="11">
+        <v>11</v>
+      </c>
+      <c r="W227" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X227" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y227" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB227" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG227" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI227" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ227" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK227" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL227" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM227" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR227" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="228" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A228" s="1">
+        <v>1</v>
+      </c>
+      <c r="B228" s="2">
+        <v>2</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D228" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E228" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F228" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G228" s="5">
+        <v>228</v>
+      </c>
+      <c r="H228" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I228" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J228" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K228" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L228" s="6">
+        <v>770</v>
+      </c>
+      <c r="M228" s="7">
+        <v>144005.85999999999</v>
+      </c>
+      <c r="N228" s="6">
+        <v>1</v>
+      </c>
+      <c r="O228" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P228" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q228" s="6">
+        <v>0</v>
+      </c>
+      <c r="R228" s="7">
+        <v>0</v>
+      </c>
+      <c r="S228" s="9">
+        <v>0</v>
+      </c>
+      <c r="T228" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U228" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V228" s="11">
+        <v>11</v>
+      </c>
+      <c r="W228" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X228" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y228" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB228" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG228" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI228" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ228" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK228" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL228" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM228" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ228" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR228" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="229" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A229" s="1">
+        <v>1</v>
+      </c>
+      <c r="B229" s="2">
+        <v>2</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D229" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E229" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F229" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G229" s="5">
+        <v>229</v>
+      </c>
+      <c r="H229" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I229" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J229" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K229" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L229" s="6">
+        <v>771</v>
+      </c>
+      <c r="M229" s="7">
+        <v>144192.88</v>
+      </c>
+      <c r="N229" s="6">
+        <v>1</v>
+      </c>
+      <c r="O229" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P229" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q229" s="6">
+        <v>0</v>
+      </c>
+      <c r="R229" s="7">
+        <v>0</v>
+      </c>
+      <c r="S229" s="9">
+        <v>0</v>
+      </c>
+      <c r="T229" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U229" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V229" s="11">
+        <v>11</v>
+      </c>
+      <c r="W229" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X229" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y229" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB229" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG229" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI229" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ229" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK229" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL229" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM229" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR229" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="230" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A230" s="1">
+        <v>1</v>
+      </c>
+      <c r="B230" s="2">
+        <v>2</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E230" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F230" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G230" s="5">
+        <v>230</v>
+      </c>
+      <c r="H230" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I230" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J230" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K230" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L230" s="6">
+        <v>772</v>
+      </c>
+      <c r="M230" s="7">
+        <v>144379.91</v>
+      </c>
+      <c r="N230" s="6">
+        <v>1</v>
+      </c>
+      <c r="O230" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P230" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q230" s="6">
+        <v>0</v>
+      </c>
+      <c r="R230" s="7">
+        <v>0</v>
+      </c>
+      <c r="S230" s="9">
+        <v>0</v>
+      </c>
+      <c r="T230" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U230" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V230" s="11">
+        <v>11</v>
+      </c>
+      <c r="W230" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X230" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y230" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB230" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG230" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI230" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ230" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK230" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL230" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM230" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ230" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR230" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="231" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A231" s="1">
+        <v>1</v>
+      </c>
+      <c r="B231" s="2">
+        <v>2</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E231" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F231" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G231" s="5">
+        <v>231</v>
+      </c>
+      <c r="H231" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I231" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J231" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K231" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L231" s="6">
+        <v>773</v>
+      </c>
+      <c r="M231" s="7">
+        <v>144566.93</v>
+      </c>
+      <c r="N231" s="6">
+        <v>1</v>
+      </c>
+      <c r="O231" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P231" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q231" s="6">
+        <v>0</v>
+      </c>
+      <c r="R231" s="7">
+        <v>0</v>
+      </c>
+      <c r="S231" s="9">
+        <v>0</v>
+      </c>
+      <c r="T231" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U231" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V231" s="11">
+        <v>11</v>
+      </c>
+      <c r="W231" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X231" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y231" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB231" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG231" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI231" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ231" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK231" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL231" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM231" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR231" s="3" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 04/05/2026 14:44:09,61
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7EF04A8-7ED3-4036-8364-3FBC54D76FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{779B1BD0-AC14-4791-ADE2-EF2558168822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5156" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5678" uniqueCount="368">
   <si>
     <t>Sel</t>
   </si>
@@ -1038,6 +1038,93 @@
   <si>
     <t>1858700135667</t>
   </si>
+  <si>
+    <t>1858700135668</t>
+  </si>
+  <si>
+    <t>1858700135669</t>
+  </si>
+  <si>
+    <t>1858700135670</t>
+  </si>
+  <si>
+    <t>1858700135671</t>
+  </si>
+  <si>
+    <t>1858700135672</t>
+  </si>
+  <si>
+    <t>1858700135673</t>
+  </si>
+  <si>
+    <t>1858700135674</t>
+  </si>
+  <si>
+    <t>1858700135675</t>
+  </si>
+  <si>
+    <t>1858700135676</t>
+  </si>
+  <si>
+    <t>1858700135677</t>
+  </si>
+  <si>
+    <t>1858700135678</t>
+  </si>
+  <si>
+    <t>1858700135679</t>
+  </si>
+  <si>
+    <t>1858700135680</t>
+  </si>
+  <si>
+    <t>1858700135681</t>
+  </si>
+  <si>
+    <t>1858700135682</t>
+  </si>
+  <si>
+    <t>1858700135683</t>
+  </si>
+  <si>
+    <t>1858700135684</t>
+  </si>
+  <si>
+    <t>1858700135685</t>
+  </si>
+  <si>
+    <t>1858700135686</t>
+  </si>
+  <si>
+    <t>1858700135687</t>
+  </si>
+  <si>
+    <t>1858700135688</t>
+  </si>
+  <si>
+    <t>1858700135689</t>
+  </si>
+  <si>
+    <t>1858700135690</t>
+  </si>
+  <si>
+    <t>1858700135691</t>
+  </si>
+  <si>
+    <t>1858700135692</t>
+  </si>
+  <si>
+    <t>1858700135693</t>
+  </si>
+  <si>
+    <t>1858700135694</t>
+  </si>
+  <si>
+    <t>1858700135695</t>
+  </si>
+  <si>
+    <t>1858700135696</t>
+  </si>
 </sst>
 </file>
 
@@ -1612,7 +1699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR285"/>
+  <dimension ref="A1:AR314"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -39803,6 +39890,3892 @@
       </c>
       <c r="AR285" s="3" t="s">
         <v>338</v>
+      </c>
+    </row>
+    <row r="286" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A286" s="1">
+        <v>1</v>
+      </c>
+      <c r="B286" s="2">
+        <v>2</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D286" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E286" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F286" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G286" s="5">
+        <v>286</v>
+      </c>
+      <c r="H286" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I286" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J286" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K286" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L286" s="6">
+        <v>828</v>
+      </c>
+      <c r="M286" s="7">
+        <v>154853.06</v>
+      </c>
+      <c r="N286" s="6">
+        <v>1</v>
+      </c>
+      <c r="O286" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P286" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q286" s="6">
+        <v>0</v>
+      </c>
+      <c r="R286" s="7">
+        <v>0</v>
+      </c>
+      <c r="S286" s="9">
+        <v>0</v>
+      </c>
+      <c r="T286" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U286" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V286" s="11">
+        <v>11</v>
+      </c>
+      <c r="W286" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X286" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y286" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB286" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG286" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI286" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ286" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK286" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM286" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR286" s="3" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="287" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A287" s="1">
+        <v>1</v>
+      </c>
+      <c r="B287" s="2">
+        <v>2</v>
+      </c>
+      <c r="C287" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D287" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E287" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F287" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G287" s="5">
+        <v>287</v>
+      </c>
+      <c r="H287" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I287" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J287" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K287" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L287" s="6">
+        <v>829</v>
+      </c>
+      <c r="M287" s="7">
+        <v>155040.07999999999</v>
+      </c>
+      <c r="N287" s="6">
+        <v>1</v>
+      </c>
+      <c r="O287" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P287" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q287" s="6">
+        <v>0</v>
+      </c>
+      <c r="R287" s="7">
+        <v>0</v>
+      </c>
+      <c r="S287" s="9">
+        <v>0</v>
+      </c>
+      <c r="T287" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U287" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V287" s="11">
+        <v>11</v>
+      </c>
+      <c r="W287" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X287" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y287" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB287" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG287" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI287" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ287" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK287" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM287" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR287" s="3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="288" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A288" s="1">
+        <v>1</v>
+      </c>
+      <c r="B288" s="2">
+        <v>2</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E288" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F288" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G288" s="5">
+        <v>288</v>
+      </c>
+      <c r="H288" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I288" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J288" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K288" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L288" s="6">
+        <v>830</v>
+      </c>
+      <c r="M288" s="7">
+        <v>155227.1</v>
+      </c>
+      <c r="N288" s="6">
+        <v>1</v>
+      </c>
+      <c r="O288" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P288" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q288" s="6">
+        <v>0</v>
+      </c>
+      <c r="R288" s="7">
+        <v>0</v>
+      </c>
+      <c r="S288" s="9">
+        <v>0</v>
+      </c>
+      <c r="T288" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U288" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V288" s="11">
+        <v>11</v>
+      </c>
+      <c r="W288" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X288" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y288" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB288" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG288" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI288" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ288" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK288" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM288" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR288" s="3" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="289" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A289" s="1">
+        <v>1</v>
+      </c>
+      <c r="B289" s="2">
+        <v>2</v>
+      </c>
+      <c r="C289" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D289" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E289" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F289" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G289" s="5">
+        <v>289</v>
+      </c>
+      <c r="H289" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I289" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J289" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K289" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L289" s="6">
+        <v>831</v>
+      </c>
+      <c r="M289" s="7">
+        <v>155414.12</v>
+      </c>
+      <c r="N289" s="6">
+        <v>1</v>
+      </c>
+      <c r="O289" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P289" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q289" s="6">
+        <v>0</v>
+      </c>
+      <c r="R289" s="7">
+        <v>0</v>
+      </c>
+      <c r="S289" s="9">
+        <v>0</v>
+      </c>
+      <c r="T289" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U289" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V289" s="11">
+        <v>11</v>
+      </c>
+      <c r="W289" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X289" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y289" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB289" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG289" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI289" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ289" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK289" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM289" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR289" s="3" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="290" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A290" s="1">
+        <v>1</v>
+      </c>
+      <c r="B290" s="2">
+        <v>2</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D290" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E290" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F290" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G290" s="5">
+        <v>290</v>
+      </c>
+      <c r="H290" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I290" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J290" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K290" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L290" s="6">
+        <v>832</v>
+      </c>
+      <c r="M290" s="7">
+        <v>155601.14000000001</v>
+      </c>
+      <c r="N290" s="6">
+        <v>1</v>
+      </c>
+      <c r="O290" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P290" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q290" s="6">
+        <v>0</v>
+      </c>
+      <c r="R290" s="7">
+        <v>0</v>
+      </c>
+      <c r="S290" s="9">
+        <v>0</v>
+      </c>
+      <c r="T290" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U290" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V290" s="11">
+        <v>11</v>
+      </c>
+      <c r="W290" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X290" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y290" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB290" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG290" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI290" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ290" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK290" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM290" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR290" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="291" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A291" s="1">
+        <v>1</v>
+      </c>
+      <c r="B291" s="2">
+        <v>2</v>
+      </c>
+      <c r="C291" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D291" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E291" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F291" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G291" s="5">
+        <v>291</v>
+      </c>
+      <c r="H291" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I291" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J291" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K291" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L291" s="6">
+        <v>833</v>
+      </c>
+      <c r="M291" s="7">
+        <v>155788.16</v>
+      </c>
+      <c r="N291" s="6">
+        <v>1</v>
+      </c>
+      <c r="O291" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P291" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q291" s="6">
+        <v>0</v>
+      </c>
+      <c r="R291" s="7">
+        <v>0</v>
+      </c>
+      <c r="S291" s="9">
+        <v>0</v>
+      </c>
+      <c r="T291" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U291" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V291" s="11">
+        <v>11</v>
+      </c>
+      <c r="W291" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X291" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y291" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB291" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG291" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI291" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ291" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK291" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM291" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR291" s="3" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="292" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A292" s="1">
+        <v>1</v>
+      </c>
+      <c r="B292" s="2">
+        <v>2</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F292" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G292" s="5">
+        <v>292</v>
+      </c>
+      <c r="H292" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I292" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J292" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K292" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L292" s="6">
+        <v>834</v>
+      </c>
+      <c r="M292" s="7">
+        <v>155975.18</v>
+      </c>
+      <c r="N292" s="6">
+        <v>1</v>
+      </c>
+      <c r="O292" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P292" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q292" s="6">
+        <v>0</v>
+      </c>
+      <c r="R292" s="7">
+        <v>0</v>
+      </c>
+      <c r="S292" s="9">
+        <v>0</v>
+      </c>
+      <c r="T292" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U292" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V292" s="11">
+        <v>11</v>
+      </c>
+      <c r="W292" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X292" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y292" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB292" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG292" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI292" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ292" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK292" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM292" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR292" s="3" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="293" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A293" s="1">
+        <v>1</v>
+      </c>
+      <c r="B293" s="2">
+        <v>2</v>
+      </c>
+      <c r="C293" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D293" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E293" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F293" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G293" s="5">
+        <v>293</v>
+      </c>
+      <c r="H293" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I293" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J293" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K293" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L293" s="6">
+        <v>835</v>
+      </c>
+      <c r="M293" s="7">
+        <v>156162.20000000001</v>
+      </c>
+      <c r="N293" s="6">
+        <v>1</v>
+      </c>
+      <c r="O293" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P293" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q293" s="6">
+        <v>0</v>
+      </c>
+      <c r="R293" s="7">
+        <v>0</v>
+      </c>
+      <c r="S293" s="9">
+        <v>0</v>
+      </c>
+      <c r="T293" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U293" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V293" s="11">
+        <v>11</v>
+      </c>
+      <c r="W293" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X293" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y293" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB293" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG293" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI293" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ293" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK293" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM293" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR293" s="3" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="294" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A294" s="1">
+        <v>1</v>
+      </c>
+      <c r="B294" s="2">
+        <v>2</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F294" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G294" s="5">
+        <v>294</v>
+      </c>
+      <c r="H294" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I294" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J294" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K294" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L294" s="6">
+        <v>836</v>
+      </c>
+      <c r="M294" s="7">
+        <v>156349.22</v>
+      </c>
+      <c r="N294" s="6">
+        <v>1</v>
+      </c>
+      <c r="O294" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P294" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q294" s="6">
+        <v>0</v>
+      </c>
+      <c r="R294" s="7">
+        <v>0</v>
+      </c>
+      <c r="S294" s="9">
+        <v>0</v>
+      </c>
+      <c r="T294" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U294" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V294" s="11">
+        <v>11</v>
+      </c>
+      <c r="W294" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X294" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y294" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB294" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG294" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI294" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ294" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK294" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM294" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR294" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="295" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A295" s="1">
+        <v>1</v>
+      </c>
+      <c r="B295" s="2">
+        <v>2</v>
+      </c>
+      <c r="C295" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E295" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F295" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G295" s="5">
+        <v>295</v>
+      </c>
+      <c r="H295" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I295" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J295" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K295" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L295" s="6">
+        <v>837</v>
+      </c>
+      <c r="M295" s="7">
+        <v>156536.24</v>
+      </c>
+      <c r="N295" s="6">
+        <v>1</v>
+      </c>
+      <c r="O295" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P295" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q295" s="6">
+        <v>0</v>
+      </c>
+      <c r="R295" s="7">
+        <v>0</v>
+      </c>
+      <c r="S295" s="9">
+        <v>0</v>
+      </c>
+      <c r="T295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U295" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V295" s="11">
+        <v>11</v>
+      </c>
+      <c r="W295" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X295" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y295" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB295" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG295" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI295" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR295" s="3" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="296" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A296" s="1">
+        <v>1</v>
+      </c>
+      <c r="B296" s="2">
+        <v>2</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F296" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G296" s="5">
+        <v>296</v>
+      </c>
+      <c r="H296" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I296" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J296" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K296" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L296" s="6">
+        <v>838</v>
+      </c>
+      <c r="M296" s="7">
+        <v>156723.26</v>
+      </c>
+      <c r="N296" s="6">
+        <v>1</v>
+      </c>
+      <c r="O296" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P296" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q296" s="6">
+        <v>0</v>
+      </c>
+      <c r="R296" s="7">
+        <v>0</v>
+      </c>
+      <c r="S296" s="9">
+        <v>0</v>
+      </c>
+      <c r="T296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U296" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V296" s="11">
+        <v>11</v>
+      </c>
+      <c r="W296" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X296" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y296" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB296" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG296" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI296" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR296" s="3" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="297" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A297" s="1">
+        <v>1</v>
+      </c>
+      <c r="B297" s="2">
+        <v>2</v>
+      </c>
+      <c r="C297" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E297" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F297" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G297" s="5">
+        <v>297</v>
+      </c>
+      <c r="H297" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I297" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J297" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K297" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L297" s="6">
+        <v>839</v>
+      </c>
+      <c r="M297" s="7">
+        <v>156910.29</v>
+      </c>
+      <c r="N297" s="6">
+        <v>1</v>
+      </c>
+      <c r="O297" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P297" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q297" s="6">
+        <v>0</v>
+      </c>
+      <c r="R297" s="7">
+        <v>0</v>
+      </c>
+      <c r="S297" s="9">
+        <v>0</v>
+      </c>
+      <c r="T297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U297" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V297" s="11">
+        <v>11</v>
+      </c>
+      <c r="W297" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X297" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y297" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB297" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG297" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI297" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR297" s="3" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="298" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A298" s="1">
+        <v>1</v>
+      </c>
+      <c r="B298" s="2">
+        <v>2</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F298" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G298" s="5">
+        <v>298</v>
+      </c>
+      <c r="H298" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I298" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J298" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K298" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L298" s="6">
+        <v>840</v>
+      </c>
+      <c r="M298" s="7">
+        <v>157097.31</v>
+      </c>
+      <c r="N298" s="6">
+        <v>1</v>
+      </c>
+      <c r="O298" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P298" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q298" s="6">
+        <v>0</v>
+      </c>
+      <c r="R298" s="7">
+        <v>0</v>
+      </c>
+      <c r="S298" s="9">
+        <v>0</v>
+      </c>
+      <c r="T298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U298" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V298" s="11">
+        <v>11</v>
+      </c>
+      <c r="W298" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X298" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y298" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB298" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG298" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI298" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR298" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="299" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A299" s="1">
+        <v>1</v>
+      </c>
+      <c r="B299" s="2">
+        <v>2</v>
+      </c>
+      <c r="C299" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D299" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E299" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F299" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G299" s="5">
+        <v>299</v>
+      </c>
+      <c r="H299" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I299" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J299" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K299" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L299" s="6">
+        <v>841</v>
+      </c>
+      <c r="M299" s="7">
+        <v>157284.32999999999</v>
+      </c>
+      <c r="N299" s="6">
+        <v>1</v>
+      </c>
+      <c r="O299" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P299" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q299" s="6">
+        <v>0</v>
+      </c>
+      <c r="R299" s="7">
+        <v>0</v>
+      </c>
+      <c r="S299" s="9">
+        <v>0</v>
+      </c>
+      <c r="T299" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U299" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V299" s="11">
+        <v>11</v>
+      </c>
+      <c r="W299" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X299" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y299" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB299" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG299" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI299" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ299" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK299" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM299" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR299" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="300" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A300" s="1">
+        <v>1</v>
+      </c>
+      <c r="B300" s="2">
+        <v>2</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F300" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G300" s="5">
+        <v>300</v>
+      </c>
+      <c r="H300" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I300" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J300" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K300" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L300" s="6">
+        <v>842</v>
+      </c>
+      <c r="M300" s="7">
+        <v>157471.35</v>
+      </c>
+      <c r="N300" s="6">
+        <v>1</v>
+      </c>
+      <c r="O300" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P300" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q300" s="6">
+        <v>0</v>
+      </c>
+      <c r="R300" s="7">
+        <v>0</v>
+      </c>
+      <c r="S300" s="9">
+        <v>0</v>
+      </c>
+      <c r="T300" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U300" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V300" s="11">
+        <v>11</v>
+      </c>
+      <c r="W300" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X300" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y300" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB300" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG300" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI300" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ300" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK300" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM300" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR300" s="3" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="301" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A301" s="1">
+        <v>1</v>
+      </c>
+      <c r="B301" s="2">
+        <v>2</v>
+      </c>
+      <c r="C301" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D301" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E301" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F301" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G301" s="5">
+        <v>301</v>
+      </c>
+      <c r="H301" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I301" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J301" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K301" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L301" s="6">
+        <v>843</v>
+      </c>
+      <c r="M301" s="7">
+        <v>157658.37</v>
+      </c>
+      <c r="N301" s="6">
+        <v>1</v>
+      </c>
+      <c r="O301" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P301" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q301" s="6">
+        <v>0</v>
+      </c>
+      <c r="R301" s="7">
+        <v>0</v>
+      </c>
+      <c r="S301" s="9">
+        <v>0</v>
+      </c>
+      <c r="T301" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U301" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V301" s="11">
+        <v>11</v>
+      </c>
+      <c r="W301" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X301" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y301" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB301" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG301" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI301" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ301" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK301" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM301" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR301" s="3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="302" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A302" s="1">
+        <v>1</v>
+      </c>
+      <c r="B302" s="2">
+        <v>2</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F302" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G302" s="5">
+        <v>302</v>
+      </c>
+      <c r="H302" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I302" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J302" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K302" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L302" s="6">
+        <v>844</v>
+      </c>
+      <c r="M302" s="7">
+        <v>157845.39000000001</v>
+      </c>
+      <c r="N302" s="6">
+        <v>1</v>
+      </c>
+      <c r="O302" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P302" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q302" s="6">
+        <v>0</v>
+      </c>
+      <c r="R302" s="7">
+        <v>0</v>
+      </c>
+      <c r="S302" s="9">
+        <v>0</v>
+      </c>
+      <c r="T302" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U302" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V302" s="11">
+        <v>11</v>
+      </c>
+      <c r="W302" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X302" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y302" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB302" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG302" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI302" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ302" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK302" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM302" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR302" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="303" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A303" s="1">
+        <v>1</v>
+      </c>
+      <c r="B303" s="2">
+        <v>2</v>
+      </c>
+      <c r="C303" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D303" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E303" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F303" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G303" s="5">
+        <v>303</v>
+      </c>
+      <c r="H303" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I303" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J303" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K303" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L303" s="6">
+        <v>845</v>
+      </c>
+      <c r="M303" s="7">
+        <v>158032.41</v>
+      </c>
+      <c r="N303" s="6">
+        <v>1</v>
+      </c>
+      <c r="O303" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P303" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q303" s="6">
+        <v>0</v>
+      </c>
+      <c r="R303" s="7">
+        <v>0</v>
+      </c>
+      <c r="S303" s="9">
+        <v>0</v>
+      </c>
+      <c r="T303" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U303" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V303" s="11">
+        <v>11</v>
+      </c>
+      <c r="W303" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X303" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y303" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB303" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG303" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI303" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ303" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK303" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM303" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR303" s="3" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="304" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A304" s="1">
+        <v>1</v>
+      </c>
+      <c r="B304" s="2">
+        <v>2</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F304" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G304" s="5">
+        <v>304</v>
+      </c>
+      <c r="H304" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I304" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J304" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K304" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L304" s="6">
+        <v>846</v>
+      </c>
+      <c r="M304" s="7">
+        <v>158219.43</v>
+      </c>
+      <c r="N304" s="6">
+        <v>1</v>
+      </c>
+      <c r="O304" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P304" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q304" s="6">
+        <v>0</v>
+      </c>
+      <c r="R304" s="7">
+        <v>0</v>
+      </c>
+      <c r="S304" s="9">
+        <v>0</v>
+      </c>
+      <c r="T304" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U304" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V304" s="11">
+        <v>11</v>
+      </c>
+      <c r="W304" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X304" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y304" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB304" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG304" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI304" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ304" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK304" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM304" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR304" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="305" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A305" s="1">
+        <v>1</v>
+      </c>
+      <c r="B305" s="2">
+        <v>2</v>
+      </c>
+      <c r="C305" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D305" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E305" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F305" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G305" s="5">
+        <v>305</v>
+      </c>
+      <c r="H305" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I305" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J305" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K305" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L305" s="6">
+        <v>847</v>
+      </c>
+      <c r="M305" s="7">
+        <v>158406.45000000001</v>
+      </c>
+      <c r="N305" s="6">
+        <v>1</v>
+      </c>
+      <c r="O305" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P305" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q305" s="6">
+        <v>0</v>
+      </c>
+      <c r="R305" s="7">
+        <v>0</v>
+      </c>
+      <c r="S305" s="9">
+        <v>0</v>
+      </c>
+      <c r="T305" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U305" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V305" s="11">
+        <v>11</v>
+      </c>
+      <c r="W305" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X305" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y305" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB305" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG305" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI305" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ305" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK305" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM305" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR305" s="3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="306" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A306" s="1">
+        <v>1</v>
+      </c>
+      <c r="B306" s="2">
+        <v>2</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F306" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G306" s="5">
+        <v>306</v>
+      </c>
+      <c r="H306" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I306" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J306" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K306" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L306" s="6">
+        <v>848</v>
+      </c>
+      <c r="M306" s="7">
+        <v>158593.47</v>
+      </c>
+      <c r="N306" s="6">
+        <v>1</v>
+      </c>
+      <c r="O306" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P306" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q306" s="6">
+        <v>0</v>
+      </c>
+      <c r="R306" s="7">
+        <v>0</v>
+      </c>
+      <c r="S306" s="9">
+        <v>0</v>
+      </c>
+      <c r="T306" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U306" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V306" s="11">
+        <v>11</v>
+      </c>
+      <c r="W306" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X306" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y306" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB306" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG306" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI306" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ306" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK306" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM306" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR306" s="3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="307" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A307" s="1">
+        <v>1</v>
+      </c>
+      <c r="B307" s="2">
+        <v>2</v>
+      </c>
+      <c r="C307" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D307" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E307" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F307" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G307" s="5">
+        <v>307</v>
+      </c>
+      <c r="H307" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I307" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J307" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K307" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L307" s="6">
+        <v>849</v>
+      </c>
+      <c r="M307" s="7">
+        <v>158780.49</v>
+      </c>
+      <c r="N307" s="6">
+        <v>1</v>
+      </c>
+      <c r="O307" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P307" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q307" s="6">
+        <v>0</v>
+      </c>
+      <c r="R307" s="7">
+        <v>0</v>
+      </c>
+      <c r="S307" s="9">
+        <v>0</v>
+      </c>
+      <c r="T307" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U307" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V307" s="11">
+        <v>11</v>
+      </c>
+      <c r="W307" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X307" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y307" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB307" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG307" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI307" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ307" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK307" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM307" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR307" s="3" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="308" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A308" s="1">
+        <v>1</v>
+      </c>
+      <c r="B308" s="2">
+        <v>2</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E308" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F308" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G308" s="5">
+        <v>308</v>
+      </c>
+      <c r="H308" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I308" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J308" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K308" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L308" s="6">
+        <v>850</v>
+      </c>
+      <c r="M308" s="7">
+        <v>158967.51</v>
+      </c>
+      <c r="N308" s="6">
+        <v>1</v>
+      </c>
+      <c r="O308" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P308" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q308" s="6">
+        <v>0</v>
+      </c>
+      <c r="R308" s="7">
+        <v>0</v>
+      </c>
+      <c r="S308" s="9">
+        <v>0</v>
+      </c>
+      <c r="T308" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U308" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V308" s="11">
+        <v>11</v>
+      </c>
+      <c r="W308" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X308" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y308" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB308" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG308" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI308" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ308" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK308" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM308" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR308" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="309" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A309" s="1">
+        <v>1</v>
+      </c>
+      <c r="B309" s="2">
+        <v>2</v>
+      </c>
+      <c r="C309" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D309" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E309" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F309" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G309" s="5">
+        <v>309</v>
+      </c>
+      <c r="H309" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I309" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J309" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K309" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L309" s="6">
+        <v>851</v>
+      </c>
+      <c r="M309" s="7">
+        <v>159154.53</v>
+      </c>
+      <c r="N309" s="6">
+        <v>1</v>
+      </c>
+      <c r="O309" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P309" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q309" s="6">
+        <v>0</v>
+      </c>
+      <c r="R309" s="7">
+        <v>0</v>
+      </c>
+      <c r="S309" s="9">
+        <v>0</v>
+      </c>
+      <c r="T309" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U309" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V309" s="11">
+        <v>11</v>
+      </c>
+      <c r="W309" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X309" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y309" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB309" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG309" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI309" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ309" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK309" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM309" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR309" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="310" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A310" s="1">
+        <v>1</v>
+      </c>
+      <c r="B310" s="2">
+        <v>2</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E310" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F310" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G310" s="5">
+        <v>310</v>
+      </c>
+      <c r="H310" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I310" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J310" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K310" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L310" s="6">
+        <v>852</v>
+      </c>
+      <c r="M310" s="7">
+        <v>159341.54999999999</v>
+      </c>
+      <c r="N310" s="6">
+        <v>1</v>
+      </c>
+      <c r="O310" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P310" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q310" s="6">
+        <v>0</v>
+      </c>
+      <c r="R310" s="7">
+        <v>0</v>
+      </c>
+      <c r="S310" s="9">
+        <v>0</v>
+      </c>
+      <c r="T310" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U310" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V310" s="11">
+        <v>11</v>
+      </c>
+      <c r="W310" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X310" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y310" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB310" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG310" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI310" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ310" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK310" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM310" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR310" s="3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="311" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A311" s="1">
+        <v>1</v>
+      </c>
+      <c r="B311" s="2">
+        <v>2</v>
+      </c>
+      <c r="C311" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D311" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E311" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F311" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G311" s="5">
+        <v>311</v>
+      </c>
+      <c r="H311" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I311" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J311" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K311" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L311" s="6">
+        <v>853</v>
+      </c>
+      <c r="M311" s="7">
+        <v>159528.57</v>
+      </c>
+      <c r="N311" s="6">
+        <v>1</v>
+      </c>
+      <c r="O311" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P311" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q311" s="6">
+        <v>0</v>
+      </c>
+      <c r="R311" s="7">
+        <v>0</v>
+      </c>
+      <c r="S311" s="9">
+        <v>0</v>
+      </c>
+      <c r="T311" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U311" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V311" s="11">
+        <v>11</v>
+      </c>
+      <c r="W311" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X311" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y311" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB311" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG311" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI311" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ311" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK311" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM311" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR311" s="3" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="312" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A312" s="1">
+        <v>1</v>
+      </c>
+      <c r="B312" s="2">
+        <v>2</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F312" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G312" s="5">
+        <v>312</v>
+      </c>
+      <c r="H312" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I312" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J312" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K312" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L312" s="6">
+        <v>854</v>
+      </c>
+      <c r="M312" s="7">
+        <v>159715.59</v>
+      </c>
+      <c r="N312" s="6">
+        <v>1</v>
+      </c>
+      <c r="O312" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P312" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q312" s="6">
+        <v>0</v>
+      </c>
+      <c r="R312" s="7">
+        <v>0</v>
+      </c>
+      <c r="S312" s="9">
+        <v>0</v>
+      </c>
+      <c r="T312" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U312" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V312" s="11">
+        <v>11</v>
+      </c>
+      <c r="W312" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X312" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y312" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB312" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG312" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI312" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ312" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK312" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM312" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR312" s="3" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="313" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A313" s="1">
+        <v>1</v>
+      </c>
+      <c r="B313" s="2">
+        <v>2</v>
+      </c>
+      <c r="C313" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D313" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E313" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F313" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G313" s="5">
+        <v>313</v>
+      </c>
+      <c r="H313" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I313" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J313" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K313" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L313" s="6">
+        <v>855</v>
+      </c>
+      <c r="M313" s="7">
+        <v>159902.62</v>
+      </c>
+      <c r="N313" s="6">
+        <v>1</v>
+      </c>
+      <c r="O313" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P313" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q313" s="6">
+        <v>0</v>
+      </c>
+      <c r="R313" s="7">
+        <v>0</v>
+      </c>
+      <c r="S313" s="9">
+        <v>0</v>
+      </c>
+      <c r="T313" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U313" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V313" s="11">
+        <v>11</v>
+      </c>
+      <c r="W313" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X313" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y313" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB313" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG313" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI313" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ313" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK313" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM313" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR313" s="3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="314" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A314" s="1">
+        <v>1</v>
+      </c>
+      <c r="B314" s="2">
+        <v>2</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D314" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E314" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F314" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G314" s="5">
+        <v>314</v>
+      </c>
+      <c r="H314" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I314" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J314" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K314" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L314" s="6">
+        <v>856</v>
+      </c>
+      <c r="M314" s="7">
+        <v>160089.64000000001</v>
+      </c>
+      <c r="N314" s="6">
+        <v>1</v>
+      </c>
+      <c r="O314" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P314" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q314" s="6">
+        <v>0</v>
+      </c>
+      <c r="R314" s="7">
+        <v>0</v>
+      </c>
+      <c r="S314" s="9">
+        <v>0</v>
+      </c>
+      <c r="T314" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U314" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V314" s="11">
+        <v>11</v>
+      </c>
+      <c r="W314" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X314" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y314" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB314" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG314" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI314" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ314" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK314" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM314" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR314" s="3" t="s">
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 04/05/2026 15:20:11,86
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{779B1BD0-AC14-4791-ADE2-EF2558168822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{98491158-14A1-4FC0-89E0-7383C1C14DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5678" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6146" uniqueCount="394">
   <si>
     <t>Sel</t>
   </si>
@@ -1125,6 +1125,84 @@
   <si>
     <t>1858700135696</t>
   </si>
+  <si>
+    <t>1858700135697</t>
+  </si>
+  <si>
+    <t>1858700135698</t>
+  </si>
+  <si>
+    <t>1858700135699</t>
+  </si>
+  <si>
+    <t>1858700135700</t>
+  </si>
+  <si>
+    <t>1858700135701</t>
+  </si>
+  <si>
+    <t>1858700135702</t>
+  </si>
+  <si>
+    <t>1858700135703</t>
+  </si>
+  <si>
+    <t>1858700135704</t>
+  </si>
+  <si>
+    <t>1858700135705</t>
+  </si>
+  <si>
+    <t>1858700135706</t>
+  </si>
+  <si>
+    <t>1858700135707</t>
+  </si>
+  <si>
+    <t>1858700135708</t>
+  </si>
+  <si>
+    <t>1858700135709</t>
+  </si>
+  <si>
+    <t>1858700135710</t>
+  </si>
+  <si>
+    <t>1858700135711</t>
+  </si>
+  <si>
+    <t>1858700135712</t>
+  </si>
+  <si>
+    <t>1858700135713</t>
+  </si>
+  <si>
+    <t>1858700135714</t>
+  </si>
+  <si>
+    <t>1858700135715</t>
+  </si>
+  <si>
+    <t>1858700135716</t>
+  </si>
+  <si>
+    <t>1858700135717</t>
+  </si>
+  <si>
+    <t>1858700135718</t>
+  </si>
+  <si>
+    <t>1858700135719</t>
+  </si>
+  <si>
+    <t>1858700135720</t>
+  </si>
+  <si>
+    <t>1858700135721</t>
+  </si>
+  <si>
+    <t>1858700135722</t>
+  </si>
 </sst>
 </file>
 
@@ -1699,7 +1777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR314"/>
+  <dimension ref="A1:AR340"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -43776,6 +43854,3490 @@
       </c>
       <c r="AR314" s="3" t="s">
         <v>367</v>
+      </c>
+    </row>
+    <row r="315" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A315" s="1">
+        <v>1</v>
+      </c>
+      <c r="B315" s="2">
+        <v>2</v>
+      </c>
+      <c r="C315" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D315" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E315" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F315" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G315" s="5">
+        <v>315</v>
+      </c>
+      <c r="H315" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I315" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J315" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K315" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L315" s="6">
+        <v>857</v>
+      </c>
+      <c r="M315" s="7">
+        <v>160276.66</v>
+      </c>
+      <c r="N315" s="6">
+        <v>1</v>
+      </c>
+      <c r="O315" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P315" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q315" s="6">
+        <v>0</v>
+      </c>
+      <c r="R315" s="7">
+        <v>0</v>
+      </c>
+      <c r="S315" s="9">
+        <v>0</v>
+      </c>
+      <c r="T315" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U315" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V315" s="11">
+        <v>11</v>
+      </c>
+      <c r="W315" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X315" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y315" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB315" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG315" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI315" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ315" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK315" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM315" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR315" s="3" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="316" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A316" s="1">
+        <v>1</v>
+      </c>
+      <c r="B316" s="2">
+        <v>2</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D316" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E316" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F316" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G316" s="5">
+        <v>316</v>
+      </c>
+      <c r="H316" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I316" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J316" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K316" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L316" s="6">
+        <v>858</v>
+      </c>
+      <c r="M316" s="7">
+        <v>160463.67999999999</v>
+      </c>
+      <c r="N316" s="6">
+        <v>1</v>
+      </c>
+      <c r="O316" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P316" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q316" s="6">
+        <v>0</v>
+      </c>
+      <c r="R316" s="7">
+        <v>0</v>
+      </c>
+      <c r="S316" s="9">
+        <v>0</v>
+      </c>
+      <c r="T316" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U316" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V316" s="11">
+        <v>11</v>
+      </c>
+      <c r="W316" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X316" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y316" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB316" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG316" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI316" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ316" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK316" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM316" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR316" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="317" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A317" s="1">
+        <v>1</v>
+      </c>
+      <c r="B317" s="2">
+        <v>2</v>
+      </c>
+      <c r="C317" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D317" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E317" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F317" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G317" s="5">
+        <v>317</v>
+      </c>
+      <c r="H317" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I317" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J317" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K317" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L317" s="6">
+        <v>859</v>
+      </c>
+      <c r="M317" s="7">
+        <v>160650.70000000001</v>
+      </c>
+      <c r="N317" s="6">
+        <v>1</v>
+      </c>
+      <c r="O317" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P317" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q317" s="6">
+        <v>0</v>
+      </c>
+      <c r="R317" s="7">
+        <v>0</v>
+      </c>
+      <c r="S317" s="9">
+        <v>0</v>
+      </c>
+      <c r="T317" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U317" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V317" s="11">
+        <v>11</v>
+      </c>
+      <c r="W317" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X317" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y317" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB317" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG317" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI317" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ317" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK317" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM317" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR317" s="3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="318" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A318" s="1">
+        <v>1</v>
+      </c>
+      <c r="B318" s="2">
+        <v>2</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D318" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E318" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F318" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G318" s="5">
+        <v>318</v>
+      </c>
+      <c r="H318" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I318" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J318" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K318" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L318" s="6">
+        <v>860</v>
+      </c>
+      <c r="M318" s="7">
+        <v>160837.72</v>
+      </c>
+      <c r="N318" s="6">
+        <v>1</v>
+      </c>
+      <c r="O318" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P318" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q318" s="6">
+        <v>0</v>
+      </c>
+      <c r="R318" s="7">
+        <v>0</v>
+      </c>
+      <c r="S318" s="9">
+        <v>0</v>
+      </c>
+      <c r="T318" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U318" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V318" s="11">
+        <v>11</v>
+      </c>
+      <c r="W318" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X318" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y318" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB318" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG318" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI318" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ318" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK318" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM318" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR318" s="3" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="319" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A319" s="1">
+        <v>1</v>
+      </c>
+      <c r="B319" s="2">
+        <v>2</v>
+      </c>
+      <c r="C319" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D319" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E319" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F319" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G319" s="5">
+        <v>319</v>
+      </c>
+      <c r="H319" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I319" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J319" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K319" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L319" s="6">
+        <v>861</v>
+      </c>
+      <c r="M319" s="7">
+        <v>161024.74</v>
+      </c>
+      <c r="N319" s="6">
+        <v>1</v>
+      </c>
+      <c r="O319" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P319" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q319" s="6">
+        <v>0</v>
+      </c>
+      <c r="R319" s="7">
+        <v>0</v>
+      </c>
+      <c r="S319" s="9">
+        <v>0</v>
+      </c>
+      <c r="T319" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U319" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V319" s="11">
+        <v>11</v>
+      </c>
+      <c r="W319" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X319" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y319" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB319" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG319" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI319" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ319" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK319" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM319" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR319" s="3" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="320" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A320" s="1">
+        <v>1</v>
+      </c>
+      <c r="B320" s="2">
+        <v>2</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D320" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E320" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F320" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G320" s="5">
+        <v>320</v>
+      </c>
+      <c r="H320" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I320" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J320" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K320" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L320" s="6">
+        <v>862</v>
+      </c>
+      <c r="M320" s="7">
+        <v>161211.76</v>
+      </c>
+      <c r="N320" s="6">
+        <v>1</v>
+      </c>
+      <c r="O320" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P320" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q320" s="6">
+        <v>0</v>
+      </c>
+      <c r="R320" s="7">
+        <v>0</v>
+      </c>
+      <c r="S320" s="9">
+        <v>0</v>
+      </c>
+      <c r="T320" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U320" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V320" s="11">
+        <v>11</v>
+      </c>
+      <c r="W320" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X320" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y320" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB320" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG320" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI320" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ320" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK320" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM320" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR320" s="3" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="321" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A321" s="1">
+        <v>1</v>
+      </c>
+      <c r="B321" s="2">
+        <v>2</v>
+      </c>
+      <c r="C321" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D321" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E321" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F321" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G321" s="5">
+        <v>321</v>
+      </c>
+      <c r="H321" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I321" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J321" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K321" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L321" s="6">
+        <v>863</v>
+      </c>
+      <c r="M321" s="7">
+        <v>161398.78</v>
+      </c>
+      <c r="N321" s="6">
+        <v>1</v>
+      </c>
+      <c r="O321" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P321" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q321" s="6">
+        <v>0</v>
+      </c>
+      <c r="R321" s="7">
+        <v>0</v>
+      </c>
+      <c r="S321" s="9">
+        <v>0</v>
+      </c>
+      <c r="T321" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U321" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V321" s="11">
+        <v>11</v>
+      </c>
+      <c r="W321" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X321" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y321" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z321" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA321" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB321" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC321" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD321" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE321" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG321" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI321" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ321" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK321" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL321" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM321" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR321" s="3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="322" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A322" s="1">
+        <v>1</v>
+      </c>
+      <c r="B322" s="2">
+        <v>2</v>
+      </c>
+      <c r="C322" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D322" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E322" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F322" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G322" s="5">
+        <v>322</v>
+      </c>
+      <c r="H322" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I322" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J322" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K322" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L322" s="6">
+        <v>864</v>
+      </c>
+      <c r="M322" s="7">
+        <v>161585.79999999999</v>
+      </c>
+      <c r="N322" s="6">
+        <v>1</v>
+      </c>
+      <c r="O322" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P322" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q322" s="6">
+        <v>0</v>
+      </c>
+      <c r="R322" s="7">
+        <v>0</v>
+      </c>
+      <c r="S322" s="9">
+        <v>0</v>
+      </c>
+      <c r="T322" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U322" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V322" s="11">
+        <v>11</v>
+      </c>
+      <c r="W322" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X322" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y322" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z322" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA322" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB322" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC322" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD322" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE322" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF322" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG322" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH322" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI322" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ322" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK322" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL322" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM322" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN322" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO322" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP322" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ322" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR322" s="3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="323" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A323" s="1">
+        <v>1</v>
+      </c>
+      <c r="B323" s="2">
+        <v>2</v>
+      </c>
+      <c r="C323" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D323" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E323" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F323" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G323" s="5">
+        <v>323</v>
+      </c>
+      <c r="H323" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I323" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J323" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K323" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L323" s="6">
+        <v>865</v>
+      </c>
+      <c r="M323" s="7">
+        <v>161772.82</v>
+      </c>
+      <c r="N323" s="6">
+        <v>1</v>
+      </c>
+      <c r="O323" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P323" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q323" s="6">
+        <v>0</v>
+      </c>
+      <c r="R323" s="7">
+        <v>0</v>
+      </c>
+      <c r="S323" s="9">
+        <v>0</v>
+      </c>
+      <c r="T323" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U323" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V323" s="11">
+        <v>11</v>
+      </c>
+      <c r="W323" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X323" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y323" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z323" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA323" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB323" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC323" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD323" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE323" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG323" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI323" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ323" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK323" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL323" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM323" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR323" s="3" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="324" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A324" s="1">
+        <v>1</v>
+      </c>
+      <c r="B324" s="2">
+        <v>2</v>
+      </c>
+      <c r="C324" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D324" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E324" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F324" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G324" s="5">
+        <v>324</v>
+      </c>
+      <c r="H324" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I324" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J324" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K324" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L324" s="6">
+        <v>866</v>
+      </c>
+      <c r="M324" s="7">
+        <v>161959.84</v>
+      </c>
+      <c r="N324" s="6">
+        <v>1</v>
+      </c>
+      <c r="O324" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P324" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q324" s="6">
+        <v>0</v>
+      </c>
+      <c r="R324" s="7">
+        <v>0</v>
+      </c>
+      <c r="S324" s="9">
+        <v>0</v>
+      </c>
+      <c r="T324" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U324" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V324" s="11">
+        <v>11</v>
+      </c>
+      <c r="W324" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X324" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y324" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z324" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA324" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB324" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC324" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD324" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE324" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG324" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI324" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ324" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK324" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL324" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM324" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR324" s="3" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="325" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A325" s="1">
+        <v>1</v>
+      </c>
+      <c r="B325" s="2">
+        <v>2</v>
+      </c>
+      <c r="C325" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D325" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E325" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F325" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G325" s="5">
+        <v>325</v>
+      </c>
+      <c r="H325" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I325" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J325" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K325" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L325" s="6">
+        <v>867</v>
+      </c>
+      <c r="M325" s="7">
+        <v>162146.85999999999</v>
+      </c>
+      <c r="N325" s="6">
+        <v>1</v>
+      </c>
+      <c r="O325" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P325" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q325" s="6">
+        <v>0</v>
+      </c>
+      <c r="R325" s="7">
+        <v>0</v>
+      </c>
+      <c r="S325" s="9">
+        <v>0</v>
+      </c>
+      <c r="T325" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U325" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V325" s="11">
+        <v>11</v>
+      </c>
+      <c r="W325" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X325" s="12">
+        <v>0.62916669999999997</v>
+      </c>
+      <c r="Y325" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z325" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA325" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB325" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC325" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD325" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE325" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG325" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI325" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ325" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK325" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL325" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM325" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR325" s="3" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="326" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A326" s="1">
+        <v>1</v>
+      </c>
+      <c r="B326" s="2">
+        <v>2</v>
+      </c>
+      <c r="C326" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D326" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E326" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F326" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G326" s="5">
+        <v>326</v>
+      </c>
+      <c r="H326" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I326" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J326" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K326" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L326" s="6">
+        <v>868</v>
+      </c>
+      <c r="M326" s="7">
+        <v>162333.88</v>
+      </c>
+      <c r="N326" s="6">
+        <v>1</v>
+      </c>
+      <c r="O326" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P326" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q326" s="6">
+        <v>0</v>
+      </c>
+      <c r="R326" s="7">
+        <v>0</v>
+      </c>
+      <c r="S326" s="9">
+        <v>0</v>
+      </c>
+      <c r="T326" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U326" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V326" s="11">
+        <v>11</v>
+      </c>
+      <c r="W326" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X326" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y326" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z326" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA326" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB326" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC326" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD326" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE326" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG326" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI326" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ326" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK326" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL326" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM326" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR326" s="3" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="327" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A327" s="1">
+        <v>1</v>
+      </c>
+      <c r="B327" s="2">
+        <v>2</v>
+      </c>
+      <c r="C327" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D327" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E327" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F327" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G327" s="5">
+        <v>327</v>
+      </c>
+      <c r="H327" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I327" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J327" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K327" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L327" s="6">
+        <v>869</v>
+      </c>
+      <c r="M327" s="7">
+        <v>162520.9</v>
+      </c>
+      <c r="N327" s="6">
+        <v>1</v>
+      </c>
+      <c r="O327" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P327" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q327" s="6">
+        <v>0</v>
+      </c>
+      <c r="R327" s="7">
+        <v>0</v>
+      </c>
+      <c r="S327" s="9">
+        <v>0</v>
+      </c>
+      <c r="T327" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U327" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V327" s="11">
+        <v>11</v>
+      </c>
+      <c r="W327" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X327" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y327" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z327" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA327" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB327" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC327" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD327" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE327" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF327" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG327" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH327" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI327" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ327" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK327" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL327" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM327" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN327" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO327" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP327" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ327" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR327" s="3" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="328" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A328" s="1">
+        <v>1</v>
+      </c>
+      <c r="B328" s="2">
+        <v>2</v>
+      </c>
+      <c r="C328" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D328" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E328" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F328" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G328" s="5">
+        <v>328</v>
+      </c>
+      <c r="H328" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I328" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J328" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K328" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L328" s="6">
+        <v>870</v>
+      </c>
+      <c r="M328" s="7">
+        <v>162707.92000000001</v>
+      </c>
+      <c r="N328" s="6">
+        <v>1</v>
+      </c>
+      <c r="O328" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P328" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q328" s="6">
+        <v>0</v>
+      </c>
+      <c r="R328" s="7">
+        <v>0</v>
+      </c>
+      <c r="S328" s="9">
+        <v>0</v>
+      </c>
+      <c r="T328" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U328" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V328" s="11">
+        <v>11</v>
+      </c>
+      <c r="W328" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X328" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y328" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z328" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA328" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB328" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC328" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD328" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE328" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF328" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG328" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH328" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI328" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ328" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK328" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL328" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM328" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN328" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO328" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP328" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ328" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR328" s="3" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="329" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A329" s="1">
+        <v>1</v>
+      </c>
+      <c r="B329" s="2">
+        <v>2</v>
+      </c>
+      <c r="C329" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D329" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E329" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F329" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G329" s="5">
+        <v>329</v>
+      </c>
+      <c r="H329" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I329" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J329" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K329" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L329" s="6">
+        <v>871</v>
+      </c>
+      <c r="M329" s="7">
+        <v>162894.94</v>
+      </c>
+      <c r="N329" s="6">
+        <v>1</v>
+      </c>
+      <c r="O329" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P329" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q329" s="6">
+        <v>0</v>
+      </c>
+      <c r="R329" s="7">
+        <v>0</v>
+      </c>
+      <c r="S329" s="9">
+        <v>0</v>
+      </c>
+      <c r="T329" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U329" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V329" s="11">
+        <v>11</v>
+      </c>
+      <c r="W329" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X329" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y329" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z329" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA329" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB329" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC329" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD329" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE329" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF329" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG329" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH329" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI329" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ329" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK329" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL329" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM329" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN329" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO329" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP329" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ329" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR329" s="3" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="330" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A330" s="1">
+        <v>1</v>
+      </c>
+      <c r="B330" s="2">
+        <v>2</v>
+      </c>
+      <c r="C330" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D330" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E330" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F330" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G330" s="5">
+        <v>330</v>
+      </c>
+      <c r="H330" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I330" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J330" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K330" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L330" s="6">
+        <v>872</v>
+      </c>
+      <c r="M330" s="7">
+        <v>163081.97</v>
+      </c>
+      <c r="N330" s="6">
+        <v>1</v>
+      </c>
+      <c r="O330" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P330" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q330" s="6">
+        <v>0</v>
+      </c>
+      <c r="R330" s="7">
+        <v>0</v>
+      </c>
+      <c r="S330" s="9">
+        <v>0</v>
+      </c>
+      <c r="T330" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U330" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V330" s="11">
+        <v>11</v>
+      </c>
+      <c r="W330" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X330" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y330" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z330" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA330" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB330" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC330" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD330" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE330" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG330" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI330" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ330" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK330" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL330" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM330" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR330" s="3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="331" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A331" s="1">
+        <v>1</v>
+      </c>
+      <c r="B331" s="2">
+        <v>2</v>
+      </c>
+      <c r="C331" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D331" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E331" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F331" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G331" s="5">
+        <v>331</v>
+      </c>
+      <c r="H331" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I331" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J331" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K331" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L331" s="6">
+        <v>873</v>
+      </c>
+      <c r="M331" s="7">
+        <v>163268.99</v>
+      </c>
+      <c r="N331" s="6">
+        <v>1</v>
+      </c>
+      <c r="O331" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P331" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q331" s="6">
+        <v>0</v>
+      </c>
+      <c r="R331" s="7">
+        <v>0</v>
+      </c>
+      <c r="S331" s="9">
+        <v>0</v>
+      </c>
+      <c r="T331" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U331" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V331" s="11">
+        <v>11</v>
+      </c>
+      <c r="W331" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X331" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y331" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z331" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA331" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB331" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC331" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD331" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE331" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG331" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI331" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ331" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK331" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL331" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM331" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR331" s="3" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="332" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A332" s="1">
+        <v>1</v>
+      </c>
+      <c r="B332" s="2">
+        <v>2</v>
+      </c>
+      <c r="C332" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D332" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E332" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F332" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G332" s="5">
+        <v>332</v>
+      </c>
+      <c r="H332" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I332" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J332" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K332" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L332" s="6">
+        <v>874</v>
+      </c>
+      <c r="M332" s="7">
+        <v>163456.01</v>
+      </c>
+      <c r="N332" s="6">
+        <v>1</v>
+      </c>
+      <c r="O332" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P332" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q332" s="6">
+        <v>0</v>
+      </c>
+      <c r="R332" s="7">
+        <v>0</v>
+      </c>
+      <c r="S332" s="9">
+        <v>0</v>
+      </c>
+      <c r="T332" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U332" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V332" s="11">
+        <v>11</v>
+      </c>
+      <c r="W332" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X332" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y332" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z332" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA332" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB332" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC332" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD332" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE332" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG332" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI332" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ332" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK332" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL332" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM332" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR332" s="3" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="333" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A333" s="1">
+        <v>1</v>
+      </c>
+      <c r="B333" s="2">
+        <v>2</v>
+      </c>
+      <c r="C333" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D333" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E333" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F333" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G333" s="5">
+        <v>333</v>
+      </c>
+      <c r="H333" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I333" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J333" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K333" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L333" s="6">
+        <v>875</v>
+      </c>
+      <c r="M333" s="7">
+        <v>163643.03</v>
+      </c>
+      <c r="N333" s="6">
+        <v>1</v>
+      </c>
+      <c r="O333" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P333" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q333" s="6">
+        <v>0</v>
+      </c>
+      <c r="R333" s="7">
+        <v>0</v>
+      </c>
+      <c r="S333" s="9">
+        <v>0</v>
+      </c>
+      <c r="T333" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U333" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V333" s="11">
+        <v>11</v>
+      </c>
+      <c r="W333" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X333" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y333" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z333" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA333" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB333" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC333" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD333" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE333" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF333" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG333" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH333" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI333" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ333" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK333" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL333" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM333" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN333" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO333" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP333" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ333" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR333" s="3" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="334" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A334" s="1">
+        <v>1</v>
+      </c>
+      <c r="B334" s="2">
+        <v>2</v>
+      </c>
+      <c r="C334" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D334" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E334" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F334" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G334" s="5">
+        <v>334</v>
+      </c>
+      <c r="H334" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I334" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J334" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K334" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L334" s="6">
+        <v>876</v>
+      </c>
+      <c r="M334" s="7">
+        <v>163830.04999999999</v>
+      </c>
+      <c r="N334" s="6">
+        <v>1</v>
+      </c>
+      <c r="O334" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P334" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q334" s="6">
+        <v>0</v>
+      </c>
+      <c r="R334" s="7">
+        <v>0</v>
+      </c>
+      <c r="S334" s="9">
+        <v>0</v>
+      </c>
+      <c r="T334" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U334" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V334" s="11">
+        <v>11</v>
+      </c>
+      <c r="W334" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X334" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y334" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB334" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG334" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI334" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ334" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK334" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM334" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR334" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="335" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A335" s="1">
+        <v>1</v>
+      </c>
+      <c r="B335" s="2">
+        <v>2</v>
+      </c>
+      <c r="C335" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D335" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E335" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F335" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G335" s="5">
+        <v>335</v>
+      </c>
+      <c r="H335" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I335" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J335" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K335" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L335" s="6">
+        <v>877</v>
+      </c>
+      <c r="M335" s="7">
+        <v>164017.07</v>
+      </c>
+      <c r="N335" s="6">
+        <v>1</v>
+      </c>
+      <c r="O335" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P335" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q335" s="6">
+        <v>0</v>
+      </c>
+      <c r="R335" s="7">
+        <v>0</v>
+      </c>
+      <c r="S335" s="9">
+        <v>0</v>
+      </c>
+      <c r="T335" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U335" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V335" s="11">
+        <v>11</v>
+      </c>
+      <c r="W335" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X335" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y335" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z335" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA335" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB335" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC335" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD335" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE335" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF335" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG335" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH335" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI335" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ335" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK335" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL335" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM335" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN335" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO335" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP335" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ335" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR335" s="3" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="336" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A336" s="1">
+        <v>1</v>
+      </c>
+      <c r="B336" s="2">
+        <v>2</v>
+      </c>
+      <c r="C336" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D336" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E336" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F336" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G336" s="5">
+        <v>336</v>
+      </c>
+      <c r="H336" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I336" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J336" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K336" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L336" s="6">
+        <v>878</v>
+      </c>
+      <c r="M336" s="7">
+        <v>164204.09</v>
+      </c>
+      <c r="N336" s="6">
+        <v>1</v>
+      </c>
+      <c r="O336" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P336" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q336" s="6">
+        <v>0</v>
+      </c>
+      <c r="R336" s="7">
+        <v>0</v>
+      </c>
+      <c r="S336" s="9">
+        <v>0</v>
+      </c>
+      <c r="T336" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U336" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V336" s="11">
+        <v>11</v>
+      </c>
+      <c r="W336" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X336" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y336" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z336" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA336" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB336" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC336" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD336" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE336" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF336" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG336" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH336" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI336" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ336" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK336" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL336" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM336" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN336" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO336" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP336" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ336" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR336" s="3" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="337" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A337" s="1">
+        <v>1</v>
+      </c>
+      <c r="B337" s="2">
+        <v>2</v>
+      </c>
+      <c r="C337" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D337" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E337" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F337" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G337" s="5">
+        <v>337</v>
+      </c>
+      <c r="H337" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I337" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J337" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K337" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L337" s="6">
+        <v>879</v>
+      </c>
+      <c r="M337" s="7">
+        <v>164391.10999999999</v>
+      </c>
+      <c r="N337" s="6">
+        <v>1</v>
+      </c>
+      <c r="O337" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P337" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q337" s="6">
+        <v>0</v>
+      </c>
+      <c r="R337" s="7">
+        <v>0</v>
+      </c>
+      <c r="S337" s="9">
+        <v>0</v>
+      </c>
+      <c r="T337" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U337" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V337" s="11">
+        <v>11</v>
+      </c>
+      <c r="W337" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X337" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y337" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z337" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA337" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB337" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC337" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD337" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE337" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG337" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI337" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ337" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK337" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL337" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM337" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR337" s="3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="338" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A338" s="1">
+        <v>1</v>
+      </c>
+      <c r="B338" s="2">
+        <v>2</v>
+      </c>
+      <c r="C338" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D338" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E338" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F338" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G338" s="5">
+        <v>338</v>
+      </c>
+      <c r="H338" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I338" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J338" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K338" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L338" s="6">
+        <v>880</v>
+      </c>
+      <c r="M338" s="7">
+        <v>164578.13</v>
+      </c>
+      <c r="N338" s="6">
+        <v>1</v>
+      </c>
+      <c r="O338" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P338" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q338" s="6">
+        <v>0</v>
+      </c>
+      <c r="R338" s="7">
+        <v>0</v>
+      </c>
+      <c r="S338" s="9">
+        <v>0</v>
+      </c>
+      <c r="T338" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U338" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V338" s="11">
+        <v>11</v>
+      </c>
+      <c r="W338" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X338" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y338" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z338" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA338" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB338" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC338" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD338" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE338" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG338" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI338" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ338" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK338" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL338" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM338" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR338" s="3" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="339" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A339" s="1">
+        <v>1</v>
+      </c>
+      <c r="B339" s="2">
+        <v>2</v>
+      </c>
+      <c r="C339" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D339" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E339" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F339" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G339" s="5">
+        <v>339</v>
+      </c>
+      <c r="H339" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I339" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J339" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K339" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L339" s="6">
+        <v>881</v>
+      </c>
+      <c r="M339" s="7">
+        <v>164765.15</v>
+      </c>
+      <c r="N339" s="6">
+        <v>1</v>
+      </c>
+      <c r="O339" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P339" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q339" s="6">
+        <v>0</v>
+      </c>
+      <c r="R339" s="7">
+        <v>0</v>
+      </c>
+      <c r="S339" s="9">
+        <v>0</v>
+      </c>
+      <c r="T339" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U339" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V339" s="11">
+        <v>11</v>
+      </c>
+      <c r="W339" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X339" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y339" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z339" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA339" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB339" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC339" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD339" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE339" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG339" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI339" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ339" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK339" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL339" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM339" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR339" s="3" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="340" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A340" s="1">
+        <v>1</v>
+      </c>
+      <c r="B340" s="2">
+        <v>2</v>
+      </c>
+      <c r="C340" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D340" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E340" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F340" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G340" s="5">
+        <v>340</v>
+      </c>
+      <c r="H340" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I340" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J340" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K340" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L340" s="6">
+        <v>882</v>
+      </c>
+      <c r="M340" s="7">
+        <v>164952.17000000001</v>
+      </c>
+      <c r="N340" s="6">
+        <v>1</v>
+      </c>
+      <c r="O340" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P340" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q340" s="6">
+        <v>0</v>
+      </c>
+      <c r="R340" s="7">
+        <v>0</v>
+      </c>
+      <c r="S340" s="9">
+        <v>0</v>
+      </c>
+      <c r="T340" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U340" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V340" s="11">
+        <v>11</v>
+      </c>
+      <c r="W340" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X340" s="12">
+        <v>0.62986109999999995</v>
+      </c>
+      <c r="Y340" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z340" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA340" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB340" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC340" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD340" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE340" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF340" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG340" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH340" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI340" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ340" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK340" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL340" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM340" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN340" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO340" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP340" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ340" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR340" s="3" t="s">
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 04/05/2026 16:45:50,82
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9D9F3EA-7A66-4517-967E-7F31C1403349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE52F25C-131A-4683-A9B3-1C001AFA55CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7172" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7550" uniqueCount="472">
   <si>
     <t>Sel</t>
   </si>
@@ -1374,6 +1374,69 @@
   <si>
     <t>1858700135779</t>
   </si>
+  <si>
+    <t>1858700135780</t>
+  </si>
+  <si>
+    <t>1858700135781</t>
+  </si>
+  <si>
+    <t>1858700135782</t>
+  </si>
+  <si>
+    <t>1858700135783</t>
+  </si>
+  <si>
+    <t>1858700135784</t>
+  </si>
+  <si>
+    <t>1858700135785</t>
+  </si>
+  <si>
+    <t>1858700135786</t>
+  </si>
+  <si>
+    <t>1858700135787</t>
+  </si>
+  <si>
+    <t>1858700135788</t>
+  </si>
+  <si>
+    <t>1858700135789</t>
+  </si>
+  <si>
+    <t>1858700135790</t>
+  </si>
+  <si>
+    <t>1858700135791</t>
+  </si>
+  <si>
+    <t>1858700135792</t>
+  </si>
+  <si>
+    <t>1858700135793</t>
+  </si>
+  <si>
+    <t>1858700135794</t>
+  </si>
+  <si>
+    <t>1858700135795</t>
+  </si>
+  <si>
+    <t>1858700135796</t>
+  </si>
+  <si>
+    <t>1858700135797</t>
+  </si>
+  <si>
+    <t>1858700135798</t>
+  </si>
+  <si>
+    <t>1858700135799</t>
+  </si>
+  <si>
+    <t>1858700135800</t>
+  </si>
 </sst>
 </file>
 
@@ -1948,7 +2011,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR397"/>
+  <dimension ref="A1:AR418"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -55147,6 +55210,2820 @@
       </c>
       <c r="AR397" s="3" t="s">
         <v>450</v>
+      </c>
+    </row>
+    <row r="398" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A398" s="1">
+        <v>1</v>
+      </c>
+      <c r="B398" s="2">
+        <v>2</v>
+      </c>
+      <c r="C398" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D398" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E398" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F398" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G398" s="5">
+        <v>434</v>
+      </c>
+      <c r="H398" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I398" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J398" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K398" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L398" s="6">
+        <v>681</v>
+      </c>
+      <c r="M398" s="7">
+        <v>127361.03</v>
+      </c>
+      <c r="N398" s="6">
+        <v>1</v>
+      </c>
+      <c r="O398" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P398" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q398" s="6">
+        <v>0</v>
+      </c>
+      <c r="R398" s="7">
+        <v>0</v>
+      </c>
+      <c r="S398" s="9">
+        <v>0</v>
+      </c>
+      <c r="T398" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U398" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V398" s="11">
+        <v>11</v>
+      </c>
+      <c r="W398" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X398" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y398" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB398" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG398" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI398" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ398" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK398" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM398" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR398" s="3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="399" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A399" s="1">
+        <v>1</v>
+      </c>
+      <c r="B399" s="2">
+        <v>2</v>
+      </c>
+      <c r="C399" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D399" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E399" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F399" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G399" s="5">
+        <v>435</v>
+      </c>
+      <c r="H399" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I399" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J399" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K399" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L399" s="6">
+        <v>682</v>
+      </c>
+      <c r="M399" s="7">
+        <v>127548.05</v>
+      </c>
+      <c r="N399" s="6">
+        <v>1</v>
+      </c>
+      <c r="O399" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P399" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q399" s="6">
+        <v>0</v>
+      </c>
+      <c r="R399" s="7">
+        <v>0</v>
+      </c>
+      <c r="S399" s="9">
+        <v>0</v>
+      </c>
+      <c r="T399" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U399" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V399" s="11">
+        <v>11</v>
+      </c>
+      <c r="W399" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X399" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y399" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB399" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG399" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI399" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ399" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK399" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM399" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR399" s="3" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="400" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A400" s="1">
+        <v>1</v>
+      </c>
+      <c r="B400" s="2">
+        <v>2</v>
+      </c>
+      <c r="C400" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D400" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E400" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F400" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G400" s="5">
+        <v>436</v>
+      </c>
+      <c r="H400" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I400" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J400" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K400" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L400" s="6">
+        <v>683</v>
+      </c>
+      <c r="M400" s="7">
+        <v>127735.07</v>
+      </c>
+      <c r="N400" s="6">
+        <v>1</v>
+      </c>
+      <c r="O400" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P400" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q400" s="6">
+        <v>0</v>
+      </c>
+      <c r="R400" s="7">
+        <v>0</v>
+      </c>
+      <c r="S400" s="9">
+        <v>0</v>
+      </c>
+      <c r="T400" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U400" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V400" s="11">
+        <v>11</v>
+      </c>
+      <c r="W400" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X400" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y400" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB400" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG400" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI400" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ400" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK400" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM400" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR400" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="401" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A401" s="1">
+        <v>1</v>
+      </c>
+      <c r="B401" s="2">
+        <v>2</v>
+      </c>
+      <c r="C401" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D401" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E401" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F401" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G401" s="5">
+        <v>437</v>
+      </c>
+      <c r="H401" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I401" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J401" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K401" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L401" s="6">
+        <v>684</v>
+      </c>
+      <c r="M401" s="7">
+        <v>127922.09</v>
+      </c>
+      <c r="N401" s="6">
+        <v>1</v>
+      </c>
+      <c r="O401" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P401" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q401" s="6">
+        <v>0</v>
+      </c>
+      <c r="R401" s="7">
+        <v>0</v>
+      </c>
+      <c r="S401" s="9">
+        <v>0</v>
+      </c>
+      <c r="T401" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U401" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V401" s="11">
+        <v>11</v>
+      </c>
+      <c r="W401" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X401" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y401" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB401" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG401" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI401" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ401" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK401" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM401" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR401" s="3" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="402" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A402" s="1">
+        <v>1</v>
+      </c>
+      <c r="B402" s="2">
+        <v>2</v>
+      </c>
+      <c r="C402" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D402" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E402" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F402" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G402" s="5">
+        <v>438</v>
+      </c>
+      <c r="H402" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I402" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J402" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K402" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L402" s="6">
+        <v>685</v>
+      </c>
+      <c r="M402" s="7">
+        <v>128109.11</v>
+      </c>
+      <c r="N402" s="6">
+        <v>1</v>
+      </c>
+      <c r="O402" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P402" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q402" s="6">
+        <v>0</v>
+      </c>
+      <c r="R402" s="7">
+        <v>0</v>
+      </c>
+      <c r="S402" s="9">
+        <v>0</v>
+      </c>
+      <c r="T402" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U402" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V402" s="11">
+        <v>11</v>
+      </c>
+      <c r="W402" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X402" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y402" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z402" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA402" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB402" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC402" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD402" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE402" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF402" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG402" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH402" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI402" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ402" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK402" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL402" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM402" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN402" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO402" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP402" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ402" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR402" s="3" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="403" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A403" s="1">
+        <v>1</v>
+      </c>
+      <c r="B403" s="2">
+        <v>2</v>
+      </c>
+      <c r="C403" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D403" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E403" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F403" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G403" s="5">
+        <v>439</v>
+      </c>
+      <c r="H403" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I403" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J403" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K403" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L403" s="6">
+        <v>686</v>
+      </c>
+      <c r="M403" s="7">
+        <v>128296.13</v>
+      </c>
+      <c r="N403" s="6">
+        <v>1</v>
+      </c>
+      <c r="O403" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P403" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q403" s="6">
+        <v>0</v>
+      </c>
+      <c r="R403" s="7">
+        <v>0</v>
+      </c>
+      <c r="S403" s="9">
+        <v>0</v>
+      </c>
+      <c r="T403" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U403" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V403" s="11">
+        <v>11</v>
+      </c>
+      <c r="W403" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X403" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y403" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z403" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA403" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB403" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC403" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD403" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE403" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF403" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG403" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH403" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI403" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ403" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK403" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL403" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM403" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN403" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO403" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP403" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ403" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR403" s="3" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="404" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A404" s="1">
+        <v>1</v>
+      </c>
+      <c r="B404" s="2">
+        <v>2</v>
+      </c>
+      <c r="C404" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D404" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E404" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F404" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G404" s="5">
+        <v>440</v>
+      </c>
+      <c r="H404" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I404" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J404" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K404" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L404" s="6">
+        <v>687</v>
+      </c>
+      <c r="M404" s="7">
+        <v>128483.15</v>
+      </c>
+      <c r="N404" s="6">
+        <v>1</v>
+      </c>
+      <c r="O404" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P404" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q404" s="6">
+        <v>0</v>
+      </c>
+      <c r="R404" s="7">
+        <v>0</v>
+      </c>
+      <c r="S404" s="9">
+        <v>0</v>
+      </c>
+      <c r="T404" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U404" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V404" s="11">
+        <v>11</v>
+      </c>
+      <c r="W404" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X404" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y404" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z404" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA404" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB404" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC404" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD404" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE404" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF404" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG404" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH404" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI404" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ404" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK404" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL404" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM404" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN404" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO404" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP404" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ404" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR404" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="405" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A405" s="1">
+        <v>1</v>
+      </c>
+      <c r="B405" s="2">
+        <v>2</v>
+      </c>
+      <c r="C405" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D405" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E405" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F405" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G405" s="5">
+        <v>441</v>
+      </c>
+      <c r="H405" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I405" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J405" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K405" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L405" s="6">
+        <v>688</v>
+      </c>
+      <c r="M405" s="7">
+        <v>128670.17</v>
+      </c>
+      <c r="N405" s="6">
+        <v>1</v>
+      </c>
+      <c r="O405" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P405" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q405" s="6">
+        <v>0</v>
+      </c>
+      <c r="R405" s="7">
+        <v>0</v>
+      </c>
+      <c r="S405" s="9">
+        <v>0</v>
+      </c>
+      <c r="T405" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U405" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V405" s="11">
+        <v>11</v>
+      </c>
+      <c r="W405" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X405" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y405" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z405" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA405" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB405" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC405" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD405" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE405" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF405" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG405" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH405" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI405" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ405" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK405" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL405" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM405" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN405" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO405" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP405" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ405" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR405" s="3" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="406" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A406" s="1">
+        <v>1</v>
+      </c>
+      <c r="B406" s="2">
+        <v>2</v>
+      </c>
+      <c r="C406" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D406" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E406" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F406" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G406" s="5">
+        <v>442</v>
+      </c>
+      <c r="H406" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I406" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J406" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K406" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L406" s="6">
+        <v>689</v>
+      </c>
+      <c r="M406" s="7">
+        <v>128857.2</v>
+      </c>
+      <c r="N406" s="6">
+        <v>1</v>
+      </c>
+      <c r="O406" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P406" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q406" s="6">
+        <v>0</v>
+      </c>
+      <c r="R406" s="7">
+        <v>0</v>
+      </c>
+      <c r="S406" s="9">
+        <v>0</v>
+      </c>
+      <c r="T406" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U406" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V406" s="11">
+        <v>11</v>
+      </c>
+      <c r="W406" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X406" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y406" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z406" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA406" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB406" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC406" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD406" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE406" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF406" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG406" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH406" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI406" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ406" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK406" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL406" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM406" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN406" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO406" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP406" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ406" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR406" s="3" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="407" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A407" s="1">
+        <v>1</v>
+      </c>
+      <c r="B407" s="2">
+        <v>2</v>
+      </c>
+      <c r="C407" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D407" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E407" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F407" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G407" s="5">
+        <v>443</v>
+      </c>
+      <c r="H407" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I407" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J407" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K407" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L407" s="6">
+        <v>690</v>
+      </c>
+      <c r="M407" s="7">
+        <v>129044.22</v>
+      </c>
+      <c r="N407" s="6">
+        <v>1</v>
+      </c>
+      <c r="O407" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P407" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q407" s="6">
+        <v>0</v>
+      </c>
+      <c r="R407" s="7">
+        <v>0</v>
+      </c>
+      <c r="S407" s="9">
+        <v>0</v>
+      </c>
+      <c r="T407" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U407" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V407" s="11">
+        <v>11</v>
+      </c>
+      <c r="W407" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X407" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y407" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z407" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA407" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB407" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC407" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD407" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE407" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF407" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG407" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH407" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI407" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ407" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK407" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL407" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM407" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN407" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO407" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP407" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ407" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR407" s="3" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="408" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A408" s="1">
+        <v>1</v>
+      </c>
+      <c r="B408" s="2">
+        <v>2</v>
+      </c>
+      <c r="C408" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D408" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E408" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F408" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G408" s="5">
+        <v>444</v>
+      </c>
+      <c r="H408" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I408" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J408" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K408" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L408" s="6">
+        <v>691</v>
+      </c>
+      <c r="M408" s="7">
+        <v>129231.24</v>
+      </c>
+      <c r="N408" s="6">
+        <v>1</v>
+      </c>
+      <c r="O408" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P408" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q408" s="6">
+        <v>0</v>
+      </c>
+      <c r="R408" s="7">
+        <v>0</v>
+      </c>
+      <c r="S408" s="9">
+        <v>0</v>
+      </c>
+      <c r="T408" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U408" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V408" s="11">
+        <v>11</v>
+      </c>
+      <c r="W408" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X408" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y408" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z408" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA408" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB408" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC408" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD408" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE408" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF408" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG408" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH408" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI408" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ408" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK408" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL408" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM408" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN408" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO408" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP408" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ408" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR408" s="3" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="409" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A409" s="1">
+        <v>1</v>
+      </c>
+      <c r="B409" s="2">
+        <v>2</v>
+      </c>
+      <c r="C409" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D409" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E409" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F409" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G409" s="5">
+        <v>445</v>
+      </c>
+      <c r="H409" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I409" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J409" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K409" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L409" s="6">
+        <v>692</v>
+      </c>
+      <c r="M409" s="7">
+        <v>129418.26</v>
+      </c>
+      <c r="N409" s="6">
+        <v>1</v>
+      </c>
+      <c r="O409" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P409" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q409" s="6">
+        <v>0</v>
+      </c>
+      <c r="R409" s="7">
+        <v>0</v>
+      </c>
+      <c r="S409" s="9">
+        <v>0</v>
+      </c>
+      <c r="T409" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U409" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V409" s="11">
+        <v>11</v>
+      </c>
+      <c r="W409" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X409" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y409" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z409" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA409" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB409" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC409" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD409" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE409" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF409" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG409" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH409" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI409" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ409" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK409" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL409" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM409" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN409" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO409" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP409" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ409" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR409" s="3" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="410" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A410" s="1">
+        <v>1</v>
+      </c>
+      <c r="B410" s="2">
+        <v>2</v>
+      </c>
+      <c r="C410" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D410" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E410" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F410" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G410" s="5">
+        <v>446</v>
+      </c>
+      <c r="H410" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I410" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J410" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K410" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L410" s="6">
+        <v>693</v>
+      </c>
+      <c r="M410" s="7">
+        <v>129605.28</v>
+      </c>
+      <c r="N410" s="6">
+        <v>1</v>
+      </c>
+      <c r="O410" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P410" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q410" s="6">
+        <v>0</v>
+      </c>
+      <c r="R410" s="7">
+        <v>0</v>
+      </c>
+      <c r="S410" s="9">
+        <v>0</v>
+      </c>
+      <c r="T410" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U410" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V410" s="11">
+        <v>11</v>
+      </c>
+      <c r="W410" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X410" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y410" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z410" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA410" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB410" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC410" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD410" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE410" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF410" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG410" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH410" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI410" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ410" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK410" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL410" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM410" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN410" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO410" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP410" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ410" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR410" s="3" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="411" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A411" s="1">
+        <v>1</v>
+      </c>
+      <c r="B411" s="2">
+        <v>2</v>
+      </c>
+      <c r="C411" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D411" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E411" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F411" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G411" s="5">
+        <v>447</v>
+      </c>
+      <c r="H411" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I411" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J411" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K411" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L411" s="6">
+        <v>694</v>
+      </c>
+      <c r="M411" s="7">
+        <v>129792.3</v>
+      </c>
+      <c r="N411" s="6">
+        <v>1</v>
+      </c>
+      <c r="O411" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P411" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q411" s="6">
+        <v>0</v>
+      </c>
+      <c r="R411" s="7">
+        <v>0</v>
+      </c>
+      <c r="S411" s="9">
+        <v>0</v>
+      </c>
+      <c r="T411" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U411" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V411" s="11">
+        <v>11</v>
+      </c>
+      <c r="W411" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X411" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y411" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z411" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA411" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB411" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC411" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD411" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE411" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG411" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI411" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ411" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK411" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL411" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM411" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ411" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR411" s="3" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="412" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A412" s="1">
+        <v>1</v>
+      </c>
+      <c r="B412" s="2">
+        <v>2</v>
+      </c>
+      <c r="C412" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D412" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E412" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F412" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G412" s="5">
+        <v>448</v>
+      </c>
+      <c r="H412" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I412" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J412" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K412" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L412" s="6">
+        <v>695</v>
+      </c>
+      <c r="M412" s="7">
+        <v>129979.32</v>
+      </c>
+      <c r="N412" s="6">
+        <v>1</v>
+      </c>
+      <c r="O412" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P412" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q412" s="6">
+        <v>0</v>
+      </c>
+      <c r="R412" s="7">
+        <v>0</v>
+      </c>
+      <c r="S412" s="9">
+        <v>0</v>
+      </c>
+      <c r="T412" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U412" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V412" s="11">
+        <v>11</v>
+      </c>
+      <c r="W412" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X412" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y412" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z412" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA412" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB412" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC412" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD412" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE412" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF412" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG412" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH412" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI412" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ412" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK412" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL412" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM412" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN412" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO412" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP412" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ412" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR412" s="3" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="413" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A413" s="1">
+        <v>1</v>
+      </c>
+      <c r="B413" s="2">
+        <v>2</v>
+      </c>
+      <c r="C413" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D413" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E413" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F413" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G413" s="5">
+        <v>449</v>
+      </c>
+      <c r="H413" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I413" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J413" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K413" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L413" s="6">
+        <v>696</v>
+      </c>
+      <c r="M413" s="7">
+        <v>130166.34</v>
+      </c>
+      <c r="N413" s="6">
+        <v>1</v>
+      </c>
+      <c r="O413" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P413" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q413" s="6">
+        <v>0</v>
+      </c>
+      <c r="R413" s="7">
+        <v>0</v>
+      </c>
+      <c r="S413" s="9">
+        <v>0</v>
+      </c>
+      <c r="T413" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U413" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V413" s="11">
+        <v>11</v>
+      </c>
+      <c r="W413" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X413" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y413" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z413" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA413" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB413" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC413" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD413" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE413" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF413" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG413" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH413" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI413" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ413" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK413" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL413" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM413" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN413" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO413" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP413" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ413" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR413" s="3" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="414" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A414" s="1">
+        <v>1</v>
+      </c>
+      <c r="B414" s="2">
+        <v>2</v>
+      </c>
+      <c r="C414" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D414" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E414" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F414" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G414" s="5">
+        <v>450</v>
+      </c>
+      <c r="H414" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I414" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J414" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K414" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L414" s="6">
+        <v>697</v>
+      </c>
+      <c r="M414" s="7">
+        <v>130353.36</v>
+      </c>
+      <c r="N414" s="6">
+        <v>1</v>
+      </c>
+      <c r="O414" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P414" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q414" s="6">
+        <v>0</v>
+      </c>
+      <c r="R414" s="7">
+        <v>0</v>
+      </c>
+      <c r="S414" s="9">
+        <v>0</v>
+      </c>
+      <c r="T414" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U414" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V414" s="11">
+        <v>11</v>
+      </c>
+      <c r="W414" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X414" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y414" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z414" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA414" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB414" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC414" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD414" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE414" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF414" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG414" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH414" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI414" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ414" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK414" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL414" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM414" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN414" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO414" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP414" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ414" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR414" s="3" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="415" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A415" s="1">
+        <v>1</v>
+      </c>
+      <c r="B415" s="2">
+        <v>2</v>
+      </c>
+      <c r="C415" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D415" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E415" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F415" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G415" s="5">
+        <v>451</v>
+      </c>
+      <c r="H415" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I415" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J415" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K415" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L415" s="6">
+        <v>698</v>
+      </c>
+      <c r="M415" s="7">
+        <v>130540.38</v>
+      </c>
+      <c r="N415" s="6">
+        <v>1</v>
+      </c>
+      <c r="O415" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P415" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q415" s="6">
+        <v>0</v>
+      </c>
+      <c r="R415" s="7">
+        <v>0</v>
+      </c>
+      <c r="S415" s="9">
+        <v>0</v>
+      </c>
+      <c r="T415" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U415" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V415" s="11">
+        <v>11</v>
+      </c>
+      <c r="W415" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X415" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y415" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z415" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA415" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB415" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC415" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD415" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE415" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF415" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG415" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH415" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI415" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ415" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK415" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL415" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM415" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN415" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO415" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP415" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ415" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR415" s="3" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="416" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A416" s="1">
+        <v>1</v>
+      </c>
+      <c r="B416" s="2">
+        <v>2</v>
+      </c>
+      <c r="C416" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D416" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E416" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F416" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G416" s="5">
+        <v>452</v>
+      </c>
+      <c r="H416" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I416" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J416" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K416" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L416" s="6">
+        <v>699</v>
+      </c>
+      <c r="M416" s="7">
+        <v>130727.4</v>
+      </c>
+      <c r="N416" s="6">
+        <v>1</v>
+      </c>
+      <c r="O416" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P416" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q416" s="6">
+        <v>0</v>
+      </c>
+      <c r="R416" s="7">
+        <v>0</v>
+      </c>
+      <c r="S416" s="9">
+        <v>0</v>
+      </c>
+      <c r="T416" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U416" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V416" s="11">
+        <v>11</v>
+      </c>
+      <c r="W416" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X416" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y416" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z416" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA416" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB416" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC416" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD416" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE416" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF416" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG416" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH416" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI416" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ416" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK416" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL416" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM416" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN416" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO416" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP416" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ416" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR416" s="3" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="417" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A417" s="1">
+        <v>1</v>
+      </c>
+      <c r="B417" s="2">
+        <v>2</v>
+      </c>
+      <c r="C417" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D417" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E417" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F417" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G417" s="5">
+        <v>453</v>
+      </c>
+      <c r="H417" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I417" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J417" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K417" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L417" s="6">
+        <v>700</v>
+      </c>
+      <c r="M417" s="7">
+        <v>130914.42</v>
+      </c>
+      <c r="N417" s="6">
+        <v>1</v>
+      </c>
+      <c r="O417" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P417" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q417" s="6">
+        <v>0</v>
+      </c>
+      <c r="R417" s="7">
+        <v>0</v>
+      </c>
+      <c r="S417" s="9">
+        <v>0</v>
+      </c>
+      <c r="T417" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U417" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V417" s="11">
+        <v>11</v>
+      </c>
+      <c r="W417" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X417" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y417" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z417" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA417" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB417" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC417" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD417" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE417" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF417" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG417" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH417" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI417" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ417" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK417" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL417" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM417" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN417" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO417" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP417" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ417" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR417" s="3" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="418" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A418" s="1">
+        <v>1</v>
+      </c>
+      <c r="B418" s="2">
+        <v>2</v>
+      </c>
+      <c r="C418" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D418" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E418" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F418" s="4">
+        <v>46146</v>
+      </c>
+      <c r="G418" s="5">
+        <v>454</v>
+      </c>
+      <c r="H418" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I418" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J418" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K418" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L418" s="6">
+        <v>701</v>
+      </c>
+      <c r="M418" s="7">
+        <v>131101.44</v>
+      </c>
+      <c r="N418" s="6">
+        <v>1</v>
+      </c>
+      <c r="O418" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P418" s="8">
+        <v>187.02</v>
+      </c>
+      <c r="Q418" s="6">
+        <v>0</v>
+      </c>
+      <c r="R418" s="7">
+        <v>0</v>
+      </c>
+      <c r="S418" s="9">
+        <v>0</v>
+      </c>
+      <c r="T418" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U418" s="10">
+        <v>64095</v>
+      </c>
+      <c r="V418" s="11">
+        <v>11</v>
+      </c>
+      <c r="W418" s="4">
+        <v>46146</v>
+      </c>
+      <c r="X418" s="12">
+        <v>0.69166669999999997</v>
+      </c>
+      <c r="Y418" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z418" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA418" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB418" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC418" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD418" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE418" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF418" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG418" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH418" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI418" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ418" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK418" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL418" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM418" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN418" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO418" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP418" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ418" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR418" s="3" t="s">
+        <v>471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 05/05/2026 13:30:36,93
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A83C9D5-D9EC-4281-BC6B-47A50662D122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{132C81BC-72A2-4260-BA23-CB92AD50750D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4292" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4400" uniqueCount="297">
   <si>
     <t>Sel</t>
   </si>
@@ -894,6 +894,24 @@
   <si>
     <t>1854300114193</t>
   </si>
+  <si>
+    <t>1854300114194</t>
+  </si>
+  <si>
+    <t>1854300114195</t>
+  </si>
+  <si>
+    <t>1854300114196</t>
+  </si>
+  <si>
+    <t>1854300114197</t>
+  </si>
+  <si>
+    <t>1854300114198</t>
+  </si>
+  <si>
+    <t>1854300114199</t>
+  </si>
 </sst>
 </file>
 
@@ -1468,7 +1486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR237"/>
+  <dimension ref="A1:AR243"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -33227,6 +33245,810 @@
       </c>
       <c r="AR237" s="3" t="s">
         <v>290</v>
+      </c>
+    </row>
+    <row r="238" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A238" s="1">
+        <v>1</v>
+      </c>
+      <c r="B238" s="2">
+        <v>2</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D238" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E238" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F238" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G238" s="5">
+        <v>262</v>
+      </c>
+      <c r="H238" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I238" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J238" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K238" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L238" s="6">
+        <v>549</v>
+      </c>
+      <c r="M238" s="7">
+        <v>108055.72</v>
+      </c>
+      <c r="N238" s="6">
+        <v>1</v>
+      </c>
+      <c r="O238" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P238" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q238" s="6">
+        <v>0</v>
+      </c>
+      <c r="R238" s="7">
+        <v>0</v>
+      </c>
+      <c r="S238" s="9">
+        <v>0</v>
+      </c>
+      <c r="T238" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U238" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V238" s="11">
+        <v>11</v>
+      </c>
+      <c r="W238" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X238" s="12">
+        <v>0.54652780000000001</v>
+      </c>
+      <c r="Y238" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z238" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA238" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB238" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC238" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD238" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE238" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF238" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG238" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH238" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI238" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ238" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK238" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL238" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM238" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN238" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO238" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP238" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ238" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR238" s="3" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="239" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A239" s="1">
+        <v>1</v>
+      </c>
+      <c r="B239" s="2">
+        <v>2</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D239" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E239" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F239" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G239" s="5">
+        <v>263</v>
+      </c>
+      <c r="H239" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I239" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J239" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K239" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L239" s="6">
+        <v>550</v>
+      </c>
+      <c r="M239" s="7">
+        <v>108252.54</v>
+      </c>
+      <c r="N239" s="6">
+        <v>1</v>
+      </c>
+      <c r="O239" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P239" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q239" s="6">
+        <v>0</v>
+      </c>
+      <c r="R239" s="7">
+        <v>0</v>
+      </c>
+      <c r="S239" s="9">
+        <v>0</v>
+      </c>
+      <c r="T239" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U239" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V239" s="11">
+        <v>11</v>
+      </c>
+      <c r="W239" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X239" s="12">
+        <v>0.54652780000000001</v>
+      </c>
+      <c r="Y239" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z239" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA239" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB239" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC239" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD239" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE239" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF239" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG239" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH239" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI239" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ239" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK239" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL239" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM239" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN239" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO239" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP239" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ239" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR239" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="240" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A240" s="1">
+        <v>1</v>
+      </c>
+      <c r="B240" s="2">
+        <v>2</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D240" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E240" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F240" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G240" s="5">
+        <v>264</v>
+      </c>
+      <c r="H240" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I240" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J240" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K240" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L240" s="6">
+        <v>551</v>
+      </c>
+      <c r="M240" s="7">
+        <v>108449.37</v>
+      </c>
+      <c r="N240" s="6">
+        <v>1</v>
+      </c>
+      <c r="O240" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P240" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q240" s="6">
+        <v>0</v>
+      </c>
+      <c r="R240" s="7">
+        <v>0</v>
+      </c>
+      <c r="S240" s="9">
+        <v>0</v>
+      </c>
+      <c r="T240" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U240" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V240" s="11">
+        <v>11</v>
+      </c>
+      <c r="W240" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X240" s="12">
+        <v>0.54652780000000001</v>
+      </c>
+      <c r="Y240" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB240" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG240" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI240" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ240" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK240" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM240" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR240" s="3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="241" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A241" s="1">
+        <v>1</v>
+      </c>
+      <c r="B241" s="2">
+        <v>2</v>
+      </c>
+      <c r="C241" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D241" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E241" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F241" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G241" s="5">
+        <v>265</v>
+      </c>
+      <c r="H241" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I241" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J241" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K241" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L241" s="6">
+        <v>552</v>
+      </c>
+      <c r="M241" s="7">
+        <v>108646.19</v>
+      </c>
+      <c r="N241" s="6">
+        <v>1</v>
+      </c>
+      <c r="O241" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P241" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q241" s="6">
+        <v>0</v>
+      </c>
+      <c r="R241" s="7">
+        <v>0</v>
+      </c>
+      <c r="S241" s="9">
+        <v>0</v>
+      </c>
+      <c r="T241" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U241" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V241" s="11">
+        <v>11</v>
+      </c>
+      <c r="W241" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X241" s="12">
+        <v>0.54652780000000001</v>
+      </c>
+      <c r="Y241" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB241" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG241" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI241" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ241" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK241" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM241" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR241" s="3" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="242" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A242" s="1">
+        <v>1</v>
+      </c>
+      <c r="B242" s="2">
+        <v>2</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E242" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F242" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G242" s="5">
+        <v>266</v>
+      </c>
+      <c r="H242" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I242" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J242" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K242" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L242" s="6">
+        <v>553</v>
+      </c>
+      <c r="M242" s="7">
+        <v>108843.01</v>
+      </c>
+      <c r="N242" s="6">
+        <v>1</v>
+      </c>
+      <c r="O242" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P242" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q242" s="6">
+        <v>0</v>
+      </c>
+      <c r="R242" s="7">
+        <v>0</v>
+      </c>
+      <c r="S242" s="9">
+        <v>0</v>
+      </c>
+      <c r="T242" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U242" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V242" s="11">
+        <v>11</v>
+      </c>
+      <c r="W242" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X242" s="12">
+        <v>0.54652780000000001</v>
+      </c>
+      <c r="Y242" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB242" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG242" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI242" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ242" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK242" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM242" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR242" s="3" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="243" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A243" s="1">
+        <v>1</v>
+      </c>
+      <c r="B243" s="2">
+        <v>2</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D243" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E243" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F243" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G243" s="5">
+        <v>267</v>
+      </c>
+      <c r="H243" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I243" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J243" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K243" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L243" s="6">
+        <v>554</v>
+      </c>
+      <c r="M243" s="7">
+        <v>109039.83</v>
+      </c>
+      <c r="N243" s="6">
+        <v>1</v>
+      </c>
+      <c r="O243" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P243" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q243" s="6">
+        <v>0</v>
+      </c>
+      <c r="R243" s="7">
+        <v>0</v>
+      </c>
+      <c r="S243" s="9">
+        <v>0</v>
+      </c>
+      <c r="T243" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U243" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V243" s="11">
+        <v>11</v>
+      </c>
+      <c r="W243" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X243" s="12">
+        <v>0.54652780000000001</v>
+      </c>
+      <c r="Y243" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB243" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG243" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI243" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ243" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK243" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM243" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR243" s="3" t="s">
+        <v>296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 05/05/2026 14:04:29,17
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{132C81BC-72A2-4260-BA23-CB92AD50750D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B50ACE2-8DDE-4CEF-B052-CDD001BCB83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4400" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4814" uniqueCount="320">
   <si>
     <t>Sel</t>
   </si>
@@ -912,6 +912,75 @@
   <si>
     <t>1854300114199</t>
   </si>
+  <si>
+    <t>1854300114200</t>
+  </si>
+  <si>
+    <t>1854300114201</t>
+  </si>
+  <si>
+    <t>1854300114202</t>
+  </si>
+  <si>
+    <t>1854300114203</t>
+  </si>
+  <si>
+    <t>1854300114204</t>
+  </si>
+  <si>
+    <t>1854300114205</t>
+  </si>
+  <si>
+    <t>1854300114206</t>
+  </si>
+  <si>
+    <t>1854300114207</t>
+  </si>
+  <si>
+    <t>1854300114208</t>
+  </si>
+  <si>
+    <t>1854300114209</t>
+  </si>
+  <si>
+    <t>1854300114212</t>
+  </si>
+  <si>
+    <t>1854300114210</t>
+  </si>
+  <si>
+    <t>1854300114211</t>
+  </si>
+  <si>
+    <t>1854300114213</t>
+  </si>
+  <si>
+    <t>1854300114214</t>
+  </si>
+  <si>
+    <t>1854300114215</t>
+  </si>
+  <si>
+    <t>1854300114216</t>
+  </si>
+  <si>
+    <t>1854300114217</t>
+  </si>
+  <si>
+    <t>1854300114218</t>
+  </si>
+  <si>
+    <t>1854300114219</t>
+  </si>
+  <si>
+    <t>1854300114220</t>
+  </si>
+  <si>
+    <t>1854300114221</t>
+  </si>
+  <si>
+    <t>1854300114222</t>
+  </si>
 </sst>
 </file>
 
@@ -1486,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR243"/>
+  <dimension ref="A1:AR266"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -34049,6 +34118,3088 @@
       </c>
       <c r="AR243" s="3" t="s">
         <v>296</v>
+      </c>
+    </row>
+    <row r="244" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A244" s="1">
+        <v>1</v>
+      </c>
+      <c r="B244" s="2">
+        <v>2</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D244" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E244" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F244" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G244" s="5">
+        <v>268</v>
+      </c>
+      <c r="H244" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I244" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J244" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K244" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L244" s="6">
+        <v>555</v>
+      </c>
+      <c r="M244" s="7">
+        <v>109236.66</v>
+      </c>
+      <c r="N244" s="6">
+        <v>1</v>
+      </c>
+      <c r="O244" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P244" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q244" s="6">
+        <v>0</v>
+      </c>
+      <c r="R244" s="7">
+        <v>0</v>
+      </c>
+      <c r="S244" s="9">
+        <v>0</v>
+      </c>
+      <c r="T244" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U244" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V244" s="11">
+        <v>11</v>
+      </c>
+      <c r="W244" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X244" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y244" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB244" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG244" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI244" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ244" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK244" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM244" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR244" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="245" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A245" s="1">
+        <v>1</v>
+      </c>
+      <c r="B245" s="2">
+        <v>2</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D245" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E245" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F245" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G245" s="5">
+        <v>269</v>
+      </c>
+      <c r="H245" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I245" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J245" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K245" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L245" s="6">
+        <v>556</v>
+      </c>
+      <c r="M245" s="7">
+        <v>109433.48</v>
+      </c>
+      <c r="N245" s="6">
+        <v>1</v>
+      </c>
+      <c r="O245" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P245" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q245" s="6">
+        <v>0</v>
+      </c>
+      <c r="R245" s="7">
+        <v>0</v>
+      </c>
+      <c r="S245" s="9">
+        <v>0</v>
+      </c>
+      <c r="T245" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U245" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V245" s="11">
+        <v>11</v>
+      </c>
+      <c r="W245" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X245" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y245" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB245" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG245" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI245" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ245" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK245" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM245" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR245" s="3" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="246" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A246" s="1">
+        <v>1</v>
+      </c>
+      <c r="B246" s="2">
+        <v>2</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D246" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E246" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F246" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G246" s="5">
+        <v>270</v>
+      </c>
+      <c r="H246" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I246" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J246" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K246" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L246" s="6">
+        <v>557</v>
+      </c>
+      <c r="M246" s="7">
+        <v>109630.3</v>
+      </c>
+      <c r="N246" s="6">
+        <v>1</v>
+      </c>
+      <c r="O246" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P246" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q246" s="6">
+        <v>0</v>
+      </c>
+      <c r="R246" s="7">
+        <v>0</v>
+      </c>
+      <c r="S246" s="9">
+        <v>0</v>
+      </c>
+      <c r="T246" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U246" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V246" s="11">
+        <v>11</v>
+      </c>
+      <c r="W246" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X246" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y246" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB246" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG246" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI246" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ246" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK246" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM246" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR246" s="3" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="247" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A247" s="1">
+        <v>1</v>
+      </c>
+      <c r="B247" s="2">
+        <v>2</v>
+      </c>
+      <c r="C247" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D247" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E247" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F247" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G247" s="5">
+        <v>271</v>
+      </c>
+      <c r="H247" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I247" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J247" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K247" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L247" s="6">
+        <v>558</v>
+      </c>
+      <c r="M247" s="7">
+        <v>109827.13</v>
+      </c>
+      <c r="N247" s="6">
+        <v>1</v>
+      </c>
+      <c r="O247" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P247" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q247" s="6">
+        <v>0</v>
+      </c>
+      <c r="R247" s="7">
+        <v>0</v>
+      </c>
+      <c r="S247" s="9">
+        <v>0</v>
+      </c>
+      <c r="T247" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U247" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V247" s="11">
+        <v>11</v>
+      </c>
+      <c r="W247" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X247" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y247" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB247" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG247" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI247" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ247" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK247" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM247" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR247" s="3" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="248" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A248" s="1">
+        <v>1</v>
+      </c>
+      <c r="B248" s="2">
+        <v>2</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E248" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F248" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G248" s="5">
+        <v>272</v>
+      </c>
+      <c r="H248" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I248" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J248" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K248" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L248" s="6">
+        <v>559</v>
+      </c>
+      <c r="M248" s="7">
+        <v>110023.95</v>
+      </c>
+      <c r="N248" s="6">
+        <v>1</v>
+      </c>
+      <c r="O248" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P248" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q248" s="6">
+        <v>0</v>
+      </c>
+      <c r="R248" s="7">
+        <v>0</v>
+      </c>
+      <c r="S248" s="9">
+        <v>0</v>
+      </c>
+      <c r="T248" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U248" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V248" s="11">
+        <v>11</v>
+      </c>
+      <c r="W248" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X248" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y248" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB248" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG248" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI248" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ248" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK248" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM248" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR248" s="3" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="249" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A249" s="1">
+        <v>1</v>
+      </c>
+      <c r="B249" s="2">
+        <v>2</v>
+      </c>
+      <c r="C249" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D249" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E249" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F249" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G249" s="5">
+        <v>273</v>
+      </c>
+      <c r="H249" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I249" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J249" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K249" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L249" s="6">
+        <v>560</v>
+      </c>
+      <c r="M249" s="7">
+        <v>110220.77</v>
+      </c>
+      <c r="N249" s="6">
+        <v>1</v>
+      </c>
+      <c r="O249" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P249" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q249" s="6">
+        <v>0</v>
+      </c>
+      <c r="R249" s="7">
+        <v>0</v>
+      </c>
+      <c r="S249" s="9">
+        <v>0</v>
+      </c>
+      <c r="T249" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U249" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V249" s="11">
+        <v>11</v>
+      </c>
+      <c r="W249" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X249" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y249" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB249" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG249" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI249" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ249" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK249" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM249" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR249" s="3" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="250" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A250" s="1">
+        <v>1</v>
+      </c>
+      <c r="B250" s="2">
+        <v>2</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E250" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F250" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G250" s="5">
+        <v>274</v>
+      </c>
+      <c r="H250" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I250" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J250" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K250" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L250" s="6">
+        <v>561</v>
+      </c>
+      <c r="M250" s="7">
+        <v>110417.59</v>
+      </c>
+      <c r="N250" s="6">
+        <v>1</v>
+      </c>
+      <c r="O250" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P250" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q250" s="6">
+        <v>0</v>
+      </c>
+      <c r="R250" s="7">
+        <v>0</v>
+      </c>
+      <c r="S250" s="9">
+        <v>0</v>
+      </c>
+      <c r="T250" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U250" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V250" s="11">
+        <v>11</v>
+      </c>
+      <c r="W250" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X250" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y250" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB250" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG250" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI250" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ250" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK250" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM250" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR250" s="3" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="251" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A251" s="1">
+        <v>1</v>
+      </c>
+      <c r="B251" s="2">
+        <v>2</v>
+      </c>
+      <c r="C251" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D251" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E251" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F251" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G251" s="5">
+        <v>275</v>
+      </c>
+      <c r="H251" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I251" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J251" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K251" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L251" s="6">
+        <v>562</v>
+      </c>
+      <c r="M251" s="7">
+        <v>110614.42</v>
+      </c>
+      <c r="N251" s="6">
+        <v>1</v>
+      </c>
+      <c r="O251" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P251" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q251" s="6">
+        <v>0</v>
+      </c>
+      <c r="R251" s="7">
+        <v>0</v>
+      </c>
+      <c r="S251" s="9">
+        <v>0</v>
+      </c>
+      <c r="T251" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U251" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V251" s="11">
+        <v>11</v>
+      </c>
+      <c r="W251" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X251" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y251" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB251" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG251" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI251" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ251" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK251" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM251" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR251" s="3" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="252" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A252" s="1">
+        <v>1</v>
+      </c>
+      <c r="B252" s="2">
+        <v>2</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E252" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F252" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G252" s="5">
+        <v>276</v>
+      </c>
+      <c r="H252" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I252" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J252" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K252" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L252" s="6">
+        <v>563</v>
+      </c>
+      <c r="M252" s="7">
+        <v>110811.24</v>
+      </c>
+      <c r="N252" s="6">
+        <v>1</v>
+      </c>
+      <c r="O252" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P252" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q252" s="6">
+        <v>0</v>
+      </c>
+      <c r="R252" s="7">
+        <v>0</v>
+      </c>
+      <c r="S252" s="9">
+        <v>0</v>
+      </c>
+      <c r="T252" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U252" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V252" s="11">
+        <v>11</v>
+      </c>
+      <c r="W252" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X252" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y252" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB252" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG252" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI252" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ252" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK252" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM252" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR252" s="3" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="253" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A253" s="1">
+        <v>1</v>
+      </c>
+      <c r="B253" s="2">
+        <v>2</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D253" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E253" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F253" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G253" s="5">
+        <v>277</v>
+      </c>
+      <c r="H253" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I253" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J253" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K253" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L253" s="6">
+        <v>564</v>
+      </c>
+      <c r="M253" s="7">
+        <v>111008.06</v>
+      </c>
+      <c r="N253" s="6">
+        <v>1</v>
+      </c>
+      <c r="O253" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P253" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q253" s="6">
+        <v>0</v>
+      </c>
+      <c r="R253" s="7">
+        <v>0</v>
+      </c>
+      <c r="S253" s="9">
+        <v>0</v>
+      </c>
+      <c r="T253" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U253" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V253" s="11">
+        <v>11</v>
+      </c>
+      <c r="W253" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X253" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y253" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB253" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG253" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI253" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ253" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK253" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM253" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR253" s="3" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="254" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A254" s="1">
+        <v>1</v>
+      </c>
+      <c r="B254" s="2">
+        <v>2</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D254" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E254" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F254" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G254" s="5">
+        <v>278</v>
+      </c>
+      <c r="H254" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I254" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J254" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K254" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L254" s="6">
+        <v>565</v>
+      </c>
+      <c r="M254" s="7">
+        <v>111204.88</v>
+      </c>
+      <c r="N254" s="6">
+        <v>1</v>
+      </c>
+      <c r="O254" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P254" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q254" s="6">
+        <v>0</v>
+      </c>
+      <c r="R254" s="7">
+        <v>0</v>
+      </c>
+      <c r="S254" s="9">
+        <v>0</v>
+      </c>
+      <c r="T254" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U254" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V254" s="11">
+        <v>11</v>
+      </c>
+      <c r="W254" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X254" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y254" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB254" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG254" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI254" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ254" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK254" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM254" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR254" s="3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="255" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A255" s="1">
+        <v>1</v>
+      </c>
+      <c r="B255" s="2">
+        <v>2</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D255" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E255" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F255" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G255" s="5">
+        <v>279</v>
+      </c>
+      <c r="H255" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I255" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J255" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K255" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L255" s="6">
+        <v>566</v>
+      </c>
+      <c r="M255" s="7">
+        <v>111401.71</v>
+      </c>
+      <c r="N255" s="6">
+        <v>1</v>
+      </c>
+      <c r="O255" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P255" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q255" s="6">
+        <v>0</v>
+      </c>
+      <c r="R255" s="7">
+        <v>0</v>
+      </c>
+      <c r="S255" s="9">
+        <v>0</v>
+      </c>
+      <c r="T255" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U255" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V255" s="11">
+        <v>11</v>
+      </c>
+      <c r="W255" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X255" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y255" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB255" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG255" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI255" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ255" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK255" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM255" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR255" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="256" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A256" s="1">
+        <v>1</v>
+      </c>
+      <c r="B256" s="2">
+        <v>2</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D256" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E256" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F256" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G256" s="5">
+        <v>280</v>
+      </c>
+      <c r="H256" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I256" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J256" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K256" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L256" s="6">
+        <v>567</v>
+      </c>
+      <c r="M256" s="7">
+        <v>111598.53</v>
+      </c>
+      <c r="N256" s="6">
+        <v>1</v>
+      </c>
+      <c r="O256" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P256" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q256" s="6">
+        <v>0</v>
+      </c>
+      <c r="R256" s="7">
+        <v>0</v>
+      </c>
+      <c r="S256" s="9">
+        <v>0</v>
+      </c>
+      <c r="T256" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U256" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V256" s="11">
+        <v>11</v>
+      </c>
+      <c r="W256" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X256" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y256" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB256" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG256" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI256" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ256" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK256" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM256" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR256" s="3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="257" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A257" s="1">
+        <v>1</v>
+      </c>
+      <c r="B257" s="2">
+        <v>2</v>
+      </c>
+      <c r="C257" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D257" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E257" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F257" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G257" s="5">
+        <v>281</v>
+      </c>
+      <c r="H257" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I257" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J257" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K257" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L257" s="6">
+        <v>568</v>
+      </c>
+      <c r="M257" s="7">
+        <v>111795.35</v>
+      </c>
+      <c r="N257" s="6">
+        <v>1</v>
+      </c>
+      <c r="O257" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P257" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q257" s="6">
+        <v>0</v>
+      </c>
+      <c r="R257" s="7">
+        <v>0</v>
+      </c>
+      <c r="S257" s="9">
+        <v>0</v>
+      </c>
+      <c r="T257" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U257" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V257" s="11">
+        <v>11</v>
+      </c>
+      <c r="W257" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X257" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y257" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB257" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG257" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI257" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ257" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK257" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM257" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR257" s="3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="258" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A258" s="1">
+        <v>1</v>
+      </c>
+      <c r="B258" s="2">
+        <v>2</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D258" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E258" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F258" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G258" s="5">
+        <v>282</v>
+      </c>
+      <c r="H258" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I258" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J258" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K258" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L258" s="6">
+        <v>569</v>
+      </c>
+      <c r="M258" s="7">
+        <v>111992.18</v>
+      </c>
+      <c r="N258" s="6">
+        <v>1</v>
+      </c>
+      <c r="O258" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P258" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q258" s="6">
+        <v>0</v>
+      </c>
+      <c r="R258" s="7">
+        <v>0</v>
+      </c>
+      <c r="S258" s="9">
+        <v>0</v>
+      </c>
+      <c r="T258" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U258" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V258" s="11">
+        <v>11</v>
+      </c>
+      <c r="W258" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X258" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y258" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB258" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG258" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI258" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ258" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK258" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM258" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR258" s="3" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="259" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A259" s="1">
+        <v>1</v>
+      </c>
+      <c r="B259" s="2">
+        <v>2</v>
+      </c>
+      <c r="C259" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D259" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E259" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F259" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G259" s="5">
+        <v>283</v>
+      </c>
+      <c r="H259" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I259" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J259" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K259" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L259" s="6">
+        <v>570</v>
+      </c>
+      <c r="M259" s="7">
+        <v>112189</v>
+      </c>
+      <c r="N259" s="6">
+        <v>1</v>
+      </c>
+      <c r="O259" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P259" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q259" s="6">
+        <v>0</v>
+      </c>
+      <c r="R259" s="7">
+        <v>0</v>
+      </c>
+      <c r="S259" s="9">
+        <v>0</v>
+      </c>
+      <c r="T259" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U259" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V259" s="11">
+        <v>11</v>
+      </c>
+      <c r="W259" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X259" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y259" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB259" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG259" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI259" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ259" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK259" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM259" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR259" s="3" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="260" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A260" s="1">
+        <v>1</v>
+      </c>
+      <c r="B260" s="2">
+        <v>2</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E260" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F260" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G260" s="5">
+        <v>284</v>
+      </c>
+      <c r="H260" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I260" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J260" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K260" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L260" s="6">
+        <v>571</v>
+      </c>
+      <c r="M260" s="7">
+        <v>112385.82</v>
+      </c>
+      <c r="N260" s="6">
+        <v>1</v>
+      </c>
+      <c r="O260" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P260" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q260" s="6">
+        <v>0</v>
+      </c>
+      <c r="R260" s="7">
+        <v>0</v>
+      </c>
+      <c r="S260" s="9">
+        <v>0</v>
+      </c>
+      <c r="T260" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U260" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V260" s="11">
+        <v>11</v>
+      </c>
+      <c r="W260" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X260" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y260" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB260" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG260" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI260" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ260" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK260" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM260" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR260" s="3" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="261" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A261" s="1">
+        <v>1</v>
+      </c>
+      <c r="B261" s="2">
+        <v>2</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D261" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E261" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F261" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G261" s="5">
+        <v>285</v>
+      </c>
+      <c r="H261" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I261" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J261" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K261" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L261" s="6">
+        <v>572</v>
+      </c>
+      <c r="M261" s="7">
+        <v>112582.64</v>
+      </c>
+      <c r="N261" s="6">
+        <v>1</v>
+      </c>
+      <c r="O261" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P261" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q261" s="6">
+        <v>0</v>
+      </c>
+      <c r="R261" s="7">
+        <v>0</v>
+      </c>
+      <c r="S261" s="9">
+        <v>0</v>
+      </c>
+      <c r="T261" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U261" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V261" s="11">
+        <v>11</v>
+      </c>
+      <c r="W261" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X261" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y261" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB261" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG261" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI261" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ261" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK261" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM261" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR261" s="3" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="262" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A262" s="1">
+        <v>1</v>
+      </c>
+      <c r="B262" s="2">
+        <v>2</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D262" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F262" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G262" s="5">
+        <v>286</v>
+      </c>
+      <c r="H262" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I262" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J262" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K262" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L262" s="6">
+        <v>573</v>
+      </c>
+      <c r="M262" s="7">
+        <v>112779.47</v>
+      </c>
+      <c r="N262" s="6">
+        <v>1</v>
+      </c>
+      <c r="O262" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P262" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q262" s="6">
+        <v>0</v>
+      </c>
+      <c r="R262" s="7">
+        <v>0</v>
+      </c>
+      <c r="S262" s="9">
+        <v>0</v>
+      </c>
+      <c r="T262" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U262" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V262" s="11">
+        <v>11</v>
+      </c>
+      <c r="W262" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X262" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y262" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB262" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG262" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI262" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ262" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK262" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM262" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR262" s="3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="263" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A263" s="1">
+        <v>1</v>
+      </c>
+      <c r="B263" s="2">
+        <v>2</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D263" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E263" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F263" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G263" s="5">
+        <v>287</v>
+      </c>
+      <c r="H263" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I263" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J263" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K263" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L263" s="6">
+        <v>574</v>
+      </c>
+      <c r="M263" s="7">
+        <v>112976.29</v>
+      </c>
+      <c r="N263" s="6">
+        <v>1</v>
+      </c>
+      <c r="O263" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P263" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q263" s="6">
+        <v>0</v>
+      </c>
+      <c r="R263" s="7">
+        <v>0</v>
+      </c>
+      <c r="S263" s="9">
+        <v>0</v>
+      </c>
+      <c r="T263" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U263" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V263" s="11">
+        <v>11</v>
+      </c>
+      <c r="W263" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X263" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y263" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB263" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG263" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI263" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ263" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK263" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM263" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR263" s="3" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="264" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A264" s="1">
+        <v>1</v>
+      </c>
+      <c r="B264" s="2">
+        <v>2</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D264" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F264" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G264" s="5">
+        <v>288</v>
+      </c>
+      <c r="H264" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I264" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J264" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K264" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L264" s="6">
+        <v>575</v>
+      </c>
+      <c r="M264" s="7">
+        <v>113173.11</v>
+      </c>
+      <c r="N264" s="6">
+        <v>1</v>
+      </c>
+      <c r="O264" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P264" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q264" s="6">
+        <v>0</v>
+      </c>
+      <c r="R264" s="7">
+        <v>0</v>
+      </c>
+      <c r="S264" s="9">
+        <v>0</v>
+      </c>
+      <c r="T264" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U264" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V264" s="11">
+        <v>11</v>
+      </c>
+      <c r="W264" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X264" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y264" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB264" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG264" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI264" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ264" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK264" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM264" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR264" s="3" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="265" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A265" s="1">
+        <v>1</v>
+      </c>
+      <c r="B265" s="2">
+        <v>2</v>
+      </c>
+      <c r="C265" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D265" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E265" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F265" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G265" s="5">
+        <v>289</v>
+      </c>
+      <c r="H265" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I265" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J265" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K265" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L265" s="6">
+        <v>576</v>
+      </c>
+      <c r="M265" s="7">
+        <v>113369.94</v>
+      </c>
+      <c r="N265" s="6">
+        <v>1</v>
+      </c>
+      <c r="O265" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P265" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q265" s="6">
+        <v>0</v>
+      </c>
+      <c r="R265" s="7">
+        <v>0</v>
+      </c>
+      <c r="S265" s="9">
+        <v>0</v>
+      </c>
+      <c r="T265" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U265" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V265" s="11">
+        <v>11</v>
+      </c>
+      <c r="W265" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X265" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y265" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB265" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG265" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI265" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ265" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK265" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM265" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR265" s="3" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="266" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A266" s="1">
+        <v>1</v>
+      </c>
+      <c r="B266" s="2">
+        <v>2</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D266" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E266" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F266" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G266" s="5">
+        <v>290</v>
+      </c>
+      <c r="H266" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I266" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J266" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K266" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L266" s="6">
+        <v>577</v>
+      </c>
+      <c r="M266" s="7">
+        <v>113566.76</v>
+      </c>
+      <c r="N266" s="6">
+        <v>1</v>
+      </c>
+      <c r="O266" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P266" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q266" s="6">
+        <v>0</v>
+      </c>
+      <c r="R266" s="7">
+        <v>0</v>
+      </c>
+      <c r="S266" s="9">
+        <v>0</v>
+      </c>
+      <c r="T266" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U266" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V266" s="11">
+        <v>11</v>
+      </c>
+      <c r="W266" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X266" s="12">
+        <v>0.56805559999999999</v>
+      </c>
+      <c r="Y266" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB266" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG266" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI266" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ266" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK266" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM266" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR266" s="3" t="s">
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 05/05/2026 14:13:57,09
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B50ACE2-8DDE-4CEF-B052-CDD001BCB83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{155BE6D4-7FAE-4782-83BA-A54F0BC9E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4814" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5372" uniqueCount="351">
   <si>
     <t>Sel</t>
   </si>
@@ -981,6 +981,99 @@
   <si>
     <t>1854300114222</t>
   </si>
+  <si>
+    <t>1854300114223</t>
+  </si>
+  <si>
+    <t>1854300114224</t>
+  </si>
+  <si>
+    <t>1854300114225</t>
+  </si>
+  <si>
+    <t>1854300114226</t>
+  </si>
+  <si>
+    <t>1854300114227</t>
+  </si>
+  <si>
+    <t>1854300114228</t>
+  </si>
+  <si>
+    <t>1854300114229</t>
+  </si>
+  <si>
+    <t>1854300114230</t>
+  </si>
+  <si>
+    <t>1854300114231</t>
+  </si>
+  <si>
+    <t>1854300114232</t>
+  </si>
+  <si>
+    <t>1854300114233</t>
+  </si>
+  <si>
+    <t>1854300114234</t>
+  </si>
+  <si>
+    <t>1854300114235</t>
+  </si>
+  <si>
+    <t>1854300114236</t>
+  </si>
+  <si>
+    <t>1854300114237</t>
+  </si>
+  <si>
+    <t>1854300114238</t>
+  </si>
+  <si>
+    <t>1854300114239</t>
+  </si>
+  <si>
+    <t>1854300114240</t>
+  </si>
+  <si>
+    <t>1854300114241</t>
+  </si>
+  <si>
+    <t>1854300114242</t>
+  </si>
+  <si>
+    <t>1854300114243</t>
+  </si>
+  <si>
+    <t>1854300114244</t>
+  </si>
+  <si>
+    <t>1854300114245</t>
+  </si>
+  <si>
+    <t>1854300114246</t>
+  </si>
+  <si>
+    <t>1854300114247</t>
+  </si>
+  <si>
+    <t>1854300114248</t>
+  </si>
+  <si>
+    <t>1854300114249</t>
+  </si>
+  <si>
+    <t>1854300114250</t>
+  </si>
+  <si>
+    <t>1854300114251</t>
+  </si>
+  <si>
+    <t>1854300114252</t>
+  </si>
+  <si>
+    <t>1854300114253</t>
+  </si>
 </sst>
 </file>
 
@@ -1555,7 +1648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR266"/>
+  <dimension ref="A1:AR297"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -37200,6 +37293,4160 @@
       </c>
       <c r="AR266" s="3" t="s">
         <v>319</v>
+      </c>
+    </row>
+    <row r="267" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A267" s="1">
+        <v>1</v>
+      </c>
+      <c r="B267" s="2">
+        <v>2</v>
+      </c>
+      <c r="C267" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D267" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E267" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F267" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G267" s="5">
+        <v>291</v>
+      </c>
+      <c r="H267" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I267" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J267" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K267" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L267" s="6">
+        <v>578</v>
+      </c>
+      <c r="M267" s="7">
+        <v>113763.58</v>
+      </c>
+      <c r="N267" s="6">
+        <v>1</v>
+      </c>
+      <c r="O267" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P267" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q267" s="6">
+        <v>0</v>
+      </c>
+      <c r="R267" s="7">
+        <v>0</v>
+      </c>
+      <c r="S267" s="9">
+        <v>0</v>
+      </c>
+      <c r="T267" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U267" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V267" s="11">
+        <v>11</v>
+      </c>
+      <c r="W267" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X267" s="12">
+        <v>0.58819440000000001</v>
+      </c>
+      <c r="Y267" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB267" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG267" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI267" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ267" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK267" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM267" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR267" s="3" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="268" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A268" s="1">
+        <v>1</v>
+      </c>
+      <c r="B268" s="2">
+        <v>2</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D268" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E268" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F268" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G268" s="5">
+        <v>292</v>
+      </c>
+      <c r="H268" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I268" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J268" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K268" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L268" s="6">
+        <v>579</v>
+      </c>
+      <c r="M268" s="7">
+        <v>113960.4</v>
+      </c>
+      <c r="N268" s="6">
+        <v>1</v>
+      </c>
+      <c r="O268" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P268" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q268" s="6">
+        <v>0</v>
+      </c>
+      <c r="R268" s="7">
+        <v>0</v>
+      </c>
+      <c r="S268" s="9">
+        <v>0</v>
+      </c>
+      <c r="T268" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U268" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V268" s="11">
+        <v>11</v>
+      </c>
+      <c r="W268" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X268" s="12">
+        <v>0.58819440000000001</v>
+      </c>
+      <c r="Y268" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z268" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA268" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB268" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC268" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD268" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE268" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF268" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG268" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH268" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI268" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ268" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK268" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL268" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM268" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN268" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO268" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP268" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ268" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR268" s="3" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="269" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A269" s="1">
+        <v>1</v>
+      </c>
+      <c r="B269" s="2">
+        <v>2</v>
+      </c>
+      <c r="C269" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D269" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E269" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F269" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G269" s="5">
+        <v>293</v>
+      </c>
+      <c r="H269" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I269" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J269" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K269" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L269" s="6">
+        <v>580</v>
+      </c>
+      <c r="M269" s="7">
+        <v>114157.23</v>
+      </c>
+      <c r="N269" s="6">
+        <v>1</v>
+      </c>
+      <c r="O269" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P269" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q269" s="6">
+        <v>0</v>
+      </c>
+      <c r="R269" s="7">
+        <v>0</v>
+      </c>
+      <c r="S269" s="9">
+        <v>0</v>
+      </c>
+      <c r="T269" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U269" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V269" s="11">
+        <v>11</v>
+      </c>
+      <c r="W269" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X269" s="12">
+        <v>0.58819440000000001</v>
+      </c>
+      <c r="Y269" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z269" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA269" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB269" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC269" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD269" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE269" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF269" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG269" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH269" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI269" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ269" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK269" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL269" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM269" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN269" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO269" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP269" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ269" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR269" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="270" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A270" s="1">
+        <v>1</v>
+      </c>
+      <c r="B270" s="2">
+        <v>2</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D270" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E270" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F270" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G270" s="5">
+        <v>294</v>
+      </c>
+      <c r="H270" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I270" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J270" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K270" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L270" s="6">
+        <v>581</v>
+      </c>
+      <c r="M270" s="7">
+        <v>114354.05</v>
+      </c>
+      <c r="N270" s="6">
+        <v>1</v>
+      </c>
+      <c r="O270" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P270" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q270" s="6">
+        <v>0</v>
+      </c>
+      <c r="R270" s="7">
+        <v>0</v>
+      </c>
+      <c r="S270" s="9">
+        <v>0</v>
+      </c>
+      <c r="T270" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U270" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V270" s="11">
+        <v>11</v>
+      </c>
+      <c r="W270" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X270" s="12">
+        <v>0.58819440000000001</v>
+      </c>
+      <c r="Y270" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z270" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA270" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB270" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC270" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD270" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE270" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF270" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG270" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH270" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI270" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ270" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK270" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL270" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM270" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN270" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO270" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP270" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ270" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR270" s="3" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="271" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A271" s="1">
+        <v>1</v>
+      </c>
+      <c r="B271" s="2">
+        <v>2</v>
+      </c>
+      <c r="C271" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D271" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E271" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F271" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G271" s="5">
+        <v>295</v>
+      </c>
+      <c r="H271" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I271" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J271" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K271" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L271" s="6">
+        <v>582</v>
+      </c>
+      <c r="M271" s="7">
+        <v>114550.87</v>
+      </c>
+      <c r="N271" s="6">
+        <v>1</v>
+      </c>
+      <c r="O271" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P271" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q271" s="6">
+        <v>0</v>
+      </c>
+      <c r="R271" s="7">
+        <v>0</v>
+      </c>
+      <c r="S271" s="9">
+        <v>0</v>
+      </c>
+      <c r="T271" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U271" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V271" s="11">
+        <v>11</v>
+      </c>
+      <c r="W271" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X271" s="12">
+        <v>0.58819440000000001</v>
+      </c>
+      <c r="Y271" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB271" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG271" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI271" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ271" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK271" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM271" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR271" s="3" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="272" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A272" s="1">
+        <v>1</v>
+      </c>
+      <c r="B272" s="2">
+        <v>2</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D272" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E272" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F272" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G272" s="5">
+        <v>296</v>
+      </c>
+      <c r="H272" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I272" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J272" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K272" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L272" s="6">
+        <v>583</v>
+      </c>
+      <c r="M272" s="7">
+        <v>114747.7</v>
+      </c>
+      <c r="N272" s="6">
+        <v>1</v>
+      </c>
+      <c r="O272" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P272" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q272" s="6">
+        <v>0</v>
+      </c>
+      <c r="R272" s="7">
+        <v>0</v>
+      </c>
+      <c r="S272" s="9">
+        <v>0</v>
+      </c>
+      <c r="T272" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U272" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V272" s="11">
+        <v>11</v>
+      </c>
+      <c r="W272" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X272" s="12">
+        <v>0.58819440000000001</v>
+      </c>
+      <c r="Y272" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB272" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG272" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI272" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ272" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK272" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM272" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR272" s="3" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="273" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A273" s="1">
+        <v>1</v>
+      </c>
+      <c r="B273" s="2">
+        <v>2</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D273" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E273" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F273" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G273" s="5">
+        <v>297</v>
+      </c>
+      <c r="H273" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I273" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J273" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K273" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L273" s="6">
+        <v>584</v>
+      </c>
+      <c r="M273" s="7">
+        <v>114944.52</v>
+      </c>
+      <c r="N273" s="6">
+        <v>1</v>
+      </c>
+      <c r="O273" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P273" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q273" s="6">
+        <v>0</v>
+      </c>
+      <c r="R273" s="7">
+        <v>0</v>
+      </c>
+      <c r="S273" s="9">
+        <v>0</v>
+      </c>
+      <c r="T273" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U273" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V273" s="11">
+        <v>11</v>
+      </c>
+      <c r="W273" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X273" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y273" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB273" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG273" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI273" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ273" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK273" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM273" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR273" s="3" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="274" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A274" s="1">
+        <v>1</v>
+      </c>
+      <c r="B274" s="2">
+        <v>2</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D274" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E274" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F274" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G274" s="5">
+        <v>298</v>
+      </c>
+      <c r="H274" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I274" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J274" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K274" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L274" s="6">
+        <v>585</v>
+      </c>
+      <c r="M274" s="7">
+        <v>115141.34</v>
+      </c>
+      <c r="N274" s="6">
+        <v>1</v>
+      </c>
+      <c r="O274" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P274" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q274" s="6">
+        <v>0</v>
+      </c>
+      <c r="R274" s="7">
+        <v>0</v>
+      </c>
+      <c r="S274" s="9">
+        <v>0</v>
+      </c>
+      <c r="T274" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U274" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V274" s="11">
+        <v>11</v>
+      </c>
+      <c r="W274" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X274" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y274" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB274" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG274" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI274" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ274" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK274" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM274" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR274" s="3" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="275" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A275" s="1">
+        <v>1</v>
+      </c>
+      <c r="B275" s="2">
+        <v>2</v>
+      </c>
+      <c r="C275" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D275" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E275" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F275" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G275" s="5">
+        <v>299</v>
+      </c>
+      <c r="H275" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I275" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J275" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K275" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L275" s="6">
+        <v>586</v>
+      </c>
+      <c r="M275" s="7">
+        <v>115338.16</v>
+      </c>
+      <c r="N275" s="6">
+        <v>1</v>
+      </c>
+      <c r="O275" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P275" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q275" s="6">
+        <v>0</v>
+      </c>
+      <c r="R275" s="7">
+        <v>0</v>
+      </c>
+      <c r="S275" s="9">
+        <v>0</v>
+      </c>
+      <c r="T275" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U275" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V275" s="11">
+        <v>11</v>
+      </c>
+      <c r="W275" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X275" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y275" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB275" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG275" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI275" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ275" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK275" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM275" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR275" s="3" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="276" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A276" s="1">
+        <v>1</v>
+      </c>
+      <c r="B276" s="2">
+        <v>2</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D276" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E276" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F276" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G276" s="5">
+        <v>300</v>
+      </c>
+      <c r="H276" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I276" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J276" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K276" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L276" s="6">
+        <v>587</v>
+      </c>
+      <c r="M276" s="7">
+        <v>115534.99</v>
+      </c>
+      <c r="N276" s="6">
+        <v>1</v>
+      </c>
+      <c r="O276" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P276" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q276" s="6">
+        <v>0</v>
+      </c>
+      <c r="R276" s="7">
+        <v>0</v>
+      </c>
+      <c r="S276" s="9">
+        <v>0</v>
+      </c>
+      <c r="T276" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U276" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V276" s="11">
+        <v>11</v>
+      </c>
+      <c r="W276" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X276" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y276" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB276" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG276" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI276" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ276" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK276" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM276" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR276" s="3" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="277" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A277" s="1">
+        <v>1</v>
+      </c>
+      <c r="B277" s="2">
+        <v>2</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D277" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E277" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F277" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G277" s="5">
+        <v>301</v>
+      </c>
+      <c r="H277" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I277" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J277" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K277" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L277" s="6">
+        <v>588</v>
+      </c>
+      <c r="M277" s="7">
+        <v>115731.81</v>
+      </c>
+      <c r="N277" s="6">
+        <v>1</v>
+      </c>
+      <c r="O277" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P277" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q277" s="6">
+        <v>0</v>
+      </c>
+      <c r="R277" s="7">
+        <v>0</v>
+      </c>
+      <c r="S277" s="9">
+        <v>0</v>
+      </c>
+      <c r="T277" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U277" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V277" s="11">
+        <v>11</v>
+      </c>
+      <c r="W277" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X277" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y277" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB277" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG277" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI277" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ277" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK277" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM277" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR277" s="3" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="278" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A278" s="1">
+        <v>1</v>
+      </c>
+      <c r="B278" s="2">
+        <v>2</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D278" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E278" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F278" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G278" s="5">
+        <v>302</v>
+      </c>
+      <c r="H278" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I278" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J278" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K278" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L278" s="6">
+        <v>589</v>
+      </c>
+      <c r="M278" s="7">
+        <v>115928.63</v>
+      </c>
+      <c r="N278" s="6">
+        <v>1</v>
+      </c>
+      <c r="O278" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P278" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q278" s="6">
+        <v>0</v>
+      </c>
+      <c r="R278" s="7">
+        <v>0</v>
+      </c>
+      <c r="S278" s="9">
+        <v>0</v>
+      </c>
+      <c r="T278" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U278" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V278" s="11">
+        <v>11</v>
+      </c>
+      <c r="W278" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X278" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y278" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB278" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG278" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI278" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ278" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK278" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM278" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR278" s="3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="279" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A279" s="1">
+        <v>1</v>
+      </c>
+      <c r="B279" s="2">
+        <v>2</v>
+      </c>
+      <c r="C279" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D279" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E279" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F279" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G279" s="5">
+        <v>303</v>
+      </c>
+      <c r="H279" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I279" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J279" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K279" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L279" s="6">
+        <v>590</v>
+      </c>
+      <c r="M279" s="7">
+        <v>116125.45</v>
+      </c>
+      <c r="N279" s="6">
+        <v>1</v>
+      </c>
+      <c r="O279" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P279" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q279" s="6">
+        <v>0</v>
+      </c>
+      <c r="R279" s="7">
+        <v>0</v>
+      </c>
+      <c r="S279" s="9">
+        <v>0</v>
+      </c>
+      <c r="T279" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U279" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V279" s="11">
+        <v>11</v>
+      </c>
+      <c r="W279" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X279" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y279" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB279" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG279" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI279" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ279" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK279" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM279" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR279" s="3" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="280" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A280" s="1">
+        <v>1</v>
+      </c>
+      <c r="B280" s="2">
+        <v>2</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D280" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E280" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F280" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G280" s="5">
+        <v>304</v>
+      </c>
+      <c r="H280" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I280" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J280" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K280" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L280" s="6">
+        <v>591</v>
+      </c>
+      <c r="M280" s="7">
+        <v>116322.28</v>
+      </c>
+      <c r="N280" s="6">
+        <v>1</v>
+      </c>
+      <c r="O280" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P280" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q280" s="6">
+        <v>0</v>
+      </c>
+      <c r="R280" s="7">
+        <v>0</v>
+      </c>
+      <c r="S280" s="9">
+        <v>0</v>
+      </c>
+      <c r="T280" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U280" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V280" s="11">
+        <v>11</v>
+      </c>
+      <c r="W280" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X280" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y280" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB280" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG280" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI280" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ280" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK280" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM280" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR280" s="3" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="281" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A281" s="1">
+        <v>1</v>
+      </c>
+      <c r="B281" s="2">
+        <v>2</v>
+      </c>
+      <c r="C281" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D281" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E281" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F281" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G281" s="5">
+        <v>305</v>
+      </c>
+      <c r="H281" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I281" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J281" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K281" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L281" s="6">
+        <v>592</v>
+      </c>
+      <c r="M281" s="7">
+        <v>116519.1</v>
+      </c>
+      <c r="N281" s="6">
+        <v>1</v>
+      </c>
+      <c r="O281" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P281" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q281" s="6">
+        <v>0</v>
+      </c>
+      <c r="R281" s="7">
+        <v>0</v>
+      </c>
+      <c r="S281" s="9">
+        <v>0</v>
+      </c>
+      <c r="T281" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U281" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V281" s="11">
+        <v>11</v>
+      </c>
+      <c r="W281" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X281" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y281" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB281" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG281" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI281" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ281" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK281" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM281" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR281" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="282" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A282" s="1">
+        <v>1</v>
+      </c>
+      <c r="B282" s="2">
+        <v>2</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D282" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E282" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F282" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G282" s="5">
+        <v>306</v>
+      </c>
+      <c r="H282" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I282" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J282" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K282" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L282" s="6">
+        <v>593</v>
+      </c>
+      <c r="M282" s="7">
+        <v>116715.92</v>
+      </c>
+      <c r="N282" s="6">
+        <v>1</v>
+      </c>
+      <c r="O282" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P282" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q282" s="6">
+        <v>0</v>
+      </c>
+      <c r="R282" s="7">
+        <v>0</v>
+      </c>
+      <c r="S282" s="9">
+        <v>0</v>
+      </c>
+      <c r="T282" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U282" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V282" s="11">
+        <v>11</v>
+      </c>
+      <c r="W282" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X282" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y282" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB282" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG282" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI282" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ282" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK282" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM282" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR282" s="3" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="283" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A283" s="1">
+        <v>1</v>
+      </c>
+      <c r="B283" s="2">
+        <v>2</v>
+      </c>
+      <c r="C283" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D283" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E283" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F283" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G283" s="5">
+        <v>307</v>
+      </c>
+      <c r="H283" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I283" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J283" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K283" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L283" s="6">
+        <v>594</v>
+      </c>
+      <c r="M283" s="7">
+        <v>116912.75</v>
+      </c>
+      <c r="N283" s="6">
+        <v>1</v>
+      </c>
+      <c r="O283" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P283" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q283" s="6">
+        <v>0</v>
+      </c>
+      <c r="R283" s="7">
+        <v>0</v>
+      </c>
+      <c r="S283" s="9">
+        <v>0</v>
+      </c>
+      <c r="T283" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U283" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V283" s="11">
+        <v>11</v>
+      </c>
+      <c r="W283" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X283" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y283" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB283" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG283" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI283" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ283" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK283" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM283" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR283" s="3" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="284" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A284" s="1">
+        <v>1</v>
+      </c>
+      <c r="B284" s="2">
+        <v>2</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D284" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E284" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F284" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G284" s="5">
+        <v>308</v>
+      </c>
+      <c r="H284" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I284" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J284" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K284" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L284" s="6">
+        <v>595</v>
+      </c>
+      <c r="M284" s="7">
+        <v>117109.57</v>
+      </c>
+      <c r="N284" s="6">
+        <v>1</v>
+      </c>
+      <c r="O284" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P284" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q284" s="6">
+        <v>0</v>
+      </c>
+      <c r="R284" s="7">
+        <v>0</v>
+      </c>
+      <c r="S284" s="9">
+        <v>0</v>
+      </c>
+      <c r="T284" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U284" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V284" s="11">
+        <v>11</v>
+      </c>
+      <c r="W284" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X284" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y284" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB284" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG284" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI284" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ284" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK284" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM284" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR284" s="3" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="285" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A285" s="1">
+        <v>1</v>
+      </c>
+      <c r="B285" s="2">
+        <v>2</v>
+      </c>
+      <c r="C285" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D285" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E285" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F285" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G285" s="5">
+        <v>309</v>
+      </c>
+      <c r="H285" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I285" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J285" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K285" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L285" s="6">
+        <v>596</v>
+      </c>
+      <c r="M285" s="7">
+        <v>117306.39</v>
+      </c>
+      <c r="N285" s="6">
+        <v>1</v>
+      </c>
+      <c r="O285" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P285" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q285" s="6">
+        <v>0</v>
+      </c>
+      <c r="R285" s="7">
+        <v>0</v>
+      </c>
+      <c r="S285" s="9">
+        <v>0</v>
+      </c>
+      <c r="T285" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U285" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V285" s="11">
+        <v>11</v>
+      </c>
+      <c r="W285" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X285" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y285" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB285" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG285" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI285" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ285" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK285" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM285" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR285" s="3" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="286" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A286" s="1">
+        <v>1</v>
+      </c>
+      <c r="B286" s="2">
+        <v>2</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D286" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E286" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F286" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G286" s="5">
+        <v>310</v>
+      </c>
+      <c r="H286" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I286" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J286" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K286" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L286" s="6">
+        <v>597</v>
+      </c>
+      <c r="M286" s="7">
+        <v>117503.21</v>
+      </c>
+      <c r="N286" s="6">
+        <v>1</v>
+      </c>
+      <c r="O286" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P286" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q286" s="6">
+        <v>0</v>
+      </c>
+      <c r="R286" s="7">
+        <v>0</v>
+      </c>
+      <c r="S286" s="9">
+        <v>0</v>
+      </c>
+      <c r="T286" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U286" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V286" s="11">
+        <v>11</v>
+      </c>
+      <c r="W286" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X286" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y286" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB286" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG286" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI286" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ286" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK286" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM286" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR286" s="3" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="287" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A287" s="1">
+        <v>1</v>
+      </c>
+      <c r="B287" s="2">
+        <v>2</v>
+      </c>
+      <c r="C287" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D287" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E287" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F287" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G287" s="5">
+        <v>311</v>
+      </c>
+      <c r="H287" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I287" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J287" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K287" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L287" s="6">
+        <v>598</v>
+      </c>
+      <c r="M287" s="7">
+        <v>117700.04</v>
+      </c>
+      <c r="N287" s="6">
+        <v>1</v>
+      </c>
+      <c r="O287" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P287" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q287" s="6">
+        <v>0</v>
+      </c>
+      <c r="R287" s="7">
+        <v>0</v>
+      </c>
+      <c r="S287" s="9">
+        <v>0</v>
+      </c>
+      <c r="T287" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U287" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V287" s="11">
+        <v>11</v>
+      </c>
+      <c r="W287" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X287" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y287" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB287" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG287" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI287" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ287" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK287" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM287" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR287" s="3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="288" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A288" s="1">
+        <v>1</v>
+      </c>
+      <c r="B288" s="2">
+        <v>2</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E288" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F288" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G288" s="5">
+        <v>312</v>
+      </c>
+      <c r="H288" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I288" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J288" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K288" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L288" s="6">
+        <v>599</v>
+      </c>
+      <c r="M288" s="7">
+        <v>117896.86</v>
+      </c>
+      <c r="N288" s="6">
+        <v>1</v>
+      </c>
+      <c r="O288" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P288" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q288" s="6">
+        <v>0</v>
+      </c>
+      <c r="R288" s="7">
+        <v>0</v>
+      </c>
+      <c r="S288" s="9">
+        <v>0</v>
+      </c>
+      <c r="T288" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U288" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V288" s="11">
+        <v>11</v>
+      </c>
+      <c r="W288" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X288" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y288" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB288" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG288" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI288" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ288" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK288" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM288" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR288" s="3" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="289" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A289" s="1">
+        <v>1</v>
+      </c>
+      <c r="B289" s="2">
+        <v>2</v>
+      </c>
+      <c r="C289" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D289" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E289" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F289" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G289" s="5">
+        <v>313</v>
+      </c>
+      <c r="H289" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I289" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J289" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K289" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L289" s="6">
+        <v>600</v>
+      </c>
+      <c r="M289" s="7">
+        <v>118093.68</v>
+      </c>
+      <c r="N289" s="6">
+        <v>1</v>
+      </c>
+      <c r="O289" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P289" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q289" s="6">
+        <v>0</v>
+      </c>
+      <c r="R289" s="7">
+        <v>0</v>
+      </c>
+      <c r="S289" s="9">
+        <v>0</v>
+      </c>
+      <c r="T289" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U289" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V289" s="11">
+        <v>11</v>
+      </c>
+      <c r="W289" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X289" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y289" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB289" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG289" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI289" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ289" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK289" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM289" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR289" s="3" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="290" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A290" s="1">
+        <v>1</v>
+      </c>
+      <c r="B290" s="2">
+        <v>2</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D290" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E290" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F290" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G290" s="5">
+        <v>314</v>
+      </c>
+      <c r="H290" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I290" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J290" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K290" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L290" s="6">
+        <v>601</v>
+      </c>
+      <c r="M290" s="7">
+        <v>118290.51</v>
+      </c>
+      <c r="N290" s="6">
+        <v>1</v>
+      </c>
+      <c r="O290" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P290" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q290" s="6">
+        <v>0</v>
+      </c>
+      <c r="R290" s="7">
+        <v>0</v>
+      </c>
+      <c r="S290" s="9">
+        <v>0</v>
+      </c>
+      <c r="T290" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U290" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V290" s="11">
+        <v>11</v>
+      </c>
+      <c r="W290" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X290" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y290" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB290" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG290" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI290" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ290" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK290" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM290" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR290" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="291" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A291" s="1">
+        <v>1</v>
+      </c>
+      <c r="B291" s="2">
+        <v>2</v>
+      </c>
+      <c r="C291" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D291" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E291" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F291" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G291" s="5">
+        <v>315</v>
+      </c>
+      <c r="H291" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I291" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J291" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K291" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L291" s="6">
+        <v>602</v>
+      </c>
+      <c r="M291" s="7">
+        <v>118487.33</v>
+      </c>
+      <c r="N291" s="6">
+        <v>1</v>
+      </c>
+      <c r="O291" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P291" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q291" s="6">
+        <v>0</v>
+      </c>
+      <c r="R291" s="7">
+        <v>0</v>
+      </c>
+      <c r="S291" s="9">
+        <v>0</v>
+      </c>
+      <c r="T291" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U291" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V291" s="11">
+        <v>11</v>
+      </c>
+      <c r="W291" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X291" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y291" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB291" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG291" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI291" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ291" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK291" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM291" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR291" s="3" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="292" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A292" s="1">
+        <v>1</v>
+      </c>
+      <c r="B292" s="2">
+        <v>2</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F292" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G292" s="5">
+        <v>316</v>
+      </c>
+      <c r="H292" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I292" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J292" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K292" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L292" s="6">
+        <v>603</v>
+      </c>
+      <c r="M292" s="7">
+        <v>118684.15</v>
+      </c>
+      <c r="N292" s="6">
+        <v>1</v>
+      </c>
+      <c r="O292" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P292" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q292" s="6">
+        <v>0</v>
+      </c>
+      <c r="R292" s="7">
+        <v>0</v>
+      </c>
+      <c r="S292" s="9">
+        <v>0</v>
+      </c>
+      <c r="T292" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U292" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V292" s="11">
+        <v>11</v>
+      </c>
+      <c r="W292" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X292" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y292" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB292" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG292" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI292" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ292" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK292" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM292" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR292" s="3" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="293" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A293" s="1">
+        <v>1</v>
+      </c>
+      <c r="B293" s="2">
+        <v>2</v>
+      </c>
+      <c r="C293" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D293" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E293" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F293" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G293" s="5">
+        <v>317</v>
+      </c>
+      <c r="H293" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I293" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J293" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K293" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L293" s="6">
+        <v>604</v>
+      </c>
+      <c r="M293" s="7">
+        <v>118880.97</v>
+      </c>
+      <c r="N293" s="6">
+        <v>1</v>
+      </c>
+      <c r="O293" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P293" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q293" s="6">
+        <v>0</v>
+      </c>
+      <c r="R293" s="7">
+        <v>0</v>
+      </c>
+      <c r="S293" s="9">
+        <v>0</v>
+      </c>
+      <c r="T293" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U293" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V293" s="11">
+        <v>11</v>
+      </c>
+      <c r="W293" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X293" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y293" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB293" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG293" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI293" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ293" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK293" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM293" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR293" s="3" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="294" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A294" s="1">
+        <v>1</v>
+      </c>
+      <c r="B294" s="2">
+        <v>2</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F294" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G294" s="5">
+        <v>318</v>
+      </c>
+      <c r="H294" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I294" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J294" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K294" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L294" s="6">
+        <v>605</v>
+      </c>
+      <c r="M294" s="7">
+        <v>119077.8</v>
+      </c>
+      <c r="N294" s="6">
+        <v>1</v>
+      </c>
+      <c r="O294" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P294" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q294" s="6">
+        <v>0</v>
+      </c>
+      <c r="R294" s="7">
+        <v>0</v>
+      </c>
+      <c r="S294" s="9">
+        <v>0</v>
+      </c>
+      <c r="T294" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U294" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V294" s="11">
+        <v>11</v>
+      </c>
+      <c r="W294" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X294" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y294" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB294" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG294" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI294" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ294" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK294" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM294" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR294" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="295" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A295" s="1">
+        <v>1</v>
+      </c>
+      <c r="B295" s="2">
+        <v>2</v>
+      </c>
+      <c r="C295" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E295" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F295" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G295" s="5">
+        <v>319</v>
+      </c>
+      <c r="H295" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I295" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J295" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K295" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L295" s="6">
+        <v>606</v>
+      </c>
+      <c r="M295" s="7">
+        <v>119274.62</v>
+      </c>
+      <c r="N295" s="6">
+        <v>1</v>
+      </c>
+      <c r="O295" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P295" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q295" s="6">
+        <v>0</v>
+      </c>
+      <c r="R295" s="7">
+        <v>0</v>
+      </c>
+      <c r="S295" s="9">
+        <v>0</v>
+      </c>
+      <c r="T295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U295" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V295" s="11">
+        <v>11</v>
+      </c>
+      <c r="W295" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X295" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y295" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB295" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG295" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI295" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR295" s="3" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="296" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A296" s="1">
+        <v>1</v>
+      </c>
+      <c r="B296" s="2">
+        <v>2</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F296" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G296" s="5">
+        <v>320</v>
+      </c>
+      <c r="H296" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I296" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J296" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K296" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L296" s="6">
+        <v>607</v>
+      </c>
+      <c r="M296" s="7">
+        <v>119471.44</v>
+      </c>
+      <c r="N296" s="6">
+        <v>1</v>
+      </c>
+      <c r="O296" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P296" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q296" s="6">
+        <v>0</v>
+      </c>
+      <c r="R296" s="7">
+        <v>0</v>
+      </c>
+      <c r="S296" s="9">
+        <v>0</v>
+      </c>
+      <c r="T296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U296" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V296" s="11">
+        <v>11</v>
+      </c>
+      <c r="W296" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X296" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y296" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB296" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG296" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI296" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR296" s="3" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="297" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A297" s="1">
+        <v>1</v>
+      </c>
+      <c r="B297" s="2">
+        <v>2</v>
+      </c>
+      <c r="C297" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E297" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F297" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G297" s="5">
+        <v>321</v>
+      </c>
+      <c r="H297" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I297" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J297" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K297" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L297" s="6">
+        <v>608</v>
+      </c>
+      <c r="M297" s="7">
+        <v>119668.27</v>
+      </c>
+      <c r="N297" s="6">
+        <v>1</v>
+      </c>
+      <c r="O297" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P297" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q297" s="6">
+        <v>0</v>
+      </c>
+      <c r="R297" s="7">
+        <v>0</v>
+      </c>
+      <c r="S297" s="9">
+        <v>0</v>
+      </c>
+      <c r="T297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U297" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V297" s="11">
+        <v>11</v>
+      </c>
+      <c r="W297" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X297" s="12">
+        <v>0.58888890000000005</v>
+      </c>
+      <c r="Y297" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB297" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG297" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI297" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR297" s="3" t="s">
+        <v>350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 05/05/2026 14:54:00,02
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{155BE6D4-7FAE-4782-83BA-A54F0BC9E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97FBE8C7-F190-402E-A97C-99BCB1F18ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5372" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5786" uniqueCount="374">
   <si>
     <t>Sel</t>
   </si>
@@ -1074,6 +1074,75 @@
   <si>
     <t>1854300114253</t>
   </si>
+  <si>
+    <t>1854300113618</t>
+  </si>
+  <si>
+    <t>1854300113619</t>
+  </si>
+  <si>
+    <t>1854300113620</t>
+  </si>
+  <si>
+    <t>1854300113621</t>
+  </si>
+  <si>
+    <t>1854300113622</t>
+  </si>
+  <si>
+    <t>1854300113623</t>
+  </si>
+  <si>
+    <t>1854300113624</t>
+  </si>
+  <si>
+    <t>1854300113625</t>
+  </si>
+  <si>
+    <t>1854300113626</t>
+  </si>
+  <si>
+    <t>1854300113627</t>
+  </si>
+  <si>
+    <t>1854300113628</t>
+  </si>
+  <si>
+    <t>1854300113629</t>
+  </si>
+  <si>
+    <t>1854300113630</t>
+  </si>
+  <si>
+    <t>1854300113631</t>
+  </si>
+  <si>
+    <t>1854300113632</t>
+  </si>
+  <si>
+    <t>1854300113633</t>
+  </si>
+  <si>
+    <t>1854300113634</t>
+  </si>
+  <si>
+    <t>1854300113635</t>
+  </si>
+  <si>
+    <t>1854300113636</t>
+  </si>
+  <si>
+    <t>1854300114254</t>
+  </si>
+  <si>
+    <t>1854300114255</t>
+  </si>
+  <si>
+    <t>1854300114256</t>
+  </si>
+  <si>
+    <t>1854300114257</t>
+  </si>
 </sst>
 </file>
 
@@ -1648,7 +1717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR297"/>
+  <dimension ref="A1:AR320"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -41447,6 +41516,3088 @@
       </c>
       <c r="AR297" s="3" t="s">
         <v>350</v>
+      </c>
+    </row>
+    <row r="298" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A298" s="1">
+        <v>1</v>
+      </c>
+      <c r="B298" s="2">
+        <v>2</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F298" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G298" s="5">
+        <v>322</v>
+      </c>
+      <c r="H298" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I298" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J298" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K298" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L298" s="6">
+        <v>609</v>
+      </c>
+      <c r="M298" s="7">
+        <v>119865.09</v>
+      </c>
+      <c r="N298" s="6">
+        <v>1</v>
+      </c>
+      <c r="O298" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P298" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q298" s="6">
+        <v>0</v>
+      </c>
+      <c r="R298" s="7">
+        <v>0</v>
+      </c>
+      <c r="S298" s="9">
+        <v>0</v>
+      </c>
+      <c r="T298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U298" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V298" s="11">
+        <v>11</v>
+      </c>
+      <c r="W298" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X298" s="12">
+        <v>0.60902780000000001</v>
+      </c>
+      <c r="Y298" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB298" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG298" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI298" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR298" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="299" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A299" s="1">
+        <v>1</v>
+      </c>
+      <c r="B299" s="2">
+        <v>2</v>
+      </c>
+      <c r="C299" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D299" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E299" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F299" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G299" s="5">
+        <v>323</v>
+      </c>
+      <c r="H299" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I299" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J299" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K299" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L299" s="6">
+        <v>610</v>
+      </c>
+      <c r="M299" s="7">
+        <v>120061.91</v>
+      </c>
+      <c r="N299" s="6">
+        <v>1</v>
+      </c>
+      <c r="O299" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P299" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q299" s="6">
+        <v>0</v>
+      </c>
+      <c r="R299" s="7">
+        <v>0</v>
+      </c>
+      <c r="S299" s="9">
+        <v>0</v>
+      </c>
+      <c r="T299" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U299" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V299" s="11">
+        <v>11</v>
+      </c>
+      <c r="W299" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X299" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y299" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB299" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG299" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI299" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ299" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK299" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM299" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR299" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="300" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A300" s="1">
+        <v>1</v>
+      </c>
+      <c r="B300" s="2">
+        <v>2</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F300" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G300" s="5">
+        <v>324</v>
+      </c>
+      <c r="H300" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I300" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J300" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K300" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L300" s="6">
+        <v>611</v>
+      </c>
+      <c r="M300" s="7">
+        <v>120258.73</v>
+      </c>
+      <c r="N300" s="6">
+        <v>1</v>
+      </c>
+      <c r="O300" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P300" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q300" s="6">
+        <v>0</v>
+      </c>
+      <c r="R300" s="7">
+        <v>0</v>
+      </c>
+      <c r="S300" s="9">
+        <v>0</v>
+      </c>
+      <c r="T300" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U300" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V300" s="11">
+        <v>11</v>
+      </c>
+      <c r="W300" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X300" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y300" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB300" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG300" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI300" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ300" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK300" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM300" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR300" s="3" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="301" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A301" s="1">
+        <v>1</v>
+      </c>
+      <c r="B301" s="2">
+        <v>2</v>
+      </c>
+      <c r="C301" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D301" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E301" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F301" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G301" s="5">
+        <v>325</v>
+      </c>
+      <c r="H301" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I301" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J301" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K301" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L301" s="6">
+        <v>612</v>
+      </c>
+      <c r="M301" s="7">
+        <v>120455.56</v>
+      </c>
+      <c r="N301" s="6">
+        <v>1</v>
+      </c>
+      <c r="O301" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P301" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q301" s="6">
+        <v>0</v>
+      </c>
+      <c r="R301" s="7">
+        <v>0</v>
+      </c>
+      <c r="S301" s="9">
+        <v>0</v>
+      </c>
+      <c r="T301" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U301" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V301" s="11">
+        <v>11</v>
+      </c>
+      <c r="W301" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X301" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y301" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB301" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG301" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI301" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ301" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK301" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM301" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR301" s="3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="302" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A302" s="1">
+        <v>1</v>
+      </c>
+      <c r="B302" s="2">
+        <v>2</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F302" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G302" s="5">
+        <v>326</v>
+      </c>
+      <c r="H302" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I302" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J302" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K302" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L302" s="6">
+        <v>613</v>
+      </c>
+      <c r="M302" s="7">
+        <v>120652.38</v>
+      </c>
+      <c r="N302" s="6">
+        <v>1</v>
+      </c>
+      <c r="O302" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P302" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q302" s="6">
+        <v>0</v>
+      </c>
+      <c r="R302" s="7">
+        <v>0</v>
+      </c>
+      <c r="S302" s="9">
+        <v>0</v>
+      </c>
+      <c r="T302" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U302" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V302" s="11">
+        <v>11</v>
+      </c>
+      <c r="W302" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X302" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y302" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB302" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG302" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI302" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ302" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK302" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM302" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR302" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="303" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A303" s="1">
+        <v>1</v>
+      </c>
+      <c r="B303" s="2">
+        <v>2</v>
+      </c>
+      <c r="C303" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D303" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E303" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F303" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G303" s="5">
+        <v>327</v>
+      </c>
+      <c r="H303" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I303" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J303" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K303" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L303" s="6">
+        <v>614</v>
+      </c>
+      <c r="M303" s="7">
+        <v>120849.2</v>
+      </c>
+      <c r="N303" s="6">
+        <v>1</v>
+      </c>
+      <c r="O303" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P303" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q303" s="6">
+        <v>0</v>
+      </c>
+      <c r="R303" s="7">
+        <v>0</v>
+      </c>
+      <c r="S303" s="9">
+        <v>0</v>
+      </c>
+      <c r="T303" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U303" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V303" s="11">
+        <v>11</v>
+      </c>
+      <c r="W303" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X303" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y303" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB303" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG303" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI303" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ303" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK303" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM303" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR303" s="3" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="304" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A304" s="1">
+        <v>1</v>
+      </c>
+      <c r="B304" s="2">
+        <v>2</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F304" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G304" s="5">
+        <v>328</v>
+      </c>
+      <c r="H304" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I304" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J304" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K304" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L304" s="6">
+        <v>615</v>
+      </c>
+      <c r="M304" s="7">
+        <v>121046.03</v>
+      </c>
+      <c r="N304" s="6">
+        <v>1</v>
+      </c>
+      <c r="O304" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P304" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q304" s="6">
+        <v>0</v>
+      </c>
+      <c r="R304" s="7">
+        <v>0</v>
+      </c>
+      <c r="S304" s="9">
+        <v>0</v>
+      </c>
+      <c r="T304" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U304" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V304" s="11">
+        <v>11</v>
+      </c>
+      <c r="W304" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X304" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y304" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB304" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG304" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI304" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ304" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK304" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL304" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM304" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ304" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR304" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="305" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A305" s="1">
+        <v>1</v>
+      </c>
+      <c r="B305" s="2">
+        <v>2</v>
+      </c>
+      <c r="C305" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D305" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E305" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F305" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G305" s="5">
+        <v>329</v>
+      </c>
+      <c r="H305" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I305" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J305" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K305" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L305" s="6">
+        <v>616</v>
+      </c>
+      <c r="M305" s="7">
+        <v>121242.85</v>
+      </c>
+      <c r="N305" s="6">
+        <v>1</v>
+      </c>
+      <c r="O305" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P305" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q305" s="6">
+        <v>0</v>
+      </c>
+      <c r="R305" s="7">
+        <v>0</v>
+      </c>
+      <c r="S305" s="9">
+        <v>0</v>
+      </c>
+      <c r="T305" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U305" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V305" s="11">
+        <v>11</v>
+      </c>
+      <c r="W305" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X305" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y305" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB305" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG305" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI305" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ305" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK305" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL305" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM305" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ305" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR305" s="3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="306" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A306" s="1">
+        <v>1</v>
+      </c>
+      <c r="B306" s="2">
+        <v>2</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F306" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G306" s="5">
+        <v>330</v>
+      </c>
+      <c r="H306" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I306" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J306" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K306" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L306" s="6">
+        <v>617</v>
+      </c>
+      <c r="M306" s="7">
+        <v>121439.67</v>
+      </c>
+      <c r="N306" s="6">
+        <v>1</v>
+      </c>
+      <c r="O306" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P306" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q306" s="6">
+        <v>0</v>
+      </c>
+      <c r="R306" s="7">
+        <v>0</v>
+      </c>
+      <c r="S306" s="9">
+        <v>0</v>
+      </c>
+      <c r="T306" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U306" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V306" s="11">
+        <v>11</v>
+      </c>
+      <c r="W306" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X306" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y306" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB306" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG306" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI306" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ306" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK306" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL306" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM306" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ306" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR306" s="3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="307" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A307" s="1">
+        <v>1</v>
+      </c>
+      <c r="B307" s="2">
+        <v>2</v>
+      </c>
+      <c r="C307" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D307" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E307" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F307" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G307" s="5">
+        <v>331</v>
+      </c>
+      <c r="H307" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I307" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J307" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K307" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L307" s="6">
+        <v>618</v>
+      </c>
+      <c r="M307" s="7">
+        <v>121636.49</v>
+      </c>
+      <c r="N307" s="6">
+        <v>1</v>
+      </c>
+      <c r="O307" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P307" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q307" s="6">
+        <v>0</v>
+      </c>
+      <c r="R307" s="7">
+        <v>0</v>
+      </c>
+      <c r="S307" s="9">
+        <v>0</v>
+      </c>
+      <c r="T307" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U307" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V307" s="11">
+        <v>11</v>
+      </c>
+      <c r="W307" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X307" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y307" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB307" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG307" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI307" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ307" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK307" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL307" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM307" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ307" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR307" s="3" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="308" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A308" s="1">
+        <v>1</v>
+      </c>
+      <c r="B308" s="2">
+        <v>2</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E308" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F308" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G308" s="5">
+        <v>332</v>
+      </c>
+      <c r="H308" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I308" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J308" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K308" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L308" s="6">
+        <v>619</v>
+      </c>
+      <c r="M308" s="7">
+        <v>121833.32</v>
+      </c>
+      <c r="N308" s="6">
+        <v>1</v>
+      </c>
+      <c r="O308" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P308" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q308" s="6">
+        <v>0</v>
+      </c>
+      <c r="R308" s="7">
+        <v>0</v>
+      </c>
+      <c r="S308" s="9">
+        <v>0</v>
+      </c>
+      <c r="T308" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U308" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V308" s="11">
+        <v>11</v>
+      </c>
+      <c r="W308" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X308" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y308" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB308" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG308" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI308" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ308" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK308" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL308" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM308" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ308" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR308" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="309" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A309" s="1">
+        <v>1</v>
+      </c>
+      <c r="B309" s="2">
+        <v>2</v>
+      </c>
+      <c r="C309" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D309" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E309" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F309" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G309" s="5">
+        <v>333</v>
+      </c>
+      <c r="H309" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I309" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J309" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K309" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L309" s="6">
+        <v>620</v>
+      </c>
+      <c r="M309" s="7">
+        <v>122030.14</v>
+      </c>
+      <c r="N309" s="6">
+        <v>1</v>
+      </c>
+      <c r="O309" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P309" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q309" s="6">
+        <v>0</v>
+      </c>
+      <c r="R309" s="7">
+        <v>0</v>
+      </c>
+      <c r="S309" s="9">
+        <v>0</v>
+      </c>
+      <c r="T309" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U309" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V309" s="11">
+        <v>11</v>
+      </c>
+      <c r="W309" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X309" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y309" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB309" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG309" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI309" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ309" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK309" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL309" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM309" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ309" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR309" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="310" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A310" s="1">
+        <v>1</v>
+      </c>
+      <c r="B310" s="2">
+        <v>2</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E310" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F310" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G310" s="5">
+        <v>334</v>
+      </c>
+      <c r="H310" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I310" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J310" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K310" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L310" s="6">
+        <v>621</v>
+      </c>
+      <c r="M310" s="7">
+        <v>122226.96</v>
+      </c>
+      <c r="N310" s="6">
+        <v>1</v>
+      </c>
+      <c r="O310" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P310" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q310" s="6">
+        <v>0</v>
+      </c>
+      <c r="R310" s="7">
+        <v>0</v>
+      </c>
+      <c r="S310" s="9">
+        <v>0</v>
+      </c>
+      <c r="T310" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U310" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V310" s="11">
+        <v>11</v>
+      </c>
+      <c r="W310" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X310" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y310" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB310" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG310" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI310" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ310" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK310" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL310" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM310" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ310" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR310" s="3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="311" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A311" s="1">
+        <v>1</v>
+      </c>
+      <c r="B311" s="2">
+        <v>2</v>
+      </c>
+      <c r="C311" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D311" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E311" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F311" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G311" s="5">
+        <v>335</v>
+      </c>
+      <c r="H311" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I311" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J311" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K311" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L311" s="6">
+        <v>622</v>
+      </c>
+      <c r="M311" s="7">
+        <v>122423.78</v>
+      </c>
+      <c r="N311" s="6">
+        <v>1</v>
+      </c>
+      <c r="O311" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P311" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q311" s="6">
+        <v>0</v>
+      </c>
+      <c r="R311" s="7">
+        <v>0</v>
+      </c>
+      <c r="S311" s="9">
+        <v>0</v>
+      </c>
+      <c r="T311" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U311" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V311" s="11">
+        <v>11</v>
+      </c>
+      <c r="W311" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X311" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y311" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB311" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG311" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI311" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ311" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK311" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL311" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM311" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ311" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR311" s="3" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="312" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A312" s="1">
+        <v>1</v>
+      </c>
+      <c r="B312" s="2">
+        <v>2</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F312" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G312" s="5">
+        <v>336</v>
+      </c>
+      <c r="H312" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I312" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J312" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K312" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L312" s="6">
+        <v>623</v>
+      </c>
+      <c r="M312" s="7">
+        <v>122620.61</v>
+      </c>
+      <c r="N312" s="6">
+        <v>1</v>
+      </c>
+      <c r="O312" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P312" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q312" s="6">
+        <v>0</v>
+      </c>
+      <c r="R312" s="7">
+        <v>0</v>
+      </c>
+      <c r="S312" s="9">
+        <v>0</v>
+      </c>
+      <c r="T312" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U312" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V312" s="11">
+        <v>11</v>
+      </c>
+      <c r="W312" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X312" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y312" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB312" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG312" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI312" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ312" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK312" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL312" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM312" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ312" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR312" s="3" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="313" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A313" s="1">
+        <v>1</v>
+      </c>
+      <c r="B313" s="2">
+        <v>2</v>
+      </c>
+      <c r="C313" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D313" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E313" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F313" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G313" s="5">
+        <v>337</v>
+      </c>
+      <c r="H313" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I313" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J313" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K313" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L313" s="6">
+        <v>624</v>
+      </c>
+      <c r="M313" s="7">
+        <v>122817.43</v>
+      </c>
+      <c r="N313" s="6">
+        <v>1</v>
+      </c>
+      <c r="O313" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P313" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q313" s="6">
+        <v>0</v>
+      </c>
+      <c r="R313" s="7">
+        <v>0</v>
+      </c>
+      <c r="S313" s="9">
+        <v>0</v>
+      </c>
+      <c r="T313" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U313" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V313" s="11">
+        <v>11</v>
+      </c>
+      <c r="W313" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X313" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y313" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB313" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG313" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI313" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ313" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK313" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL313" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM313" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ313" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR313" s="3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="314" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A314" s="1">
+        <v>1</v>
+      </c>
+      <c r="B314" s="2">
+        <v>2</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D314" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E314" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F314" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G314" s="5">
+        <v>338</v>
+      </c>
+      <c r="H314" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I314" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J314" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K314" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L314" s="6">
+        <v>625</v>
+      </c>
+      <c r="M314" s="7">
+        <v>123014.25</v>
+      </c>
+      <c r="N314" s="6">
+        <v>1</v>
+      </c>
+      <c r="O314" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P314" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q314" s="6">
+        <v>0</v>
+      </c>
+      <c r="R314" s="7">
+        <v>0</v>
+      </c>
+      <c r="S314" s="9">
+        <v>0</v>
+      </c>
+      <c r="T314" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U314" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V314" s="11">
+        <v>11</v>
+      </c>
+      <c r="W314" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X314" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y314" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB314" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG314" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI314" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ314" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK314" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL314" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM314" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ314" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR314" s="3" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="315" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A315" s="1">
+        <v>1</v>
+      </c>
+      <c r="B315" s="2">
+        <v>2</v>
+      </c>
+      <c r="C315" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D315" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E315" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F315" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G315" s="5">
+        <v>339</v>
+      </c>
+      <c r="H315" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I315" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J315" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K315" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L315" s="6">
+        <v>626</v>
+      </c>
+      <c r="M315" s="7">
+        <v>123211.08</v>
+      </c>
+      <c r="N315" s="6">
+        <v>1</v>
+      </c>
+      <c r="O315" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P315" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q315" s="6">
+        <v>0</v>
+      </c>
+      <c r="R315" s="7">
+        <v>0</v>
+      </c>
+      <c r="S315" s="9">
+        <v>0</v>
+      </c>
+      <c r="T315" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U315" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V315" s="11">
+        <v>11</v>
+      </c>
+      <c r="W315" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X315" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y315" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB315" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG315" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI315" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ315" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK315" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL315" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM315" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ315" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR315" s="3" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="316" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A316" s="1">
+        <v>1</v>
+      </c>
+      <c r="B316" s="2">
+        <v>2</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D316" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E316" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F316" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G316" s="5">
+        <v>340</v>
+      </c>
+      <c r="H316" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I316" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J316" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K316" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L316" s="6">
+        <v>627</v>
+      </c>
+      <c r="M316" s="7">
+        <v>123407.9</v>
+      </c>
+      <c r="N316" s="6">
+        <v>1</v>
+      </c>
+      <c r="O316" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P316" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q316" s="6">
+        <v>0</v>
+      </c>
+      <c r="R316" s="7">
+        <v>0</v>
+      </c>
+      <c r="S316" s="9">
+        <v>0</v>
+      </c>
+      <c r="T316" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U316" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V316" s="11">
+        <v>11</v>
+      </c>
+      <c r="W316" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X316" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y316" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB316" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG316" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI316" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ316" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK316" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL316" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM316" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ316" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR316" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="317" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A317" s="1">
+        <v>1</v>
+      </c>
+      <c r="B317" s="2">
+        <v>2</v>
+      </c>
+      <c r="C317" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D317" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E317" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F317" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G317" s="5">
+        <v>341</v>
+      </c>
+      <c r="H317" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I317" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J317" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K317" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L317" s="6">
+        <v>628</v>
+      </c>
+      <c r="M317" s="7">
+        <v>123604.72</v>
+      </c>
+      <c r="N317" s="6">
+        <v>1</v>
+      </c>
+      <c r="O317" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P317" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q317" s="6">
+        <v>0</v>
+      </c>
+      <c r="R317" s="7">
+        <v>0</v>
+      </c>
+      <c r="S317" s="9">
+        <v>0</v>
+      </c>
+      <c r="T317" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U317" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V317" s="11">
+        <v>11</v>
+      </c>
+      <c r="W317" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X317" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y317" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB317" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG317" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI317" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ317" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK317" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL317" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM317" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ317" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR317" s="3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="318" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A318" s="1">
+        <v>1</v>
+      </c>
+      <c r="B318" s="2">
+        <v>2</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D318" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E318" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F318" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G318" s="5">
+        <v>342</v>
+      </c>
+      <c r="H318" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I318" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J318" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K318" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L318" s="6">
+        <v>629</v>
+      </c>
+      <c r="M318" s="7">
+        <v>123801.54</v>
+      </c>
+      <c r="N318" s="6">
+        <v>1</v>
+      </c>
+      <c r="O318" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P318" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q318" s="6">
+        <v>0</v>
+      </c>
+      <c r="R318" s="7">
+        <v>0</v>
+      </c>
+      <c r="S318" s="9">
+        <v>0</v>
+      </c>
+      <c r="T318" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U318" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V318" s="11">
+        <v>11</v>
+      </c>
+      <c r="W318" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X318" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y318" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB318" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG318" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI318" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ318" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK318" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL318" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM318" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR318" s="3" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="319" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A319" s="1">
+        <v>1</v>
+      </c>
+      <c r="B319" s="2">
+        <v>2</v>
+      </c>
+      <c r="C319" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D319" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E319" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F319" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G319" s="5">
+        <v>343</v>
+      </c>
+      <c r="H319" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I319" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J319" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K319" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L319" s="6">
+        <v>630</v>
+      </c>
+      <c r="M319" s="7">
+        <v>123998.37</v>
+      </c>
+      <c r="N319" s="6">
+        <v>1</v>
+      </c>
+      <c r="O319" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P319" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q319" s="6">
+        <v>0</v>
+      </c>
+      <c r="R319" s="7">
+        <v>0</v>
+      </c>
+      <c r="S319" s="9">
+        <v>0</v>
+      </c>
+      <c r="T319" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U319" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V319" s="11">
+        <v>11</v>
+      </c>
+      <c r="W319" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X319" s="12">
+        <v>0.60972219999999999</v>
+      </c>
+      <c r="Y319" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB319" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG319" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI319" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ319" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK319" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL319" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM319" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ319" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR319" s="3" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="320" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A320" s="1">
+        <v>1</v>
+      </c>
+      <c r="B320" s="2">
+        <v>2</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D320" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E320" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F320" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G320" s="5">
+        <v>344</v>
+      </c>
+      <c r="H320" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I320" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J320" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K320" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L320" s="6">
+        <v>631</v>
+      </c>
+      <c r="M320" s="7">
+        <v>124195.19</v>
+      </c>
+      <c r="N320" s="6">
+        <v>1</v>
+      </c>
+      <c r="O320" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P320" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q320" s="6">
+        <v>0</v>
+      </c>
+      <c r="R320" s="7">
+        <v>0</v>
+      </c>
+      <c r="S320" s="9">
+        <v>0</v>
+      </c>
+      <c r="T320" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U320" s="10">
+        <v>64146</v>
+      </c>
+      <c r="V320" s="11">
+        <v>11</v>
+      </c>
+      <c r="W320" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X320" s="12">
+        <v>0.61041670000000003</v>
+      </c>
+      <c r="Y320" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB320" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG320" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI320" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ320" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK320" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL320" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM320" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR320" s="3" t="s">
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 05/05/2026 16:19:43,05
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6266A02C-2A61-4FC7-B4B1-6724B2620219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A940F76-5D8A-4533-9875-AFB7E81C6DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6812" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7244" uniqueCount="455">
   <si>
     <t>Sel</t>
   </si>
@@ -1314,6 +1314,78 @@
   <si>
     <t>1854300113693</t>
   </si>
+  <si>
+    <t>1854300113694</t>
+  </si>
+  <si>
+    <t>1854300113695</t>
+  </si>
+  <si>
+    <t>1854300113696</t>
+  </si>
+  <si>
+    <t>1854300113697</t>
+  </si>
+  <si>
+    <t>1854300113698</t>
+  </si>
+  <si>
+    <t>1854300113699</t>
+  </si>
+  <si>
+    <t>1854300113700</t>
+  </si>
+  <si>
+    <t>1854300113701</t>
+  </si>
+  <si>
+    <t>1854300113702</t>
+  </si>
+  <si>
+    <t>1854300113703</t>
+  </si>
+  <si>
+    <t>1854300113704</t>
+  </si>
+  <si>
+    <t>1854300113705</t>
+  </si>
+  <si>
+    <t>1854300113706</t>
+  </si>
+  <si>
+    <t>1854300113707</t>
+  </si>
+  <si>
+    <t>1854300113708</t>
+  </si>
+  <si>
+    <t>1854300113709</t>
+  </si>
+  <si>
+    <t>1854300113710</t>
+  </si>
+  <si>
+    <t>1854300113711</t>
+  </si>
+  <si>
+    <t>1854300113712</t>
+  </si>
+  <si>
+    <t>1854300113713</t>
+  </si>
+  <si>
+    <t>1854300113714</t>
+  </si>
+  <si>
+    <t>1854300113715</t>
+  </si>
+  <si>
+    <t>1854300113716</t>
+  </si>
+  <si>
+    <t>1854300113717</t>
+  </si>
 </sst>
 </file>
 
@@ -1888,7 +1960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR377"/>
+  <dimension ref="A1:AR401"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -52407,6 +52479,3222 @@
       </c>
       <c r="AR377" s="3" t="s">
         <v>430</v>
+      </c>
+    </row>
+    <row r="378" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A378" s="1">
+        <v>1</v>
+      </c>
+      <c r="B378" s="2">
+        <v>2</v>
+      </c>
+      <c r="C378" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D378" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E378" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F378" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G378" s="5">
+        <v>402</v>
+      </c>
+      <c r="H378" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I378" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J378" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K378" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L378" s="6">
+        <v>689</v>
+      </c>
+      <c r="M378" s="7">
+        <v>135610.91</v>
+      </c>
+      <c r="N378" s="6">
+        <v>1</v>
+      </c>
+      <c r="O378" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P378" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q378" s="6">
+        <v>0</v>
+      </c>
+      <c r="R378" s="7">
+        <v>0</v>
+      </c>
+      <c r="S378" s="9">
+        <v>0</v>
+      </c>
+      <c r="T378" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U378" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V378" s="11">
+        <v>11</v>
+      </c>
+      <c r="W378" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X378" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y378" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB378" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG378" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI378" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ378" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK378" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM378" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR378" s="3" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="379" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A379" s="1">
+        <v>1</v>
+      </c>
+      <c r="B379" s="2">
+        <v>2</v>
+      </c>
+      <c r="C379" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D379" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E379" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F379" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G379" s="5">
+        <v>403</v>
+      </c>
+      <c r="H379" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I379" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J379" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K379" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L379" s="6">
+        <v>690</v>
+      </c>
+      <c r="M379" s="7">
+        <v>135807.74</v>
+      </c>
+      <c r="N379" s="6">
+        <v>1</v>
+      </c>
+      <c r="O379" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P379" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q379" s="6">
+        <v>0</v>
+      </c>
+      <c r="R379" s="7">
+        <v>0</v>
+      </c>
+      <c r="S379" s="9">
+        <v>0</v>
+      </c>
+      <c r="T379" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U379" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V379" s="11">
+        <v>11</v>
+      </c>
+      <c r="W379" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X379" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y379" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB379" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG379" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI379" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ379" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK379" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM379" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR379" s="3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="380" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A380" s="1">
+        <v>1</v>
+      </c>
+      <c r="B380" s="2">
+        <v>2</v>
+      </c>
+      <c r="C380" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D380" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E380" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F380" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G380" s="5">
+        <v>404</v>
+      </c>
+      <c r="H380" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I380" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J380" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K380" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L380" s="6">
+        <v>691</v>
+      </c>
+      <c r="M380" s="7">
+        <v>136004.56</v>
+      </c>
+      <c r="N380" s="6">
+        <v>1</v>
+      </c>
+      <c r="O380" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P380" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q380" s="6">
+        <v>0</v>
+      </c>
+      <c r="R380" s="7">
+        <v>0</v>
+      </c>
+      <c r="S380" s="9">
+        <v>0</v>
+      </c>
+      <c r="T380" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U380" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V380" s="11">
+        <v>11</v>
+      </c>
+      <c r="W380" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X380" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y380" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB380" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG380" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI380" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ380" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK380" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM380" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR380" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="381" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A381" s="1">
+        <v>1</v>
+      </c>
+      <c r="B381" s="2">
+        <v>2</v>
+      </c>
+      <c r="C381" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D381" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E381" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F381" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G381" s="5">
+        <v>405</v>
+      </c>
+      <c r="H381" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I381" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J381" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K381" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L381" s="6">
+        <v>692</v>
+      </c>
+      <c r="M381" s="7">
+        <v>136201.38</v>
+      </c>
+      <c r="N381" s="6">
+        <v>1</v>
+      </c>
+      <c r="O381" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P381" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q381" s="6">
+        <v>0</v>
+      </c>
+      <c r="R381" s="7">
+        <v>0</v>
+      </c>
+      <c r="S381" s="9">
+        <v>0</v>
+      </c>
+      <c r="T381" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U381" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V381" s="11">
+        <v>11</v>
+      </c>
+      <c r="W381" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X381" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y381" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB381" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG381" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI381" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ381" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK381" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM381" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR381" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="382" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A382" s="1">
+        <v>1</v>
+      </c>
+      <c r="B382" s="2">
+        <v>2</v>
+      </c>
+      <c r="C382" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D382" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E382" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F382" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G382" s="5">
+        <v>406</v>
+      </c>
+      <c r="H382" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I382" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J382" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K382" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L382" s="6">
+        <v>693</v>
+      </c>
+      <c r="M382" s="7">
+        <v>136398.20000000001</v>
+      </c>
+      <c r="N382" s="6">
+        <v>1</v>
+      </c>
+      <c r="O382" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P382" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q382" s="6">
+        <v>0</v>
+      </c>
+      <c r="R382" s="7">
+        <v>0</v>
+      </c>
+      <c r="S382" s="9">
+        <v>0</v>
+      </c>
+      <c r="T382" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U382" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V382" s="11">
+        <v>11</v>
+      </c>
+      <c r="W382" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X382" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y382" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB382" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG382" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI382" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ382" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK382" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM382" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR382" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="383" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A383" s="1">
+        <v>1</v>
+      </c>
+      <c r="B383" s="2">
+        <v>2</v>
+      </c>
+      <c r="C383" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D383" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E383" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F383" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G383" s="5">
+        <v>407</v>
+      </c>
+      <c r="H383" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I383" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J383" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K383" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L383" s="6">
+        <v>694</v>
+      </c>
+      <c r="M383" s="7">
+        <v>136595.03</v>
+      </c>
+      <c r="N383" s="6">
+        <v>1</v>
+      </c>
+      <c r="O383" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P383" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q383" s="6">
+        <v>0</v>
+      </c>
+      <c r="R383" s="7">
+        <v>0</v>
+      </c>
+      <c r="S383" s="9">
+        <v>0</v>
+      </c>
+      <c r="T383" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U383" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V383" s="11">
+        <v>11</v>
+      </c>
+      <c r="W383" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X383" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y383" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB383" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG383" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI383" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ383" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK383" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM383" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR383" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="384" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A384" s="1">
+        <v>1</v>
+      </c>
+      <c r="B384" s="2">
+        <v>2</v>
+      </c>
+      <c r="C384" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D384" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E384" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F384" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G384" s="5">
+        <v>408</v>
+      </c>
+      <c r="H384" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I384" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J384" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K384" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L384" s="6">
+        <v>695</v>
+      </c>
+      <c r="M384" s="7">
+        <v>136791.85</v>
+      </c>
+      <c r="N384" s="6">
+        <v>1</v>
+      </c>
+      <c r="O384" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P384" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q384" s="6">
+        <v>0</v>
+      </c>
+      <c r="R384" s="7">
+        <v>0</v>
+      </c>
+      <c r="S384" s="9">
+        <v>0</v>
+      </c>
+      <c r="T384" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U384" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V384" s="11">
+        <v>11</v>
+      </c>
+      <c r="W384" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X384" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y384" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB384" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG384" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI384" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ384" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK384" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM384" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR384" s="3" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="385" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A385" s="1">
+        <v>1</v>
+      </c>
+      <c r="B385" s="2">
+        <v>2</v>
+      </c>
+      <c r="C385" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D385" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E385" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F385" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G385" s="5">
+        <v>409</v>
+      </c>
+      <c r="H385" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I385" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J385" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K385" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L385" s="6">
+        <v>696</v>
+      </c>
+      <c r="M385" s="7">
+        <v>136988.67000000001</v>
+      </c>
+      <c r="N385" s="6">
+        <v>1</v>
+      </c>
+      <c r="O385" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P385" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q385" s="6">
+        <v>0</v>
+      </c>
+      <c r="R385" s="7">
+        <v>0</v>
+      </c>
+      <c r="S385" s="9">
+        <v>0</v>
+      </c>
+      <c r="T385" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U385" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V385" s="11">
+        <v>11</v>
+      </c>
+      <c r="W385" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X385" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y385" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB385" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG385" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI385" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ385" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK385" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM385" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR385" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="386" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A386" s="1">
+        <v>1</v>
+      </c>
+      <c r="B386" s="2">
+        <v>2</v>
+      </c>
+      <c r="C386" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D386" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E386" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F386" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G386" s="5">
+        <v>410</v>
+      </c>
+      <c r="H386" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I386" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J386" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K386" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L386" s="6">
+        <v>697</v>
+      </c>
+      <c r="M386" s="7">
+        <v>137185.5</v>
+      </c>
+      <c r="N386" s="6">
+        <v>1</v>
+      </c>
+      <c r="O386" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P386" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q386" s="6">
+        <v>0</v>
+      </c>
+      <c r="R386" s="7">
+        <v>0</v>
+      </c>
+      <c r="S386" s="9">
+        <v>0</v>
+      </c>
+      <c r="T386" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U386" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V386" s="11">
+        <v>11</v>
+      </c>
+      <c r="W386" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X386" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y386" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB386" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG386" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI386" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ386" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK386" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM386" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR386" s="3" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="387" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A387" s="1">
+        <v>1</v>
+      </c>
+      <c r="B387" s="2">
+        <v>2</v>
+      </c>
+      <c r="C387" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D387" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E387" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F387" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G387" s="5">
+        <v>411</v>
+      </c>
+      <c r="H387" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I387" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J387" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K387" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L387" s="6">
+        <v>698</v>
+      </c>
+      <c r="M387" s="7">
+        <v>137382.32</v>
+      </c>
+      <c r="N387" s="6">
+        <v>1</v>
+      </c>
+      <c r="O387" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P387" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q387" s="6">
+        <v>0</v>
+      </c>
+      <c r="R387" s="7">
+        <v>0</v>
+      </c>
+      <c r="S387" s="9">
+        <v>0</v>
+      </c>
+      <c r="T387" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U387" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V387" s="11">
+        <v>11</v>
+      </c>
+      <c r="W387" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X387" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y387" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB387" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG387" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI387" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ387" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK387" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM387" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR387" s="3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="388" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A388" s="1">
+        <v>1</v>
+      </c>
+      <c r="B388" s="2">
+        <v>2</v>
+      </c>
+      <c r="C388" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D388" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E388" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F388" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G388" s="5">
+        <v>412</v>
+      </c>
+      <c r="H388" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I388" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J388" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K388" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L388" s="6">
+        <v>699</v>
+      </c>
+      <c r="M388" s="7">
+        <v>137579.14000000001</v>
+      </c>
+      <c r="N388" s="6">
+        <v>1</v>
+      </c>
+      <c r="O388" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P388" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q388" s="6">
+        <v>0</v>
+      </c>
+      <c r="R388" s="7">
+        <v>0</v>
+      </c>
+      <c r="S388" s="9">
+        <v>0</v>
+      </c>
+      <c r="T388" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U388" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V388" s="11">
+        <v>11</v>
+      </c>
+      <c r="W388" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X388" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y388" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z388" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA388" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB388" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC388" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD388" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE388" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG388" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI388" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ388" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK388" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL388" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM388" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ388" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR388" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="389" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A389" s="1">
+        <v>1</v>
+      </c>
+      <c r="B389" s="2">
+        <v>2</v>
+      </c>
+      <c r="C389" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D389" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E389" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F389" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G389" s="5">
+        <v>413</v>
+      </c>
+      <c r="H389" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I389" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J389" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K389" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L389" s="6">
+        <v>700</v>
+      </c>
+      <c r="M389" s="7">
+        <v>137775.96</v>
+      </c>
+      <c r="N389" s="6">
+        <v>1</v>
+      </c>
+      <c r="O389" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P389" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q389" s="6">
+        <v>0</v>
+      </c>
+      <c r="R389" s="7">
+        <v>0</v>
+      </c>
+      <c r="S389" s="9">
+        <v>0</v>
+      </c>
+      <c r="T389" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U389" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V389" s="11">
+        <v>11</v>
+      </c>
+      <c r="W389" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X389" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y389" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z389" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA389" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB389" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC389" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD389" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE389" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF389" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG389" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH389" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI389" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ389" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK389" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL389" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM389" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN389" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO389" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP389" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ389" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR389" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="390" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A390" s="1">
+        <v>1</v>
+      </c>
+      <c r="B390" s="2">
+        <v>2</v>
+      </c>
+      <c r="C390" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D390" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E390" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F390" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G390" s="5">
+        <v>414</v>
+      </c>
+      <c r="H390" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I390" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J390" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K390" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L390" s="6">
+        <v>701</v>
+      </c>
+      <c r="M390" s="7">
+        <v>137972.79</v>
+      </c>
+      <c r="N390" s="6">
+        <v>1</v>
+      </c>
+      <c r="O390" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P390" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q390" s="6">
+        <v>0</v>
+      </c>
+      <c r="R390" s="7">
+        <v>0</v>
+      </c>
+      <c r="S390" s="9">
+        <v>0</v>
+      </c>
+      <c r="T390" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U390" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V390" s="11">
+        <v>11</v>
+      </c>
+      <c r="W390" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X390" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y390" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z390" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA390" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB390" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC390" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD390" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE390" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF390" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG390" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH390" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI390" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ390" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK390" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL390" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM390" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN390" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO390" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP390" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ390" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR390" s="3" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="391" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A391" s="1">
+        <v>1</v>
+      </c>
+      <c r="B391" s="2">
+        <v>2</v>
+      </c>
+      <c r="C391" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D391" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E391" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F391" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G391" s="5">
+        <v>415</v>
+      </c>
+      <c r="H391" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I391" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J391" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K391" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L391" s="6">
+        <v>702</v>
+      </c>
+      <c r="M391" s="7">
+        <v>138169.60999999999</v>
+      </c>
+      <c r="N391" s="6">
+        <v>1</v>
+      </c>
+      <c r="O391" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P391" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q391" s="6">
+        <v>0</v>
+      </c>
+      <c r="R391" s="7">
+        <v>0</v>
+      </c>
+      <c r="S391" s="9">
+        <v>0</v>
+      </c>
+      <c r="T391" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U391" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V391" s="11">
+        <v>11</v>
+      </c>
+      <c r="W391" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X391" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y391" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z391" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA391" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB391" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC391" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD391" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE391" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF391" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG391" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH391" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI391" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ391" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK391" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL391" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM391" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN391" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO391" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP391" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ391" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR391" s="3" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="392" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A392" s="1">
+        <v>1</v>
+      </c>
+      <c r="B392" s="2">
+        <v>2</v>
+      </c>
+      <c r="C392" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D392" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E392" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F392" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G392" s="5">
+        <v>416</v>
+      </c>
+      <c r="H392" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I392" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J392" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K392" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L392" s="6">
+        <v>703</v>
+      </c>
+      <c r="M392" s="7">
+        <v>138366.43</v>
+      </c>
+      <c r="N392" s="6">
+        <v>1</v>
+      </c>
+      <c r="O392" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P392" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q392" s="6">
+        <v>0</v>
+      </c>
+      <c r="R392" s="7">
+        <v>0</v>
+      </c>
+      <c r="S392" s="9">
+        <v>0</v>
+      </c>
+      <c r="T392" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U392" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V392" s="11">
+        <v>11</v>
+      </c>
+      <c r="W392" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X392" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y392" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z392" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA392" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB392" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC392" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD392" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE392" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF392" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG392" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH392" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI392" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ392" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK392" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL392" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM392" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN392" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO392" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP392" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ392" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR392" s="3" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="393" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A393" s="1">
+        <v>1</v>
+      </c>
+      <c r="B393" s="2">
+        <v>2</v>
+      </c>
+      <c r="C393" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D393" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E393" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F393" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G393" s="5">
+        <v>417</v>
+      </c>
+      <c r="H393" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I393" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J393" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K393" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L393" s="6">
+        <v>704</v>
+      </c>
+      <c r="M393" s="7">
+        <v>138563.25</v>
+      </c>
+      <c r="N393" s="6">
+        <v>1</v>
+      </c>
+      <c r="O393" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P393" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q393" s="6">
+        <v>0</v>
+      </c>
+      <c r="R393" s="7">
+        <v>0</v>
+      </c>
+      <c r="S393" s="9">
+        <v>0</v>
+      </c>
+      <c r="T393" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U393" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V393" s="11">
+        <v>11</v>
+      </c>
+      <c r="W393" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X393" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y393" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z393" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA393" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB393" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC393" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD393" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE393" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF393" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG393" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH393" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI393" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ393" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK393" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL393" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM393" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN393" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO393" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP393" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ393" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR393" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="394" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A394" s="1">
+        <v>1</v>
+      </c>
+      <c r="B394" s="2">
+        <v>2</v>
+      </c>
+      <c r="C394" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D394" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E394" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F394" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G394" s="5">
+        <v>418</v>
+      </c>
+      <c r="H394" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I394" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J394" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K394" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L394" s="6">
+        <v>705</v>
+      </c>
+      <c r="M394" s="7">
+        <v>138760.07999999999</v>
+      </c>
+      <c r="N394" s="6">
+        <v>1</v>
+      </c>
+      <c r="O394" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P394" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q394" s="6">
+        <v>0</v>
+      </c>
+      <c r="R394" s="7">
+        <v>0</v>
+      </c>
+      <c r="S394" s="9">
+        <v>0</v>
+      </c>
+      <c r="T394" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U394" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V394" s="11">
+        <v>11</v>
+      </c>
+      <c r="W394" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X394" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y394" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z394" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA394" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB394" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC394" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD394" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE394" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF394" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG394" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH394" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI394" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ394" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK394" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL394" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM394" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN394" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO394" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP394" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ394" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR394" s="3" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="395" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A395" s="1">
+        <v>1</v>
+      </c>
+      <c r="B395" s="2">
+        <v>2</v>
+      </c>
+      <c r="C395" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D395" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E395" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F395" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G395" s="5">
+        <v>419</v>
+      </c>
+      <c r="H395" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I395" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J395" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K395" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L395" s="6">
+        <v>706</v>
+      </c>
+      <c r="M395" s="7">
+        <v>138956.9</v>
+      </c>
+      <c r="N395" s="6">
+        <v>1</v>
+      </c>
+      <c r="O395" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P395" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q395" s="6">
+        <v>0</v>
+      </c>
+      <c r="R395" s="7">
+        <v>0</v>
+      </c>
+      <c r="S395" s="9">
+        <v>0</v>
+      </c>
+      <c r="T395" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U395" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V395" s="11">
+        <v>11</v>
+      </c>
+      <c r="W395" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X395" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y395" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z395" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA395" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB395" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC395" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD395" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE395" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF395" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG395" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH395" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI395" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ395" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK395" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL395" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM395" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN395" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO395" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP395" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ395" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR395" s="3" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="396" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A396" s="1">
+        <v>1</v>
+      </c>
+      <c r="B396" s="2">
+        <v>2</v>
+      </c>
+      <c r="C396" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D396" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E396" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F396" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G396" s="5">
+        <v>420</v>
+      </c>
+      <c r="H396" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I396" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J396" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K396" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L396" s="6">
+        <v>707</v>
+      </c>
+      <c r="M396" s="7">
+        <v>139153.72</v>
+      </c>
+      <c r="N396" s="6">
+        <v>1</v>
+      </c>
+      <c r="O396" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P396" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q396" s="6">
+        <v>0</v>
+      </c>
+      <c r="R396" s="7">
+        <v>0</v>
+      </c>
+      <c r="S396" s="9">
+        <v>0</v>
+      </c>
+      <c r="T396" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U396" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V396" s="11">
+        <v>11</v>
+      </c>
+      <c r="W396" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X396" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y396" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z396" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA396" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB396" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC396" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD396" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE396" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF396" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG396" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH396" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI396" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ396" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK396" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL396" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM396" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN396" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO396" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP396" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ396" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR396" s="3" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="397" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A397" s="1">
+        <v>1</v>
+      </c>
+      <c r="B397" s="2">
+        <v>2</v>
+      </c>
+      <c r="C397" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D397" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E397" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F397" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G397" s="5">
+        <v>421</v>
+      </c>
+      <c r="H397" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I397" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J397" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K397" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L397" s="6">
+        <v>708</v>
+      </c>
+      <c r="M397" s="7">
+        <v>139350.54999999999</v>
+      </c>
+      <c r="N397" s="6">
+        <v>1</v>
+      </c>
+      <c r="O397" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P397" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q397" s="6">
+        <v>0</v>
+      </c>
+      <c r="R397" s="7">
+        <v>0</v>
+      </c>
+      <c r="S397" s="9">
+        <v>0</v>
+      </c>
+      <c r="T397" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U397" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V397" s="11">
+        <v>11</v>
+      </c>
+      <c r="W397" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X397" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y397" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z397" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA397" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB397" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC397" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD397" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE397" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF397" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG397" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH397" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI397" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ397" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK397" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL397" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM397" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN397" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO397" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP397" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ397" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR397" s="3" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="398" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A398" s="1">
+        <v>1</v>
+      </c>
+      <c r="B398" s="2">
+        <v>2</v>
+      </c>
+      <c r="C398" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D398" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E398" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F398" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G398" s="5">
+        <v>422</v>
+      </c>
+      <c r="H398" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I398" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J398" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K398" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L398" s="6">
+        <v>709</v>
+      </c>
+      <c r="M398" s="7">
+        <v>139547.37</v>
+      </c>
+      <c r="N398" s="6">
+        <v>1</v>
+      </c>
+      <c r="O398" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P398" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q398" s="6">
+        <v>0</v>
+      </c>
+      <c r="R398" s="7">
+        <v>0</v>
+      </c>
+      <c r="S398" s="9">
+        <v>0</v>
+      </c>
+      <c r="T398" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U398" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V398" s="11">
+        <v>11</v>
+      </c>
+      <c r="W398" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X398" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y398" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB398" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG398" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI398" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ398" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK398" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL398" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM398" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ398" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR398" s="3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="399" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A399" s="1">
+        <v>1</v>
+      </c>
+      <c r="B399" s="2">
+        <v>2</v>
+      </c>
+      <c r="C399" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D399" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E399" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F399" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G399" s="5">
+        <v>423</v>
+      </c>
+      <c r="H399" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I399" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J399" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K399" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L399" s="6">
+        <v>710</v>
+      </c>
+      <c r="M399" s="7">
+        <v>139744.19</v>
+      </c>
+      <c r="N399" s="6">
+        <v>1</v>
+      </c>
+      <c r="O399" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P399" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q399" s="6">
+        <v>0</v>
+      </c>
+      <c r="R399" s="7">
+        <v>0</v>
+      </c>
+      <c r="S399" s="9">
+        <v>0</v>
+      </c>
+      <c r="T399" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U399" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V399" s="11">
+        <v>11</v>
+      </c>
+      <c r="W399" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X399" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y399" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB399" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG399" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI399" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ399" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK399" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL399" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM399" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ399" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR399" s="3" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="400" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A400" s="1">
+        <v>1</v>
+      </c>
+      <c r="B400" s="2">
+        <v>2</v>
+      </c>
+      <c r="C400" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D400" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E400" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F400" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G400" s="5">
+        <v>424</v>
+      </c>
+      <c r="H400" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I400" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J400" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K400" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L400" s="6">
+        <v>711</v>
+      </c>
+      <c r="M400" s="7">
+        <v>139941.01</v>
+      </c>
+      <c r="N400" s="6">
+        <v>1</v>
+      </c>
+      <c r="O400" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P400" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q400" s="6">
+        <v>0</v>
+      </c>
+      <c r="R400" s="7">
+        <v>0</v>
+      </c>
+      <c r="S400" s="9">
+        <v>0</v>
+      </c>
+      <c r="T400" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U400" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V400" s="11">
+        <v>11</v>
+      </c>
+      <c r="W400" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X400" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y400" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB400" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG400" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI400" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ400" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK400" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL400" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM400" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ400" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR400" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="401" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A401" s="1">
+        <v>1</v>
+      </c>
+      <c r="B401" s="2">
+        <v>2</v>
+      </c>
+      <c r="C401" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D401" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E401" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F401" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G401" s="5">
+        <v>425</v>
+      </c>
+      <c r="H401" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I401" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J401" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K401" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L401" s="6">
+        <v>712</v>
+      </c>
+      <c r="M401" s="7">
+        <v>140137.84</v>
+      </c>
+      <c r="N401" s="6">
+        <v>1</v>
+      </c>
+      <c r="O401" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P401" s="8">
+        <v>196.82</v>
+      </c>
+      <c r="Q401" s="6">
+        <v>0</v>
+      </c>
+      <c r="R401" s="7">
+        <v>0</v>
+      </c>
+      <c r="S401" s="9">
+        <v>0</v>
+      </c>
+      <c r="T401" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U401" s="10">
+        <v>64144</v>
+      </c>
+      <c r="V401" s="11">
+        <v>11</v>
+      </c>
+      <c r="W401" s="4">
+        <v>46147</v>
+      </c>
+      <c r="X401" s="12">
+        <v>0.67152780000000001</v>
+      </c>
+      <c r="Y401" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB401" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG401" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI401" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ401" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK401" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM401" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR401" s="3" t="s">
+        <v>454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 06/05/2026 12:35:27,30
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BEC1EE8-3696-4E31-8ACE-FCA66F0A2E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5D4D624-1BE5-477F-8A9C-3411996A789C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3554" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4022" uniqueCount="278">
   <si>
     <t>Sel</t>
   </si>
@@ -777,6 +777,84 @@
   <si>
     <t>1858700135868</t>
   </si>
+  <si>
+    <t>1858700135869</t>
+  </si>
+  <si>
+    <t>1858700135870</t>
+  </si>
+  <si>
+    <t>1858700135871</t>
+  </si>
+  <si>
+    <t>1858700135872</t>
+  </si>
+  <si>
+    <t>1858700135873</t>
+  </si>
+  <si>
+    <t>1858700135874</t>
+  </si>
+  <si>
+    <t>1858700135875</t>
+  </si>
+  <si>
+    <t>1858700135876</t>
+  </si>
+  <si>
+    <t>1858700135877</t>
+  </si>
+  <si>
+    <t>1858700135878</t>
+  </si>
+  <si>
+    <t>1858700135879</t>
+  </si>
+  <si>
+    <t>1858700135880</t>
+  </si>
+  <si>
+    <t>1858700135881</t>
+  </si>
+  <si>
+    <t>1858700135882</t>
+  </si>
+  <si>
+    <t>1858700135883</t>
+  </si>
+  <si>
+    <t>1858700135884</t>
+  </si>
+  <si>
+    <t>1858700135885</t>
+  </si>
+  <si>
+    <t>1858700135886</t>
+  </si>
+  <si>
+    <t>1858700135887</t>
+  </si>
+  <si>
+    <t>1858700135888</t>
+  </si>
+  <si>
+    <t>1858700135889</t>
+  </si>
+  <si>
+    <t>1858700135890</t>
+  </si>
+  <si>
+    <t>1858700135891</t>
+  </si>
+  <si>
+    <t>1858700135892</t>
+  </si>
+  <si>
+    <t>1858700135893</t>
+  </si>
+  <si>
+    <t>1858700135894</t>
+  </si>
 </sst>
 </file>
 
@@ -1351,7 +1429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR196"/>
+  <dimension ref="A1:AR222"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -27616,6 +27694,3490 @@
       </c>
       <c r="AR196" s="3" t="s">
         <v>251</v>
+      </c>
+    </row>
+    <row r="197" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A197" s="1">
+        <v>1</v>
+      </c>
+      <c r="B197" s="2">
+        <v>2</v>
+      </c>
+      <c r="C197" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D197" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E197" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F197" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G197" s="5">
+        <v>56</v>
+      </c>
+      <c r="H197" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I197" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J197" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K197" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L197" s="6">
+        <v>511</v>
+      </c>
+      <c r="M197" s="7">
+        <v>96059.01</v>
+      </c>
+      <c r="N197" s="6">
+        <v>1</v>
+      </c>
+      <c r="O197" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P197" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q197" s="6">
+        <v>0</v>
+      </c>
+      <c r="R197" s="7">
+        <v>0</v>
+      </c>
+      <c r="S197" s="9">
+        <v>0</v>
+      </c>
+      <c r="T197" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U197" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V197" s="11">
+        <v>11</v>
+      </c>
+      <c r="W197" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X197" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y197" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB197" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG197" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI197" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ197" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK197" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL197" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM197" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ197" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR197" s="3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="198" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A198" s="1">
+        <v>1</v>
+      </c>
+      <c r="B198" s="2">
+        <v>2</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E198" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F198" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G198" s="5">
+        <v>57</v>
+      </c>
+      <c r="H198" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I198" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J198" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K198" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L198" s="6">
+        <v>512</v>
+      </c>
+      <c r="M198" s="7">
+        <v>96247</v>
+      </c>
+      <c r="N198" s="6">
+        <v>1</v>
+      </c>
+      <c r="O198" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P198" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q198" s="6">
+        <v>0</v>
+      </c>
+      <c r="R198" s="7">
+        <v>0</v>
+      </c>
+      <c r="S198" s="9">
+        <v>0</v>
+      </c>
+      <c r="T198" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U198" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V198" s="11">
+        <v>11</v>
+      </c>
+      <c r="W198" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X198" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y198" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB198" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG198" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI198" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ198" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK198" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL198" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM198" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR198" s="3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="199" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A199" s="1">
+        <v>1</v>
+      </c>
+      <c r="B199" s="2">
+        <v>2</v>
+      </c>
+      <c r="C199" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E199" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F199" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G199" s="5">
+        <v>58</v>
+      </c>
+      <c r="H199" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I199" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J199" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K199" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L199" s="6">
+        <v>513</v>
+      </c>
+      <c r="M199" s="7">
+        <v>96434.98</v>
+      </c>
+      <c r="N199" s="6">
+        <v>1</v>
+      </c>
+      <c r="O199" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P199" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q199" s="6">
+        <v>0</v>
+      </c>
+      <c r="R199" s="7">
+        <v>0</v>
+      </c>
+      <c r="S199" s="9">
+        <v>0</v>
+      </c>
+      <c r="T199" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U199" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V199" s="11">
+        <v>11</v>
+      </c>
+      <c r="W199" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X199" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y199" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB199" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG199" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI199" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ199" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK199" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL199" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM199" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ199" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR199" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="200" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A200" s="1">
+        <v>1</v>
+      </c>
+      <c r="B200" s="2">
+        <v>2</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E200" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F200" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G200" s="5">
+        <v>59</v>
+      </c>
+      <c r="H200" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I200" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J200" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K200" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L200" s="6">
+        <v>514</v>
+      </c>
+      <c r="M200" s="7">
+        <v>96622.96</v>
+      </c>
+      <c r="N200" s="6">
+        <v>1</v>
+      </c>
+      <c r="O200" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P200" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q200" s="6">
+        <v>0</v>
+      </c>
+      <c r="R200" s="7">
+        <v>0</v>
+      </c>
+      <c r="S200" s="9">
+        <v>0</v>
+      </c>
+      <c r="T200" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U200" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V200" s="11">
+        <v>11</v>
+      </c>
+      <c r="W200" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X200" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y200" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB200" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG200" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI200" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ200" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK200" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL200" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM200" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR200" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="201" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A201" s="1">
+        <v>1</v>
+      </c>
+      <c r="B201" s="2">
+        <v>2</v>
+      </c>
+      <c r="C201" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D201" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E201" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F201" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G201" s="5">
+        <v>60</v>
+      </c>
+      <c r="H201" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I201" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J201" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K201" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L201" s="6">
+        <v>515</v>
+      </c>
+      <c r="M201" s="7">
+        <v>96810.94</v>
+      </c>
+      <c r="N201" s="6">
+        <v>1</v>
+      </c>
+      <c r="O201" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P201" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q201" s="6">
+        <v>0</v>
+      </c>
+      <c r="R201" s="7">
+        <v>0</v>
+      </c>
+      <c r="S201" s="9">
+        <v>0</v>
+      </c>
+      <c r="T201" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U201" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V201" s="11">
+        <v>11</v>
+      </c>
+      <c r="W201" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X201" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y201" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB201" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG201" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI201" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ201" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK201" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL201" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM201" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ201" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR201" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="202" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A202" s="1">
+        <v>1</v>
+      </c>
+      <c r="B202" s="2">
+        <v>2</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E202" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F202" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G202" s="5">
+        <v>61</v>
+      </c>
+      <c r="H202" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I202" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J202" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K202" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L202" s="6">
+        <v>516</v>
+      </c>
+      <c r="M202" s="7">
+        <v>96998.93</v>
+      </c>
+      <c r="N202" s="6">
+        <v>1</v>
+      </c>
+      <c r="O202" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P202" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q202" s="6">
+        <v>0</v>
+      </c>
+      <c r="R202" s="7">
+        <v>0</v>
+      </c>
+      <c r="S202" s="9">
+        <v>0</v>
+      </c>
+      <c r="T202" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U202" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V202" s="11">
+        <v>11</v>
+      </c>
+      <c r="W202" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X202" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y202" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB202" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG202" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI202" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ202" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK202" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL202" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM202" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR202" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="203" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A203" s="1">
+        <v>1</v>
+      </c>
+      <c r="B203" s="2">
+        <v>2</v>
+      </c>
+      <c r="C203" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D203" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E203" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F203" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G203" s="5">
+        <v>62</v>
+      </c>
+      <c r="H203" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I203" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J203" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K203" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L203" s="6">
+        <v>517</v>
+      </c>
+      <c r="M203" s="7">
+        <v>97186.91</v>
+      </c>
+      <c r="N203" s="6">
+        <v>1</v>
+      </c>
+      <c r="O203" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P203" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q203" s="6">
+        <v>0</v>
+      </c>
+      <c r="R203" s="7">
+        <v>0</v>
+      </c>
+      <c r="S203" s="9">
+        <v>0</v>
+      </c>
+      <c r="T203" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U203" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V203" s="11">
+        <v>11</v>
+      </c>
+      <c r="W203" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X203" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y203" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB203" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG203" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI203" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ203" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK203" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL203" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM203" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ203" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR203" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="204" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A204" s="1">
+        <v>1</v>
+      </c>
+      <c r="B204" s="2">
+        <v>2</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D204" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E204" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F204" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G204" s="5">
+        <v>63</v>
+      </c>
+      <c r="H204" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I204" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J204" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K204" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L204" s="6">
+        <v>518</v>
+      </c>
+      <c r="M204" s="7">
+        <v>97374.89</v>
+      </c>
+      <c r="N204" s="6">
+        <v>1</v>
+      </c>
+      <c r="O204" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P204" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q204" s="6">
+        <v>0</v>
+      </c>
+      <c r="R204" s="7">
+        <v>0</v>
+      </c>
+      <c r="S204" s="9">
+        <v>0</v>
+      </c>
+      <c r="T204" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U204" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V204" s="11">
+        <v>11</v>
+      </c>
+      <c r="W204" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X204" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y204" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z204" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA204" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB204" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC204" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD204" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE204" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG204" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI204" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ204" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK204" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL204" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM204" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR204" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="205" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A205" s="1">
+        <v>1</v>
+      </c>
+      <c r="B205" s="2">
+        <v>2</v>
+      </c>
+      <c r="C205" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D205" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E205" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F205" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G205" s="5">
+        <v>64</v>
+      </c>
+      <c r="H205" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I205" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J205" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K205" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L205" s="6">
+        <v>519</v>
+      </c>
+      <c r="M205" s="7">
+        <v>97562.87</v>
+      </c>
+      <c r="N205" s="6">
+        <v>1</v>
+      </c>
+      <c r="O205" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P205" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q205" s="6">
+        <v>0</v>
+      </c>
+      <c r="R205" s="7">
+        <v>0</v>
+      </c>
+      <c r="S205" s="9">
+        <v>0</v>
+      </c>
+      <c r="T205" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U205" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V205" s="11">
+        <v>11</v>
+      </c>
+      <c r="W205" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X205" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y205" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z205" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA205" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB205" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC205" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD205" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE205" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF205" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG205" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH205" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI205" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ205" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK205" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL205" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM205" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN205" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO205" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP205" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ205" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR205" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="206" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A206" s="1">
+        <v>1</v>
+      </c>
+      <c r="B206" s="2">
+        <v>2</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D206" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E206" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F206" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G206" s="5">
+        <v>65</v>
+      </c>
+      <c r="H206" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I206" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J206" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K206" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L206" s="6">
+        <v>520</v>
+      </c>
+      <c r="M206" s="7">
+        <v>97750.86</v>
+      </c>
+      <c r="N206" s="6">
+        <v>1</v>
+      </c>
+      <c r="O206" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P206" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q206" s="6">
+        <v>0</v>
+      </c>
+      <c r="R206" s="7">
+        <v>0</v>
+      </c>
+      <c r="S206" s="9">
+        <v>0</v>
+      </c>
+      <c r="T206" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U206" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V206" s="11">
+        <v>11</v>
+      </c>
+      <c r="W206" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X206" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y206" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z206" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA206" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB206" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC206" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD206" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE206" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG206" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI206" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ206" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK206" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL206" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM206" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR206" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="207" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A207" s="1">
+        <v>1</v>
+      </c>
+      <c r="B207" s="2">
+        <v>2</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D207" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E207" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F207" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G207" s="5">
+        <v>66</v>
+      </c>
+      <c r="H207" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I207" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J207" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K207" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L207" s="6">
+        <v>521</v>
+      </c>
+      <c r="M207" s="7">
+        <v>97938.84</v>
+      </c>
+      <c r="N207" s="6">
+        <v>1</v>
+      </c>
+      <c r="O207" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P207" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q207" s="6">
+        <v>0</v>
+      </c>
+      <c r="R207" s="7">
+        <v>0</v>
+      </c>
+      <c r="S207" s="9">
+        <v>0</v>
+      </c>
+      <c r="T207" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U207" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V207" s="11">
+        <v>11</v>
+      </c>
+      <c r="W207" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X207" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y207" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB207" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG207" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI207" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ207" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK207" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM207" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR207" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="208" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A208" s="1">
+        <v>1</v>
+      </c>
+      <c r="B208" s="2">
+        <v>2</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F208" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G208" s="5">
+        <v>67</v>
+      </c>
+      <c r="H208" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I208" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J208" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K208" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L208" s="6">
+        <v>522</v>
+      </c>
+      <c r="M208" s="7">
+        <v>98126.82</v>
+      </c>
+      <c r="N208" s="6">
+        <v>1</v>
+      </c>
+      <c r="O208" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P208" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q208" s="6">
+        <v>0</v>
+      </c>
+      <c r="R208" s="7">
+        <v>0</v>
+      </c>
+      <c r="S208" s="9">
+        <v>0</v>
+      </c>
+      <c r="T208" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U208" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V208" s="11">
+        <v>11</v>
+      </c>
+      <c r="W208" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X208" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y208" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB208" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG208" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI208" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ208" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK208" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM208" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR208" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="209" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A209" s="1">
+        <v>1</v>
+      </c>
+      <c r="B209" s="2">
+        <v>2</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D209" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E209" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F209" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G209" s="5">
+        <v>68</v>
+      </c>
+      <c r="H209" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I209" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J209" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K209" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L209" s="6">
+        <v>523</v>
+      </c>
+      <c r="M209" s="7">
+        <v>98314.8</v>
+      </c>
+      <c r="N209" s="6">
+        <v>1</v>
+      </c>
+      <c r="O209" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P209" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q209" s="6">
+        <v>0</v>
+      </c>
+      <c r="R209" s="7">
+        <v>0</v>
+      </c>
+      <c r="S209" s="9">
+        <v>0</v>
+      </c>
+      <c r="T209" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U209" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V209" s="11">
+        <v>11</v>
+      </c>
+      <c r="W209" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X209" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y209" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z209" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA209" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB209" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC209" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD209" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE209" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF209" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG209" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH209" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI209" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ209" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK209" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL209" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM209" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN209" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO209" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP209" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ209" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR209" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="210" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A210" s="1">
+        <v>1</v>
+      </c>
+      <c r="B210" s="2">
+        <v>2</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D210" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E210" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F210" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G210" s="5">
+        <v>69</v>
+      </c>
+      <c r="H210" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I210" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J210" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K210" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L210" s="6">
+        <v>524</v>
+      </c>
+      <c r="M210" s="7">
+        <v>98502.79</v>
+      </c>
+      <c r="N210" s="6">
+        <v>1</v>
+      </c>
+      <c r="O210" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P210" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q210" s="6">
+        <v>0</v>
+      </c>
+      <c r="R210" s="7">
+        <v>0</v>
+      </c>
+      <c r="S210" s="9">
+        <v>0</v>
+      </c>
+      <c r="T210" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U210" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V210" s="11">
+        <v>11</v>
+      </c>
+      <c r="W210" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X210" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y210" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB210" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG210" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI210" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ210" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK210" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL210" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM210" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ210" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR210" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="211" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A211" s="1">
+        <v>1</v>
+      </c>
+      <c r="B211" s="2">
+        <v>2</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D211" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E211" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F211" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G211" s="5">
+        <v>70</v>
+      </c>
+      <c r="H211" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I211" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J211" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K211" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L211" s="6">
+        <v>525</v>
+      </c>
+      <c r="M211" s="7">
+        <v>98690.77</v>
+      </c>
+      <c r="N211" s="6">
+        <v>1</v>
+      </c>
+      <c r="O211" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P211" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q211" s="6">
+        <v>0</v>
+      </c>
+      <c r="R211" s="7">
+        <v>0</v>
+      </c>
+      <c r="S211" s="9">
+        <v>0</v>
+      </c>
+      <c r="T211" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U211" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V211" s="11">
+        <v>11</v>
+      </c>
+      <c r="W211" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X211" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y211" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB211" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG211" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI211" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ211" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK211" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL211" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM211" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ211" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR211" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="212" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A212" s="1">
+        <v>1</v>
+      </c>
+      <c r="B212" s="2">
+        <v>2</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E212" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F212" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G212" s="5">
+        <v>71</v>
+      </c>
+      <c r="H212" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I212" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J212" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K212" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L212" s="6">
+        <v>526</v>
+      </c>
+      <c r="M212" s="7">
+        <v>98878.75</v>
+      </c>
+      <c r="N212" s="6">
+        <v>1</v>
+      </c>
+      <c r="O212" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P212" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q212" s="6">
+        <v>0</v>
+      </c>
+      <c r="R212" s="7">
+        <v>0</v>
+      </c>
+      <c r="S212" s="9">
+        <v>0</v>
+      </c>
+      <c r="T212" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U212" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V212" s="11">
+        <v>11</v>
+      </c>
+      <c r="W212" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X212" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y212" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB212" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG212" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI212" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ212" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK212" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL212" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM212" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ212" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR212" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="213" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A213" s="1">
+        <v>1</v>
+      </c>
+      <c r="B213" s="2">
+        <v>2</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D213" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E213" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F213" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G213" s="5">
+        <v>72</v>
+      </c>
+      <c r="H213" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I213" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J213" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K213" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L213" s="6">
+        <v>527</v>
+      </c>
+      <c r="M213" s="7">
+        <v>99066.73</v>
+      </c>
+      <c r="N213" s="6">
+        <v>1</v>
+      </c>
+      <c r="O213" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P213" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q213" s="6">
+        <v>0</v>
+      </c>
+      <c r="R213" s="7">
+        <v>0</v>
+      </c>
+      <c r="S213" s="9">
+        <v>0</v>
+      </c>
+      <c r="T213" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U213" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V213" s="11">
+        <v>11</v>
+      </c>
+      <c r="W213" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X213" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y213" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB213" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG213" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI213" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ213" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK213" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL213" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM213" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ213" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR213" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="214" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A214" s="1">
+        <v>1</v>
+      </c>
+      <c r="B214" s="2">
+        <v>2</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E214" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F214" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G214" s="5">
+        <v>73</v>
+      </c>
+      <c r="H214" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I214" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J214" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K214" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L214" s="6">
+        <v>528</v>
+      </c>
+      <c r="M214" s="7">
+        <v>99254.720000000001</v>
+      </c>
+      <c r="N214" s="6">
+        <v>1</v>
+      </c>
+      <c r="O214" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P214" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q214" s="6">
+        <v>0</v>
+      </c>
+      <c r="R214" s="7">
+        <v>0</v>
+      </c>
+      <c r="S214" s="9">
+        <v>0</v>
+      </c>
+      <c r="T214" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U214" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V214" s="11">
+        <v>11</v>
+      </c>
+      <c r="W214" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X214" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y214" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB214" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG214" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI214" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ214" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK214" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL214" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM214" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ214" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR214" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="215" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A215" s="1">
+        <v>1</v>
+      </c>
+      <c r="B215" s="2">
+        <v>2</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D215" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E215" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F215" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G215" s="5">
+        <v>74</v>
+      </c>
+      <c r="H215" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I215" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J215" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K215" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L215" s="6">
+        <v>529</v>
+      </c>
+      <c r="M215" s="7">
+        <v>99442.7</v>
+      </c>
+      <c r="N215" s="6">
+        <v>1</v>
+      </c>
+      <c r="O215" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P215" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q215" s="6">
+        <v>0</v>
+      </c>
+      <c r="R215" s="7">
+        <v>0</v>
+      </c>
+      <c r="S215" s="9">
+        <v>0</v>
+      </c>
+      <c r="T215" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U215" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V215" s="11">
+        <v>11</v>
+      </c>
+      <c r="W215" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X215" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y215" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB215" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG215" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI215" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ215" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK215" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL215" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM215" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ215" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR215" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="216" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A216" s="1">
+        <v>1</v>
+      </c>
+      <c r="B216" s="2">
+        <v>2</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E216" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F216" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G216" s="5">
+        <v>75</v>
+      </c>
+      <c r="H216" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I216" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J216" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K216" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L216" s="6">
+        <v>530</v>
+      </c>
+      <c r="M216" s="7">
+        <v>99630.68</v>
+      </c>
+      <c r="N216" s="6">
+        <v>1</v>
+      </c>
+      <c r="O216" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P216" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q216" s="6">
+        <v>0</v>
+      </c>
+      <c r="R216" s="7">
+        <v>0</v>
+      </c>
+      <c r="S216" s="9">
+        <v>0</v>
+      </c>
+      <c r="T216" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U216" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V216" s="11">
+        <v>11</v>
+      </c>
+      <c r="W216" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X216" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y216" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB216" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG216" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI216" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ216" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK216" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL216" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM216" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ216" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR216" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="217" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A217" s="1">
+        <v>1</v>
+      </c>
+      <c r="B217" s="2">
+        <v>2</v>
+      </c>
+      <c r="C217" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E217" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F217" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G217" s="5">
+        <v>76</v>
+      </c>
+      <c r="H217" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I217" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J217" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K217" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L217" s="6">
+        <v>531</v>
+      </c>
+      <c r="M217" s="7">
+        <v>99818.66</v>
+      </c>
+      <c r="N217" s="6">
+        <v>1</v>
+      </c>
+      <c r="O217" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P217" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q217" s="6">
+        <v>0</v>
+      </c>
+      <c r="R217" s="7">
+        <v>0</v>
+      </c>
+      <c r="S217" s="9">
+        <v>0</v>
+      </c>
+      <c r="T217" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U217" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V217" s="11">
+        <v>11</v>
+      </c>
+      <c r="W217" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X217" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y217" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB217" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG217" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI217" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ217" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK217" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL217" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM217" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ217" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR217" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="218" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A218" s="1">
+        <v>1</v>
+      </c>
+      <c r="B218" s="2">
+        <v>2</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D218" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E218" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F218" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G218" s="5">
+        <v>77</v>
+      </c>
+      <c r="H218" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I218" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J218" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K218" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L218" s="6">
+        <v>532</v>
+      </c>
+      <c r="M218" s="7">
+        <v>100006.65</v>
+      </c>
+      <c r="N218" s="6">
+        <v>1</v>
+      </c>
+      <c r="O218" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P218" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q218" s="6">
+        <v>0</v>
+      </c>
+      <c r="R218" s="7">
+        <v>0</v>
+      </c>
+      <c r="S218" s="9">
+        <v>0</v>
+      </c>
+      <c r="T218" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U218" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V218" s="11">
+        <v>11</v>
+      </c>
+      <c r="W218" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X218" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y218" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB218" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG218" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI218" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ218" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK218" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL218" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM218" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ218" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR218" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="219" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A219" s="1">
+        <v>1</v>
+      </c>
+      <c r="B219" s="2">
+        <v>2</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D219" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E219" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F219" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G219" s="5">
+        <v>78</v>
+      </c>
+      <c r="H219" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I219" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J219" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K219" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L219" s="6">
+        <v>533</v>
+      </c>
+      <c r="M219" s="7">
+        <v>100194.63</v>
+      </c>
+      <c r="N219" s="6">
+        <v>1</v>
+      </c>
+      <c r="O219" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P219" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q219" s="6">
+        <v>0</v>
+      </c>
+      <c r="R219" s="7">
+        <v>0</v>
+      </c>
+      <c r="S219" s="9">
+        <v>0</v>
+      </c>
+      <c r="T219" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U219" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V219" s="11">
+        <v>11</v>
+      </c>
+      <c r="W219" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X219" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y219" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB219" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG219" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI219" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ219" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK219" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL219" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM219" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ219" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR219" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="220" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A220" s="1">
+        <v>1</v>
+      </c>
+      <c r="B220" s="2">
+        <v>2</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E220" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F220" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G220" s="5">
+        <v>79</v>
+      </c>
+      <c r="H220" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I220" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J220" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K220" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L220" s="6">
+        <v>534</v>
+      </c>
+      <c r="M220" s="7">
+        <v>100382.61</v>
+      </c>
+      <c r="N220" s="6">
+        <v>1</v>
+      </c>
+      <c r="O220" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P220" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q220" s="6">
+        <v>0</v>
+      </c>
+      <c r="R220" s="7">
+        <v>0</v>
+      </c>
+      <c r="S220" s="9">
+        <v>0</v>
+      </c>
+      <c r="T220" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U220" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V220" s="11">
+        <v>11</v>
+      </c>
+      <c r="W220" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X220" s="12">
+        <v>0.50486109999999995</v>
+      </c>
+      <c r="Y220" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB220" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG220" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI220" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ220" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK220" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL220" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM220" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ220" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR220" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="221" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A221" s="1">
+        <v>1</v>
+      </c>
+      <c r="B221" s="2">
+        <v>2</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D221" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E221" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F221" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G221" s="5">
+        <v>80</v>
+      </c>
+      <c r="H221" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I221" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J221" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K221" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L221" s="6">
+        <v>535</v>
+      </c>
+      <c r="M221" s="7">
+        <v>100570.59</v>
+      </c>
+      <c r="N221" s="6">
+        <v>1</v>
+      </c>
+      <c r="O221" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P221" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q221" s="6">
+        <v>0</v>
+      </c>
+      <c r="R221" s="7">
+        <v>0</v>
+      </c>
+      <c r="S221" s="9">
+        <v>0</v>
+      </c>
+      <c r="T221" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U221" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V221" s="11">
+        <v>11</v>
+      </c>
+      <c r="W221" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X221" s="12">
+        <v>0.50486109999999995</v>
+      </c>
+      <c r="Y221" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB221" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG221" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI221" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ221" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK221" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL221" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM221" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR221" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="222" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A222" s="1">
+        <v>1</v>
+      </c>
+      <c r="B222" s="2">
+        <v>2</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E222" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F222" s="4">
+        <v>46148</v>
+      </c>
+      <c r="G222" s="5">
+        <v>81</v>
+      </c>
+      <c r="H222" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I222" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J222" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K222" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L222" s="6">
+        <v>536</v>
+      </c>
+      <c r="M222" s="7">
+        <v>100758.57</v>
+      </c>
+      <c r="N222" s="6">
+        <v>1</v>
+      </c>
+      <c r="O222" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="P222" s="8">
+        <v>187.98</v>
+      </c>
+      <c r="Q222" s="6">
+        <v>0</v>
+      </c>
+      <c r="R222" s="7">
+        <v>0</v>
+      </c>
+      <c r="S222" s="9">
+        <v>0</v>
+      </c>
+      <c r="T222" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U222" s="10">
+        <v>64174</v>
+      </c>
+      <c r="V222" s="11">
+        <v>11</v>
+      </c>
+      <c r="W222" s="4">
+        <v>46148</v>
+      </c>
+      <c r="X222" s="12">
+        <v>0.50486109999999995</v>
+      </c>
+      <c r="Y222" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB222" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG222" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI222" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ222" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK222" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL222" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM222" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ222" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR222" s="3" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 07/05/2026 14:01:50,76
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE161816-689B-4CC9-BA23-DEF8D70F76F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0ED81052-1984-4A48-8284-534170816429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4886" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5066" uniqueCount="338">
   <si>
     <t>Sel</t>
   </si>
@@ -1005,6 +1005,36 @@
   <si>
     <t>1881300000040</t>
   </si>
+  <si>
+    <t>1881300000041</t>
+  </si>
+  <si>
+    <t>1881300000042</t>
+  </si>
+  <si>
+    <t>1881300000043</t>
+  </si>
+  <si>
+    <t>1881300000044</t>
+  </si>
+  <si>
+    <t>1881300000045</t>
+  </si>
+  <si>
+    <t>1881300000046</t>
+  </si>
+  <si>
+    <t>1881300000047</t>
+  </si>
+  <si>
+    <t>1881300000048</t>
+  </si>
+  <si>
+    <t>1881300000049</t>
+  </si>
+  <si>
+    <t>1881300000050</t>
+  </si>
 </sst>
 </file>
 
@@ -1579,7 +1609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR270"/>
+  <dimension ref="A1:AR280"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -37760,6 +37790,1346 @@
       </c>
       <c r="AR270" s="3" t="s">
         <v>327</v>
+      </c>
+    </row>
+    <row r="271" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A271" s="1">
+        <v>1</v>
+      </c>
+      <c r="B271" s="2">
+        <v>2</v>
+      </c>
+      <c r="C271" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D271" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E271" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F271" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G271" s="5">
+        <v>40</v>
+      </c>
+      <c r="H271" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I271" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J271" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K271" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L271" s="6">
+        <v>39</v>
+      </c>
+      <c r="M271" s="7">
+        <v>0</v>
+      </c>
+      <c r="N271" s="6">
+        <v>1</v>
+      </c>
+      <c r="O271" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P271" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q271" s="6">
+        <v>0</v>
+      </c>
+      <c r="R271" s="7">
+        <v>0</v>
+      </c>
+      <c r="S271" s="9">
+        <v>0</v>
+      </c>
+      <c r="T271" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U271" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V271" s="11">
+        <v>11</v>
+      </c>
+      <c r="W271" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X271" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y271" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB271" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG271" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI271" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ271" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK271" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL271" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM271" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ271" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR271" s="3" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="272" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A272" s="1">
+        <v>1</v>
+      </c>
+      <c r="B272" s="2">
+        <v>2</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D272" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E272" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F272" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G272" s="5">
+        <v>41</v>
+      </c>
+      <c r="H272" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I272" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J272" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K272" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L272" s="6">
+        <v>40</v>
+      </c>
+      <c r="M272" s="7">
+        <v>0</v>
+      </c>
+      <c r="N272" s="6">
+        <v>1</v>
+      </c>
+      <c r="O272" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P272" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q272" s="6">
+        <v>0</v>
+      </c>
+      <c r="R272" s="7">
+        <v>0</v>
+      </c>
+      <c r="S272" s="9">
+        <v>0</v>
+      </c>
+      <c r="T272" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U272" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V272" s="11">
+        <v>11</v>
+      </c>
+      <c r="W272" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X272" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y272" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB272" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG272" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI272" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ272" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK272" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL272" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM272" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ272" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR272" s="3" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="273" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A273" s="1">
+        <v>1</v>
+      </c>
+      <c r="B273" s="2">
+        <v>2</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D273" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E273" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F273" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G273" s="5">
+        <v>42</v>
+      </c>
+      <c r="H273" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I273" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J273" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K273" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L273" s="6">
+        <v>41</v>
+      </c>
+      <c r="M273" s="7">
+        <v>0</v>
+      </c>
+      <c r="N273" s="6">
+        <v>1</v>
+      </c>
+      <c r="O273" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P273" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q273" s="6">
+        <v>0</v>
+      </c>
+      <c r="R273" s="7">
+        <v>0</v>
+      </c>
+      <c r="S273" s="9">
+        <v>0</v>
+      </c>
+      <c r="T273" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U273" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V273" s="11">
+        <v>11</v>
+      </c>
+      <c r="W273" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X273" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y273" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB273" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG273" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI273" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ273" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK273" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL273" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM273" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ273" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR273" s="3" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="274" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A274" s="1">
+        <v>1</v>
+      </c>
+      <c r="B274" s="2">
+        <v>2</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D274" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E274" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F274" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G274" s="5">
+        <v>43</v>
+      </c>
+      <c r="H274" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I274" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J274" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K274" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L274" s="6">
+        <v>42</v>
+      </c>
+      <c r="M274" s="7">
+        <v>0</v>
+      </c>
+      <c r="N274" s="6">
+        <v>1</v>
+      </c>
+      <c r="O274" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P274" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q274" s="6">
+        <v>0</v>
+      </c>
+      <c r="R274" s="7">
+        <v>0</v>
+      </c>
+      <c r="S274" s="9">
+        <v>0</v>
+      </c>
+      <c r="T274" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U274" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V274" s="11">
+        <v>11</v>
+      </c>
+      <c r="W274" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X274" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y274" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB274" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG274" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI274" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ274" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK274" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL274" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM274" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ274" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR274" s="3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="275" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A275" s="1">
+        <v>1</v>
+      </c>
+      <c r="B275" s="2">
+        <v>2</v>
+      </c>
+      <c r="C275" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D275" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E275" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F275" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G275" s="5">
+        <v>44</v>
+      </c>
+      <c r="H275" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I275" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J275" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K275" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L275" s="6">
+        <v>43</v>
+      </c>
+      <c r="M275" s="7">
+        <v>0</v>
+      </c>
+      <c r="N275" s="6">
+        <v>1</v>
+      </c>
+      <c r="O275" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P275" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q275" s="6">
+        <v>0</v>
+      </c>
+      <c r="R275" s="7">
+        <v>0</v>
+      </c>
+      <c r="S275" s="9">
+        <v>0</v>
+      </c>
+      <c r="T275" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U275" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V275" s="11">
+        <v>11</v>
+      </c>
+      <c r="W275" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X275" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y275" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB275" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG275" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI275" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ275" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK275" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL275" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM275" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ275" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR275" s="3" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="276" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A276" s="1">
+        <v>1</v>
+      </c>
+      <c r="B276" s="2">
+        <v>2</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D276" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E276" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F276" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G276" s="5">
+        <v>45</v>
+      </c>
+      <c r="H276" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I276" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J276" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K276" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L276" s="6">
+        <v>44</v>
+      </c>
+      <c r="M276" s="7">
+        <v>0</v>
+      </c>
+      <c r="N276" s="6">
+        <v>1</v>
+      </c>
+      <c r="O276" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P276" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q276" s="6">
+        <v>0</v>
+      </c>
+      <c r="R276" s="7">
+        <v>0</v>
+      </c>
+      <c r="S276" s="9">
+        <v>0</v>
+      </c>
+      <c r="T276" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U276" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V276" s="11">
+        <v>11</v>
+      </c>
+      <c r="W276" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X276" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y276" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB276" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG276" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI276" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ276" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK276" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL276" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM276" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ276" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR276" s="3" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="277" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A277" s="1">
+        <v>1</v>
+      </c>
+      <c r="B277" s="2">
+        <v>2</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D277" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E277" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F277" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G277" s="5">
+        <v>46</v>
+      </c>
+      <c r="H277" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I277" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J277" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K277" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L277" s="6">
+        <v>45</v>
+      </c>
+      <c r="M277" s="7">
+        <v>0</v>
+      </c>
+      <c r="N277" s="6">
+        <v>1</v>
+      </c>
+      <c r="O277" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P277" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q277" s="6">
+        <v>0</v>
+      </c>
+      <c r="R277" s="7">
+        <v>0</v>
+      </c>
+      <c r="S277" s="9">
+        <v>0</v>
+      </c>
+      <c r="T277" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U277" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V277" s="11">
+        <v>11</v>
+      </c>
+      <c r="W277" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X277" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y277" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB277" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG277" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI277" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ277" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK277" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL277" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM277" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ277" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR277" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="278" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A278" s="1">
+        <v>1</v>
+      </c>
+      <c r="B278" s="2">
+        <v>2</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D278" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E278" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F278" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G278" s="5">
+        <v>47</v>
+      </c>
+      <c r="H278" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I278" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J278" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K278" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L278" s="6">
+        <v>46</v>
+      </c>
+      <c r="M278" s="7">
+        <v>0</v>
+      </c>
+      <c r="N278" s="6">
+        <v>1</v>
+      </c>
+      <c r="O278" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P278" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q278" s="6">
+        <v>0</v>
+      </c>
+      <c r="R278" s="7">
+        <v>0</v>
+      </c>
+      <c r="S278" s="9">
+        <v>0</v>
+      </c>
+      <c r="T278" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U278" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V278" s="11">
+        <v>11</v>
+      </c>
+      <c r="W278" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X278" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y278" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB278" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG278" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI278" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ278" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK278" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL278" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM278" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ278" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR278" s="3" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="279" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A279" s="1">
+        <v>1</v>
+      </c>
+      <c r="B279" s="2">
+        <v>2</v>
+      </c>
+      <c r="C279" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D279" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E279" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F279" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G279" s="5">
+        <v>48</v>
+      </c>
+      <c r="H279" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I279" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J279" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K279" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L279" s="6">
+        <v>47</v>
+      </c>
+      <c r="M279" s="7">
+        <v>0</v>
+      </c>
+      <c r="N279" s="6">
+        <v>1</v>
+      </c>
+      <c r="O279" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P279" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q279" s="6">
+        <v>0</v>
+      </c>
+      <c r="R279" s="7">
+        <v>0</v>
+      </c>
+      <c r="S279" s="9">
+        <v>0</v>
+      </c>
+      <c r="T279" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U279" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V279" s="11">
+        <v>11</v>
+      </c>
+      <c r="W279" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X279" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y279" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB279" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG279" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI279" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ279" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK279" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL279" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM279" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ279" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR279" s="3" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="280" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A280" s="1">
+        <v>1</v>
+      </c>
+      <c r="B280" s="2">
+        <v>2</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D280" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E280" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F280" s="4">
+        <v>46149</v>
+      </c>
+      <c r="G280" s="5">
+        <v>49</v>
+      </c>
+      <c r="H280" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I280" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J280" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K280" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L280" s="6">
+        <v>48</v>
+      </c>
+      <c r="M280" s="7">
+        <v>0</v>
+      </c>
+      <c r="N280" s="6">
+        <v>1</v>
+      </c>
+      <c r="O280" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="P280" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q280" s="6">
+        <v>0</v>
+      </c>
+      <c r="R280" s="7">
+        <v>0</v>
+      </c>
+      <c r="S280" s="9">
+        <v>0</v>
+      </c>
+      <c r="T280" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U280" s="10">
+        <v>64180</v>
+      </c>
+      <c r="V280" s="11">
+        <v>11</v>
+      </c>
+      <c r="W280" s="4">
+        <v>46149</v>
+      </c>
+      <c r="X280" s="12">
+        <v>0.56597220000000004</v>
+      </c>
+      <c r="Y280" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB280" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG280" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI280" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ280" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK280" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM280" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR280" s="3" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 11/05/2026  9:02:43,93
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0381C91E-225A-423A-A887-A258A41F473C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B00D992-9021-4696-8309-1292F04A40A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="63">
   <si>
     <t>Sel</t>
   </si>
@@ -200,6 +200,15 @@
   </si>
   <si>
     <t>1871400011212</t>
+  </si>
+  <si>
+    <t>1871400011213</t>
+  </si>
+  <si>
+    <t>1871400011214</t>
+  </si>
+  <si>
+    <t>1871400011215</t>
   </si>
 </sst>
 </file>
@@ -775,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR6"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -1580,6 +1589,408 @@
       </c>
       <c r="AR6" s="3" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G7" s="5">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" s="6">
+        <v>868</v>
+      </c>
+      <c r="M7" s="7">
+        <v>362836.4</v>
+      </c>
+      <c r="N7" s="6">
+        <v>1</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P7" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q7" s="6">
+        <v>0</v>
+      </c>
+      <c r="R7" s="7">
+        <v>0</v>
+      </c>
+      <c r="S7" s="9">
+        <v>0</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U7" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V7" s="11">
+        <v>11</v>
+      </c>
+      <c r="W7" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X7" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y7" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG7" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK7" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR7" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2">
+        <v>2</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G8" s="5">
+        <v>7</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L8" s="6">
+        <v>869</v>
+      </c>
+      <c r="M8" s="7">
+        <v>363254.42</v>
+      </c>
+      <c r="N8" s="6">
+        <v>1</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P8" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q8" s="6">
+        <v>0</v>
+      </c>
+      <c r="R8" s="7">
+        <v>0</v>
+      </c>
+      <c r="S8" s="9">
+        <v>0</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U8" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V8" s="11">
+        <v>11</v>
+      </c>
+      <c r="W8" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X8" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y8" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG8" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK8" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM8" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR8" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2">
+        <v>2</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G9" s="5">
+        <v>8</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L9" s="6">
+        <v>870</v>
+      </c>
+      <c r="M9" s="7">
+        <v>363672.43</v>
+      </c>
+      <c r="N9" s="6">
+        <v>1</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P9" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="7">
+        <v>0</v>
+      </c>
+      <c r="S9" s="9">
+        <v>0</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U9" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V9" s="11">
+        <v>11</v>
+      </c>
+      <c r="W9" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X9" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y9" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG9" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI9" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK9" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR9" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 11/05/2026  9:51:32,09
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0ED0E235-ADAC-448D-B549-9A9EA43C8CE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15243E96-E8B2-408A-81B9-FC13BA33FB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1772" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2168" uniqueCount="177">
   <si>
     <t>Sel</t>
   </si>
@@ -451,6 +451,63 @@
     <t>1858700136651</t>
   </si>
   <si>
+    <t>1858700136652</t>
+  </si>
+  <si>
+    <t>1858700136653</t>
+  </si>
+  <si>
+    <t>1858700136654</t>
+  </si>
+  <si>
+    <t>1858700136655</t>
+  </si>
+  <si>
+    <t>1858700136656</t>
+  </si>
+  <si>
+    <t>1858700136657</t>
+  </si>
+  <si>
+    <t>1858700136658</t>
+  </si>
+  <si>
+    <t>1858700136659</t>
+  </si>
+  <si>
+    <t>1858700136660</t>
+  </si>
+  <si>
+    <t>1858700136661</t>
+  </si>
+  <si>
+    <t>1858700136662</t>
+  </si>
+  <si>
+    <t>1858700136663</t>
+  </si>
+  <si>
+    <t>1858700136664</t>
+  </si>
+  <si>
+    <t>1858700136665</t>
+  </si>
+  <si>
+    <t>1858700136666</t>
+  </si>
+  <si>
+    <t>1858700136667</t>
+  </si>
+  <si>
+    <t>1858700136668</t>
+  </si>
+  <si>
+    <t>1858700136669</t>
+  </si>
+  <si>
+    <t>1858700136670</t>
+  </si>
+  <si>
     <t>10016354</t>
   </si>
   <si>
@@ -485,6 +542,15 @@
   </si>
   <si>
     <t>1871400011215</t>
+  </si>
+  <si>
+    <t>1871400011216</t>
+  </si>
+  <si>
+    <t>1871400011217</t>
+  </si>
+  <si>
+    <t>1871400011218</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR97"/>
+  <dimension ref="A1:AR119"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -12997,10 +13063,10 @@
         <v>2</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>46</v>
@@ -13009,7 +13075,7 @@
         <v>46153</v>
       </c>
       <c r="G90" s="5">
-        <v>1</v>
+        <v>198</v>
       </c>
       <c r="H90" s="3" t="s">
         <v>47</v>
@@ -13024,19 +13090,19 @@
         <v>50</v>
       </c>
       <c r="L90" s="6">
-        <v>863</v>
+        <v>734</v>
       </c>
       <c r="M90" s="7">
-        <v>360746.33</v>
+        <v>138602.35999999999</v>
       </c>
       <c r="N90" s="6">
         <v>1</v>
       </c>
       <c r="O90" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P90" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q90" s="6">
         <v>0</v>
@@ -13051,7 +13117,7 @@
         <v>52</v>
       </c>
       <c r="U90" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V90" s="11">
         <v>11</v>
@@ -13060,7 +13126,7 @@
         <v>46153</v>
       </c>
       <c r="X90" s="12">
-        <v>0.31597219999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y90" s="10">
         <v>0</v>
@@ -13093,7 +13159,7 @@
         <v>53</v>
       </c>
       <c r="AI90" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="AJ90" s="3" t="s">
         <v>52</v>
@@ -13120,7 +13186,7 @@
         <v>53</v>
       </c>
       <c r="AR90" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="91" spans="1:44" x14ac:dyDescent="0.3">
@@ -13131,10 +13197,10 @@
         <v>2</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>46</v>
@@ -13143,7 +13209,7 @@
         <v>46153</v>
       </c>
       <c r="G91" s="5">
-        <v>2</v>
+        <v>199</v>
       </c>
       <c r="H91" s="3" t="s">
         <v>47</v>
@@ -13158,19 +13224,19 @@
         <v>50</v>
       </c>
       <c r="L91" s="6">
-        <v>864</v>
+        <v>735</v>
       </c>
       <c r="M91" s="7">
-        <v>361164.35</v>
+        <v>138791.19</v>
       </c>
       <c r="N91" s="6">
         <v>1</v>
       </c>
       <c r="O91" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P91" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q91" s="6">
         <v>0</v>
@@ -13185,7 +13251,7 @@
         <v>52</v>
       </c>
       <c r="U91" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V91" s="11">
         <v>11</v>
@@ -13194,7 +13260,7 @@
         <v>46153</v>
       </c>
       <c r="X91" s="12">
-        <v>0.31597219999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y91" s="10">
         <v>0</v>
@@ -13227,7 +13293,7 @@
         <v>53</v>
       </c>
       <c r="AI91" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="AJ91" s="3" t="s">
         <v>52</v>
@@ -13254,7 +13320,7 @@
         <v>53</v>
       </c>
       <c r="AR91" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="92" spans="1:44" x14ac:dyDescent="0.3">
@@ -13265,10 +13331,10 @@
         <v>2</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>46</v>
@@ -13277,7 +13343,7 @@
         <v>46153</v>
       </c>
       <c r="G92" s="5">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>47</v>
@@ -13292,19 +13358,19 @@
         <v>50</v>
       </c>
       <c r="L92" s="6">
-        <v>865</v>
+        <v>736</v>
       </c>
       <c r="M92" s="7">
-        <v>361582.36</v>
+        <v>138980.01999999999</v>
       </c>
       <c r="N92" s="6">
         <v>1</v>
       </c>
       <c r="O92" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P92" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q92" s="6">
         <v>0</v>
@@ -13319,7 +13385,7 @@
         <v>52</v>
       </c>
       <c r="U92" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V92" s="11">
         <v>11</v>
@@ -13328,7 +13394,7 @@
         <v>46153</v>
       </c>
       <c r="X92" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y92" s="10">
         <v>0</v>
@@ -13361,7 +13427,7 @@
         <v>53</v>
       </c>
       <c r="AI92" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="AJ92" s="3" t="s">
         <v>52</v>
@@ -13388,7 +13454,7 @@
         <v>53</v>
       </c>
       <c r="AR92" s="3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="93" spans="1:44" x14ac:dyDescent="0.3">
@@ -13399,10 +13465,10 @@
         <v>2</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>46</v>
@@ -13411,7 +13477,7 @@
         <v>46153</v>
       </c>
       <c r="G93" s="5">
-        <v>4</v>
+        <v>201</v>
       </c>
       <c r="H93" s="3" t="s">
         <v>47</v>
@@ -13426,19 +13492,19 @@
         <v>50</v>
       </c>
       <c r="L93" s="6">
-        <v>866</v>
+        <v>737</v>
       </c>
       <c r="M93" s="7">
-        <v>362000.38</v>
+        <v>139168.85</v>
       </c>
       <c r="N93" s="6">
         <v>1</v>
       </c>
       <c r="O93" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P93" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q93" s="6">
         <v>0</v>
@@ -13453,7 +13519,7 @@
         <v>52</v>
       </c>
       <c r="U93" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V93" s="11">
         <v>11</v>
@@ -13462,7 +13528,7 @@
         <v>46153</v>
       </c>
       <c r="X93" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y93" s="10">
         <v>0</v>
@@ -13495,34 +13561,34 @@
         <v>53</v>
       </c>
       <c r="AI93" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ93" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK93" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM93" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR93" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="AJ93" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK93" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL93" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM93" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN93" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO93" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP93" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ93" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR93" s="3" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="94" spans="1:44" x14ac:dyDescent="0.3">
@@ -13533,10 +13599,10 @@
         <v>2</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E94" s="3" t="s">
         <v>46</v>
@@ -13545,7 +13611,7 @@
         <v>46153</v>
       </c>
       <c r="G94" s="5">
-        <v>5</v>
+        <v>202</v>
       </c>
       <c r="H94" s="3" t="s">
         <v>47</v>
@@ -13560,19 +13626,19 @@
         <v>50</v>
       </c>
       <c r="L94" s="6">
-        <v>867</v>
+        <v>738</v>
       </c>
       <c r="M94" s="7">
-        <v>362418.39</v>
+        <v>139357.68</v>
       </c>
       <c r="N94" s="6">
         <v>1</v>
       </c>
       <c r="O94" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P94" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q94" s="6">
         <v>0</v>
@@ -13587,7 +13653,7 @@
         <v>52</v>
       </c>
       <c r="U94" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V94" s="11">
         <v>11</v>
@@ -13596,7 +13662,7 @@
         <v>46153</v>
       </c>
       <c r="X94" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y94" s="10">
         <v>0</v>
@@ -13629,7 +13695,7 @@
         <v>53</v>
       </c>
       <c r="AI94" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="AJ94" s="3" t="s">
         <v>52</v>
@@ -13656,7 +13722,7 @@
         <v>53</v>
       </c>
       <c r="AR94" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="95" spans="1:44" x14ac:dyDescent="0.3">
@@ -13667,10 +13733,10 @@
         <v>2</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>46</v>
@@ -13679,7 +13745,7 @@
         <v>46153</v>
       </c>
       <c r="G95" s="5">
-        <v>6</v>
+        <v>203</v>
       </c>
       <c r="H95" s="3" t="s">
         <v>47</v>
@@ -13694,19 +13760,19 @@
         <v>50</v>
       </c>
       <c r="L95" s="6">
-        <v>868</v>
+        <v>739</v>
       </c>
       <c r="M95" s="7">
-        <v>362836.4</v>
+        <v>139546.51</v>
       </c>
       <c r="N95" s="6">
         <v>1</v>
       </c>
       <c r="O95" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P95" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q95" s="6">
         <v>0</v>
@@ -13721,7 +13787,7 @@
         <v>52</v>
       </c>
       <c r="U95" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V95" s="11">
         <v>11</v>
@@ -13730,7 +13796,7 @@
         <v>46153</v>
       </c>
       <c r="X95" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y95" s="10">
         <v>0</v>
@@ -13763,7 +13829,7 @@
         <v>53</v>
       </c>
       <c r="AI95" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="AJ95" s="3" t="s">
         <v>52</v>
@@ -13790,7 +13856,7 @@
         <v>53</v>
       </c>
       <c r="AR95" s="3" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="96" spans="1:44" x14ac:dyDescent="0.3">
@@ -13801,10 +13867,10 @@
         <v>2</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>46</v>
@@ -13813,7 +13879,7 @@
         <v>46153</v>
       </c>
       <c r="G96" s="5">
-        <v>7</v>
+        <v>204</v>
       </c>
       <c r="H96" s="3" t="s">
         <v>47</v>
@@ -13828,19 +13894,19 @@
         <v>50</v>
       </c>
       <c r="L96" s="6">
-        <v>869</v>
+        <v>740</v>
       </c>
       <c r="M96" s="7">
-        <v>363254.42</v>
+        <v>139735.35</v>
       </c>
       <c r="N96" s="6">
         <v>1</v>
       </c>
       <c r="O96" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P96" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q96" s="6">
         <v>0</v>
@@ -13855,7 +13921,7 @@
         <v>52</v>
       </c>
       <c r="U96" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V96" s="11">
         <v>11</v>
@@ -13864,7 +13930,7 @@
         <v>46153</v>
       </c>
       <c r="X96" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.39930559999999998</v>
       </c>
       <c r="Y96" s="10">
         <v>0</v>
@@ -13897,7 +13963,7 @@
         <v>53</v>
       </c>
       <c r="AI96" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="AJ96" s="3" t="s">
         <v>52</v>
@@ -13924,7 +13990,7 @@
         <v>53</v>
       </c>
       <c r="AR96" s="3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="97" spans="1:44" x14ac:dyDescent="0.3">
@@ -13935,10 +14001,10 @@
         <v>2</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>46</v>
@@ -13947,7 +14013,7 @@
         <v>46153</v>
       </c>
       <c r="G97" s="5">
-        <v>8</v>
+        <v>205</v>
       </c>
       <c r="H97" s="3" t="s">
         <v>47</v>
@@ -13962,19 +14028,19 @@
         <v>50</v>
       </c>
       <c r="L97" s="6">
-        <v>870</v>
+        <v>741</v>
       </c>
       <c r="M97" s="7">
-        <v>363672.43</v>
+        <v>139924.18</v>
       </c>
       <c r="N97" s="6">
         <v>1</v>
       </c>
       <c r="O97" s="3" t="s">
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="P97" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q97" s="6">
         <v>0</v>
@@ -13989,7 +14055,7 @@
         <v>52</v>
       </c>
       <c r="U97" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V97" s="11">
         <v>11</v>
@@ -13998,67 +14064,3015 @@
         <v>46153</v>
       </c>
       <c r="X97" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y97" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB97" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG97" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI97" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ97" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK97" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM97" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR97" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="98" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A98" s="1">
+        <v>1</v>
+      </c>
+      <c r="B98" s="2">
+        <v>2</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E98" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F98" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G98" s="5">
+        <v>206</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I98" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J98" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K98" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L98" s="6">
+        <v>742</v>
+      </c>
+      <c r="M98" s="7">
+        <v>140113.01</v>
+      </c>
+      <c r="N98" s="6">
+        <v>1</v>
+      </c>
+      <c r="O98" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P98" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q98" s="6">
+        <v>0</v>
+      </c>
+      <c r="R98" s="7">
+        <v>0</v>
+      </c>
+      <c r="S98" s="9">
+        <v>0</v>
+      </c>
+      <c r="T98" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U98" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V98" s="11">
+        <v>11</v>
+      </c>
+      <c r="W98" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X98" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y98" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB98" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG98" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI98" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ98" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK98" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM98" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR98" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="99" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A99" s="1">
+        <v>1</v>
+      </c>
+      <c r="B99" s="2">
+        <v>2</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F99" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G99" s="5">
+        <v>207</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J99" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K99" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L99" s="6">
+        <v>743</v>
+      </c>
+      <c r="M99" s="7">
+        <v>140301.84</v>
+      </c>
+      <c r="N99" s="6">
+        <v>1</v>
+      </c>
+      <c r="O99" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P99" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q99" s="6">
+        <v>0</v>
+      </c>
+      <c r="R99" s="7">
+        <v>0</v>
+      </c>
+      <c r="S99" s="9">
+        <v>0</v>
+      </c>
+      <c r="T99" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U99" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V99" s="11">
+        <v>11</v>
+      </c>
+      <c r="W99" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X99" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y99" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB99" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG99" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI99" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ99" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK99" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM99" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR99" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="100" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A100" s="1">
+        <v>1</v>
+      </c>
+      <c r="B100" s="2">
+        <v>2</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F100" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G100" s="5">
+        <v>208</v>
+      </c>
+      <c r="H100" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I100" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J100" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K100" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L100" s="6">
+        <v>744</v>
+      </c>
+      <c r="M100" s="7">
+        <v>140490.67000000001</v>
+      </c>
+      <c r="N100" s="6">
+        <v>1</v>
+      </c>
+      <c r="O100" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P100" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q100" s="6">
+        <v>0</v>
+      </c>
+      <c r="R100" s="7">
+        <v>0</v>
+      </c>
+      <c r="S100" s="9">
+        <v>0</v>
+      </c>
+      <c r="T100" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U100" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V100" s="11">
+        <v>11</v>
+      </c>
+      <c r="W100" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X100" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y100" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB100" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG100" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI100" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ100" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK100" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM100" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR100" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="101" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A101" s="1">
+        <v>1</v>
+      </c>
+      <c r="B101" s="2">
+        <v>2</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F101" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G101" s="5">
+        <v>209</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I101" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J101" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K101" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L101" s="6">
+        <v>745</v>
+      </c>
+      <c r="M101" s="7">
+        <v>140679.5</v>
+      </c>
+      <c r="N101" s="6">
+        <v>1</v>
+      </c>
+      <c r="O101" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P101" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q101" s="6">
+        <v>0</v>
+      </c>
+      <c r="R101" s="7">
+        <v>0</v>
+      </c>
+      <c r="S101" s="9">
+        <v>0</v>
+      </c>
+      <c r="T101" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U101" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V101" s="11">
+        <v>11</v>
+      </c>
+      <c r="W101" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X101" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y101" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB101" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG101" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI101" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ101" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK101" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM101" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR101" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="102" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A102" s="1">
+        <v>1</v>
+      </c>
+      <c r="B102" s="2">
+        <v>2</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F102" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G102" s="5">
+        <v>210</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I102" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J102" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K102" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L102" s="6">
+        <v>746</v>
+      </c>
+      <c r="M102" s="7">
+        <v>140868.32999999999</v>
+      </c>
+      <c r="N102" s="6">
+        <v>1</v>
+      </c>
+      <c r="O102" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P102" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q102" s="6">
+        <v>0</v>
+      </c>
+      <c r="R102" s="7">
+        <v>0</v>
+      </c>
+      <c r="S102" s="9">
+        <v>0</v>
+      </c>
+      <c r="T102" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U102" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V102" s="11">
+        <v>11</v>
+      </c>
+      <c r="W102" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X102" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y102" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB102" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG102" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI102" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ102" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK102" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM102" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR102" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="103" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>1</v>
+      </c>
+      <c r="B103" s="2">
+        <v>2</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F103" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G103" s="5">
+        <v>211</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I103" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J103" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K103" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L103" s="6">
+        <v>747</v>
+      </c>
+      <c r="M103" s="7">
+        <v>141057.17000000001</v>
+      </c>
+      <c r="N103" s="6">
+        <v>1</v>
+      </c>
+      <c r="O103" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P103" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q103" s="6">
+        <v>0</v>
+      </c>
+      <c r="R103" s="7">
+        <v>0</v>
+      </c>
+      <c r="S103" s="9">
+        <v>0</v>
+      </c>
+      <c r="T103" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U103" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V103" s="11">
+        <v>11</v>
+      </c>
+      <c r="W103" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X103" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y103" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB103" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG103" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI103" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ103" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK103" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM103" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR103" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="104" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
+        <v>1</v>
+      </c>
+      <c r="B104" s="2">
+        <v>2</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F104" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G104" s="5">
+        <v>212</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I104" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J104" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K104" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L104" s="6">
+        <v>748</v>
+      </c>
+      <c r="M104" s="7">
+        <v>141246</v>
+      </c>
+      <c r="N104" s="6">
+        <v>1</v>
+      </c>
+      <c r="O104" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P104" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q104" s="6">
+        <v>0</v>
+      </c>
+      <c r="R104" s="7">
+        <v>0</v>
+      </c>
+      <c r="S104" s="9">
+        <v>0</v>
+      </c>
+      <c r="T104" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U104" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V104" s="11">
+        <v>11</v>
+      </c>
+      <c r="W104" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X104" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y104" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB104" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG104" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI104" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ104" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK104" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM104" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR104" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="105" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A105" s="1">
+        <v>1</v>
+      </c>
+      <c r="B105" s="2">
+        <v>2</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F105" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G105" s="5">
+        <v>213</v>
+      </c>
+      <c r="H105" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I105" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J105" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K105" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L105" s="6">
+        <v>749</v>
+      </c>
+      <c r="M105" s="7">
+        <v>141434.82999999999</v>
+      </c>
+      <c r="N105" s="6">
+        <v>1</v>
+      </c>
+      <c r="O105" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P105" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q105" s="6">
+        <v>0</v>
+      </c>
+      <c r="R105" s="7">
+        <v>0</v>
+      </c>
+      <c r="S105" s="9">
+        <v>0</v>
+      </c>
+      <c r="T105" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U105" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V105" s="11">
+        <v>11</v>
+      </c>
+      <c r="W105" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X105" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y105" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB105" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG105" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI105" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ105" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK105" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM105" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR105" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="106" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A106" s="1">
+        <v>1</v>
+      </c>
+      <c r="B106" s="2">
+        <v>2</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F106" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G106" s="5">
+        <v>214</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I106" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J106" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K106" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L106" s="6">
+        <v>750</v>
+      </c>
+      <c r="M106" s="7">
+        <v>141623.66</v>
+      </c>
+      <c r="N106" s="6">
+        <v>1</v>
+      </c>
+      <c r="O106" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P106" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q106" s="6">
+        <v>0</v>
+      </c>
+      <c r="R106" s="7">
+        <v>0</v>
+      </c>
+      <c r="S106" s="9">
+        <v>0</v>
+      </c>
+      <c r="T106" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U106" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V106" s="11">
+        <v>11</v>
+      </c>
+      <c r="W106" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X106" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y106" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB106" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG106" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI106" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ106" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK106" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM106" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR106" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="107" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A107" s="1">
+        <v>1</v>
+      </c>
+      <c r="B107" s="2">
+        <v>2</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F107" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G107" s="5">
+        <v>215</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I107" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J107" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K107" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L107" s="6">
+        <v>751</v>
+      </c>
+      <c r="M107" s="7">
+        <v>141812.49</v>
+      </c>
+      <c r="N107" s="6">
+        <v>1</v>
+      </c>
+      <c r="O107" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P107" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q107" s="6">
+        <v>0</v>
+      </c>
+      <c r="R107" s="7">
+        <v>0</v>
+      </c>
+      <c r="S107" s="9">
+        <v>0</v>
+      </c>
+      <c r="T107" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U107" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V107" s="11">
+        <v>11</v>
+      </c>
+      <c r="W107" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X107" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y107" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB107" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG107" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI107" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ107" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK107" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM107" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR107" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="108" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A108" s="1">
+        <v>1</v>
+      </c>
+      <c r="B108" s="2">
+        <v>2</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F108" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G108" s="5">
+        <v>216</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I108" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J108" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K108" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L108" s="6">
+        <v>752</v>
+      </c>
+      <c r="M108" s="7">
+        <v>142001.32</v>
+      </c>
+      <c r="N108" s="6">
+        <v>1</v>
+      </c>
+      <c r="O108" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P108" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q108" s="6">
+        <v>0</v>
+      </c>
+      <c r="R108" s="7">
+        <v>0</v>
+      </c>
+      <c r="S108" s="9">
+        <v>0</v>
+      </c>
+      <c r="T108" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U108" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V108" s="11">
+        <v>11</v>
+      </c>
+      <c r="W108" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X108" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y108" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB108" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG108" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI108" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ108" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK108" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM108" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR108" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="109" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A109" s="1">
+        <v>1</v>
+      </c>
+      <c r="B109" s="2">
+        <v>2</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F109" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G109" s="5">
+        <v>1</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I109" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J109" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K109" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L109" s="6">
+        <v>863</v>
+      </c>
+      <c r="M109" s="7">
+        <v>360746.33</v>
+      </c>
+      <c r="N109" s="6">
+        <v>1</v>
+      </c>
+      <c r="O109" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P109" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q109" s="6">
+        <v>0</v>
+      </c>
+      <c r="R109" s="7">
+        <v>0</v>
+      </c>
+      <c r="S109" s="9">
+        <v>0</v>
+      </c>
+      <c r="T109" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U109" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V109" s="11">
+        <v>11</v>
+      </c>
+      <c r="W109" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X109" s="12">
+        <v>0.31597219999999998</v>
+      </c>
+      <c r="Y109" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB109" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG109" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI109" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ109" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK109" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM109" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR109" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="110" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
+        <v>1</v>
+      </c>
+      <c r="B110" s="2">
+        <v>2</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F110" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G110" s="5">
+        <v>2</v>
+      </c>
+      <c r="H110" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I110" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J110" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K110" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L110" s="6">
+        <v>864</v>
+      </c>
+      <c r="M110" s="7">
+        <v>361164.35</v>
+      </c>
+      <c r="N110" s="6">
+        <v>1</v>
+      </c>
+      <c r="O110" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P110" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q110" s="6">
+        <v>0</v>
+      </c>
+      <c r="R110" s="7">
+        <v>0</v>
+      </c>
+      <c r="S110" s="9">
+        <v>0</v>
+      </c>
+      <c r="T110" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U110" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V110" s="11">
+        <v>11</v>
+      </c>
+      <c r="W110" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X110" s="12">
+        <v>0.31597219999999998</v>
+      </c>
+      <c r="Y110" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB110" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG110" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI110" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ110" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK110" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM110" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR110" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="111" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
+        <v>1</v>
+      </c>
+      <c r="B111" s="2">
+        <v>2</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F111" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G111" s="5">
+        <v>3</v>
+      </c>
+      <c r="H111" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I111" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J111" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K111" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L111" s="6">
+        <v>865</v>
+      </c>
+      <c r="M111" s="7">
+        <v>361582.36</v>
+      </c>
+      <c r="N111" s="6">
+        <v>1</v>
+      </c>
+      <c r="O111" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P111" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q111" s="6">
+        <v>0</v>
+      </c>
+      <c r="R111" s="7">
+        <v>0</v>
+      </c>
+      <c r="S111" s="9">
+        <v>0</v>
+      </c>
+      <c r="T111" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U111" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V111" s="11">
+        <v>11</v>
+      </c>
+      <c r="W111" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X111" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y111" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB111" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG111" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI111" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ111" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK111" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM111" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR111" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="112" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A112" s="1">
+        <v>1</v>
+      </c>
+      <c r="B112" s="2">
+        <v>2</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F112" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G112" s="5">
+        <v>4</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I112" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J112" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K112" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L112" s="6">
+        <v>866</v>
+      </c>
+      <c r="M112" s="7">
+        <v>362000.38</v>
+      </c>
+      <c r="N112" s="6">
+        <v>1</v>
+      </c>
+      <c r="O112" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P112" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q112" s="6">
+        <v>0</v>
+      </c>
+      <c r="R112" s="7">
+        <v>0</v>
+      </c>
+      <c r="S112" s="9">
+        <v>0</v>
+      </c>
+      <c r="T112" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U112" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V112" s="11">
+        <v>11</v>
+      </c>
+      <c r="W112" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X112" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y112" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB112" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG112" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI112" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ112" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK112" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM112" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR112" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="113" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
+        <v>1</v>
+      </c>
+      <c r="B113" s="2">
+        <v>2</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E113" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F113" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G113" s="5">
+        <v>5</v>
+      </c>
+      <c r="H113" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J113" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K113" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L113" s="6">
+        <v>867</v>
+      </c>
+      <c r="M113" s="7">
+        <v>362418.39</v>
+      </c>
+      <c r="N113" s="6">
+        <v>1</v>
+      </c>
+      <c r="O113" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P113" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q113" s="6">
+        <v>0</v>
+      </c>
+      <c r="R113" s="7">
+        <v>0</v>
+      </c>
+      <c r="S113" s="9">
+        <v>0</v>
+      </c>
+      <c r="T113" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U113" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V113" s="11">
+        <v>11</v>
+      </c>
+      <c r="W113" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X113" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y113" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB113" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG113" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI113" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ113" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK113" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM113" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR113" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="114" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
+        <v>1</v>
+      </c>
+      <c r="B114" s="2">
+        <v>2</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F114" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G114" s="5">
+        <v>6</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I114" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J114" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K114" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L114" s="6">
+        <v>868</v>
+      </c>
+      <c r="M114" s="7">
+        <v>362836.4</v>
+      </c>
+      <c r="N114" s="6">
+        <v>1</v>
+      </c>
+      <c r="O114" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P114" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q114" s="6">
+        <v>0</v>
+      </c>
+      <c r="R114" s="7">
+        <v>0</v>
+      </c>
+      <c r="S114" s="9">
+        <v>0</v>
+      </c>
+      <c r="T114" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U114" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V114" s="11">
+        <v>11</v>
+      </c>
+      <c r="W114" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X114" s="12">
         <v>0.35763889999999998</v>
       </c>
-      <c r="Y97" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z97" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA97" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB97" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC97" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD97" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE97" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF97" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG97" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH97" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI97" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="AJ97" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK97" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL97" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM97" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN97" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO97" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP97" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ97" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR97" s="3" t="s">
-        <v>154</v>
+      <c r="Y114" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB114" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG114" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI114" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ114" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK114" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM114" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR114" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="115" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
+        <v>1</v>
+      </c>
+      <c r="B115" s="2">
+        <v>2</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F115" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G115" s="5">
+        <v>7</v>
+      </c>
+      <c r="H115" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I115" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J115" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K115" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L115" s="6">
+        <v>869</v>
+      </c>
+      <c r="M115" s="7">
+        <v>363254.42</v>
+      </c>
+      <c r="N115" s="6">
+        <v>1</v>
+      </c>
+      <c r="O115" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P115" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q115" s="6">
+        <v>0</v>
+      </c>
+      <c r="R115" s="7">
+        <v>0</v>
+      </c>
+      <c r="S115" s="9">
+        <v>0</v>
+      </c>
+      <c r="T115" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U115" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V115" s="11">
+        <v>11</v>
+      </c>
+      <c r="W115" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X115" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y115" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB115" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG115" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI115" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ115" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK115" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM115" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR115" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="116" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
+        <v>1</v>
+      </c>
+      <c r="B116" s="2">
+        <v>2</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F116" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G116" s="5">
+        <v>8</v>
+      </c>
+      <c r="H116" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I116" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J116" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K116" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L116" s="6">
+        <v>870</v>
+      </c>
+      <c r="M116" s="7">
+        <v>363672.43</v>
+      </c>
+      <c r="N116" s="6">
+        <v>1</v>
+      </c>
+      <c r="O116" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P116" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q116" s="6">
+        <v>0</v>
+      </c>
+      <c r="R116" s="7">
+        <v>0</v>
+      </c>
+      <c r="S116" s="9">
+        <v>0</v>
+      </c>
+      <c r="T116" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U116" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V116" s="11">
+        <v>11</v>
+      </c>
+      <c r="W116" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X116" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y116" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB116" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG116" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI116" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ116" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK116" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM116" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR116" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="117" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>1</v>
+      </c>
+      <c r="B117" s="2">
+        <v>2</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F117" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G117" s="5">
+        <v>9</v>
+      </c>
+      <c r="H117" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I117" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J117" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K117" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L117" s="6">
+        <v>871</v>
+      </c>
+      <c r="M117" s="7">
+        <v>364090.45</v>
+      </c>
+      <c r="N117" s="6">
+        <v>1</v>
+      </c>
+      <c r="O117" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P117" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q117" s="6">
+        <v>0</v>
+      </c>
+      <c r="R117" s="7">
+        <v>0</v>
+      </c>
+      <c r="S117" s="9">
+        <v>0</v>
+      </c>
+      <c r="T117" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U117" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V117" s="11">
+        <v>11</v>
+      </c>
+      <c r="W117" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X117" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y117" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB117" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG117" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI117" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ117" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK117" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM117" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR117" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="118" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>1</v>
+      </c>
+      <c r="B118" s="2">
+        <v>2</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F118" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G118" s="5">
+        <v>10</v>
+      </c>
+      <c r="H118" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I118" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J118" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K118" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L118" s="6">
+        <v>872</v>
+      </c>
+      <c r="M118" s="7">
+        <v>364508.46</v>
+      </c>
+      <c r="N118" s="6">
+        <v>1</v>
+      </c>
+      <c r="O118" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P118" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q118" s="6">
+        <v>0</v>
+      </c>
+      <c r="R118" s="7">
+        <v>0</v>
+      </c>
+      <c r="S118" s="9">
+        <v>0</v>
+      </c>
+      <c r="T118" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U118" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V118" s="11">
+        <v>11</v>
+      </c>
+      <c r="W118" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X118" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y118" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB118" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG118" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI118" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ118" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK118" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM118" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR118" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="119" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
+        <v>1</v>
+      </c>
+      <c r="B119" s="2">
+        <v>2</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F119" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G119" s="5">
+        <v>11</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I119" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J119" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K119" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L119" s="6">
+        <v>873</v>
+      </c>
+      <c r="M119" s="7">
+        <v>364926.48</v>
+      </c>
+      <c r="N119" s="6">
+        <v>1</v>
+      </c>
+      <c r="O119" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="P119" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q119" s="6">
+        <v>0</v>
+      </c>
+      <c r="R119" s="7">
+        <v>0</v>
+      </c>
+      <c r="S119" s="9">
+        <v>0</v>
+      </c>
+      <c r="T119" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U119" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V119" s="11">
+        <v>11</v>
+      </c>
+      <c r="W119" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X119" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y119" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB119" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG119" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI119" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ119" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK119" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM119" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR119" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 11/05/2026 10:29:56,92
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15243E96-E8B2-408A-81B9-FC13BA33FB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1FA80C2-FC2E-457A-91FD-EE733D75C966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2168" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2582" uniqueCount="200">
   <si>
     <t>Sel</t>
   </si>
@@ -506,6 +506,75 @@
   </si>
   <si>
     <t>1858700136670</t>
+  </si>
+  <si>
+    <t>1858700136671</t>
+  </si>
+  <si>
+    <t>1858700136672</t>
+  </si>
+  <si>
+    <t>1858700136673</t>
+  </si>
+  <si>
+    <t>1858700136674</t>
+  </si>
+  <si>
+    <t>1858700136675</t>
+  </si>
+  <si>
+    <t>1858700136676</t>
+  </si>
+  <si>
+    <t>1858700136677</t>
+  </si>
+  <si>
+    <t>1858700136678</t>
+  </si>
+  <si>
+    <t>1858700136679</t>
+  </si>
+  <si>
+    <t>1858700136680</t>
+  </si>
+  <si>
+    <t>1858700136681</t>
+  </si>
+  <si>
+    <t>1858700136682</t>
+  </si>
+  <si>
+    <t>1858700136683</t>
+  </si>
+  <si>
+    <t>1858700136684</t>
+  </si>
+  <si>
+    <t>1858700136685</t>
+  </si>
+  <si>
+    <t>1858700136686</t>
+  </si>
+  <si>
+    <t>1858700136687</t>
+  </si>
+  <si>
+    <t>1858700136688</t>
+  </si>
+  <si>
+    <t>1858700136689</t>
+  </si>
+  <si>
+    <t>1858700136690</t>
+  </si>
+  <si>
+    <t>1858700136691</t>
+  </si>
+  <si>
+    <t>1858700136692</t>
+  </si>
+  <si>
+    <t>1858700136693</t>
   </si>
   <si>
     <t>10016354</t>
@@ -1126,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR119"/>
+  <dimension ref="A1:AR142"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -15609,10 +15678,10 @@
         <v>2</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>46</v>
@@ -15621,7 +15690,7 @@
         <v>46153</v>
       </c>
       <c r="G109" s="5">
-        <v>1</v>
+        <v>218</v>
       </c>
       <c r="H109" s="3" t="s">
         <v>47</v>
@@ -15636,19 +15705,19 @@
         <v>50</v>
       </c>
       <c r="L109" s="6">
-        <v>863</v>
+        <v>727</v>
       </c>
       <c r="M109" s="7">
-        <v>360746.33</v>
+        <v>137280.53</v>
       </c>
       <c r="N109" s="6">
         <v>1</v>
       </c>
       <c r="O109" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P109" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q109" s="6">
         <v>0</v>
@@ -15663,7 +15732,7 @@
         <v>52</v>
       </c>
       <c r="U109" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V109" s="11">
         <v>11</v>
@@ -15672,7 +15741,7 @@
         <v>46153</v>
       </c>
       <c r="X109" s="12">
-        <v>0.31597219999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y109" s="10">
         <v>0</v>
@@ -15705,7 +15774,7 @@
         <v>53</v>
       </c>
       <c r="AI109" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ109" s="3" t="s">
         <v>52</v>
@@ -15732,7 +15801,7 @@
         <v>53</v>
       </c>
       <c r="AR109" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="110" spans="1:44" x14ac:dyDescent="0.3">
@@ -15743,10 +15812,10 @@
         <v>2</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E110" s="3" t="s">
         <v>46</v>
@@ -15755,7 +15824,7 @@
         <v>46153</v>
       </c>
       <c r="G110" s="5">
-        <v>2</v>
+        <v>219</v>
       </c>
       <c r="H110" s="3" t="s">
         <v>47</v>
@@ -15770,19 +15839,19 @@
         <v>50</v>
       </c>
       <c r="L110" s="6">
-        <v>864</v>
+        <v>728</v>
       </c>
       <c r="M110" s="7">
-        <v>361164.35</v>
+        <v>137469.37</v>
       </c>
       <c r="N110" s="6">
         <v>1</v>
       </c>
       <c r="O110" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P110" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q110" s="6">
         <v>0</v>
@@ -15797,7 +15866,7 @@
         <v>52</v>
       </c>
       <c r="U110" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V110" s="11">
         <v>11</v>
@@ -15806,7 +15875,7 @@
         <v>46153</v>
       </c>
       <c r="X110" s="12">
-        <v>0.31597219999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y110" s="10">
         <v>0</v>
@@ -15839,7 +15908,7 @@
         <v>53</v>
       </c>
       <c r="AI110" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ110" s="3" t="s">
         <v>52</v>
@@ -15866,7 +15935,7 @@
         <v>53</v>
       </c>
       <c r="AR110" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="111" spans="1:44" x14ac:dyDescent="0.3">
@@ -15877,10 +15946,10 @@
         <v>2</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E111" s="3" t="s">
         <v>46</v>
@@ -15889,7 +15958,7 @@
         <v>46153</v>
       </c>
       <c r="G111" s="5">
-        <v>3</v>
+        <v>220</v>
       </c>
       <c r="H111" s="3" t="s">
         <v>47</v>
@@ -15904,19 +15973,19 @@
         <v>50</v>
       </c>
       <c r="L111" s="6">
-        <v>865</v>
+        <v>729</v>
       </c>
       <c r="M111" s="7">
-        <v>361582.36</v>
+        <v>137658.20000000001</v>
       </c>
       <c r="N111" s="6">
         <v>1</v>
       </c>
       <c r="O111" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P111" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q111" s="6">
         <v>0</v>
@@ -15931,7 +16000,7 @@
         <v>52</v>
       </c>
       <c r="U111" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V111" s="11">
         <v>11</v>
@@ -15940,7 +16009,7 @@
         <v>46153</v>
       </c>
       <c r="X111" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y111" s="10">
         <v>0</v>
@@ -15973,7 +16042,7 @@
         <v>53</v>
       </c>
       <c r="AI111" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ111" s="3" t="s">
         <v>52</v>
@@ -16000,7 +16069,7 @@
         <v>53</v>
       </c>
       <c r="AR111" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="112" spans="1:44" x14ac:dyDescent="0.3">
@@ -16011,10 +16080,10 @@
         <v>2</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E112" s="3" t="s">
         <v>46</v>
@@ -16023,7 +16092,7 @@
         <v>46153</v>
       </c>
       <c r="G112" s="5">
-        <v>4</v>
+        <v>221</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>47</v>
@@ -16038,19 +16107,19 @@
         <v>50</v>
       </c>
       <c r="L112" s="6">
-        <v>866</v>
+        <v>730</v>
       </c>
       <c r="M112" s="7">
-        <v>362000.38</v>
+        <v>137847.03</v>
       </c>
       <c r="N112" s="6">
         <v>1</v>
       </c>
       <c r="O112" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P112" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q112" s="6">
         <v>0</v>
@@ -16065,7 +16134,7 @@
         <v>52</v>
       </c>
       <c r="U112" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V112" s="11">
         <v>11</v>
@@ -16074,7 +16143,7 @@
         <v>46153</v>
       </c>
       <c r="X112" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y112" s="10">
         <v>0</v>
@@ -16107,34 +16176,34 @@
         <v>53</v>
       </c>
       <c r="AI112" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ112" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK112" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM112" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR112" s="3" t="s">
         <v>165</v>
-      </c>
-      <c r="AJ112" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK112" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL112" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM112" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN112" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO112" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP112" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ112" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR112" s="3" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="113" spans="1:44" x14ac:dyDescent="0.3">
@@ -16145,10 +16214,10 @@
         <v>2</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E113" s="3" t="s">
         <v>46</v>
@@ -16157,7 +16226,7 @@
         <v>46153</v>
       </c>
       <c r="G113" s="5">
-        <v>5</v>
+        <v>222</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>47</v>
@@ -16172,19 +16241,19 @@
         <v>50</v>
       </c>
       <c r="L113" s="6">
-        <v>867</v>
+        <v>731</v>
       </c>
       <c r="M113" s="7">
-        <v>362418.39</v>
+        <v>138035.85999999999</v>
       </c>
       <c r="N113" s="6">
         <v>1</v>
       </c>
       <c r="O113" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P113" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q113" s="6">
         <v>0</v>
@@ -16199,7 +16268,7 @@
         <v>52</v>
       </c>
       <c r="U113" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V113" s="11">
         <v>11</v>
@@ -16208,7 +16277,7 @@
         <v>46153</v>
       </c>
       <c r="X113" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y113" s="10">
         <v>0</v>
@@ -16241,7 +16310,7 @@
         <v>53</v>
       </c>
       <c r="AI113" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ113" s="3" t="s">
         <v>52</v>
@@ -16268,7 +16337,7 @@
         <v>53</v>
       </c>
       <c r="AR113" s="3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="114" spans="1:44" x14ac:dyDescent="0.3">
@@ -16279,10 +16348,10 @@
         <v>2</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E114" s="3" t="s">
         <v>46</v>
@@ -16291,7 +16360,7 @@
         <v>46153</v>
       </c>
       <c r="G114" s="5">
-        <v>6</v>
+        <v>223</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>47</v>
@@ -16306,19 +16375,19 @@
         <v>50</v>
       </c>
       <c r="L114" s="6">
-        <v>868</v>
+        <v>732</v>
       </c>
       <c r="M114" s="7">
-        <v>362836.4</v>
+        <v>138224.69</v>
       </c>
       <c r="N114" s="6">
         <v>1</v>
       </c>
       <c r="O114" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P114" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q114" s="6">
         <v>0</v>
@@ -16333,7 +16402,7 @@
         <v>52</v>
       </c>
       <c r="U114" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V114" s="11">
         <v>11</v>
@@ -16342,7 +16411,7 @@
         <v>46153</v>
       </c>
       <c r="X114" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y114" s="10">
         <v>0</v>
@@ -16375,7 +16444,7 @@
         <v>53</v>
       </c>
       <c r="AI114" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ114" s="3" t="s">
         <v>52</v>
@@ -16402,7 +16471,7 @@
         <v>53</v>
       </c>
       <c r="AR114" s="3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="115" spans="1:44" x14ac:dyDescent="0.3">
@@ -16413,10 +16482,10 @@
         <v>2</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E115" s="3" t="s">
         <v>46</v>
@@ -16425,7 +16494,7 @@
         <v>46153</v>
       </c>
       <c r="G115" s="5">
-        <v>7</v>
+        <v>224</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>47</v>
@@ -16440,19 +16509,19 @@
         <v>50</v>
       </c>
       <c r="L115" s="6">
-        <v>869</v>
+        <v>733</v>
       </c>
       <c r="M115" s="7">
-        <v>363254.42</v>
+        <v>138413.51999999999</v>
       </c>
       <c r="N115" s="6">
         <v>1</v>
       </c>
       <c r="O115" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P115" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q115" s="6">
         <v>0</v>
@@ -16467,7 +16536,7 @@
         <v>52</v>
       </c>
       <c r="U115" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V115" s="11">
         <v>11</v>
@@ -16476,7 +16545,7 @@
         <v>46153</v>
       </c>
       <c r="X115" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y115" s="10">
         <v>0</v>
@@ -16509,7 +16578,7 @@
         <v>53</v>
       </c>
       <c r="AI115" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ115" s="3" t="s">
         <v>52</v>
@@ -16536,7 +16605,7 @@
         <v>53</v>
       </c>
       <c r="AR115" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="116" spans="1:44" x14ac:dyDescent="0.3">
@@ -16547,10 +16616,10 @@
         <v>2</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E116" s="3" t="s">
         <v>46</v>
@@ -16559,7 +16628,7 @@
         <v>46153</v>
       </c>
       <c r="G116" s="5">
-        <v>8</v>
+        <v>225</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>47</v>
@@ -16574,19 +16643,19 @@
         <v>50</v>
       </c>
       <c r="L116" s="6">
-        <v>870</v>
+        <v>734</v>
       </c>
       <c r="M116" s="7">
-        <v>363672.43</v>
+        <v>138602.35999999999</v>
       </c>
       <c r="N116" s="6">
         <v>1</v>
       </c>
       <c r="O116" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P116" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q116" s="6">
         <v>0</v>
@@ -16601,7 +16670,7 @@
         <v>52</v>
       </c>
       <c r="U116" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V116" s="11">
         <v>11</v>
@@ -16610,7 +16679,7 @@
         <v>46153</v>
       </c>
       <c r="X116" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y116" s="10">
         <v>0</v>
@@ -16643,7 +16712,7 @@
         <v>53</v>
       </c>
       <c r="AI116" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ116" s="3" t="s">
         <v>52</v>
@@ -16670,7 +16739,7 @@
         <v>53</v>
       </c>
       <c r="AR116" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="117" spans="1:44" x14ac:dyDescent="0.3">
@@ -16681,10 +16750,10 @@
         <v>2</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E117" s="3" t="s">
         <v>46</v>
@@ -16693,7 +16762,7 @@
         <v>46153</v>
       </c>
       <c r="G117" s="5">
-        <v>9</v>
+        <v>226</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>47</v>
@@ -16708,19 +16777,19 @@
         <v>50</v>
       </c>
       <c r="L117" s="6">
-        <v>871</v>
+        <v>735</v>
       </c>
       <c r="M117" s="7">
-        <v>364090.45</v>
+        <v>138791.19</v>
       </c>
       <c r="N117" s="6">
         <v>1</v>
       </c>
       <c r="O117" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P117" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q117" s="6">
         <v>0</v>
@@ -16735,7 +16804,7 @@
         <v>52</v>
       </c>
       <c r="U117" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V117" s="11">
         <v>11</v>
@@ -16744,7 +16813,7 @@
         <v>46153</v>
       </c>
       <c r="X117" s="12">
-        <v>0.39930559999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y117" s="10">
         <v>0</v>
@@ -16777,7 +16846,7 @@
         <v>53</v>
       </c>
       <c r="AI117" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ117" s="3" t="s">
         <v>52</v>
@@ -16804,7 +16873,7 @@
         <v>53</v>
       </c>
       <c r="AR117" s="3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="118" spans="1:44" x14ac:dyDescent="0.3">
@@ -16815,10 +16884,10 @@
         <v>2</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E118" s="3" t="s">
         <v>46</v>
@@ -16827,7 +16896,7 @@
         <v>46153</v>
       </c>
       <c r="G118" s="5">
-        <v>10</v>
+        <v>227</v>
       </c>
       <c r="H118" s="3" t="s">
         <v>47</v>
@@ -16842,19 +16911,19 @@
         <v>50</v>
       </c>
       <c r="L118" s="6">
-        <v>872</v>
+        <v>736</v>
       </c>
       <c r="M118" s="7">
-        <v>364508.46</v>
+        <v>138980.01999999999</v>
       </c>
       <c r="N118" s="6">
         <v>1</v>
       </c>
       <c r="O118" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P118" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q118" s="6">
         <v>0</v>
@@ -16869,7 +16938,7 @@
         <v>52</v>
       </c>
       <c r="U118" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V118" s="11">
         <v>11</v>
@@ -16878,7 +16947,7 @@
         <v>46153</v>
       </c>
       <c r="X118" s="12">
-        <v>0.39930559999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y118" s="10">
         <v>0</v>
@@ -16911,7 +16980,7 @@
         <v>53</v>
       </c>
       <c r="AI118" s="3" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="AJ118" s="3" t="s">
         <v>52</v>
@@ -16938,7 +17007,7 @@
         <v>53</v>
       </c>
       <c r="AR118" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="119" spans="1:44" x14ac:dyDescent="0.3">
@@ -16949,10 +17018,10 @@
         <v>2</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>163</v>
+        <v>45</v>
       </c>
       <c r="E119" s="3" t="s">
         <v>46</v>
@@ -16961,7 +17030,7 @@
         <v>46153</v>
       </c>
       <c r="G119" s="5">
-        <v>11</v>
+        <v>228</v>
       </c>
       <c r="H119" s="3" t="s">
         <v>47</v>
@@ -16976,19 +17045,19 @@
         <v>50</v>
       </c>
       <c r="L119" s="6">
-        <v>873</v>
+        <v>737</v>
       </c>
       <c r="M119" s="7">
-        <v>364926.48</v>
+        <v>139168.85</v>
       </c>
       <c r="N119" s="6">
         <v>1</v>
       </c>
       <c r="O119" s="3" t="s">
-        <v>164</v>
+        <v>51</v>
       </c>
       <c r="P119" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q119" s="6">
         <v>0</v>
@@ -17003,7 +17072,7 @@
         <v>52</v>
       </c>
       <c r="U119" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V119" s="11">
         <v>11</v>
@@ -17012,67 +17081,3149 @@
         <v>46153</v>
       </c>
       <c r="X119" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y119" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB119" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG119" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI119" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ119" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK119" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM119" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR119" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="120" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
+        <v>1</v>
+      </c>
+      <c r="B120" s="2">
+        <v>2</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F120" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G120" s="5">
+        <v>229</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I120" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J120" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K120" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L120" s="6">
+        <v>738</v>
+      </c>
+      <c r="M120" s="7">
+        <v>139357.68</v>
+      </c>
+      <c r="N120" s="6">
+        <v>1</v>
+      </c>
+      <c r="O120" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P120" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q120" s="6">
+        <v>0</v>
+      </c>
+      <c r="R120" s="7">
+        <v>0</v>
+      </c>
+      <c r="S120" s="9">
+        <v>0</v>
+      </c>
+      <c r="T120" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U120" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V120" s="11">
+        <v>11</v>
+      </c>
+      <c r="W120" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X120" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y120" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB120" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG120" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI120" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ120" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK120" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM120" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR120" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="121" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
+        <v>1</v>
+      </c>
+      <c r="B121" s="2">
+        <v>2</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F121" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G121" s="5">
+        <v>230</v>
+      </c>
+      <c r="H121" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I121" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J121" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K121" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L121" s="6">
+        <v>739</v>
+      </c>
+      <c r="M121" s="7">
+        <v>139546.51</v>
+      </c>
+      <c r="N121" s="6">
+        <v>1</v>
+      </c>
+      <c r="O121" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P121" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q121" s="6">
+        <v>0</v>
+      </c>
+      <c r="R121" s="7">
+        <v>0</v>
+      </c>
+      <c r="S121" s="9">
+        <v>0</v>
+      </c>
+      <c r="T121" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U121" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V121" s="11">
+        <v>11</v>
+      </c>
+      <c r="W121" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X121" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y121" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB121" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG121" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI121" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ121" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK121" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM121" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR121" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="122" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>1</v>
+      </c>
+      <c r="B122" s="2">
+        <v>2</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F122" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G122" s="5">
+        <v>231</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I122" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J122" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K122" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L122" s="6">
+        <v>740</v>
+      </c>
+      <c r="M122" s="7">
+        <v>139735.35</v>
+      </c>
+      <c r="N122" s="6">
+        <v>1</v>
+      </c>
+      <c r="O122" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P122" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q122" s="6">
+        <v>0</v>
+      </c>
+      <c r="R122" s="7">
+        <v>0</v>
+      </c>
+      <c r="S122" s="9">
+        <v>0</v>
+      </c>
+      <c r="T122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U122" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V122" s="11">
+        <v>11</v>
+      </c>
+      <c r="W122" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X122" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y122" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB122" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG122" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI122" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK122" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM122" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR122" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="123" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
+        <v>1</v>
+      </c>
+      <c r="B123" s="2">
+        <v>2</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F123" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G123" s="5">
+        <v>232</v>
+      </c>
+      <c r="H123" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I123" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J123" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K123" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L123" s="6">
+        <v>741</v>
+      </c>
+      <c r="M123" s="7">
+        <v>139924.18</v>
+      </c>
+      <c r="N123" s="6">
+        <v>1</v>
+      </c>
+      <c r="O123" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P123" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q123" s="6">
+        <v>0</v>
+      </c>
+      <c r="R123" s="7">
+        <v>0</v>
+      </c>
+      <c r="S123" s="9">
+        <v>0</v>
+      </c>
+      <c r="T123" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U123" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V123" s="11">
+        <v>11</v>
+      </c>
+      <c r="W123" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X123" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y123" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB123" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG123" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI123" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ123" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK123" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM123" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR123" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="124" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>1</v>
+      </c>
+      <c r="B124" s="2">
+        <v>2</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F124" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G124" s="5">
+        <v>233</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I124" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J124" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K124" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L124" s="6">
+        <v>742</v>
+      </c>
+      <c r="M124" s="7">
+        <v>140113.01</v>
+      </c>
+      <c r="N124" s="6">
+        <v>1</v>
+      </c>
+      <c r="O124" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P124" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q124" s="6">
+        <v>0</v>
+      </c>
+      <c r="R124" s="7">
+        <v>0</v>
+      </c>
+      <c r="S124" s="9">
+        <v>0</v>
+      </c>
+      <c r="T124" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U124" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V124" s="11">
+        <v>11</v>
+      </c>
+      <c r="W124" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X124" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y124" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB124" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG124" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI124" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ124" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK124" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM124" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR124" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="125" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
+        <v>1</v>
+      </c>
+      <c r="B125" s="2">
+        <v>2</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F125" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G125" s="5">
+        <v>234</v>
+      </c>
+      <c r="H125" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I125" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J125" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K125" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L125" s="6">
+        <v>743</v>
+      </c>
+      <c r="M125" s="7">
+        <v>140301.84</v>
+      </c>
+      <c r="N125" s="6">
+        <v>1</v>
+      </c>
+      <c r="O125" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P125" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q125" s="6">
+        <v>0</v>
+      </c>
+      <c r="R125" s="7">
+        <v>0</v>
+      </c>
+      <c r="S125" s="9">
+        <v>0</v>
+      </c>
+      <c r="T125" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U125" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V125" s="11">
+        <v>11</v>
+      </c>
+      <c r="W125" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X125" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y125" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB125" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG125" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI125" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ125" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK125" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM125" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR125" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="126" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A126" s="1">
+        <v>1</v>
+      </c>
+      <c r="B126" s="2">
+        <v>2</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F126" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G126" s="5">
+        <v>235</v>
+      </c>
+      <c r="H126" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I126" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J126" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K126" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L126" s="6">
+        <v>744</v>
+      </c>
+      <c r="M126" s="7">
+        <v>140490.67000000001</v>
+      </c>
+      <c r="N126" s="6">
+        <v>1</v>
+      </c>
+      <c r="O126" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P126" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q126" s="6">
+        <v>0</v>
+      </c>
+      <c r="R126" s="7">
+        <v>0</v>
+      </c>
+      <c r="S126" s="9">
+        <v>0</v>
+      </c>
+      <c r="T126" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U126" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V126" s="11">
+        <v>11</v>
+      </c>
+      <c r="W126" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X126" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y126" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB126" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG126" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI126" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ126" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK126" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM126" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR126" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="127" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A127" s="1">
+        <v>1</v>
+      </c>
+      <c r="B127" s="2">
+        <v>2</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E127" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F127" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G127" s="5">
+        <v>236</v>
+      </c>
+      <c r="H127" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I127" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J127" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K127" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L127" s="6">
+        <v>745</v>
+      </c>
+      <c r="M127" s="7">
+        <v>140679.5</v>
+      </c>
+      <c r="N127" s="6">
+        <v>1</v>
+      </c>
+      <c r="O127" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P127" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q127" s="6">
+        <v>0</v>
+      </c>
+      <c r="R127" s="7">
+        <v>0</v>
+      </c>
+      <c r="S127" s="9">
+        <v>0</v>
+      </c>
+      <c r="T127" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U127" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V127" s="11">
+        <v>11</v>
+      </c>
+      <c r="W127" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X127" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y127" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB127" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG127" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI127" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ127" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK127" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM127" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR127" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="128" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A128" s="1">
+        <v>1</v>
+      </c>
+      <c r="B128" s="2">
+        <v>2</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F128" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G128" s="5">
+        <v>237</v>
+      </c>
+      <c r="H128" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I128" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J128" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K128" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L128" s="6">
+        <v>746</v>
+      </c>
+      <c r="M128" s="7">
+        <v>140868.32999999999</v>
+      </c>
+      <c r="N128" s="6">
+        <v>1</v>
+      </c>
+      <c r="O128" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P128" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q128" s="6">
+        <v>0</v>
+      </c>
+      <c r="R128" s="7">
+        <v>0</v>
+      </c>
+      <c r="S128" s="9">
+        <v>0</v>
+      </c>
+      <c r="T128" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U128" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V128" s="11">
+        <v>11</v>
+      </c>
+      <c r="W128" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X128" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y128" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB128" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG128" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI128" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ128" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK128" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM128" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR128" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="129" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A129" s="1">
+        <v>1</v>
+      </c>
+      <c r="B129" s="2">
+        <v>2</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E129" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F129" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G129" s="5">
+        <v>238</v>
+      </c>
+      <c r="H129" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I129" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J129" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K129" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L129" s="6">
+        <v>747</v>
+      </c>
+      <c r="M129" s="7">
+        <v>141057.17000000001</v>
+      </c>
+      <c r="N129" s="6">
+        <v>1</v>
+      </c>
+      <c r="O129" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P129" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q129" s="6">
+        <v>0</v>
+      </c>
+      <c r="R129" s="7">
+        <v>0</v>
+      </c>
+      <c r="S129" s="9">
+        <v>0</v>
+      </c>
+      <c r="T129" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U129" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V129" s="11">
+        <v>11</v>
+      </c>
+      <c r="W129" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X129" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y129" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z129" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA129" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB129" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC129" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD129" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE129" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF129" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG129" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH129" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI129" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ129" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK129" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL129" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM129" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN129" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO129" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP129" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ129" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR129" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="130" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A130" s="1">
+        <v>1</v>
+      </c>
+      <c r="B130" s="2">
+        <v>2</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F130" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G130" s="5">
+        <v>239</v>
+      </c>
+      <c r="H130" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I130" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J130" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K130" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L130" s="6">
+        <v>748</v>
+      </c>
+      <c r="M130" s="7">
+        <v>141246</v>
+      </c>
+      <c r="N130" s="6">
+        <v>1</v>
+      </c>
+      <c r="O130" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P130" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q130" s="6">
+        <v>0</v>
+      </c>
+      <c r="R130" s="7">
+        <v>0</v>
+      </c>
+      <c r="S130" s="9">
+        <v>0</v>
+      </c>
+      <c r="T130" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U130" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V130" s="11">
+        <v>11</v>
+      </c>
+      <c r="W130" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X130" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y130" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z130" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA130" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB130" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC130" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD130" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE130" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG130" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI130" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ130" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK130" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL130" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM130" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR130" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="131" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A131" s="1">
+        <v>1</v>
+      </c>
+      <c r="B131" s="2">
+        <v>2</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E131" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F131" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G131" s="5">
+        <v>240</v>
+      </c>
+      <c r="H131" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I131" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J131" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K131" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L131" s="6">
+        <v>749</v>
+      </c>
+      <c r="M131" s="7">
+        <v>141434.82999999999</v>
+      </c>
+      <c r="N131" s="6">
+        <v>1</v>
+      </c>
+      <c r="O131" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P131" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q131" s="6">
+        <v>0</v>
+      </c>
+      <c r="R131" s="7">
+        <v>0</v>
+      </c>
+      <c r="S131" s="9">
+        <v>0</v>
+      </c>
+      <c r="T131" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U131" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V131" s="11">
+        <v>11</v>
+      </c>
+      <c r="W131" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X131" s="12">
+        <v>0.42013889999999998</v>
+      </c>
+      <c r="Y131" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z131" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA131" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB131" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC131" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD131" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE131" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF131" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG131" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH131" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI131" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ131" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK131" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL131" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM131" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN131" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO131" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP131" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ131" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR131" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="132" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A132" s="1">
+        <v>1</v>
+      </c>
+      <c r="B132" s="2">
+        <v>2</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F132" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G132" s="5">
+        <v>1</v>
+      </c>
+      <c r="H132" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I132" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J132" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K132" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L132" s="6">
+        <v>863</v>
+      </c>
+      <c r="M132" s="7">
+        <v>360746.33</v>
+      </c>
+      <c r="N132" s="6">
+        <v>1</v>
+      </c>
+      <c r="O132" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P132" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q132" s="6">
+        <v>0</v>
+      </c>
+      <c r="R132" s="7">
+        <v>0</v>
+      </c>
+      <c r="S132" s="9">
+        <v>0</v>
+      </c>
+      <c r="T132" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U132" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V132" s="11">
+        <v>11</v>
+      </c>
+      <c r="W132" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X132" s="12">
+        <v>0.31597219999999998</v>
+      </c>
+      <c r="Y132" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB132" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG132" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI132" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ132" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK132" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL132" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM132" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR132" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="133" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A133" s="1">
+        <v>1</v>
+      </c>
+      <c r="B133" s="2">
+        <v>2</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F133" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G133" s="5">
+        <v>2</v>
+      </c>
+      <c r="H133" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I133" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J133" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K133" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L133" s="6">
+        <v>864</v>
+      </c>
+      <c r="M133" s="7">
+        <v>361164.35</v>
+      </c>
+      <c r="N133" s="6">
+        <v>1</v>
+      </c>
+      <c r="O133" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P133" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q133" s="6">
+        <v>0</v>
+      </c>
+      <c r="R133" s="7">
+        <v>0</v>
+      </c>
+      <c r="S133" s="9">
+        <v>0</v>
+      </c>
+      <c r="T133" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U133" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V133" s="11">
+        <v>11</v>
+      </c>
+      <c r="W133" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X133" s="12">
+        <v>0.31597219999999998</v>
+      </c>
+      <c r="Y133" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB133" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG133" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI133" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ133" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK133" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL133" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM133" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ133" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR133" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="134" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A134" s="1">
+        <v>1</v>
+      </c>
+      <c r="B134" s="2">
+        <v>2</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F134" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G134" s="5">
+        <v>3</v>
+      </c>
+      <c r="H134" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I134" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J134" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K134" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L134" s="6">
+        <v>865</v>
+      </c>
+      <c r="M134" s="7">
+        <v>361582.36</v>
+      </c>
+      <c r="N134" s="6">
+        <v>1</v>
+      </c>
+      <c r="O134" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P134" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q134" s="6">
+        <v>0</v>
+      </c>
+      <c r="R134" s="7">
+        <v>0</v>
+      </c>
+      <c r="S134" s="9">
+        <v>0</v>
+      </c>
+      <c r="T134" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U134" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V134" s="11">
+        <v>11</v>
+      </c>
+      <c r="W134" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X134" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y134" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB134" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG134" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI134" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ134" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK134" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL134" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM134" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR134" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="135" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A135" s="1">
+        <v>1</v>
+      </c>
+      <c r="B135" s="2">
+        <v>2</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E135" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F135" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G135" s="5">
+        <v>4</v>
+      </c>
+      <c r="H135" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I135" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J135" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K135" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L135" s="6">
+        <v>866</v>
+      </c>
+      <c r="M135" s="7">
+        <v>362000.38</v>
+      </c>
+      <c r="N135" s="6">
+        <v>1</v>
+      </c>
+      <c r="O135" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P135" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q135" s="6">
+        <v>0</v>
+      </c>
+      <c r="R135" s="7">
+        <v>0</v>
+      </c>
+      <c r="S135" s="9">
+        <v>0</v>
+      </c>
+      <c r="T135" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U135" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V135" s="11">
+        <v>11</v>
+      </c>
+      <c r="W135" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X135" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y135" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB135" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG135" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI135" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ135" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK135" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL135" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM135" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ135" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR135" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="136" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A136" s="1">
+        <v>1</v>
+      </c>
+      <c r="B136" s="2">
+        <v>2</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F136" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G136" s="5">
+        <v>5</v>
+      </c>
+      <c r="H136" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I136" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J136" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K136" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L136" s="6">
+        <v>867</v>
+      </c>
+      <c r="M136" s="7">
+        <v>362418.39</v>
+      </c>
+      <c r="N136" s="6">
+        <v>1</v>
+      </c>
+      <c r="O136" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P136" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q136" s="6">
+        <v>0</v>
+      </c>
+      <c r="R136" s="7">
+        <v>0</v>
+      </c>
+      <c r="S136" s="9">
+        <v>0</v>
+      </c>
+      <c r="T136" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U136" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V136" s="11">
+        <v>11</v>
+      </c>
+      <c r="W136" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X136" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y136" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB136" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG136" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI136" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ136" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK136" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL136" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM136" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR136" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="137" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A137" s="1">
+        <v>1</v>
+      </c>
+      <c r="B137" s="2">
+        <v>2</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F137" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G137" s="5">
+        <v>6</v>
+      </c>
+      <c r="H137" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I137" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J137" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K137" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L137" s="6">
+        <v>868</v>
+      </c>
+      <c r="M137" s="7">
+        <v>362836.4</v>
+      </c>
+      <c r="N137" s="6">
+        <v>1</v>
+      </c>
+      <c r="O137" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P137" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q137" s="6">
+        <v>0</v>
+      </c>
+      <c r="R137" s="7">
+        <v>0</v>
+      </c>
+      <c r="S137" s="9">
+        <v>0</v>
+      </c>
+      <c r="T137" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U137" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V137" s="11">
+        <v>11</v>
+      </c>
+      <c r="W137" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X137" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y137" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB137" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG137" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI137" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ137" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK137" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL137" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM137" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ137" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR137" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="138" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A138" s="1">
+        <v>1</v>
+      </c>
+      <c r="B138" s="2">
+        <v>2</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F138" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G138" s="5">
+        <v>7</v>
+      </c>
+      <c r="H138" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I138" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J138" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K138" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L138" s="6">
+        <v>869</v>
+      </c>
+      <c r="M138" s="7">
+        <v>363254.42</v>
+      </c>
+      <c r="N138" s="6">
+        <v>1</v>
+      </c>
+      <c r="O138" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P138" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q138" s="6">
+        <v>0</v>
+      </c>
+      <c r="R138" s="7">
+        <v>0</v>
+      </c>
+      <c r="S138" s="9">
+        <v>0</v>
+      </c>
+      <c r="T138" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U138" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V138" s="11">
+        <v>11</v>
+      </c>
+      <c r="W138" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X138" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y138" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB138" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG138" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI138" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ138" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK138" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL138" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM138" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR138" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="139" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A139" s="1">
+        <v>1</v>
+      </c>
+      <c r="B139" s="2">
+        <v>2</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E139" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F139" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G139" s="5">
+        <v>8</v>
+      </c>
+      <c r="H139" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I139" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J139" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K139" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L139" s="6">
+        <v>870</v>
+      </c>
+      <c r="M139" s="7">
+        <v>363672.43</v>
+      </c>
+      <c r="N139" s="6">
+        <v>1</v>
+      </c>
+      <c r="O139" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P139" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q139" s="6">
+        <v>0</v>
+      </c>
+      <c r="R139" s="7">
+        <v>0</v>
+      </c>
+      <c r="S139" s="9">
+        <v>0</v>
+      </c>
+      <c r="T139" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U139" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V139" s="11">
+        <v>11</v>
+      </c>
+      <c r="W139" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X139" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y139" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB139" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG139" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI139" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ139" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK139" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL139" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM139" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ139" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR139" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="140" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A140" s="1">
+        <v>1</v>
+      </c>
+      <c r="B140" s="2">
+        <v>2</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F140" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G140" s="5">
+        <v>9</v>
+      </c>
+      <c r="H140" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I140" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J140" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K140" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L140" s="6">
+        <v>871</v>
+      </c>
+      <c r="M140" s="7">
+        <v>364090.45</v>
+      </c>
+      <c r="N140" s="6">
+        <v>1</v>
+      </c>
+      <c r="O140" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P140" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q140" s="6">
+        <v>0</v>
+      </c>
+      <c r="R140" s="7">
+        <v>0</v>
+      </c>
+      <c r="S140" s="9">
+        <v>0</v>
+      </c>
+      <c r="T140" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U140" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V140" s="11">
+        <v>11</v>
+      </c>
+      <c r="W140" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X140" s="12">
         <v>0.39930559999999998</v>
       </c>
-      <c r="Y119" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z119" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA119" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB119" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC119" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD119" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE119" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF119" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG119" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH119" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI119" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="AJ119" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK119" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL119" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM119" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN119" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO119" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP119" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ119" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR119" s="3" t="s">
-        <v>176</v>
+      <c r="Y140" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB140" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG140" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI140" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ140" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK140" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL140" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM140" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR140" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="141" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A141" s="1">
+        <v>1</v>
+      </c>
+      <c r="B141" s="2">
+        <v>2</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E141" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F141" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G141" s="5">
+        <v>10</v>
+      </c>
+      <c r="H141" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I141" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J141" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K141" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L141" s="6">
+        <v>872</v>
+      </c>
+      <c r="M141" s="7">
+        <v>364508.46</v>
+      </c>
+      <c r="N141" s="6">
+        <v>1</v>
+      </c>
+      <c r="O141" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P141" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q141" s="6">
+        <v>0</v>
+      </c>
+      <c r="R141" s="7">
+        <v>0</v>
+      </c>
+      <c r="S141" s="9">
+        <v>0</v>
+      </c>
+      <c r="T141" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U141" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V141" s="11">
+        <v>11</v>
+      </c>
+      <c r="W141" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X141" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y141" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB141" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG141" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI141" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ141" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK141" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL141" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM141" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR141" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="142" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A142" s="1">
+        <v>1</v>
+      </c>
+      <c r="B142" s="2">
+        <v>2</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F142" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G142" s="5">
+        <v>11</v>
+      </c>
+      <c r="H142" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I142" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J142" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K142" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L142" s="6">
+        <v>873</v>
+      </c>
+      <c r="M142" s="7">
+        <v>364926.48</v>
+      </c>
+      <c r="N142" s="6">
+        <v>1</v>
+      </c>
+      <c r="O142" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P142" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q142" s="6">
+        <v>0</v>
+      </c>
+      <c r="R142" s="7">
+        <v>0</v>
+      </c>
+      <c r="S142" s="9">
+        <v>0</v>
+      </c>
+      <c r="T142" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U142" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V142" s="11">
+        <v>11</v>
+      </c>
+      <c r="W142" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X142" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y142" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB142" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG142" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI142" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ142" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK142" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL142" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM142" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR142" s="3" t="s">
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 11/05/2026 12:08:55,62
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DCF74DDC-02B5-44AE-BF67-F2E2EC71215A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D452AD0A-3E2C-43B4-AAE6-14DD260626E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4346" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4832" uniqueCount="325">
   <si>
     <t>Sel</t>
   </si>
@@ -871,6 +871,87 @@
     <t>1858700136791</t>
   </si>
   <si>
+    <t>1858700136792</t>
+  </si>
+  <si>
+    <t>1858700136793</t>
+  </si>
+  <si>
+    <t>1858700136794</t>
+  </si>
+  <si>
+    <t>1858700136795</t>
+  </si>
+  <si>
+    <t>1858700136796</t>
+  </si>
+  <si>
+    <t>1858700136797</t>
+  </si>
+  <si>
+    <t>1858700136798</t>
+  </si>
+  <si>
+    <t>1858700136799</t>
+  </si>
+  <si>
+    <t>1858700136800</t>
+  </si>
+  <si>
+    <t>1858700136801</t>
+  </si>
+  <si>
+    <t>1858700136802</t>
+  </si>
+  <si>
+    <t>1858700136803</t>
+  </si>
+  <si>
+    <t>1858700136804</t>
+  </si>
+  <si>
+    <t>1858700136805</t>
+  </si>
+  <si>
+    <t>1858700136806</t>
+  </si>
+  <si>
+    <t>1858700136807</t>
+  </si>
+  <si>
+    <t>1858700136808</t>
+  </si>
+  <si>
+    <t>1858700136809</t>
+  </si>
+  <si>
+    <t>1858700136810</t>
+  </si>
+  <si>
+    <t>1858700136811</t>
+  </si>
+  <si>
+    <t>1858700136812</t>
+  </si>
+  <si>
+    <t>1858700136813</t>
+  </si>
+  <si>
+    <t>1858700136814</t>
+  </si>
+  <si>
+    <t>1858700136815</t>
+  </si>
+  <si>
+    <t>1858700136816</t>
+  </si>
+  <si>
+    <t>1858700136817</t>
+  </si>
+  <si>
+    <t>1858700136818</t>
+  </si>
+  <si>
     <t>10016354</t>
   </si>
   <si>
@@ -1489,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR240"/>
+  <dimension ref="A1:AR267"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -32186,10 +32267,10 @@
         <v>2</v>
       </c>
       <c r="C230" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D230" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E230" s="3" t="s">
         <v>46</v>
@@ -32198,7 +32279,7 @@
         <v>46153</v>
       </c>
       <c r="G230" s="5">
-        <v>1</v>
+        <v>339</v>
       </c>
       <c r="H230" s="3" t="s">
         <v>47</v>
@@ -32213,19 +32294,19 @@
         <v>50</v>
       </c>
       <c r="L230" s="6">
-        <v>863</v>
+        <v>848</v>
       </c>
       <c r="M230" s="7">
-        <v>360746.33</v>
+        <v>160129.15</v>
       </c>
       <c r="N230" s="6">
         <v>1</v>
       </c>
       <c r="O230" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P230" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q230" s="6">
         <v>0</v>
@@ -32240,7 +32321,7 @@
         <v>52</v>
       </c>
       <c r="U230" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V230" s="11">
         <v>11</v>
@@ -32249,7 +32330,7 @@
         <v>46153</v>
       </c>
       <c r="X230" s="12">
-        <v>0.31597219999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y230" s="10">
         <v>0</v>
@@ -32282,7 +32363,7 @@
         <v>53</v>
       </c>
       <c r="AI230" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ230" s="3" t="s">
         <v>52</v>
@@ -32309,7 +32390,7 @@
         <v>53</v>
       </c>
       <c r="AR230" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
     </row>
     <row r="231" spans="1:44" x14ac:dyDescent="0.3">
@@ -32320,10 +32401,10 @@
         <v>2</v>
       </c>
       <c r="C231" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D231" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E231" s="3" t="s">
         <v>46</v>
@@ -32332,7 +32413,7 @@
         <v>46153</v>
       </c>
       <c r="G231" s="5">
-        <v>2</v>
+        <v>340</v>
       </c>
       <c r="H231" s="3" t="s">
         <v>47</v>
@@ -32347,19 +32428,19 @@
         <v>50</v>
       </c>
       <c r="L231" s="6">
-        <v>864</v>
+        <v>849</v>
       </c>
       <c r="M231" s="7">
-        <v>361164.35</v>
+        <v>160317.98000000001</v>
       </c>
       <c r="N231" s="6">
         <v>1</v>
       </c>
       <c r="O231" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P231" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q231" s="6">
         <v>0</v>
@@ -32374,7 +32455,7 @@
         <v>52</v>
       </c>
       <c r="U231" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V231" s="11">
         <v>11</v>
@@ -32383,7 +32464,7 @@
         <v>46153</v>
       </c>
       <c r="X231" s="12">
-        <v>0.31597219999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y231" s="10">
         <v>0</v>
@@ -32416,7 +32497,7 @@
         <v>53</v>
       </c>
       <c r="AI231" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ231" s="3" t="s">
         <v>52</v>
@@ -32443,7 +32524,7 @@
         <v>53</v>
       </c>
       <c r="AR231" s="3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
     </row>
     <row r="232" spans="1:44" x14ac:dyDescent="0.3">
@@ -32454,10 +32535,10 @@
         <v>2</v>
       </c>
       <c r="C232" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D232" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E232" s="3" t="s">
         <v>46</v>
@@ -32466,7 +32547,7 @@
         <v>46153</v>
       </c>
       <c r="G232" s="5">
-        <v>3</v>
+        <v>341</v>
       </c>
       <c r="H232" s="3" t="s">
         <v>47</v>
@@ -32481,19 +32562,19 @@
         <v>50</v>
       </c>
       <c r="L232" s="6">
-        <v>865</v>
+        <v>850</v>
       </c>
       <c r="M232" s="7">
-        <v>361582.36</v>
+        <v>160506.82</v>
       </c>
       <c r="N232" s="6">
         <v>1</v>
       </c>
       <c r="O232" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P232" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q232" s="6">
         <v>0</v>
@@ -32508,7 +32589,7 @@
         <v>52</v>
       </c>
       <c r="U232" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V232" s="11">
         <v>11</v>
@@ -32517,7 +32598,7 @@
         <v>46153</v>
       </c>
       <c r="X232" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y232" s="10">
         <v>0</v>
@@ -32550,7 +32631,7 @@
         <v>53</v>
       </c>
       <c r="AI232" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ232" s="3" t="s">
         <v>52</v>
@@ -32577,7 +32658,7 @@
         <v>53</v>
       </c>
       <c r="AR232" s="3" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="233" spans="1:44" x14ac:dyDescent="0.3">
@@ -32588,10 +32669,10 @@
         <v>2</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D233" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E233" s="3" t="s">
         <v>46</v>
@@ -32600,7 +32681,7 @@
         <v>46153</v>
       </c>
       <c r="G233" s="5">
-        <v>4</v>
+        <v>342</v>
       </c>
       <c r="H233" s="3" t="s">
         <v>47</v>
@@ -32615,19 +32696,19 @@
         <v>50</v>
       </c>
       <c r="L233" s="6">
-        <v>866</v>
+        <v>851</v>
       </c>
       <c r="M233" s="7">
-        <v>362000.38</v>
+        <v>160695.65</v>
       </c>
       <c r="N233" s="6">
         <v>1</v>
       </c>
       <c r="O233" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P233" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q233" s="6">
         <v>0</v>
@@ -32642,7 +32723,7 @@
         <v>52</v>
       </c>
       <c r="U233" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V233" s="11">
         <v>11</v>
@@ -32651,7 +32732,7 @@
         <v>46153</v>
       </c>
       <c r="X233" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y233" s="10">
         <v>0</v>
@@ -32684,34 +32765,34 @@
         <v>53</v>
       </c>
       <c r="AI233" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ233" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK233" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL233" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM233" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR233" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="AJ233" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK233" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL233" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM233" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN233" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO233" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP233" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ233" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR233" s="3" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="234" spans="1:44" x14ac:dyDescent="0.3">
@@ -32722,10 +32803,10 @@
         <v>2</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D234" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E234" s="3" t="s">
         <v>46</v>
@@ -32734,7 +32815,7 @@
         <v>46153</v>
       </c>
       <c r="G234" s="5">
-        <v>5</v>
+        <v>343</v>
       </c>
       <c r="H234" s="3" t="s">
         <v>47</v>
@@ -32749,19 +32830,19 @@
         <v>50</v>
       </c>
       <c r="L234" s="6">
-        <v>867</v>
+        <v>852</v>
       </c>
       <c r="M234" s="7">
-        <v>362418.39</v>
+        <v>160884.48000000001</v>
       </c>
       <c r="N234" s="6">
         <v>1</v>
       </c>
       <c r="O234" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P234" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q234" s="6">
         <v>0</v>
@@ -32776,7 +32857,7 @@
         <v>52</v>
       </c>
       <c r="U234" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V234" s="11">
         <v>11</v>
@@ -32785,7 +32866,7 @@
         <v>46153</v>
       </c>
       <c r="X234" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y234" s="10">
         <v>0</v>
@@ -32818,7 +32899,7 @@
         <v>53</v>
       </c>
       <c r="AI234" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ234" s="3" t="s">
         <v>52</v>
@@ -32845,7 +32926,7 @@
         <v>53</v>
       </c>
       <c r="AR234" s="3" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="235" spans="1:44" x14ac:dyDescent="0.3">
@@ -32856,10 +32937,10 @@
         <v>2</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D235" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E235" s="3" t="s">
         <v>46</v>
@@ -32868,7 +32949,7 @@
         <v>46153</v>
       </c>
       <c r="G235" s="5">
-        <v>6</v>
+        <v>344</v>
       </c>
       <c r="H235" s="3" t="s">
         <v>47</v>
@@ -32883,19 +32964,19 @@
         <v>50</v>
       </c>
       <c r="L235" s="6">
-        <v>868</v>
+        <v>853</v>
       </c>
       <c r="M235" s="7">
-        <v>362836.4</v>
+        <v>161073.31</v>
       </c>
       <c r="N235" s="6">
         <v>1</v>
       </c>
       <c r="O235" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P235" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q235" s="6">
         <v>0</v>
@@ -32910,7 +32991,7 @@
         <v>52</v>
       </c>
       <c r="U235" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V235" s="11">
         <v>11</v>
@@ -32919,7 +33000,7 @@
         <v>46153</v>
       </c>
       <c r="X235" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y235" s="10">
         <v>0</v>
@@ -32952,7 +33033,7 @@
         <v>53</v>
       </c>
       <c r="AI235" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ235" s="3" t="s">
         <v>52</v>
@@ -32979,7 +33060,7 @@
         <v>53</v>
       </c>
       <c r="AR235" s="3" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="236" spans="1:44" x14ac:dyDescent="0.3">
@@ -32990,10 +33071,10 @@
         <v>2</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D236" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E236" s="3" t="s">
         <v>46</v>
@@ -33002,7 +33083,7 @@
         <v>46153</v>
       </c>
       <c r="G236" s="5">
-        <v>7</v>
+        <v>345</v>
       </c>
       <c r="H236" s="3" t="s">
         <v>47</v>
@@ -33017,19 +33098,19 @@
         <v>50</v>
       </c>
       <c r="L236" s="6">
-        <v>869</v>
+        <v>854</v>
       </c>
       <c r="M236" s="7">
-        <v>363254.42</v>
+        <v>161262.14000000001</v>
       </c>
       <c r="N236" s="6">
         <v>1</v>
       </c>
       <c r="O236" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P236" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q236" s="6">
         <v>0</v>
@@ -33044,7 +33125,7 @@
         <v>52</v>
       </c>
       <c r="U236" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V236" s="11">
         <v>11</v>
@@ -33053,7 +33134,7 @@
         <v>46153</v>
       </c>
       <c r="X236" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y236" s="10">
         <v>0</v>
@@ -33086,7 +33167,7 @@
         <v>53</v>
       </c>
       <c r="AI236" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ236" s="3" t="s">
         <v>52</v>
@@ -33113,7 +33194,7 @@
         <v>53</v>
       </c>
       <c r="AR236" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="237" spans="1:44" x14ac:dyDescent="0.3">
@@ -33124,10 +33205,10 @@
         <v>2</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D237" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E237" s="3" t="s">
         <v>46</v>
@@ -33136,7 +33217,7 @@
         <v>46153</v>
       </c>
       <c r="G237" s="5">
-        <v>8</v>
+        <v>346</v>
       </c>
       <c r="H237" s="3" t="s">
         <v>47</v>
@@ -33151,19 +33232,19 @@
         <v>50</v>
       </c>
       <c r="L237" s="6">
-        <v>870</v>
+        <v>855</v>
       </c>
       <c r="M237" s="7">
-        <v>363672.43</v>
+        <v>161450.97</v>
       </c>
       <c r="N237" s="6">
         <v>1</v>
       </c>
       <c r="O237" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P237" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q237" s="6">
         <v>0</v>
@@ -33178,7 +33259,7 @@
         <v>52</v>
       </c>
       <c r="U237" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V237" s="11">
         <v>11</v>
@@ -33187,7 +33268,7 @@
         <v>46153</v>
       </c>
       <c r="X237" s="12">
-        <v>0.35763889999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y237" s="10">
         <v>0</v>
@@ -33220,7 +33301,7 @@
         <v>53</v>
       </c>
       <c r="AI237" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ237" s="3" t="s">
         <v>52</v>
@@ -33247,7 +33328,7 @@
         <v>53</v>
       </c>
       <c r="AR237" s="3" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="238" spans="1:44" x14ac:dyDescent="0.3">
@@ -33258,10 +33339,10 @@
         <v>2</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D238" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E238" s="3" t="s">
         <v>46</v>
@@ -33270,7 +33351,7 @@
         <v>46153</v>
       </c>
       <c r="G238" s="5">
-        <v>9</v>
+        <v>347</v>
       </c>
       <c r="H238" s="3" t="s">
         <v>47</v>
@@ -33285,19 +33366,19 @@
         <v>50</v>
       </c>
       <c r="L238" s="6">
-        <v>871</v>
+        <v>856</v>
       </c>
       <c r="M238" s="7">
-        <v>364090.45</v>
+        <v>161639.79999999999</v>
       </c>
       <c r="N238" s="6">
         <v>1</v>
       </c>
       <c r="O238" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P238" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q238" s="6">
         <v>0</v>
@@ -33312,7 +33393,7 @@
         <v>52</v>
       </c>
       <c r="U238" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V238" s="11">
         <v>11</v>
@@ -33321,7 +33402,7 @@
         <v>46153</v>
       </c>
       <c r="X238" s="12">
-        <v>0.39930559999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y238" s="10">
         <v>0</v>
@@ -33354,7 +33435,7 @@
         <v>53</v>
       </c>
       <c r="AI238" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ238" s="3" t="s">
         <v>52</v>
@@ -33381,7 +33462,7 @@
         <v>53</v>
       </c>
       <c r="AR238" s="3" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="239" spans="1:44" x14ac:dyDescent="0.3">
@@ -33392,10 +33473,10 @@
         <v>2</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D239" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E239" s="3" t="s">
         <v>46</v>
@@ -33404,7 +33485,7 @@
         <v>46153</v>
       </c>
       <c r="G239" s="5">
-        <v>10</v>
+        <v>348</v>
       </c>
       <c r="H239" s="3" t="s">
         <v>47</v>
@@ -33419,19 +33500,19 @@
         <v>50</v>
       </c>
       <c r="L239" s="6">
-        <v>872</v>
+        <v>857</v>
       </c>
       <c r="M239" s="7">
-        <v>364508.46</v>
+        <v>161828.64000000001</v>
       </c>
       <c r="N239" s="6">
         <v>1</v>
       </c>
       <c r="O239" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P239" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q239" s="6">
         <v>0</v>
@@ -33446,7 +33527,7 @@
         <v>52</v>
       </c>
       <c r="U239" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V239" s="11">
         <v>11</v>
@@ -33455,7 +33536,7 @@
         <v>46153</v>
       </c>
       <c r="X239" s="12">
-        <v>0.39930559999999998</v>
+        <v>0.50347220000000004</v>
       </c>
       <c r="Y239" s="10">
         <v>0</v>
@@ -33488,7 +33569,7 @@
         <v>53</v>
       </c>
       <c r="AI239" s="3" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
       <c r="AJ239" s="3" t="s">
         <v>52</v>
@@ -33515,7 +33596,7 @@
         <v>53</v>
       </c>
       <c r="AR239" s="3" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="240" spans="1:44" x14ac:dyDescent="0.3">
@@ -33526,10 +33607,10 @@
         <v>2</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>283</v>
+        <v>44</v>
       </c>
       <c r="D240" s="3" t="s">
-        <v>284</v>
+        <v>45</v>
       </c>
       <c r="E240" s="3" t="s">
         <v>46</v>
@@ -33538,7 +33619,7 @@
         <v>46153</v>
       </c>
       <c r="G240" s="5">
-        <v>11</v>
+        <v>349</v>
       </c>
       <c r="H240" s="3" t="s">
         <v>47</v>
@@ -33553,19 +33634,19 @@
         <v>50</v>
       </c>
       <c r="L240" s="6">
-        <v>873</v>
+        <v>858</v>
       </c>
       <c r="M240" s="7">
-        <v>364926.48</v>
+        <v>162017.47</v>
       </c>
       <c r="N240" s="6">
         <v>1</v>
       </c>
       <c r="O240" s="3" t="s">
-        <v>285</v>
+        <v>51</v>
       </c>
       <c r="P240" s="8">
-        <v>418.01</v>
+        <v>188.83</v>
       </c>
       <c r="Q240" s="6">
         <v>0</v>
@@ -33580,7 +33661,7 @@
         <v>52</v>
       </c>
       <c r="U240" s="10">
-        <v>64026</v>
+        <v>64209</v>
       </c>
       <c r="V240" s="11">
         <v>11</v>
@@ -33589,67 +33670,3685 @@
         <v>46153</v>
       </c>
       <c r="X240" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y240" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB240" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG240" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI240" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ240" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK240" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL240" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM240" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ240" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR240" s="3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="241" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A241" s="1">
+        <v>1</v>
+      </c>
+      <c r="B241" s="2">
+        <v>2</v>
+      </c>
+      <c r="C241" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D241" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E241" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F241" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G241" s="5">
+        <v>350</v>
+      </c>
+      <c r="H241" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I241" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J241" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K241" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L241" s="6">
+        <v>859</v>
+      </c>
+      <c r="M241" s="7">
+        <v>162206.29999999999</v>
+      </c>
+      <c r="N241" s="6">
+        <v>1</v>
+      </c>
+      <c r="O241" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P241" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q241" s="6">
+        <v>0</v>
+      </c>
+      <c r="R241" s="7">
+        <v>0</v>
+      </c>
+      <c r="S241" s="9">
+        <v>0</v>
+      </c>
+      <c r="T241" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U241" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V241" s="11">
+        <v>11</v>
+      </c>
+      <c r="W241" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X241" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y241" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB241" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG241" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI241" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ241" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK241" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL241" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM241" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ241" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR241" s="3" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="242" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A242" s="1">
+        <v>1</v>
+      </c>
+      <c r="B242" s="2">
+        <v>2</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E242" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F242" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G242" s="5">
+        <v>351</v>
+      </c>
+      <c r="H242" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I242" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J242" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K242" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L242" s="6">
+        <v>860</v>
+      </c>
+      <c r="M242" s="7">
+        <v>162395.13</v>
+      </c>
+      <c r="N242" s="6">
+        <v>1</v>
+      </c>
+      <c r="O242" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P242" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q242" s="6">
+        <v>0</v>
+      </c>
+      <c r="R242" s="7">
+        <v>0</v>
+      </c>
+      <c r="S242" s="9">
+        <v>0</v>
+      </c>
+      <c r="T242" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U242" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V242" s="11">
+        <v>11</v>
+      </c>
+      <c r="W242" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X242" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y242" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB242" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG242" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI242" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ242" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK242" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL242" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM242" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ242" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR242" s="3" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="243" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A243" s="1">
+        <v>1</v>
+      </c>
+      <c r="B243" s="2">
+        <v>2</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D243" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E243" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F243" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G243" s="5">
+        <v>352</v>
+      </c>
+      <c r="H243" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I243" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J243" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K243" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L243" s="6">
+        <v>861</v>
+      </c>
+      <c r="M243" s="7">
+        <v>162583.96</v>
+      </c>
+      <c r="N243" s="6">
+        <v>1</v>
+      </c>
+      <c r="O243" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P243" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q243" s="6">
+        <v>0</v>
+      </c>
+      <c r="R243" s="7">
+        <v>0</v>
+      </c>
+      <c r="S243" s="9">
+        <v>0</v>
+      </c>
+      <c r="T243" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U243" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V243" s="11">
+        <v>11</v>
+      </c>
+      <c r="W243" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X243" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y243" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB243" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG243" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI243" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ243" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK243" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL243" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM243" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ243" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR243" s="3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="244" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A244" s="1">
+        <v>1</v>
+      </c>
+      <c r="B244" s="2">
+        <v>2</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D244" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E244" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F244" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G244" s="5">
+        <v>353</v>
+      </c>
+      <c r="H244" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I244" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J244" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K244" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L244" s="6">
+        <v>862</v>
+      </c>
+      <c r="M244" s="7">
+        <v>162772.79</v>
+      </c>
+      <c r="N244" s="6">
+        <v>1</v>
+      </c>
+      <c r="O244" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P244" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q244" s="6">
+        <v>0</v>
+      </c>
+      <c r="R244" s="7">
+        <v>0</v>
+      </c>
+      <c r="S244" s="9">
+        <v>0</v>
+      </c>
+      <c r="T244" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U244" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V244" s="11">
+        <v>11</v>
+      </c>
+      <c r="W244" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X244" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y244" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB244" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG244" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI244" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ244" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK244" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL244" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM244" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ244" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR244" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="245" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A245" s="1">
+        <v>1</v>
+      </c>
+      <c r="B245" s="2">
+        <v>2</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D245" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E245" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F245" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G245" s="5">
+        <v>354</v>
+      </c>
+      <c r="H245" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I245" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J245" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K245" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L245" s="6">
+        <v>863</v>
+      </c>
+      <c r="M245" s="7">
+        <v>162961.63</v>
+      </c>
+      <c r="N245" s="6">
+        <v>1</v>
+      </c>
+      <c r="O245" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P245" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q245" s="6">
+        <v>0</v>
+      </c>
+      <c r="R245" s="7">
+        <v>0</v>
+      </c>
+      <c r="S245" s="9">
+        <v>0</v>
+      </c>
+      <c r="T245" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U245" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V245" s="11">
+        <v>11</v>
+      </c>
+      <c r="W245" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X245" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y245" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB245" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG245" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI245" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ245" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK245" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL245" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM245" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ245" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR245" s="3" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="246" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A246" s="1">
+        <v>1</v>
+      </c>
+      <c r="B246" s="2">
+        <v>2</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D246" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E246" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F246" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G246" s="5">
+        <v>355</v>
+      </c>
+      <c r="H246" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I246" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J246" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K246" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L246" s="6">
+        <v>864</v>
+      </c>
+      <c r="M246" s="7">
+        <v>163150.46</v>
+      </c>
+      <c r="N246" s="6">
+        <v>1</v>
+      </c>
+      <c r="O246" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P246" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q246" s="6">
+        <v>0</v>
+      </c>
+      <c r="R246" s="7">
+        <v>0</v>
+      </c>
+      <c r="S246" s="9">
+        <v>0</v>
+      </c>
+      <c r="T246" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U246" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V246" s="11">
+        <v>11</v>
+      </c>
+      <c r="W246" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X246" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y246" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB246" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG246" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI246" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ246" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK246" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL246" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM246" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ246" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR246" s="3" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="247" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A247" s="1">
+        <v>1</v>
+      </c>
+      <c r="B247" s="2">
+        <v>2</v>
+      </c>
+      <c r="C247" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D247" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E247" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F247" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G247" s="5">
+        <v>356</v>
+      </c>
+      <c r="H247" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I247" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J247" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K247" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L247" s="6">
+        <v>865</v>
+      </c>
+      <c r="M247" s="7">
+        <v>163339.29</v>
+      </c>
+      <c r="N247" s="6">
+        <v>1</v>
+      </c>
+      <c r="O247" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P247" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q247" s="6">
+        <v>0</v>
+      </c>
+      <c r="R247" s="7">
+        <v>0</v>
+      </c>
+      <c r="S247" s="9">
+        <v>0</v>
+      </c>
+      <c r="T247" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U247" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V247" s="11">
+        <v>11</v>
+      </c>
+      <c r="W247" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X247" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y247" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB247" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG247" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI247" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ247" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK247" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL247" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM247" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ247" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR247" s="3" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="248" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A248" s="1">
+        <v>1</v>
+      </c>
+      <c r="B248" s="2">
+        <v>2</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E248" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F248" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G248" s="5">
+        <v>357</v>
+      </c>
+      <c r="H248" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I248" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J248" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K248" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L248" s="6">
+        <v>866</v>
+      </c>
+      <c r="M248" s="7">
+        <v>163528.12</v>
+      </c>
+      <c r="N248" s="6">
+        <v>1</v>
+      </c>
+      <c r="O248" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P248" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q248" s="6">
+        <v>0</v>
+      </c>
+      <c r="R248" s="7">
+        <v>0</v>
+      </c>
+      <c r="S248" s="9">
+        <v>0</v>
+      </c>
+      <c r="T248" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U248" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V248" s="11">
+        <v>11</v>
+      </c>
+      <c r="W248" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X248" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y248" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB248" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG248" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI248" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ248" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK248" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL248" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM248" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ248" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR248" s="3" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="249" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A249" s="1">
+        <v>1</v>
+      </c>
+      <c r="B249" s="2">
+        <v>2</v>
+      </c>
+      <c r="C249" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D249" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E249" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F249" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G249" s="5">
+        <v>358</v>
+      </c>
+      <c r="H249" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I249" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J249" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K249" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L249" s="6">
+        <v>867</v>
+      </c>
+      <c r="M249" s="7">
+        <v>163716.95000000001</v>
+      </c>
+      <c r="N249" s="6">
+        <v>1</v>
+      </c>
+      <c r="O249" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P249" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q249" s="6">
+        <v>0</v>
+      </c>
+      <c r="R249" s="7">
+        <v>0</v>
+      </c>
+      <c r="S249" s="9">
+        <v>0</v>
+      </c>
+      <c r="T249" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U249" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V249" s="11">
+        <v>11</v>
+      </c>
+      <c r="W249" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X249" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y249" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB249" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG249" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI249" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ249" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK249" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL249" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM249" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ249" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR249" s="3" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="250" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A250" s="1">
+        <v>1</v>
+      </c>
+      <c r="B250" s="2">
+        <v>2</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E250" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F250" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G250" s="5">
+        <v>359</v>
+      </c>
+      <c r="H250" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I250" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J250" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K250" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L250" s="6">
+        <v>868</v>
+      </c>
+      <c r="M250" s="7">
+        <v>163905.78</v>
+      </c>
+      <c r="N250" s="6">
+        <v>1</v>
+      </c>
+      <c r="O250" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P250" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q250" s="6">
+        <v>0</v>
+      </c>
+      <c r="R250" s="7">
+        <v>0</v>
+      </c>
+      <c r="S250" s="9">
+        <v>0</v>
+      </c>
+      <c r="T250" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U250" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V250" s="11">
+        <v>11</v>
+      </c>
+      <c r="W250" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X250" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y250" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB250" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG250" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI250" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ250" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK250" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL250" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM250" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ250" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR250" s="3" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="251" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A251" s="1">
+        <v>1</v>
+      </c>
+      <c r="B251" s="2">
+        <v>2</v>
+      </c>
+      <c r="C251" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D251" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E251" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F251" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G251" s="5">
+        <v>360</v>
+      </c>
+      <c r="H251" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I251" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J251" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K251" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L251" s="6">
+        <v>869</v>
+      </c>
+      <c r="M251" s="7">
+        <v>164094.60999999999</v>
+      </c>
+      <c r="N251" s="6">
+        <v>1</v>
+      </c>
+      <c r="O251" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P251" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q251" s="6">
+        <v>0</v>
+      </c>
+      <c r="R251" s="7">
+        <v>0</v>
+      </c>
+      <c r="S251" s="9">
+        <v>0</v>
+      </c>
+      <c r="T251" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U251" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V251" s="11">
+        <v>11</v>
+      </c>
+      <c r="W251" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X251" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y251" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB251" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG251" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI251" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ251" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK251" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL251" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM251" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ251" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR251" s="3" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="252" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A252" s="1">
+        <v>1</v>
+      </c>
+      <c r="B252" s="2">
+        <v>2</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E252" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F252" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G252" s="5">
+        <v>361</v>
+      </c>
+      <c r="H252" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I252" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J252" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K252" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L252" s="6">
+        <v>870</v>
+      </c>
+      <c r="M252" s="7">
+        <v>164283.45000000001</v>
+      </c>
+      <c r="N252" s="6">
+        <v>1</v>
+      </c>
+      <c r="O252" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P252" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q252" s="6">
+        <v>0</v>
+      </c>
+      <c r="R252" s="7">
+        <v>0</v>
+      </c>
+      <c r="S252" s="9">
+        <v>0</v>
+      </c>
+      <c r="T252" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U252" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V252" s="11">
+        <v>11</v>
+      </c>
+      <c r="W252" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X252" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y252" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB252" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG252" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI252" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ252" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK252" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL252" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM252" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ252" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR252" s="3" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="253" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A253" s="1">
+        <v>1</v>
+      </c>
+      <c r="B253" s="2">
+        <v>2</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D253" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E253" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F253" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G253" s="5">
+        <v>362</v>
+      </c>
+      <c r="H253" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I253" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J253" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K253" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L253" s="6">
+        <v>871</v>
+      </c>
+      <c r="M253" s="7">
+        <v>164472.28</v>
+      </c>
+      <c r="N253" s="6">
+        <v>1</v>
+      </c>
+      <c r="O253" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P253" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q253" s="6">
+        <v>0</v>
+      </c>
+      <c r="R253" s="7">
+        <v>0</v>
+      </c>
+      <c r="S253" s="9">
+        <v>0</v>
+      </c>
+      <c r="T253" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U253" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V253" s="11">
+        <v>11</v>
+      </c>
+      <c r="W253" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X253" s="12">
+        <v>0.50347220000000004</v>
+      </c>
+      <c r="Y253" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB253" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG253" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI253" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ253" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK253" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL253" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM253" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ253" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR253" s="3" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="254" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A254" s="1">
+        <v>1</v>
+      </c>
+      <c r="B254" s="2">
+        <v>2</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D254" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E254" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F254" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G254" s="5">
+        <v>363</v>
+      </c>
+      <c r="H254" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I254" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J254" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K254" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L254" s="6">
+        <v>872</v>
+      </c>
+      <c r="M254" s="7">
+        <v>164661.10999999999</v>
+      </c>
+      <c r="N254" s="6">
+        <v>1</v>
+      </c>
+      <c r="O254" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P254" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q254" s="6">
+        <v>0</v>
+      </c>
+      <c r="R254" s="7">
+        <v>0</v>
+      </c>
+      <c r="S254" s="9">
+        <v>0</v>
+      </c>
+      <c r="T254" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U254" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V254" s="11">
+        <v>11</v>
+      </c>
+      <c r="W254" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X254" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y254" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB254" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG254" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI254" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ254" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK254" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL254" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM254" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ254" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR254" s="3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="255" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A255" s="1">
+        <v>1</v>
+      </c>
+      <c r="B255" s="2">
+        <v>2</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D255" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E255" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F255" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G255" s="5">
+        <v>364</v>
+      </c>
+      <c r="H255" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I255" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J255" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K255" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L255" s="6">
+        <v>873</v>
+      </c>
+      <c r="M255" s="7">
+        <v>164849.94</v>
+      </c>
+      <c r="N255" s="6">
+        <v>1</v>
+      </c>
+      <c r="O255" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P255" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q255" s="6">
+        <v>0</v>
+      </c>
+      <c r="R255" s="7">
+        <v>0</v>
+      </c>
+      <c r="S255" s="9">
+        <v>0</v>
+      </c>
+      <c r="T255" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U255" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V255" s="11">
+        <v>11</v>
+      </c>
+      <c r="W255" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X255" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y255" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB255" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG255" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI255" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ255" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK255" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL255" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM255" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ255" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR255" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="256" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A256" s="1">
+        <v>1</v>
+      </c>
+      <c r="B256" s="2">
+        <v>2</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D256" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E256" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F256" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G256" s="5">
+        <v>365</v>
+      </c>
+      <c r="H256" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I256" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J256" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K256" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L256" s="6">
+        <v>874</v>
+      </c>
+      <c r="M256" s="7">
+        <v>165038.76999999999</v>
+      </c>
+      <c r="N256" s="6">
+        <v>1</v>
+      </c>
+      <c r="O256" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P256" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q256" s="6">
+        <v>0</v>
+      </c>
+      <c r="R256" s="7">
+        <v>0</v>
+      </c>
+      <c r="S256" s="9">
+        <v>0</v>
+      </c>
+      <c r="T256" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U256" s="10">
+        <v>64209</v>
+      </c>
+      <c r="V256" s="11">
+        <v>11</v>
+      </c>
+      <c r="W256" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X256" s="12">
+        <v>0.50416669999999997</v>
+      </c>
+      <c r="Y256" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB256" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG256" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI256" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ256" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK256" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL256" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM256" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ256" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR256" s="3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="257" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A257" s="1">
+        <v>1</v>
+      </c>
+      <c r="B257" s="2">
+        <v>2</v>
+      </c>
+      <c r="C257" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D257" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E257" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F257" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G257" s="5">
+        <v>1</v>
+      </c>
+      <c r="H257" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I257" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J257" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K257" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L257" s="6">
+        <v>863</v>
+      </c>
+      <c r="M257" s="7">
+        <v>360746.33</v>
+      </c>
+      <c r="N257" s="6">
+        <v>1</v>
+      </c>
+      <c r="O257" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P257" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q257" s="6">
+        <v>0</v>
+      </c>
+      <c r="R257" s="7">
+        <v>0</v>
+      </c>
+      <c r="S257" s="9">
+        <v>0</v>
+      </c>
+      <c r="T257" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U257" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V257" s="11">
+        <v>11</v>
+      </c>
+      <c r="W257" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X257" s="12">
+        <v>0.31597219999999998</v>
+      </c>
+      <c r="Y257" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB257" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG257" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI257" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ257" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK257" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL257" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM257" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ257" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR257" s="3" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="258" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A258" s="1">
+        <v>1</v>
+      </c>
+      <c r="B258" s="2">
+        <v>2</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D258" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E258" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F258" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G258" s="5">
+        <v>2</v>
+      </c>
+      <c r="H258" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I258" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J258" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K258" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L258" s="6">
+        <v>864</v>
+      </c>
+      <c r="M258" s="7">
+        <v>361164.35</v>
+      </c>
+      <c r="N258" s="6">
+        <v>1</v>
+      </c>
+      <c r="O258" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P258" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q258" s="6">
+        <v>0</v>
+      </c>
+      <c r="R258" s="7">
+        <v>0</v>
+      </c>
+      <c r="S258" s="9">
+        <v>0</v>
+      </c>
+      <c r="T258" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U258" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V258" s="11">
+        <v>11</v>
+      </c>
+      <c r="W258" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X258" s="12">
+        <v>0.31597219999999998</v>
+      </c>
+      <c r="Y258" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB258" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG258" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI258" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ258" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK258" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL258" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM258" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ258" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR258" s="3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="259" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A259" s="1">
+        <v>1</v>
+      </c>
+      <c r="B259" s="2">
+        <v>2</v>
+      </c>
+      <c r="C259" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D259" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E259" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F259" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G259" s="5">
+        <v>3</v>
+      </c>
+      <c r="H259" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I259" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J259" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K259" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L259" s="6">
+        <v>865</v>
+      </c>
+      <c r="M259" s="7">
+        <v>361582.36</v>
+      </c>
+      <c r="N259" s="6">
+        <v>1</v>
+      </c>
+      <c r="O259" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P259" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q259" s="6">
+        <v>0</v>
+      </c>
+      <c r="R259" s="7">
+        <v>0</v>
+      </c>
+      <c r="S259" s="9">
+        <v>0</v>
+      </c>
+      <c r="T259" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U259" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V259" s="11">
+        <v>11</v>
+      </c>
+      <c r="W259" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X259" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y259" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB259" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG259" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI259" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ259" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK259" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL259" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM259" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ259" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR259" s="3" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="260" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A260" s="1">
+        <v>1</v>
+      </c>
+      <c r="B260" s="2">
+        <v>2</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E260" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F260" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G260" s="5">
+        <v>4</v>
+      </c>
+      <c r="H260" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I260" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J260" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K260" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L260" s="6">
+        <v>866</v>
+      </c>
+      <c r="M260" s="7">
+        <v>362000.38</v>
+      </c>
+      <c r="N260" s="6">
+        <v>1</v>
+      </c>
+      <c r="O260" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P260" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q260" s="6">
+        <v>0</v>
+      </c>
+      <c r="R260" s="7">
+        <v>0</v>
+      </c>
+      <c r="S260" s="9">
+        <v>0</v>
+      </c>
+      <c r="T260" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U260" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V260" s="11">
+        <v>11</v>
+      </c>
+      <c r="W260" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X260" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y260" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB260" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG260" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI260" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ260" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK260" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL260" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM260" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ260" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR260" s="3" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="261" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A261" s="1">
+        <v>1</v>
+      </c>
+      <c r="B261" s="2">
+        <v>2</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D261" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E261" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F261" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G261" s="5">
+        <v>5</v>
+      </c>
+      <c r="H261" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I261" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J261" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K261" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L261" s="6">
+        <v>867</v>
+      </c>
+      <c r="M261" s="7">
+        <v>362418.39</v>
+      </c>
+      <c r="N261" s="6">
+        <v>1</v>
+      </c>
+      <c r="O261" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P261" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q261" s="6">
+        <v>0</v>
+      </c>
+      <c r="R261" s="7">
+        <v>0</v>
+      </c>
+      <c r="S261" s="9">
+        <v>0</v>
+      </c>
+      <c r="T261" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U261" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V261" s="11">
+        <v>11</v>
+      </c>
+      <c r="W261" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X261" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y261" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB261" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG261" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI261" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ261" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK261" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL261" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM261" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ261" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR261" s="3" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="262" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A262" s="1">
+        <v>1</v>
+      </c>
+      <c r="B262" s="2">
+        <v>2</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D262" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F262" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G262" s="5">
+        <v>6</v>
+      </c>
+      <c r="H262" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I262" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J262" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K262" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L262" s="6">
+        <v>868</v>
+      </c>
+      <c r="M262" s="7">
+        <v>362836.4</v>
+      </c>
+      <c r="N262" s="6">
+        <v>1</v>
+      </c>
+      <c r="O262" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P262" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q262" s="6">
+        <v>0</v>
+      </c>
+      <c r="R262" s="7">
+        <v>0</v>
+      </c>
+      <c r="S262" s="9">
+        <v>0</v>
+      </c>
+      <c r="T262" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U262" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V262" s="11">
+        <v>11</v>
+      </c>
+      <c r="W262" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X262" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y262" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB262" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG262" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI262" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ262" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK262" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL262" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM262" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ262" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR262" s="3" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="263" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A263" s="1">
+        <v>1</v>
+      </c>
+      <c r="B263" s="2">
+        <v>2</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D263" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E263" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F263" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G263" s="5">
+        <v>7</v>
+      </c>
+      <c r="H263" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I263" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J263" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K263" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L263" s="6">
+        <v>869</v>
+      </c>
+      <c r="M263" s="7">
+        <v>363254.42</v>
+      </c>
+      <c r="N263" s="6">
+        <v>1</v>
+      </c>
+      <c r="O263" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P263" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q263" s="6">
+        <v>0</v>
+      </c>
+      <c r="R263" s="7">
+        <v>0</v>
+      </c>
+      <c r="S263" s="9">
+        <v>0</v>
+      </c>
+      <c r="T263" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U263" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V263" s="11">
+        <v>11</v>
+      </c>
+      <c r="W263" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X263" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y263" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB263" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG263" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI263" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ263" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK263" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL263" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM263" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ263" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR263" s="3" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="264" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A264" s="1">
+        <v>1</v>
+      </c>
+      <c r="B264" s="2">
+        <v>2</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D264" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F264" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G264" s="5">
+        <v>8</v>
+      </c>
+      <c r="H264" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I264" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J264" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K264" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L264" s="6">
+        <v>870</v>
+      </c>
+      <c r="M264" s="7">
+        <v>363672.43</v>
+      </c>
+      <c r="N264" s="6">
+        <v>1</v>
+      </c>
+      <c r="O264" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P264" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q264" s="6">
+        <v>0</v>
+      </c>
+      <c r="R264" s="7">
+        <v>0</v>
+      </c>
+      <c r="S264" s="9">
+        <v>0</v>
+      </c>
+      <c r="T264" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U264" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V264" s="11">
+        <v>11</v>
+      </c>
+      <c r="W264" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X264" s="12">
+        <v>0.35763889999999998</v>
+      </c>
+      <c r="Y264" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB264" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG264" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI264" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ264" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK264" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL264" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM264" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ264" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR264" s="3" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="265" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A265" s="1">
+        <v>1</v>
+      </c>
+      <c r="B265" s="2">
+        <v>2</v>
+      </c>
+      <c r="C265" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D265" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E265" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F265" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G265" s="5">
+        <v>9</v>
+      </c>
+      <c r="H265" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I265" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J265" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K265" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L265" s="6">
+        <v>871</v>
+      </c>
+      <c r="M265" s="7">
+        <v>364090.45</v>
+      </c>
+      <c r="N265" s="6">
+        <v>1</v>
+      </c>
+      <c r="O265" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P265" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q265" s="6">
+        <v>0</v>
+      </c>
+      <c r="R265" s="7">
+        <v>0</v>
+      </c>
+      <c r="S265" s="9">
+        <v>0</v>
+      </c>
+      <c r="T265" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U265" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V265" s="11">
+        <v>11</v>
+      </c>
+      <c r="W265" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X265" s="12">
         <v>0.39930559999999998</v>
       </c>
-      <c r="Y240" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z240" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA240" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB240" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC240" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD240" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE240" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF240" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG240" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH240" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI240" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="AJ240" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK240" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL240" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM240" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN240" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO240" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP240" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ240" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR240" s="3" t="s">
-        <v>297</v>
+      <c r="Y265" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB265" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG265" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI265" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ265" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK265" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL265" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM265" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ265" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR265" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="266" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A266" s="1">
+        <v>1</v>
+      </c>
+      <c r="B266" s="2">
+        <v>2</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D266" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E266" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F266" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G266" s="5">
+        <v>10</v>
+      </c>
+      <c r="H266" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I266" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J266" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K266" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L266" s="6">
+        <v>872</v>
+      </c>
+      <c r="M266" s="7">
+        <v>364508.46</v>
+      </c>
+      <c r="N266" s="6">
+        <v>1</v>
+      </c>
+      <c r="O266" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P266" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q266" s="6">
+        <v>0</v>
+      </c>
+      <c r="R266" s="7">
+        <v>0</v>
+      </c>
+      <c r="S266" s="9">
+        <v>0</v>
+      </c>
+      <c r="T266" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U266" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V266" s="11">
+        <v>11</v>
+      </c>
+      <c r="W266" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X266" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y266" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB266" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG266" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI266" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ266" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK266" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL266" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM266" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ266" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR266" s="3" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="267" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A267" s="1">
+        <v>1</v>
+      </c>
+      <c r="B267" s="2">
+        <v>2</v>
+      </c>
+      <c r="C267" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="D267" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E267" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F267" s="4">
+        <v>46153</v>
+      </c>
+      <c r="G267" s="5">
+        <v>11</v>
+      </c>
+      <c r="H267" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I267" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J267" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K267" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L267" s="6">
+        <v>873</v>
+      </c>
+      <c r="M267" s="7">
+        <v>364926.48</v>
+      </c>
+      <c r="N267" s="6">
+        <v>1</v>
+      </c>
+      <c r="O267" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="P267" s="8">
+        <v>418.01</v>
+      </c>
+      <c r="Q267" s="6">
+        <v>0</v>
+      </c>
+      <c r="R267" s="7">
+        <v>0</v>
+      </c>
+      <c r="S267" s="9">
+        <v>0</v>
+      </c>
+      <c r="T267" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U267" s="10">
+        <v>64026</v>
+      </c>
+      <c r="V267" s="11">
+        <v>11</v>
+      </c>
+      <c r="W267" s="4">
+        <v>46153</v>
+      </c>
+      <c r="X267" s="12">
+        <v>0.39930559999999998</v>
+      </c>
+      <c r="Y267" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB267" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG267" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI267" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AJ267" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK267" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL267" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM267" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ267" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR267" s="3" t="s">
+        <v>324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 12/05/2026 16:41:51,11
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B02F167-469C-43A7-B4BD-89FCC2035726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2DFBC8E-F5B3-4222-AD8B-78FAB5A4265B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9116" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9260" uniqueCount="572">
   <si>
     <t>Sel</t>
   </si>
@@ -1540,6 +1540,30 @@
     <t>1879900000192</t>
   </si>
   <si>
+    <t>1879900000193</t>
+  </si>
+  <si>
+    <t>1879900000194</t>
+  </si>
+  <si>
+    <t>1879900000195</t>
+  </si>
+  <si>
+    <t>1879900000196</t>
+  </si>
+  <si>
+    <t>1879900000197</t>
+  </si>
+  <si>
+    <t>1879900000198</t>
+  </si>
+  <si>
+    <t>1879900000199</t>
+  </si>
+  <si>
+    <t>1879900000200</t>
+  </si>
+  <si>
     <t>36118965</t>
   </si>
   <si>
@@ -2287,7 +2311,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR505"/>
+  <dimension ref="A1:AR513"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -62464,7 +62488,7 @@
         <v>2</v>
       </c>
       <c r="C450" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D450" s="3" t="s">
         <v>45</v>
@@ -62476,7 +62500,7 @@
         <v>46154</v>
       </c>
       <c r="G450" s="5">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="H450" s="3" t="s">
         <v>47</v>
@@ -62491,19 +62515,19 @@
         <v>50</v>
       </c>
       <c r="L450" s="6">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="M450" s="7">
-        <v>6355.14</v>
+        <v>12746.5</v>
       </c>
       <c r="N450" s="6">
         <v>1</v>
       </c>
       <c r="O450" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P450" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q450" s="6">
         <v>0</v>
@@ -62518,7 +62542,7 @@
         <v>52</v>
       </c>
       <c r="U450" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V450" s="11">
         <v>11</v>
@@ -62527,7 +62551,7 @@
         <v>46154</v>
       </c>
       <c r="X450" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67291670000000003</v>
       </c>
       <c r="Y450" s="10">
         <v>0</v>
@@ -62587,7 +62611,7 @@
         <v>53</v>
       </c>
       <c r="AR450" s="3" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="451" spans="1:44" x14ac:dyDescent="0.3">
@@ -62598,7 +62622,7 @@
         <v>2</v>
       </c>
       <c r="C451" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D451" s="3" t="s">
         <v>45</v>
@@ -62610,7 +62634,7 @@
         <v>46154</v>
       </c>
       <c r="G451" s="5">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="H451" s="3" t="s">
         <v>47</v>
@@ -62625,19 +62649,19 @@
         <v>50</v>
       </c>
       <c r="L451" s="6">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="M451" s="7">
-        <v>6644.01</v>
+        <v>13121.4</v>
       </c>
       <c r="N451" s="6">
         <v>1</v>
       </c>
       <c r="O451" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P451" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q451" s="6">
         <v>0</v>
@@ -62652,7 +62676,7 @@
         <v>52</v>
       </c>
       <c r="U451" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V451" s="11">
         <v>11</v>
@@ -62661,7 +62685,7 @@
         <v>46154</v>
       </c>
       <c r="X451" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67291670000000003</v>
       </c>
       <c r="Y451" s="10">
         <v>0</v>
@@ -62721,7 +62745,7 @@
         <v>53</v>
       </c>
       <c r="AR451" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="452" spans="1:44" x14ac:dyDescent="0.3">
@@ -62732,7 +62756,7 @@
         <v>2</v>
       </c>
       <c r="C452" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D452" s="3" t="s">
         <v>45</v>
@@ -62744,7 +62768,7 @@
         <v>46154</v>
       </c>
       <c r="G452" s="5">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H452" s="3" t="s">
         <v>47</v>
@@ -62759,19 +62783,19 @@
         <v>50</v>
       </c>
       <c r="L452" s="6">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="M452" s="7">
-        <v>6932.88</v>
+        <v>13496.29</v>
       </c>
       <c r="N452" s="6">
         <v>1</v>
       </c>
       <c r="O452" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P452" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q452" s="6">
         <v>0</v>
@@ -62786,7 +62810,7 @@
         <v>52</v>
       </c>
       <c r="U452" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V452" s="11">
         <v>11</v>
@@ -62795,7 +62819,7 @@
         <v>46154</v>
       </c>
       <c r="X452" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67361110000000002</v>
       </c>
       <c r="Y452" s="10">
         <v>0</v>
@@ -62855,7 +62879,7 @@
         <v>53</v>
       </c>
       <c r="AR452" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="453" spans="1:44" x14ac:dyDescent="0.3">
@@ -62866,7 +62890,7 @@
         <v>2</v>
       </c>
       <c r="C453" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D453" s="3" t="s">
         <v>45</v>
@@ -62878,7 +62902,7 @@
         <v>46154</v>
       </c>
       <c r="G453" s="5">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H453" s="3" t="s">
         <v>47</v>
@@ -62893,19 +62917,19 @@
         <v>50</v>
       </c>
       <c r="L453" s="6">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="M453" s="7">
-        <v>7221.75</v>
+        <v>13871.19</v>
       </c>
       <c r="N453" s="6">
         <v>1</v>
       </c>
       <c r="O453" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P453" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q453" s="6">
         <v>0</v>
@@ -62920,7 +62944,7 @@
         <v>52</v>
       </c>
       <c r="U453" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V453" s="11">
         <v>11</v>
@@ -62929,7 +62953,7 @@
         <v>46154</v>
       </c>
       <c r="X453" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67361110000000002</v>
       </c>
       <c r="Y453" s="10">
         <v>0</v>
@@ -62989,7 +63013,7 @@
         <v>53</v>
       </c>
       <c r="AR453" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="454" spans="1:44" x14ac:dyDescent="0.3">
@@ -63000,7 +63024,7 @@
         <v>2</v>
       </c>
       <c r="C454" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D454" s="3" t="s">
         <v>45</v>
@@ -63012,7 +63036,7 @@
         <v>46154</v>
       </c>
       <c r="G454" s="5">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="H454" s="3" t="s">
         <v>47</v>
@@ -63027,19 +63051,19 @@
         <v>50</v>
       </c>
       <c r="L454" s="6">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="M454" s="7">
-        <v>7510.62</v>
+        <v>14246.09</v>
       </c>
       <c r="N454" s="6">
         <v>1</v>
       </c>
       <c r="O454" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P454" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q454" s="6">
         <v>0</v>
@@ -63054,7 +63078,7 @@
         <v>52</v>
       </c>
       <c r="U454" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V454" s="11">
         <v>11</v>
@@ -63063,7 +63087,7 @@
         <v>46154</v>
       </c>
       <c r="X454" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67361110000000002</v>
       </c>
       <c r="Y454" s="10">
         <v>0</v>
@@ -63123,7 +63147,7 @@
         <v>53</v>
       </c>
       <c r="AR454" s="3" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="455" spans="1:44" x14ac:dyDescent="0.3">
@@ -63134,7 +63158,7 @@
         <v>2</v>
       </c>
       <c r="C455" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D455" s="3" t="s">
         <v>45</v>
@@ -63146,7 +63170,7 @@
         <v>46154</v>
       </c>
       <c r="G455" s="5">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="H455" s="3" t="s">
         <v>47</v>
@@ -63161,19 +63185,19 @@
         <v>50</v>
       </c>
       <c r="L455" s="6">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="M455" s="7">
-        <v>7799.49</v>
+        <v>14620.99</v>
       </c>
       <c r="N455" s="6">
         <v>1</v>
       </c>
       <c r="O455" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P455" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q455" s="6">
         <v>0</v>
@@ -63188,7 +63212,7 @@
         <v>52</v>
       </c>
       <c r="U455" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V455" s="11">
         <v>11</v>
@@ -63197,7 +63221,7 @@
         <v>46154</v>
       </c>
       <c r="X455" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67361110000000002</v>
       </c>
       <c r="Y455" s="10">
         <v>0</v>
@@ -63257,7 +63281,7 @@
         <v>53</v>
       </c>
       <c r="AR455" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="456" spans="1:44" x14ac:dyDescent="0.3">
@@ -63268,7 +63292,7 @@
         <v>2</v>
       </c>
       <c r="C456" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D456" s="3" t="s">
         <v>45</v>
@@ -63280,7 +63304,7 @@
         <v>46154</v>
       </c>
       <c r="G456" s="5">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H456" s="3" t="s">
         <v>47</v>
@@ -63295,19 +63319,19 @@
         <v>50</v>
       </c>
       <c r="L456" s="6">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="M456" s="7">
-        <v>8088.36</v>
+        <v>14995.88</v>
       </c>
       <c r="N456" s="6">
         <v>1</v>
       </c>
       <c r="O456" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P456" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q456" s="6">
         <v>0</v>
@@ -63322,7 +63346,7 @@
         <v>52</v>
       </c>
       <c r="U456" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V456" s="11">
         <v>11</v>
@@ -63331,7 +63355,7 @@
         <v>46154</v>
       </c>
       <c r="X456" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67361110000000002</v>
       </c>
       <c r="Y456" s="10">
         <v>0</v>
@@ -63391,7 +63415,7 @@
         <v>53</v>
       </c>
       <c r="AR456" s="3" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="457" spans="1:44" x14ac:dyDescent="0.3">
@@ -63402,7 +63426,7 @@
         <v>2</v>
       </c>
       <c r="C457" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="D457" s="3" t="s">
         <v>45</v>
@@ -63414,7 +63438,7 @@
         <v>46154</v>
       </c>
       <c r="G457" s="5">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H457" s="3" t="s">
         <v>47</v>
@@ -63429,19 +63453,19 @@
         <v>50</v>
       </c>
       <c r="L457" s="6">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="M457" s="7">
-        <v>8377.23</v>
+        <v>15370.78</v>
       </c>
       <c r="N457" s="6">
         <v>1</v>
       </c>
       <c r="O457" s="3" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="P457" s="8">
-        <v>288.87</v>
+        <v>374.9</v>
       </c>
       <c r="Q457" s="6">
         <v>0</v>
@@ -63456,7 +63480,7 @@
         <v>52</v>
       </c>
       <c r="U457" s="10">
-        <v>64285</v>
+        <v>64288</v>
       </c>
       <c r="V457" s="11">
         <v>11</v>
@@ -63465,7 +63489,7 @@
         <v>46154</v>
       </c>
       <c r="X457" s="12">
-        <v>0.38194440000000002</v>
+        <v>0.67361110000000002</v>
       </c>
       <c r="Y457" s="10">
         <v>0</v>
@@ -63525,7 +63549,7 @@
         <v>53</v>
       </c>
       <c r="AR457" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="458" spans="1:44" x14ac:dyDescent="0.3">
@@ -63536,7 +63560,7 @@
         <v>2</v>
       </c>
       <c r="C458" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D458" s="3" t="s">
         <v>45</v>
@@ -63548,7 +63572,7 @@
         <v>46154</v>
       </c>
       <c r="G458" s="5">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="H458" s="3" t="s">
         <v>47</v>
@@ -63563,16 +63587,16 @@
         <v>50</v>
       </c>
       <c r="L458" s="6">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="M458" s="7">
-        <v>8666.1</v>
+        <v>6355.14</v>
       </c>
       <c r="N458" s="6">
         <v>1</v>
       </c>
       <c r="O458" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P458" s="8">
         <v>288.87</v>
@@ -63670,7 +63694,7 @@
         <v>2</v>
       </c>
       <c r="C459" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D459" s="3" t="s">
         <v>45</v>
@@ -63682,7 +63706,7 @@
         <v>46154</v>
       </c>
       <c r="G459" s="5">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H459" s="3" t="s">
         <v>47</v>
@@ -63697,16 +63721,16 @@
         <v>50</v>
       </c>
       <c r="L459" s="6">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="M459" s="7">
-        <v>8954.9699999999993</v>
+        <v>6644.01</v>
       </c>
       <c r="N459" s="6">
         <v>1</v>
       </c>
       <c r="O459" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P459" s="8">
         <v>288.87</v>
@@ -63804,7 +63828,7 @@
         <v>2</v>
       </c>
       <c r="C460" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D460" s="3" t="s">
         <v>45</v>
@@ -63816,7 +63840,7 @@
         <v>46154</v>
       </c>
       <c r="G460" s="5">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H460" s="3" t="s">
         <v>47</v>
@@ -63831,16 +63855,16 @@
         <v>50</v>
       </c>
       <c r="L460" s="6">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="M460" s="7">
-        <v>9243.84</v>
+        <v>6932.88</v>
       </c>
       <c r="N460" s="6">
         <v>1</v>
       </c>
       <c r="O460" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P460" s="8">
         <v>288.87</v>
@@ -63938,7 +63962,7 @@
         <v>2</v>
       </c>
       <c r="C461" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D461" s="3" t="s">
         <v>45</v>
@@ -63950,7 +63974,7 @@
         <v>46154</v>
       </c>
       <c r="G461" s="5">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H461" s="3" t="s">
         <v>47</v>
@@ -63965,16 +63989,16 @@
         <v>50</v>
       </c>
       <c r="L461" s="6">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="M461" s="7">
-        <v>9532.7099999999991</v>
+        <v>7221.75</v>
       </c>
       <c r="N461" s="6">
         <v>1</v>
       </c>
       <c r="O461" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P461" s="8">
         <v>288.87</v>
@@ -64072,7 +64096,7 @@
         <v>2</v>
       </c>
       <c r="C462" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D462" s="3" t="s">
         <v>45</v>
@@ -64084,7 +64108,7 @@
         <v>46154</v>
       </c>
       <c r="G462" s="5">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="H462" s="3" t="s">
         <v>47</v>
@@ -64099,16 +64123,16 @@
         <v>50</v>
       </c>
       <c r="L462" s="6">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="M462" s="7">
-        <v>9821.58</v>
+        <v>7510.62</v>
       </c>
       <c r="N462" s="6">
         <v>1</v>
       </c>
       <c r="O462" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P462" s="8">
         <v>288.87</v>
@@ -64206,7 +64230,7 @@
         <v>2</v>
       </c>
       <c r="C463" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D463" s="3" t="s">
         <v>45</v>
@@ -64218,7 +64242,7 @@
         <v>46154</v>
       </c>
       <c r="G463" s="5">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H463" s="3" t="s">
         <v>47</v>
@@ -64233,16 +64257,16 @@
         <v>50</v>
       </c>
       <c r="L463" s="6">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="M463" s="7">
-        <v>10110.450000000001</v>
+        <v>7799.49</v>
       </c>
       <c r="N463" s="6">
         <v>1</v>
       </c>
       <c r="O463" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P463" s="8">
         <v>288.87</v>
@@ -64340,7 +64364,7 @@
         <v>2</v>
       </c>
       <c r="C464" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D464" s="3" t="s">
         <v>45</v>
@@ -64352,7 +64376,7 @@
         <v>46154</v>
       </c>
       <c r="G464" s="5">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="H464" s="3" t="s">
         <v>47</v>
@@ -64367,16 +64391,16 @@
         <v>50</v>
       </c>
       <c r="L464" s="6">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M464" s="7">
-        <v>10399.32</v>
+        <v>8088.36</v>
       </c>
       <c r="N464" s="6">
         <v>1</v>
       </c>
       <c r="O464" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P464" s="8">
         <v>288.87</v>
@@ -64474,7 +64498,7 @@
         <v>2</v>
       </c>
       <c r="C465" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D465" s="3" t="s">
         <v>45</v>
@@ -64486,7 +64510,7 @@
         <v>46154</v>
       </c>
       <c r="G465" s="5">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="H465" s="3" t="s">
         <v>47</v>
@@ -64501,16 +64525,16 @@
         <v>50</v>
       </c>
       <c r="L465" s="6">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M465" s="7">
-        <v>10688.19</v>
+        <v>8377.23</v>
       </c>
       <c r="N465" s="6">
         <v>1</v>
       </c>
       <c r="O465" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P465" s="8">
         <v>288.87</v>
@@ -64608,7 +64632,7 @@
         <v>2</v>
       </c>
       <c r="C466" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D466" s="3" t="s">
         <v>45</v>
@@ -64620,7 +64644,7 @@
         <v>46154</v>
       </c>
       <c r="G466" s="5">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="H466" s="3" t="s">
         <v>47</v>
@@ -64635,16 +64659,16 @@
         <v>50</v>
       </c>
       <c r="L466" s="6">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="M466" s="7">
-        <v>10977.06</v>
+        <v>8666.1</v>
       </c>
       <c r="N466" s="6">
         <v>1</v>
       </c>
       <c r="O466" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P466" s="8">
         <v>288.87</v>
@@ -64742,7 +64766,7 @@
         <v>2</v>
       </c>
       <c r="C467" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D467" s="3" t="s">
         <v>45</v>
@@ -64754,7 +64778,7 @@
         <v>46154</v>
       </c>
       <c r="G467" s="5">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H467" s="3" t="s">
         <v>47</v>
@@ -64769,16 +64793,16 @@
         <v>50</v>
       </c>
       <c r="L467" s="6">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="M467" s="7">
-        <v>11265.93</v>
+        <v>8954.9699999999993</v>
       </c>
       <c r="N467" s="6">
         <v>1</v>
       </c>
       <c r="O467" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P467" s="8">
         <v>288.87</v>
@@ -64876,7 +64900,7 @@
         <v>2</v>
       </c>
       <c r="C468" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D468" s="3" t="s">
         <v>45</v>
@@ -64888,7 +64912,7 @@
         <v>46154</v>
       </c>
       <c r="G468" s="5">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H468" s="3" t="s">
         <v>47</v>
@@ -64903,16 +64927,16 @@
         <v>50</v>
       </c>
       <c r="L468" s="6">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="M468" s="7">
-        <v>11554.8</v>
+        <v>9243.84</v>
       </c>
       <c r="N468" s="6">
         <v>1</v>
       </c>
       <c r="O468" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P468" s="8">
         <v>288.87</v>
@@ -64939,7 +64963,7 @@
         <v>46154</v>
       </c>
       <c r="X468" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y468" s="10">
         <v>0</v>
@@ -65010,7 +65034,7 @@
         <v>2</v>
       </c>
       <c r="C469" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D469" s="3" t="s">
         <v>45</v>
@@ -65022,7 +65046,7 @@
         <v>46154</v>
       </c>
       <c r="G469" s="5">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H469" s="3" t="s">
         <v>47</v>
@@ -65037,16 +65061,16 @@
         <v>50</v>
       </c>
       <c r="L469" s="6">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="M469" s="7">
-        <v>11843.67</v>
+        <v>9532.7099999999991</v>
       </c>
       <c r="N469" s="6">
         <v>1</v>
       </c>
       <c r="O469" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P469" s="8">
         <v>288.87</v>
@@ -65073,7 +65097,7 @@
         <v>46154</v>
       </c>
       <c r="X469" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y469" s="10">
         <v>0</v>
@@ -65144,7 +65168,7 @@
         <v>2</v>
       </c>
       <c r="C470" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D470" s="3" t="s">
         <v>45</v>
@@ -65156,7 +65180,7 @@
         <v>46154</v>
       </c>
       <c r="G470" s="5">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="H470" s="3" t="s">
         <v>47</v>
@@ -65171,16 +65195,16 @@
         <v>50</v>
       </c>
       <c r="L470" s="6">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M470" s="7">
-        <v>12132.54</v>
+        <v>9821.58</v>
       </c>
       <c r="N470" s="6">
         <v>1</v>
       </c>
       <c r="O470" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P470" s="8">
         <v>288.87</v>
@@ -65207,7 +65231,7 @@
         <v>46154</v>
       </c>
       <c r="X470" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y470" s="10">
         <v>0</v>
@@ -65278,7 +65302,7 @@
         <v>2</v>
       </c>
       <c r="C471" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D471" s="3" t="s">
         <v>45</v>
@@ -65290,7 +65314,7 @@
         <v>46154</v>
       </c>
       <c r="G471" s="5">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="H471" s="3" t="s">
         <v>47</v>
@@ -65305,16 +65329,16 @@
         <v>50</v>
       </c>
       <c r="L471" s="6">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="M471" s="7">
-        <v>12421.41</v>
+        <v>10110.450000000001</v>
       </c>
       <c r="N471" s="6">
         <v>1</v>
       </c>
       <c r="O471" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P471" s="8">
         <v>288.87</v>
@@ -65341,7 +65365,7 @@
         <v>46154</v>
       </c>
       <c r="X471" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y471" s="10">
         <v>0</v>
@@ -65412,7 +65436,7 @@
         <v>2</v>
       </c>
       <c r="C472" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D472" s="3" t="s">
         <v>45</v>
@@ -65424,7 +65448,7 @@
         <v>46154</v>
       </c>
       <c r="G472" s="5">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="H472" s="3" t="s">
         <v>47</v>
@@ -65439,16 +65463,16 @@
         <v>50</v>
       </c>
       <c r="L472" s="6">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="M472" s="7">
-        <v>12710.28</v>
+        <v>10399.32</v>
       </c>
       <c r="N472" s="6">
         <v>1</v>
       </c>
       <c r="O472" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P472" s="8">
         <v>288.87</v>
@@ -65475,7 +65499,7 @@
         <v>46154</v>
       </c>
       <c r="X472" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y472" s="10">
         <v>0</v>
@@ -65546,7 +65570,7 @@
         <v>2</v>
       </c>
       <c r="C473" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D473" s="3" t="s">
         <v>45</v>
@@ -65558,7 +65582,7 @@
         <v>46154</v>
       </c>
       <c r="G473" s="5">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H473" s="3" t="s">
         <v>47</v>
@@ -65573,16 +65597,16 @@
         <v>50</v>
       </c>
       <c r="L473" s="6">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="M473" s="7">
-        <v>12999.15</v>
+        <v>10688.19</v>
       </c>
       <c r="N473" s="6">
         <v>1</v>
       </c>
       <c r="O473" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P473" s="8">
         <v>288.87</v>
@@ -65609,7 +65633,7 @@
         <v>46154</v>
       </c>
       <c r="X473" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y473" s="10">
         <v>0</v>
@@ -65680,7 +65704,7 @@
         <v>2</v>
       </c>
       <c r="C474" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D474" s="3" t="s">
         <v>45</v>
@@ -65692,7 +65716,7 @@
         <v>46154</v>
       </c>
       <c r="G474" s="5">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="H474" s="3" t="s">
         <v>47</v>
@@ -65707,16 +65731,16 @@
         <v>50</v>
       </c>
       <c r="L474" s="6">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="M474" s="7">
-        <v>13288.02</v>
+        <v>10977.06</v>
       </c>
       <c r="N474" s="6">
         <v>1</v>
       </c>
       <c r="O474" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P474" s="8">
         <v>288.87</v>
@@ -65743,7 +65767,7 @@
         <v>46154</v>
       </c>
       <c r="X474" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y474" s="10">
         <v>0</v>
@@ -65814,7 +65838,7 @@
         <v>2</v>
       </c>
       <c r="C475" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D475" s="3" t="s">
         <v>45</v>
@@ -65826,7 +65850,7 @@
         <v>46154</v>
       </c>
       <c r="G475" s="5">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="H475" s="3" t="s">
         <v>47</v>
@@ -65841,16 +65865,16 @@
         <v>50</v>
       </c>
       <c r="L475" s="6">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="M475" s="7">
-        <v>13576.89</v>
+        <v>11265.93</v>
       </c>
       <c r="N475" s="6">
         <v>1</v>
       </c>
       <c r="O475" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P475" s="8">
         <v>288.87</v>
@@ -65877,7 +65901,7 @@
         <v>46154</v>
       </c>
       <c r="X475" s="12">
-        <v>0.40208329999999998</v>
+        <v>0.38194440000000002</v>
       </c>
       <c r="Y475" s="10">
         <v>0</v>
@@ -65948,7 +65972,7 @@
         <v>2</v>
       </c>
       <c r="C476" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D476" s="3" t="s">
         <v>45</v>
@@ -65960,7 +65984,7 @@
         <v>46154</v>
       </c>
       <c r="G476" s="5">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="H476" s="3" t="s">
         <v>47</v>
@@ -65975,16 +65999,16 @@
         <v>50</v>
       </c>
       <c r="L476" s="6">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="M476" s="7">
-        <v>13865.76</v>
+        <v>11554.8</v>
       </c>
       <c r="N476" s="6">
         <v>1</v>
       </c>
       <c r="O476" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P476" s="8">
         <v>288.87</v>
@@ -66011,7 +66035,7 @@
         <v>46154</v>
       </c>
       <c r="X476" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y476" s="10">
         <v>0</v>
@@ -66082,7 +66106,7 @@
         <v>2</v>
       </c>
       <c r="C477" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D477" s="3" t="s">
         <v>45</v>
@@ -66094,7 +66118,7 @@
         <v>46154</v>
       </c>
       <c r="G477" s="5">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="H477" s="3" t="s">
         <v>47</v>
@@ -66109,16 +66133,16 @@
         <v>50</v>
       </c>
       <c r="L477" s="6">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="M477" s="7">
-        <v>14154.63</v>
+        <v>11843.67</v>
       </c>
       <c r="N477" s="6">
         <v>1</v>
       </c>
       <c r="O477" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P477" s="8">
         <v>288.87</v>
@@ -66145,7 +66169,7 @@
         <v>46154</v>
       </c>
       <c r="X477" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y477" s="10">
         <v>0</v>
@@ -66216,7 +66240,7 @@
         <v>2</v>
       </c>
       <c r="C478" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D478" s="3" t="s">
         <v>45</v>
@@ -66228,7 +66252,7 @@
         <v>46154</v>
       </c>
       <c r="G478" s="5">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="H478" s="3" t="s">
         <v>47</v>
@@ -66243,16 +66267,16 @@
         <v>50</v>
       </c>
       <c r="L478" s="6">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="M478" s="7">
-        <v>14443.5</v>
+        <v>12132.54</v>
       </c>
       <c r="N478" s="6">
         <v>1</v>
       </c>
       <c r="O478" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P478" s="8">
         <v>288.87</v>
@@ -66279,7 +66303,7 @@
         <v>46154</v>
       </c>
       <c r="X478" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y478" s="10">
         <v>0</v>
@@ -66350,7 +66374,7 @@
         <v>2</v>
       </c>
       <c r="C479" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D479" s="3" t="s">
         <v>45</v>
@@ -66362,7 +66386,7 @@
         <v>46154</v>
       </c>
       <c r="G479" s="5">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H479" s="3" t="s">
         <v>47</v>
@@ -66377,16 +66401,16 @@
         <v>50</v>
       </c>
       <c r="L479" s="6">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="M479" s="7">
-        <v>14732.37</v>
+        <v>12421.41</v>
       </c>
       <c r="N479" s="6">
         <v>1</v>
       </c>
       <c r="O479" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P479" s="8">
         <v>288.87</v>
@@ -66413,7 +66437,7 @@
         <v>46154</v>
       </c>
       <c r="X479" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y479" s="10">
         <v>0</v>
@@ -66484,7 +66508,7 @@
         <v>2</v>
       </c>
       <c r="C480" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D480" s="3" t="s">
         <v>45</v>
@@ -66496,7 +66520,7 @@
         <v>46154</v>
       </c>
       <c r="G480" s="5">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H480" s="3" t="s">
         <v>47</v>
@@ -66511,16 +66535,16 @@
         <v>50</v>
       </c>
       <c r="L480" s="6">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="M480" s="7">
-        <v>15021.24</v>
+        <v>12710.28</v>
       </c>
       <c r="N480" s="6">
         <v>1</v>
       </c>
       <c r="O480" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P480" s="8">
         <v>288.87</v>
@@ -66547,7 +66571,7 @@
         <v>46154</v>
       </c>
       <c r="X480" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y480" s="10">
         <v>0</v>
@@ -66618,7 +66642,7 @@
         <v>2</v>
       </c>
       <c r="C481" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D481" s="3" t="s">
         <v>45</v>
@@ -66630,7 +66654,7 @@
         <v>46154</v>
       </c>
       <c r="G481" s="5">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="H481" s="3" t="s">
         <v>47</v>
@@ -66645,16 +66669,16 @@
         <v>50</v>
       </c>
       <c r="L481" s="6">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="M481" s="7">
-        <v>15310.11</v>
+        <v>12999.15</v>
       </c>
       <c r="N481" s="6">
         <v>1</v>
       </c>
       <c r="O481" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P481" s="8">
         <v>288.87</v>
@@ -66681,7 +66705,7 @@
         <v>46154</v>
       </c>
       <c r="X481" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y481" s="10">
         <v>0</v>
@@ -66752,7 +66776,7 @@
         <v>2</v>
       </c>
       <c r="C482" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D482" s="3" t="s">
         <v>45</v>
@@ -66764,7 +66788,7 @@
         <v>46154</v>
       </c>
       <c r="G482" s="5">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="H482" s="3" t="s">
         <v>47</v>
@@ -66779,16 +66803,16 @@
         <v>50</v>
       </c>
       <c r="L482" s="6">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="M482" s="7">
-        <v>15598.98</v>
+        <v>13288.02</v>
       </c>
       <c r="N482" s="6">
         <v>1</v>
       </c>
       <c r="O482" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P482" s="8">
         <v>288.87</v>
@@ -66815,7 +66839,7 @@
         <v>46154</v>
       </c>
       <c r="X482" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y482" s="10">
         <v>0</v>
@@ -66886,7 +66910,7 @@
         <v>2</v>
       </c>
       <c r="C483" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D483" s="3" t="s">
         <v>45</v>
@@ -66898,7 +66922,7 @@
         <v>46154</v>
       </c>
       <c r="G483" s="5">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="H483" s="3" t="s">
         <v>47</v>
@@ -66913,16 +66937,16 @@
         <v>50</v>
       </c>
       <c r="L483" s="6">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="M483" s="7">
-        <v>15887.85</v>
+        <v>13576.89</v>
       </c>
       <c r="N483" s="6">
         <v>1</v>
       </c>
       <c r="O483" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P483" s="8">
         <v>288.87</v>
@@ -66949,7 +66973,7 @@
         <v>46154</v>
       </c>
       <c r="X483" s="12">
-        <v>0.42291669999999998</v>
+        <v>0.40208329999999998</v>
       </c>
       <c r="Y483" s="10">
         <v>0</v>
@@ -67020,7 +67044,7 @@
         <v>2</v>
       </c>
       <c r="C484" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D484" s="3" t="s">
         <v>45</v>
@@ -67032,7 +67056,7 @@
         <v>46154</v>
       </c>
       <c r="G484" s="5">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H484" s="3" t="s">
         <v>47</v>
@@ -67047,16 +67071,16 @@
         <v>50</v>
       </c>
       <c r="L484" s="6">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="M484" s="7">
-        <v>16176.72</v>
+        <v>13865.76</v>
       </c>
       <c r="N484" s="6">
         <v>1</v>
       </c>
       <c r="O484" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P484" s="8">
         <v>288.87</v>
@@ -67083,7 +67107,7 @@
         <v>46154</v>
       </c>
       <c r="X484" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y484" s="10">
         <v>0</v>
@@ -67154,7 +67178,7 @@
         <v>2</v>
       </c>
       <c r="C485" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D485" s="3" t="s">
         <v>45</v>
@@ -67166,7 +67190,7 @@
         <v>46154</v>
       </c>
       <c r="G485" s="5">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="H485" s="3" t="s">
         <v>47</v>
@@ -67181,16 +67205,16 @@
         <v>50</v>
       </c>
       <c r="L485" s="6">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="M485" s="7">
-        <v>16465.59</v>
+        <v>14154.63</v>
       </c>
       <c r="N485" s="6">
         <v>1</v>
       </c>
       <c r="O485" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P485" s="8">
         <v>288.87</v>
@@ -67217,7 +67241,7 @@
         <v>46154</v>
       </c>
       <c r="X485" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y485" s="10">
         <v>0</v>
@@ -67288,7 +67312,7 @@
         <v>2</v>
       </c>
       <c r="C486" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D486" s="3" t="s">
         <v>45</v>
@@ -67300,7 +67324,7 @@
         <v>46154</v>
       </c>
       <c r="G486" s="5">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="H486" s="3" t="s">
         <v>47</v>
@@ -67315,16 +67339,16 @@
         <v>50</v>
       </c>
       <c r="L486" s="6">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M486" s="7">
-        <v>16754.46</v>
+        <v>14443.5</v>
       </c>
       <c r="N486" s="6">
         <v>1</v>
       </c>
       <c r="O486" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P486" s="8">
         <v>288.87</v>
@@ -67351,7 +67375,7 @@
         <v>46154</v>
       </c>
       <c r="X486" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y486" s="10">
         <v>0</v>
@@ -67422,7 +67446,7 @@
         <v>2</v>
       </c>
       <c r="C487" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D487" s="3" t="s">
         <v>45</v>
@@ -67434,7 +67458,7 @@
         <v>46154</v>
       </c>
       <c r="G487" s="5">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="H487" s="3" t="s">
         <v>47</v>
@@ -67449,16 +67473,16 @@
         <v>50</v>
       </c>
       <c r="L487" s="6">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="M487" s="7">
-        <v>17043.330000000002</v>
+        <v>14732.37</v>
       </c>
       <c r="N487" s="6">
         <v>1</v>
       </c>
       <c r="O487" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P487" s="8">
         <v>288.87</v>
@@ -67485,7 +67509,7 @@
         <v>46154</v>
       </c>
       <c r="X487" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y487" s="10">
         <v>0</v>
@@ -67556,7 +67580,7 @@
         <v>2</v>
       </c>
       <c r="C488" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D488" s="3" t="s">
         <v>45</v>
@@ -67568,7 +67592,7 @@
         <v>46154</v>
       </c>
       <c r="G488" s="5">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="H488" s="3" t="s">
         <v>47</v>
@@ -67583,16 +67607,16 @@
         <v>50</v>
       </c>
       <c r="L488" s="6">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="M488" s="7">
-        <v>17332.2</v>
+        <v>15021.24</v>
       </c>
       <c r="N488" s="6">
         <v>1</v>
       </c>
       <c r="O488" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P488" s="8">
         <v>288.87</v>
@@ -67619,7 +67643,7 @@
         <v>46154</v>
       </c>
       <c r="X488" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y488" s="10">
         <v>0</v>
@@ -67690,7 +67714,7 @@
         <v>2</v>
       </c>
       <c r="C489" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D489" s="3" t="s">
         <v>45</v>
@@ -67702,7 +67726,7 @@
         <v>46154</v>
       </c>
       <c r="G489" s="5">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H489" s="3" t="s">
         <v>47</v>
@@ -67717,16 +67741,16 @@
         <v>50</v>
       </c>
       <c r="L489" s="6">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="M489" s="7">
-        <v>17621.07</v>
+        <v>15310.11</v>
       </c>
       <c r="N489" s="6">
         <v>1</v>
       </c>
       <c r="O489" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P489" s="8">
         <v>288.87</v>
@@ -67753,7 +67777,7 @@
         <v>46154</v>
       </c>
       <c r="X489" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y489" s="10">
         <v>0</v>
@@ -67824,7 +67848,7 @@
         <v>2</v>
       </c>
       <c r="C490" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D490" s="3" t="s">
         <v>45</v>
@@ -67836,7 +67860,7 @@
         <v>46154</v>
       </c>
       <c r="G490" s="5">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H490" s="3" t="s">
         <v>47</v>
@@ -67851,16 +67875,16 @@
         <v>50</v>
       </c>
       <c r="L490" s="6">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="M490" s="7">
-        <v>17909.939999999999</v>
+        <v>15598.98</v>
       </c>
       <c r="N490" s="6">
         <v>1</v>
       </c>
       <c r="O490" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P490" s="8">
         <v>288.87</v>
@@ -67887,7 +67911,7 @@
         <v>46154</v>
       </c>
       <c r="X490" s="12">
-        <v>0.44444440000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y490" s="10">
         <v>0</v>
@@ -67958,7 +67982,7 @@
         <v>2</v>
       </c>
       <c r="C491" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D491" s="3" t="s">
         <v>45</v>
@@ -67970,7 +67994,7 @@
         <v>46154</v>
       </c>
       <c r="G491" s="5">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="H491" s="3" t="s">
         <v>47</v>
@@ -67985,16 +68009,16 @@
         <v>50</v>
       </c>
       <c r="L491" s="6">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="M491" s="7">
-        <v>18198.810000000001</v>
+        <v>15887.85</v>
       </c>
       <c r="N491" s="6">
         <v>1</v>
       </c>
       <c r="O491" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P491" s="8">
         <v>288.87</v>
@@ -68021,7 +68045,7 @@
         <v>46154</v>
       </c>
       <c r="X491" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.42291669999999998</v>
       </c>
       <c r="Y491" s="10">
         <v>0</v>
@@ -68092,7 +68116,7 @@
         <v>2</v>
       </c>
       <c r="C492" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D492" s="3" t="s">
         <v>45</v>
@@ -68104,7 +68128,7 @@
         <v>46154</v>
       </c>
       <c r="G492" s="5">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H492" s="3" t="s">
         <v>47</v>
@@ -68119,16 +68143,16 @@
         <v>50</v>
       </c>
       <c r="L492" s="6">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="M492" s="7">
-        <v>18487.68</v>
+        <v>16176.72</v>
       </c>
       <c r="N492" s="6">
         <v>1</v>
       </c>
       <c r="O492" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P492" s="8">
         <v>288.87</v>
@@ -68155,7 +68179,7 @@
         <v>46154</v>
       </c>
       <c r="X492" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y492" s="10">
         <v>0</v>
@@ -68226,7 +68250,7 @@
         <v>2</v>
       </c>
       <c r="C493" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D493" s="3" t="s">
         <v>45</v>
@@ -68238,7 +68262,7 @@
         <v>46154</v>
       </c>
       <c r="G493" s="5">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="H493" s="3" t="s">
         <v>47</v>
@@ -68253,16 +68277,16 @@
         <v>50</v>
       </c>
       <c r="L493" s="6">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="M493" s="7">
-        <v>18776.55</v>
+        <v>16465.59</v>
       </c>
       <c r="N493" s="6">
         <v>1</v>
       </c>
       <c r="O493" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P493" s="8">
         <v>288.87</v>
@@ -68289,7 +68313,7 @@
         <v>46154</v>
       </c>
       <c r="X493" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y493" s="10">
         <v>0</v>
@@ -68360,7 +68384,7 @@
         <v>2</v>
       </c>
       <c r="C494" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D494" s="3" t="s">
         <v>45</v>
@@ -68372,7 +68396,7 @@
         <v>46154</v>
       </c>
       <c r="G494" s="5">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="H494" s="3" t="s">
         <v>47</v>
@@ -68387,16 +68411,16 @@
         <v>50</v>
       </c>
       <c r="L494" s="6">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="M494" s="7">
-        <v>19065.419999999998</v>
+        <v>16754.46</v>
       </c>
       <c r="N494" s="6">
         <v>1</v>
       </c>
       <c r="O494" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P494" s="8">
         <v>288.87</v>
@@ -68423,7 +68447,7 @@
         <v>46154</v>
       </c>
       <c r="X494" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y494" s="10">
         <v>0</v>
@@ -68494,7 +68518,7 @@
         <v>2</v>
       </c>
       <c r="C495" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D495" s="3" t="s">
         <v>45</v>
@@ -68506,7 +68530,7 @@
         <v>46154</v>
       </c>
       <c r="G495" s="5">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="H495" s="3" t="s">
         <v>47</v>
@@ -68521,16 +68545,16 @@
         <v>50</v>
       </c>
       <c r="L495" s="6">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="M495" s="7">
-        <v>19354.29</v>
+        <v>17043.330000000002</v>
       </c>
       <c r="N495" s="6">
         <v>1</v>
       </c>
       <c r="O495" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P495" s="8">
         <v>288.87</v>
@@ -68557,7 +68581,7 @@
         <v>46154</v>
       </c>
       <c r="X495" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y495" s="10">
         <v>0</v>
@@ -68628,7 +68652,7 @@
         <v>2</v>
       </c>
       <c r="C496" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D496" s="3" t="s">
         <v>45</v>
@@ -68640,7 +68664,7 @@
         <v>46154</v>
       </c>
       <c r="G496" s="5">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="H496" s="3" t="s">
         <v>47</v>
@@ -68655,16 +68679,16 @@
         <v>50</v>
       </c>
       <c r="L496" s="6">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="M496" s="7">
-        <v>19643.16</v>
+        <v>17332.2</v>
       </c>
       <c r="N496" s="6">
         <v>1</v>
       </c>
       <c r="O496" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P496" s="8">
         <v>288.87</v>
@@ -68691,7 +68715,7 @@
         <v>46154</v>
       </c>
       <c r="X496" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y496" s="10">
         <v>0</v>
@@ -68762,7 +68786,7 @@
         <v>2</v>
       </c>
       <c r="C497" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D497" s="3" t="s">
         <v>45</v>
@@ -68774,7 +68798,7 @@
         <v>46154</v>
       </c>
       <c r="G497" s="5">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="H497" s="3" t="s">
         <v>47</v>
@@ -68789,16 +68813,16 @@
         <v>50</v>
       </c>
       <c r="L497" s="6">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="M497" s="7">
-        <v>19932.03</v>
+        <v>17621.07</v>
       </c>
       <c r="N497" s="6">
         <v>1</v>
       </c>
       <c r="O497" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P497" s="8">
         <v>288.87</v>
@@ -68825,7 +68849,7 @@
         <v>46154</v>
       </c>
       <c r="X497" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y497" s="10">
         <v>0</v>
@@ -68896,7 +68920,7 @@
         <v>2</v>
       </c>
       <c r="C498" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D498" s="3" t="s">
         <v>45</v>
@@ -68908,7 +68932,7 @@
         <v>46154</v>
       </c>
       <c r="G498" s="5">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="H498" s="3" t="s">
         <v>47</v>
@@ -68923,16 +68947,16 @@
         <v>50</v>
       </c>
       <c r="L498" s="6">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="M498" s="7">
-        <v>20220.900000000001</v>
+        <v>17909.939999999999</v>
       </c>
       <c r="N498" s="6">
         <v>1</v>
       </c>
       <c r="O498" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P498" s="8">
         <v>288.87</v>
@@ -68959,7 +68983,7 @@
         <v>46154</v>
       </c>
       <c r="X498" s="12">
-        <v>0.46527780000000002</v>
+        <v>0.44444440000000002</v>
       </c>
       <c r="Y498" s="10">
         <v>0</v>
@@ -69030,7 +69054,7 @@
         <v>2</v>
       </c>
       <c r="C499" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D499" s="3" t="s">
         <v>45</v>
@@ -69042,7 +69066,7 @@
         <v>46154</v>
       </c>
       <c r="G499" s="5">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="H499" s="3" t="s">
         <v>47</v>
@@ -69057,16 +69081,16 @@
         <v>50</v>
       </c>
       <c r="L499" s="6">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="M499" s="7">
-        <v>20509.77</v>
+        <v>18198.810000000001</v>
       </c>
       <c r="N499" s="6">
         <v>1</v>
       </c>
       <c r="O499" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P499" s="8">
         <v>288.87</v>
@@ -69093,7 +69117,7 @@
         <v>46154</v>
       </c>
       <c r="X499" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y499" s="10">
         <v>0</v>
@@ -69164,7 +69188,7 @@
         <v>2</v>
       </c>
       <c r="C500" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D500" s="3" t="s">
         <v>45</v>
@@ -69176,7 +69200,7 @@
         <v>46154</v>
       </c>
       <c r="G500" s="5">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="H500" s="3" t="s">
         <v>47</v>
@@ -69191,16 +69215,16 @@
         <v>50</v>
       </c>
       <c r="L500" s="6">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="M500" s="7">
-        <v>20798.64</v>
+        <v>18487.68</v>
       </c>
       <c r="N500" s="6">
         <v>1</v>
       </c>
       <c r="O500" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P500" s="8">
         <v>288.87</v>
@@ -69227,7 +69251,7 @@
         <v>46154</v>
       </c>
       <c r="X500" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y500" s="10">
         <v>0</v>
@@ -69298,7 +69322,7 @@
         <v>2</v>
       </c>
       <c r="C501" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D501" s="3" t="s">
         <v>45</v>
@@ -69310,7 +69334,7 @@
         <v>46154</v>
       </c>
       <c r="G501" s="5">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="H501" s="3" t="s">
         <v>47</v>
@@ -69325,16 +69349,16 @@
         <v>50</v>
       </c>
       <c r="L501" s="6">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="M501" s="7">
-        <v>21087.51</v>
+        <v>18776.55</v>
       </c>
       <c r="N501" s="6">
         <v>1</v>
       </c>
       <c r="O501" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P501" s="8">
         <v>288.87</v>
@@ -69361,7 +69385,7 @@
         <v>46154</v>
       </c>
       <c r="X501" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y501" s="10">
         <v>0</v>
@@ -69432,7 +69456,7 @@
         <v>2</v>
       </c>
       <c r="C502" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D502" s="3" t="s">
         <v>45</v>
@@ -69444,7 +69468,7 @@
         <v>46154</v>
       </c>
       <c r="G502" s="5">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="H502" s="3" t="s">
         <v>47</v>
@@ -69459,16 +69483,16 @@
         <v>50</v>
       </c>
       <c r="L502" s="6">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M502" s="7">
-        <v>21376.38</v>
+        <v>19065.419999999998</v>
       </c>
       <c r="N502" s="6">
         <v>1</v>
       </c>
       <c r="O502" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P502" s="8">
         <v>288.87</v>
@@ -69495,7 +69519,7 @@
         <v>46154</v>
       </c>
       <c r="X502" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y502" s="10">
         <v>0</v>
@@ -69566,7 +69590,7 @@
         <v>2</v>
       </c>
       <c r="C503" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D503" s="3" t="s">
         <v>45</v>
@@ -69578,7 +69602,7 @@
         <v>46154</v>
       </c>
       <c r="G503" s="5">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="H503" s="3" t="s">
         <v>47</v>
@@ -69593,16 +69617,16 @@
         <v>50</v>
       </c>
       <c r="L503" s="6">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="M503" s="7">
-        <v>21665.25</v>
+        <v>19354.29</v>
       </c>
       <c r="N503" s="6">
         <v>1</v>
       </c>
       <c r="O503" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P503" s="8">
         <v>288.87</v>
@@ -69629,7 +69653,7 @@
         <v>46154</v>
       </c>
       <c r="X503" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y503" s="10">
         <v>0</v>
@@ -69700,7 +69724,7 @@
         <v>2</v>
       </c>
       <c r="C504" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D504" s="3" t="s">
         <v>45</v>
@@ -69712,7 +69736,7 @@
         <v>46154</v>
       </c>
       <c r="G504" s="5">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="H504" s="3" t="s">
         <v>47</v>
@@ -69727,16 +69751,16 @@
         <v>50</v>
       </c>
       <c r="L504" s="6">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="M504" s="7">
-        <v>21954.12</v>
+        <v>19643.16</v>
       </c>
       <c r="N504" s="6">
         <v>1</v>
       </c>
       <c r="O504" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P504" s="8">
         <v>288.87</v>
@@ -69763,7 +69787,7 @@
         <v>46154</v>
       </c>
       <c r="X504" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y504" s="10">
         <v>0</v>
@@ -69834,7 +69858,7 @@
         <v>2</v>
       </c>
       <c r="C505" s="3" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D505" s="3" t="s">
         <v>45</v>
@@ -69846,7 +69870,7 @@
         <v>46154</v>
       </c>
       <c r="G505" s="5">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="H505" s="3" t="s">
         <v>47</v>
@@ -69861,16 +69885,16 @@
         <v>50</v>
       </c>
       <c r="L505" s="6">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="M505" s="7">
-        <v>22242.99</v>
+        <v>19932.03</v>
       </c>
       <c r="N505" s="6">
         <v>1</v>
       </c>
       <c r="O505" s="3" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="P505" s="8">
         <v>288.87</v>
@@ -69897,7 +69921,7 @@
         <v>46154</v>
       </c>
       <c r="X505" s="12">
-        <v>0.54861110000000002</v>
+        <v>0.46527780000000002</v>
       </c>
       <c r="Y505" s="10">
         <v>0</v>
@@ -69958,6 +69982,1078 @@
       </c>
       <c r="AR505" s="3" t="s">
         <v>563</v>
+      </c>
+    </row>
+    <row r="506" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A506" s="1">
+        <v>1</v>
+      </c>
+      <c r="B506" s="2">
+        <v>2</v>
+      </c>
+      <c r="C506" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D506" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E506" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F506" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G506" s="5">
+        <v>76</v>
+      </c>
+      <c r="H506" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I506" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J506" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K506" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L506" s="6">
+        <v>70</v>
+      </c>
+      <c r="M506" s="7">
+        <v>20220.900000000001</v>
+      </c>
+      <c r="N506" s="6">
+        <v>1</v>
+      </c>
+      <c r="O506" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P506" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q506" s="6">
+        <v>0</v>
+      </c>
+      <c r="R506" s="7">
+        <v>0</v>
+      </c>
+      <c r="S506" s="9">
+        <v>0</v>
+      </c>
+      <c r="T506" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U506" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V506" s="11">
+        <v>11</v>
+      </c>
+      <c r="W506" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X506" s="12">
+        <v>0.46527780000000002</v>
+      </c>
+      <c r="Y506" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z506" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA506" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB506" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC506" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD506" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE506" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF506" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG506" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH506" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI506" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ506" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK506" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL506" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM506" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN506" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO506" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP506" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ506" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR506" s="3" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="507" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A507" s="1">
+        <v>1</v>
+      </c>
+      <c r="B507" s="2">
+        <v>2</v>
+      </c>
+      <c r="C507" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D507" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E507" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F507" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G507" s="5">
+        <v>98</v>
+      </c>
+      <c r="H507" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I507" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J507" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K507" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L507" s="6">
+        <v>71</v>
+      </c>
+      <c r="M507" s="7">
+        <v>20509.77</v>
+      </c>
+      <c r="N507" s="6">
+        <v>1</v>
+      </c>
+      <c r="O507" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P507" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q507" s="6">
+        <v>0</v>
+      </c>
+      <c r="R507" s="7">
+        <v>0</v>
+      </c>
+      <c r="S507" s="9">
+        <v>0</v>
+      </c>
+      <c r="T507" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U507" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V507" s="11">
+        <v>11</v>
+      </c>
+      <c r="W507" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X507" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y507" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z507" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA507" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB507" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC507" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD507" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE507" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF507" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG507" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH507" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI507" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ507" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK507" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL507" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM507" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN507" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO507" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP507" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ507" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR507" s="3" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="508" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A508" s="1">
+        <v>1</v>
+      </c>
+      <c r="B508" s="2">
+        <v>2</v>
+      </c>
+      <c r="C508" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D508" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E508" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F508" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G508" s="5">
+        <v>99</v>
+      </c>
+      <c r="H508" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I508" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J508" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K508" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L508" s="6">
+        <v>72</v>
+      </c>
+      <c r="M508" s="7">
+        <v>20798.64</v>
+      </c>
+      <c r="N508" s="6">
+        <v>1</v>
+      </c>
+      <c r="O508" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P508" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q508" s="6">
+        <v>0</v>
+      </c>
+      <c r="R508" s="7">
+        <v>0</v>
+      </c>
+      <c r="S508" s="9">
+        <v>0</v>
+      </c>
+      <c r="T508" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U508" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V508" s="11">
+        <v>11</v>
+      </c>
+      <c r="W508" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X508" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y508" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z508" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA508" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB508" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC508" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD508" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE508" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF508" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG508" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH508" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI508" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ508" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK508" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL508" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM508" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN508" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO508" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP508" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ508" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR508" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="509" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A509" s="1">
+        <v>1</v>
+      </c>
+      <c r="B509" s="2">
+        <v>2</v>
+      </c>
+      <c r="C509" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D509" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E509" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F509" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G509" s="5">
+        <v>100</v>
+      </c>
+      <c r="H509" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I509" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J509" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K509" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L509" s="6">
+        <v>73</v>
+      </c>
+      <c r="M509" s="7">
+        <v>21087.51</v>
+      </c>
+      <c r="N509" s="6">
+        <v>1</v>
+      </c>
+      <c r="O509" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P509" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q509" s="6">
+        <v>0</v>
+      </c>
+      <c r="R509" s="7">
+        <v>0</v>
+      </c>
+      <c r="S509" s="9">
+        <v>0</v>
+      </c>
+      <c r="T509" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U509" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V509" s="11">
+        <v>11</v>
+      </c>
+      <c r="W509" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X509" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y509" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z509" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA509" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB509" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC509" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD509" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE509" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF509" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG509" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH509" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI509" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ509" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK509" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL509" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM509" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN509" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO509" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP509" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ509" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR509" s="3" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="510" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A510" s="1">
+        <v>1</v>
+      </c>
+      <c r="B510" s="2">
+        <v>2</v>
+      </c>
+      <c r="C510" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D510" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E510" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F510" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G510" s="5">
+        <v>101</v>
+      </c>
+      <c r="H510" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I510" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J510" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K510" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L510" s="6">
+        <v>74</v>
+      </c>
+      <c r="M510" s="7">
+        <v>21376.38</v>
+      </c>
+      <c r="N510" s="6">
+        <v>1</v>
+      </c>
+      <c r="O510" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P510" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q510" s="6">
+        <v>0</v>
+      </c>
+      <c r="R510" s="7">
+        <v>0</v>
+      </c>
+      <c r="S510" s="9">
+        <v>0</v>
+      </c>
+      <c r="T510" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U510" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V510" s="11">
+        <v>11</v>
+      </c>
+      <c r="W510" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X510" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y510" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z510" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA510" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB510" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC510" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD510" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE510" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF510" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG510" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH510" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI510" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ510" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK510" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL510" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM510" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN510" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO510" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP510" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ510" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR510" s="3" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="511" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A511" s="1">
+        <v>1</v>
+      </c>
+      <c r="B511" s="2">
+        <v>2</v>
+      </c>
+      <c r="C511" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D511" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E511" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F511" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G511" s="5">
+        <v>102</v>
+      </c>
+      <c r="H511" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I511" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J511" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K511" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L511" s="6">
+        <v>75</v>
+      </c>
+      <c r="M511" s="7">
+        <v>21665.25</v>
+      </c>
+      <c r="N511" s="6">
+        <v>1</v>
+      </c>
+      <c r="O511" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P511" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q511" s="6">
+        <v>0</v>
+      </c>
+      <c r="R511" s="7">
+        <v>0</v>
+      </c>
+      <c r="S511" s="9">
+        <v>0</v>
+      </c>
+      <c r="T511" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U511" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V511" s="11">
+        <v>11</v>
+      </c>
+      <c r="W511" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X511" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y511" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z511" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA511" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB511" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC511" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD511" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE511" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF511" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG511" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH511" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI511" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ511" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK511" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL511" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM511" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN511" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO511" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP511" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ511" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR511" s="3" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="512" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A512" s="1">
+        <v>1</v>
+      </c>
+      <c r="B512" s="2">
+        <v>2</v>
+      </c>
+      <c r="C512" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D512" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E512" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F512" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G512" s="5">
+        <v>103</v>
+      </c>
+      <c r="H512" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I512" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J512" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K512" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L512" s="6">
+        <v>76</v>
+      </c>
+      <c r="M512" s="7">
+        <v>21954.12</v>
+      </c>
+      <c r="N512" s="6">
+        <v>1</v>
+      </c>
+      <c r="O512" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P512" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q512" s="6">
+        <v>0</v>
+      </c>
+      <c r="R512" s="7">
+        <v>0</v>
+      </c>
+      <c r="S512" s="9">
+        <v>0</v>
+      </c>
+      <c r="T512" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U512" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V512" s="11">
+        <v>11</v>
+      </c>
+      <c r="W512" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X512" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y512" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z512" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA512" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB512" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC512" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD512" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE512" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF512" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG512" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH512" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI512" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ512" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK512" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL512" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM512" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN512" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO512" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP512" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ512" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR512" s="3" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="513" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A513" s="1">
+        <v>1</v>
+      </c>
+      <c r="B513" s="2">
+        <v>2</v>
+      </c>
+      <c r="C513" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D513" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E513" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F513" s="4">
+        <v>46154</v>
+      </c>
+      <c r="G513" s="5">
+        <v>104</v>
+      </c>
+      <c r="H513" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I513" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J513" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K513" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L513" s="6">
+        <v>77</v>
+      </c>
+      <c r="M513" s="7">
+        <v>22242.99</v>
+      </c>
+      <c r="N513" s="6">
+        <v>1</v>
+      </c>
+      <c r="O513" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="P513" s="8">
+        <v>288.87</v>
+      </c>
+      <c r="Q513" s="6">
+        <v>0</v>
+      </c>
+      <c r="R513" s="7">
+        <v>0</v>
+      </c>
+      <c r="S513" s="9">
+        <v>0</v>
+      </c>
+      <c r="T513" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U513" s="10">
+        <v>64285</v>
+      </c>
+      <c r="V513" s="11">
+        <v>11</v>
+      </c>
+      <c r="W513" s="4">
+        <v>46154</v>
+      </c>
+      <c r="X513" s="12">
+        <v>0.54861110000000002</v>
+      </c>
+      <c r="Y513" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z513" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA513" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB513" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC513" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD513" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE513" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF513" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG513" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH513" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI513" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ513" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK513" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL513" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM513" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN513" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO513" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP513" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ513" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR513" s="3" t="s">
+        <v>571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 13/05/2026  9:00:04,12
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{278B1858-7896-43F4-BDAD-8C8E621174C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D041A8AF-2944-435C-B37F-8476DAF63921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="132">
   <si>
     <t>Sel</t>
   </si>
@@ -335,6 +335,87 @@
   </si>
   <si>
     <t>1858700137666</t>
+  </si>
+  <si>
+    <t>1858700137667</t>
+  </si>
+  <si>
+    <t>1858700137668</t>
+  </si>
+  <si>
+    <t>1858700137669</t>
+  </si>
+  <si>
+    <t>1858700137670</t>
+  </si>
+  <si>
+    <t>1858700137671</t>
+  </si>
+  <si>
+    <t>1858700137672</t>
+  </si>
+  <si>
+    <t>1858700137673</t>
+  </si>
+  <si>
+    <t>1858700137674</t>
+  </si>
+  <si>
+    <t>1858700137675</t>
+  </si>
+  <si>
+    <t>1858700137676</t>
+  </si>
+  <si>
+    <t>1858700137677</t>
+  </si>
+  <si>
+    <t>1858700137678</t>
+  </si>
+  <si>
+    <t>1858700137679</t>
+  </si>
+  <si>
+    <t>1858700137680</t>
+  </si>
+  <si>
+    <t>1858700137681</t>
+  </si>
+  <si>
+    <t>1858700137682</t>
+  </si>
+  <si>
+    <t>1858700137683</t>
+  </si>
+  <si>
+    <t>1858700137684</t>
+  </si>
+  <si>
+    <t>1858700137685</t>
+  </si>
+  <si>
+    <t>1858700137686</t>
+  </si>
+  <si>
+    <t>1858700137687</t>
+  </si>
+  <si>
+    <t>1858700137688</t>
+  </si>
+  <si>
+    <t>1858700137689</t>
+  </si>
+  <si>
+    <t>1858700137690</t>
+  </si>
+  <si>
+    <t>1858700137691</t>
+  </si>
+  <si>
+    <t>1858700137692</t>
+  </si>
+  <si>
+    <t>1858700137693</t>
   </si>
 </sst>
 </file>
@@ -910,7 +991,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR51"/>
+  <dimension ref="A1:AR78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -7745,6 +7826,3624 @@
       </c>
       <c r="AR51" s="3" t="s">
         <v>104</v>
+      </c>
+    </row>
+    <row r="52" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>1</v>
+      </c>
+      <c r="B52" s="2">
+        <v>2</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F52" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G52" s="5">
+        <v>54</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L52" s="6">
+        <v>1693</v>
+      </c>
+      <c r="M52" s="7">
+        <v>319691.81</v>
+      </c>
+      <c r="N52" s="6">
+        <v>1</v>
+      </c>
+      <c r="O52" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P52" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q52" s="6">
+        <v>0</v>
+      </c>
+      <c r="R52" s="7">
+        <v>0</v>
+      </c>
+      <c r="S52" s="9">
+        <v>0</v>
+      </c>
+      <c r="T52" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U52" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V52" s="11">
+        <v>11</v>
+      </c>
+      <c r="W52" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X52" s="12">
+        <v>0.3618056</v>
+      </c>
+      <c r="Y52" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB52" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG52" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI52" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ52" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK52" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM52" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR52" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="53" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>1</v>
+      </c>
+      <c r="B53" s="2">
+        <v>2</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F53" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G53" s="5">
+        <v>55</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L53" s="6">
+        <v>1694</v>
+      </c>
+      <c r="M53" s="7">
+        <v>319880.64</v>
+      </c>
+      <c r="N53" s="6">
+        <v>1</v>
+      </c>
+      <c r="O53" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P53" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q53" s="6">
+        <v>0</v>
+      </c>
+      <c r="R53" s="7">
+        <v>0</v>
+      </c>
+      <c r="S53" s="9">
+        <v>0</v>
+      </c>
+      <c r="T53" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U53" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V53" s="11">
+        <v>11</v>
+      </c>
+      <c r="W53" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X53" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y53" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB53" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG53" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI53" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ53" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK53" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM53" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR53" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="54" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>1</v>
+      </c>
+      <c r="B54" s="2">
+        <v>2</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G54" s="5">
+        <v>56</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J54" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K54" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L54" s="6">
+        <v>1695</v>
+      </c>
+      <c r="M54" s="7">
+        <v>320069.46999999997</v>
+      </c>
+      <c r="N54" s="6">
+        <v>1</v>
+      </c>
+      <c r="O54" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P54" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q54" s="6">
+        <v>0</v>
+      </c>
+      <c r="R54" s="7">
+        <v>0</v>
+      </c>
+      <c r="S54" s="9">
+        <v>0</v>
+      </c>
+      <c r="T54" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U54" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V54" s="11">
+        <v>11</v>
+      </c>
+      <c r="W54" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X54" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y54" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB54" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG54" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI54" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ54" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK54" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM54" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR54" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="55" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>1</v>
+      </c>
+      <c r="B55" s="2">
+        <v>2</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F55" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G55" s="5">
+        <v>57</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J55" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L55" s="6">
+        <v>1696</v>
+      </c>
+      <c r="M55" s="7">
+        <v>320258.3</v>
+      </c>
+      <c r="N55" s="6">
+        <v>1</v>
+      </c>
+      <c r="O55" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P55" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q55" s="6">
+        <v>0</v>
+      </c>
+      <c r="R55" s="7">
+        <v>0</v>
+      </c>
+      <c r="S55" s="9">
+        <v>0</v>
+      </c>
+      <c r="T55" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U55" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V55" s="11">
+        <v>11</v>
+      </c>
+      <c r="W55" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X55" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y55" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB55" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG55" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI55" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ55" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK55" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM55" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR55" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="56" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A56" s="1">
+        <v>1</v>
+      </c>
+      <c r="B56" s="2">
+        <v>2</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F56" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G56" s="5">
+        <v>58</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L56" s="6">
+        <v>1697</v>
+      </c>
+      <c r="M56" s="7">
+        <v>320447.14</v>
+      </c>
+      <c r="N56" s="6">
+        <v>1</v>
+      </c>
+      <c r="O56" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P56" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q56" s="6">
+        <v>0</v>
+      </c>
+      <c r="R56" s="7">
+        <v>0</v>
+      </c>
+      <c r="S56" s="9">
+        <v>0</v>
+      </c>
+      <c r="T56" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U56" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V56" s="11">
+        <v>11</v>
+      </c>
+      <c r="W56" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X56" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y56" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB56" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG56" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI56" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ56" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK56" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM56" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR56" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="57" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A57" s="1">
+        <v>1</v>
+      </c>
+      <c r="B57" s="2">
+        <v>2</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F57" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G57" s="5">
+        <v>59</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L57" s="6">
+        <v>1698</v>
+      </c>
+      <c r="M57" s="7">
+        <v>320635.96999999997</v>
+      </c>
+      <c r="N57" s="6">
+        <v>1</v>
+      </c>
+      <c r="O57" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P57" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q57" s="6">
+        <v>0</v>
+      </c>
+      <c r="R57" s="7">
+        <v>0</v>
+      </c>
+      <c r="S57" s="9">
+        <v>0</v>
+      </c>
+      <c r="T57" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U57" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V57" s="11">
+        <v>11</v>
+      </c>
+      <c r="W57" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X57" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y57" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB57" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG57" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI57" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ57" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK57" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM57" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR57" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="58" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A58" s="1">
+        <v>1</v>
+      </c>
+      <c r="B58" s="2">
+        <v>2</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F58" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G58" s="5">
+        <v>60</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J58" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L58" s="6">
+        <v>1699</v>
+      </c>
+      <c r="M58" s="7">
+        <v>320824.8</v>
+      </c>
+      <c r="N58" s="6">
+        <v>1</v>
+      </c>
+      <c r="O58" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P58" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q58" s="6">
+        <v>0</v>
+      </c>
+      <c r="R58" s="7">
+        <v>0</v>
+      </c>
+      <c r="S58" s="9">
+        <v>0</v>
+      </c>
+      <c r="T58" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U58" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V58" s="11">
+        <v>11</v>
+      </c>
+      <c r="W58" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X58" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y58" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB58" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG58" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI58" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ58" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK58" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM58" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR58" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="59" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>1</v>
+      </c>
+      <c r="B59" s="2">
+        <v>2</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F59" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G59" s="5">
+        <v>61</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J59" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K59" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L59" s="6">
+        <v>1700</v>
+      </c>
+      <c r="M59" s="7">
+        <v>321013.63</v>
+      </c>
+      <c r="N59" s="6">
+        <v>1</v>
+      </c>
+      <c r="O59" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P59" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q59" s="6">
+        <v>0</v>
+      </c>
+      <c r="R59" s="7">
+        <v>0</v>
+      </c>
+      <c r="S59" s="9">
+        <v>0</v>
+      </c>
+      <c r="T59" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U59" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V59" s="11">
+        <v>11</v>
+      </c>
+      <c r="W59" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X59" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y59" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB59" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG59" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI59" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ59" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK59" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM59" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR59" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="60" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
+        <v>1</v>
+      </c>
+      <c r="B60" s="2">
+        <v>2</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F60" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G60" s="5">
+        <v>62</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I60" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J60" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K60" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L60" s="6">
+        <v>1701</v>
+      </c>
+      <c r="M60" s="7">
+        <v>321202.46000000002</v>
+      </c>
+      <c r="N60" s="6">
+        <v>1</v>
+      </c>
+      <c r="O60" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P60" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q60" s="6">
+        <v>0</v>
+      </c>
+      <c r="R60" s="7">
+        <v>0</v>
+      </c>
+      <c r="S60" s="9">
+        <v>0</v>
+      </c>
+      <c r="T60" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U60" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V60" s="11">
+        <v>11</v>
+      </c>
+      <c r="W60" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X60" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y60" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB60" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG60" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI60" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ60" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK60" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM60" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR60" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="61" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>1</v>
+      </c>
+      <c r="B61" s="2">
+        <v>2</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F61" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G61" s="5">
+        <v>63</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J61" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K61" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L61" s="6">
+        <v>1702</v>
+      </c>
+      <c r="M61" s="7">
+        <v>321391.28999999998</v>
+      </c>
+      <c r="N61" s="6">
+        <v>1</v>
+      </c>
+      <c r="O61" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P61" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q61" s="6">
+        <v>0</v>
+      </c>
+      <c r="R61" s="7">
+        <v>0</v>
+      </c>
+      <c r="S61" s="9">
+        <v>0</v>
+      </c>
+      <c r="T61" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U61" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V61" s="11">
+        <v>11</v>
+      </c>
+      <c r="W61" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X61" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y61" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB61" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG61" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI61" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ61" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK61" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM61" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR61" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="62" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>1</v>
+      </c>
+      <c r="B62" s="2">
+        <v>2</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F62" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G62" s="5">
+        <v>64</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L62" s="6">
+        <v>1703</v>
+      </c>
+      <c r="M62" s="7">
+        <v>321580.13</v>
+      </c>
+      <c r="N62" s="6">
+        <v>1</v>
+      </c>
+      <c r="O62" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P62" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q62" s="6">
+        <v>0</v>
+      </c>
+      <c r="R62" s="7">
+        <v>0</v>
+      </c>
+      <c r="S62" s="9">
+        <v>0</v>
+      </c>
+      <c r="T62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U62" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V62" s="11">
+        <v>11</v>
+      </c>
+      <c r="W62" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X62" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y62" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB62" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG62" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI62" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK62" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM62" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR62" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>1</v>
+      </c>
+      <c r="B63" s="2">
+        <v>2</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F63" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G63" s="5">
+        <v>65</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K63" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L63" s="6">
+        <v>1704</v>
+      </c>
+      <c r="M63" s="7">
+        <v>321768.96000000002</v>
+      </c>
+      <c r="N63" s="6">
+        <v>1</v>
+      </c>
+      <c r="O63" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P63" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q63" s="6">
+        <v>0</v>
+      </c>
+      <c r="R63" s="7">
+        <v>0</v>
+      </c>
+      <c r="S63" s="9">
+        <v>0</v>
+      </c>
+      <c r="T63" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U63" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V63" s="11">
+        <v>11</v>
+      </c>
+      <c r="W63" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X63" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y63" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB63" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG63" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI63" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ63" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK63" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM63" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR63" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="64" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>1</v>
+      </c>
+      <c r="B64" s="2">
+        <v>2</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F64" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G64" s="5">
+        <v>66</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K64" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L64" s="6">
+        <v>1705</v>
+      </c>
+      <c r="M64" s="7">
+        <v>321957.78999999998</v>
+      </c>
+      <c r="N64" s="6">
+        <v>1</v>
+      </c>
+      <c r="O64" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P64" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q64" s="6">
+        <v>0</v>
+      </c>
+      <c r="R64" s="7">
+        <v>0</v>
+      </c>
+      <c r="S64" s="9">
+        <v>0</v>
+      </c>
+      <c r="T64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U64" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V64" s="11">
+        <v>11</v>
+      </c>
+      <c r="W64" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X64" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y64" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB64" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG64" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI64" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK64" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM64" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR64" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="65" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>1</v>
+      </c>
+      <c r="B65" s="2">
+        <v>2</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F65" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G65" s="5">
+        <v>67</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K65" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L65" s="6">
+        <v>1706</v>
+      </c>
+      <c r="M65" s="7">
+        <v>322146.62</v>
+      </c>
+      <c r="N65" s="6">
+        <v>1</v>
+      </c>
+      <c r="O65" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P65" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q65" s="6">
+        <v>0</v>
+      </c>
+      <c r="R65" s="7">
+        <v>0</v>
+      </c>
+      <c r="S65" s="9">
+        <v>0</v>
+      </c>
+      <c r="T65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U65" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V65" s="11">
+        <v>11</v>
+      </c>
+      <c r="W65" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X65" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y65" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG65" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI65" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR65" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>1</v>
+      </c>
+      <c r="B66" s="2">
+        <v>2</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F66" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G66" s="5">
+        <v>68</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K66" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L66" s="6">
+        <v>1707</v>
+      </c>
+      <c r="M66" s="7">
+        <v>322335.45</v>
+      </c>
+      <c r="N66" s="6">
+        <v>1</v>
+      </c>
+      <c r="O66" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P66" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q66" s="6">
+        <v>0</v>
+      </c>
+      <c r="R66" s="7">
+        <v>0</v>
+      </c>
+      <c r="S66" s="9">
+        <v>0</v>
+      </c>
+      <c r="T66" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U66" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V66" s="11">
+        <v>11</v>
+      </c>
+      <c r="W66" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X66" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y66" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB66" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG66" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI66" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ66" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK66" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM66" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR66" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="67" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>1</v>
+      </c>
+      <c r="B67" s="2">
+        <v>2</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F67" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G67" s="5">
+        <v>69</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L67" s="6">
+        <v>1708</v>
+      </c>
+      <c r="M67" s="7">
+        <v>322524.28000000003</v>
+      </c>
+      <c r="N67" s="6">
+        <v>1</v>
+      </c>
+      <c r="O67" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P67" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q67" s="6">
+        <v>0</v>
+      </c>
+      <c r="R67" s="7">
+        <v>0</v>
+      </c>
+      <c r="S67" s="9">
+        <v>0</v>
+      </c>
+      <c r="T67" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U67" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V67" s="11">
+        <v>11</v>
+      </c>
+      <c r="W67" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X67" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y67" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB67" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG67" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI67" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ67" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK67" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM67" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR67" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="68" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
+        <v>1</v>
+      </c>
+      <c r="B68" s="2">
+        <v>2</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F68" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G68" s="5">
+        <v>70</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J68" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K68" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L68" s="6">
+        <v>1709</v>
+      </c>
+      <c r="M68" s="7">
+        <v>322713.11</v>
+      </c>
+      <c r="N68" s="6">
+        <v>1</v>
+      </c>
+      <c r="O68" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P68" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q68" s="6">
+        <v>0</v>
+      </c>
+      <c r="R68" s="7">
+        <v>0</v>
+      </c>
+      <c r="S68" s="9">
+        <v>0</v>
+      </c>
+      <c r="T68" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U68" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V68" s="11">
+        <v>11</v>
+      </c>
+      <c r="W68" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X68" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y68" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB68" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG68" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI68" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ68" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK68" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM68" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR68" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="69" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
+        <v>1</v>
+      </c>
+      <c r="B69" s="2">
+        <v>2</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F69" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G69" s="5">
+        <v>71</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J69" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L69" s="6">
+        <v>1710</v>
+      </c>
+      <c r="M69" s="7">
+        <v>322901.95</v>
+      </c>
+      <c r="N69" s="6">
+        <v>1</v>
+      </c>
+      <c r="O69" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P69" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q69" s="6">
+        <v>0</v>
+      </c>
+      <c r="R69" s="7">
+        <v>0</v>
+      </c>
+      <c r="S69" s="9">
+        <v>0</v>
+      </c>
+      <c r="T69" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U69" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V69" s="11">
+        <v>11</v>
+      </c>
+      <c r="W69" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X69" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y69" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB69" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG69" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI69" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ69" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK69" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM69" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR69" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
+        <v>1</v>
+      </c>
+      <c r="B70" s="2">
+        <v>2</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F70" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G70" s="5">
+        <v>72</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L70" s="6">
+        <v>1711</v>
+      </c>
+      <c r="M70" s="7">
+        <v>323090.78000000003</v>
+      </c>
+      <c r="N70" s="6">
+        <v>1</v>
+      </c>
+      <c r="O70" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P70" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q70" s="6">
+        <v>0</v>
+      </c>
+      <c r="R70" s="7">
+        <v>0</v>
+      </c>
+      <c r="S70" s="9">
+        <v>0</v>
+      </c>
+      <c r="T70" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U70" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V70" s="11">
+        <v>11</v>
+      </c>
+      <c r="W70" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X70" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y70" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB70" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG70" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI70" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ70" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK70" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM70" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR70" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
+        <v>1</v>
+      </c>
+      <c r="B71" s="2">
+        <v>2</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F71" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G71" s="5">
+        <v>73</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L71" s="6">
+        <v>1712</v>
+      </c>
+      <c r="M71" s="7">
+        <v>323279.61</v>
+      </c>
+      <c r="N71" s="6">
+        <v>1</v>
+      </c>
+      <c r="O71" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P71" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q71" s="6">
+        <v>0</v>
+      </c>
+      <c r="R71" s="7">
+        <v>0</v>
+      </c>
+      <c r="S71" s="9">
+        <v>0</v>
+      </c>
+      <c r="T71" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U71" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V71" s="11">
+        <v>11</v>
+      </c>
+      <c r="W71" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X71" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y71" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB71" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG71" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI71" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ71" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK71" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM71" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR71" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="72" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
+        <v>1</v>
+      </c>
+      <c r="B72" s="2">
+        <v>2</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F72" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G72" s="5">
+        <v>74</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L72" s="6">
+        <v>1713</v>
+      </c>
+      <c r="M72" s="7">
+        <v>323468.44</v>
+      </c>
+      <c r="N72" s="6">
+        <v>1</v>
+      </c>
+      <c r="O72" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P72" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q72" s="6">
+        <v>0</v>
+      </c>
+      <c r="R72" s="7">
+        <v>0</v>
+      </c>
+      <c r="S72" s="9">
+        <v>0</v>
+      </c>
+      <c r="T72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U72" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V72" s="11">
+        <v>11</v>
+      </c>
+      <c r="W72" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X72" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y72" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB72" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG72" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI72" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK72" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM72" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR72" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
+        <v>1</v>
+      </c>
+      <c r="B73" s="2">
+        <v>2</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F73" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G73" s="5">
+        <v>75</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K73" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L73" s="6">
+        <v>1714</v>
+      </c>
+      <c r="M73" s="7">
+        <v>323657.27</v>
+      </c>
+      <c r="N73" s="6">
+        <v>1</v>
+      </c>
+      <c r="O73" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P73" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q73" s="6">
+        <v>0</v>
+      </c>
+      <c r="R73" s="7">
+        <v>0</v>
+      </c>
+      <c r="S73" s="9">
+        <v>0</v>
+      </c>
+      <c r="T73" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U73" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V73" s="11">
+        <v>11</v>
+      </c>
+      <c r="W73" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X73" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y73" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB73" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG73" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI73" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ73" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK73" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM73" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR73" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
+        <v>1</v>
+      </c>
+      <c r="B74" s="2">
+        <v>2</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F74" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G74" s="5">
+        <v>76</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K74" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L74" s="6">
+        <v>1715</v>
+      </c>
+      <c r="M74" s="7">
+        <v>323846.09999999998</v>
+      </c>
+      <c r="N74" s="6">
+        <v>1</v>
+      </c>
+      <c r="O74" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P74" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q74" s="6">
+        <v>0</v>
+      </c>
+      <c r="R74" s="7">
+        <v>0</v>
+      </c>
+      <c r="S74" s="9">
+        <v>0</v>
+      </c>
+      <c r="T74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U74" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V74" s="11">
+        <v>11</v>
+      </c>
+      <c r="W74" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X74" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y74" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB74" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG74" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI74" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK74" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM74" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR74" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="75" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
+        <v>1</v>
+      </c>
+      <c r="B75" s="2">
+        <v>2</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F75" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G75" s="5">
+        <v>77</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K75" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L75" s="6">
+        <v>1716</v>
+      </c>
+      <c r="M75" s="7">
+        <v>324034.94</v>
+      </c>
+      <c r="N75" s="6">
+        <v>1</v>
+      </c>
+      <c r="O75" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P75" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q75" s="6">
+        <v>0</v>
+      </c>
+      <c r="R75" s="7">
+        <v>0</v>
+      </c>
+      <c r="S75" s="9">
+        <v>0</v>
+      </c>
+      <c r="T75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U75" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V75" s="11">
+        <v>11</v>
+      </c>
+      <c r="W75" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X75" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y75" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB75" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG75" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI75" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK75" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM75" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR75" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="76" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
+        <v>1</v>
+      </c>
+      <c r="B76" s="2">
+        <v>2</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F76" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G76" s="5">
+        <v>78</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L76" s="6">
+        <v>1717</v>
+      </c>
+      <c r="M76" s="7">
+        <v>324223.77</v>
+      </c>
+      <c r="N76" s="6">
+        <v>1</v>
+      </c>
+      <c r="O76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P76" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q76" s="6">
+        <v>0</v>
+      </c>
+      <c r="R76" s="7">
+        <v>0</v>
+      </c>
+      <c r="S76" s="9">
+        <v>0</v>
+      </c>
+      <c r="T76" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U76" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V76" s="11">
+        <v>11</v>
+      </c>
+      <c r="W76" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X76" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y76" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB76" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG76" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI76" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ76" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK76" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM76" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR76" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="77" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
+        <v>1</v>
+      </c>
+      <c r="B77" s="2">
+        <v>2</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F77" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G77" s="5">
+        <v>79</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K77" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L77" s="6">
+        <v>1718</v>
+      </c>
+      <c r="M77" s="7">
+        <v>324412.59999999998</v>
+      </c>
+      <c r="N77" s="6">
+        <v>1</v>
+      </c>
+      <c r="O77" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P77" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q77" s="6">
+        <v>0</v>
+      </c>
+      <c r="R77" s="7">
+        <v>0</v>
+      </c>
+      <c r="S77" s="9">
+        <v>0</v>
+      </c>
+      <c r="T77" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U77" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V77" s="11">
+        <v>11</v>
+      </c>
+      <c r="W77" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X77" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y77" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB77" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG77" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI77" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ77" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK77" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM77" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR77" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
+        <v>1</v>
+      </c>
+      <c r="B78" s="2">
+        <v>2</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F78" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G78" s="5">
+        <v>80</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L78" s="6">
+        <v>1719</v>
+      </c>
+      <c r="M78" s="7">
+        <v>324601.43</v>
+      </c>
+      <c r="N78" s="6">
+        <v>1</v>
+      </c>
+      <c r="O78" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P78" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q78" s="6">
+        <v>0</v>
+      </c>
+      <c r="R78" s="7">
+        <v>0</v>
+      </c>
+      <c r="S78" s="9">
+        <v>0</v>
+      </c>
+      <c r="T78" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U78" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V78" s="11">
+        <v>11</v>
+      </c>
+      <c r="W78" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X78" s="12">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="Y78" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB78" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG78" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI78" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ78" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK78" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM78" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR78" s="3" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 13/05/2026  9:21:12,91
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D041A8AF-2944-435C-B37F-8476DAF63921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD32733D-8E9E-4A47-BCAA-A236BAE39486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1790" uniqueCount="152">
   <si>
     <t>Sel</t>
   </si>
@@ -416,6 +416,66 @@
   </si>
   <si>
     <t>1858700137693</t>
+  </si>
+  <si>
+    <t>1858700137694</t>
+  </si>
+  <si>
+    <t>1858700137695</t>
+  </si>
+  <si>
+    <t>1858700137696</t>
+  </si>
+  <si>
+    <t>1858700137697</t>
+  </si>
+  <si>
+    <t>1858700137698</t>
+  </si>
+  <si>
+    <t>1858700137699</t>
+  </si>
+  <si>
+    <t>1858700137700</t>
+  </si>
+  <si>
+    <t>1858700137701</t>
+  </si>
+  <si>
+    <t>1858700137702</t>
+  </si>
+  <si>
+    <t>1858700137703</t>
+  </si>
+  <si>
+    <t>1858700137704</t>
+  </si>
+  <si>
+    <t>1858700137705</t>
+  </si>
+  <si>
+    <t>1858700137706</t>
+  </si>
+  <si>
+    <t>1858700137707</t>
+  </si>
+  <si>
+    <t>1858700137708</t>
+  </si>
+  <si>
+    <t>1858700137709</t>
+  </si>
+  <si>
+    <t>1858700137710</t>
+  </si>
+  <si>
+    <t>1858700137711</t>
+  </si>
+  <si>
+    <t>1858700137712</t>
+  </si>
+  <si>
+    <t>1858700137713</t>
   </si>
 </sst>
 </file>
@@ -991,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR78"/>
+  <dimension ref="A1:AR98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -11444,6 +11504,2686 @@
       </c>
       <c r="AR78" s="3" t="s">
         <v>131</v>
+      </c>
+    </row>
+    <row r="79" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
+        <v>1</v>
+      </c>
+      <c r="B79" s="2">
+        <v>2</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F79" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G79" s="5">
+        <v>81</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L79" s="6">
+        <v>1720</v>
+      </c>
+      <c r="M79" s="7">
+        <v>324790.26</v>
+      </c>
+      <c r="N79" s="6">
+        <v>1</v>
+      </c>
+      <c r="O79" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P79" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q79" s="6">
+        <v>0</v>
+      </c>
+      <c r="R79" s="7">
+        <v>0</v>
+      </c>
+      <c r="S79" s="9">
+        <v>0</v>
+      </c>
+      <c r="T79" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U79" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V79" s="11">
+        <v>11</v>
+      </c>
+      <c r="W79" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X79" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y79" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB79" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG79" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI79" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ79" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK79" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM79" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR79" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="80" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
+        <v>1</v>
+      </c>
+      <c r="B80" s="2">
+        <v>2</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F80" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G80" s="5">
+        <v>82</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I80" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J80" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K80" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L80" s="6">
+        <v>1721</v>
+      </c>
+      <c r="M80" s="7">
+        <v>324979.09000000003</v>
+      </c>
+      <c r="N80" s="6">
+        <v>1</v>
+      </c>
+      <c r="O80" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P80" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q80" s="6">
+        <v>0</v>
+      </c>
+      <c r="R80" s="7">
+        <v>0</v>
+      </c>
+      <c r="S80" s="9">
+        <v>0</v>
+      </c>
+      <c r="T80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U80" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V80" s="11">
+        <v>11</v>
+      </c>
+      <c r="W80" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X80" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y80" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB80" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG80" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI80" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK80" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM80" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR80" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
+        <v>1</v>
+      </c>
+      <c r="B81" s="2">
+        <v>2</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F81" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G81" s="5">
+        <v>83</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I81" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K81" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L81" s="6">
+        <v>1722</v>
+      </c>
+      <c r="M81" s="7">
+        <v>325167.92</v>
+      </c>
+      <c r="N81" s="6">
+        <v>1</v>
+      </c>
+      <c r="O81" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P81" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q81" s="6">
+        <v>0</v>
+      </c>
+      <c r="R81" s="7">
+        <v>0</v>
+      </c>
+      <c r="S81" s="9">
+        <v>0</v>
+      </c>
+      <c r="T81" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U81" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V81" s="11">
+        <v>11</v>
+      </c>
+      <c r="W81" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X81" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y81" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB81" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG81" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI81" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ81" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK81" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM81" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR81" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="82" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
+        <v>1</v>
+      </c>
+      <c r="B82" s="2">
+        <v>2</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F82" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G82" s="5">
+        <v>84</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L82" s="6">
+        <v>1723</v>
+      </c>
+      <c r="M82" s="7">
+        <v>325356.76</v>
+      </c>
+      <c r="N82" s="6">
+        <v>1</v>
+      </c>
+      <c r="O82" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P82" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q82" s="6">
+        <v>0</v>
+      </c>
+      <c r="R82" s="7">
+        <v>0</v>
+      </c>
+      <c r="S82" s="9">
+        <v>0</v>
+      </c>
+      <c r="T82" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U82" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V82" s="11">
+        <v>11</v>
+      </c>
+      <c r="W82" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X82" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y82" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB82" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG82" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI82" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ82" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK82" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL82" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM82" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR82" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="83" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
+        <v>1</v>
+      </c>
+      <c r="B83" s="2">
+        <v>2</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F83" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G83" s="5">
+        <v>85</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I83" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J83" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K83" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L83" s="6">
+        <v>1724</v>
+      </c>
+      <c r="M83" s="7">
+        <v>325545.59000000003</v>
+      </c>
+      <c r="N83" s="6">
+        <v>1</v>
+      </c>
+      <c r="O83" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P83" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q83" s="6">
+        <v>0</v>
+      </c>
+      <c r="R83" s="7">
+        <v>0</v>
+      </c>
+      <c r="S83" s="9">
+        <v>0</v>
+      </c>
+      <c r="T83" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U83" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V83" s="11">
+        <v>11</v>
+      </c>
+      <c r="W83" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X83" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y83" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB83" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG83" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI83" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ83" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK83" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL83" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM83" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ83" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR83" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="84" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
+        <v>1</v>
+      </c>
+      <c r="B84" s="2">
+        <v>2</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F84" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G84" s="5">
+        <v>86</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I84" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L84" s="6">
+        <v>1725</v>
+      </c>
+      <c r="M84" s="7">
+        <v>325734.42</v>
+      </c>
+      <c r="N84" s="6">
+        <v>1</v>
+      </c>
+      <c r="O84" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P84" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q84" s="6">
+        <v>0</v>
+      </c>
+      <c r="R84" s="7">
+        <v>0</v>
+      </c>
+      <c r="S84" s="9">
+        <v>0</v>
+      </c>
+      <c r="T84" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U84" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V84" s="11">
+        <v>11</v>
+      </c>
+      <c r="W84" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X84" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y84" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB84" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG84" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI84" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ84" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK84" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL84" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM84" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR84" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="85" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
+        <v>1</v>
+      </c>
+      <c r="B85" s="2">
+        <v>2</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F85" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G85" s="5">
+        <v>87</v>
+      </c>
+      <c r="H85" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J85" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K85" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L85" s="6">
+        <v>1726</v>
+      </c>
+      <c r="M85" s="7">
+        <v>325923.25</v>
+      </c>
+      <c r="N85" s="6">
+        <v>1</v>
+      </c>
+      <c r="O85" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P85" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q85" s="6">
+        <v>0</v>
+      </c>
+      <c r="R85" s="7">
+        <v>0</v>
+      </c>
+      <c r="S85" s="9">
+        <v>0</v>
+      </c>
+      <c r="T85" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U85" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V85" s="11">
+        <v>11</v>
+      </c>
+      <c r="W85" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X85" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y85" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB85" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG85" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI85" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ85" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK85" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL85" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM85" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR85" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="86" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
+        <v>1</v>
+      </c>
+      <c r="B86" s="2">
+        <v>2</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F86" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G86" s="5">
+        <v>88</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J86" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K86" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L86" s="6">
+        <v>1727</v>
+      </c>
+      <c r="M86" s="7">
+        <v>326112.08</v>
+      </c>
+      <c r="N86" s="6">
+        <v>1</v>
+      </c>
+      <c r="O86" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P86" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q86" s="6">
+        <v>0</v>
+      </c>
+      <c r="R86" s="7">
+        <v>0</v>
+      </c>
+      <c r="S86" s="9">
+        <v>0</v>
+      </c>
+      <c r="T86" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U86" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V86" s="11">
+        <v>11</v>
+      </c>
+      <c r="W86" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X86" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y86" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB86" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG86" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI86" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ86" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK86" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL86" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM86" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR86" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="87" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
+        <v>1</v>
+      </c>
+      <c r="B87" s="2">
+        <v>2</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F87" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G87" s="5">
+        <v>89</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I87" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J87" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K87" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L87" s="6">
+        <v>1728</v>
+      </c>
+      <c r="M87" s="7">
+        <v>326300.90999999997</v>
+      </c>
+      <c r="N87" s="6">
+        <v>1</v>
+      </c>
+      <c r="O87" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P87" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q87" s="6">
+        <v>0</v>
+      </c>
+      <c r="R87" s="7">
+        <v>0</v>
+      </c>
+      <c r="S87" s="9">
+        <v>0</v>
+      </c>
+      <c r="T87" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U87" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V87" s="11">
+        <v>11</v>
+      </c>
+      <c r="W87" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X87" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y87" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB87" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG87" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI87" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ87" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK87" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL87" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM87" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ87" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR87" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="88" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
+        <v>1</v>
+      </c>
+      <c r="B88" s="2">
+        <v>2</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F88" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G88" s="5">
+        <v>90</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I88" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L88" s="6">
+        <v>1729</v>
+      </c>
+      <c r="M88" s="7">
+        <v>326489.75</v>
+      </c>
+      <c r="N88" s="6">
+        <v>1</v>
+      </c>
+      <c r="O88" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P88" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q88" s="6">
+        <v>0</v>
+      </c>
+      <c r="R88" s="7">
+        <v>0</v>
+      </c>
+      <c r="S88" s="9">
+        <v>0</v>
+      </c>
+      <c r="T88" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U88" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V88" s="11">
+        <v>11</v>
+      </c>
+      <c r="W88" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X88" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y88" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB88" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG88" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI88" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ88" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK88" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL88" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM88" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR88" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="89" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>1</v>
+      </c>
+      <c r="B89" s="2">
+        <v>2</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F89" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G89" s="5">
+        <v>91</v>
+      </c>
+      <c r="H89" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I89" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J89" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K89" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L89" s="6">
+        <v>1730</v>
+      </c>
+      <c r="M89" s="7">
+        <v>326678.58</v>
+      </c>
+      <c r="N89" s="6">
+        <v>1</v>
+      </c>
+      <c r="O89" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P89" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q89" s="6">
+        <v>0</v>
+      </c>
+      <c r="R89" s="7">
+        <v>0</v>
+      </c>
+      <c r="S89" s="9">
+        <v>0</v>
+      </c>
+      <c r="T89" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U89" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V89" s="11">
+        <v>11</v>
+      </c>
+      <c r="W89" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X89" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y89" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB89" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG89" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI89" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ89" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK89" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL89" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM89" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ89" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR89" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="90" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
+        <v>1</v>
+      </c>
+      <c r="B90" s="2">
+        <v>2</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F90" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G90" s="5">
+        <v>92</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I90" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J90" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K90" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L90" s="6">
+        <v>1731</v>
+      </c>
+      <c r="M90" s="7">
+        <v>326867.40999999997</v>
+      </c>
+      <c r="N90" s="6">
+        <v>1</v>
+      </c>
+      <c r="O90" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P90" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q90" s="6">
+        <v>0</v>
+      </c>
+      <c r="R90" s="7">
+        <v>0</v>
+      </c>
+      <c r="S90" s="9">
+        <v>0</v>
+      </c>
+      <c r="T90" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U90" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V90" s="11">
+        <v>11</v>
+      </c>
+      <c r="W90" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X90" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y90" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB90" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG90" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI90" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ90" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK90" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL90" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM90" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR90" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="91" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A91" s="1">
+        <v>1</v>
+      </c>
+      <c r="B91" s="2">
+        <v>2</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F91" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G91" s="5">
+        <v>93</v>
+      </c>
+      <c r="H91" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I91" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J91" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K91" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L91" s="6">
+        <v>1732</v>
+      </c>
+      <c r="M91" s="7">
+        <v>327056.24</v>
+      </c>
+      <c r="N91" s="6">
+        <v>1</v>
+      </c>
+      <c r="O91" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P91" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q91" s="6">
+        <v>0</v>
+      </c>
+      <c r="R91" s="7">
+        <v>0</v>
+      </c>
+      <c r="S91" s="9">
+        <v>0</v>
+      </c>
+      <c r="T91" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U91" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V91" s="11">
+        <v>11</v>
+      </c>
+      <c r="W91" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X91" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y91" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z91" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA91" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB91" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC91" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD91" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE91" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF91" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG91" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH91" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI91" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ91" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK91" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL91" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM91" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN91" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO91" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP91" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ91" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR91" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="92" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A92" s="1">
+        <v>1</v>
+      </c>
+      <c r="B92" s="2">
+        <v>2</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F92" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G92" s="5">
+        <v>94</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I92" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J92" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K92" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L92" s="6">
+        <v>1733</v>
+      </c>
+      <c r="M92" s="7">
+        <v>327245.07</v>
+      </c>
+      <c r="N92" s="6">
+        <v>1</v>
+      </c>
+      <c r="O92" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P92" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q92" s="6">
+        <v>0</v>
+      </c>
+      <c r="R92" s="7">
+        <v>0</v>
+      </c>
+      <c r="S92" s="9">
+        <v>0</v>
+      </c>
+      <c r="T92" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U92" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V92" s="11">
+        <v>11</v>
+      </c>
+      <c r="W92" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X92" s="12">
+        <v>0.3826389</v>
+      </c>
+      <c r="Y92" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z92" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA92" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB92" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC92" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD92" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE92" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG92" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI92" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ92" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK92" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL92" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM92" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR92" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="93" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A93" s="1">
+        <v>1</v>
+      </c>
+      <c r="B93" s="2">
+        <v>2</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F93" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G93" s="5">
+        <v>95</v>
+      </c>
+      <c r="H93" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I93" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J93" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K93" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L93" s="6">
+        <v>1734</v>
+      </c>
+      <c r="M93" s="7">
+        <v>327433.90000000002</v>
+      </c>
+      <c r="N93" s="6">
+        <v>1</v>
+      </c>
+      <c r="O93" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P93" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q93" s="6">
+        <v>0</v>
+      </c>
+      <c r="R93" s="7">
+        <v>0</v>
+      </c>
+      <c r="S93" s="9">
+        <v>0</v>
+      </c>
+      <c r="T93" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U93" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V93" s="11">
+        <v>11</v>
+      </c>
+      <c r="W93" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X93" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y93" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB93" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG93" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI93" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ93" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK93" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL93" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM93" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR93" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="94" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A94" s="1">
+        <v>1</v>
+      </c>
+      <c r="B94" s="2">
+        <v>2</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F94" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G94" s="5">
+        <v>96</v>
+      </c>
+      <c r="H94" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I94" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J94" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K94" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L94" s="6">
+        <v>1735</v>
+      </c>
+      <c r="M94" s="7">
+        <v>327622.73</v>
+      </c>
+      <c r="N94" s="6">
+        <v>1</v>
+      </c>
+      <c r="O94" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P94" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q94" s="6">
+        <v>0</v>
+      </c>
+      <c r="R94" s="7">
+        <v>0</v>
+      </c>
+      <c r="S94" s="9">
+        <v>0</v>
+      </c>
+      <c r="T94" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U94" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V94" s="11">
+        <v>11</v>
+      </c>
+      <c r="W94" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X94" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y94" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z94" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA94" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB94" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC94" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD94" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE94" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG94" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI94" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ94" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK94" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL94" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM94" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR94" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="95" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A95" s="1">
+        <v>1</v>
+      </c>
+      <c r="B95" s="2">
+        <v>2</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F95" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G95" s="5">
+        <v>97</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I95" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J95" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K95" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L95" s="6">
+        <v>1736</v>
+      </c>
+      <c r="M95" s="7">
+        <v>327811.57</v>
+      </c>
+      <c r="N95" s="6">
+        <v>1</v>
+      </c>
+      <c r="O95" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P95" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q95" s="6">
+        <v>0</v>
+      </c>
+      <c r="R95" s="7">
+        <v>0</v>
+      </c>
+      <c r="S95" s="9">
+        <v>0</v>
+      </c>
+      <c r="T95" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U95" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V95" s="11">
+        <v>11</v>
+      </c>
+      <c r="W95" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X95" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y95" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z95" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA95" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB95" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC95" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD95" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE95" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF95" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG95" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH95" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI95" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ95" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK95" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL95" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM95" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN95" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO95" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP95" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ95" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR95" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="96" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A96" s="1">
+        <v>1</v>
+      </c>
+      <c r="B96" s="2">
+        <v>2</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E96" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F96" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G96" s="5">
+        <v>98</v>
+      </c>
+      <c r="H96" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I96" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J96" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K96" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L96" s="6">
+        <v>1737</v>
+      </c>
+      <c r="M96" s="7">
+        <v>328000.40000000002</v>
+      </c>
+      <c r="N96" s="6">
+        <v>1</v>
+      </c>
+      <c r="O96" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P96" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q96" s="6">
+        <v>0</v>
+      </c>
+      <c r="R96" s="7">
+        <v>0</v>
+      </c>
+      <c r="S96" s="9">
+        <v>0</v>
+      </c>
+      <c r="T96" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U96" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V96" s="11">
+        <v>11</v>
+      </c>
+      <c r="W96" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X96" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y96" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z96" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA96" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB96" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC96" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD96" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE96" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG96" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI96" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ96" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK96" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL96" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM96" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR96" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="97" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A97" s="1">
+        <v>1</v>
+      </c>
+      <c r="B97" s="2">
+        <v>2</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F97" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G97" s="5">
+        <v>99</v>
+      </c>
+      <c r="H97" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I97" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J97" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K97" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L97" s="6">
+        <v>1738</v>
+      </c>
+      <c r="M97" s="7">
+        <v>328189.23</v>
+      </c>
+      <c r="N97" s="6">
+        <v>1</v>
+      </c>
+      <c r="O97" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P97" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q97" s="6">
+        <v>0</v>
+      </c>
+      <c r="R97" s="7">
+        <v>0</v>
+      </c>
+      <c r="S97" s="9">
+        <v>0</v>
+      </c>
+      <c r="T97" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U97" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V97" s="11">
+        <v>11</v>
+      </c>
+      <c r="W97" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X97" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y97" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB97" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG97" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI97" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ97" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK97" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL97" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM97" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ97" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR97" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="98" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A98" s="1">
+        <v>1</v>
+      </c>
+      <c r="B98" s="2">
+        <v>2</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E98" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F98" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G98" s="5">
+        <v>100</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I98" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J98" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K98" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L98" s="6">
+        <v>1739</v>
+      </c>
+      <c r="M98" s="7">
+        <v>328378.06</v>
+      </c>
+      <c r="N98" s="6">
+        <v>1</v>
+      </c>
+      <c r="O98" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P98" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q98" s="6">
+        <v>0</v>
+      </c>
+      <c r="R98" s="7">
+        <v>0</v>
+      </c>
+      <c r="S98" s="9">
+        <v>0</v>
+      </c>
+      <c r="T98" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U98" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V98" s="11">
+        <v>11</v>
+      </c>
+      <c r="W98" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X98" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y98" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB98" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG98" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI98" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ98" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK98" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL98" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM98" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR98" s="3" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 13/05/2026  9:45:01,96
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD32733D-8E9E-4A47-BCAA-A236BAE39486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FBB24F5-04A3-42B6-B843-840848549A4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1790" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2330" uniqueCount="182">
   <si>
     <t>Sel</t>
   </si>
@@ -476,6 +476,96 @@
   </si>
   <si>
     <t>1858700137713</t>
+  </si>
+  <si>
+    <t>1858700137714</t>
+  </si>
+  <si>
+    <t>1858700137715</t>
+  </si>
+  <si>
+    <t>1858700137716</t>
+  </si>
+  <si>
+    <t>1858700137717</t>
+  </si>
+  <si>
+    <t>1858700137718</t>
+  </si>
+  <si>
+    <t>1858700137719</t>
+  </si>
+  <si>
+    <t>1858700137720</t>
+  </si>
+  <si>
+    <t>1858700137721</t>
+  </si>
+  <si>
+    <t>1858700137722</t>
+  </si>
+  <si>
+    <t>1858700137723</t>
+  </si>
+  <si>
+    <t>1858700137724</t>
+  </si>
+  <si>
+    <t>1858700137725</t>
+  </si>
+  <si>
+    <t>1858700137726</t>
+  </si>
+  <si>
+    <t>1858700137727</t>
+  </si>
+  <si>
+    <t>1858700137728</t>
+  </si>
+  <si>
+    <t>1858700137729</t>
+  </si>
+  <si>
+    <t>1858700137730</t>
+  </si>
+  <si>
+    <t>1858700137731</t>
+  </si>
+  <si>
+    <t>1858700137732</t>
+  </si>
+  <si>
+    <t>1858700137733</t>
+  </si>
+  <si>
+    <t>1858700137734</t>
+  </si>
+  <si>
+    <t>1858700137735</t>
+  </si>
+  <si>
+    <t>1858700137736</t>
+  </si>
+  <si>
+    <t>1858700137737</t>
+  </si>
+  <si>
+    <t>1858700137738</t>
+  </si>
+  <si>
+    <t>1858700137739</t>
+  </si>
+  <si>
+    <t>1858700137740</t>
+  </si>
+  <si>
+    <t>1858700137741</t>
+  </si>
+  <si>
+    <t>1858700137742</t>
+  </si>
+  <si>
+    <t>1858700137743</t>
   </si>
 </sst>
 </file>
@@ -1051,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR98"/>
+  <dimension ref="A1:AR128"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -14184,6 +14274,4026 @@
       </c>
       <c r="AR98" s="3" t="s">
         <v>151</v>
+      </c>
+    </row>
+    <row r="99" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A99" s="1">
+        <v>1</v>
+      </c>
+      <c r="B99" s="2">
+        <v>2</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F99" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G99" s="5">
+        <v>101</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J99" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K99" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L99" s="6">
+        <v>1740</v>
+      </c>
+      <c r="M99" s="7">
+        <v>328566.89</v>
+      </c>
+      <c r="N99" s="6">
+        <v>1</v>
+      </c>
+      <c r="O99" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P99" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q99" s="6">
+        <v>0</v>
+      </c>
+      <c r="R99" s="7">
+        <v>0</v>
+      </c>
+      <c r="S99" s="9">
+        <v>0</v>
+      </c>
+      <c r="T99" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U99" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V99" s="11">
+        <v>11</v>
+      </c>
+      <c r="W99" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X99" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y99" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB99" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG99" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI99" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ99" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK99" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL99" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM99" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ99" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR99" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="100" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A100" s="1">
+        <v>1</v>
+      </c>
+      <c r="B100" s="2">
+        <v>2</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F100" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G100" s="5">
+        <v>102</v>
+      </c>
+      <c r="H100" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I100" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J100" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K100" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L100" s="6">
+        <v>1741</v>
+      </c>
+      <c r="M100" s="7">
+        <v>328755.71999999997</v>
+      </c>
+      <c r="N100" s="6">
+        <v>1</v>
+      </c>
+      <c r="O100" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P100" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q100" s="6">
+        <v>0</v>
+      </c>
+      <c r="R100" s="7">
+        <v>0</v>
+      </c>
+      <c r="S100" s="9">
+        <v>0</v>
+      </c>
+      <c r="T100" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U100" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V100" s="11">
+        <v>11</v>
+      </c>
+      <c r="W100" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X100" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y100" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB100" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG100" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI100" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ100" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK100" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL100" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM100" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR100" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="101" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A101" s="1">
+        <v>1</v>
+      </c>
+      <c r="B101" s="2">
+        <v>2</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F101" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G101" s="5">
+        <v>103</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I101" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J101" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K101" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L101" s="6">
+        <v>1742</v>
+      </c>
+      <c r="M101" s="7">
+        <v>328944.56</v>
+      </c>
+      <c r="N101" s="6">
+        <v>1</v>
+      </c>
+      <c r="O101" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P101" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q101" s="6">
+        <v>0</v>
+      </c>
+      <c r="R101" s="7">
+        <v>0</v>
+      </c>
+      <c r="S101" s="9">
+        <v>0</v>
+      </c>
+      <c r="T101" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U101" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V101" s="11">
+        <v>11</v>
+      </c>
+      <c r="W101" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X101" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y101" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB101" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG101" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI101" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ101" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK101" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL101" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM101" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ101" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR101" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="102" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A102" s="1">
+        <v>1</v>
+      </c>
+      <c r="B102" s="2">
+        <v>2</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F102" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G102" s="5">
+        <v>104</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I102" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J102" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K102" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L102" s="6">
+        <v>1743</v>
+      </c>
+      <c r="M102" s="7">
+        <v>329133.39</v>
+      </c>
+      <c r="N102" s="6">
+        <v>1</v>
+      </c>
+      <c r="O102" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P102" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q102" s="6">
+        <v>0</v>
+      </c>
+      <c r="R102" s="7">
+        <v>0</v>
+      </c>
+      <c r="S102" s="9">
+        <v>0</v>
+      </c>
+      <c r="T102" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U102" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V102" s="11">
+        <v>11</v>
+      </c>
+      <c r="W102" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X102" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y102" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB102" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG102" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI102" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ102" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK102" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL102" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM102" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR102" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="103" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>1</v>
+      </c>
+      <c r="B103" s="2">
+        <v>2</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F103" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G103" s="5">
+        <v>105</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I103" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J103" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K103" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L103" s="6">
+        <v>1744</v>
+      </c>
+      <c r="M103" s="7">
+        <v>329322.21999999997</v>
+      </c>
+      <c r="N103" s="6">
+        <v>1</v>
+      </c>
+      <c r="O103" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P103" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q103" s="6">
+        <v>0</v>
+      </c>
+      <c r="R103" s="7">
+        <v>0</v>
+      </c>
+      <c r="S103" s="9">
+        <v>0</v>
+      </c>
+      <c r="T103" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U103" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V103" s="11">
+        <v>11</v>
+      </c>
+      <c r="W103" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X103" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y103" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB103" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG103" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI103" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ103" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK103" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL103" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM103" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ103" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR103" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="104" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
+        <v>1</v>
+      </c>
+      <c r="B104" s="2">
+        <v>2</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F104" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G104" s="5">
+        <v>106</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I104" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J104" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K104" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L104" s="6">
+        <v>1745</v>
+      </c>
+      <c r="M104" s="7">
+        <v>329511.05</v>
+      </c>
+      <c r="N104" s="6">
+        <v>1</v>
+      </c>
+      <c r="O104" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P104" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q104" s="6">
+        <v>0</v>
+      </c>
+      <c r="R104" s="7">
+        <v>0</v>
+      </c>
+      <c r="S104" s="9">
+        <v>0</v>
+      </c>
+      <c r="T104" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U104" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V104" s="11">
+        <v>11</v>
+      </c>
+      <c r="W104" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X104" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y104" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB104" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG104" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI104" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ104" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK104" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL104" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM104" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR104" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="105" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A105" s="1">
+        <v>1</v>
+      </c>
+      <c r="B105" s="2">
+        <v>2</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F105" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G105" s="5">
+        <v>107</v>
+      </c>
+      <c r="H105" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I105" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J105" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K105" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L105" s="6">
+        <v>1746</v>
+      </c>
+      <c r="M105" s="7">
+        <v>329699.88</v>
+      </c>
+      <c r="N105" s="6">
+        <v>1</v>
+      </c>
+      <c r="O105" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P105" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q105" s="6">
+        <v>0</v>
+      </c>
+      <c r="R105" s="7">
+        <v>0</v>
+      </c>
+      <c r="S105" s="9">
+        <v>0</v>
+      </c>
+      <c r="T105" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U105" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V105" s="11">
+        <v>11</v>
+      </c>
+      <c r="W105" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X105" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y105" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB105" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG105" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI105" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ105" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK105" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL105" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM105" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ105" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR105" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="106" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A106" s="1">
+        <v>1</v>
+      </c>
+      <c r="B106" s="2">
+        <v>2</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F106" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G106" s="5">
+        <v>108</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I106" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J106" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K106" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L106" s="6">
+        <v>1747</v>
+      </c>
+      <c r="M106" s="7">
+        <v>329888.71000000002</v>
+      </c>
+      <c r="N106" s="6">
+        <v>1</v>
+      </c>
+      <c r="O106" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P106" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q106" s="6">
+        <v>0</v>
+      </c>
+      <c r="R106" s="7">
+        <v>0</v>
+      </c>
+      <c r="S106" s="9">
+        <v>0</v>
+      </c>
+      <c r="T106" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U106" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V106" s="11">
+        <v>11</v>
+      </c>
+      <c r="W106" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X106" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y106" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB106" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG106" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI106" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ106" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK106" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL106" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM106" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR106" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="107" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A107" s="1">
+        <v>1</v>
+      </c>
+      <c r="B107" s="2">
+        <v>2</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F107" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G107" s="5">
+        <v>109</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I107" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J107" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K107" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L107" s="6">
+        <v>1748</v>
+      </c>
+      <c r="M107" s="7">
+        <v>330077.53999999998</v>
+      </c>
+      <c r="N107" s="6">
+        <v>1</v>
+      </c>
+      <c r="O107" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P107" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q107" s="6">
+        <v>0</v>
+      </c>
+      <c r="R107" s="7">
+        <v>0</v>
+      </c>
+      <c r="S107" s="9">
+        <v>0</v>
+      </c>
+      <c r="T107" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U107" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V107" s="11">
+        <v>11</v>
+      </c>
+      <c r="W107" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X107" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y107" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB107" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG107" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI107" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ107" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK107" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL107" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM107" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ107" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR107" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="108" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A108" s="1">
+        <v>1</v>
+      </c>
+      <c r="B108" s="2">
+        <v>2</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F108" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G108" s="5">
+        <v>110</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I108" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J108" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K108" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L108" s="6">
+        <v>1749</v>
+      </c>
+      <c r="M108" s="7">
+        <v>330266.38</v>
+      </c>
+      <c r="N108" s="6">
+        <v>1</v>
+      </c>
+      <c r="O108" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P108" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q108" s="6">
+        <v>0</v>
+      </c>
+      <c r="R108" s="7">
+        <v>0</v>
+      </c>
+      <c r="S108" s="9">
+        <v>0</v>
+      </c>
+      <c r="T108" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U108" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V108" s="11">
+        <v>11</v>
+      </c>
+      <c r="W108" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X108" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y108" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB108" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG108" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI108" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ108" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK108" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL108" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM108" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR108" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="109" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A109" s="1">
+        <v>1</v>
+      </c>
+      <c r="B109" s="2">
+        <v>2</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F109" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G109" s="5">
+        <v>111</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I109" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J109" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K109" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L109" s="6">
+        <v>1750</v>
+      </c>
+      <c r="M109" s="7">
+        <v>330455.21000000002</v>
+      </c>
+      <c r="N109" s="6">
+        <v>1</v>
+      </c>
+      <c r="O109" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P109" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q109" s="6">
+        <v>0</v>
+      </c>
+      <c r="R109" s="7">
+        <v>0</v>
+      </c>
+      <c r="S109" s="9">
+        <v>0</v>
+      </c>
+      <c r="T109" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U109" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V109" s="11">
+        <v>11</v>
+      </c>
+      <c r="W109" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X109" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y109" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB109" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG109" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI109" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ109" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK109" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL109" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM109" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ109" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR109" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="110" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
+        <v>1</v>
+      </c>
+      <c r="B110" s="2">
+        <v>2</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F110" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G110" s="5">
+        <v>112</v>
+      </c>
+      <c r="H110" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I110" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J110" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K110" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L110" s="6">
+        <v>1751</v>
+      </c>
+      <c r="M110" s="7">
+        <v>330644.03999999998</v>
+      </c>
+      <c r="N110" s="6">
+        <v>1</v>
+      </c>
+      <c r="O110" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P110" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q110" s="6">
+        <v>0</v>
+      </c>
+      <c r="R110" s="7">
+        <v>0</v>
+      </c>
+      <c r="S110" s="9">
+        <v>0</v>
+      </c>
+      <c r="T110" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U110" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V110" s="11">
+        <v>11</v>
+      </c>
+      <c r="W110" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X110" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y110" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB110" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG110" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI110" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ110" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK110" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL110" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM110" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR110" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="111" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
+        <v>1</v>
+      </c>
+      <c r="B111" s="2">
+        <v>2</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F111" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G111" s="5">
+        <v>113</v>
+      </c>
+      <c r="H111" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I111" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J111" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K111" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L111" s="6">
+        <v>1752</v>
+      </c>
+      <c r="M111" s="7">
+        <v>330832.87</v>
+      </c>
+      <c r="N111" s="6">
+        <v>1</v>
+      </c>
+      <c r="O111" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P111" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q111" s="6">
+        <v>0</v>
+      </c>
+      <c r="R111" s="7">
+        <v>0</v>
+      </c>
+      <c r="S111" s="9">
+        <v>0</v>
+      </c>
+      <c r="T111" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U111" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V111" s="11">
+        <v>11</v>
+      </c>
+      <c r="W111" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X111" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y111" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB111" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG111" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI111" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ111" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK111" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL111" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM111" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ111" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR111" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="112" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A112" s="1">
+        <v>1</v>
+      </c>
+      <c r="B112" s="2">
+        <v>2</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F112" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G112" s="5">
+        <v>114</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I112" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J112" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K112" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L112" s="6">
+        <v>1753</v>
+      </c>
+      <c r="M112" s="7">
+        <v>331021.7</v>
+      </c>
+      <c r="N112" s="6">
+        <v>1</v>
+      </c>
+      <c r="O112" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P112" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q112" s="6">
+        <v>0</v>
+      </c>
+      <c r="R112" s="7">
+        <v>0</v>
+      </c>
+      <c r="S112" s="9">
+        <v>0</v>
+      </c>
+      <c r="T112" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U112" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V112" s="11">
+        <v>11</v>
+      </c>
+      <c r="W112" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X112" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y112" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB112" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG112" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI112" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ112" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK112" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL112" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM112" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR112" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="113" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
+        <v>1</v>
+      </c>
+      <c r="B113" s="2">
+        <v>2</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E113" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F113" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G113" s="5">
+        <v>115</v>
+      </c>
+      <c r="H113" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J113" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K113" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L113" s="6">
+        <v>1754</v>
+      </c>
+      <c r="M113" s="7">
+        <v>331210.53000000003</v>
+      </c>
+      <c r="N113" s="6">
+        <v>1</v>
+      </c>
+      <c r="O113" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P113" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q113" s="6">
+        <v>0</v>
+      </c>
+      <c r="R113" s="7">
+        <v>0</v>
+      </c>
+      <c r="S113" s="9">
+        <v>0</v>
+      </c>
+      <c r="T113" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U113" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V113" s="11">
+        <v>11</v>
+      </c>
+      <c r="W113" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X113" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y113" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB113" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG113" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI113" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ113" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK113" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL113" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM113" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR113" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="114" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
+        <v>1</v>
+      </c>
+      <c r="B114" s="2">
+        <v>2</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F114" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G114" s="5">
+        <v>116</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I114" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J114" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K114" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L114" s="6">
+        <v>1755</v>
+      </c>
+      <c r="M114" s="7">
+        <v>331399.37</v>
+      </c>
+      <c r="N114" s="6">
+        <v>1</v>
+      </c>
+      <c r="O114" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P114" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q114" s="6">
+        <v>0</v>
+      </c>
+      <c r="R114" s="7">
+        <v>0</v>
+      </c>
+      <c r="S114" s="9">
+        <v>0</v>
+      </c>
+      <c r="T114" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U114" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V114" s="11">
+        <v>11</v>
+      </c>
+      <c r="W114" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X114" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y114" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB114" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG114" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI114" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ114" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK114" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL114" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM114" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR114" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="115" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
+        <v>1</v>
+      </c>
+      <c r="B115" s="2">
+        <v>2</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F115" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G115" s="5">
+        <v>117</v>
+      </c>
+      <c r="H115" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I115" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J115" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K115" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L115" s="6">
+        <v>1756</v>
+      </c>
+      <c r="M115" s="7">
+        <v>331588.2</v>
+      </c>
+      <c r="N115" s="6">
+        <v>1</v>
+      </c>
+      <c r="O115" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P115" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q115" s="6">
+        <v>0</v>
+      </c>
+      <c r="R115" s="7">
+        <v>0</v>
+      </c>
+      <c r="S115" s="9">
+        <v>0</v>
+      </c>
+      <c r="T115" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U115" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V115" s="11">
+        <v>11</v>
+      </c>
+      <c r="W115" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X115" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y115" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB115" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG115" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI115" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ115" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK115" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL115" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM115" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ115" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR115" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="116" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
+        <v>1</v>
+      </c>
+      <c r="B116" s="2">
+        <v>2</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F116" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G116" s="5">
+        <v>118</v>
+      </c>
+      <c r="H116" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I116" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J116" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K116" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L116" s="6">
+        <v>1757</v>
+      </c>
+      <c r="M116" s="7">
+        <v>331777.03000000003</v>
+      </c>
+      <c r="N116" s="6">
+        <v>1</v>
+      </c>
+      <c r="O116" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P116" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q116" s="6">
+        <v>0</v>
+      </c>
+      <c r="R116" s="7">
+        <v>0</v>
+      </c>
+      <c r="S116" s="9">
+        <v>0</v>
+      </c>
+      <c r="T116" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U116" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V116" s="11">
+        <v>11</v>
+      </c>
+      <c r="W116" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X116" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y116" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB116" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG116" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI116" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ116" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK116" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL116" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM116" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR116" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="117" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>1</v>
+      </c>
+      <c r="B117" s="2">
+        <v>2</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F117" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G117" s="5">
+        <v>119</v>
+      </c>
+      <c r="H117" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I117" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J117" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K117" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L117" s="6">
+        <v>1758</v>
+      </c>
+      <c r="M117" s="7">
+        <v>331965.86</v>
+      </c>
+      <c r="N117" s="6">
+        <v>1</v>
+      </c>
+      <c r="O117" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P117" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q117" s="6">
+        <v>0</v>
+      </c>
+      <c r="R117" s="7">
+        <v>0</v>
+      </c>
+      <c r="S117" s="9">
+        <v>0</v>
+      </c>
+      <c r="T117" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U117" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V117" s="11">
+        <v>11</v>
+      </c>
+      <c r="W117" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X117" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y117" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB117" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG117" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI117" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ117" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK117" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL117" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM117" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ117" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR117" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="118" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>1</v>
+      </c>
+      <c r="B118" s="2">
+        <v>2</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F118" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G118" s="5">
+        <v>120</v>
+      </c>
+      <c r="H118" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I118" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J118" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K118" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L118" s="6">
+        <v>1759</v>
+      </c>
+      <c r="M118" s="7">
+        <v>332154.69</v>
+      </c>
+      <c r="N118" s="6">
+        <v>1</v>
+      </c>
+      <c r="O118" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P118" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q118" s="6">
+        <v>0</v>
+      </c>
+      <c r="R118" s="7">
+        <v>0</v>
+      </c>
+      <c r="S118" s="9">
+        <v>0</v>
+      </c>
+      <c r="T118" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U118" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V118" s="11">
+        <v>11</v>
+      </c>
+      <c r="W118" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X118" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y118" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB118" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG118" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI118" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ118" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK118" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL118" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM118" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR118" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="119" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
+        <v>1</v>
+      </c>
+      <c r="B119" s="2">
+        <v>2</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F119" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G119" s="5">
+        <v>121</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I119" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J119" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K119" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L119" s="6">
+        <v>1760</v>
+      </c>
+      <c r="M119" s="7">
+        <v>332343.52</v>
+      </c>
+      <c r="N119" s="6">
+        <v>1</v>
+      </c>
+      <c r="O119" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P119" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q119" s="6">
+        <v>0</v>
+      </c>
+      <c r="R119" s="7">
+        <v>0</v>
+      </c>
+      <c r="S119" s="9">
+        <v>0</v>
+      </c>
+      <c r="T119" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U119" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V119" s="11">
+        <v>11</v>
+      </c>
+      <c r="W119" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X119" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y119" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB119" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG119" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI119" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ119" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK119" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL119" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM119" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ119" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR119" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="120" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
+        <v>1</v>
+      </c>
+      <c r="B120" s="2">
+        <v>2</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F120" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G120" s="5">
+        <v>122</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I120" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J120" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K120" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L120" s="6">
+        <v>1761</v>
+      </c>
+      <c r="M120" s="7">
+        <v>332532.34999999998</v>
+      </c>
+      <c r="N120" s="6">
+        <v>1</v>
+      </c>
+      <c r="O120" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P120" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q120" s="6">
+        <v>0</v>
+      </c>
+      <c r="R120" s="7">
+        <v>0</v>
+      </c>
+      <c r="S120" s="9">
+        <v>0</v>
+      </c>
+      <c r="T120" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U120" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V120" s="11">
+        <v>11</v>
+      </c>
+      <c r="W120" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X120" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y120" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB120" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG120" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI120" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ120" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK120" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL120" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM120" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR120" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="121" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
+        <v>1</v>
+      </c>
+      <c r="B121" s="2">
+        <v>2</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F121" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G121" s="5">
+        <v>123</v>
+      </c>
+      <c r="H121" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I121" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J121" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K121" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L121" s="6">
+        <v>1762</v>
+      </c>
+      <c r="M121" s="7">
+        <v>332721.19</v>
+      </c>
+      <c r="N121" s="6">
+        <v>1</v>
+      </c>
+      <c r="O121" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P121" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q121" s="6">
+        <v>0</v>
+      </c>
+      <c r="R121" s="7">
+        <v>0</v>
+      </c>
+      <c r="S121" s="9">
+        <v>0</v>
+      </c>
+      <c r="T121" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U121" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V121" s="11">
+        <v>11</v>
+      </c>
+      <c r="W121" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X121" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y121" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB121" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG121" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI121" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ121" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK121" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL121" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM121" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ121" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR121" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="122" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>1</v>
+      </c>
+      <c r="B122" s="2">
+        <v>2</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F122" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G122" s="5">
+        <v>124</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I122" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J122" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K122" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L122" s="6">
+        <v>1763</v>
+      </c>
+      <c r="M122" s="7">
+        <v>332910.02</v>
+      </c>
+      <c r="N122" s="6">
+        <v>1</v>
+      </c>
+      <c r="O122" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P122" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q122" s="6">
+        <v>0</v>
+      </c>
+      <c r="R122" s="7">
+        <v>0</v>
+      </c>
+      <c r="S122" s="9">
+        <v>0</v>
+      </c>
+      <c r="T122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U122" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V122" s="11">
+        <v>11</v>
+      </c>
+      <c r="W122" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X122" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y122" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB122" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG122" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI122" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK122" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM122" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR122" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="123" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
+        <v>1</v>
+      </c>
+      <c r="B123" s="2">
+        <v>2</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F123" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G123" s="5">
+        <v>125</v>
+      </c>
+      <c r="H123" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I123" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J123" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K123" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L123" s="6">
+        <v>1764</v>
+      </c>
+      <c r="M123" s="7">
+        <v>333098.84999999998</v>
+      </c>
+      <c r="N123" s="6">
+        <v>1</v>
+      </c>
+      <c r="O123" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P123" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q123" s="6">
+        <v>0</v>
+      </c>
+      <c r="R123" s="7">
+        <v>0</v>
+      </c>
+      <c r="S123" s="9">
+        <v>0</v>
+      </c>
+      <c r="T123" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U123" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V123" s="11">
+        <v>11</v>
+      </c>
+      <c r="W123" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X123" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y123" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB123" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG123" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI123" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ123" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK123" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL123" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM123" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ123" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR123" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="124" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>1</v>
+      </c>
+      <c r="B124" s="2">
+        <v>2</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F124" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G124" s="5">
+        <v>126</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I124" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J124" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K124" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L124" s="6">
+        <v>1765</v>
+      </c>
+      <c r="M124" s="7">
+        <v>333287.67999999999</v>
+      </c>
+      <c r="N124" s="6">
+        <v>1</v>
+      </c>
+      <c r="O124" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P124" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q124" s="6">
+        <v>0</v>
+      </c>
+      <c r="R124" s="7">
+        <v>0</v>
+      </c>
+      <c r="S124" s="9">
+        <v>0</v>
+      </c>
+      <c r="T124" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U124" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V124" s="11">
+        <v>11</v>
+      </c>
+      <c r="W124" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X124" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y124" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB124" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG124" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI124" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ124" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK124" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL124" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM124" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR124" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="125" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
+        <v>1</v>
+      </c>
+      <c r="B125" s="2">
+        <v>2</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F125" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G125" s="5">
+        <v>127</v>
+      </c>
+      <c r="H125" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I125" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J125" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K125" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L125" s="6">
+        <v>1766</v>
+      </c>
+      <c r="M125" s="7">
+        <v>333476.51</v>
+      </c>
+      <c r="N125" s="6">
+        <v>1</v>
+      </c>
+      <c r="O125" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P125" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q125" s="6">
+        <v>0</v>
+      </c>
+      <c r="R125" s="7">
+        <v>0</v>
+      </c>
+      <c r="S125" s="9">
+        <v>0</v>
+      </c>
+      <c r="T125" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U125" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V125" s="11">
+        <v>11</v>
+      </c>
+      <c r="W125" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X125" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y125" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB125" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG125" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI125" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ125" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK125" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL125" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM125" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ125" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR125" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="126" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A126" s="1">
+        <v>1</v>
+      </c>
+      <c r="B126" s="2">
+        <v>2</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F126" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G126" s="5">
+        <v>128</v>
+      </c>
+      <c r="H126" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I126" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J126" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K126" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L126" s="6">
+        <v>1767</v>
+      </c>
+      <c r="M126" s="7">
+        <v>333665.34000000003</v>
+      </c>
+      <c r="N126" s="6">
+        <v>1</v>
+      </c>
+      <c r="O126" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P126" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q126" s="6">
+        <v>0</v>
+      </c>
+      <c r="R126" s="7">
+        <v>0</v>
+      </c>
+      <c r="S126" s="9">
+        <v>0</v>
+      </c>
+      <c r="T126" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U126" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V126" s="11">
+        <v>11</v>
+      </c>
+      <c r="W126" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X126" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y126" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB126" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG126" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI126" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ126" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK126" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL126" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM126" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR126" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="127" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A127" s="1">
+        <v>1</v>
+      </c>
+      <c r="B127" s="2">
+        <v>2</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E127" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F127" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G127" s="5">
+        <v>129</v>
+      </c>
+      <c r="H127" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I127" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J127" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K127" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L127" s="6">
+        <v>1768</v>
+      </c>
+      <c r="M127" s="7">
+        <v>333854.18</v>
+      </c>
+      <c r="N127" s="6">
+        <v>1</v>
+      </c>
+      <c r="O127" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P127" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q127" s="6">
+        <v>0</v>
+      </c>
+      <c r="R127" s="7">
+        <v>0</v>
+      </c>
+      <c r="S127" s="9">
+        <v>0</v>
+      </c>
+      <c r="T127" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U127" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V127" s="11">
+        <v>11</v>
+      </c>
+      <c r="W127" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X127" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y127" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB127" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG127" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI127" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ127" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK127" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL127" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM127" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ127" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR127" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="128" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A128" s="1">
+        <v>1</v>
+      </c>
+      <c r="B128" s="2">
+        <v>2</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F128" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G128" s="5">
+        <v>130</v>
+      </c>
+      <c r="H128" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I128" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J128" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K128" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L128" s="6">
+        <v>1769</v>
+      </c>
+      <c r="M128" s="7">
+        <v>334043.01</v>
+      </c>
+      <c r="N128" s="6">
+        <v>1</v>
+      </c>
+      <c r="O128" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P128" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q128" s="6">
+        <v>0</v>
+      </c>
+      <c r="R128" s="7">
+        <v>0</v>
+      </c>
+      <c r="S128" s="9">
+        <v>0</v>
+      </c>
+      <c r="T128" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U128" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V128" s="11">
+        <v>11</v>
+      </c>
+      <c r="W128" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X128" s="12">
+        <v>0.4034722</v>
+      </c>
+      <c r="Y128" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB128" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG128" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI128" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ128" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK128" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL128" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM128" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR128" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 13/05/2026 12:49:14,93
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D0DBAC3-CB5B-4727-9BC0-2772364A617D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2AC7E95-A748-4E14-A3E2-5BC70F37679F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5048" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5480" uniqueCount="357">
   <si>
     <t>Sel</t>
   </si>
@@ -1020,6 +1020,78 @@
   <si>
     <t>1858700137894</t>
   </si>
+  <si>
+    <t>1858700137895</t>
+  </si>
+  <si>
+    <t>1858700137896</t>
+  </si>
+  <si>
+    <t>1858700137897</t>
+  </si>
+  <si>
+    <t>1858700137898</t>
+  </si>
+  <si>
+    <t>1858700137899</t>
+  </si>
+  <si>
+    <t>1858700137900</t>
+  </si>
+  <si>
+    <t>1858700137901</t>
+  </si>
+  <si>
+    <t>1858700137902</t>
+  </si>
+  <si>
+    <t>1858700137903</t>
+  </si>
+  <si>
+    <t>1858700137904</t>
+  </si>
+  <si>
+    <t>1858700137905</t>
+  </si>
+  <si>
+    <t>1858700137906</t>
+  </si>
+  <si>
+    <t>1858700137907</t>
+  </si>
+  <si>
+    <t>1858700137908</t>
+  </si>
+  <si>
+    <t>1858700137909</t>
+  </si>
+  <si>
+    <t>1858700137910</t>
+  </si>
+  <si>
+    <t>1858700137911</t>
+  </si>
+  <si>
+    <t>1858700137912</t>
+  </si>
+  <si>
+    <t>1858700137913</t>
+  </si>
+  <si>
+    <t>1858700137914</t>
+  </si>
+  <si>
+    <t>1858700137915</t>
+  </si>
+  <si>
+    <t>1858700137916</t>
+  </si>
+  <si>
+    <t>1858700137917</t>
+  </si>
+  <si>
+    <t>1858700137918</t>
+  </si>
 </sst>
 </file>
 
@@ -1594,7 +1666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR279"/>
+  <dimension ref="A1:AR303"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -38981,6 +39053,3222 @@
       </c>
       <c r="AR279" s="3" t="s">
         <v>332</v>
+      </c>
+    </row>
+    <row r="280" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A280" s="1">
+        <v>1</v>
+      </c>
+      <c r="B280" s="2">
+        <v>2</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D280" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E280" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F280" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G280" s="5">
+        <v>282</v>
+      </c>
+      <c r="H280" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I280" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J280" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K280" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L280" s="6">
+        <v>1921</v>
+      </c>
+      <c r="M280" s="7">
+        <v>362745.4</v>
+      </c>
+      <c r="N280" s="6">
+        <v>1</v>
+      </c>
+      <c r="O280" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P280" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q280" s="6">
+        <v>0</v>
+      </c>
+      <c r="R280" s="7">
+        <v>0</v>
+      </c>
+      <c r="S280" s="9">
+        <v>0</v>
+      </c>
+      <c r="T280" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U280" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V280" s="11">
+        <v>11</v>
+      </c>
+      <c r="W280" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X280" s="12">
+        <v>0.50694439999999996</v>
+      </c>
+      <c r="Y280" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB280" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG280" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI280" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ280" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK280" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL280" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM280" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ280" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR280" s="3" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="281" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A281" s="1">
+        <v>1</v>
+      </c>
+      <c r="B281" s="2">
+        <v>2</v>
+      </c>
+      <c r="C281" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D281" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E281" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F281" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G281" s="5">
+        <v>283</v>
+      </c>
+      <c r="H281" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I281" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J281" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K281" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L281" s="6">
+        <v>1922</v>
+      </c>
+      <c r="M281" s="7">
+        <v>362934.23</v>
+      </c>
+      <c r="N281" s="6">
+        <v>1</v>
+      </c>
+      <c r="O281" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P281" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q281" s="6">
+        <v>0</v>
+      </c>
+      <c r="R281" s="7">
+        <v>0</v>
+      </c>
+      <c r="S281" s="9">
+        <v>0</v>
+      </c>
+      <c r="T281" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U281" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V281" s="11">
+        <v>11</v>
+      </c>
+      <c r="W281" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X281" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y281" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB281" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG281" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI281" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ281" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK281" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL281" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM281" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ281" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR281" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="282" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A282" s="1">
+        <v>1</v>
+      </c>
+      <c r="B282" s="2">
+        <v>2</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D282" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E282" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F282" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G282" s="5">
+        <v>284</v>
+      </c>
+      <c r="H282" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I282" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J282" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K282" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L282" s="6">
+        <v>1923</v>
+      </c>
+      <c r="M282" s="7">
+        <v>363123.07</v>
+      </c>
+      <c r="N282" s="6">
+        <v>1</v>
+      </c>
+      <c r="O282" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P282" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q282" s="6">
+        <v>0</v>
+      </c>
+      <c r="R282" s="7">
+        <v>0</v>
+      </c>
+      <c r="S282" s="9">
+        <v>0</v>
+      </c>
+      <c r="T282" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U282" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V282" s="11">
+        <v>11</v>
+      </c>
+      <c r="W282" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X282" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y282" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB282" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG282" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI282" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ282" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK282" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL282" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM282" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ282" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR282" s="3" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="283" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A283" s="1">
+        <v>1</v>
+      </c>
+      <c r="B283" s="2">
+        <v>2</v>
+      </c>
+      <c r="C283" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D283" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E283" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F283" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G283" s="5">
+        <v>285</v>
+      </c>
+      <c r="H283" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I283" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J283" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K283" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L283" s="6">
+        <v>1924</v>
+      </c>
+      <c r="M283" s="7">
+        <v>363311.9</v>
+      </c>
+      <c r="N283" s="6">
+        <v>1</v>
+      </c>
+      <c r="O283" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P283" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q283" s="6">
+        <v>0</v>
+      </c>
+      <c r="R283" s="7">
+        <v>0</v>
+      </c>
+      <c r="S283" s="9">
+        <v>0</v>
+      </c>
+      <c r="T283" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U283" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V283" s="11">
+        <v>11</v>
+      </c>
+      <c r="W283" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X283" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y283" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB283" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG283" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI283" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ283" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK283" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL283" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM283" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ283" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR283" s="3" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="284" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A284" s="1">
+        <v>1</v>
+      </c>
+      <c r="B284" s="2">
+        <v>2</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D284" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E284" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F284" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G284" s="5">
+        <v>286</v>
+      </c>
+      <c r="H284" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I284" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J284" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K284" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L284" s="6">
+        <v>1925</v>
+      </c>
+      <c r="M284" s="7">
+        <v>363500.73</v>
+      </c>
+      <c r="N284" s="6">
+        <v>1</v>
+      </c>
+      <c r="O284" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P284" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q284" s="6">
+        <v>0</v>
+      </c>
+      <c r="R284" s="7">
+        <v>0</v>
+      </c>
+      <c r="S284" s="9">
+        <v>0</v>
+      </c>
+      <c r="T284" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U284" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V284" s="11">
+        <v>11</v>
+      </c>
+      <c r="W284" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X284" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y284" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB284" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG284" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI284" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ284" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK284" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL284" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM284" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ284" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR284" s="3" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="285" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A285" s="1">
+        <v>1</v>
+      </c>
+      <c r="B285" s="2">
+        <v>2</v>
+      </c>
+      <c r="C285" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D285" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E285" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F285" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G285" s="5">
+        <v>287</v>
+      </c>
+      <c r="H285" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I285" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J285" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K285" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L285" s="6">
+        <v>1926</v>
+      </c>
+      <c r="M285" s="7">
+        <v>363689.56</v>
+      </c>
+      <c r="N285" s="6">
+        <v>1</v>
+      </c>
+      <c r="O285" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P285" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q285" s="6">
+        <v>0</v>
+      </c>
+      <c r="R285" s="7">
+        <v>0</v>
+      </c>
+      <c r="S285" s="9">
+        <v>0</v>
+      </c>
+      <c r="T285" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U285" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V285" s="11">
+        <v>11</v>
+      </c>
+      <c r="W285" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X285" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y285" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB285" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG285" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI285" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ285" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK285" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL285" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM285" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ285" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR285" s="3" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="286" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A286" s="1">
+        <v>1</v>
+      </c>
+      <c r="B286" s="2">
+        <v>2</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D286" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E286" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F286" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G286" s="5">
+        <v>288</v>
+      </c>
+      <c r="H286" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I286" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J286" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K286" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L286" s="6">
+        <v>1927</v>
+      </c>
+      <c r="M286" s="7">
+        <v>363878.39</v>
+      </c>
+      <c r="N286" s="6">
+        <v>1</v>
+      </c>
+      <c r="O286" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P286" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q286" s="6">
+        <v>0</v>
+      </c>
+      <c r="R286" s="7">
+        <v>0</v>
+      </c>
+      <c r="S286" s="9">
+        <v>0</v>
+      </c>
+      <c r="T286" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U286" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V286" s="11">
+        <v>11</v>
+      </c>
+      <c r="W286" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X286" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y286" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB286" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG286" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI286" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ286" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK286" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL286" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM286" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ286" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR286" s="3" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="287" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A287" s="1">
+        <v>1</v>
+      </c>
+      <c r="B287" s="2">
+        <v>2</v>
+      </c>
+      <c r="C287" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D287" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E287" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F287" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G287" s="5">
+        <v>289</v>
+      </c>
+      <c r="H287" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I287" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J287" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K287" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L287" s="6">
+        <v>1928</v>
+      </c>
+      <c r="M287" s="7">
+        <v>364067.22</v>
+      </c>
+      <c r="N287" s="6">
+        <v>1</v>
+      </c>
+      <c r="O287" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P287" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q287" s="6">
+        <v>0</v>
+      </c>
+      <c r="R287" s="7">
+        <v>0</v>
+      </c>
+      <c r="S287" s="9">
+        <v>0</v>
+      </c>
+      <c r="T287" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U287" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V287" s="11">
+        <v>11</v>
+      </c>
+      <c r="W287" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X287" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y287" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB287" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG287" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI287" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ287" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK287" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL287" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM287" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ287" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR287" s="3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="288" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A288" s="1">
+        <v>1</v>
+      </c>
+      <c r="B288" s="2">
+        <v>2</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E288" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F288" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G288" s="5">
+        <v>290</v>
+      </c>
+      <c r="H288" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I288" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J288" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K288" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L288" s="6">
+        <v>1929</v>
+      </c>
+      <c r="M288" s="7">
+        <v>364256.05</v>
+      </c>
+      <c r="N288" s="6">
+        <v>1</v>
+      </c>
+      <c r="O288" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P288" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q288" s="6">
+        <v>0</v>
+      </c>
+      <c r="R288" s="7">
+        <v>0</v>
+      </c>
+      <c r="S288" s="9">
+        <v>0</v>
+      </c>
+      <c r="T288" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U288" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V288" s="11">
+        <v>11</v>
+      </c>
+      <c r="W288" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X288" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y288" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB288" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG288" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI288" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ288" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK288" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL288" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM288" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ288" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR288" s="3" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="289" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A289" s="1">
+        <v>1</v>
+      </c>
+      <c r="B289" s="2">
+        <v>2</v>
+      </c>
+      <c r="C289" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D289" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E289" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F289" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G289" s="5">
+        <v>291</v>
+      </c>
+      <c r="H289" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I289" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J289" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K289" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L289" s="6">
+        <v>1930</v>
+      </c>
+      <c r="M289" s="7">
+        <v>364444.89</v>
+      </c>
+      <c r="N289" s="6">
+        <v>1</v>
+      </c>
+      <c r="O289" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P289" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q289" s="6">
+        <v>0</v>
+      </c>
+      <c r="R289" s="7">
+        <v>0</v>
+      </c>
+      <c r="S289" s="9">
+        <v>0</v>
+      </c>
+      <c r="T289" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U289" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V289" s="11">
+        <v>11</v>
+      </c>
+      <c r="W289" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X289" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y289" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB289" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG289" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI289" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ289" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK289" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL289" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM289" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ289" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR289" s="3" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="290" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A290" s="1">
+        <v>1</v>
+      </c>
+      <c r="B290" s="2">
+        <v>2</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D290" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E290" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F290" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G290" s="5">
+        <v>292</v>
+      </c>
+      <c r="H290" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I290" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J290" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K290" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L290" s="6">
+        <v>1931</v>
+      </c>
+      <c r="M290" s="7">
+        <v>364633.72</v>
+      </c>
+      <c r="N290" s="6">
+        <v>1</v>
+      </c>
+      <c r="O290" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P290" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q290" s="6">
+        <v>0</v>
+      </c>
+      <c r="R290" s="7">
+        <v>0</v>
+      </c>
+      <c r="S290" s="9">
+        <v>0</v>
+      </c>
+      <c r="T290" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U290" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V290" s="11">
+        <v>11</v>
+      </c>
+      <c r="W290" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X290" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y290" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB290" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG290" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI290" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ290" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK290" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL290" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM290" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ290" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR290" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="291" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A291" s="1">
+        <v>1</v>
+      </c>
+      <c r="B291" s="2">
+        <v>2</v>
+      </c>
+      <c r="C291" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D291" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E291" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F291" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G291" s="5">
+        <v>293</v>
+      </c>
+      <c r="H291" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I291" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J291" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K291" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L291" s="6">
+        <v>1932</v>
+      </c>
+      <c r="M291" s="7">
+        <v>364822.55</v>
+      </c>
+      <c r="N291" s="6">
+        <v>1</v>
+      </c>
+      <c r="O291" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P291" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q291" s="6">
+        <v>0</v>
+      </c>
+      <c r="R291" s="7">
+        <v>0</v>
+      </c>
+      <c r="S291" s="9">
+        <v>0</v>
+      </c>
+      <c r="T291" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U291" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V291" s="11">
+        <v>11</v>
+      </c>
+      <c r="W291" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X291" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y291" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB291" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG291" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI291" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ291" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK291" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL291" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM291" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ291" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR291" s="3" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="292" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A292" s="1">
+        <v>1</v>
+      </c>
+      <c r="B292" s="2">
+        <v>2</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F292" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G292" s="5">
+        <v>294</v>
+      </c>
+      <c r="H292" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I292" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J292" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K292" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L292" s="6">
+        <v>1933</v>
+      </c>
+      <c r="M292" s="7">
+        <v>365011.38</v>
+      </c>
+      <c r="N292" s="6">
+        <v>1</v>
+      </c>
+      <c r="O292" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P292" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q292" s="6">
+        <v>0</v>
+      </c>
+      <c r="R292" s="7">
+        <v>0</v>
+      </c>
+      <c r="S292" s="9">
+        <v>0</v>
+      </c>
+      <c r="T292" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U292" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V292" s="11">
+        <v>11</v>
+      </c>
+      <c r="W292" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X292" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y292" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB292" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG292" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI292" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ292" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK292" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL292" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM292" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ292" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR292" s="3" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="293" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A293" s="1">
+        <v>1</v>
+      </c>
+      <c r="B293" s="2">
+        <v>2</v>
+      </c>
+      <c r="C293" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D293" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E293" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F293" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G293" s="5">
+        <v>295</v>
+      </c>
+      <c r="H293" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I293" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J293" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K293" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L293" s="6">
+        <v>1934</v>
+      </c>
+      <c r="M293" s="7">
+        <v>365200.21</v>
+      </c>
+      <c r="N293" s="6">
+        <v>1</v>
+      </c>
+      <c r="O293" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P293" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q293" s="6">
+        <v>0</v>
+      </c>
+      <c r="R293" s="7">
+        <v>0</v>
+      </c>
+      <c r="S293" s="9">
+        <v>0</v>
+      </c>
+      <c r="T293" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U293" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V293" s="11">
+        <v>11</v>
+      </c>
+      <c r="W293" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X293" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y293" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB293" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG293" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI293" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ293" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK293" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL293" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM293" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ293" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR293" s="3" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="294" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A294" s="1">
+        <v>1</v>
+      </c>
+      <c r="B294" s="2">
+        <v>2</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F294" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G294" s="5">
+        <v>296</v>
+      </c>
+      <c r="H294" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I294" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J294" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K294" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L294" s="6">
+        <v>1935</v>
+      </c>
+      <c r="M294" s="7">
+        <v>365389.04</v>
+      </c>
+      <c r="N294" s="6">
+        <v>1</v>
+      </c>
+      <c r="O294" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P294" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q294" s="6">
+        <v>0</v>
+      </c>
+      <c r="R294" s="7">
+        <v>0</v>
+      </c>
+      <c r="S294" s="9">
+        <v>0</v>
+      </c>
+      <c r="T294" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U294" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V294" s="11">
+        <v>11</v>
+      </c>
+      <c r="W294" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X294" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y294" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB294" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG294" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI294" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ294" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK294" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL294" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM294" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ294" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR294" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="295" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A295" s="1">
+        <v>1</v>
+      </c>
+      <c r="B295" s="2">
+        <v>2</v>
+      </c>
+      <c r="C295" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E295" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F295" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G295" s="5">
+        <v>297</v>
+      </c>
+      <c r="H295" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I295" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J295" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K295" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L295" s="6">
+        <v>1936</v>
+      </c>
+      <c r="M295" s="7">
+        <v>365577.88</v>
+      </c>
+      <c r="N295" s="6">
+        <v>1</v>
+      </c>
+      <c r="O295" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P295" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q295" s="6">
+        <v>0</v>
+      </c>
+      <c r="R295" s="7">
+        <v>0</v>
+      </c>
+      <c r="S295" s="9">
+        <v>0</v>
+      </c>
+      <c r="T295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U295" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V295" s="11">
+        <v>11</v>
+      </c>
+      <c r="W295" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X295" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y295" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB295" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG295" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI295" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR295" s="3" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="296" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A296" s="1">
+        <v>1</v>
+      </c>
+      <c r="B296" s="2">
+        <v>2</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F296" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G296" s="5">
+        <v>298</v>
+      </c>
+      <c r="H296" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I296" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J296" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K296" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L296" s="6">
+        <v>1937</v>
+      </c>
+      <c r="M296" s="7">
+        <v>365766.71</v>
+      </c>
+      <c r="N296" s="6">
+        <v>1</v>
+      </c>
+      <c r="O296" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P296" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q296" s="6">
+        <v>0</v>
+      </c>
+      <c r="R296" s="7">
+        <v>0</v>
+      </c>
+      <c r="S296" s="9">
+        <v>0</v>
+      </c>
+      <c r="T296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U296" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V296" s="11">
+        <v>11</v>
+      </c>
+      <c r="W296" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X296" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y296" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB296" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG296" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI296" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR296" s="3" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="297" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A297" s="1">
+        <v>1</v>
+      </c>
+      <c r="B297" s="2">
+        <v>2</v>
+      </c>
+      <c r="C297" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E297" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F297" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G297" s="5">
+        <v>299</v>
+      </c>
+      <c r="H297" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I297" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J297" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K297" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L297" s="6">
+        <v>1938</v>
+      </c>
+      <c r="M297" s="7">
+        <v>365955.54</v>
+      </c>
+      <c r="N297" s="6">
+        <v>1</v>
+      </c>
+      <c r="O297" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P297" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q297" s="6">
+        <v>0</v>
+      </c>
+      <c r="R297" s="7">
+        <v>0</v>
+      </c>
+      <c r="S297" s="9">
+        <v>0</v>
+      </c>
+      <c r="T297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U297" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V297" s="11">
+        <v>11</v>
+      </c>
+      <c r="W297" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X297" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y297" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB297" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG297" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI297" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR297" s="3" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="298" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A298" s="1">
+        <v>1</v>
+      </c>
+      <c r="B298" s="2">
+        <v>2</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F298" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G298" s="5">
+        <v>300</v>
+      </c>
+      <c r="H298" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I298" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J298" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K298" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L298" s="6">
+        <v>1939</v>
+      </c>
+      <c r="M298" s="7">
+        <v>366144.37</v>
+      </c>
+      <c r="N298" s="6">
+        <v>1</v>
+      </c>
+      <c r="O298" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P298" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q298" s="6">
+        <v>0</v>
+      </c>
+      <c r="R298" s="7">
+        <v>0</v>
+      </c>
+      <c r="S298" s="9">
+        <v>0</v>
+      </c>
+      <c r="T298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U298" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V298" s="11">
+        <v>11</v>
+      </c>
+      <c r="W298" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X298" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y298" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB298" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG298" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI298" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR298" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="299" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A299" s="1">
+        <v>1</v>
+      </c>
+      <c r="B299" s="2">
+        <v>2</v>
+      </c>
+      <c r="C299" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D299" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E299" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F299" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G299" s="5">
+        <v>301</v>
+      </c>
+      <c r="H299" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I299" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J299" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K299" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L299" s="6">
+        <v>1940</v>
+      </c>
+      <c r="M299" s="7">
+        <v>366333.2</v>
+      </c>
+      <c r="N299" s="6">
+        <v>1</v>
+      </c>
+      <c r="O299" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P299" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q299" s="6">
+        <v>0</v>
+      </c>
+      <c r="R299" s="7">
+        <v>0</v>
+      </c>
+      <c r="S299" s="9">
+        <v>0</v>
+      </c>
+      <c r="T299" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U299" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V299" s="11">
+        <v>11</v>
+      </c>
+      <c r="W299" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X299" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y299" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB299" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG299" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI299" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ299" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK299" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL299" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM299" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ299" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR299" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="300" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A300" s="1">
+        <v>1</v>
+      </c>
+      <c r="B300" s="2">
+        <v>2</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F300" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G300" s="5">
+        <v>302</v>
+      </c>
+      <c r="H300" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I300" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J300" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K300" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L300" s="6">
+        <v>1941</v>
+      </c>
+      <c r="M300" s="7">
+        <v>366522.03</v>
+      </c>
+      <c r="N300" s="6">
+        <v>1</v>
+      </c>
+      <c r="O300" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P300" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q300" s="6">
+        <v>0</v>
+      </c>
+      <c r="R300" s="7">
+        <v>0</v>
+      </c>
+      <c r="S300" s="9">
+        <v>0</v>
+      </c>
+      <c r="T300" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U300" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V300" s="11">
+        <v>11</v>
+      </c>
+      <c r="W300" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X300" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y300" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB300" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG300" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI300" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ300" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK300" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL300" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM300" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ300" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR300" s="3" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="301" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A301" s="1">
+        <v>1</v>
+      </c>
+      <c r="B301" s="2">
+        <v>2</v>
+      </c>
+      <c r="C301" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D301" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E301" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F301" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G301" s="5">
+        <v>303</v>
+      </c>
+      <c r="H301" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I301" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J301" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K301" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L301" s="6">
+        <v>1942</v>
+      </c>
+      <c r="M301" s="7">
+        <v>366710.86</v>
+      </c>
+      <c r="N301" s="6">
+        <v>1</v>
+      </c>
+      <c r="O301" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P301" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q301" s="6">
+        <v>0</v>
+      </c>
+      <c r="R301" s="7">
+        <v>0</v>
+      </c>
+      <c r="S301" s="9">
+        <v>0</v>
+      </c>
+      <c r="T301" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U301" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V301" s="11">
+        <v>11</v>
+      </c>
+      <c r="W301" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X301" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y301" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB301" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG301" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI301" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ301" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK301" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL301" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM301" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ301" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR301" s="3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="302" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A302" s="1">
+        <v>1</v>
+      </c>
+      <c r="B302" s="2">
+        <v>2</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F302" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G302" s="5">
+        <v>304</v>
+      </c>
+      <c r="H302" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I302" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J302" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K302" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L302" s="6">
+        <v>1943</v>
+      </c>
+      <c r="M302" s="7">
+        <v>366899.7</v>
+      </c>
+      <c r="N302" s="6">
+        <v>1</v>
+      </c>
+      <c r="O302" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P302" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q302" s="6">
+        <v>0</v>
+      </c>
+      <c r="R302" s="7">
+        <v>0</v>
+      </c>
+      <c r="S302" s="9">
+        <v>0</v>
+      </c>
+      <c r="T302" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U302" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V302" s="11">
+        <v>11</v>
+      </c>
+      <c r="W302" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X302" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y302" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB302" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG302" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI302" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ302" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK302" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL302" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM302" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ302" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR302" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="303" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A303" s="1">
+        <v>1</v>
+      </c>
+      <c r="B303" s="2">
+        <v>2</v>
+      </c>
+      <c r="C303" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D303" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E303" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F303" s="4">
+        <v>46155</v>
+      </c>
+      <c r="G303" s="5">
+        <v>305</v>
+      </c>
+      <c r="H303" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I303" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J303" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K303" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L303" s="6">
+        <v>1944</v>
+      </c>
+      <c r="M303" s="7">
+        <v>367088.53</v>
+      </c>
+      <c r="N303" s="6">
+        <v>1</v>
+      </c>
+      <c r="O303" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P303" s="8">
+        <v>188.83</v>
+      </c>
+      <c r="Q303" s="6">
+        <v>0</v>
+      </c>
+      <c r="R303" s="7">
+        <v>0</v>
+      </c>
+      <c r="S303" s="9">
+        <v>0</v>
+      </c>
+      <c r="T303" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U303" s="10">
+        <v>64296</v>
+      </c>
+      <c r="V303" s="11">
+        <v>11</v>
+      </c>
+      <c r="W303" s="4">
+        <v>46155</v>
+      </c>
+      <c r="X303" s="12">
+        <v>0.5076389</v>
+      </c>
+      <c r="Y303" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB303" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG303" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI303" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ303" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK303" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL303" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM303" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ303" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR303" s="3" t="s">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026  9:28:56,93
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72281DD0-0D89-463A-A26B-5D6EEF0E743A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{464B751D-058F-4702-A462-F15C43DF552F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2204" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2222" uniqueCount="181">
   <si>
     <t>Sel</t>
   </si>
@@ -511,13 +511,22 @@
     <t>1854300114808</t>
   </si>
   <si>
+    <t>10016351</t>
+  </si>
+  <si>
+    <t>FORNO ELETRICO NARDELLI EMBUTIR INOX 60 LITROS - NARDELLI EMBUTIR INOX 60 LITROS - 127 V</t>
+  </si>
+  <si>
+    <t>FORNOE</t>
+  </si>
+  <si>
+    <t>1858400002936</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
     <t>FORNO ELETRICO NARDELLI E50 BLACK 50L - NARDELLI E50 BLACK 50 L - 127 V</t>
-  </si>
-  <si>
-    <t>FORNOE</t>
   </si>
   <si>
     <t>1879800000219</t>
@@ -1129,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR121"/>
+  <dimension ref="A1:AR122"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -15773,10 +15782,10 @@
         <v>50</v>
       </c>
       <c r="L110" s="6">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="M110" s="7">
-        <v>26267.89</v>
+        <v>16637.939999999999</v>
       </c>
       <c r="N110" s="6">
         <v>1</v>
@@ -15785,7 +15794,7 @@
         <v>164</v>
       </c>
       <c r="P110" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q110" s="6">
         <v>0</v>
@@ -15800,7 +15809,7 @@
         <v>52</v>
       </c>
       <c r="U110" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V110" s="11">
         <v>11</v>
@@ -15809,7 +15818,7 @@
         <v>46156</v>
       </c>
       <c r="X110" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.37847219999999998</v>
       </c>
       <c r="Y110" s="10">
         <v>0</v>
@@ -15880,7 +15889,7 @@
         <v>2</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>45</v>
@@ -15892,7 +15901,7 @@
         <v>46156</v>
       </c>
       <c r="G111" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H111" s="3" t="s">
         <v>47</v>
@@ -15907,16 +15916,16 @@
         <v>50</v>
       </c>
       <c r="L111" s="6">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M111" s="7">
-        <v>26648.59</v>
+        <v>26267.89</v>
       </c>
       <c r="N111" s="6">
         <v>1</v>
       </c>
       <c r="O111" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P111" s="8">
         <v>380.69</v>
@@ -16003,7 +16012,7 @@
         <v>53</v>
       </c>
       <c r="AR111" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="112" spans="1:44" x14ac:dyDescent="0.3">
@@ -16014,7 +16023,7 @@
         <v>2</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>45</v>
@@ -16026,7 +16035,7 @@
         <v>46156</v>
       </c>
       <c r="G112" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>47</v>
@@ -16041,16 +16050,16 @@
         <v>50</v>
       </c>
       <c r="L112" s="6">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M112" s="7">
-        <v>27029.279999999999</v>
+        <v>26648.59</v>
       </c>
       <c r="N112" s="6">
         <v>1</v>
       </c>
       <c r="O112" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P112" s="8">
         <v>380.69</v>
@@ -16137,7 +16146,7 @@
         <v>53</v>
       </c>
       <c r="AR112" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="113" spans="1:44" x14ac:dyDescent="0.3">
@@ -16148,7 +16157,7 @@
         <v>2</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>45</v>
@@ -16160,7 +16169,7 @@
         <v>46156</v>
       </c>
       <c r="G113" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>47</v>
@@ -16175,16 +16184,16 @@
         <v>50</v>
       </c>
       <c r="L113" s="6">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M113" s="7">
-        <v>27409.98</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N113" s="6">
         <v>1</v>
       </c>
       <c r="O113" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P113" s="8">
         <v>380.69</v>
@@ -16271,7 +16280,7 @@
         <v>53</v>
       </c>
       <c r="AR113" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="114" spans="1:44" x14ac:dyDescent="0.3">
@@ -16282,7 +16291,7 @@
         <v>2</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>45</v>
@@ -16294,7 +16303,7 @@
         <v>46156</v>
       </c>
       <c r="G114" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>47</v>
@@ -16309,16 +16318,16 @@
         <v>50</v>
       </c>
       <c r="L114" s="6">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M114" s="7">
-        <v>27790.67</v>
+        <v>27409.98</v>
       </c>
       <c r="N114" s="6">
         <v>1</v>
       </c>
       <c r="O114" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P114" s="8">
         <v>380.69</v>
@@ -16405,7 +16414,7 @@
         <v>53</v>
       </c>
       <c r="AR114" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="115" spans="1:44" x14ac:dyDescent="0.3">
@@ -16416,7 +16425,7 @@
         <v>2</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>45</v>
@@ -16428,7 +16437,7 @@
         <v>46156</v>
       </c>
       <c r="G115" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>47</v>
@@ -16443,16 +16452,16 @@
         <v>50</v>
       </c>
       <c r="L115" s="6">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M115" s="7">
-        <v>28171.360000000001</v>
+        <v>27790.67</v>
       </c>
       <c r="N115" s="6">
         <v>1</v>
       </c>
       <c r="O115" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P115" s="8">
         <v>380.69</v>
@@ -16539,7 +16548,7 @@
         <v>53</v>
       </c>
       <c r="AR115" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="116" spans="1:44" x14ac:dyDescent="0.3">
@@ -16550,7 +16559,7 @@
         <v>2</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>45</v>
@@ -16562,7 +16571,7 @@
         <v>46156</v>
       </c>
       <c r="G116" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>47</v>
@@ -16577,16 +16586,16 @@
         <v>50</v>
       </c>
       <c r="L116" s="6">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M116" s="7">
-        <v>28552.06</v>
+        <v>28171.360000000001</v>
       </c>
       <c r="N116" s="6">
         <v>1</v>
       </c>
       <c r="O116" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P116" s="8">
         <v>380.69</v>
@@ -16613,7 +16622,7 @@
         <v>46156</v>
       </c>
       <c r="X116" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y116" s="10">
         <v>0</v>
@@ -16673,7 +16682,7 @@
         <v>53</v>
       </c>
       <c r="AR116" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="117" spans="1:44" x14ac:dyDescent="0.3">
@@ -16684,7 +16693,7 @@
         <v>2</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>45</v>
@@ -16696,7 +16705,7 @@
         <v>46156</v>
       </c>
       <c r="G117" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>47</v>
@@ -16711,16 +16720,16 @@
         <v>50</v>
       </c>
       <c r="L117" s="6">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M117" s="7">
-        <v>28932.75</v>
+        <v>28552.06</v>
       </c>
       <c r="N117" s="6">
         <v>1</v>
       </c>
       <c r="O117" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P117" s="8">
         <v>380.69</v>
@@ -16807,7 +16816,7 @@
         <v>53</v>
       </c>
       <c r="AR117" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="118" spans="1:44" x14ac:dyDescent="0.3">
@@ -16818,7 +16827,7 @@
         <v>2</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>45</v>
@@ -16830,7 +16839,7 @@
         <v>46156</v>
       </c>
       <c r="G118" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H118" s="3" t="s">
         <v>47</v>
@@ -16845,16 +16854,16 @@
         <v>50</v>
       </c>
       <c r="L118" s="6">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M118" s="7">
-        <v>29313.45</v>
+        <v>28932.75</v>
       </c>
       <c r="N118" s="6">
         <v>1</v>
       </c>
       <c r="O118" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P118" s="8">
         <v>380.69</v>
@@ -16941,7 +16950,7 @@
         <v>53</v>
       </c>
       <c r="AR118" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="119" spans="1:44" x14ac:dyDescent="0.3">
@@ -16952,7 +16961,7 @@
         <v>2</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>45</v>
@@ -16964,7 +16973,7 @@
         <v>46156</v>
       </c>
       <c r="G119" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H119" s="3" t="s">
         <v>47</v>
@@ -16979,16 +16988,16 @@
         <v>50</v>
       </c>
       <c r="L119" s="6">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M119" s="7">
-        <v>29694.14</v>
+        <v>29313.45</v>
       </c>
       <c r="N119" s="6">
         <v>1</v>
       </c>
       <c r="O119" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P119" s="8">
         <v>380.69</v>
@@ -17015,7 +17024,7 @@
         <v>46156</v>
       </c>
       <c r="X119" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y119" s="10">
         <v>0</v>
@@ -17075,7 +17084,7 @@
         <v>53</v>
       </c>
       <c r="AR119" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="120" spans="1:44" x14ac:dyDescent="0.3">
@@ -17086,7 +17095,7 @@
         <v>2</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>45</v>
@@ -17098,7 +17107,7 @@
         <v>46156</v>
       </c>
       <c r="G120" s="5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H120" s="3" t="s">
         <v>47</v>
@@ -17113,16 +17122,16 @@
         <v>50</v>
       </c>
       <c r="L120" s="6">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M120" s="7">
-        <v>30074.83</v>
+        <v>29694.14</v>
       </c>
       <c r="N120" s="6">
         <v>1</v>
       </c>
       <c r="O120" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P120" s="8">
         <v>380.69</v>
@@ -17209,7 +17218,7 @@
         <v>53</v>
       </c>
       <c r="AR120" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="121" spans="1:44" x14ac:dyDescent="0.3">
@@ -17220,7 +17229,7 @@
         <v>2</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>45</v>
@@ -17232,7 +17241,7 @@
         <v>46156</v>
       </c>
       <c r="G121" s="5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>47</v>
@@ -17247,16 +17256,16 @@
         <v>50</v>
       </c>
       <c r="L121" s="6">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M121" s="7">
-        <v>30455.53</v>
+        <v>30074.83</v>
       </c>
       <c r="N121" s="6">
         <v>1</v>
       </c>
       <c r="O121" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="P121" s="8">
         <v>380.69</v>
@@ -17343,7 +17352,141 @@
         <v>53</v>
       </c>
       <c r="AR121" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="122" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>1</v>
+      </c>
+      <c r="B122" s="2">
+        <v>2</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F122" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G122" s="5">
+        <v>12</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I122" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J122" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K122" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L122" s="6">
+        <v>80</v>
+      </c>
+      <c r="M122" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N122" s="6">
+        <v>1</v>
+      </c>
+      <c r="O122" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="P122" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q122" s="6">
+        <v>0</v>
+      </c>
+      <c r="R122" s="7">
+        <v>0</v>
+      </c>
+      <c r="S122" s="9">
+        <v>0</v>
+      </c>
+      <c r="T122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U122" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V122" s="11">
+        <v>11</v>
+      </c>
+      <c r="W122" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X122" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y122" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB122" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG122" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI122" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK122" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL122" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM122" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR122" s="3" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 10:39:51,56
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4173D9E-670A-4A4E-96D1-2E8FCF15148C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CA4D90A-DC2D-4552-9785-38FDACD4E296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3734" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3770" uniqueCount="267">
   <si>
     <t>Sel</t>
   </si>
@@ -772,6 +772,12 @@
     <t>1858400002937</t>
   </si>
   <si>
+    <t>1858400002938</t>
+  </si>
+  <si>
+    <t>1858400002939</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -1390,7 +1396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR206"/>
+  <dimension ref="A1:AR208"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -27263,7 +27269,7 @@
         <v>2</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D194" s="3" t="s">
         <v>45</v>
@@ -27275,7 +27281,7 @@
         <v>46156</v>
       </c>
       <c r="G194" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H194" s="3" t="s">
         <v>47</v>
@@ -27290,19 +27296,19 @@
         <v>50</v>
       </c>
       <c r="L194" s="6">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="M194" s="7">
-        <v>26267.89</v>
+        <v>17537.29</v>
       </c>
       <c r="N194" s="6">
         <v>1</v>
       </c>
       <c r="O194" s="3" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="P194" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q194" s="6">
         <v>0</v>
@@ -27317,7 +27323,7 @@
         <v>52</v>
       </c>
       <c r="U194" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V194" s="11">
         <v>11</v>
@@ -27326,7 +27332,7 @@
         <v>46156</v>
       </c>
       <c r="X194" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.44097219999999998</v>
       </c>
       <c r="Y194" s="10">
         <v>0</v>
@@ -27386,7 +27392,7 @@
         <v>53</v>
       </c>
       <c r="AR194" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="195" spans="1:44" x14ac:dyDescent="0.3">
@@ -27397,7 +27403,7 @@
         <v>2</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D195" s="3" t="s">
         <v>45</v>
@@ -27409,7 +27415,7 @@
         <v>46156</v>
       </c>
       <c r="G195" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H195" s="3" t="s">
         <v>47</v>
@@ -27424,19 +27430,19 @@
         <v>50</v>
       </c>
       <c r="L195" s="6">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="M195" s="7">
-        <v>26648.59</v>
+        <v>17986.96</v>
       </c>
       <c r="N195" s="6">
         <v>1</v>
       </c>
       <c r="O195" s="3" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="P195" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q195" s="6">
         <v>0</v>
@@ -27451,7 +27457,7 @@
         <v>52</v>
       </c>
       <c r="U195" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V195" s="11">
         <v>11</v>
@@ -27460,7 +27466,7 @@
         <v>46156</v>
       </c>
       <c r="X195" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.44097219999999998</v>
       </c>
       <c r="Y195" s="10">
         <v>0</v>
@@ -27520,7 +27526,7 @@
         <v>53</v>
       </c>
       <c r="AR195" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="196" spans="1:44" x14ac:dyDescent="0.3">
@@ -27531,7 +27537,7 @@
         <v>2</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D196" s="3" t="s">
         <v>45</v>
@@ -27543,7 +27549,7 @@
         <v>46156</v>
       </c>
       <c r="G196" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H196" s="3" t="s">
         <v>47</v>
@@ -27558,16 +27564,16 @@
         <v>50</v>
       </c>
       <c r="L196" s="6">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M196" s="7">
-        <v>27029.279999999999</v>
+        <v>26267.89</v>
       </c>
       <c r="N196" s="6">
         <v>1</v>
       </c>
       <c r="O196" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P196" s="8">
         <v>380.69</v>
@@ -27665,7 +27671,7 @@
         <v>2</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D197" s="3" t="s">
         <v>45</v>
@@ -27677,7 +27683,7 @@
         <v>46156</v>
       </c>
       <c r="G197" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H197" s="3" t="s">
         <v>47</v>
@@ -27692,16 +27698,16 @@
         <v>50</v>
       </c>
       <c r="L197" s="6">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M197" s="7">
-        <v>27409.98</v>
+        <v>26648.59</v>
       </c>
       <c r="N197" s="6">
         <v>1</v>
       </c>
       <c r="O197" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P197" s="8">
         <v>380.69</v>
@@ -27799,7 +27805,7 @@
         <v>2</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>45</v>
@@ -27811,7 +27817,7 @@
         <v>46156</v>
       </c>
       <c r="G198" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H198" s="3" t="s">
         <v>47</v>
@@ -27826,16 +27832,16 @@
         <v>50</v>
       </c>
       <c r="L198" s="6">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="M198" s="7">
-        <v>27790.67</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N198" s="6">
         <v>1</v>
       </c>
       <c r="O198" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P198" s="8">
         <v>380.69</v>
@@ -27933,7 +27939,7 @@
         <v>2</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D199" s="3" t="s">
         <v>45</v>
@@ -27945,7 +27951,7 @@
         <v>46156</v>
       </c>
       <c r="G199" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H199" s="3" t="s">
         <v>47</v>
@@ -27960,16 +27966,16 @@
         <v>50</v>
       </c>
       <c r="L199" s="6">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M199" s="7">
-        <v>28171.360000000001</v>
+        <v>27409.98</v>
       </c>
       <c r="N199" s="6">
         <v>1</v>
       </c>
       <c r="O199" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P199" s="8">
         <v>380.69</v>
@@ -28067,7 +28073,7 @@
         <v>2</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D200" s="3" t="s">
         <v>45</v>
@@ -28079,7 +28085,7 @@
         <v>46156</v>
       </c>
       <c r="G200" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H200" s="3" t="s">
         <v>47</v>
@@ -28094,16 +28100,16 @@
         <v>50</v>
       </c>
       <c r="L200" s="6">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M200" s="7">
-        <v>28552.06</v>
+        <v>27790.67</v>
       </c>
       <c r="N200" s="6">
         <v>1</v>
       </c>
       <c r="O200" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P200" s="8">
         <v>380.69</v>
@@ -28130,7 +28136,7 @@
         <v>46156</v>
       </c>
       <c r="X200" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y200" s="10">
         <v>0</v>
@@ -28201,7 +28207,7 @@
         <v>2</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D201" s="3" t="s">
         <v>45</v>
@@ -28213,7 +28219,7 @@
         <v>46156</v>
       </c>
       <c r="G201" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H201" s="3" t="s">
         <v>47</v>
@@ -28228,16 +28234,16 @@
         <v>50</v>
       </c>
       <c r="L201" s="6">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M201" s="7">
-        <v>28932.75</v>
+        <v>28171.360000000001</v>
       </c>
       <c r="N201" s="6">
         <v>1</v>
       </c>
       <c r="O201" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P201" s="8">
         <v>380.69</v>
@@ -28264,7 +28270,7 @@
         <v>46156</v>
       </c>
       <c r="X201" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y201" s="10">
         <v>0</v>
@@ -28335,7 +28341,7 @@
         <v>2</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D202" s="3" t="s">
         <v>45</v>
@@ -28347,7 +28353,7 @@
         <v>46156</v>
       </c>
       <c r="G202" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H202" s="3" t="s">
         <v>47</v>
@@ -28362,16 +28368,16 @@
         <v>50</v>
       </c>
       <c r="L202" s="6">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M202" s="7">
-        <v>29313.45</v>
+        <v>28552.06</v>
       </c>
       <c r="N202" s="6">
         <v>1</v>
       </c>
       <c r="O202" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P202" s="8">
         <v>380.69</v>
@@ -28469,7 +28475,7 @@
         <v>2</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D203" s="3" t="s">
         <v>45</v>
@@ -28481,7 +28487,7 @@
         <v>46156</v>
       </c>
       <c r="G203" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H203" s="3" t="s">
         <v>47</v>
@@ -28496,16 +28502,16 @@
         <v>50</v>
       </c>
       <c r="L203" s="6">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="M203" s="7">
-        <v>29694.14</v>
+        <v>28932.75</v>
       </c>
       <c r="N203" s="6">
         <v>1</v>
       </c>
       <c r="O203" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P203" s="8">
         <v>380.69</v>
@@ -28532,7 +28538,7 @@
         <v>46156</v>
       </c>
       <c r="X203" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y203" s="10">
         <v>0</v>
@@ -28603,7 +28609,7 @@
         <v>2</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D204" s="3" t="s">
         <v>45</v>
@@ -28615,7 +28621,7 @@
         <v>46156</v>
       </c>
       <c r="G204" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H204" s="3" t="s">
         <v>47</v>
@@ -28630,16 +28636,16 @@
         <v>50</v>
       </c>
       <c r="L204" s="6">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="M204" s="7">
-        <v>30074.83</v>
+        <v>29313.45</v>
       </c>
       <c r="N204" s="6">
         <v>1</v>
       </c>
       <c r="O204" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P204" s="8">
         <v>380.69</v>
@@ -28666,7 +28672,7 @@
         <v>46156</v>
       </c>
       <c r="X204" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y204" s="10">
         <v>0</v>
@@ -28737,7 +28743,7 @@
         <v>2</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D205" s="3" t="s">
         <v>45</v>
@@ -28749,7 +28755,7 @@
         <v>46156</v>
       </c>
       <c r="G205" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H205" s="3" t="s">
         <v>47</v>
@@ -28764,16 +28770,16 @@
         <v>50</v>
       </c>
       <c r="L205" s="6">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="M205" s="7">
-        <v>30455.53</v>
+        <v>29694.14</v>
       </c>
       <c r="N205" s="6">
         <v>1</v>
       </c>
       <c r="O205" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P205" s="8">
         <v>380.69</v>
@@ -28871,7 +28877,7 @@
         <v>2</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D206" s="3" t="s">
         <v>45</v>
@@ -28883,7 +28889,7 @@
         <v>46156</v>
       </c>
       <c r="G206" s="5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H206" s="3" t="s">
         <v>47</v>
@@ -28898,16 +28904,16 @@
         <v>50</v>
       </c>
       <c r="L206" s="6">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="M206" s="7">
-        <v>30836.22</v>
+        <v>30074.83</v>
       </c>
       <c r="N206" s="6">
         <v>1</v>
       </c>
       <c r="O206" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="P206" s="8">
         <v>380.69</v>
@@ -28934,7 +28940,7 @@
         <v>46156</v>
       </c>
       <c r="X206" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.35972219999999999</v>
       </c>
       <c r="Y206" s="10">
         <v>0</v>
@@ -28995,6 +29001,274 @@
       </c>
       <c r="AR206" s="3" t="s">
         <v>264</v>
+      </c>
+    </row>
+    <row r="207" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A207" s="1">
+        <v>1</v>
+      </c>
+      <c r="B207" s="2">
+        <v>2</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D207" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E207" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F207" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G207" s="5">
+        <v>12</v>
+      </c>
+      <c r="H207" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I207" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J207" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K207" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L207" s="6">
+        <v>80</v>
+      </c>
+      <c r="M207" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N207" s="6">
+        <v>1</v>
+      </c>
+      <c r="O207" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="P207" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q207" s="6">
+        <v>0</v>
+      </c>
+      <c r="R207" s="7">
+        <v>0</v>
+      </c>
+      <c r="S207" s="9">
+        <v>0</v>
+      </c>
+      <c r="T207" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U207" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V207" s="11">
+        <v>11</v>
+      </c>
+      <c r="W207" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X207" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y207" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB207" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG207" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI207" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ207" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK207" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL207" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM207" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ207" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR207" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="208" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A208" s="1">
+        <v>1</v>
+      </c>
+      <c r="B208" s="2">
+        <v>2</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F208" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G208" s="5">
+        <v>13</v>
+      </c>
+      <c r="H208" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I208" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J208" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K208" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L208" s="6">
+        <v>81</v>
+      </c>
+      <c r="M208" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N208" s="6">
+        <v>1</v>
+      </c>
+      <c r="O208" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="P208" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q208" s="6">
+        <v>0</v>
+      </c>
+      <c r="R208" s="7">
+        <v>0</v>
+      </c>
+      <c r="S208" s="9">
+        <v>0</v>
+      </c>
+      <c r="T208" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U208" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V208" s="11">
+        <v>11</v>
+      </c>
+      <c r="W208" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X208" s="12">
+        <v>0.40138889999999999</v>
+      </c>
+      <c r="Y208" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB208" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG208" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI208" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AJ208" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK208" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL208" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM208" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ208" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR208" s="3" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 11:38:47,18
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8ACB123-58A8-444A-A844-F5CDDB004F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{952512EC-3C21-4323-98A1-5ABF5906095E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5318" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5390" uniqueCount="357">
   <si>
     <t>Sel</t>
   </si>
@@ -1036,6 +1036,18 @@
     <t>1858400002943</t>
   </si>
   <si>
+    <t>1858400002944</t>
+  </si>
+  <si>
+    <t>1858400002945</t>
+  </si>
+  <si>
+    <t>1858400002946</t>
+  </si>
+  <si>
+    <t>1858400002947</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -1654,7 +1666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR294"/>
+  <dimension ref="A1:AR298"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -39319,7 +39331,7 @@
         <v>2</v>
       </c>
       <c r="C282" s="3" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="D282" s="3" t="s">
         <v>45</v>
@@ -39331,7 +39343,7 @@
         <v>46156</v>
       </c>
       <c r="G282" s="5">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H282" s="3" t="s">
         <v>47</v>
@@ -39346,19 +39358,19 @@
         <v>50</v>
       </c>
       <c r="L282" s="6">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="M282" s="7">
-        <v>26267.89</v>
+        <v>20235.330000000002</v>
       </c>
       <c r="N282" s="6">
         <v>1</v>
       </c>
       <c r="O282" s="3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="P282" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q282" s="6">
         <v>0</v>
@@ -39373,7 +39385,7 @@
         <v>52</v>
       </c>
       <c r="U282" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V282" s="11">
         <v>11</v>
@@ -39382,7 +39394,7 @@
         <v>46156</v>
       </c>
       <c r="X282" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y282" s="10">
         <v>0</v>
@@ -39442,7 +39454,7 @@
         <v>53</v>
       </c>
       <c r="AR282" s="3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="283" spans="1:44" x14ac:dyDescent="0.3">
@@ -39453,7 +39465,7 @@
         <v>2</v>
       </c>
       <c r="C283" s="3" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="D283" s="3" t="s">
         <v>45</v>
@@ -39465,7 +39477,7 @@
         <v>46156</v>
       </c>
       <c r="G283" s="5">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H283" s="3" t="s">
         <v>47</v>
@@ -39480,19 +39492,19 @@
         <v>50</v>
       </c>
       <c r="L283" s="6">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="M283" s="7">
-        <v>26648.59</v>
+        <v>20685</v>
       </c>
       <c r="N283" s="6">
         <v>1</v>
       </c>
       <c r="O283" s="3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="P283" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q283" s="6">
         <v>0</v>
@@ -39507,7 +39519,7 @@
         <v>52</v>
       </c>
       <c r="U283" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V283" s="11">
         <v>11</v>
@@ -39516,7 +39528,7 @@
         <v>46156</v>
       </c>
       <c r="X283" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y283" s="10">
         <v>0</v>
@@ -39576,7 +39588,7 @@
         <v>53</v>
       </c>
       <c r="AR283" s="3" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="284" spans="1:44" x14ac:dyDescent="0.3">
@@ -39587,7 +39599,7 @@
         <v>2</v>
       </c>
       <c r="C284" s="3" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="D284" s="3" t="s">
         <v>45</v>
@@ -39599,7 +39611,7 @@
         <v>46156</v>
       </c>
       <c r="G284" s="5">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="H284" s="3" t="s">
         <v>47</v>
@@ -39614,19 +39626,19 @@
         <v>50</v>
       </c>
       <c r="L284" s="6">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="M284" s="7">
-        <v>27029.279999999999</v>
+        <v>21134.68</v>
       </c>
       <c r="N284" s="6">
         <v>1</v>
       </c>
       <c r="O284" s="3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="P284" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q284" s="6">
         <v>0</v>
@@ -39641,7 +39653,7 @@
         <v>52</v>
       </c>
       <c r="U284" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V284" s="11">
         <v>11</v>
@@ -39650,7 +39662,7 @@
         <v>46156</v>
       </c>
       <c r="X284" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y284" s="10">
         <v>0</v>
@@ -39710,7 +39722,7 @@
         <v>53</v>
       </c>
       <c r="AR284" s="3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="285" spans="1:44" x14ac:dyDescent="0.3">
@@ -39721,7 +39733,7 @@
         <v>2</v>
       </c>
       <c r="C285" s="3" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="D285" s="3" t="s">
         <v>45</v>
@@ -39733,7 +39745,7 @@
         <v>46156</v>
       </c>
       <c r="G285" s="5">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H285" s="3" t="s">
         <v>47</v>
@@ -39748,19 +39760,19 @@
         <v>50</v>
       </c>
       <c r="L285" s="6">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="M285" s="7">
-        <v>27409.98</v>
+        <v>21584.35</v>
       </c>
       <c r="N285" s="6">
         <v>1</v>
       </c>
       <c r="O285" s="3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="P285" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q285" s="6">
         <v>0</v>
@@ -39775,7 +39787,7 @@
         <v>52</v>
       </c>
       <c r="U285" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V285" s="11">
         <v>11</v>
@@ -39784,7 +39796,7 @@
         <v>46156</v>
       </c>
       <c r="X285" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y285" s="10">
         <v>0</v>
@@ -39844,7 +39856,7 @@
         <v>53</v>
       </c>
       <c r="AR285" s="3" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="286" spans="1:44" x14ac:dyDescent="0.3">
@@ -39855,7 +39867,7 @@
         <v>2</v>
       </c>
       <c r="C286" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D286" s="3" t="s">
         <v>45</v>
@@ -39867,7 +39879,7 @@
         <v>46156</v>
       </c>
       <c r="G286" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H286" s="3" t="s">
         <v>47</v>
@@ -39882,16 +39894,16 @@
         <v>50</v>
       </c>
       <c r="L286" s="6">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M286" s="7">
-        <v>27790.67</v>
+        <v>26267.89</v>
       </c>
       <c r="N286" s="6">
         <v>1</v>
       </c>
       <c r="O286" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P286" s="8">
         <v>380.69</v>
@@ -39989,7 +40001,7 @@
         <v>2</v>
       </c>
       <c r="C287" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D287" s="3" t="s">
         <v>45</v>
@@ -40001,7 +40013,7 @@
         <v>46156</v>
       </c>
       <c r="G287" s="5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H287" s="3" t="s">
         <v>47</v>
@@ -40016,16 +40028,16 @@
         <v>50</v>
       </c>
       <c r="L287" s="6">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="M287" s="7">
-        <v>28171.360000000001</v>
+        <v>26648.59</v>
       </c>
       <c r="N287" s="6">
         <v>1</v>
       </c>
       <c r="O287" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P287" s="8">
         <v>380.69</v>
@@ -40123,7 +40135,7 @@
         <v>2</v>
       </c>
       <c r="C288" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D288" s="3" t="s">
         <v>45</v>
@@ -40135,7 +40147,7 @@
         <v>46156</v>
       </c>
       <c r="G288" s="5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H288" s="3" t="s">
         <v>47</v>
@@ -40150,16 +40162,16 @@
         <v>50</v>
       </c>
       <c r="L288" s="6">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="M288" s="7">
-        <v>28552.06</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N288" s="6">
         <v>1</v>
       </c>
       <c r="O288" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P288" s="8">
         <v>380.69</v>
@@ -40186,7 +40198,7 @@
         <v>46156</v>
       </c>
       <c r="X288" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y288" s="10">
         <v>0</v>
@@ -40257,7 +40269,7 @@
         <v>2</v>
       </c>
       <c r="C289" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D289" s="3" t="s">
         <v>45</v>
@@ -40269,7 +40281,7 @@
         <v>46156</v>
       </c>
       <c r="G289" s="5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H289" s="3" t="s">
         <v>47</v>
@@ -40284,16 +40296,16 @@
         <v>50</v>
       </c>
       <c r="L289" s="6">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="M289" s="7">
-        <v>28932.75</v>
+        <v>27409.98</v>
       </c>
       <c r="N289" s="6">
         <v>1</v>
       </c>
       <c r="O289" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P289" s="8">
         <v>380.69</v>
@@ -40320,7 +40332,7 @@
         <v>46156</v>
       </c>
       <c r="X289" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y289" s="10">
         <v>0</v>
@@ -40391,7 +40403,7 @@
         <v>2</v>
       </c>
       <c r="C290" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D290" s="3" t="s">
         <v>45</v>
@@ -40403,7 +40415,7 @@
         <v>46156</v>
       </c>
       <c r="G290" s="5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H290" s="3" t="s">
         <v>47</v>
@@ -40418,16 +40430,16 @@
         <v>50</v>
       </c>
       <c r="L290" s="6">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M290" s="7">
-        <v>29313.45</v>
+        <v>27790.67</v>
       </c>
       <c r="N290" s="6">
         <v>1</v>
       </c>
       <c r="O290" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P290" s="8">
         <v>380.69</v>
@@ -40454,7 +40466,7 @@
         <v>46156</v>
       </c>
       <c r="X290" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y290" s="10">
         <v>0</v>
@@ -40525,7 +40537,7 @@
         <v>2</v>
       </c>
       <c r="C291" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D291" s="3" t="s">
         <v>45</v>
@@ -40537,7 +40549,7 @@
         <v>46156</v>
       </c>
       <c r="G291" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H291" s="3" t="s">
         <v>47</v>
@@ -40552,16 +40564,16 @@
         <v>50</v>
       </c>
       <c r="L291" s="6">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="M291" s="7">
-        <v>29694.14</v>
+        <v>28171.360000000001</v>
       </c>
       <c r="N291" s="6">
         <v>1</v>
       </c>
       <c r="O291" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P291" s="8">
         <v>380.69</v>
@@ -40588,7 +40600,7 @@
         <v>46156</v>
       </c>
       <c r="X291" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y291" s="10">
         <v>0</v>
@@ -40659,7 +40671,7 @@
         <v>2</v>
       </c>
       <c r="C292" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D292" s="3" t="s">
         <v>45</v>
@@ -40671,7 +40683,7 @@
         <v>46156</v>
       </c>
       <c r="G292" s="5">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H292" s="3" t="s">
         <v>47</v>
@@ -40686,16 +40698,16 @@
         <v>50</v>
       </c>
       <c r="L292" s="6">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="M292" s="7">
-        <v>30074.83</v>
+        <v>28552.06</v>
       </c>
       <c r="N292" s="6">
         <v>1</v>
       </c>
       <c r="O292" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P292" s="8">
         <v>380.69</v>
@@ -40722,7 +40734,7 @@
         <v>46156</v>
       </c>
       <c r="X292" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y292" s="10">
         <v>0</v>
@@ -40793,7 +40805,7 @@
         <v>2</v>
       </c>
       <c r="C293" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D293" s="3" t="s">
         <v>45</v>
@@ -40805,7 +40817,7 @@
         <v>46156</v>
       </c>
       <c r="G293" s="5">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H293" s="3" t="s">
         <v>47</v>
@@ -40820,16 +40832,16 @@
         <v>50</v>
       </c>
       <c r="L293" s="6">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="M293" s="7">
-        <v>30455.53</v>
+        <v>28932.75</v>
       </c>
       <c r="N293" s="6">
         <v>1</v>
       </c>
       <c r="O293" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P293" s="8">
         <v>380.69</v>
@@ -40856,7 +40868,7 @@
         <v>46156</v>
       </c>
       <c r="X293" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y293" s="10">
         <v>0</v>
@@ -40927,7 +40939,7 @@
         <v>2</v>
       </c>
       <c r="C294" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D294" s="3" t="s">
         <v>45</v>
@@ -40939,7 +40951,7 @@
         <v>46156</v>
       </c>
       <c r="G294" s="5">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H294" s="3" t="s">
         <v>47</v>
@@ -40954,16 +40966,16 @@
         <v>50</v>
       </c>
       <c r="L294" s="6">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="M294" s="7">
-        <v>30836.22</v>
+        <v>29313.45</v>
       </c>
       <c r="N294" s="6">
         <v>1</v>
       </c>
       <c r="O294" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="P294" s="8">
         <v>380.69</v>
@@ -40990,7 +41002,7 @@
         <v>46156</v>
       </c>
       <c r="X294" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y294" s="10">
         <v>0</v>
@@ -41051,6 +41063,542 @@
       </c>
       <c r="AR294" s="3" t="s">
         <v>352</v>
+      </c>
+    </row>
+    <row r="295" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A295" s="1">
+        <v>1</v>
+      </c>
+      <c r="B295" s="2">
+        <v>2</v>
+      </c>
+      <c r="C295" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E295" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F295" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G295" s="5">
+        <v>10</v>
+      </c>
+      <c r="H295" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I295" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J295" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K295" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L295" s="6">
+        <v>78</v>
+      </c>
+      <c r="M295" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N295" s="6">
+        <v>1</v>
+      </c>
+      <c r="O295" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="P295" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q295" s="6">
+        <v>0</v>
+      </c>
+      <c r="R295" s="7">
+        <v>0</v>
+      </c>
+      <c r="S295" s="9">
+        <v>0</v>
+      </c>
+      <c r="T295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U295" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V295" s="11">
+        <v>11</v>
+      </c>
+      <c r="W295" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X295" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y295" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB295" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG295" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI295" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="AJ295" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL295" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM295" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ295" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR295" s="3" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="296" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A296" s="1">
+        <v>1</v>
+      </c>
+      <c r="B296" s="2">
+        <v>2</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F296" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G296" s="5">
+        <v>11</v>
+      </c>
+      <c r="H296" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I296" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J296" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K296" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L296" s="6">
+        <v>79</v>
+      </c>
+      <c r="M296" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N296" s="6">
+        <v>1</v>
+      </c>
+      <c r="O296" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="P296" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q296" s="6">
+        <v>0</v>
+      </c>
+      <c r="R296" s="7">
+        <v>0</v>
+      </c>
+      <c r="S296" s="9">
+        <v>0</v>
+      </c>
+      <c r="T296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U296" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V296" s="11">
+        <v>11</v>
+      </c>
+      <c r="W296" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X296" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y296" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB296" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG296" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI296" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="AJ296" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL296" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM296" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ296" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR296" s="3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="297" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A297" s="1">
+        <v>1</v>
+      </c>
+      <c r="B297" s="2">
+        <v>2</v>
+      </c>
+      <c r="C297" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E297" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F297" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G297" s="5">
+        <v>12</v>
+      </c>
+      <c r="H297" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I297" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J297" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K297" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L297" s="6">
+        <v>80</v>
+      </c>
+      <c r="M297" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N297" s="6">
+        <v>1</v>
+      </c>
+      <c r="O297" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="P297" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q297" s="6">
+        <v>0</v>
+      </c>
+      <c r="R297" s="7">
+        <v>0</v>
+      </c>
+      <c r="S297" s="9">
+        <v>0</v>
+      </c>
+      <c r="T297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U297" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V297" s="11">
+        <v>11</v>
+      </c>
+      <c r="W297" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X297" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y297" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB297" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG297" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI297" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="AJ297" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL297" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM297" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ297" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR297" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="298" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A298" s="1">
+        <v>1</v>
+      </c>
+      <c r="B298" s="2">
+        <v>2</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F298" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G298" s="5">
+        <v>13</v>
+      </c>
+      <c r="H298" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I298" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J298" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K298" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L298" s="6">
+        <v>81</v>
+      </c>
+      <c r="M298" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N298" s="6">
+        <v>1</v>
+      </c>
+      <c r="O298" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="P298" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q298" s="6">
+        <v>0</v>
+      </c>
+      <c r="R298" s="7">
+        <v>0</v>
+      </c>
+      <c r="S298" s="9">
+        <v>0</v>
+      </c>
+      <c r="T298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U298" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V298" s="11">
+        <v>11</v>
+      </c>
+      <c r="W298" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X298" s="12">
+        <v>0.40138889999999999</v>
+      </c>
+      <c r="Y298" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB298" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG298" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI298" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="AJ298" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL298" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM298" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ298" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR298" s="3" t="s">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 13:18:33,25
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80AEEEF9-F277-44C6-AD9D-B64F3DF3BE57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADE07338-81D0-45E5-9117-B3CB0972D0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6434" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6686" uniqueCount="429">
   <si>
     <t>Sel</t>
   </si>
@@ -1177,6 +1177,36 @@
     <t>1854300115030</t>
   </si>
   <si>
+    <t>1854300115031</t>
+  </si>
+  <si>
+    <t>1854300115032</t>
+  </si>
+  <si>
+    <t>1854300115033</t>
+  </si>
+  <si>
+    <t>1854300115034</t>
+  </si>
+  <si>
+    <t>1854300115035</t>
+  </si>
+  <si>
+    <t>1854300115036</t>
+  </si>
+  <si>
+    <t>1854300115037</t>
+  </si>
+  <si>
+    <t>1854300115038</t>
+  </si>
+  <si>
+    <t>1854300115039</t>
+  </si>
+  <si>
+    <t>1854300115040</t>
+  </si>
+  <si>
     <t>10016351</t>
   </si>
   <si>
@@ -1220,6 +1250,18 @@
   </si>
   <si>
     <t>1858400002947</t>
+  </si>
+  <si>
+    <t>1858400002948</t>
+  </si>
+  <si>
+    <t>1858400002949</t>
+  </si>
+  <si>
+    <t>1858400002950</t>
+  </si>
+  <si>
+    <t>1858400002951</t>
   </si>
   <si>
     <t>10018965</t>
@@ -1840,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR356"/>
+  <dimension ref="A1:AR370"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -46205,7 +46247,7 @@
         <v>2</v>
       </c>
       <c r="C332" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D332" s="3" t="s">
         <v>45</v>
@@ -46217,7 +46259,7 @@
         <v>46156</v>
       </c>
       <c r="G332" s="5">
-        <v>1</v>
+        <v>378</v>
       </c>
       <c r="H332" s="3" t="s">
         <v>47</v>
@@ -46232,19 +46274,19 @@
         <v>50</v>
       </c>
       <c r="L332" s="6">
-        <v>37</v>
+        <v>595</v>
       </c>
       <c r="M332" s="7">
-        <v>16637.939999999999</v>
+        <v>117595.35</v>
       </c>
       <c r="N332" s="6">
         <v>1</v>
       </c>
       <c r="O332" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P332" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q332" s="6">
         <v>0</v>
@@ -46259,7 +46301,7 @@
         <v>52</v>
       </c>
       <c r="U332" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V332" s="11">
         <v>11</v>
@@ -46268,7 +46310,7 @@
         <v>46156</v>
       </c>
       <c r="X332" s="12">
-        <v>0.37847219999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y332" s="10">
         <v>0</v>
@@ -46301,7 +46343,7 @@
         <v>53</v>
       </c>
       <c r="AI332" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ332" s="3" t="s">
         <v>52</v>
@@ -46328,7 +46370,7 @@
         <v>53</v>
       </c>
       <c r="AR332" s="3" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="333" spans="1:44" x14ac:dyDescent="0.3">
@@ -46339,7 +46381,7 @@
         <v>2</v>
       </c>
       <c r="C333" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D333" s="3" t="s">
         <v>45</v>
@@ -46351,7 +46393,7 @@
         <v>46156</v>
       </c>
       <c r="G333" s="5">
-        <v>2</v>
+        <v>379</v>
       </c>
       <c r="H333" s="3" t="s">
         <v>47</v>
@@ -46366,19 +46408,19 @@
         <v>50</v>
       </c>
       <c r="L333" s="6">
-        <v>38</v>
+        <v>596</v>
       </c>
       <c r="M333" s="7">
-        <v>17087.61</v>
+        <v>117792.99</v>
       </c>
       <c r="N333" s="6">
         <v>1</v>
       </c>
       <c r="O333" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P333" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q333" s="6">
         <v>0</v>
@@ -46393,7 +46435,7 @@
         <v>52</v>
       </c>
       <c r="U333" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V333" s="11">
         <v>11</v>
@@ -46402,7 +46444,7 @@
         <v>46156</v>
       </c>
       <c r="X333" s="12">
-        <v>0.42013889999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y333" s="10">
         <v>0</v>
@@ -46435,7 +46477,7 @@
         <v>53</v>
       </c>
       <c r="AI333" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ333" s="3" t="s">
         <v>52</v>
@@ -46462,7 +46504,7 @@
         <v>53</v>
       </c>
       <c r="AR333" s="3" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="334" spans="1:44" x14ac:dyDescent="0.3">
@@ -46473,7 +46515,7 @@
         <v>2</v>
       </c>
       <c r="C334" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D334" s="3" t="s">
         <v>45</v>
@@ -46485,7 +46527,7 @@
         <v>46156</v>
       </c>
       <c r="G334" s="5">
-        <v>3</v>
+        <v>380</v>
       </c>
       <c r="H334" s="3" t="s">
         <v>47</v>
@@ -46500,19 +46542,19 @@
         <v>50</v>
       </c>
       <c r="L334" s="6">
-        <v>39</v>
+        <v>597</v>
       </c>
       <c r="M334" s="7">
-        <v>17537.29</v>
+        <v>117990.63</v>
       </c>
       <c r="N334" s="6">
         <v>1</v>
       </c>
       <c r="O334" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P334" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q334" s="6">
         <v>0</v>
@@ -46527,7 +46569,7 @@
         <v>52</v>
       </c>
       <c r="U334" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V334" s="11">
         <v>11</v>
@@ -46536,7 +46578,7 @@
         <v>46156</v>
       </c>
       <c r="X334" s="12">
-        <v>0.44097219999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y334" s="10">
         <v>0</v>
@@ -46569,34 +46611,34 @@
         <v>53</v>
       </c>
       <c r="AI334" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ334" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK334" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL334" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM334" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ334" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR334" s="3" t="s">
         <v>387</v>
-      </c>
-      <c r="AJ334" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK334" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL334" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM334" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN334" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO334" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP334" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ334" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR334" s="3" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="335" spans="1:44" x14ac:dyDescent="0.3">
@@ -46607,7 +46649,7 @@
         <v>2</v>
       </c>
       <c r="C335" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D335" s="3" t="s">
         <v>45</v>
@@ -46619,7 +46661,7 @@
         <v>46156</v>
       </c>
       <c r="G335" s="5">
-        <v>4</v>
+        <v>381</v>
       </c>
       <c r="H335" s="3" t="s">
         <v>47</v>
@@ -46634,19 +46676,19 @@
         <v>50</v>
       </c>
       <c r="L335" s="6">
-        <v>40</v>
+        <v>598</v>
       </c>
       <c r="M335" s="7">
-        <v>17986.96</v>
+        <v>118188.27</v>
       </c>
       <c r="N335" s="6">
         <v>1</v>
       </c>
       <c r="O335" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P335" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q335" s="6">
         <v>0</v>
@@ -46661,7 +46703,7 @@
         <v>52</v>
       </c>
       <c r="U335" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V335" s="11">
         <v>11</v>
@@ -46670,7 +46712,7 @@
         <v>46156</v>
       </c>
       <c r="X335" s="12">
-        <v>0.44097219999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y335" s="10">
         <v>0</v>
@@ -46703,7 +46745,7 @@
         <v>53</v>
       </c>
       <c r="AI335" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ335" s="3" t="s">
         <v>52</v>
@@ -46730,7 +46772,7 @@
         <v>53</v>
       </c>
       <c r="AR335" s="3" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="336" spans="1:44" x14ac:dyDescent="0.3">
@@ -46741,7 +46783,7 @@
         <v>2</v>
       </c>
       <c r="C336" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D336" s="3" t="s">
         <v>45</v>
@@ -46753,7 +46795,7 @@
         <v>46156</v>
       </c>
       <c r="G336" s="5">
-        <v>5</v>
+        <v>382</v>
       </c>
       <c r="H336" s="3" t="s">
         <v>47</v>
@@ -46768,19 +46810,19 @@
         <v>50</v>
       </c>
       <c r="L336" s="6">
-        <v>41</v>
+        <v>599</v>
       </c>
       <c r="M336" s="7">
-        <v>18436.63</v>
+        <v>118385.91</v>
       </c>
       <c r="N336" s="6">
         <v>1</v>
       </c>
       <c r="O336" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P336" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q336" s="6">
         <v>0</v>
@@ -46795,7 +46837,7 @@
         <v>52</v>
       </c>
       <c r="U336" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V336" s="11">
         <v>11</v>
@@ -46804,7 +46846,7 @@
         <v>46156</v>
       </c>
       <c r="X336" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y336" s="10">
         <v>0</v>
@@ -46837,7 +46879,7 @@
         <v>53</v>
       </c>
       <c r="AI336" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ336" s="3" t="s">
         <v>52</v>
@@ -46864,7 +46906,7 @@
         <v>53</v>
       </c>
       <c r="AR336" s="3" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="337" spans="1:44" x14ac:dyDescent="0.3">
@@ -46875,7 +46917,7 @@
         <v>2</v>
       </c>
       <c r="C337" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D337" s="3" t="s">
         <v>45</v>
@@ -46887,7 +46929,7 @@
         <v>46156</v>
       </c>
       <c r="G337" s="5">
-        <v>6</v>
+        <v>383</v>
       </c>
       <c r="H337" s="3" t="s">
         <v>47</v>
@@ -46902,19 +46944,19 @@
         <v>50</v>
       </c>
       <c r="L337" s="6">
-        <v>42</v>
+        <v>600</v>
       </c>
       <c r="M337" s="7">
-        <v>18886.310000000001</v>
+        <v>118583.55</v>
       </c>
       <c r="N337" s="6">
         <v>1</v>
       </c>
       <c r="O337" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P337" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q337" s="6">
         <v>0</v>
@@ -46929,7 +46971,7 @@
         <v>52</v>
       </c>
       <c r="U337" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V337" s="11">
         <v>11</v>
@@ -46938,7 +46980,7 @@
         <v>46156</v>
       </c>
       <c r="X337" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y337" s="10">
         <v>0</v>
@@ -46971,7 +47013,7 @@
         <v>53</v>
       </c>
       <c r="AI337" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ337" s="3" t="s">
         <v>52</v>
@@ -46998,7 +47040,7 @@
         <v>53</v>
       </c>
       <c r="AR337" s="3" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="338" spans="1:44" x14ac:dyDescent="0.3">
@@ -47009,7 +47051,7 @@
         <v>2</v>
       </c>
       <c r="C338" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D338" s="3" t="s">
         <v>45</v>
@@ -47021,7 +47063,7 @@
         <v>46156</v>
       </c>
       <c r="G338" s="5">
-        <v>7</v>
+        <v>384</v>
       </c>
       <c r="H338" s="3" t="s">
         <v>47</v>
@@ -47036,19 +47078,19 @@
         <v>50</v>
       </c>
       <c r="L338" s="6">
-        <v>43</v>
+        <v>601</v>
       </c>
       <c r="M338" s="7">
-        <v>19335.98</v>
+        <v>118781.19</v>
       </c>
       <c r="N338" s="6">
         <v>1</v>
       </c>
       <c r="O338" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P338" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q338" s="6">
         <v>0</v>
@@ -47063,7 +47105,7 @@
         <v>52</v>
       </c>
       <c r="U338" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V338" s="11">
         <v>11</v>
@@ -47072,7 +47114,7 @@
         <v>46156</v>
       </c>
       <c r="X338" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y338" s="10">
         <v>0</v>
@@ -47105,7 +47147,7 @@
         <v>53</v>
       </c>
       <c r="AI338" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ338" s="3" t="s">
         <v>52</v>
@@ -47132,7 +47174,7 @@
         <v>53</v>
       </c>
       <c r="AR338" s="3" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="339" spans="1:44" x14ac:dyDescent="0.3">
@@ -47143,7 +47185,7 @@
         <v>2</v>
       </c>
       <c r="C339" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D339" s="3" t="s">
         <v>45</v>
@@ -47155,7 +47197,7 @@
         <v>46156</v>
       </c>
       <c r="G339" s="5">
-        <v>8</v>
+        <v>385</v>
       </c>
       <c r="H339" s="3" t="s">
         <v>47</v>
@@ -47170,19 +47212,19 @@
         <v>50</v>
       </c>
       <c r="L339" s="6">
-        <v>44</v>
+        <v>602</v>
       </c>
       <c r="M339" s="7">
-        <v>19785.66</v>
+        <v>118978.83</v>
       </c>
       <c r="N339" s="6">
         <v>1</v>
       </c>
       <c r="O339" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P339" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q339" s="6">
         <v>0</v>
@@ -47197,7 +47239,7 @@
         <v>52</v>
       </c>
       <c r="U339" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V339" s="11">
         <v>11</v>
@@ -47206,7 +47248,7 @@
         <v>46156</v>
       </c>
       <c r="X339" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y339" s="10">
         <v>0</v>
@@ -47239,7 +47281,7 @@
         <v>53</v>
       </c>
       <c r="AI339" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ339" s="3" t="s">
         <v>52</v>
@@ -47266,7 +47308,7 @@
         <v>53</v>
       </c>
       <c r="AR339" s="3" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="340" spans="1:44" x14ac:dyDescent="0.3">
@@ -47277,7 +47319,7 @@
         <v>2</v>
       </c>
       <c r="C340" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D340" s="3" t="s">
         <v>45</v>
@@ -47289,7 +47331,7 @@
         <v>46156</v>
       </c>
       <c r="G340" s="5">
-        <v>9</v>
+        <v>386</v>
       </c>
       <c r="H340" s="3" t="s">
         <v>47</v>
@@ -47304,19 +47346,19 @@
         <v>50</v>
       </c>
       <c r="L340" s="6">
-        <v>45</v>
+        <v>603</v>
       </c>
       <c r="M340" s="7">
-        <v>20235.330000000002</v>
+        <v>119176.46</v>
       </c>
       <c r="N340" s="6">
         <v>1</v>
       </c>
       <c r="O340" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P340" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q340" s="6">
         <v>0</v>
@@ -47331,7 +47373,7 @@
         <v>52</v>
       </c>
       <c r="U340" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V340" s="11">
         <v>11</v>
@@ -47340,7 +47382,7 @@
         <v>46156</v>
       </c>
       <c r="X340" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y340" s="10">
         <v>0</v>
@@ -47373,7 +47415,7 @@
         <v>53</v>
       </c>
       <c r="AI340" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ340" s="3" t="s">
         <v>52</v>
@@ -47400,7 +47442,7 @@
         <v>53</v>
       </c>
       <c r="AR340" s="3" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="341" spans="1:44" x14ac:dyDescent="0.3">
@@ -47411,7 +47453,7 @@
         <v>2</v>
       </c>
       <c r="C341" s="3" t="s">
-        <v>385</v>
+        <v>44</v>
       </c>
       <c r="D341" s="3" t="s">
         <v>45</v>
@@ -47423,7 +47465,7 @@
         <v>46156</v>
       </c>
       <c r="G341" s="5">
-        <v>10</v>
+        <v>387</v>
       </c>
       <c r="H341" s="3" t="s">
         <v>47</v>
@@ -47438,19 +47480,19 @@
         <v>50</v>
       </c>
       <c r="L341" s="6">
-        <v>46</v>
+        <v>604</v>
       </c>
       <c r="M341" s="7">
-        <v>20685</v>
+        <v>119374.1</v>
       </c>
       <c r="N341" s="6">
         <v>1</v>
       </c>
       <c r="O341" s="3" t="s">
-        <v>386</v>
+        <v>51</v>
       </c>
       <c r="P341" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q341" s="6">
         <v>0</v>
@@ -47465,7 +47507,7 @@
         <v>52</v>
       </c>
       <c r="U341" s="10">
-        <v>64218</v>
+        <v>64301</v>
       </c>
       <c r="V341" s="11">
         <v>11</v>
@@ -47474,7 +47516,7 @@
         <v>46156</v>
       </c>
       <c r="X341" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.54652780000000001</v>
       </c>
       <c r="Y341" s="10">
         <v>0</v>
@@ -47507,7 +47549,7 @@
         <v>53</v>
       </c>
       <c r="AI341" s="3" t="s">
-        <v>387</v>
+        <v>54</v>
       </c>
       <c r="AJ341" s="3" t="s">
         <v>52</v>
@@ -47534,7 +47576,7 @@
         <v>53</v>
       </c>
       <c r="AR341" s="3" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="342" spans="1:44" x14ac:dyDescent="0.3">
@@ -47545,7 +47587,7 @@
         <v>2</v>
       </c>
       <c r="C342" s="3" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="D342" s="3" t="s">
         <v>45</v>
@@ -47557,7 +47599,7 @@
         <v>46156</v>
       </c>
       <c r="G342" s="5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H342" s="3" t="s">
         <v>47</v>
@@ -47572,16 +47614,16 @@
         <v>50</v>
       </c>
       <c r="L342" s="6">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M342" s="7">
-        <v>21134.68</v>
+        <v>16637.939999999999</v>
       </c>
       <c r="N342" s="6">
         <v>1</v>
       </c>
       <c r="O342" s="3" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
       <c r="P342" s="8">
         <v>449.67</v>
@@ -47608,7 +47650,7 @@
         <v>46156</v>
       </c>
       <c r="X342" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.37847219999999998</v>
       </c>
       <c r="Y342" s="10">
         <v>0</v>
@@ -47641,7 +47683,7 @@
         <v>53</v>
       </c>
       <c r="AI342" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ342" s="3" t="s">
         <v>52</v>
@@ -47679,7 +47721,7 @@
         <v>2</v>
       </c>
       <c r="C343" s="3" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="D343" s="3" t="s">
         <v>45</v>
@@ -47691,7 +47733,7 @@
         <v>46156</v>
       </c>
       <c r="G343" s="5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H343" s="3" t="s">
         <v>47</v>
@@ -47706,16 +47748,16 @@
         <v>50</v>
       </c>
       <c r="L343" s="6">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="M343" s="7">
-        <v>21584.35</v>
+        <v>17087.61</v>
       </c>
       <c r="N343" s="6">
         <v>1</v>
       </c>
       <c r="O343" s="3" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
       <c r="P343" s="8">
         <v>449.67</v>
@@ -47742,7 +47784,7 @@
         <v>46156</v>
       </c>
       <c r="X343" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y343" s="10">
         <v>0</v>
@@ -47775,7 +47817,7 @@
         <v>53</v>
       </c>
       <c r="AI343" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ343" s="3" t="s">
         <v>52</v>
@@ -47813,7 +47855,7 @@
         <v>2</v>
       </c>
       <c r="C344" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D344" s="3" t="s">
         <v>45</v>
@@ -47825,7 +47867,7 @@
         <v>46156</v>
       </c>
       <c r="G344" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H344" s="3" t="s">
         <v>47</v>
@@ -47840,19 +47882,19 @@
         <v>50</v>
       </c>
       <c r="L344" s="6">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="M344" s="7">
-        <v>26267.89</v>
+        <v>17537.29</v>
       </c>
       <c r="N344" s="6">
         <v>1</v>
       </c>
       <c r="O344" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P344" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q344" s="6">
         <v>0</v>
@@ -47867,7 +47909,7 @@
         <v>52</v>
       </c>
       <c r="U344" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V344" s="11">
         <v>11</v>
@@ -47876,7 +47918,7 @@
         <v>46156</v>
       </c>
       <c r="X344" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.44097219999999998</v>
       </c>
       <c r="Y344" s="10">
         <v>0</v>
@@ -47909,7 +47951,7 @@
         <v>53</v>
       </c>
       <c r="AI344" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ344" s="3" t="s">
         <v>52</v>
@@ -47936,7 +47978,7 @@
         <v>53</v>
       </c>
       <c r="AR344" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="345" spans="1:44" x14ac:dyDescent="0.3">
@@ -47947,7 +47989,7 @@
         <v>2</v>
       </c>
       <c r="C345" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D345" s="3" t="s">
         <v>45</v>
@@ -47959,7 +48001,7 @@
         <v>46156</v>
       </c>
       <c r="G345" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H345" s="3" t="s">
         <v>47</v>
@@ -47974,19 +48016,19 @@
         <v>50</v>
       </c>
       <c r="L345" s="6">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="M345" s="7">
-        <v>26648.59</v>
+        <v>17986.96</v>
       </c>
       <c r="N345" s="6">
         <v>1</v>
       </c>
       <c r="O345" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P345" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q345" s="6">
         <v>0</v>
@@ -48001,7 +48043,7 @@
         <v>52</v>
       </c>
       <c r="U345" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V345" s="11">
         <v>11</v>
@@ -48010,7 +48052,7 @@
         <v>46156</v>
       </c>
       <c r="X345" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.44097219999999998</v>
       </c>
       <c r="Y345" s="10">
         <v>0</v>
@@ -48043,7 +48085,7 @@
         <v>53</v>
       </c>
       <c r="AI345" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ345" s="3" t="s">
         <v>52</v>
@@ -48070,7 +48112,7 @@
         <v>53</v>
       </c>
       <c r="AR345" s="3" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="346" spans="1:44" x14ac:dyDescent="0.3">
@@ -48081,7 +48123,7 @@
         <v>2</v>
       </c>
       <c r="C346" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D346" s="3" t="s">
         <v>45</v>
@@ -48093,7 +48135,7 @@
         <v>46156</v>
       </c>
       <c r="G346" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H346" s="3" t="s">
         <v>47</v>
@@ -48108,19 +48150,19 @@
         <v>50</v>
       </c>
       <c r="L346" s="6">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="M346" s="7">
-        <v>27029.279999999999</v>
+        <v>18436.63</v>
       </c>
       <c r="N346" s="6">
         <v>1</v>
       </c>
       <c r="O346" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P346" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q346" s="6">
         <v>0</v>
@@ -48135,7 +48177,7 @@
         <v>52</v>
       </c>
       <c r="U346" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V346" s="11">
         <v>11</v>
@@ -48144,7 +48186,7 @@
         <v>46156</v>
       </c>
       <c r="X346" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y346" s="10">
         <v>0</v>
@@ -48177,7 +48219,7 @@
         <v>53</v>
       </c>
       <c r="AI346" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ346" s="3" t="s">
         <v>52</v>
@@ -48204,7 +48246,7 @@
         <v>53</v>
       </c>
       <c r="AR346" s="3" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="347" spans="1:44" x14ac:dyDescent="0.3">
@@ -48215,7 +48257,7 @@
         <v>2</v>
       </c>
       <c r="C347" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D347" s="3" t="s">
         <v>45</v>
@@ -48227,7 +48269,7 @@
         <v>46156</v>
       </c>
       <c r="G347" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H347" s="3" t="s">
         <v>47</v>
@@ -48242,19 +48284,19 @@
         <v>50</v>
       </c>
       <c r="L347" s="6">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="M347" s="7">
-        <v>27409.98</v>
+        <v>18886.310000000001</v>
       </c>
       <c r="N347" s="6">
         <v>1</v>
       </c>
       <c r="O347" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P347" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q347" s="6">
         <v>0</v>
@@ -48269,7 +48311,7 @@
         <v>52</v>
       </c>
       <c r="U347" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V347" s="11">
         <v>11</v>
@@ -48278,7 +48320,7 @@
         <v>46156</v>
       </c>
       <c r="X347" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y347" s="10">
         <v>0</v>
@@ -48311,7 +48353,7 @@
         <v>53</v>
       </c>
       <c r="AI347" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ347" s="3" t="s">
         <v>52</v>
@@ -48338,7 +48380,7 @@
         <v>53</v>
       </c>
       <c r="AR347" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="348" spans="1:44" x14ac:dyDescent="0.3">
@@ -48349,7 +48391,7 @@
         <v>2</v>
       </c>
       <c r="C348" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D348" s="3" t="s">
         <v>45</v>
@@ -48361,7 +48403,7 @@
         <v>46156</v>
       </c>
       <c r="G348" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H348" s="3" t="s">
         <v>47</v>
@@ -48376,19 +48418,19 @@
         <v>50</v>
       </c>
       <c r="L348" s="6">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="M348" s="7">
-        <v>27790.67</v>
+        <v>19335.98</v>
       </c>
       <c r="N348" s="6">
         <v>1</v>
       </c>
       <c r="O348" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P348" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q348" s="6">
         <v>0</v>
@@ -48403,7 +48445,7 @@
         <v>52</v>
       </c>
       <c r="U348" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V348" s="11">
         <v>11</v>
@@ -48412,7 +48454,7 @@
         <v>46156</v>
       </c>
       <c r="X348" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y348" s="10">
         <v>0</v>
@@ -48445,7 +48487,7 @@
         <v>53</v>
       </c>
       <c r="AI348" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ348" s="3" t="s">
         <v>52</v>
@@ -48472,7 +48514,7 @@
         <v>53</v>
       </c>
       <c r="AR348" s="3" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="349" spans="1:44" x14ac:dyDescent="0.3">
@@ -48483,7 +48525,7 @@
         <v>2</v>
       </c>
       <c r="C349" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D349" s="3" t="s">
         <v>45</v>
@@ -48495,7 +48537,7 @@
         <v>46156</v>
       </c>
       <c r="G349" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H349" s="3" t="s">
         <v>47</v>
@@ -48510,19 +48552,19 @@
         <v>50</v>
       </c>
       <c r="L349" s="6">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="M349" s="7">
-        <v>28171.360000000001</v>
+        <v>19785.66</v>
       </c>
       <c r="N349" s="6">
         <v>1</v>
       </c>
       <c r="O349" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P349" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q349" s="6">
         <v>0</v>
@@ -48537,7 +48579,7 @@
         <v>52</v>
       </c>
       <c r="U349" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V349" s="11">
         <v>11</v>
@@ -48546,7 +48588,7 @@
         <v>46156</v>
       </c>
       <c r="X349" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y349" s="10">
         <v>0</v>
@@ -48579,7 +48621,7 @@
         <v>53</v>
       </c>
       <c r="AI349" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ349" s="3" t="s">
         <v>52</v>
@@ -48606,7 +48648,7 @@
         <v>53</v>
       </c>
       <c r="AR349" s="3" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="350" spans="1:44" x14ac:dyDescent="0.3">
@@ -48617,7 +48659,7 @@
         <v>2</v>
       </c>
       <c r="C350" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D350" s="3" t="s">
         <v>45</v>
@@ -48629,7 +48671,7 @@
         <v>46156</v>
       </c>
       <c r="G350" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H350" s="3" t="s">
         <v>47</v>
@@ -48644,19 +48686,19 @@
         <v>50</v>
       </c>
       <c r="L350" s="6">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="M350" s="7">
-        <v>28552.06</v>
+        <v>20235.330000000002</v>
       </c>
       <c r="N350" s="6">
         <v>1</v>
       </c>
       <c r="O350" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P350" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q350" s="6">
         <v>0</v>
@@ -48671,7 +48713,7 @@
         <v>52</v>
       </c>
       <c r="U350" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V350" s="11">
         <v>11</v>
@@ -48680,7 +48722,7 @@
         <v>46156</v>
       </c>
       <c r="X350" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y350" s="10">
         <v>0</v>
@@ -48713,7 +48755,7 @@
         <v>53</v>
       </c>
       <c r="AI350" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ350" s="3" t="s">
         <v>52</v>
@@ -48740,7 +48782,7 @@
         <v>53</v>
       </c>
       <c r="AR350" s="3" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="351" spans="1:44" x14ac:dyDescent="0.3">
@@ -48751,7 +48793,7 @@
         <v>2</v>
       </c>
       <c r="C351" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D351" s="3" t="s">
         <v>45</v>
@@ -48763,7 +48805,7 @@
         <v>46156</v>
       </c>
       <c r="G351" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H351" s="3" t="s">
         <v>47</v>
@@ -48778,19 +48820,19 @@
         <v>50</v>
       </c>
       <c r="L351" s="6">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="M351" s="7">
-        <v>28932.75</v>
+        <v>20685</v>
       </c>
       <c r="N351" s="6">
         <v>1</v>
       </c>
       <c r="O351" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P351" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q351" s="6">
         <v>0</v>
@@ -48805,7 +48847,7 @@
         <v>52</v>
       </c>
       <c r="U351" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V351" s="11">
         <v>11</v>
@@ -48814,7 +48856,7 @@
         <v>46156</v>
       </c>
       <c r="X351" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y351" s="10">
         <v>0</v>
@@ -48847,7 +48889,7 @@
         <v>53</v>
       </c>
       <c r="AI351" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ351" s="3" t="s">
         <v>52</v>
@@ -48874,7 +48916,7 @@
         <v>53</v>
       </c>
       <c r="AR351" s="3" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="352" spans="1:44" x14ac:dyDescent="0.3">
@@ -48885,7 +48927,7 @@
         <v>2</v>
       </c>
       <c r="C352" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D352" s="3" t="s">
         <v>45</v>
@@ -48897,7 +48939,7 @@
         <v>46156</v>
       </c>
       <c r="G352" s="5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H352" s="3" t="s">
         <v>47</v>
@@ -48912,19 +48954,19 @@
         <v>50</v>
       </c>
       <c r="L352" s="6">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="M352" s="7">
-        <v>29313.45</v>
+        <v>21134.68</v>
       </c>
       <c r="N352" s="6">
         <v>1</v>
       </c>
       <c r="O352" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P352" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q352" s="6">
         <v>0</v>
@@ -48939,7 +48981,7 @@
         <v>52</v>
       </c>
       <c r="U352" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V352" s="11">
         <v>11</v>
@@ -48948,7 +48990,7 @@
         <v>46156</v>
       </c>
       <c r="X352" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y352" s="10">
         <v>0</v>
@@ -48981,7 +49023,7 @@
         <v>53</v>
       </c>
       <c r="AI352" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ352" s="3" t="s">
         <v>52</v>
@@ -49008,7 +49050,7 @@
         <v>53</v>
       </c>
       <c r="AR352" s="3" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="353" spans="1:44" x14ac:dyDescent="0.3">
@@ -49019,7 +49061,7 @@
         <v>2</v>
       </c>
       <c r="C353" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D353" s="3" t="s">
         <v>45</v>
@@ -49031,7 +49073,7 @@
         <v>46156</v>
       </c>
       <c r="G353" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H353" s="3" t="s">
         <v>47</v>
@@ -49046,19 +49088,19 @@
         <v>50</v>
       </c>
       <c r="L353" s="6">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="M353" s="7">
-        <v>29694.14</v>
+        <v>21584.35</v>
       </c>
       <c r="N353" s="6">
         <v>1</v>
       </c>
       <c r="O353" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P353" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q353" s="6">
         <v>0</v>
@@ -49073,7 +49115,7 @@
         <v>52</v>
       </c>
       <c r="U353" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V353" s="11">
         <v>11</v>
@@ -49082,7 +49124,7 @@
         <v>46156</v>
       </c>
       <c r="X353" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y353" s="10">
         <v>0</v>
@@ -49115,7 +49157,7 @@
         <v>53</v>
       </c>
       <c r="AI353" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ353" s="3" t="s">
         <v>52</v>
@@ -49142,7 +49184,7 @@
         <v>53</v>
       </c>
       <c r="AR353" s="3" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="354" spans="1:44" x14ac:dyDescent="0.3">
@@ -49153,7 +49195,7 @@
         <v>2</v>
       </c>
       <c r="C354" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D354" s="3" t="s">
         <v>45</v>
@@ -49165,7 +49207,7 @@
         <v>46156</v>
       </c>
       <c r="G354" s="5">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H354" s="3" t="s">
         <v>47</v>
@@ -49180,19 +49222,19 @@
         <v>50</v>
       </c>
       <c r="L354" s="6">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="M354" s="7">
-        <v>30074.83</v>
+        <v>22034.03</v>
       </c>
       <c r="N354" s="6">
         <v>1</v>
       </c>
       <c r="O354" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P354" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q354" s="6">
         <v>0</v>
@@ -49207,7 +49249,7 @@
         <v>52</v>
       </c>
       <c r="U354" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V354" s="11">
         <v>11</v>
@@ -49216,7 +49258,7 @@
         <v>46156</v>
       </c>
       <c r="X354" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.54513889999999998</v>
       </c>
       <c r="Y354" s="10">
         <v>0</v>
@@ -49249,7 +49291,7 @@
         <v>53</v>
       </c>
       <c r="AI354" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ354" s="3" t="s">
         <v>52</v>
@@ -49276,7 +49318,7 @@
         <v>53</v>
       </c>
       <c r="AR354" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="355" spans="1:44" x14ac:dyDescent="0.3">
@@ -49287,7 +49329,7 @@
         <v>2</v>
       </c>
       <c r="C355" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D355" s="3" t="s">
         <v>45</v>
@@ -49299,7 +49341,7 @@
         <v>46156</v>
       </c>
       <c r="G355" s="5">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H355" s="3" t="s">
         <v>47</v>
@@ -49314,19 +49356,19 @@
         <v>50</v>
       </c>
       <c r="L355" s="6">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="M355" s="7">
-        <v>30455.53</v>
+        <v>22483.7</v>
       </c>
       <c r="N355" s="6">
         <v>1</v>
       </c>
       <c r="O355" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P355" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q355" s="6">
         <v>0</v>
@@ -49341,7 +49383,7 @@
         <v>52</v>
       </c>
       <c r="U355" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V355" s="11">
         <v>11</v>
@@ -49350,7 +49392,7 @@
         <v>46156</v>
       </c>
       <c r="X355" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.54513889999999998</v>
       </c>
       <c r="Y355" s="10">
         <v>0</v>
@@ -49383,7 +49425,7 @@
         <v>53</v>
       </c>
       <c r="AI355" s="3" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="AJ355" s="3" t="s">
         <v>52</v>
@@ -49410,7 +49452,7 @@
         <v>53</v>
       </c>
       <c r="AR355" s="3" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="356" spans="1:44" x14ac:dyDescent="0.3">
@@ -49421,7 +49463,7 @@
         <v>2</v>
       </c>
       <c r="C356" s="3" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="D356" s="3" t="s">
         <v>45</v>
@@ -49433,7 +49475,7 @@
         <v>46156</v>
       </c>
       <c r="G356" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H356" s="3" t="s">
         <v>47</v>
@@ -49448,19 +49490,19 @@
         <v>50</v>
       </c>
       <c r="L356" s="6">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="M356" s="7">
-        <v>30836.22</v>
+        <v>22933.38</v>
       </c>
       <c r="N356" s="6">
         <v>1</v>
       </c>
       <c r="O356" s="3" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="P356" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q356" s="6">
         <v>0</v>
@@ -49475,7 +49517,7 @@
         <v>52</v>
       </c>
       <c r="U356" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V356" s="11">
         <v>11</v>
@@ -49484,67 +49526,1943 @@
         <v>46156</v>
       </c>
       <c r="X356" s="12">
+        <v>0.54513889999999998</v>
+      </c>
+      <c r="Y356" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB356" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG356" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI356" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ356" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK356" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM356" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR356" s="3" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="357" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A357" s="1">
+        <v>1</v>
+      </c>
+      <c r="B357" s="2">
+        <v>2</v>
+      </c>
+      <c r="C357" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D357" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E357" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F357" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G357" s="5">
+        <v>16</v>
+      </c>
+      <c r="H357" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I357" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J357" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K357" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L357" s="6">
+        <v>52</v>
+      </c>
+      <c r="M357" s="7">
+        <v>23383.05</v>
+      </c>
+      <c r="N357" s="6">
+        <v>1</v>
+      </c>
+      <c r="O357" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="P357" s="8">
+        <v>449.67</v>
+      </c>
+      <c r="Q357" s="6">
+        <v>0</v>
+      </c>
+      <c r="R357" s="7">
+        <v>0</v>
+      </c>
+      <c r="S357" s="9">
+        <v>0</v>
+      </c>
+      <c r="T357" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U357" s="10">
+        <v>64218</v>
+      </c>
+      <c r="V357" s="11">
+        <v>11</v>
+      </c>
+      <c r="W357" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X357" s="12">
+        <v>0.54513889999999998</v>
+      </c>
+      <c r="Y357" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB357" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG357" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI357" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ357" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK357" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM357" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR357" s="3" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="358" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A358" s="1">
+        <v>1</v>
+      </c>
+      <c r="B358" s="2">
+        <v>2</v>
+      </c>
+      <c r="C358" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D358" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E358" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F358" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G358" s="5">
+        <v>1</v>
+      </c>
+      <c r="H358" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I358" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J358" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K358" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L358" s="6">
+        <v>69</v>
+      </c>
+      <c r="M358" s="7">
+        <v>26267.89</v>
+      </c>
+      <c r="N358" s="6">
+        <v>1</v>
+      </c>
+      <c r="O358" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P358" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q358" s="6">
+        <v>0</v>
+      </c>
+      <c r="R358" s="7">
+        <v>0</v>
+      </c>
+      <c r="S358" s="9">
+        <v>0</v>
+      </c>
+      <c r="T358" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U358" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V358" s="11">
+        <v>11</v>
+      </c>
+      <c r="W358" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X358" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y358" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB358" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG358" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI358" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ358" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK358" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM358" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR358" s="3" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="359" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A359" s="1">
+        <v>1</v>
+      </c>
+      <c r="B359" s="2">
+        <v>2</v>
+      </c>
+      <c r="C359" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D359" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E359" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F359" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G359" s="5">
+        <v>2</v>
+      </c>
+      <c r="H359" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I359" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J359" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K359" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L359" s="6">
+        <v>70</v>
+      </c>
+      <c r="M359" s="7">
+        <v>26648.59</v>
+      </c>
+      <c r="N359" s="6">
+        <v>1</v>
+      </c>
+      <c r="O359" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P359" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q359" s="6">
+        <v>0</v>
+      </c>
+      <c r="R359" s="7">
+        <v>0</v>
+      </c>
+      <c r="S359" s="9">
+        <v>0</v>
+      </c>
+      <c r="T359" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U359" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V359" s="11">
+        <v>11</v>
+      </c>
+      <c r="W359" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X359" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y359" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB359" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG359" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI359" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ359" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK359" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM359" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR359" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="360" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A360" s="1">
+        <v>1</v>
+      </c>
+      <c r="B360" s="2">
+        <v>2</v>
+      </c>
+      <c r="C360" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D360" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E360" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F360" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G360" s="5">
+        <v>3</v>
+      </c>
+      <c r="H360" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I360" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J360" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K360" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L360" s="6">
+        <v>71</v>
+      </c>
+      <c r="M360" s="7">
+        <v>27029.279999999999</v>
+      </c>
+      <c r="N360" s="6">
+        <v>1</v>
+      </c>
+      <c r="O360" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P360" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q360" s="6">
+        <v>0</v>
+      </c>
+      <c r="R360" s="7">
+        <v>0</v>
+      </c>
+      <c r="S360" s="9">
+        <v>0</v>
+      </c>
+      <c r="T360" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U360" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V360" s="11">
+        <v>11</v>
+      </c>
+      <c r="W360" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X360" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y360" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB360" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG360" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI360" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ360" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK360" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM360" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR360" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="361" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A361" s="1">
+        <v>1</v>
+      </c>
+      <c r="B361" s="2">
+        <v>2</v>
+      </c>
+      <c r="C361" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D361" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E361" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F361" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G361" s="5">
+        <v>4</v>
+      </c>
+      <c r="H361" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I361" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J361" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K361" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L361" s="6">
+        <v>72</v>
+      </c>
+      <c r="M361" s="7">
+        <v>27409.98</v>
+      </c>
+      <c r="N361" s="6">
+        <v>1</v>
+      </c>
+      <c r="O361" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P361" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q361" s="6">
+        <v>0</v>
+      </c>
+      <c r="R361" s="7">
+        <v>0</v>
+      </c>
+      <c r="S361" s="9">
+        <v>0</v>
+      </c>
+      <c r="T361" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U361" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V361" s="11">
+        <v>11</v>
+      </c>
+      <c r="W361" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X361" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y361" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB361" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG361" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI361" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ361" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK361" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM361" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR361" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="362" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A362" s="1">
+        <v>1</v>
+      </c>
+      <c r="B362" s="2">
+        <v>2</v>
+      </c>
+      <c r="C362" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D362" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E362" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F362" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G362" s="5">
+        <v>5</v>
+      </c>
+      <c r="H362" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I362" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J362" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K362" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L362" s="6">
+        <v>73</v>
+      </c>
+      <c r="M362" s="7">
+        <v>27790.67</v>
+      </c>
+      <c r="N362" s="6">
+        <v>1</v>
+      </c>
+      <c r="O362" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P362" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q362" s="6">
+        <v>0</v>
+      </c>
+      <c r="R362" s="7">
+        <v>0</v>
+      </c>
+      <c r="S362" s="9">
+        <v>0</v>
+      </c>
+      <c r="T362" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U362" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V362" s="11">
+        <v>11</v>
+      </c>
+      <c r="W362" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X362" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y362" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB362" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG362" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI362" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ362" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK362" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM362" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR362" s="3" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="363" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A363" s="1">
+        <v>1</v>
+      </c>
+      <c r="B363" s="2">
+        <v>2</v>
+      </c>
+      <c r="C363" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D363" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E363" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F363" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G363" s="5">
+        <v>6</v>
+      </c>
+      <c r="H363" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I363" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J363" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K363" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L363" s="6">
+        <v>74</v>
+      </c>
+      <c r="M363" s="7">
+        <v>28171.360000000001</v>
+      </c>
+      <c r="N363" s="6">
+        <v>1</v>
+      </c>
+      <c r="O363" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P363" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q363" s="6">
+        <v>0</v>
+      </c>
+      <c r="R363" s="7">
+        <v>0</v>
+      </c>
+      <c r="S363" s="9">
+        <v>0</v>
+      </c>
+      <c r="T363" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U363" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V363" s="11">
+        <v>11</v>
+      </c>
+      <c r="W363" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X363" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y363" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB363" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG363" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI363" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ363" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK363" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM363" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR363" s="3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="364" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A364" s="1">
+        <v>1</v>
+      </c>
+      <c r="B364" s="2">
+        <v>2</v>
+      </c>
+      <c r="C364" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E364" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F364" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G364" s="5">
+        <v>7</v>
+      </c>
+      <c r="H364" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I364" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J364" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K364" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L364" s="6">
+        <v>75</v>
+      </c>
+      <c r="M364" s="7">
+        <v>28552.06</v>
+      </c>
+      <c r="N364" s="6">
+        <v>1</v>
+      </c>
+      <c r="O364" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P364" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q364" s="6">
+        <v>0</v>
+      </c>
+      <c r="R364" s="7">
+        <v>0</v>
+      </c>
+      <c r="S364" s="9">
+        <v>0</v>
+      </c>
+      <c r="T364" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U364" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V364" s="11">
+        <v>11</v>
+      </c>
+      <c r="W364" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X364" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y364" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB364" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG364" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI364" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ364" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK364" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM364" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR364" s="3" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="365" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A365" s="1">
+        <v>1</v>
+      </c>
+      <c r="B365" s="2">
+        <v>2</v>
+      </c>
+      <c r="C365" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D365" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E365" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F365" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G365" s="5">
+        <v>8</v>
+      </c>
+      <c r="H365" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I365" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J365" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K365" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L365" s="6">
+        <v>76</v>
+      </c>
+      <c r="M365" s="7">
+        <v>28932.75</v>
+      </c>
+      <c r="N365" s="6">
+        <v>1</v>
+      </c>
+      <c r="O365" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P365" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q365" s="6">
+        <v>0</v>
+      </c>
+      <c r="R365" s="7">
+        <v>0</v>
+      </c>
+      <c r="S365" s="9">
+        <v>0</v>
+      </c>
+      <c r="T365" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U365" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V365" s="11">
+        <v>11</v>
+      </c>
+      <c r="W365" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X365" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y365" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z365" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA365" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB365" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC365" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD365" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE365" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF365" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG365" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH365" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI365" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ365" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK365" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL365" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM365" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN365" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO365" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP365" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ365" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR365" s="3" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="366" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A366" s="1">
+        <v>1</v>
+      </c>
+      <c r="B366" s="2">
+        <v>2</v>
+      </c>
+      <c r="C366" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D366" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E366" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F366" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G366" s="5">
+        <v>9</v>
+      </c>
+      <c r="H366" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I366" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J366" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K366" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L366" s="6">
+        <v>77</v>
+      </c>
+      <c r="M366" s="7">
+        <v>29313.45</v>
+      </c>
+      <c r="N366" s="6">
+        <v>1</v>
+      </c>
+      <c r="O366" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P366" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q366" s="6">
+        <v>0</v>
+      </c>
+      <c r="R366" s="7">
+        <v>0</v>
+      </c>
+      <c r="S366" s="9">
+        <v>0</v>
+      </c>
+      <c r="T366" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U366" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V366" s="11">
+        <v>11</v>
+      </c>
+      <c r="W366" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X366" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y366" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z366" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA366" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB366" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC366" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD366" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE366" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF366" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG366" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH366" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI366" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ366" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK366" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL366" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM366" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN366" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO366" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP366" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ366" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR366" s="3" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="367" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A367" s="1">
+        <v>1</v>
+      </c>
+      <c r="B367" s="2">
+        <v>2</v>
+      </c>
+      <c r="C367" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D367" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E367" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F367" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G367" s="5">
+        <v>10</v>
+      </c>
+      <c r="H367" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I367" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J367" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K367" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L367" s="6">
+        <v>78</v>
+      </c>
+      <c r="M367" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N367" s="6">
+        <v>1</v>
+      </c>
+      <c r="O367" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P367" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q367" s="6">
+        <v>0</v>
+      </c>
+      <c r="R367" s="7">
+        <v>0</v>
+      </c>
+      <c r="S367" s="9">
+        <v>0</v>
+      </c>
+      <c r="T367" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U367" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V367" s="11">
+        <v>11</v>
+      </c>
+      <c r="W367" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X367" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y367" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z367" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA367" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB367" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC367" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD367" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE367" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF367" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG367" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH367" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI367" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ367" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK367" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL367" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM367" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN367" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO367" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP367" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ367" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR367" s="3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="368" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A368" s="1">
+        <v>1</v>
+      </c>
+      <c r="B368" s="2">
+        <v>2</v>
+      </c>
+      <c r="C368" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D368" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E368" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F368" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G368" s="5">
+        <v>11</v>
+      </c>
+      <c r="H368" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I368" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J368" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K368" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L368" s="6">
+        <v>79</v>
+      </c>
+      <c r="M368" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N368" s="6">
+        <v>1</v>
+      </c>
+      <c r="O368" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P368" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q368" s="6">
+        <v>0</v>
+      </c>
+      <c r="R368" s="7">
+        <v>0</v>
+      </c>
+      <c r="S368" s="9">
+        <v>0</v>
+      </c>
+      <c r="T368" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U368" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V368" s="11">
+        <v>11</v>
+      </c>
+      <c r="W368" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X368" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y368" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z368" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA368" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB368" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC368" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD368" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE368" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF368" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG368" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH368" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI368" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ368" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK368" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL368" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM368" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN368" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO368" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP368" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ368" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR368" s="3" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="369" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A369" s="1">
+        <v>1</v>
+      </c>
+      <c r="B369" s="2">
+        <v>2</v>
+      </c>
+      <c r="C369" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D369" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E369" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F369" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G369" s="5">
+        <v>12</v>
+      </c>
+      <c r="H369" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I369" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J369" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K369" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L369" s="6">
+        <v>80</v>
+      </c>
+      <c r="M369" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N369" s="6">
+        <v>1</v>
+      </c>
+      <c r="O369" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P369" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q369" s="6">
+        <v>0</v>
+      </c>
+      <c r="R369" s="7">
+        <v>0</v>
+      </c>
+      <c r="S369" s="9">
+        <v>0</v>
+      </c>
+      <c r="T369" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U369" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V369" s="11">
+        <v>11</v>
+      </c>
+      <c r="W369" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X369" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y369" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z369" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA369" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB369" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC369" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD369" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE369" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF369" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG369" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH369" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI369" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ369" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK369" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL369" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM369" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN369" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO369" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP369" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ369" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR369" s="3" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="370" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A370" s="1">
+        <v>1</v>
+      </c>
+      <c r="B370" s="2">
+        <v>2</v>
+      </c>
+      <c r="C370" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D370" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E370" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F370" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G370" s="5">
+        <v>13</v>
+      </c>
+      <c r="H370" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I370" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J370" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K370" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L370" s="6">
+        <v>81</v>
+      </c>
+      <c r="M370" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N370" s="6">
+        <v>1</v>
+      </c>
+      <c r="O370" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="P370" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q370" s="6">
+        <v>0</v>
+      </c>
+      <c r="R370" s="7">
+        <v>0</v>
+      </c>
+      <c r="S370" s="9">
+        <v>0</v>
+      </c>
+      <c r="T370" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U370" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V370" s="11">
+        <v>11</v>
+      </c>
+      <c r="W370" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X370" s="12">
         <v>0.40138889999999999</v>
       </c>
-      <c r="Y356" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z356" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA356" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB356" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC356" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD356" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE356" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF356" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG356" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH356" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI356" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="AJ356" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK356" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL356" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM356" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN356" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO356" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP356" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ356" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR356" s="3" t="s">
-        <v>414</v>
+      <c r="Y370" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z370" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA370" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB370" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC370" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD370" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE370" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF370" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG370" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH370" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI370" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ370" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK370" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL370" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM370" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN370" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO370" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP370" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ370" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR370" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 13:36:24,72
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADE07338-81D0-45E5-9117-B3CB0972D0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{542B7D29-1343-4464-AFA5-E5F6D1DB211D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6686" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6812" uniqueCount="436">
   <si>
     <t>Sel</t>
   </si>
@@ -1264,6 +1264,27 @@
     <t>1858400002951</t>
   </si>
   <si>
+    <t>1858400002952</t>
+  </si>
+  <si>
+    <t>1858400002953</t>
+  </si>
+  <si>
+    <t>1858400002954</t>
+  </si>
+  <si>
+    <t>1858400002955</t>
+  </si>
+  <si>
+    <t>1858400002956</t>
+  </si>
+  <si>
+    <t>1858400002957</t>
+  </si>
+  <si>
+    <t>1858400002958</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -1882,7 +1903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR370"/>
+  <dimension ref="A1:AR377"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -49731,7 +49752,7 @@
         <v>2</v>
       </c>
       <c r="C358" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D358" s="3" t="s">
         <v>45</v>
@@ -49743,7 +49764,7 @@
         <v>46156</v>
       </c>
       <c r="G358" s="5">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="H358" s="3" t="s">
         <v>47</v>
@@ -49758,19 +49779,19 @@
         <v>50</v>
       </c>
       <c r="L358" s="6">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="M358" s="7">
-        <v>26267.89</v>
+        <v>23832.720000000001</v>
       </c>
       <c r="N358" s="6">
         <v>1</v>
       </c>
       <c r="O358" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P358" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q358" s="6">
         <v>0</v>
@@ -49785,7 +49806,7 @@
         <v>52</v>
       </c>
       <c r="U358" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V358" s="11">
         <v>11</v>
@@ -49794,7 +49815,7 @@
         <v>46156</v>
       </c>
       <c r="X358" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y358" s="10">
         <v>0</v>
@@ -49854,7 +49875,7 @@
         <v>53</v>
       </c>
       <c r="AR358" s="3" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="359" spans="1:44" x14ac:dyDescent="0.3">
@@ -49865,7 +49886,7 @@
         <v>2</v>
       </c>
       <c r="C359" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D359" s="3" t="s">
         <v>45</v>
@@ -49877,7 +49898,7 @@
         <v>46156</v>
       </c>
       <c r="G359" s="5">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H359" s="3" t="s">
         <v>47</v>
@@ -49892,19 +49913,19 @@
         <v>50</v>
       </c>
       <c r="L359" s="6">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="M359" s="7">
-        <v>26648.59</v>
+        <v>24282.400000000001</v>
       </c>
       <c r="N359" s="6">
         <v>1</v>
       </c>
       <c r="O359" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P359" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q359" s="6">
         <v>0</v>
@@ -49919,7 +49940,7 @@
         <v>52</v>
       </c>
       <c r="U359" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V359" s="11">
         <v>11</v>
@@ -49928,7 +49949,7 @@
         <v>46156</v>
       </c>
       <c r="X359" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y359" s="10">
         <v>0</v>
@@ -49988,7 +50009,7 @@
         <v>53</v>
       </c>
       <c r="AR359" s="3" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="360" spans="1:44" x14ac:dyDescent="0.3">
@@ -49999,7 +50020,7 @@
         <v>2</v>
       </c>
       <c r="C360" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D360" s="3" t="s">
         <v>45</v>
@@ -50011,7 +50032,7 @@
         <v>46156</v>
       </c>
       <c r="G360" s="5">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H360" s="3" t="s">
         <v>47</v>
@@ -50026,19 +50047,19 @@
         <v>50</v>
       </c>
       <c r="L360" s="6">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="M360" s="7">
-        <v>27029.279999999999</v>
+        <v>24732.07</v>
       </c>
       <c r="N360" s="6">
         <v>1</v>
       </c>
       <c r="O360" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P360" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q360" s="6">
         <v>0</v>
@@ -50053,7 +50074,7 @@
         <v>52</v>
       </c>
       <c r="U360" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V360" s="11">
         <v>11</v>
@@ -50062,7 +50083,7 @@
         <v>46156</v>
       </c>
       <c r="X360" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y360" s="10">
         <v>0</v>
@@ -50122,7 +50143,7 @@
         <v>53</v>
       </c>
       <c r="AR360" s="3" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="361" spans="1:44" x14ac:dyDescent="0.3">
@@ -50133,7 +50154,7 @@
         <v>2</v>
       </c>
       <c r="C361" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D361" s="3" t="s">
         <v>45</v>
@@ -50145,7 +50166,7 @@
         <v>46156</v>
       </c>
       <c r="G361" s="5">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="H361" s="3" t="s">
         <v>47</v>
@@ -50160,19 +50181,19 @@
         <v>50</v>
       </c>
       <c r="L361" s="6">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="M361" s="7">
-        <v>27409.98</v>
+        <v>25181.75</v>
       </c>
       <c r="N361" s="6">
         <v>1</v>
       </c>
       <c r="O361" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P361" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q361" s="6">
         <v>0</v>
@@ -50187,7 +50208,7 @@
         <v>52</v>
       </c>
       <c r="U361" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V361" s="11">
         <v>11</v>
@@ -50196,7 +50217,7 @@
         <v>46156</v>
       </c>
       <c r="X361" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y361" s="10">
         <v>0</v>
@@ -50256,7 +50277,7 @@
         <v>53</v>
       </c>
       <c r="AR361" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="362" spans="1:44" x14ac:dyDescent="0.3">
@@ -50267,7 +50288,7 @@
         <v>2</v>
       </c>
       <c r="C362" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D362" s="3" t="s">
         <v>45</v>
@@ -50279,7 +50300,7 @@
         <v>46156</v>
       </c>
       <c r="G362" s="5">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="H362" s="3" t="s">
         <v>47</v>
@@ -50294,19 +50315,19 @@
         <v>50</v>
       </c>
       <c r="L362" s="6">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="M362" s="7">
-        <v>27790.67</v>
+        <v>25631.42</v>
       </c>
       <c r="N362" s="6">
         <v>1</v>
       </c>
       <c r="O362" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P362" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q362" s="6">
         <v>0</v>
@@ -50321,7 +50342,7 @@
         <v>52</v>
       </c>
       <c r="U362" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V362" s="11">
         <v>11</v>
@@ -50330,7 +50351,7 @@
         <v>46156</v>
       </c>
       <c r="X362" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y362" s="10">
         <v>0</v>
@@ -50390,7 +50411,7 @@
         <v>53</v>
       </c>
       <c r="AR362" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="363" spans="1:44" x14ac:dyDescent="0.3">
@@ -50401,7 +50422,7 @@
         <v>2</v>
       </c>
       <c r="C363" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D363" s="3" t="s">
         <v>45</v>
@@ -50413,7 +50434,7 @@
         <v>46156</v>
       </c>
       <c r="G363" s="5">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="H363" s="3" t="s">
         <v>47</v>
@@ -50428,19 +50449,19 @@
         <v>50</v>
       </c>
       <c r="L363" s="6">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="M363" s="7">
-        <v>28171.360000000001</v>
+        <v>26081.09</v>
       </c>
       <c r="N363" s="6">
         <v>1</v>
       </c>
       <c r="O363" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P363" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q363" s="6">
         <v>0</v>
@@ -50455,7 +50476,7 @@
         <v>52</v>
       </c>
       <c r="U363" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V363" s="11">
         <v>11</v>
@@ -50464,7 +50485,7 @@
         <v>46156</v>
       </c>
       <c r="X363" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y363" s="10">
         <v>0</v>
@@ -50524,7 +50545,7 @@
         <v>53</v>
       </c>
       <c r="AR363" s="3" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="364" spans="1:44" x14ac:dyDescent="0.3">
@@ -50535,7 +50556,7 @@
         <v>2</v>
       </c>
       <c r="C364" s="3" t="s">
-        <v>414</v>
+        <v>395</v>
       </c>
       <c r="D364" s="3" t="s">
         <v>45</v>
@@ -50547,7 +50568,7 @@
         <v>46156</v>
       </c>
       <c r="G364" s="5">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H364" s="3" t="s">
         <v>47</v>
@@ -50562,19 +50583,19 @@
         <v>50</v>
       </c>
       <c r="L364" s="6">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="M364" s="7">
-        <v>28552.06</v>
+        <v>26530.77</v>
       </c>
       <c r="N364" s="6">
         <v>1</v>
       </c>
       <c r="O364" s="3" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="P364" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q364" s="6">
         <v>0</v>
@@ -50589,7 +50610,7 @@
         <v>52</v>
       </c>
       <c r="U364" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V364" s="11">
         <v>11</v>
@@ -50598,7 +50619,7 @@
         <v>46156</v>
       </c>
       <c r="X364" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y364" s="10">
         <v>0</v>
@@ -50658,7 +50679,7 @@
         <v>53</v>
       </c>
       <c r="AR364" s="3" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="365" spans="1:44" x14ac:dyDescent="0.3">
@@ -50669,7 +50690,7 @@
         <v>2</v>
       </c>
       <c r="C365" s="3" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D365" s="3" t="s">
         <v>45</v>
@@ -50681,7 +50702,7 @@
         <v>46156</v>
       </c>
       <c r="G365" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H365" s="3" t="s">
         <v>47</v>
@@ -50696,16 +50717,16 @@
         <v>50</v>
       </c>
       <c r="L365" s="6">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="M365" s="7">
-        <v>28932.75</v>
+        <v>26267.89</v>
       </c>
       <c r="N365" s="6">
         <v>1</v>
       </c>
       <c r="O365" s="3" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="P365" s="8">
         <v>380.69</v>
@@ -50732,7 +50753,7 @@
         <v>46156</v>
       </c>
       <c r="X365" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y365" s="10">
         <v>0</v>
@@ -50803,7 +50824,7 @@
         <v>2</v>
       </c>
       <c r="C366" s="3" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D366" s="3" t="s">
         <v>45</v>
@@ -50815,7 +50836,7 @@
         <v>46156</v>
       </c>
       <c r="G366" s="5">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H366" s="3" t="s">
         <v>47</v>
@@ -50830,16 +50851,16 @@
         <v>50</v>
       </c>
       <c r="L366" s="6">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="M366" s="7">
-        <v>29313.45</v>
+        <v>26648.59</v>
       </c>
       <c r="N366" s="6">
         <v>1</v>
       </c>
       <c r="O366" s="3" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="P366" s="8">
         <v>380.69</v>
@@ -50866,7 +50887,7 @@
         <v>46156</v>
       </c>
       <c r="X366" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y366" s="10">
         <v>0</v>
@@ -50937,7 +50958,7 @@
         <v>2</v>
       </c>
       <c r="C367" s="3" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D367" s="3" t="s">
         <v>45</v>
@@ -50949,7 +50970,7 @@
         <v>46156</v>
       </c>
       <c r="G367" s="5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H367" s="3" t="s">
         <v>47</v>
@@ -50964,16 +50985,16 @@
         <v>50</v>
       </c>
       <c r="L367" s="6">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="M367" s="7">
-        <v>29694.14</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N367" s="6">
         <v>1</v>
       </c>
       <c r="O367" s="3" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="P367" s="8">
         <v>380.69</v>
@@ -51000,7 +51021,7 @@
         <v>46156</v>
       </c>
       <c r="X367" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y367" s="10">
         <v>0</v>
@@ -51071,7 +51092,7 @@
         <v>2</v>
       </c>
       <c r="C368" s="3" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D368" s="3" t="s">
         <v>45</v>
@@ -51083,7 +51104,7 @@
         <v>46156</v>
       </c>
       <c r="G368" s="5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="H368" s="3" t="s">
         <v>47</v>
@@ -51098,16 +51119,16 @@
         <v>50</v>
       </c>
       <c r="L368" s="6">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="M368" s="7">
-        <v>30074.83</v>
+        <v>27409.98</v>
       </c>
       <c r="N368" s="6">
         <v>1</v>
       </c>
       <c r="O368" s="3" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="P368" s="8">
         <v>380.69</v>
@@ -51134,7 +51155,7 @@
         <v>46156</v>
       </c>
       <c r="X368" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y368" s="10">
         <v>0</v>
@@ -51205,7 +51226,7 @@
         <v>2</v>
       </c>
       <c r="C369" s="3" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D369" s="3" t="s">
         <v>45</v>
@@ -51217,7 +51238,7 @@
         <v>46156</v>
       </c>
       <c r="G369" s="5">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H369" s="3" t="s">
         <v>47</v>
@@ -51232,16 +51253,16 @@
         <v>50</v>
       </c>
       <c r="L369" s="6">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="M369" s="7">
-        <v>30455.53</v>
+        <v>27790.67</v>
       </c>
       <c r="N369" s="6">
         <v>1</v>
       </c>
       <c r="O369" s="3" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="P369" s="8">
         <v>380.69</v>
@@ -51268,7 +51289,7 @@
         <v>46156</v>
       </c>
       <c r="X369" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y369" s="10">
         <v>0</v>
@@ -51339,7 +51360,7 @@
         <v>2</v>
       </c>
       <c r="C370" s="3" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D370" s="3" t="s">
         <v>45</v>
@@ -51351,7 +51372,7 @@
         <v>46156</v>
       </c>
       <c r="G370" s="5">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H370" s="3" t="s">
         <v>47</v>
@@ -51366,16 +51387,16 @@
         <v>50</v>
       </c>
       <c r="L370" s="6">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="M370" s="7">
-        <v>30836.22</v>
+        <v>28171.360000000001</v>
       </c>
       <c r="N370" s="6">
         <v>1</v>
       </c>
       <c r="O370" s="3" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="P370" s="8">
         <v>380.69</v>
@@ -51402,7 +51423,7 @@
         <v>46156</v>
       </c>
       <c r="X370" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y370" s="10">
         <v>0</v>
@@ -51463,6 +51484,944 @@
       </c>
       <c r="AR370" s="3" t="s">
         <v>428</v>
+      </c>
+    </row>
+    <row r="371" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A371" s="1">
+        <v>1</v>
+      </c>
+      <c r="B371" s="2">
+        <v>2</v>
+      </c>
+      <c r="C371" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D371" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E371" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F371" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G371" s="5">
+        <v>7</v>
+      </c>
+      <c r="H371" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I371" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J371" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K371" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L371" s="6">
+        <v>75</v>
+      </c>
+      <c r="M371" s="7">
+        <v>28552.06</v>
+      </c>
+      <c r="N371" s="6">
+        <v>1</v>
+      </c>
+      <c r="O371" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P371" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q371" s="6">
+        <v>0</v>
+      </c>
+      <c r="R371" s="7">
+        <v>0</v>
+      </c>
+      <c r="S371" s="9">
+        <v>0</v>
+      </c>
+      <c r="T371" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U371" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V371" s="11">
+        <v>11</v>
+      </c>
+      <c r="W371" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X371" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y371" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z371" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA371" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB371" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC371" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD371" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE371" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF371" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG371" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH371" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI371" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ371" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK371" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL371" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM371" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN371" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO371" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP371" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ371" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR371" s="3" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="372" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A372" s="1">
+        <v>1</v>
+      </c>
+      <c r="B372" s="2">
+        <v>2</v>
+      </c>
+      <c r="C372" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D372" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E372" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F372" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G372" s="5">
+        <v>8</v>
+      </c>
+      <c r="H372" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I372" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J372" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K372" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L372" s="6">
+        <v>76</v>
+      </c>
+      <c r="M372" s="7">
+        <v>28932.75</v>
+      </c>
+      <c r="N372" s="6">
+        <v>1</v>
+      </c>
+      <c r="O372" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P372" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q372" s="6">
+        <v>0</v>
+      </c>
+      <c r="R372" s="7">
+        <v>0</v>
+      </c>
+      <c r="S372" s="9">
+        <v>0</v>
+      </c>
+      <c r="T372" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U372" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V372" s="11">
+        <v>11</v>
+      </c>
+      <c r="W372" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X372" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y372" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z372" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA372" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB372" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC372" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD372" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE372" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF372" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG372" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH372" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI372" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ372" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK372" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL372" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM372" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN372" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO372" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP372" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ372" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR372" s="3" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="373" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A373" s="1">
+        <v>1</v>
+      </c>
+      <c r="B373" s="2">
+        <v>2</v>
+      </c>
+      <c r="C373" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D373" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E373" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F373" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G373" s="5">
+        <v>9</v>
+      </c>
+      <c r="H373" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I373" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J373" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K373" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L373" s="6">
+        <v>77</v>
+      </c>
+      <c r="M373" s="7">
+        <v>29313.45</v>
+      </c>
+      <c r="N373" s="6">
+        <v>1</v>
+      </c>
+      <c r="O373" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P373" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q373" s="6">
+        <v>0</v>
+      </c>
+      <c r="R373" s="7">
+        <v>0</v>
+      </c>
+      <c r="S373" s="9">
+        <v>0</v>
+      </c>
+      <c r="T373" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U373" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V373" s="11">
+        <v>11</v>
+      </c>
+      <c r="W373" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X373" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y373" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB373" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG373" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI373" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ373" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK373" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM373" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR373" s="3" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="374" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A374" s="1">
+        <v>1</v>
+      </c>
+      <c r="B374" s="2">
+        <v>2</v>
+      </c>
+      <c r="C374" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D374" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E374" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F374" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G374" s="5">
+        <v>10</v>
+      </c>
+      <c r="H374" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I374" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J374" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K374" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L374" s="6">
+        <v>78</v>
+      </c>
+      <c r="M374" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N374" s="6">
+        <v>1</v>
+      </c>
+      <c r="O374" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P374" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q374" s="6">
+        <v>0</v>
+      </c>
+      <c r="R374" s="7">
+        <v>0</v>
+      </c>
+      <c r="S374" s="9">
+        <v>0</v>
+      </c>
+      <c r="T374" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U374" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V374" s="11">
+        <v>11</v>
+      </c>
+      <c r="W374" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X374" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y374" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB374" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG374" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI374" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ374" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK374" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM374" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR374" s="3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="375" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A375" s="1">
+        <v>1</v>
+      </c>
+      <c r="B375" s="2">
+        <v>2</v>
+      </c>
+      <c r="C375" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D375" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E375" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F375" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G375" s="5">
+        <v>11</v>
+      </c>
+      <c r="H375" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I375" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J375" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K375" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L375" s="6">
+        <v>79</v>
+      </c>
+      <c r="M375" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N375" s="6">
+        <v>1</v>
+      </c>
+      <c r="O375" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P375" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q375" s="6">
+        <v>0</v>
+      </c>
+      <c r="R375" s="7">
+        <v>0</v>
+      </c>
+      <c r="S375" s="9">
+        <v>0</v>
+      </c>
+      <c r="T375" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U375" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V375" s="11">
+        <v>11</v>
+      </c>
+      <c r="W375" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X375" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y375" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB375" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG375" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI375" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ375" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK375" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM375" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR375" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="376" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A376" s="1">
+        <v>1</v>
+      </c>
+      <c r="B376" s="2">
+        <v>2</v>
+      </c>
+      <c r="C376" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D376" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E376" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F376" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G376" s="5">
+        <v>12</v>
+      </c>
+      <c r="H376" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I376" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J376" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K376" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L376" s="6">
+        <v>80</v>
+      </c>
+      <c r="M376" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N376" s="6">
+        <v>1</v>
+      </c>
+      <c r="O376" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P376" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q376" s="6">
+        <v>0</v>
+      </c>
+      <c r="R376" s="7">
+        <v>0</v>
+      </c>
+      <c r="S376" s="9">
+        <v>0</v>
+      </c>
+      <c r="T376" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U376" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V376" s="11">
+        <v>11</v>
+      </c>
+      <c r="W376" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X376" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y376" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB376" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG376" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI376" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ376" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK376" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM376" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR376" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="377" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A377" s="1">
+        <v>1</v>
+      </c>
+      <c r="B377" s="2">
+        <v>2</v>
+      </c>
+      <c r="C377" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D377" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E377" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F377" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G377" s="5">
+        <v>13</v>
+      </c>
+      <c r="H377" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I377" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J377" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K377" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L377" s="6">
+        <v>81</v>
+      </c>
+      <c r="M377" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N377" s="6">
+        <v>1</v>
+      </c>
+      <c r="O377" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="P377" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q377" s="6">
+        <v>0</v>
+      </c>
+      <c r="R377" s="7">
+        <v>0</v>
+      </c>
+      <c r="S377" s="9">
+        <v>0</v>
+      </c>
+      <c r="T377" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U377" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V377" s="11">
+        <v>11</v>
+      </c>
+      <c r="W377" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X377" s="12">
+        <v>0.40138889999999999</v>
+      </c>
+      <c r="Y377" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB377" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG377" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI377" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ377" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK377" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM377" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR377" s="3" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 14:16:28,96
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FF33AE6-83F9-4DCF-85C7-54352984A57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45E08581-16AF-43B0-A555-49B8398B5224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7874" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8108" uniqueCount="508">
   <si>
     <t>Sel</t>
   </si>
@@ -1378,6 +1378,45 @@
     <t>1854300115097</t>
   </si>
   <si>
+    <t>1854300115098</t>
+  </si>
+  <si>
+    <t>1854300115099</t>
+  </si>
+  <si>
+    <t>1854300115100</t>
+  </si>
+  <si>
+    <t>1854300115101</t>
+  </si>
+  <si>
+    <t>1854300115102</t>
+  </si>
+  <si>
+    <t>1854300115103</t>
+  </si>
+  <si>
+    <t>1854300115104</t>
+  </si>
+  <si>
+    <t>1854300115105</t>
+  </si>
+  <si>
+    <t>1854300115106</t>
+  </si>
+  <si>
+    <t>1854300115107</t>
+  </si>
+  <si>
+    <t>1854300115108</t>
+  </si>
+  <si>
+    <t>1854300115109</t>
+  </si>
+  <si>
+    <t>1854300115110</t>
+  </si>
+  <si>
     <t>10016351</t>
   </si>
   <si>
@@ -2080,7 +2119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR436"/>
+  <dimension ref="A1:AR449"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -55423,7 +55462,7 @@
         <v>2</v>
       </c>
       <c r="C399" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D399" s="3" t="s">
         <v>45</v>
@@ -55435,7 +55474,7 @@
         <v>46156</v>
       </c>
       <c r="G399" s="5">
-        <v>1</v>
+        <v>447</v>
       </c>
       <c r="H399" s="3" t="s">
         <v>47</v>
@@ -55450,19 +55489,19 @@
         <v>50</v>
       </c>
       <c r="L399" s="6">
-        <v>37</v>
+        <v>663</v>
       </c>
       <c r="M399" s="7">
-        <v>16637.939999999999</v>
+        <v>131034.82</v>
       </c>
       <c r="N399" s="6">
         <v>1</v>
       </c>
       <c r="O399" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P399" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q399" s="6">
         <v>0</v>
@@ -55477,7 +55516,7 @@
         <v>52</v>
       </c>
       <c r="U399" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V399" s="11">
         <v>11</v>
@@ -55486,7 +55525,7 @@
         <v>46156</v>
       </c>
       <c r="X399" s="12">
-        <v>0.37847219999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y399" s="10">
         <v>0</v>
@@ -55519,7 +55558,7 @@
         <v>53</v>
       </c>
       <c r="AI399" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ399" s="3" t="s">
         <v>52</v>
@@ -55546,7 +55585,7 @@
         <v>53</v>
       </c>
       <c r="AR399" s="3" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="400" spans="1:44" x14ac:dyDescent="0.3">
@@ -55557,7 +55596,7 @@
         <v>2</v>
       </c>
       <c r="C400" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D400" s="3" t="s">
         <v>45</v>
@@ -55569,7 +55608,7 @@
         <v>46156</v>
       </c>
       <c r="G400" s="5">
-        <v>2</v>
+        <v>448</v>
       </c>
       <c r="H400" s="3" t="s">
         <v>47</v>
@@ -55584,19 +55623,19 @@
         <v>50</v>
       </c>
       <c r="L400" s="6">
-        <v>38</v>
+        <v>664</v>
       </c>
       <c r="M400" s="7">
-        <v>17087.61</v>
+        <v>131232.46</v>
       </c>
       <c r="N400" s="6">
         <v>1</v>
       </c>
       <c r="O400" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P400" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q400" s="6">
         <v>0</v>
@@ -55611,7 +55650,7 @@
         <v>52</v>
       </c>
       <c r="U400" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V400" s="11">
         <v>11</v>
@@ -55620,7 +55659,7 @@
         <v>46156</v>
       </c>
       <c r="X400" s="12">
-        <v>0.42013889999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y400" s="10">
         <v>0</v>
@@ -55653,7 +55692,7 @@
         <v>53</v>
       </c>
       <c r="AI400" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ400" s="3" t="s">
         <v>52</v>
@@ -55680,7 +55719,7 @@
         <v>53</v>
       </c>
       <c r="AR400" s="3" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="401" spans="1:44" x14ac:dyDescent="0.3">
@@ -55691,7 +55730,7 @@
         <v>2</v>
       </c>
       <c r="C401" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D401" s="3" t="s">
         <v>45</v>
@@ -55703,7 +55742,7 @@
         <v>46156</v>
       </c>
       <c r="G401" s="5">
-        <v>3</v>
+        <v>449</v>
       </c>
       <c r="H401" s="3" t="s">
         <v>47</v>
@@ -55718,19 +55757,19 @@
         <v>50</v>
       </c>
       <c r="L401" s="6">
-        <v>39</v>
+        <v>665</v>
       </c>
       <c r="M401" s="7">
-        <v>17537.29</v>
+        <v>131430.1</v>
       </c>
       <c r="N401" s="6">
         <v>1</v>
       </c>
       <c r="O401" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P401" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q401" s="6">
         <v>0</v>
@@ -55745,7 +55784,7 @@
         <v>52</v>
       </c>
       <c r="U401" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V401" s="11">
         <v>11</v>
@@ -55754,7 +55793,7 @@
         <v>46156</v>
       </c>
       <c r="X401" s="12">
-        <v>0.44097219999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y401" s="10">
         <v>0</v>
@@ -55787,34 +55826,34 @@
         <v>53</v>
       </c>
       <c r="AI401" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ401" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK401" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL401" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM401" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ401" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR401" s="3" t="s">
         <v>454</v>
-      </c>
-      <c r="AJ401" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK401" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL401" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM401" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN401" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO401" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP401" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ401" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR401" s="3" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="402" spans="1:44" x14ac:dyDescent="0.3">
@@ -55825,7 +55864,7 @@
         <v>2</v>
       </c>
       <c r="C402" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D402" s="3" t="s">
         <v>45</v>
@@ -55837,7 +55876,7 @@
         <v>46156</v>
       </c>
       <c r="G402" s="5">
-        <v>4</v>
+        <v>450</v>
       </c>
       <c r="H402" s="3" t="s">
         <v>47</v>
@@ -55852,19 +55891,19 @@
         <v>50</v>
       </c>
       <c r="L402" s="6">
-        <v>40</v>
+        <v>666</v>
       </c>
       <c r="M402" s="7">
-        <v>17986.96</v>
+        <v>131627.74</v>
       </c>
       <c r="N402" s="6">
         <v>1</v>
       </c>
       <c r="O402" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P402" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q402" s="6">
         <v>0</v>
@@ -55879,7 +55918,7 @@
         <v>52</v>
       </c>
       <c r="U402" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V402" s="11">
         <v>11</v>
@@ -55888,7 +55927,7 @@
         <v>46156</v>
       </c>
       <c r="X402" s="12">
-        <v>0.44097219999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y402" s="10">
         <v>0</v>
@@ -55921,7 +55960,7 @@
         <v>53</v>
       </c>
       <c r="AI402" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ402" s="3" t="s">
         <v>52</v>
@@ -55948,7 +55987,7 @@
         <v>53</v>
       </c>
       <c r="AR402" s="3" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="403" spans="1:44" x14ac:dyDescent="0.3">
@@ -55959,7 +55998,7 @@
         <v>2</v>
       </c>
       <c r="C403" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D403" s="3" t="s">
         <v>45</v>
@@ -55971,7 +56010,7 @@
         <v>46156</v>
       </c>
       <c r="G403" s="5">
-        <v>5</v>
+        <v>451</v>
       </c>
       <c r="H403" s="3" t="s">
         <v>47</v>
@@ -55986,19 +56025,19 @@
         <v>50</v>
       </c>
       <c r="L403" s="6">
-        <v>41</v>
+        <v>667</v>
       </c>
       <c r="M403" s="7">
-        <v>18436.63</v>
+        <v>131825.38</v>
       </c>
       <c r="N403" s="6">
         <v>1</v>
       </c>
       <c r="O403" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P403" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q403" s="6">
         <v>0</v>
@@ -56013,7 +56052,7 @@
         <v>52</v>
       </c>
       <c r="U403" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V403" s="11">
         <v>11</v>
@@ -56022,7 +56061,7 @@
         <v>46156</v>
       </c>
       <c r="X403" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y403" s="10">
         <v>0</v>
@@ -56055,7 +56094,7 @@
         <v>53</v>
       </c>
       <c r="AI403" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ403" s="3" t="s">
         <v>52</v>
@@ -56082,7 +56121,7 @@
         <v>53</v>
       </c>
       <c r="AR403" s="3" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="404" spans="1:44" x14ac:dyDescent="0.3">
@@ -56093,7 +56132,7 @@
         <v>2</v>
       </c>
       <c r="C404" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D404" s="3" t="s">
         <v>45</v>
@@ -56105,7 +56144,7 @@
         <v>46156</v>
       </c>
       <c r="G404" s="5">
-        <v>6</v>
+        <v>452</v>
       </c>
       <c r="H404" s="3" t="s">
         <v>47</v>
@@ -56120,19 +56159,19 @@
         <v>50</v>
       </c>
       <c r="L404" s="6">
-        <v>42</v>
+        <v>668</v>
       </c>
       <c r="M404" s="7">
-        <v>18886.310000000001</v>
+        <v>132023.01999999999</v>
       </c>
       <c r="N404" s="6">
         <v>1</v>
       </c>
       <c r="O404" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P404" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q404" s="6">
         <v>0</v>
@@ -56147,7 +56186,7 @@
         <v>52</v>
       </c>
       <c r="U404" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V404" s="11">
         <v>11</v>
@@ -56156,7 +56195,7 @@
         <v>46156</v>
       </c>
       <c r="X404" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y404" s="10">
         <v>0</v>
@@ -56189,7 +56228,7 @@
         <v>53</v>
       </c>
       <c r="AI404" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ404" s="3" t="s">
         <v>52</v>
@@ -56216,7 +56255,7 @@
         <v>53</v>
       </c>
       <c r="AR404" s="3" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="405" spans="1:44" x14ac:dyDescent="0.3">
@@ -56227,7 +56266,7 @@
         <v>2</v>
       </c>
       <c r="C405" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D405" s="3" t="s">
         <v>45</v>
@@ -56239,7 +56278,7 @@
         <v>46156</v>
       </c>
       <c r="G405" s="5">
-        <v>7</v>
+        <v>453</v>
       </c>
       <c r="H405" s="3" t="s">
         <v>47</v>
@@ -56254,19 +56293,19 @@
         <v>50</v>
       </c>
       <c r="L405" s="6">
-        <v>43</v>
+        <v>669</v>
       </c>
       <c r="M405" s="7">
-        <v>19335.98</v>
+        <v>132220.66</v>
       </c>
       <c r="N405" s="6">
         <v>1</v>
       </c>
       <c r="O405" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P405" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q405" s="6">
         <v>0</v>
@@ -56281,7 +56320,7 @@
         <v>52</v>
       </c>
       <c r="U405" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V405" s="11">
         <v>11</v>
@@ -56290,7 +56329,7 @@
         <v>46156</v>
       </c>
       <c r="X405" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y405" s="10">
         <v>0</v>
@@ -56323,7 +56362,7 @@
         <v>53</v>
       </c>
       <c r="AI405" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ405" s="3" t="s">
         <v>52</v>
@@ -56350,7 +56389,7 @@
         <v>53</v>
       </c>
       <c r="AR405" s="3" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="406" spans="1:44" x14ac:dyDescent="0.3">
@@ -56361,7 +56400,7 @@
         <v>2</v>
       </c>
       <c r="C406" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D406" s="3" t="s">
         <v>45</v>
@@ -56373,7 +56412,7 @@
         <v>46156</v>
       </c>
       <c r="G406" s="5">
-        <v>8</v>
+        <v>454</v>
       </c>
       <c r="H406" s="3" t="s">
         <v>47</v>
@@ -56388,19 +56427,19 @@
         <v>50</v>
       </c>
       <c r="L406" s="6">
-        <v>44</v>
+        <v>670</v>
       </c>
       <c r="M406" s="7">
-        <v>19785.66</v>
+        <v>132418.29</v>
       </c>
       <c r="N406" s="6">
         <v>1</v>
       </c>
       <c r="O406" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P406" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q406" s="6">
         <v>0</v>
@@ -56415,7 +56454,7 @@
         <v>52</v>
       </c>
       <c r="U406" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V406" s="11">
         <v>11</v>
@@ -56424,7 +56463,7 @@
         <v>46156</v>
       </c>
       <c r="X406" s="12">
-        <v>0.46180559999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y406" s="10">
         <v>0</v>
@@ -56457,7 +56496,7 @@
         <v>53</v>
       </c>
       <c r="AI406" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ406" s="3" t="s">
         <v>52</v>
@@ -56484,7 +56523,7 @@
         <v>53</v>
       </c>
       <c r="AR406" s="3" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="407" spans="1:44" x14ac:dyDescent="0.3">
@@ -56495,7 +56534,7 @@
         <v>2</v>
       </c>
       <c r="C407" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D407" s="3" t="s">
         <v>45</v>
@@ -56507,7 +56546,7 @@
         <v>46156</v>
       </c>
       <c r="G407" s="5">
-        <v>9</v>
+        <v>455</v>
       </c>
       <c r="H407" s="3" t="s">
         <v>47</v>
@@ -56522,19 +56561,19 @@
         <v>50</v>
       </c>
       <c r="L407" s="6">
-        <v>45</v>
+        <v>671</v>
       </c>
       <c r="M407" s="7">
-        <v>20235.330000000002</v>
+        <v>132615.93</v>
       </c>
       <c r="N407" s="6">
         <v>1</v>
       </c>
       <c r="O407" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P407" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q407" s="6">
         <v>0</v>
@@ -56549,7 +56588,7 @@
         <v>52</v>
       </c>
       <c r="U407" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V407" s="11">
         <v>11</v>
@@ -56558,7 +56597,7 @@
         <v>46156</v>
       </c>
       <c r="X407" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y407" s="10">
         <v>0</v>
@@ -56591,7 +56630,7 @@
         <v>53</v>
       </c>
       <c r="AI407" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ407" s="3" t="s">
         <v>52</v>
@@ -56618,7 +56657,7 @@
         <v>53</v>
       </c>
       <c r="AR407" s="3" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="408" spans="1:44" x14ac:dyDescent="0.3">
@@ -56629,7 +56668,7 @@
         <v>2</v>
       </c>
       <c r="C408" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D408" s="3" t="s">
         <v>45</v>
@@ -56641,7 +56680,7 @@
         <v>46156</v>
       </c>
       <c r="G408" s="5">
-        <v>10</v>
+        <v>456</v>
       </c>
       <c r="H408" s="3" t="s">
         <v>47</v>
@@ -56656,19 +56695,19 @@
         <v>50</v>
       </c>
       <c r="L408" s="6">
-        <v>46</v>
+        <v>672</v>
       </c>
       <c r="M408" s="7">
-        <v>20685</v>
+        <v>132813.57</v>
       </c>
       <c r="N408" s="6">
         <v>1</v>
       </c>
       <c r="O408" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P408" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q408" s="6">
         <v>0</v>
@@ -56683,7 +56722,7 @@
         <v>52</v>
       </c>
       <c r="U408" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V408" s="11">
         <v>11</v>
@@ -56692,7 +56731,7 @@
         <v>46156</v>
       </c>
       <c r="X408" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y408" s="10">
         <v>0</v>
@@ -56725,7 +56764,7 @@
         <v>53</v>
       </c>
       <c r="AI408" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ408" s="3" t="s">
         <v>52</v>
@@ -56752,7 +56791,7 @@
         <v>53</v>
       </c>
       <c r="AR408" s="3" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="409" spans="1:44" x14ac:dyDescent="0.3">
@@ -56763,7 +56802,7 @@
         <v>2</v>
       </c>
       <c r="C409" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D409" s="3" t="s">
         <v>45</v>
@@ -56775,7 +56814,7 @@
         <v>46156</v>
       </c>
       <c r="G409" s="5">
-        <v>11</v>
+        <v>457</v>
       </c>
       <c r="H409" s="3" t="s">
         <v>47</v>
@@ -56790,19 +56829,19 @@
         <v>50</v>
       </c>
       <c r="L409" s="6">
-        <v>47</v>
+        <v>673</v>
       </c>
       <c r="M409" s="7">
-        <v>21134.68</v>
+        <v>133011.21</v>
       </c>
       <c r="N409" s="6">
         <v>1</v>
       </c>
       <c r="O409" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P409" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q409" s="6">
         <v>0</v>
@@ -56817,7 +56856,7 @@
         <v>52</v>
       </c>
       <c r="U409" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V409" s="11">
         <v>11</v>
@@ -56826,7 +56865,7 @@
         <v>46156</v>
       </c>
       <c r="X409" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y409" s="10">
         <v>0</v>
@@ -56859,7 +56898,7 @@
         <v>53</v>
       </c>
       <c r="AI409" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ409" s="3" t="s">
         <v>52</v>
@@ -56886,7 +56925,7 @@
         <v>53</v>
       </c>
       <c r="AR409" s="3" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="410" spans="1:44" x14ac:dyDescent="0.3">
@@ -56897,7 +56936,7 @@
         <v>2</v>
       </c>
       <c r="C410" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D410" s="3" t="s">
         <v>45</v>
@@ -56909,7 +56948,7 @@
         <v>46156</v>
       </c>
       <c r="G410" s="5">
-        <v>12</v>
+        <v>458</v>
       </c>
       <c r="H410" s="3" t="s">
         <v>47</v>
@@ -56924,19 +56963,19 @@
         <v>50</v>
       </c>
       <c r="L410" s="6">
-        <v>48</v>
+        <v>674</v>
       </c>
       <c r="M410" s="7">
-        <v>21584.35</v>
+        <v>133208.85</v>
       </c>
       <c r="N410" s="6">
         <v>1</v>
       </c>
       <c r="O410" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P410" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q410" s="6">
         <v>0</v>
@@ -56951,7 +56990,7 @@
         <v>52</v>
       </c>
       <c r="U410" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V410" s="11">
         <v>11</v>
@@ -56960,7 +56999,7 @@
         <v>46156</v>
       </c>
       <c r="X410" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y410" s="10">
         <v>0</v>
@@ -56993,7 +57032,7 @@
         <v>53</v>
       </c>
       <c r="AI410" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ410" s="3" t="s">
         <v>52</v>
@@ -57020,7 +57059,7 @@
         <v>53</v>
       </c>
       <c r="AR410" s="3" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="411" spans="1:44" x14ac:dyDescent="0.3">
@@ -57031,7 +57070,7 @@
         <v>2</v>
       </c>
       <c r="C411" s="3" t="s">
-        <v>452</v>
+        <v>44</v>
       </c>
       <c r="D411" s="3" t="s">
         <v>45</v>
@@ -57043,7 +57082,7 @@
         <v>46156</v>
       </c>
       <c r="G411" s="5">
-        <v>13</v>
+        <v>459</v>
       </c>
       <c r="H411" s="3" t="s">
         <v>47</v>
@@ -57058,19 +57097,19 @@
         <v>50</v>
       </c>
       <c r="L411" s="6">
-        <v>49</v>
+        <v>675</v>
       </c>
       <c r="M411" s="7">
-        <v>22034.03</v>
+        <v>133406.49</v>
       </c>
       <c r="N411" s="6">
         <v>1</v>
       </c>
       <c r="O411" s="3" t="s">
-        <v>453</v>
+        <v>51</v>
       </c>
       <c r="P411" s="8">
-        <v>449.67</v>
+        <v>197.64</v>
       </c>
       <c r="Q411" s="6">
         <v>0</v>
@@ -57085,7 +57124,7 @@
         <v>52</v>
       </c>
       <c r="U411" s="10">
-        <v>64218</v>
+        <v>64344</v>
       </c>
       <c r="V411" s="11">
         <v>11</v>
@@ -57094,7 +57133,7 @@
         <v>46156</v>
       </c>
       <c r="X411" s="12">
-        <v>0.54513889999999998</v>
+        <v>0.59166669999999999</v>
       </c>
       <c r="Y411" s="10">
         <v>0</v>
@@ -57127,7 +57166,7 @@
         <v>53</v>
       </c>
       <c r="AI411" s="3" t="s">
-        <v>454</v>
+        <v>54</v>
       </c>
       <c r="AJ411" s="3" t="s">
         <v>52</v>
@@ -57154,7 +57193,7 @@
         <v>53</v>
       </c>
       <c r="AR411" s="3" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="412" spans="1:44" x14ac:dyDescent="0.3">
@@ -57165,7 +57204,7 @@
         <v>2</v>
       </c>
       <c r="C412" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D412" s="3" t="s">
         <v>45</v>
@@ -57177,7 +57216,7 @@
         <v>46156</v>
       </c>
       <c r="G412" s="5">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H412" s="3" t="s">
         <v>47</v>
@@ -57192,16 +57231,16 @@
         <v>50</v>
       </c>
       <c r="L412" s="6">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="M412" s="7">
-        <v>22483.7</v>
+        <v>16637.939999999999</v>
       </c>
       <c r="N412" s="6">
         <v>1</v>
       </c>
       <c r="O412" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P412" s="8">
         <v>449.67</v>
@@ -57228,7 +57267,7 @@
         <v>46156</v>
       </c>
       <c r="X412" s="12">
-        <v>0.54513889999999998</v>
+        <v>0.37847219999999998</v>
       </c>
       <c r="Y412" s="10">
         <v>0</v>
@@ -57261,7 +57300,7 @@
         <v>53</v>
       </c>
       <c r="AI412" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ412" s="3" t="s">
         <v>52</v>
@@ -57299,7 +57338,7 @@
         <v>2</v>
       </c>
       <c r="C413" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D413" s="3" t="s">
         <v>45</v>
@@ -57311,7 +57350,7 @@
         <v>46156</v>
       </c>
       <c r="G413" s="5">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H413" s="3" t="s">
         <v>47</v>
@@ -57326,16 +57365,16 @@
         <v>50</v>
       </c>
       <c r="L413" s="6">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="M413" s="7">
-        <v>22933.38</v>
+        <v>17087.61</v>
       </c>
       <c r="N413" s="6">
         <v>1</v>
       </c>
       <c r="O413" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P413" s="8">
         <v>449.67</v>
@@ -57362,7 +57401,7 @@
         <v>46156</v>
       </c>
       <c r="X413" s="12">
-        <v>0.54513889999999998</v>
+        <v>0.42013889999999998</v>
       </c>
       <c r="Y413" s="10">
         <v>0</v>
@@ -57395,7 +57434,7 @@
         <v>53</v>
       </c>
       <c r="AI413" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ413" s="3" t="s">
         <v>52</v>
@@ -57433,7 +57472,7 @@
         <v>2</v>
       </c>
       <c r="C414" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D414" s="3" t="s">
         <v>45</v>
@@ -57445,7 +57484,7 @@
         <v>46156</v>
       </c>
       <c r="G414" s="5">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="H414" s="3" t="s">
         <v>47</v>
@@ -57460,16 +57499,16 @@
         <v>50</v>
       </c>
       <c r="L414" s="6">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="M414" s="7">
-        <v>23383.05</v>
+        <v>17537.29</v>
       </c>
       <c r="N414" s="6">
         <v>1</v>
       </c>
       <c r="O414" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P414" s="8">
         <v>449.67</v>
@@ -57496,7 +57535,7 @@
         <v>46156</v>
       </c>
       <c r="X414" s="12">
-        <v>0.54513889999999998</v>
+        <v>0.44097219999999998</v>
       </c>
       <c r="Y414" s="10">
         <v>0</v>
@@ -57529,7 +57568,7 @@
         <v>53</v>
       </c>
       <c r="AI414" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ414" s="3" t="s">
         <v>52</v>
@@ -57567,7 +57606,7 @@
         <v>2</v>
       </c>
       <c r="C415" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D415" s="3" t="s">
         <v>45</v>
@@ -57579,7 +57618,7 @@
         <v>46156</v>
       </c>
       <c r="G415" s="5">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H415" s="3" t="s">
         <v>47</v>
@@ -57594,16 +57633,16 @@
         <v>50</v>
       </c>
       <c r="L415" s="6">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="M415" s="7">
-        <v>23832.720000000001</v>
+        <v>17986.96</v>
       </c>
       <c r="N415" s="6">
         <v>1</v>
       </c>
       <c r="O415" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P415" s="8">
         <v>449.67</v>
@@ -57630,7 +57669,7 @@
         <v>46156</v>
       </c>
       <c r="X415" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.44097219999999998</v>
       </c>
       <c r="Y415" s="10">
         <v>0</v>
@@ -57663,7 +57702,7 @@
         <v>53</v>
       </c>
       <c r="AI415" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ415" s="3" t="s">
         <v>52</v>
@@ -57701,7 +57740,7 @@
         <v>2</v>
       </c>
       <c r="C416" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D416" s="3" t="s">
         <v>45</v>
@@ -57713,7 +57752,7 @@
         <v>46156</v>
       </c>
       <c r="G416" s="5">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="H416" s="3" t="s">
         <v>47</v>
@@ -57728,16 +57767,16 @@
         <v>50</v>
       </c>
       <c r="L416" s="6">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="M416" s="7">
-        <v>24282.400000000001</v>
+        <v>18436.63</v>
       </c>
       <c r="N416" s="6">
         <v>1</v>
       </c>
       <c r="O416" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P416" s="8">
         <v>449.67</v>
@@ -57764,7 +57803,7 @@
         <v>46156</v>
       </c>
       <c r="X416" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y416" s="10">
         <v>0</v>
@@ -57797,7 +57836,7 @@
         <v>53</v>
       </c>
       <c r="AI416" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ416" s="3" t="s">
         <v>52</v>
@@ -57835,7 +57874,7 @@
         <v>2</v>
       </c>
       <c r="C417" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D417" s="3" t="s">
         <v>45</v>
@@ -57847,7 +57886,7 @@
         <v>46156</v>
       </c>
       <c r="G417" s="5">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H417" s="3" t="s">
         <v>47</v>
@@ -57862,16 +57901,16 @@
         <v>50</v>
       </c>
       <c r="L417" s="6">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="M417" s="7">
-        <v>24732.07</v>
+        <v>18886.310000000001</v>
       </c>
       <c r="N417" s="6">
         <v>1</v>
       </c>
       <c r="O417" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P417" s="8">
         <v>449.67</v>
@@ -57898,7 +57937,7 @@
         <v>46156</v>
       </c>
       <c r="X417" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y417" s="10">
         <v>0</v>
@@ -57931,7 +57970,7 @@
         <v>53</v>
       </c>
       <c r="AI417" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ417" s="3" t="s">
         <v>52</v>
@@ -57969,7 +58008,7 @@
         <v>2</v>
       </c>
       <c r="C418" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D418" s="3" t="s">
         <v>45</v>
@@ -57981,7 +58020,7 @@
         <v>46156</v>
       </c>
       <c r="G418" s="5">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="H418" s="3" t="s">
         <v>47</v>
@@ -57996,16 +58035,16 @@
         <v>50</v>
       </c>
       <c r="L418" s="6">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="M418" s="7">
-        <v>25181.75</v>
+        <v>19335.98</v>
       </c>
       <c r="N418" s="6">
         <v>1</v>
       </c>
       <c r="O418" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P418" s="8">
         <v>449.67</v>
@@ -58032,7 +58071,7 @@
         <v>46156</v>
       </c>
       <c r="X418" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y418" s="10">
         <v>0</v>
@@ -58065,7 +58104,7 @@
         <v>53</v>
       </c>
       <c r="AI418" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ418" s="3" t="s">
         <v>52</v>
@@ -58103,7 +58142,7 @@
         <v>2</v>
       </c>
       <c r="C419" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D419" s="3" t="s">
         <v>45</v>
@@ -58115,7 +58154,7 @@
         <v>46156</v>
       </c>
       <c r="G419" s="5">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="H419" s="3" t="s">
         <v>47</v>
@@ -58130,16 +58169,16 @@
         <v>50</v>
       </c>
       <c r="L419" s="6">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="M419" s="7">
-        <v>25631.42</v>
+        <v>19785.66</v>
       </c>
       <c r="N419" s="6">
         <v>1</v>
       </c>
       <c r="O419" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P419" s="8">
         <v>449.67</v>
@@ -58166,7 +58205,7 @@
         <v>46156</v>
       </c>
       <c r="X419" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y419" s="10">
         <v>0</v>
@@ -58199,7 +58238,7 @@
         <v>53</v>
       </c>
       <c r="AI419" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ419" s="3" t="s">
         <v>52</v>
@@ -58237,7 +58276,7 @@
         <v>2</v>
       </c>
       <c r="C420" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D420" s="3" t="s">
         <v>45</v>
@@ -58249,7 +58288,7 @@
         <v>46156</v>
       </c>
       <c r="G420" s="5">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="H420" s="3" t="s">
         <v>47</v>
@@ -58264,16 +58303,16 @@
         <v>50</v>
       </c>
       <c r="L420" s="6">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="M420" s="7">
-        <v>26081.09</v>
+        <v>20235.330000000002</v>
       </c>
       <c r="N420" s="6">
         <v>1</v>
       </c>
       <c r="O420" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P420" s="8">
         <v>449.67</v>
@@ -58300,7 +58339,7 @@
         <v>46156</v>
       </c>
       <c r="X420" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y420" s="10">
         <v>0</v>
@@ -58333,7 +58372,7 @@
         <v>53</v>
       </c>
       <c r="AI420" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ420" s="3" t="s">
         <v>52</v>
@@ -58371,7 +58410,7 @@
         <v>2</v>
       </c>
       <c r="C421" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D421" s="3" t="s">
         <v>45</v>
@@ -58383,7 +58422,7 @@
         <v>46156</v>
       </c>
       <c r="G421" s="5">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H421" s="3" t="s">
         <v>47</v>
@@ -58398,16 +58437,16 @@
         <v>50</v>
       </c>
       <c r="L421" s="6">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="M421" s="7">
-        <v>26530.77</v>
+        <v>20685</v>
       </c>
       <c r="N421" s="6">
         <v>1</v>
       </c>
       <c r="O421" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P421" s="8">
         <v>449.67</v>
@@ -58434,7 +58473,7 @@
         <v>46156</v>
       </c>
       <c r="X421" s="12">
-        <v>0.56597220000000004</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y421" s="10">
         <v>0</v>
@@ -58467,7 +58506,7 @@
         <v>53</v>
       </c>
       <c r="AI421" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ421" s="3" t="s">
         <v>52</v>
@@ -58505,7 +58544,7 @@
         <v>2</v>
       </c>
       <c r="C422" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D422" s="3" t="s">
         <v>45</v>
@@ -58517,7 +58556,7 @@
         <v>46156</v>
       </c>
       <c r="G422" s="5">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H422" s="3" t="s">
         <v>47</v>
@@ -58532,16 +58571,16 @@
         <v>50</v>
       </c>
       <c r="L422" s="6">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="M422" s="7">
-        <v>26980.44</v>
+        <v>21134.68</v>
       </c>
       <c r="N422" s="6">
         <v>1</v>
       </c>
       <c r="O422" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P422" s="8">
         <v>449.67</v>
@@ -58568,7 +58607,7 @@
         <v>46156</v>
       </c>
       <c r="X422" s="12">
-        <v>0.58680560000000004</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y422" s="10">
         <v>0</v>
@@ -58601,7 +58640,7 @@
         <v>53</v>
       </c>
       <c r="AI422" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ422" s="3" t="s">
         <v>52</v>
@@ -58639,7 +58678,7 @@
         <v>2</v>
       </c>
       <c r="C423" s="3" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="D423" s="3" t="s">
         <v>45</v>
@@ -58651,7 +58690,7 @@
         <v>46156</v>
       </c>
       <c r="G423" s="5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H423" s="3" t="s">
         <v>47</v>
@@ -58666,16 +58705,16 @@
         <v>50</v>
       </c>
       <c r="L423" s="6">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="M423" s="7">
-        <v>27430.12</v>
+        <v>21584.35</v>
       </c>
       <c r="N423" s="6">
         <v>1</v>
       </c>
       <c r="O423" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="P423" s="8">
         <v>449.67</v>
@@ -58702,7 +58741,7 @@
         <v>46156</v>
       </c>
       <c r="X423" s="12">
-        <v>0.58680560000000004</v>
+        <v>0.48263889999999998</v>
       </c>
       <c r="Y423" s="10">
         <v>0</v>
@@ -58735,7 +58774,7 @@
         <v>53</v>
       </c>
       <c r="AI423" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ423" s="3" t="s">
         <v>52</v>
@@ -58773,7 +58812,7 @@
         <v>2</v>
       </c>
       <c r="C424" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D424" s="3" t="s">
         <v>45</v>
@@ -58785,7 +58824,7 @@
         <v>46156</v>
       </c>
       <c r="G424" s="5">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H424" s="3" t="s">
         <v>47</v>
@@ -58800,19 +58839,19 @@
         <v>50</v>
       </c>
       <c r="L424" s="6">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="M424" s="7">
-        <v>26267.89</v>
+        <v>22034.03</v>
       </c>
       <c r="N424" s="6">
         <v>1</v>
       </c>
       <c r="O424" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P424" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q424" s="6">
         <v>0</v>
@@ -58827,7 +58866,7 @@
         <v>52</v>
       </c>
       <c r="U424" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V424" s="11">
         <v>11</v>
@@ -58836,7 +58875,7 @@
         <v>46156</v>
       </c>
       <c r="X424" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.54513889999999998</v>
       </c>
       <c r="Y424" s="10">
         <v>0</v>
@@ -58869,7 +58908,7 @@
         <v>53</v>
       </c>
       <c r="AI424" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ424" s="3" t="s">
         <v>52</v>
@@ -58896,7 +58935,7 @@
         <v>53</v>
       </c>
       <c r="AR424" s="3" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="425" spans="1:44" x14ac:dyDescent="0.3">
@@ -58907,7 +58946,7 @@
         <v>2</v>
       </c>
       <c r="C425" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D425" s="3" t="s">
         <v>45</v>
@@ -58919,7 +58958,7 @@
         <v>46156</v>
       </c>
       <c r="G425" s="5">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H425" s="3" t="s">
         <v>47</v>
@@ -58934,19 +58973,19 @@
         <v>50</v>
       </c>
       <c r="L425" s="6">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="M425" s="7">
-        <v>26648.59</v>
+        <v>22483.7</v>
       </c>
       <c r="N425" s="6">
         <v>1</v>
       </c>
       <c r="O425" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P425" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q425" s="6">
         <v>0</v>
@@ -58961,7 +59000,7 @@
         <v>52</v>
       </c>
       <c r="U425" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V425" s="11">
         <v>11</v>
@@ -58970,7 +59009,7 @@
         <v>46156</v>
       </c>
       <c r="X425" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.54513889999999998</v>
       </c>
       <c r="Y425" s="10">
         <v>0</v>
@@ -59003,7 +59042,7 @@
         <v>53</v>
       </c>
       <c r="AI425" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ425" s="3" t="s">
         <v>52</v>
@@ -59030,7 +59069,7 @@
         <v>53</v>
       </c>
       <c r="AR425" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="426" spans="1:44" x14ac:dyDescent="0.3">
@@ -59041,7 +59080,7 @@
         <v>2</v>
       </c>
       <c r="C426" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D426" s="3" t="s">
         <v>45</v>
@@ -59053,7 +59092,7 @@
         <v>46156</v>
       </c>
       <c r="G426" s="5">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="H426" s="3" t="s">
         <v>47</v>
@@ -59068,19 +59107,19 @@
         <v>50</v>
       </c>
       <c r="L426" s="6">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="M426" s="7">
-        <v>27029.279999999999</v>
+        <v>22933.38</v>
       </c>
       <c r="N426" s="6">
         <v>1</v>
       </c>
       <c r="O426" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P426" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q426" s="6">
         <v>0</v>
@@ -59095,7 +59134,7 @@
         <v>52</v>
       </c>
       <c r="U426" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V426" s="11">
         <v>11</v>
@@ -59104,7 +59143,7 @@
         <v>46156</v>
       </c>
       <c r="X426" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.54513889999999998</v>
       </c>
       <c r="Y426" s="10">
         <v>0</v>
@@ -59137,7 +59176,7 @@
         <v>53</v>
       </c>
       <c r="AI426" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ426" s="3" t="s">
         <v>52</v>
@@ -59164,7 +59203,7 @@
         <v>53</v>
       </c>
       <c r="AR426" s="3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="427" spans="1:44" x14ac:dyDescent="0.3">
@@ -59175,7 +59214,7 @@
         <v>2</v>
       </c>
       <c r="C427" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D427" s="3" t="s">
         <v>45</v>
@@ -59187,7 +59226,7 @@
         <v>46156</v>
       </c>
       <c r="G427" s="5">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H427" s="3" t="s">
         <v>47</v>
@@ -59202,19 +59241,19 @@
         <v>50</v>
       </c>
       <c r="L427" s="6">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="M427" s="7">
-        <v>27409.98</v>
+        <v>23383.05</v>
       </c>
       <c r="N427" s="6">
         <v>1</v>
       </c>
       <c r="O427" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P427" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q427" s="6">
         <v>0</v>
@@ -59229,7 +59268,7 @@
         <v>52</v>
       </c>
       <c r="U427" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V427" s="11">
         <v>11</v>
@@ -59238,7 +59277,7 @@
         <v>46156</v>
       </c>
       <c r="X427" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.54513889999999998</v>
       </c>
       <c r="Y427" s="10">
         <v>0</v>
@@ -59271,7 +59310,7 @@
         <v>53</v>
       </c>
       <c r="AI427" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ427" s="3" t="s">
         <v>52</v>
@@ -59298,7 +59337,7 @@
         <v>53</v>
       </c>
       <c r="AR427" s="3" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="428" spans="1:44" x14ac:dyDescent="0.3">
@@ -59309,7 +59348,7 @@
         <v>2</v>
       </c>
       <c r="C428" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D428" s="3" t="s">
         <v>45</v>
@@ -59321,7 +59360,7 @@
         <v>46156</v>
       </c>
       <c r="G428" s="5">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H428" s="3" t="s">
         <v>47</v>
@@ -59336,19 +59375,19 @@
         <v>50</v>
       </c>
       <c r="L428" s="6">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="M428" s="7">
-        <v>27790.67</v>
+        <v>23832.720000000001</v>
       </c>
       <c r="N428" s="6">
         <v>1</v>
       </c>
       <c r="O428" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P428" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q428" s="6">
         <v>0</v>
@@ -59363,7 +59402,7 @@
         <v>52</v>
       </c>
       <c r="U428" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V428" s="11">
         <v>11</v>
@@ -59372,7 +59411,7 @@
         <v>46156</v>
       </c>
       <c r="X428" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y428" s="10">
         <v>0</v>
@@ -59405,7 +59444,7 @@
         <v>53</v>
       </c>
       <c r="AI428" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ428" s="3" t="s">
         <v>52</v>
@@ -59432,7 +59471,7 @@
         <v>53</v>
       </c>
       <c r="AR428" s="3" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="429" spans="1:44" x14ac:dyDescent="0.3">
@@ -59443,7 +59482,7 @@
         <v>2</v>
       </c>
       <c r="C429" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D429" s="3" t="s">
         <v>45</v>
@@ -59455,7 +59494,7 @@
         <v>46156</v>
       </c>
       <c r="G429" s="5">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H429" s="3" t="s">
         <v>47</v>
@@ -59470,19 +59509,19 @@
         <v>50</v>
       </c>
       <c r="L429" s="6">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="M429" s="7">
-        <v>28171.360000000001</v>
+        <v>24282.400000000001</v>
       </c>
       <c r="N429" s="6">
         <v>1</v>
       </c>
       <c r="O429" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P429" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q429" s="6">
         <v>0</v>
@@ -59497,7 +59536,7 @@
         <v>52</v>
       </c>
       <c r="U429" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V429" s="11">
         <v>11</v>
@@ -59506,7 +59545,7 @@
         <v>46156</v>
       </c>
       <c r="X429" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y429" s="10">
         <v>0</v>
@@ -59539,7 +59578,7 @@
         <v>53</v>
       </c>
       <c r="AI429" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ429" s="3" t="s">
         <v>52</v>
@@ -59566,7 +59605,7 @@
         <v>53</v>
       </c>
       <c r="AR429" s="3" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="430" spans="1:44" x14ac:dyDescent="0.3">
@@ -59577,7 +59616,7 @@
         <v>2</v>
       </c>
       <c r="C430" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D430" s="3" t="s">
         <v>45</v>
@@ -59589,7 +59628,7 @@
         <v>46156</v>
       </c>
       <c r="G430" s="5">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="H430" s="3" t="s">
         <v>47</v>
@@ -59604,19 +59643,19 @@
         <v>50</v>
       </c>
       <c r="L430" s="6">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="M430" s="7">
-        <v>28552.06</v>
+        <v>24732.07</v>
       </c>
       <c r="N430" s="6">
         <v>1</v>
       </c>
       <c r="O430" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P430" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q430" s="6">
         <v>0</v>
@@ -59631,7 +59670,7 @@
         <v>52</v>
       </c>
       <c r="U430" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V430" s="11">
         <v>11</v>
@@ -59640,7 +59679,7 @@
         <v>46156</v>
       </c>
       <c r="X430" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y430" s="10">
         <v>0</v>
@@ -59673,7 +59712,7 @@
         <v>53</v>
       </c>
       <c r="AI430" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ430" s="3" t="s">
         <v>52</v>
@@ -59700,7 +59739,7 @@
         <v>53</v>
       </c>
       <c r="AR430" s="3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="431" spans="1:44" x14ac:dyDescent="0.3">
@@ -59711,7 +59750,7 @@
         <v>2</v>
       </c>
       <c r="C431" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D431" s="3" t="s">
         <v>45</v>
@@ -59723,7 +59762,7 @@
         <v>46156</v>
       </c>
       <c r="G431" s="5">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="H431" s="3" t="s">
         <v>47</v>
@@ -59738,19 +59777,19 @@
         <v>50</v>
       </c>
       <c r="L431" s="6">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="M431" s="7">
-        <v>28932.75</v>
+        <v>25181.75</v>
       </c>
       <c r="N431" s="6">
         <v>1</v>
       </c>
       <c r="O431" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P431" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q431" s="6">
         <v>0</v>
@@ -59765,7 +59804,7 @@
         <v>52</v>
       </c>
       <c r="U431" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V431" s="11">
         <v>11</v>
@@ -59774,7 +59813,7 @@
         <v>46156</v>
       </c>
       <c r="X431" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y431" s="10">
         <v>0</v>
@@ -59807,7 +59846,7 @@
         <v>53</v>
       </c>
       <c r="AI431" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ431" s="3" t="s">
         <v>52</v>
@@ -59834,7 +59873,7 @@
         <v>53</v>
       </c>
       <c r="AR431" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="432" spans="1:44" x14ac:dyDescent="0.3">
@@ -59845,7 +59884,7 @@
         <v>2</v>
       </c>
       <c r="C432" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D432" s="3" t="s">
         <v>45</v>
@@ -59857,7 +59896,7 @@
         <v>46156</v>
       </c>
       <c r="G432" s="5">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H432" s="3" t="s">
         <v>47</v>
@@ -59872,19 +59911,19 @@
         <v>50</v>
       </c>
       <c r="L432" s="6">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="M432" s="7">
-        <v>29313.45</v>
+        <v>25631.42</v>
       </c>
       <c r="N432" s="6">
         <v>1</v>
       </c>
       <c r="O432" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P432" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q432" s="6">
         <v>0</v>
@@ -59899,7 +59938,7 @@
         <v>52</v>
       </c>
       <c r="U432" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V432" s="11">
         <v>11</v>
@@ -59908,7 +59947,7 @@
         <v>46156</v>
       </c>
       <c r="X432" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y432" s="10">
         <v>0</v>
@@ -59941,7 +59980,7 @@
         <v>53</v>
       </c>
       <c r="AI432" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ432" s="3" t="s">
         <v>52</v>
@@ -59968,7 +60007,7 @@
         <v>53</v>
       </c>
       <c r="AR432" s="3" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="433" spans="1:44" x14ac:dyDescent="0.3">
@@ -59979,7 +60018,7 @@
         <v>2</v>
       </c>
       <c r="C433" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D433" s="3" t="s">
         <v>45</v>
@@ -59991,7 +60030,7 @@
         <v>46156</v>
       </c>
       <c r="G433" s="5">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H433" s="3" t="s">
         <v>47</v>
@@ -60006,19 +60045,19 @@
         <v>50</v>
       </c>
       <c r="L433" s="6">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="M433" s="7">
-        <v>29694.14</v>
+        <v>26081.09</v>
       </c>
       <c r="N433" s="6">
         <v>1</v>
       </c>
       <c r="O433" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P433" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q433" s="6">
         <v>0</v>
@@ -60033,7 +60072,7 @@
         <v>52</v>
       </c>
       <c r="U433" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V433" s="11">
         <v>11</v>
@@ -60042,7 +60081,7 @@
         <v>46156</v>
       </c>
       <c r="X433" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y433" s="10">
         <v>0</v>
@@ -60075,7 +60114,7 @@
         <v>53</v>
       </c>
       <c r="AI433" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ433" s="3" t="s">
         <v>52</v>
@@ -60102,7 +60141,7 @@
         <v>53</v>
       </c>
       <c r="AR433" s="3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="434" spans="1:44" x14ac:dyDescent="0.3">
@@ -60113,7 +60152,7 @@
         <v>2</v>
       </c>
       <c r="C434" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D434" s="3" t="s">
         <v>45</v>
@@ -60125,7 +60164,7 @@
         <v>46156</v>
       </c>
       <c r="G434" s="5">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="H434" s="3" t="s">
         <v>47</v>
@@ -60140,19 +60179,19 @@
         <v>50</v>
       </c>
       <c r="L434" s="6">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="M434" s="7">
-        <v>30074.83</v>
+        <v>26530.77</v>
       </c>
       <c r="N434" s="6">
         <v>1</v>
       </c>
       <c r="O434" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P434" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q434" s="6">
         <v>0</v>
@@ -60167,7 +60206,7 @@
         <v>52</v>
       </c>
       <c r="U434" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V434" s="11">
         <v>11</v>
@@ -60176,7 +60215,7 @@
         <v>46156</v>
       </c>
       <c r="X434" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.56597220000000004</v>
       </c>
       <c r="Y434" s="10">
         <v>0</v>
@@ -60209,7 +60248,7 @@
         <v>53</v>
       </c>
       <c r="AI434" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ434" s="3" t="s">
         <v>52</v>
@@ -60236,7 +60275,7 @@
         <v>53</v>
       </c>
       <c r="AR434" s="3" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="435" spans="1:44" x14ac:dyDescent="0.3">
@@ -60247,7 +60286,7 @@
         <v>2</v>
       </c>
       <c r="C435" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D435" s="3" t="s">
         <v>45</v>
@@ -60259,7 +60298,7 @@
         <v>46156</v>
       </c>
       <c r="G435" s="5">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="H435" s="3" t="s">
         <v>47</v>
@@ -60274,19 +60313,19 @@
         <v>50</v>
       </c>
       <c r="L435" s="6">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="M435" s="7">
-        <v>30455.53</v>
+        <v>26980.44</v>
       </c>
       <c r="N435" s="6">
         <v>1</v>
       </c>
       <c r="O435" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P435" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q435" s="6">
         <v>0</v>
@@ -60301,7 +60340,7 @@
         <v>52</v>
       </c>
       <c r="U435" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V435" s="11">
         <v>11</v>
@@ -60310,7 +60349,7 @@
         <v>46156</v>
       </c>
       <c r="X435" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.58680560000000004</v>
       </c>
       <c r="Y435" s="10">
         <v>0</v>
@@ -60343,7 +60382,7 @@
         <v>53</v>
       </c>
       <c r="AI435" s="3" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="AJ435" s="3" t="s">
         <v>52</v>
@@ -60370,7 +60409,7 @@
         <v>53</v>
       </c>
       <c r="AR435" s="3" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="436" spans="1:44" x14ac:dyDescent="0.3">
@@ -60381,7 +60420,7 @@
         <v>2</v>
       </c>
       <c r="C436" s="3" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D436" s="3" t="s">
         <v>45</v>
@@ -60393,7 +60432,7 @@
         <v>46156</v>
       </c>
       <c r="G436" s="5">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H436" s="3" t="s">
         <v>47</v>
@@ -60408,19 +60447,19 @@
         <v>50</v>
       </c>
       <c r="L436" s="6">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="M436" s="7">
-        <v>30836.22</v>
+        <v>27430.12</v>
       </c>
       <c r="N436" s="6">
         <v>1</v>
       </c>
       <c r="O436" s="3" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P436" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q436" s="6">
         <v>0</v>
@@ -60435,7 +60474,7 @@
         <v>52</v>
       </c>
       <c r="U436" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V436" s="11">
         <v>11</v>
@@ -60444,67 +60483,1809 @@
         <v>46156</v>
       </c>
       <c r="X436" s="12">
+        <v>0.58680560000000004</v>
+      </c>
+      <c r="Y436" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z436" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA436" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB436" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC436" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD436" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE436" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF436" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG436" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH436" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI436" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ436" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK436" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL436" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM436" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN436" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO436" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP436" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ436" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR436" s="3" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="437" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A437" s="1">
+        <v>1</v>
+      </c>
+      <c r="B437" s="2">
+        <v>2</v>
+      </c>
+      <c r="C437" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D437" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E437" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F437" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G437" s="5">
+        <v>1</v>
+      </c>
+      <c r="H437" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I437" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J437" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K437" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L437" s="6">
+        <v>69</v>
+      </c>
+      <c r="M437" s="7">
+        <v>26267.89</v>
+      </c>
+      <c r="N437" s="6">
+        <v>1</v>
+      </c>
+      <c r="O437" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P437" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q437" s="6">
+        <v>0</v>
+      </c>
+      <c r="R437" s="7">
+        <v>0</v>
+      </c>
+      <c r="S437" s="9">
+        <v>0</v>
+      </c>
+      <c r="T437" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U437" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V437" s="11">
+        <v>11</v>
+      </c>
+      <c r="W437" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X437" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y437" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z437" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA437" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB437" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC437" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD437" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE437" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF437" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG437" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH437" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI437" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ437" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK437" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL437" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM437" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN437" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO437" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP437" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ437" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR437" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="438" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A438" s="1">
+        <v>1</v>
+      </c>
+      <c r="B438" s="2">
+        <v>2</v>
+      </c>
+      <c r="C438" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D438" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E438" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F438" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G438" s="5">
+        <v>2</v>
+      </c>
+      <c r="H438" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I438" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J438" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K438" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L438" s="6">
+        <v>70</v>
+      </c>
+      <c r="M438" s="7">
+        <v>26648.59</v>
+      </c>
+      <c r="N438" s="6">
+        <v>1</v>
+      </c>
+      <c r="O438" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P438" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q438" s="6">
+        <v>0</v>
+      </c>
+      <c r="R438" s="7">
+        <v>0</v>
+      </c>
+      <c r="S438" s="9">
+        <v>0</v>
+      </c>
+      <c r="T438" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U438" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V438" s="11">
+        <v>11</v>
+      </c>
+      <c r="W438" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X438" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y438" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z438" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA438" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB438" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC438" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD438" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE438" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF438" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG438" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH438" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI438" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ438" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK438" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL438" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM438" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN438" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO438" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP438" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ438" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR438" s="3" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="439" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A439" s="1">
+        <v>1</v>
+      </c>
+      <c r="B439" s="2">
+        <v>2</v>
+      </c>
+      <c r="C439" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D439" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E439" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F439" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G439" s="5">
+        <v>3</v>
+      </c>
+      <c r="H439" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I439" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J439" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K439" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L439" s="6">
+        <v>71</v>
+      </c>
+      <c r="M439" s="7">
+        <v>27029.279999999999</v>
+      </c>
+      <c r="N439" s="6">
+        <v>1</v>
+      </c>
+      <c r="O439" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P439" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q439" s="6">
+        <v>0</v>
+      </c>
+      <c r="R439" s="7">
+        <v>0</v>
+      </c>
+      <c r="S439" s="9">
+        <v>0</v>
+      </c>
+      <c r="T439" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U439" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V439" s="11">
+        <v>11</v>
+      </c>
+      <c r="W439" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X439" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y439" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z439" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA439" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB439" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC439" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD439" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE439" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF439" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG439" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH439" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI439" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ439" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK439" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL439" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM439" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN439" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO439" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP439" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ439" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR439" s="3" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="440" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A440" s="1">
+        <v>1</v>
+      </c>
+      <c r="B440" s="2">
+        <v>2</v>
+      </c>
+      <c r="C440" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D440" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E440" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F440" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G440" s="5">
+        <v>4</v>
+      </c>
+      <c r="H440" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I440" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J440" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K440" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L440" s="6">
+        <v>72</v>
+      </c>
+      <c r="M440" s="7">
+        <v>27409.98</v>
+      </c>
+      <c r="N440" s="6">
+        <v>1</v>
+      </c>
+      <c r="O440" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P440" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q440" s="6">
+        <v>0</v>
+      </c>
+      <c r="R440" s="7">
+        <v>0</v>
+      </c>
+      <c r="S440" s="9">
+        <v>0</v>
+      </c>
+      <c r="T440" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U440" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V440" s="11">
+        <v>11</v>
+      </c>
+      <c r="W440" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X440" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y440" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z440" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA440" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB440" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC440" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD440" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE440" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF440" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG440" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH440" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI440" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ440" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK440" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL440" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM440" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN440" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO440" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP440" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ440" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR440" s="3" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="441" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A441" s="1">
+        <v>1</v>
+      </c>
+      <c r="B441" s="2">
+        <v>2</v>
+      </c>
+      <c r="C441" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D441" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E441" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F441" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G441" s="5">
+        <v>5</v>
+      </c>
+      <c r="H441" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I441" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J441" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K441" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L441" s="6">
+        <v>73</v>
+      </c>
+      <c r="M441" s="7">
+        <v>27790.67</v>
+      </c>
+      <c r="N441" s="6">
+        <v>1</v>
+      </c>
+      <c r="O441" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P441" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q441" s="6">
+        <v>0</v>
+      </c>
+      <c r="R441" s="7">
+        <v>0</v>
+      </c>
+      <c r="S441" s="9">
+        <v>0</v>
+      </c>
+      <c r="T441" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U441" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V441" s="11">
+        <v>11</v>
+      </c>
+      <c r="W441" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X441" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y441" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z441" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA441" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB441" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC441" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD441" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE441" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF441" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG441" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH441" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI441" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ441" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK441" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL441" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM441" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN441" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO441" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP441" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ441" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR441" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="442" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A442" s="1">
+        <v>1</v>
+      </c>
+      <c r="B442" s="2">
+        <v>2</v>
+      </c>
+      <c r="C442" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D442" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E442" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F442" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G442" s="5">
+        <v>6</v>
+      </c>
+      <c r="H442" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I442" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J442" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K442" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L442" s="6">
+        <v>74</v>
+      </c>
+      <c r="M442" s="7">
+        <v>28171.360000000001</v>
+      </c>
+      <c r="N442" s="6">
+        <v>1</v>
+      </c>
+      <c r="O442" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P442" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q442" s="6">
+        <v>0</v>
+      </c>
+      <c r="R442" s="7">
+        <v>0</v>
+      </c>
+      <c r="S442" s="9">
+        <v>0</v>
+      </c>
+      <c r="T442" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U442" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V442" s="11">
+        <v>11</v>
+      </c>
+      <c r="W442" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X442" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y442" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z442" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA442" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB442" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC442" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD442" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE442" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF442" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG442" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH442" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI442" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ442" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK442" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL442" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM442" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN442" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO442" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP442" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ442" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR442" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="443" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A443" s="1">
+        <v>1</v>
+      </c>
+      <c r="B443" s="2">
+        <v>2</v>
+      </c>
+      <c r="C443" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D443" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E443" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F443" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G443" s="5">
+        <v>7</v>
+      </c>
+      <c r="H443" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I443" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J443" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K443" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L443" s="6">
+        <v>75</v>
+      </c>
+      <c r="M443" s="7">
+        <v>28552.06</v>
+      </c>
+      <c r="N443" s="6">
+        <v>1</v>
+      </c>
+      <c r="O443" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P443" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q443" s="6">
+        <v>0</v>
+      </c>
+      <c r="R443" s="7">
+        <v>0</v>
+      </c>
+      <c r="S443" s="9">
+        <v>0</v>
+      </c>
+      <c r="T443" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U443" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V443" s="11">
+        <v>11</v>
+      </c>
+      <c r="W443" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X443" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y443" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z443" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA443" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB443" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC443" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD443" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE443" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF443" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG443" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH443" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI443" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ443" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK443" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL443" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM443" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN443" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO443" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP443" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ443" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR443" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="444" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A444" s="1">
+        <v>1</v>
+      </c>
+      <c r="B444" s="2">
+        <v>2</v>
+      </c>
+      <c r="C444" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D444" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E444" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F444" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G444" s="5">
+        <v>8</v>
+      </c>
+      <c r="H444" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I444" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J444" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K444" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L444" s="6">
+        <v>76</v>
+      </c>
+      <c r="M444" s="7">
+        <v>28932.75</v>
+      </c>
+      <c r="N444" s="6">
+        <v>1</v>
+      </c>
+      <c r="O444" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P444" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q444" s="6">
+        <v>0</v>
+      </c>
+      <c r="R444" s="7">
+        <v>0</v>
+      </c>
+      <c r="S444" s="9">
+        <v>0</v>
+      </c>
+      <c r="T444" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U444" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V444" s="11">
+        <v>11</v>
+      </c>
+      <c r="W444" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X444" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y444" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z444" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA444" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB444" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC444" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD444" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE444" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF444" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG444" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH444" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI444" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ444" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK444" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL444" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM444" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN444" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO444" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP444" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ444" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR444" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="445" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A445" s="1">
+        <v>1</v>
+      </c>
+      <c r="B445" s="2">
+        <v>2</v>
+      </c>
+      <c r="C445" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D445" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E445" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F445" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G445" s="5">
+        <v>9</v>
+      </c>
+      <c r="H445" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I445" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J445" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K445" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L445" s="6">
+        <v>77</v>
+      </c>
+      <c r="M445" s="7">
+        <v>29313.45</v>
+      </c>
+      <c r="N445" s="6">
+        <v>1</v>
+      </c>
+      <c r="O445" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P445" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q445" s="6">
+        <v>0</v>
+      </c>
+      <c r="R445" s="7">
+        <v>0</v>
+      </c>
+      <c r="S445" s="9">
+        <v>0</v>
+      </c>
+      <c r="T445" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U445" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V445" s="11">
+        <v>11</v>
+      </c>
+      <c r="W445" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X445" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y445" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z445" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA445" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB445" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC445" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD445" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE445" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF445" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG445" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH445" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI445" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ445" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK445" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL445" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM445" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN445" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO445" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP445" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ445" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR445" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="446" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A446" s="1">
+        <v>1</v>
+      </c>
+      <c r="B446" s="2">
+        <v>2</v>
+      </c>
+      <c r="C446" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D446" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E446" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F446" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G446" s="5">
+        <v>10</v>
+      </c>
+      <c r="H446" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I446" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J446" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K446" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L446" s="6">
+        <v>78</v>
+      </c>
+      <c r="M446" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N446" s="6">
+        <v>1</v>
+      </c>
+      <c r="O446" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P446" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q446" s="6">
+        <v>0</v>
+      </c>
+      <c r="R446" s="7">
+        <v>0</v>
+      </c>
+      <c r="S446" s="9">
+        <v>0</v>
+      </c>
+      <c r="T446" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U446" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V446" s="11">
+        <v>11</v>
+      </c>
+      <c r="W446" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X446" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y446" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB446" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG446" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI446" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ446" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK446" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM446" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR446" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="447" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A447" s="1">
+        <v>1</v>
+      </c>
+      <c r="B447" s="2">
+        <v>2</v>
+      </c>
+      <c r="C447" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D447" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E447" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F447" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G447" s="5">
+        <v>11</v>
+      </c>
+      <c r="H447" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I447" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J447" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K447" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L447" s="6">
+        <v>79</v>
+      </c>
+      <c r="M447" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N447" s="6">
+        <v>1</v>
+      </c>
+      <c r="O447" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P447" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q447" s="6">
+        <v>0</v>
+      </c>
+      <c r="R447" s="7">
+        <v>0</v>
+      </c>
+      <c r="S447" s="9">
+        <v>0</v>
+      </c>
+      <c r="T447" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U447" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V447" s="11">
+        <v>11</v>
+      </c>
+      <c r="W447" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X447" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y447" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB447" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG447" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI447" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ447" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK447" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM447" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR447" s="3" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="448" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A448" s="1">
+        <v>1</v>
+      </c>
+      <c r="B448" s="2">
+        <v>2</v>
+      </c>
+      <c r="C448" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D448" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E448" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F448" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G448" s="5">
+        <v>12</v>
+      </c>
+      <c r="H448" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I448" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J448" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K448" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L448" s="6">
+        <v>80</v>
+      </c>
+      <c r="M448" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N448" s="6">
+        <v>1</v>
+      </c>
+      <c r="O448" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P448" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q448" s="6">
+        <v>0</v>
+      </c>
+      <c r="R448" s="7">
+        <v>0</v>
+      </c>
+      <c r="S448" s="9">
+        <v>0</v>
+      </c>
+      <c r="T448" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U448" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V448" s="11">
+        <v>11</v>
+      </c>
+      <c r="W448" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X448" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y448" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z448" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA448" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB448" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC448" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD448" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE448" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF448" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG448" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH448" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI448" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ448" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK448" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL448" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM448" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN448" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO448" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP448" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ448" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR448" s="3" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="449" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A449" s="1">
+        <v>1</v>
+      </c>
+      <c r="B449" s="2">
+        <v>2</v>
+      </c>
+      <c r="C449" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D449" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E449" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F449" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G449" s="5">
+        <v>13</v>
+      </c>
+      <c r="H449" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I449" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J449" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K449" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L449" s="6">
+        <v>81</v>
+      </c>
+      <c r="M449" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N449" s="6">
+        <v>1</v>
+      </c>
+      <c r="O449" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="P449" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q449" s="6">
+        <v>0</v>
+      </c>
+      <c r="R449" s="7">
+        <v>0</v>
+      </c>
+      <c r="S449" s="9">
+        <v>0</v>
+      </c>
+      <c r="T449" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U449" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V449" s="11">
+        <v>11</v>
+      </c>
+      <c r="W449" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X449" s="12">
         <v>0.40138889999999999</v>
       </c>
-      <c r="Y436" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z436" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA436" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB436" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC436" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD436" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE436" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF436" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG436" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH436" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI436" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="AJ436" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK436" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL436" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM436" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN436" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO436" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP436" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ436" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR436" s="3" t="s">
-        <v>494</v>
+      <c r="Y449" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z449" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA449" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB449" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC449" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD449" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE449" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF449" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG449" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH449" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI449" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ449" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK449" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL449" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM449" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN449" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO449" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP449" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ449" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR449" s="3" t="s">
+        <v>507</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 14:38:10,90
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45E08581-16AF-43B0-A555-49B8398B5224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35B24BE7-55B7-469D-BFAC-56DF115994E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8108" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8270" uniqueCount="517">
   <si>
     <t>Sel</t>
   </si>
@@ -1501,6 +1501,33 @@
     <t>1858400002960</t>
   </si>
   <si>
+    <t>1858400002961</t>
+  </si>
+  <si>
+    <t>1858400002962</t>
+  </si>
+  <si>
+    <t>1858400002963</t>
+  </si>
+  <si>
+    <t>1858400002964</t>
+  </si>
+  <si>
+    <t>1858400002965</t>
+  </si>
+  <si>
+    <t>1858400002966</t>
+  </si>
+  <si>
+    <t>1858400002967</t>
+  </si>
+  <si>
+    <t>1858400002968</t>
+  </si>
+  <si>
+    <t>1858400002969</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -2119,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR449"/>
+  <dimension ref="A1:AR458"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -60554,7 +60581,7 @@
         <v>2</v>
       </c>
       <c r="C437" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D437" s="3" t="s">
         <v>45</v>
@@ -60566,7 +60593,7 @@
         <v>46156</v>
       </c>
       <c r="G437" s="5">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="H437" s="3" t="s">
         <v>47</v>
@@ -60581,19 +60608,19 @@
         <v>50</v>
       </c>
       <c r="L437" s="6">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M437" s="7">
-        <v>26267.89</v>
+        <v>27879.79</v>
       </c>
       <c r="N437" s="6">
         <v>1</v>
       </c>
       <c r="O437" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P437" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q437" s="6">
         <v>0</v>
@@ -60608,7 +60635,7 @@
         <v>52</v>
       </c>
       <c r="U437" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V437" s="11">
         <v>11</v>
@@ -60617,7 +60644,7 @@
         <v>46156</v>
       </c>
       <c r="X437" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y437" s="10">
         <v>0</v>
@@ -60677,7 +60704,7 @@
         <v>53</v>
       </c>
       <c r="AR437" s="3" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="438" spans="1:44" x14ac:dyDescent="0.3">
@@ -60688,7 +60715,7 @@
         <v>2</v>
       </c>
       <c r="C438" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D438" s="3" t="s">
         <v>45</v>
@@ -60700,7 +60727,7 @@
         <v>46156</v>
       </c>
       <c r="G438" s="5">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H438" s="3" t="s">
         <v>47</v>
@@ -60715,19 +60742,19 @@
         <v>50</v>
       </c>
       <c r="L438" s="6">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="M438" s="7">
-        <v>26648.59</v>
+        <v>28329.46</v>
       </c>
       <c r="N438" s="6">
         <v>1</v>
       </c>
       <c r="O438" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P438" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q438" s="6">
         <v>0</v>
@@ -60742,7 +60769,7 @@
         <v>52</v>
       </c>
       <c r="U438" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V438" s="11">
         <v>11</v>
@@ -60751,7 +60778,7 @@
         <v>46156</v>
       </c>
       <c r="X438" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y438" s="10">
         <v>0</v>
@@ -60811,7 +60838,7 @@
         <v>53</v>
       </c>
       <c r="AR438" s="3" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="439" spans="1:44" x14ac:dyDescent="0.3">
@@ -60822,7 +60849,7 @@
         <v>2</v>
       </c>
       <c r="C439" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D439" s="3" t="s">
         <v>45</v>
@@ -60834,7 +60861,7 @@
         <v>46156</v>
       </c>
       <c r="G439" s="5">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="H439" s="3" t="s">
         <v>47</v>
@@ -60849,19 +60876,19 @@
         <v>50</v>
       </c>
       <c r="L439" s="6">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="M439" s="7">
-        <v>27029.279999999999</v>
+        <v>28779.14</v>
       </c>
       <c r="N439" s="6">
         <v>1</v>
       </c>
       <c r="O439" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P439" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q439" s="6">
         <v>0</v>
@@ -60876,7 +60903,7 @@
         <v>52</v>
       </c>
       <c r="U439" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V439" s="11">
         <v>11</v>
@@ -60885,7 +60912,7 @@
         <v>46156</v>
       </c>
       <c r="X439" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y439" s="10">
         <v>0</v>
@@ -60945,7 +60972,7 @@
         <v>53</v>
       </c>
       <c r="AR439" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="440" spans="1:44" x14ac:dyDescent="0.3">
@@ -60956,7 +60983,7 @@
         <v>2</v>
       </c>
       <c r="C440" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D440" s="3" t="s">
         <v>45</v>
@@ -60968,7 +60995,7 @@
         <v>46156</v>
       </c>
       <c r="G440" s="5">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="H440" s="3" t="s">
         <v>47</v>
@@ -60983,19 +61010,19 @@
         <v>50</v>
       </c>
       <c r="L440" s="6">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="M440" s="7">
-        <v>27409.98</v>
+        <v>29228.81</v>
       </c>
       <c r="N440" s="6">
         <v>1</v>
       </c>
       <c r="O440" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P440" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q440" s="6">
         <v>0</v>
@@ -61010,7 +61037,7 @@
         <v>52</v>
       </c>
       <c r="U440" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V440" s="11">
         <v>11</v>
@@ -61019,7 +61046,7 @@
         <v>46156</v>
       </c>
       <c r="X440" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y440" s="10">
         <v>0</v>
@@ -61079,7 +61106,7 @@
         <v>53</v>
       </c>
       <c r="AR440" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="441" spans="1:44" x14ac:dyDescent="0.3">
@@ -61090,7 +61117,7 @@
         <v>2</v>
       </c>
       <c r="C441" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D441" s="3" t="s">
         <v>45</v>
@@ -61102,7 +61129,7 @@
         <v>46156</v>
       </c>
       <c r="G441" s="5">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H441" s="3" t="s">
         <v>47</v>
@@ -61117,19 +61144,19 @@
         <v>50</v>
       </c>
       <c r="L441" s="6">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="M441" s="7">
-        <v>27790.67</v>
+        <v>29678.49</v>
       </c>
       <c r="N441" s="6">
         <v>1</v>
       </c>
       <c r="O441" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P441" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q441" s="6">
         <v>0</v>
@@ -61144,7 +61171,7 @@
         <v>52</v>
       </c>
       <c r="U441" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V441" s="11">
         <v>11</v>
@@ -61153,7 +61180,7 @@
         <v>46156</v>
       </c>
       <c r="X441" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y441" s="10">
         <v>0</v>
@@ -61213,7 +61240,7 @@
         <v>53</v>
       </c>
       <c r="AR441" s="3" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="442" spans="1:44" x14ac:dyDescent="0.3">
@@ -61224,7 +61251,7 @@
         <v>2</v>
       </c>
       <c r="C442" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D442" s="3" t="s">
         <v>45</v>
@@ -61236,7 +61263,7 @@
         <v>46156</v>
       </c>
       <c r="G442" s="5">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="H442" s="3" t="s">
         <v>47</v>
@@ -61251,19 +61278,19 @@
         <v>50</v>
       </c>
       <c r="L442" s="6">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="M442" s="7">
-        <v>28171.360000000001</v>
+        <v>30128.16</v>
       </c>
       <c r="N442" s="6">
         <v>1</v>
       </c>
       <c r="O442" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P442" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q442" s="6">
         <v>0</v>
@@ -61278,7 +61305,7 @@
         <v>52</v>
       </c>
       <c r="U442" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V442" s="11">
         <v>11</v>
@@ -61287,7 +61314,7 @@
         <v>46156</v>
       </c>
       <c r="X442" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y442" s="10">
         <v>0</v>
@@ -61347,7 +61374,7 @@
         <v>53</v>
       </c>
       <c r="AR442" s="3" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="443" spans="1:44" x14ac:dyDescent="0.3">
@@ -61358,7 +61385,7 @@
         <v>2</v>
       </c>
       <c r="C443" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D443" s="3" t="s">
         <v>45</v>
@@ -61370,7 +61397,7 @@
         <v>46156</v>
       </c>
       <c r="G443" s="5">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="H443" s="3" t="s">
         <v>47</v>
@@ -61385,19 +61412,19 @@
         <v>50</v>
       </c>
       <c r="L443" s="6">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="M443" s="7">
-        <v>28552.06</v>
+        <v>30577.83</v>
       </c>
       <c r="N443" s="6">
         <v>1</v>
       </c>
       <c r="O443" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P443" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q443" s="6">
         <v>0</v>
@@ -61412,7 +61439,7 @@
         <v>52</v>
       </c>
       <c r="U443" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V443" s="11">
         <v>11</v>
@@ -61421,7 +61448,7 @@
         <v>46156</v>
       </c>
       <c r="X443" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y443" s="10">
         <v>0</v>
@@ -61481,7 +61508,7 @@
         <v>53</v>
       </c>
       <c r="AR443" s="3" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="444" spans="1:44" x14ac:dyDescent="0.3">
@@ -61492,7 +61519,7 @@
         <v>2</v>
       </c>
       <c r="C444" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D444" s="3" t="s">
         <v>45</v>
@@ -61504,7 +61531,7 @@
         <v>46156</v>
       </c>
       <c r="G444" s="5">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="H444" s="3" t="s">
         <v>47</v>
@@ -61519,19 +61546,19 @@
         <v>50</v>
       </c>
       <c r="L444" s="6">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="M444" s="7">
-        <v>28932.75</v>
+        <v>31027.51</v>
       </c>
       <c r="N444" s="6">
         <v>1</v>
       </c>
       <c r="O444" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P444" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q444" s="6">
         <v>0</v>
@@ -61546,7 +61573,7 @@
         <v>52</v>
       </c>
       <c r="U444" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V444" s="11">
         <v>11</v>
@@ -61555,7 +61582,7 @@
         <v>46156</v>
       </c>
       <c r="X444" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y444" s="10">
         <v>0</v>
@@ -61615,7 +61642,7 @@
         <v>53</v>
       </c>
       <c r="AR444" s="3" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="445" spans="1:44" x14ac:dyDescent="0.3">
@@ -61626,7 +61653,7 @@
         <v>2</v>
       </c>
       <c r="C445" s="3" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="D445" s="3" t="s">
         <v>45</v>
@@ -61638,7 +61665,7 @@
         <v>46156</v>
       </c>
       <c r="G445" s="5">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H445" s="3" t="s">
         <v>47</v>
@@ -61653,19 +61680,19 @@
         <v>50</v>
       </c>
       <c r="L445" s="6">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="M445" s="7">
-        <v>29313.45</v>
+        <v>31477.18</v>
       </c>
       <c r="N445" s="6">
         <v>1</v>
       </c>
       <c r="O445" s="3" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="P445" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q445" s="6">
         <v>0</v>
@@ -61680,7 +61707,7 @@
         <v>52</v>
       </c>
       <c r="U445" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V445" s="11">
         <v>11</v>
@@ -61689,7 +61716,7 @@
         <v>46156</v>
       </c>
       <c r="X445" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.60763889999999998</v>
       </c>
       <c r="Y445" s="10">
         <v>0</v>
@@ -61749,7 +61776,7 @@
         <v>53</v>
       </c>
       <c r="AR445" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="446" spans="1:44" x14ac:dyDescent="0.3">
@@ -61760,7 +61787,7 @@
         <v>2</v>
       </c>
       <c r="C446" s="3" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="D446" s="3" t="s">
         <v>45</v>
@@ -61772,7 +61799,7 @@
         <v>46156</v>
       </c>
       <c r="G446" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H446" s="3" t="s">
         <v>47</v>
@@ -61787,16 +61814,16 @@
         <v>50</v>
       </c>
       <c r="L446" s="6">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="M446" s="7">
-        <v>29694.14</v>
+        <v>26267.89</v>
       </c>
       <c r="N446" s="6">
         <v>1</v>
       </c>
       <c r="O446" s="3" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="P446" s="8">
         <v>380.69</v>
@@ -61823,7 +61850,7 @@
         <v>46156</v>
       </c>
       <c r="X446" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y446" s="10">
         <v>0</v>
@@ -61894,7 +61921,7 @@
         <v>2</v>
       </c>
       <c r="C447" s="3" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="D447" s="3" t="s">
         <v>45</v>
@@ -61906,7 +61933,7 @@
         <v>46156</v>
       </c>
       <c r="G447" s="5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H447" s="3" t="s">
         <v>47</v>
@@ -61921,16 +61948,16 @@
         <v>50</v>
       </c>
       <c r="L447" s="6">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="M447" s="7">
-        <v>30074.83</v>
+        <v>26648.59</v>
       </c>
       <c r="N447" s="6">
         <v>1</v>
       </c>
       <c r="O447" s="3" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="P447" s="8">
         <v>380.69</v>
@@ -61957,7 +61984,7 @@
         <v>46156</v>
       </c>
       <c r="X447" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y447" s="10">
         <v>0</v>
@@ -62028,7 +62055,7 @@
         <v>2</v>
       </c>
       <c r="C448" s="3" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="D448" s="3" t="s">
         <v>45</v>
@@ -62040,7 +62067,7 @@
         <v>46156</v>
       </c>
       <c r="G448" s="5">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H448" s="3" t="s">
         <v>47</v>
@@ -62055,16 +62082,16 @@
         <v>50</v>
       </c>
       <c r="L448" s="6">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="M448" s="7">
-        <v>30455.53</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N448" s="6">
         <v>1</v>
       </c>
       <c r="O448" s="3" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="P448" s="8">
         <v>380.69</v>
@@ -62091,7 +62118,7 @@
         <v>46156</v>
       </c>
       <c r="X448" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y448" s="10">
         <v>0</v>
@@ -62162,7 +62189,7 @@
         <v>2</v>
       </c>
       <c r="C449" s="3" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="D449" s="3" t="s">
         <v>45</v>
@@ -62174,7 +62201,7 @@
         <v>46156</v>
       </c>
       <c r="G449" s="5">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H449" s="3" t="s">
         <v>47</v>
@@ -62189,16 +62216,16 @@
         <v>50</v>
       </c>
       <c r="L449" s="6">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="M449" s="7">
-        <v>30836.22</v>
+        <v>27409.98</v>
       </c>
       <c r="N449" s="6">
         <v>1</v>
       </c>
       <c r="O449" s="3" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="P449" s="8">
         <v>380.69</v>
@@ -62225,7 +62252,7 @@
         <v>46156</v>
       </c>
       <c r="X449" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y449" s="10">
         <v>0</v>
@@ -62286,6 +62313,1212 @@
       </c>
       <c r="AR449" s="3" t="s">
         <v>507</v>
+      </c>
+    </row>
+    <row r="450" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A450" s="1">
+        <v>1</v>
+      </c>
+      <c r="B450" s="2">
+        <v>2</v>
+      </c>
+      <c r="C450" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D450" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E450" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F450" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G450" s="5">
+        <v>5</v>
+      </c>
+      <c r="H450" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I450" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J450" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K450" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L450" s="6">
+        <v>73</v>
+      </c>
+      <c r="M450" s="7">
+        <v>27790.67</v>
+      </c>
+      <c r="N450" s="6">
+        <v>1</v>
+      </c>
+      <c r="O450" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P450" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q450" s="6">
+        <v>0</v>
+      </c>
+      <c r="R450" s="7">
+        <v>0</v>
+      </c>
+      <c r="S450" s="9">
+        <v>0</v>
+      </c>
+      <c r="T450" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U450" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V450" s="11">
+        <v>11</v>
+      </c>
+      <c r="W450" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X450" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y450" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z450" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA450" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB450" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC450" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD450" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE450" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF450" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG450" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH450" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI450" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ450" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK450" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL450" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM450" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN450" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO450" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP450" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ450" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR450" s="3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="451" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A451" s="1">
+        <v>1</v>
+      </c>
+      <c r="B451" s="2">
+        <v>2</v>
+      </c>
+      <c r="C451" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D451" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E451" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F451" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G451" s="5">
+        <v>6</v>
+      </c>
+      <c r="H451" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I451" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J451" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K451" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L451" s="6">
+        <v>74</v>
+      </c>
+      <c r="M451" s="7">
+        <v>28171.360000000001</v>
+      </c>
+      <c r="N451" s="6">
+        <v>1</v>
+      </c>
+      <c r="O451" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P451" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q451" s="6">
+        <v>0</v>
+      </c>
+      <c r="R451" s="7">
+        <v>0</v>
+      </c>
+      <c r="S451" s="9">
+        <v>0</v>
+      </c>
+      <c r="T451" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U451" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V451" s="11">
+        <v>11</v>
+      </c>
+      <c r="W451" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X451" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y451" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z451" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA451" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB451" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC451" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD451" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE451" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF451" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG451" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH451" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI451" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ451" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK451" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL451" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM451" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN451" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO451" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP451" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ451" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR451" s="3" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="452" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A452" s="1">
+        <v>1</v>
+      </c>
+      <c r="B452" s="2">
+        <v>2</v>
+      </c>
+      <c r="C452" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D452" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E452" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F452" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G452" s="5">
+        <v>7</v>
+      </c>
+      <c r="H452" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I452" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J452" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K452" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L452" s="6">
+        <v>75</v>
+      </c>
+      <c r="M452" s="7">
+        <v>28552.06</v>
+      </c>
+      <c r="N452" s="6">
+        <v>1</v>
+      </c>
+      <c r="O452" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P452" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q452" s="6">
+        <v>0</v>
+      </c>
+      <c r="R452" s="7">
+        <v>0</v>
+      </c>
+      <c r="S452" s="9">
+        <v>0</v>
+      </c>
+      <c r="T452" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U452" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V452" s="11">
+        <v>11</v>
+      </c>
+      <c r="W452" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X452" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y452" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z452" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA452" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB452" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC452" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD452" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE452" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF452" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG452" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH452" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI452" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ452" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK452" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL452" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM452" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN452" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO452" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP452" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ452" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR452" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="453" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A453" s="1">
+        <v>1</v>
+      </c>
+      <c r="B453" s="2">
+        <v>2</v>
+      </c>
+      <c r="C453" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D453" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E453" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F453" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G453" s="5">
+        <v>8</v>
+      </c>
+      <c r="H453" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I453" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J453" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K453" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L453" s="6">
+        <v>76</v>
+      </c>
+      <c r="M453" s="7">
+        <v>28932.75</v>
+      </c>
+      <c r="N453" s="6">
+        <v>1</v>
+      </c>
+      <c r="O453" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P453" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q453" s="6">
+        <v>0</v>
+      </c>
+      <c r="R453" s="7">
+        <v>0</v>
+      </c>
+      <c r="S453" s="9">
+        <v>0</v>
+      </c>
+      <c r="T453" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U453" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V453" s="11">
+        <v>11</v>
+      </c>
+      <c r="W453" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X453" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y453" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z453" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA453" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB453" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC453" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD453" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE453" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF453" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG453" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH453" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI453" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ453" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK453" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL453" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM453" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN453" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO453" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP453" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ453" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR453" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="454" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A454" s="1">
+        <v>1</v>
+      </c>
+      <c r="B454" s="2">
+        <v>2</v>
+      </c>
+      <c r="C454" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D454" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E454" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F454" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G454" s="5">
+        <v>9</v>
+      </c>
+      <c r="H454" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I454" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J454" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K454" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L454" s="6">
+        <v>77</v>
+      </c>
+      <c r="M454" s="7">
+        <v>29313.45</v>
+      </c>
+      <c r="N454" s="6">
+        <v>1</v>
+      </c>
+      <c r="O454" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P454" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q454" s="6">
+        <v>0</v>
+      </c>
+      <c r="R454" s="7">
+        <v>0</v>
+      </c>
+      <c r="S454" s="9">
+        <v>0</v>
+      </c>
+      <c r="T454" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U454" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V454" s="11">
+        <v>11</v>
+      </c>
+      <c r="W454" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X454" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y454" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z454" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA454" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB454" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC454" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD454" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE454" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF454" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG454" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH454" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI454" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ454" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK454" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL454" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM454" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN454" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO454" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP454" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ454" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR454" s="3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="455" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A455" s="1">
+        <v>1</v>
+      </c>
+      <c r="B455" s="2">
+        <v>2</v>
+      </c>
+      <c r="C455" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D455" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E455" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F455" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G455" s="5">
+        <v>10</v>
+      </c>
+      <c r="H455" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I455" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J455" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K455" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L455" s="6">
+        <v>78</v>
+      </c>
+      <c r="M455" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N455" s="6">
+        <v>1</v>
+      </c>
+      <c r="O455" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P455" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q455" s="6">
+        <v>0</v>
+      </c>
+      <c r="R455" s="7">
+        <v>0</v>
+      </c>
+      <c r="S455" s="9">
+        <v>0</v>
+      </c>
+      <c r="T455" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U455" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V455" s="11">
+        <v>11</v>
+      </c>
+      <c r="W455" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X455" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y455" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z455" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA455" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB455" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC455" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD455" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE455" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF455" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG455" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH455" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI455" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ455" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK455" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL455" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM455" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN455" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO455" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP455" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ455" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR455" s="3" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="456" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A456" s="1">
+        <v>1</v>
+      </c>
+      <c r="B456" s="2">
+        <v>2</v>
+      </c>
+      <c r="C456" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D456" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E456" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F456" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G456" s="5">
+        <v>11</v>
+      </c>
+      <c r="H456" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I456" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J456" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K456" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L456" s="6">
+        <v>79</v>
+      </c>
+      <c r="M456" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N456" s="6">
+        <v>1</v>
+      </c>
+      <c r="O456" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P456" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q456" s="6">
+        <v>0</v>
+      </c>
+      <c r="R456" s="7">
+        <v>0</v>
+      </c>
+      <c r="S456" s="9">
+        <v>0</v>
+      </c>
+      <c r="T456" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U456" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V456" s="11">
+        <v>11</v>
+      </c>
+      <c r="W456" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X456" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y456" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z456" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA456" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB456" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC456" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD456" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE456" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF456" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG456" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH456" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI456" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ456" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK456" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL456" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM456" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN456" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO456" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP456" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ456" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR456" s="3" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="457" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A457" s="1">
+        <v>1</v>
+      </c>
+      <c r="B457" s="2">
+        <v>2</v>
+      </c>
+      <c r="C457" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D457" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E457" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F457" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G457" s="5">
+        <v>12</v>
+      </c>
+      <c r="H457" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I457" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J457" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K457" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L457" s="6">
+        <v>80</v>
+      </c>
+      <c r="M457" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N457" s="6">
+        <v>1</v>
+      </c>
+      <c r="O457" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P457" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q457" s="6">
+        <v>0</v>
+      </c>
+      <c r="R457" s="7">
+        <v>0</v>
+      </c>
+      <c r="S457" s="9">
+        <v>0</v>
+      </c>
+      <c r="T457" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U457" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V457" s="11">
+        <v>11</v>
+      </c>
+      <c r="W457" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X457" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y457" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z457" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA457" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB457" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC457" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD457" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE457" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF457" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG457" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH457" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI457" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ457" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK457" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL457" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM457" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN457" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO457" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP457" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ457" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR457" s="3" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="458" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A458" s="1">
+        <v>1</v>
+      </c>
+      <c r="B458" s="2">
+        <v>2</v>
+      </c>
+      <c r="C458" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D458" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E458" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F458" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G458" s="5">
+        <v>13</v>
+      </c>
+      <c r="H458" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I458" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J458" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K458" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L458" s="6">
+        <v>81</v>
+      </c>
+      <c r="M458" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N458" s="6">
+        <v>1</v>
+      </c>
+      <c r="O458" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="P458" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q458" s="6">
+        <v>0</v>
+      </c>
+      <c r="R458" s="7">
+        <v>0</v>
+      </c>
+      <c r="S458" s="9">
+        <v>0</v>
+      </c>
+      <c r="T458" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U458" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V458" s="11">
+        <v>11</v>
+      </c>
+      <c r="W458" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X458" s="12">
+        <v>0.40138889999999999</v>
+      </c>
+      <c r="Y458" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z458" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA458" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB458" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC458" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD458" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE458" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF458" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG458" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH458" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI458" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="AJ458" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK458" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL458" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM458" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN458" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO458" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP458" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ458" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR458" s="3" t="s">
+        <v>516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 15:37:55,75
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51F15F87-692E-4E62-8FA0-1AB24C2AD6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A70C098-4BC4-456C-B237-923101275D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9962" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10052" uniqueCount="616">
   <si>
     <t>Sel</t>
   </si>
@@ -1810,6 +1810,21 @@
     <t>1858400002975</t>
   </si>
   <si>
+    <t>1858400002976</t>
+  </si>
+  <si>
+    <t>1858400002977</t>
+  </si>
+  <si>
+    <t>1858400002978</t>
+  </si>
+  <si>
+    <t>1858400002979</t>
+  </si>
+  <si>
+    <t>1858400002980</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -2428,7 +2443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR552"/>
+  <dimension ref="A1:AR557"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -74665,7 +74680,7 @@
         <v>2</v>
       </c>
       <c r="C540" s="3" t="s">
-        <v>596</v>
+        <v>553</v>
       </c>
       <c r="D540" s="3" t="s">
         <v>45</v>
@@ -74677,7 +74692,7 @@
         <v>46156</v>
       </c>
       <c r="G540" s="5">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="H540" s="3" t="s">
         <v>47</v>
@@ -74692,19 +74707,19 @@
         <v>50</v>
       </c>
       <c r="L540" s="6">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="M540" s="7">
-        <v>26267.89</v>
+        <v>34624.9</v>
       </c>
       <c r="N540" s="6">
         <v>1</v>
       </c>
       <c r="O540" s="3" t="s">
-        <v>597</v>
+        <v>554</v>
       </c>
       <c r="P540" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q540" s="6">
         <v>0</v>
@@ -74719,7 +74734,7 @@
         <v>52</v>
       </c>
       <c r="U540" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V540" s="11">
         <v>11</v>
@@ -74728,7 +74743,7 @@
         <v>46156</v>
       </c>
       <c r="X540" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.64930560000000004</v>
       </c>
       <c r="Y540" s="10">
         <v>0</v>
@@ -74788,7 +74803,7 @@
         <v>53</v>
       </c>
       <c r="AR540" s="3" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="541" spans="1:44" x14ac:dyDescent="0.3">
@@ -74799,7 +74814,7 @@
         <v>2</v>
       </c>
       <c r="C541" s="3" t="s">
-        <v>596</v>
+        <v>553</v>
       </c>
       <c r="D541" s="3" t="s">
         <v>45</v>
@@ -74811,7 +74826,7 @@
         <v>46156</v>
       </c>
       <c r="G541" s="5">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="H541" s="3" t="s">
         <v>47</v>
@@ -74826,19 +74841,19 @@
         <v>50</v>
       </c>
       <c r="L541" s="6">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="M541" s="7">
-        <v>26648.59</v>
+        <v>35074.57</v>
       </c>
       <c r="N541" s="6">
         <v>1</v>
       </c>
       <c r="O541" s="3" t="s">
-        <v>597</v>
+        <v>554</v>
       </c>
       <c r="P541" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q541" s="6">
         <v>0</v>
@@ -74853,7 +74868,7 @@
         <v>52</v>
       </c>
       <c r="U541" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V541" s="11">
         <v>11</v>
@@ -74862,7 +74877,7 @@
         <v>46156</v>
       </c>
       <c r="X541" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.64930560000000004</v>
       </c>
       <c r="Y541" s="10">
         <v>0</v>
@@ -74922,7 +74937,7 @@
         <v>53</v>
       </c>
       <c r="AR541" s="3" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="542" spans="1:44" x14ac:dyDescent="0.3">
@@ -74933,7 +74948,7 @@
         <v>2</v>
       </c>
       <c r="C542" s="3" t="s">
-        <v>596</v>
+        <v>553</v>
       </c>
       <c r="D542" s="3" t="s">
         <v>45</v>
@@ -74945,7 +74960,7 @@
         <v>46156</v>
       </c>
       <c r="G542" s="5">
-        <v>3</v>
+        <v>43</v>
       </c>
       <c r="H542" s="3" t="s">
         <v>47</v>
@@ -74960,19 +74975,19 @@
         <v>50</v>
       </c>
       <c r="L542" s="6">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="M542" s="7">
-        <v>27029.279999999999</v>
+        <v>35524.25</v>
       </c>
       <c r="N542" s="6">
         <v>1</v>
       </c>
       <c r="O542" s="3" t="s">
-        <v>597</v>
+        <v>554</v>
       </c>
       <c r="P542" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q542" s="6">
         <v>0</v>
@@ -74987,7 +75002,7 @@
         <v>52</v>
       </c>
       <c r="U542" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V542" s="11">
         <v>11</v>
@@ -74996,7 +75011,7 @@
         <v>46156</v>
       </c>
       <c r="X542" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.64930560000000004</v>
       </c>
       <c r="Y542" s="10">
         <v>0</v>
@@ -75056,7 +75071,7 @@
         <v>53</v>
       </c>
       <c r="AR542" s="3" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="543" spans="1:44" x14ac:dyDescent="0.3">
@@ -75067,7 +75082,7 @@
         <v>2</v>
       </c>
       <c r="C543" s="3" t="s">
-        <v>596</v>
+        <v>553</v>
       </c>
       <c r="D543" s="3" t="s">
         <v>45</v>
@@ -75079,7 +75094,7 @@
         <v>46156</v>
       </c>
       <c r="G543" s="5">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="H543" s="3" t="s">
         <v>47</v>
@@ -75094,19 +75109,19 @@
         <v>50</v>
       </c>
       <c r="L543" s="6">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="M543" s="7">
-        <v>27409.98</v>
+        <v>35973.919999999998</v>
       </c>
       <c r="N543" s="6">
         <v>1</v>
       </c>
       <c r="O543" s="3" t="s">
-        <v>597</v>
+        <v>554</v>
       </c>
       <c r="P543" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q543" s="6">
         <v>0</v>
@@ -75121,7 +75136,7 @@
         <v>52</v>
       </c>
       <c r="U543" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V543" s="11">
         <v>11</v>
@@ -75130,7 +75145,7 @@
         <v>46156</v>
       </c>
       <c r="X543" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.64930560000000004</v>
       </c>
       <c r="Y543" s="10">
         <v>0</v>
@@ -75190,7 +75205,7 @@
         <v>53</v>
       </c>
       <c r="AR543" s="3" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="544" spans="1:44" x14ac:dyDescent="0.3">
@@ -75201,7 +75216,7 @@
         <v>2</v>
       </c>
       <c r="C544" s="3" t="s">
-        <v>596</v>
+        <v>553</v>
       </c>
       <c r="D544" s="3" t="s">
         <v>45</v>
@@ -75213,7 +75228,7 @@
         <v>46156</v>
       </c>
       <c r="G544" s="5">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="H544" s="3" t="s">
         <v>47</v>
@@ -75228,19 +75243,19 @@
         <v>50</v>
       </c>
       <c r="L544" s="6">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="M544" s="7">
-        <v>27790.67</v>
+        <v>36423.599999999999</v>
       </c>
       <c r="N544" s="6">
         <v>1</v>
       </c>
       <c r="O544" s="3" t="s">
-        <v>597</v>
+        <v>554</v>
       </c>
       <c r="P544" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q544" s="6">
         <v>0</v>
@@ -75255,7 +75270,7 @@
         <v>52</v>
       </c>
       <c r="U544" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V544" s="11">
         <v>11</v>
@@ -75264,7 +75279,7 @@
         <v>46156</v>
       </c>
       <c r="X544" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.64930560000000004</v>
       </c>
       <c r="Y544" s="10">
         <v>0</v>
@@ -75324,7 +75339,7 @@
         <v>53</v>
       </c>
       <c r="AR544" s="3" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
     </row>
     <row r="545" spans="1:44" x14ac:dyDescent="0.3">
@@ -75335,7 +75350,7 @@
         <v>2</v>
       </c>
       <c r="C545" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D545" s="3" t="s">
         <v>45</v>
@@ -75347,7 +75362,7 @@
         <v>46156</v>
       </c>
       <c r="G545" s="5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H545" s="3" t="s">
         <v>47</v>
@@ -75362,16 +75377,16 @@
         <v>50</v>
       </c>
       <c r="L545" s="6">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="M545" s="7">
-        <v>28171.360000000001</v>
+        <v>26267.89</v>
       </c>
       <c r="N545" s="6">
         <v>1</v>
       </c>
       <c r="O545" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P545" s="8">
         <v>380.69</v>
@@ -75469,7 +75484,7 @@
         <v>2</v>
       </c>
       <c r="C546" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D546" s="3" t="s">
         <v>45</v>
@@ -75481,7 +75496,7 @@
         <v>46156</v>
       </c>
       <c r="G546" s="5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H546" s="3" t="s">
         <v>47</v>
@@ -75496,16 +75511,16 @@
         <v>50</v>
       </c>
       <c r="L546" s="6">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="M546" s="7">
-        <v>28552.06</v>
+        <v>26648.59</v>
       </c>
       <c r="N546" s="6">
         <v>1</v>
       </c>
       <c r="O546" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P546" s="8">
         <v>380.69</v>
@@ -75532,7 +75547,7 @@
         <v>46156</v>
       </c>
       <c r="X546" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y546" s="10">
         <v>0</v>
@@ -75603,7 +75618,7 @@
         <v>2</v>
       </c>
       <c r="C547" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D547" s="3" t="s">
         <v>45</v>
@@ -75615,7 +75630,7 @@
         <v>46156</v>
       </c>
       <c r="G547" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H547" s="3" t="s">
         <v>47</v>
@@ -75630,16 +75645,16 @@
         <v>50</v>
       </c>
       <c r="L547" s="6">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="M547" s="7">
-        <v>28932.75</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N547" s="6">
         <v>1</v>
       </c>
       <c r="O547" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P547" s="8">
         <v>380.69</v>
@@ -75666,7 +75681,7 @@
         <v>46156</v>
       </c>
       <c r="X547" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y547" s="10">
         <v>0</v>
@@ -75737,7 +75752,7 @@
         <v>2</v>
       </c>
       <c r="C548" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D548" s="3" t="s">
         <v>45</v>
@@ -75749,7 +75764,7 @@
         <v>46156</v>
       </c>
       <c r="G548" s="5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H548" s="3" t="s">
         <v>47</v>
@@ -75764,16 +75779,16 @@
         <v>50</v>
       </c>
       <c r="L548" s="6">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="M548" s="7">
-        <v>29313.45</v>
+        <v>27409.98</v>
       </c>
       <c r="N548" s="6">
         <v>1</v>
       </c>
       <c r="O548" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P548" s="8">
         <v>380.69</v>
@@ -75800,7 +75815,7 @@
         <v>46156</v>
       </c>
       <c r="X548" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y548" s="10">
         <v>0</v>
@@ -75871,7 +75886,7 @@
         <v>2</v>
       </c>
       <c r="C549" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D549" s="3" t="s">
         <v>45</v>
@@ -75883,7 +75898,7 @@
         <v>46156</v>
       </c>
       <c r="G549" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H549" s="3" t="s">
         <v>47</v>
@@ -75898,16 +75913,16 @@
         <v>50</v>
       </c>
       <c r="L549" s="6">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M549" s="7">
-        <v>29694.14</v>
+        <v>27790.67</v>
       </c>
       <c r="N549" s="6">
         <v>1</v>
       </c>
       <c r="O549" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P549" s="8">
         <v>380.69</v>
@@ -75934,7 +75949,7 @@
         <v>46156</v>
       </c>
       <c r="X549" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y549" s="10">
         <v>0</v>
@@ -76005,7 +76020,7 @@
         <v>2</v>
       </c>
       <c r="C550" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D550" s="3" t="s">
         <v>45</v>
@@ -76017,7 +76032,7 @@
         <v>46156</v>
       </c>
       <c r="G550" s="5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H550" s="3" t="s">
         <v>47</v>
@@ -76032,16 +76047,16 @@
         <v>50</v>
       </c>
       <c r="L550" s="6">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="M550" s="7">
-        <v>30074.83</v>
+        <v>28171.360000000001</v>
       </c>
       <c r="N550" s="6">
         <v>1</v>
       </c>
       <c r="O550" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P550" s="8">
         <v>380.69</v>
@@ -76068,7 +76083,7 @@
         <v>46156</v>
       </c>
       <c r="X550" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y550" s="10">
         <v>0</v>
@@ -76139,7 +76154,7 @@
         <v>2</v>
       </c>
       <c r="C551" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D551" s="3" t="s">
         <v>45</v>
@@ -76151,7 +76166,7 @@
         <v>46156</v>
       </c>
       <c r="G551" s="5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H551" s="3" t="s">
         <v>47</v>
@@ -76166,16 +76181,16 @@
         <v>50</v>
       </c>
       <c r="L551" s="6">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="M551" s="7">
-        <v>30455.53</v>
+        <v>28552.06</v>
       </c>
       <c r="N551" s="6">
         <v>1</v>
       </c>
       <c r="O551" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P551" s="8">
         <v>380.69</v>
@@ -76202,7 +76217,7 @@
         <v>46156</v>
       </c>
       <c r="X551" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y551" s="10">
         <v>0</v>
@@ -76273,7 +76288,7 @@
         <v>2</v>
       </c>
       <c r="C552" s="3" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D552" s="3" t="s">
         <v>45</v>
@@ -76285,7 +76300,7 @@
         <v>46156</v>
       </c>
       <c r="G552" s="5">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H552" s="3" t="s">
         <v>47</v>
@@ -76300,16 +76315,16 @@
         <v>50</v>
       </c>
       <c r="L552" s="6">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="M552" s="7">
-        <v>30836.22</v>
+        <v>28932.75</v>
       </c>
       <c r="N552" s="6">
         <v>1</v>
       </c>
       <c r="O552" s="3" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="P552" s="8">
         <v>380.69</v>
@@ -76336,7 +76351,7 @@
         <v>46156</v>
       </c>
       <c r="X552" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y552" s="10">
         <v>0</v>
@@ -76397,6 +76412,676 @@
       </c>
       <c r="AR552" s="3" t="s">
         <v>610</v>
+      </c>
+    </row>
+    <row r="553" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A553" s="1">
+        <v>1</v>
+      </c>
+      <c r="B553" s="2">
+        <v>2</v>
+      </c>
+      <c r="C553" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D553" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E553" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F553" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G553" s="5">
+        <v>9</v>
+      </c>
+      <c r="H553" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I553" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J553" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K553" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L553" s="6">
+        <v>77</v>
+      </c>
+      <c r="M553" s="7">
+        <v>29313.45</v>
+      </c>
+      <c r="N553" s="6">
+        <v>1</v>
+      </c>
+      <c r="O553" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="P553" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q553" s="6">
+        <v>0</v>
+      </c>
+      <c r="R553" s="7">
+        <v>0</v>
+      </c>
+      <c r="S553" s="9">
+        <v>0</v>
+      </c>
+      <c r="T553" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U553" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V553" s="11">
+        <v>11</v>
+      </c>
+      <c r="W553" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X553" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y553" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z553" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA553" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB553" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC553" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD553" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE553" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF553" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG553" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH553" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI553" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="AJ553" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK553" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL553" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM553" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN553" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO553" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP553" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ553" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR553" s="3" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="554" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A554" s="1">
+        <v>1</v>
+      </c>
+      <c r="B554" s="2">
+        <v>2</v>
+      </c>
+      <c r="C554" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D554" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E554" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F554" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G554" s="5">
+        <v>10</v>
+      </c>
+      <c r="H554" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I554" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J554" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K554" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L554" s="6">
+        <v>78</v>
+      </c>
+      <c r="M554" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N554" s="6">
+        <v>1</v>
+      </c>
+      <c r="O554" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="P554" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q554" s="6">
+        <v>0</v>
+      </c>
+      <c r="R554" s="7">
+        <v>0</v>
+      </c>
+      <c r="S554" s="9">
+        <v>0</v>
+      </c>
+      <c r="T554" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U554" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V554" s="11">
+        <v>11</v>
+      </c>
+      <c r="W554" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X554" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y554" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z554" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA554" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB554" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC554" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD554" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE554" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF554" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG554" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH554" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI554" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="AJ554" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK554" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL554" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM554" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN554" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO554" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP554" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ554" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR554" s="3" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="555" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A555" s="1">
+        <v>1</v>
+      </c>
+      <c r="B555" s="2">
+        <v>2</v>
+      </c>
+      <c r="C555" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D555" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E555" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F555" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G555" s="5">
+        <v>11</v>
+      </c>
+      <c r="H555" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I555" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J555" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K555" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L555" s="6">
+        <v>79</v>
+      </c>
+      <c r="M555" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N555" s="6">
+        <v>1</v>
+      </c>
+      <c r="O555" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="P555" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q555" s="6">
+        <v>0</v>
+      </c>
+      <c r="R555" s="7">
+        <v>0</v>
+      </c>
+      <c r="S555" s="9">
+        <v>0</v>
+      </c>
+      <c r="T555" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U555" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V555" s="11">
+        <v>11</v>
+      </c>
+      <c r="W555" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X555" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y555" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z555" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA555" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB555" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC555" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD555" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE555" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF555" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG555" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH555" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI555" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="AJ555" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK555" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL555" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM555" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN555" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO555" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP555" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ555" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR555" s="3" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="556" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A556" s="1">
+        <v>1</v>
+      </c>
+      <c r="B556" s="2">
+        <v>2</v>
+      </c>
+      <c r="C556" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D556" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E556" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F556" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G556" s="5">
+        <v>12</v>
+      </c>
+      <c r="H556" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I556" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J556" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K556" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L556" s="6">
+        <v>80</v>
+      </c>
+      <c r="M556" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N556" s="6">
+        <v>1</v>
+      </c>
+      <c r="O556" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="P556" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q556" s="6">
+        <v>0</v>
+      </c>
+      <c r="R556" s="7">
+        <v>0</v>
+      </c>
+      <c r="S556" s="9">
+        <v>0</v>
+      </c>
+      <c r="T556" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U556" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V556" s="11">
+        <v>11</v>
+      </c>
+      <c r="W556" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X556" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y556" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z556" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA556" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB556" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC556" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD556" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE556" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF556" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG556" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH556" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI556" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="AJ556" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK556" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL556" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM556" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN556" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO556" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP556" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ556" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR556" s="3" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="557" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A557" s="1">
+        <v>1</v>
+      </c>
+      <c r="B557" s="2">
+        <v>2</v>
+      </c>
+      <c r="C557" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D557" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E557" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F557" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G557" s="5">
+        <v>13</v>
+      </c>
+      <c r="H557" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I557" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J557" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K557" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L557" s="6">
+        <v>81</v>
+      </c>
+      <c r="M557" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N557" s="6">
+        <v>1</v>
+      </c>
+      <c r="O557" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="P557" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q557" s="6">
+        <v>0</v>
+      </c>
+      <c r="R557" s="7">
+        <v>0</v>
+      </c>
+      <c r="S557" s="9">
+        <v>0</v>
+      </c>
+      <c r="T557" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U557" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V557" s="11">
+        <v>11</v>
+      </c>
+      <c r="W557" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X557" s="12">
+        <v>0.40138889999999999</v>
+      </c>
+      <c r="Y557" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z557" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA557" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB557" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC557" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD557" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE557" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF557" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG557" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH557" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI557" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="AJ557" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK557" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL557" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM557" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN557" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO557" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP557" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ557" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR557" s="3" t="s">
+        <v>615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 16:44:24,62
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CC5E28E-F300-4ACD-941D-77B1BB63AA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C6010BA-3AA0-4FD8-9554-5A98A572EFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11528" uniqueCount="698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11600" uniqueCount="702">
   <si>
     <t>Sel</t>
   </si>
@@ -2071,6 +2071,18 @@
     <t>1858400002983</t>
   </si>
   <si>
+    <t>1858400002984</t>
+  </si>
+  <si>
+    <t>1858400002985</t>
+  </si>
+  <si>
+    <t>1858400002986</t>
+  </si>
+  <si>
+    <t>1858400002987</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -2689,7 +2701,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR639"/>
+  <dimension ref="A1:AR643"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -86584,7 +86596,7 @@
         <v>2</v>
       </c>
       <c r="C627" s="3" t="s">
-        <v>683</v>
+        <v>632</v>
       </c>
       <c r="D627" s="3" t="s">
         <v>45</v>
@@ -86596,7 +86608,7 @@
         <v>46156</v>
       </c>
       <c r="G627" s="5">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="H627" s="3" t="s">
         <v>47</v>
@@ -86611,19 +86623,19 @@
         <v>50</v>
       </c>
       <c r="L627" s="6">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="M627" s="7">
-        <v>26267.89</v>
+        <v>38222.29</v>
       </c>
       <c r="N627" s="6">
         <v>1</v>
       </c>
       <c r="O627" s="3" t="s">
-        <v>684</v>
+        <v>633</v>
       </c>
       <c r="P627" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q627" s="6">
         <v>0</v>
@@ -86638,7 +86650,7 @@
         <v>52</v>
       </c>
       <c r="U627" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V627" s="11">
         <v>11</v>
@@ -86647,7 +86659,7 @@
         <v>46156</v>
       </c>
       <c r="X627" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.69097220000000004</v>
       </c>
       <c r="Y627" s="10">
         <v>0</v>
@@ -86707,7 +86719,7 @@
         <v>53</v>
       </c>
       <c r="AR627" s="3" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="628" spans="1:44" x14ac:dyDescent="0.3">
@@ -86718,7 +86730,7 @@
         <v>2</v>
       </c>
       <c r="C628" s="3" t="s">
-        <v>683</v>
+        <v>632</v>
       </c>
       <c r="D628" s="3" t="s">
         <v>45</v>
@@ -86730,7 +86742,7 @@
         <v>46156</v>
       </c>
       <c r="G628" s="5">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="H628" s="3" t="s">
         <v>47</v>
@@ -86745,19 +86757,19 @@
         <v>50</v>
       </c>
       <c r="L628" s="6">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="M628" s="7">
-        <v>26648.59</v>
+        <v>38671.97</v>
       </c>
       <c r="N628" s="6">
         <v>1</v>
       </c>
       <c r="O628" s="3" t="s">
-        <v>684</v>
+        <v>633</v>
       </c>
       <c r="P628" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q628" s="6">
         <v>0</v>
@@ -86772,7 +86784,7 @@
         <v>52</v>
       </c>
       <c r="U628" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V628" s="11">
         <v>11</v>
@@ -86781,7 +86793,7 @@
         <v>46156</v>
       </c>
       <c r="X628" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.69097220000000004</v>
       </c>
       <c r="Y628" s="10">
         <v>0</v>
@@ -86841,7 +86853,7 @@
         <v>53</v>
       </c>
       <c r="AR628" s="3" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="629" spans="1:44" x14ac:dyDescent="0.3">
@@ -86852,7 +86864,7 @@
         <v>2</v>
       </c>
       <c r="C629" s="3" t="s">
-        <v>683</v>
+        <v>632</v>
       </c>
       <c r="D629" s="3" t="s">
         <v>45</v>
@@ -86864,7 +86876,7 @@
         <v>46156</v>
       </c>
       <c r="G629" s="5">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="H629" s="3" t="s">
         <v>47</v>
@@ -86879,19 +86891,19 @@
         <v>50</v>
       </c>
       <c r="L629" s="6">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="M629" s="7">
-        <v>27029.279999999999</v>
+        <v>39121.64</v>
       </c>
       <c r="N629" s="6">
         <v>1</v>
       </c>
       <c r="O629" s="3" t="s">
-        <v>684</v>
+        <v>633</v>
       </c>
       <c r="P629" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q629" s="6">
         <v>0</v>
@@ -86906,7 +86918,7 @@
         <v>52</v>
       </c>
       <c r="U629" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V629" s="11">
         <v>11</v>
@@ -86915,7 +86927,7 @@
         <v>46156</v>
       </c>
       <c r="X629" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.69097220000000004</v>
       </c>
       <c r="Y629" s="10">
         <v>0</v>
@@ -86975,7 +86987,7 @@
         <v>53</v>
       </c>
       <c r="AR629" s="3" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
     </row>
     <row r="630" spans="1:44" x14ac:dyDescent="0.3">
@@ -86986,7 +86998,7 @@
         <v>2</v>
       </c>
       <c r="C630" s="3" t="s">
-        <v>683</v>
+        <v>632</v>
       </c>
       <c r="D630" s="3" t="s">
         <v>45</v>
@@ -86998,7 +87010,7 @@
         <v>46156</v>
       </c>
       <c r="G630" s="5">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="H630" s="3" t="s">
         <v>47</v>
@@ -87013,19 +87025,19 @@
         <v>50</v>
       </c>
       <c r="L630" s="6">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M630" s="7">
-        <v>27409.98</v>
+        <v>39571.31</v>
       </c>
       <c r="N630" s="6">
         <v>1</v>
       </c>
       <c r="O630" s="3" t="s">
-        <v>684</v>
+        <v>633</v>
       </c>
       <c r="P630" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q630" s="6">
         <v>0</v>
@@ -87040,7 +87052,7 @@
         <v>52</v>
       </c>
       <c r="U630" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V630" s="11">
         <v>11</v>
@@ -87049,7 +87061,7 @@
         <v>46156</v>
       </c>
       <c r="X630" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.69097220000000004</v>
       </c>
       <c r="Y630" s="10">
         <v>0</v>
@@ -87109,7 +87121,7 @@
         <v>53</v>
       </c>
       <c r="AR630" s="3" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="631" spans="1:44" x14ac:dyDescent="0.3">
@@ -87120,7 +87132,7 @@
         <v>2</v>
       </c>
       <c r="C631" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D631" s="3" t="s">
         <v>45</v>
@@ -87132,7 +87144,7 @@
         <v>46156</v>
       </c>
       <c r="G631" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H631" s="3" t="s">
         <v>47</v>
@@ -87147,16 +87159,16 @@
         <v>50</v>
       </c>
       <c r="L631" s="6">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M631" s="7">
-        <v>27790.67</v>
+        <v>26267.89</v>
       </c>
       <c r="N631" s="6">
         <v>1</v>
       </c>
       <c r="O631" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P631" s="8">
         <v>380.69</v>
@@ -87254,7 +87266,7 @@
         <v>2</v>
       </c>
       <c r="C632" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D632" s="3" t="s">
         <v>45</v>
@@ -87266,7 +87278,7 @@
         <v>46156</v>
       </c>
       <c r="G632" s="5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H632" s="3" t="s">
         <v>47</v>
@@ -87281,16 +87293,16 @@
         <v>50</v>
       </c>
       <c r="L632" s="6">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="M632" s="7">
-        <v>28171.360000000001</v>
+        <v>26648.59</v>
       </c>
       <c r="N632" s="6">
         <v>1</v>
       </c>
       <c r="O632" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P632" s="8">
         <v>380.69</v>
@@ -87388,7 +87400,7 @@
         <v>2</v>
       </c>
       <c r="C633" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D633" s="3" t="s">
         <v>45</v>
@@ -87400,7 +87412,7 @@
         <v>46156</v>
       </c>
       <c r="G633" s="5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H633" s="3" t="s">
         <v>47</v>
@@ -87415,16 +87427,16 @@
         <v>50</v>
       </c>
       <c r="L633" s="6">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="M633" s="7">
-        <v>28552.06</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N633" s="6">
         <v>1</v>
       </c>
       <c r="O633" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P633" s="8">
         <v>380.69</v>
@@ -87451,7 +87463,7 @@
         <v>46156</v>
       </c>
       <c r="X633" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y633" s="10">
         <v>0</v>
@@ -87522,7 +87534,7 @@
         <v>2</v>
       </c>
       <c r="C634" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D634" s="3" t="s">
         <v>45</v>
@@ -87534,7 +87546,7 @@
         <v>46156</v>
       </c>
       <c r="G634" s="5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H634" s="3" t="s">
         <v>47</v>
@@ -87549,16 +87561,16 @@
         <v>50</v>
       </c>
       <c r="L634" s="6">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="M634" s="7">
-        <v>28932.75</v>
+        <v>27409.98</v>
       </c>
       <c r="N634" s="6">
         <v>1</v>
       </c>
       <c r="O634" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P634" s="8">
         <v>380.69</v>
@@ -87585,7 +87597,7 @@
         <v>46156</v>
       </c>
       <c r="X634" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y634" s="10">
         <v>0</v>
@@ -87656,7 +87668,7 @@
         <v>2</v>
       </c>
       <c r="C635" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D635" s="3" t="s">
         <v>45</v>
@@ -87668,7 +87680,7 @@
         <v>46156</v>
       </c>
       <c r="G635" s="5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H635" s="3" t="s">
         <v>47</v>
@@ -87683,16 +87695,16 @@
         <v>50</v>
       </c>
       <c r="L635" s="6">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M635" s="7">
-        <v>29313.45</v>
+        <v>27790.67</v>
       </c>
       <c r="N635" s="6">
         <v>1</v>
       </c>
       <c r="O635" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P635" s="8">
         <v>380.69</v>
@@ -87719,7 +87731,7 @@
         <v>46156</v>
       </c>
       <c r="X635" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y635" s="10">
         <v>0</v>
@@ -87790,7 +87802,7 @@
         <v>2</v>
       </c>
       <c r="C636" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D636" s="3" t="s">
         <v>45</v>
@@ -87802,7 +87814,7 @@
         <v>46156</v>
       </c>
       <c r="G636" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H636" s="3" t="s">
         <v>47</v>
@@ -87817,16 +87829,16 @@
         <v>50</v>
       </c>
       <c r="L636" s="6">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="M636" s="7">
-        <v>29694.14</v>
+        <v>28171.360000000001</v>
       </c>
       <c r="N636" s="6">
         <v>1</v>
       </c>
       <c r="O636" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P636" s="8">
         <v>380.69</v>
@@ -87853,7 +87865,7 @@
         <v>46156</v>
       </c>
       <c r="X636" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y636" s="10">
         <v>0</v>
@@ -87924,7 +87936,7 @@
         <v>2</v>
       </c>
       <c r="C637" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D637" s="3" t="s">
         <v>45</v>
@@ -87936,7 +87948,7 @@
         <v>46156</v>
       </c>
       <c r="G637" s="5">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H637" s="3" t="s">
         <v>47</v>
@@ -87951,16 +87963,16 @@
         <v>50</v>
       </c>
       <c r="L637" s="6">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="M637" s="7">
-        <v>30074.83</v>
+        <v>28552.06</v>
       </c>
       <c r="N637" s="6">
         <v>1</v>
       </c>
       <c r="O637" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P637" s="8">
         <v>380.69</v>
@@ -87987,7 +87999,7 @@
         <v>46156</v>
       </c>
       <c r="X637" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y637" s="10">
         <v>0</v>
@@ -88058,7 +88070,7 @@
         <v>2</v>
       </c>
       <c r="C638" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D638" s="3" t="s">
         <v>45</v>
@@ -88070,7 +88082,7 @@
         <v>46156</v>
       </c>
       <c r="G638" s="5">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H638" s="3" t="s">
         <v>47</v>
@@ -88085,16 +88097,16 @@
         <v>50</v>
       </c>
       <c r="L638" s="6">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="M638" s="7">
-        <v>30455.53</v>
+        <v>28932.75</v>
       </c>
       <c r="N638" s="6">
         <v>1</v>
       </c>
       <c r="O638" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P638" s="8">
         <v>380.69</v>
@@ -88121,7 +88133,7 @@
         <v>46156</v>
       </c>
       <c r="X638" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y638" s="10">
         <v>0</v>
@@ -88192,7 +88204,7 @@
         <v>2</v>
       </c>
       <c r="C639" s="3" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D639" s="3" t="s">
         <v>45</v>
@@ -88204,7 +88216,7 @@
         <v>46156</v>
       </c>
       <c r="G639" s="5">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H639" s="3" t="s">
         <v>47</v>
@@ -88219,16 +88231,16 @@
         <v>50</v>
       </c>
       <c r="L639" s="6">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="M639" s="7">
-        <v>30836.22</v>
+        <v>29313.45</v>
       </c>
       <c r="N639" s="6">
         <v>1</v>
       </c>
       <c r="O639" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="P639" s="8">
         <v>380.69</v>
@@ -88255,7 +88267,7 @@
         <v>46156</v>
       </c>
       <c r="X639" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.33888889999999999</v>
       </c>
       <c r="Y639" s="10">
         <v>0</v>
@@ -88316,6 +88328,542 @@
       </c>
       <c r="AR639" s="3" t="s">
         <v>697</v>
+      </c>
+    </row>
+    <row r="640" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A640" s="1">
+        <v>1</v>
+      </c>
+      <c r="B640" s="2">
+        <v>2</v>
+      </c>
+      <c r="C640" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D640" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E640" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F640" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G640" s="5">
+        <v>10</v>
+      </c>
+      <c r="H640" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I640" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J640" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K640" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L640" s="6">
+        <v>78</v>
+      </c>
+      <c r="M640" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N640" s="6">
+        <v>1</v>
+      </c>
+      <c r="O640" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="P640" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q640" s="6">
+        <v>0</v>
+      </c>
+      <c r="R640" s="7">
+        <v>0</v>
+      </c>
+      <c r="S640" s="9">
+        <v>0</v>
+      </c>
+      <c r="T640" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U640" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V640" s="11">
+        <v>11</v>
+      </c>
+      <c r="W640" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X640" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y640" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z640" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA640" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB640" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC640" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD640" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE640" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF640" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG640" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH640" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI640" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ640" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK640" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL640" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM640" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN640" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO640" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP640" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ640" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR640" s="3" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="641" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A641" s="1">
+        <v>1</v>
+      </c>
+      <c r="B641" s="2">
+        <v>2</v>
+      </c>
+      <c r="C641" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D641" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E641" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F641" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G641" s="5">
+        <v>11</v>
+      </c>
+      <c r="H641" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I641" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J641" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K641" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L641" s="6">
+        <v>79</v>
+      </c>
+      <c r="M641" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N641" s="6">
+        <v>1</v>
+      </c>
+      <c r="O641" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="P641" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q641" s="6">
+        <v>0</v>
+      </c>
+      <c r="R641" s="7">
+        <v>0</v>
+      </c>
+      <c r="S641" s="9">
+        <v>0</v>
+      </c>
+      <c r="T641" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U641" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V641" s="11">
+        <v>11</v>
+      </c>
+      <c r="W641" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X641" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y641" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z641" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA641" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB641" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC641" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD641" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE641" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF641" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG641" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH641" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI641" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ641" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK641" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL641" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM641" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN641" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO641" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP641" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ641" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR641" s="3" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="642" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A642" s="1">
+        <v>1</v>
+      </c>
+      <c r="B642" s="2">
+        <v>2</v>
+      </c>
+      <c r="C642" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D642" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E642" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F642" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G642" s="5">
+        <v>12</v>
+      </c>
+      <c r="H642" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I642" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J642" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K642" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L642" s="6">
+        <v>80</v>
+      </c>
+      <c r="M642" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N642" s="6">
+        <v>1</v>
+      </c>
+      <c r="O642" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="P642" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q642" s="6">
+        <v>0</v>
+      </c>
+      <c r="R642" s="7">
+        <v>0</v>
+      </c>
+      <c r="S642" s="9">
+        <v>0</v>
+      </c>
+      <c r="T642" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U642" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V642" s="11">
+        <v>11</v>
+      </c>
+      <c r="W642" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X642" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y642" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z642" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA642" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB642" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC642" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD642" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE642" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF642" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG642" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH642" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI642" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ642" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK642" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL642" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM642" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN642" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO642" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP642" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ642" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR642" s="3" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="643" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A643" s="1">
+        <v>1</v>
+      </c>
+      <c r="B643" s="2">
+        <v>2</v>
+      </c>
+      <c r="C643" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D643" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E643" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F643" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G643" s="5">
+        <v>13</v>
+      </c>
+      <c r="H643" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I643" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J643" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K643" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L643" s="6">
+        <v>81</v>
+      </c>
+      <c r="M643" s="7">
+        <v>30836.22</v>
+      </c>
+      <c r="N643" s="6">
+        <v>1</v>
+      </c>
+      <c r="O643" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="P643" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q643" s="6">
+        <v>0</v>
+      </c>
+      <c r="R643" s="7">
+        <v>0</v>
+      </c>
+      <c r="S643" s="9">
+        <v>0</v>
+      </c>
+      <c r="T643" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U643" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V643" s="11">
+        <v>11</v>
+      </c>
+      <c r="W643" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X643" s="12">
+        <v>0.40138889999999999</v>
+      </c>
+      <c r="Y643" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z643" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA643" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB643" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC643" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD643" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE643" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF643" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG643" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH643" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI643" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ643" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK643" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL643" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM643" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN643" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO643" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP643" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ643" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR643" s="3" t="s">
+        <v>701</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/05/2026 17:13:29,69
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EF37385-8453-4F81-8FEB-75FD52452856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F961AC0-9851-4251-9A4D-A8401D9AC285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11600" uniqueCount="702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11744" uniqueCount="710">
   <si>
     <t>Sel</t>
   </si>
@@ -2083,6 +2083,30 @@
     <t>1858400002987</t>
   </si>
   <si>
+    <t>1858400002988</t>
+  </si>
+  <si>
+    <t>1858400002989</t>
+  </si>
+  <si>
+    <t>1858400002990</t>
+  </si>
+  <si>
+    <t>1858400002991</t>
+  </si>
+  <si>
+    <t>1858400002992</t>
+  </si>
+  <si>
+    <t>1858400002993</t>
+  </si>
+  <si>
+    <t>1858400002994</t>
+  </si>
+  <si>
+    <t>1858400002995</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
@@ -2701,7 +2725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR643"/>
+  <dimension ref="A1:AR651"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -87132,7 +87156,7 @@
         <v>2</v>
       </c>
       <c r="C631" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D631" s="3" t="s">
         <v>45</v>
@@ -87144,7 +87168,7 @@
         <v>46156</v>
       </c>
       <c r="G631" s="5">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="H631" s="3" t="s">
         <v>47</v>
@@ -87159,19 +87183,19 @@
         <v>50</v>
       </c>
       <c r="L631" s="6">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="M631" s="7">
-        <v>26267.89</v>
+        <v>40020.99</v>
       </c>
       <c r="N631" s="6">
         <v>1</v>
       </c>
       <c r="O631" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P631" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q631" s="6">
         <v>0</v>
@@ -87186,7 +87210,7 @@
         <v>52</v>
       </c>
       <c r="U631" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V631" s="11">
         <v>11</v>
@@ -87195,7 +87219,7 @@
         <v>46156</v>
       </c>
       <c r="X631" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.71180560000000004</v>
       </c>
       <c r="Y631" s="10">
         <v>0</v>
@@ -87255,7 +87279,7 @@
         <v>53</v>
       </c>
       <c r="AR631" s="3" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="632" spans="1:44" x14ac:dyDescent="0.3">
@@ -87266,7 +87290,7 @@
         <v>2</v>
       </c>
       <c r="C632" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D632" s="3" t="s">
         <v>45</v>
@@ -87278,7 +87302,7 @@
         <v>46156</v>
       </c>
       <c r="G632" s="5">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="H632" s="3" t="s">
         <v>47</v>
@@ -87293,19 +87317,19 @@
         <v>50</v>
       </c>
       <c r="L632" s="6">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="M632" s="7">
-        <v>26648.59</v>
+        <v>40470.660000000003</v>
       </c>
       <c r="N632" s="6">
         <v>1</v>
       </c>
       <c r="O632" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P632" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q632" s="6">
         <v>0</v>
@@ -87320,7 +87344,7 @@
         <v>52</v>
       </c>
       <c r="U632" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V632" s="11">
         <v>11</v>
@@ -87329,7 +87353,7 @@
         <v>46156</v>
       </c>
       <c r="X632" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.71180560000000004</v>
       </c>
       <c r="Y632" s="10">
         <v>0</v>
@@ -87389,7 +87413,7 @@
         <v>53</v>
       </c>
       <c r="AR632" s="3" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="633" spans="1:44" x14ac:dyDescent="0.3">
@@ -87400,7 +87424,7 @@
         <v>2</v>
       </c>
       <c r="C633" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D633" s="3" t="s">
         <v>45</v>
@@ -87412,7 +87436,7 @@
         <v>46156</v>
       </c>
       <c r="G633" s="5">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="H633" s="3" t="s">
         <v>47</v>
@@ -87427,19 +87451,19 @@
         <v>50</v>
       </c>
       <c r="L633" s="6">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="M633" s="7">
-        <v>27029.279999999999</v>
+        <v>40920.339999999997</v>
       </c>
       <c r="N633" s="6">
         <v>1</v>
       </c>
       <c r="O633" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P633" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q633" s="6">
         <v>0</v>
@@ -87454,7 +87478,7 @@
         <v>52</v>
       </c>
       <c r="U633" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V633" s="11">
         <v>11</v>
@@ -87463,7 +87487,7 @@
         <v>46156</v>
       </c>
       <c r="X633" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.71180560000000004</v>
       </c>
       <c r="Y633" s="10">
         <v>0</v>
@@ -87523,7 +87547,7 @@
         <v>53</v>
       </c>
       <c r="AR633" s="3" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
     </row>
     <row r="634" spans="1:44" x14ac:dyDescent="0.3">
@@ -87534,7 +87558,7 @@
         <v>2</v>
       </c>
       <c r="C634" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D634" s="3" t="s">
         <v>45</v>
@@ -87546,7 +87570,7 @@
         <v>46156</v>
       </c>
       <c r="G634" s="5">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="H634" s="3" t="s">
         <v>47</v>
@@ -87561,19 +87585,19 @@
         <v>50</v>
       </c>
       <c r="L634" s="6">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="M634" s="7">
-        <v>27409.98</v>
+        <v>41370.01</v>
       </c>
       <c r="N634" s="6">
         <v>1</v>
       </c>
       <c r="O634" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P634" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q634" s="6">
         <v>0</v>
@@ -87588,7 +87612,7 @@
         <v>52</v>
       </c>
       <c r="U634" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V634" s="11">
         <v>11</v>
@@ -87597,7 +87621,7 @@
         <v>46156</v>
       </c>
       <c r="X634" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.71180560000000004</v>
       </c>
       <c r="Y634" s="10">
         <v>0</v>
@@ -87657,7 +87681,7 @@
         <v>53</v>
       </c>
       <c r="AR634" s="3" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="635" spans="1:44" x14ac:dyDescent="0.3">
@@ -87668,7 +87692,7 @@
         <v>2</v>
       </c>
       <c r="C635" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D635" s="3" t="s">
         <v>45</v>
@@ -87680,7 +87704,7 @@
         <v>46156</v>
       </c>
       <c r="G635" s="5">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="H635" s="3" t="s">
         <v>47</v>
@@ -87695,19 +87719,19 @@
         <v>50</v>
       </c>
       <c r="L635" s="6">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="M635" s="7">
-        <v>27790.67</v>
+        <v>41819.68</v>
       </c>
       <c r="N635" s="6">
         <v>1</v>
       </c>
       <c r="O635" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P635" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q635" s="6">
         <v>0</v>
@@ -87722,7 +87746,7 @@
         <v>52</v>
       </c>
       <c r="U635" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V635" s="11">
         <v>11</v>
@@ -87731,7 +87755,7 @@
         <v>46156</v>
       </c>
       <c r="X635" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.71250000000000002</v>
       </c>
       <c r="Y635" s="10">
         <v>0</v>
@@ -87791,7 +87815,7 @@
         <v>53</v>
       </c>
       <c r="AR635" s="3" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
     </row>
     <row r="636" spans="1:44" x14ac:dyDescent="0.3">
@@ -87802,7 +87826,7 @@
         <v>2</v>
       </c>
       <c r="C636" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D636" s="3" t="s">
         <v>45</v>
@@ -87814,7 +87838,7 @@
         <v>46156</v>
       </c>
       <c r="G636" s="5">
-        <v>6</v>
+        <v>58</v>
       </c>
       <c r="H636" s="3" t="s">
         <v>47</v>
@@ -87829,19 +87853,19 @@
         <v>50</v>
       </c>
       <c r="L636" s="6">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="M636" s="7">
-        <v>28171.360000000001</v>
+        <v>42269.36</v>
       </c>
       <c r="N636" s="6">
         <v>1</v>
       </c>
       <c r="O636" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P636" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q636" s="6">
         <v>0</v>
@@ -87856,7 +87880,7 @@
         <v>52</v>
       </c>
       <c r="U636" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V636" s="11">
         <v>11</v>
@@ -87865,7 +87889,7 @@
         <v>46156</v>
       </c>
       <c r="X636" s="12">
-        <v>0.29722219999999999</v>
+        <v>0.71250000000000002</v>
       </c>
       <c r="Y636" s="10">
         <v>0</v>
@@ -87925,7 +87949,7 @@
         <v>53</v>
       </c>
       <c r="AR636" s="3" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
     </row>
     <row r="637" spans="1:44" x14ac:dyDescent="0.3">
@@ -87936,7 +87960,7 @@
         <v>2</v>
       </c>
       <c r="C637" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D637" s="3" t="s">
         <v>45</v>
@@ -87948,7 +87972,7 @@
         <v>46156</v>
       </c>
       <c r="G637" s="5">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="H637" s="3" t="s">
         <v>47</v>
@@ -87963,19 +87987,19 @@
         <v>50</v>
       </c>
       <c r="L637" s="6">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="M637" s="7">
-        <v>28552.06</v>
+        <v>42719.03</v>
       </c>
       <c r="N637" s="6">
         <v>1</v>
       </c>
       <c r="O637" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P637" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q637" s="6">
         <v>0</v>
@@ -87990,7 +88014,7 @@
         <v>52</v>
       </c>
       <c r="U637" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V637" s="11">
         <v>11</v>
@@ -87999,7 +88023,7 @@
         <v>46156</v>
       </c>
       <c r="X637" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.71250000000000002</v>
       </c>
       <c r="Y637" s="10">
         <v>0</v>
@@ -88059,7 +88083,7 @@
         <v>53</v>
       </c>
       <c r="AR637" s="3" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
     </row>
     <row r="638" spans="1:44" x14ac:dyDescent="0.3">
@@ -88070,7 +88094,7 @@
         <v>2</v>
       </c>
       <c r="C638" s="3" t="s">
-        <v>687</v>
+        <v>632</v>
       </c>
       <c r="D638" s="3" t="s">
         <v>45</v>
@@ -88082,7 +88106,7 @@
         <v>46156</v>
       </c>
       <c r="G638" s="5">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="H638" s="3" t="s">
         <v>47</v>
@@ -88097,19 +88121,19 @@
         <v>50</v>
       </c>
       <c r="L638" s="6">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="M638" s="7">
-        <v>28932.75</v>
+        <v>43168.71</v>
       </c>
       <c r="N638" s="6">
         <v>1</v>
       </c>
       <c r="O638" s="3" t="s">
-        <v>688</v>
+        <v>633</v>
       </c>
       <c r="P638" s="8">
-        <v>380.69</v>
+        <v>449.67</v>
       </c>
       <c r="Q638" s="6">
         <v>0</v>
@@ -88124,7 +88148,7 @@
         <v>52</v>
       </c>
       <c r="U638" s="10">
-        <v>64287</v>
+        <v>64218</v>
       </c>
       <c r="V638" s="11">
         <v>11</v>
@@ -88133,7 +88157,7 @@
         <v>46156</v>
       </c>
       <c r="X638" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.71250000000000002</v>
       </c>
       <c r="Y638" s="10">
         <v>0</v>
@@ -88193,7 +88217,7 @@
         <v>53</v>
       </c>
       <c r="AR638" s="3" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
     </row>
     <row r="639" spans="1:44" x14ac:dyDescent="0.3">
@@ -88204,7 +88228,7 @@
         <v>2</v>
       </c>
       <c r="C639" s="3" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="D639" s="3" t="s">
         <v>45</v>
@@ -88216,7 +88240,7 @@
         <v>46156</v>
       </c>
       <c r="G639" s="5">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H639" s="3" t="s">
         <v>47</v>
@@ -88231,16 +88255,16 @@
         <v>50</v>
       </c>
       <c r="L639" s="6">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="M639" s="7">
-        <v>29313.45</v>
+        <v>26267.89</v>
       </c>
       <c r="N639" s="6">
         <v>1</v>
       </c>
       <c r="O639" s="3" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="P639" s="8">
         <v>380.69</v>
@@ -88267,7 +88291,7 @@
         <v>46156</v>
       </c>
       <c r="X639" s="12">
-        <v>0.33888889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y639" s="10">
         <v>0</v>
@@ -88338,7 +88362,7 @@
         <v>2</v>
       </c>
       <c r="C640" s="3" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="D640" s="3" t="s">
         <v>45</v>
@@ -88350,7 +88374,7 @@
         <v>46156</v>
       </c>
       <c r="G640" s="5">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H640" s="3" t="s">
         <v>47</v>
@@ -88365,16 +88389,16 @@
         <v>50</v>
       </c>
       <c r="L640" s="6">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="M640" s="7">
-        <v>29694.14</v>
+        <v>26648.59</v>
       </c>
       <c r="N640" s="6">
         <v>1</v>
       </c>
       <c r="O640" s="3" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="P640" s="8">
         <v>380.69</v>
@@ -88401,7 +88425,7 @@
         <v>46156</v>
       </c>
       <c r="X640" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y640" s="10">
         <v>0</v>
@@ -88472,7 +88496,7 @@
         <v>2</v>
       </c>
       <c r="C641" s="3" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="D641" s="3" t="s">
         <v>45</v>
@@ -88484,7 +88508,7 @@
         <v>46156</v>
       </c>
       <c r="G641" s="5">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H641" s="3" t="s">
         <v>47</v>
@@ -88499,16 +88523,16 @@
         <v>50</v>
       </c>
       <c r="L641" s="6">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="M641" s="7">
-        <v>30074.83</v>
+        <v>27029.279999999999</v>
       </c>
       <c r="N641" s="6">
         <v>1</v>
       </c>
       <c r="O641" s="3" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="P641" s="8">
         <v>380.69</v>
@@ -88535,7 +88559,7 @@
         <v>46156</v>
       </c>
       <c r="X641" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y641" s="10">
         <v>0</v>
@@ -88606,7 +88630,7 @@
         <v>2</v>
       </c>
       <c r="C642" s="3" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="D642" s="3" t="s">
         <v>45</v>
@@ -88618,7 +88642,7 @@
         <v>46156</v>
       </c>
       <c r="G642" s="5">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H642" s="3" t="s">
         <v>47</v>
@@ -88633,16 +88657,16 @@
         <v>50</v>
       </c>
       <c r="L642" s="6">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="M642" s="7">
-        <v>30455.53</v>
+        <v>27409.98</v>
       </c>
       <c r="N642" s="6">
         <v>1</v>
       </c>
       <c r="O642" s="3" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="P642" s="8">
         <v>380.69</v>
@@ -88669,7 +88693,7 @@
         <v>46156</v>
       </c>
       <c r="X642" s="12">
-        <v>0.35972219999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y642" s="10">
         <v>0</v>
@@ -88740,7 +88764,7 @@
         <v>2</v>
       </c>
       <c r="C643" s="3" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="D643" s="3" t="s">
         <v>45</v>
@@ -88752,7 +88776,7 @@
         <v>46156</v>
       </c>
       <c r="G643" s="5">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H643" s="3" t="s">
         <v>47</v>
@@ -88767,16 +88791,16 @@
         <v>50</v>
       </c>
       <c r="L643" s="6">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="M643" s="7">
-        <v>30836.22</v>
+        <v>27790.67</v>
       </c>
       <c r="N643" s="6">
         <v>1</v>
       </c>
       <c r="O643" s="3" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="P643" s="8">
         <v>380.69</v>
@@ -88803,7 +88827,7 @@
         <v>46156</v>
       </c>
       <c r="X643" s="12">
-        <v>0.40138889999999999</v>
+        <v>0.29722219999999999</v>
       </c>
       <c r="Y643" s="10">
         <v>0</v>
@@ -88864,6 +88888,1078 @@
       </c>
       <c r="AR643" s="3" t="s">
         <v>701</v>
+      </c>
+    </row>
+    <row r="644" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A644" s="1">
+        <v>1</v>
+      </c>
+      <c r="B644" s="2">
+        <v>2</v>
+      </c>
+      <c r="C644" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D644" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E644" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F644" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G644" s="5">
+        <v>6</v>
+      </c>
+      <c r="H644" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I644" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J644" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K644" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L644" s="6">
+        <v>74</v>
+      </c>
+      <c r="M644" s="7">
+        <v>28171.360000000001</v>
+      </c>
+      <c r="N644" s="6">
+        <v>1</v>
+      </c>
+      <c r="O644" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P644" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q644" s="6">
+        <v>0</v>
+      </c>
+      <c r="R644" s="7">
+        <v>0</v>
+      </c>
+      <c r="S644" s="9">
+        <v>0</v>
+      </c>
+      <c r="T644" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U644" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V644" s="11">
+        <v>11</v>
+      </c>
+      <c r="W644" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X644" s="12">
+        <v>0.29722219999999999</v>
+      </c>
+      <c r="Y644" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z644" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA644" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB644" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC644" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD644" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE644" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF644" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG644" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH644" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI644" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ644" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK644" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL644" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM644" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN644" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO644" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP644" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ644" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR644" s="3" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="645" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A645" s="1">
+        <v>1</v>
+      </c>
+      <c r="B645" s="2">
+        <v>2</v>
+      </c>
+      <c r="C645" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D645" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E645" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F645" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G645" s="5">
+        <v>7</v>
+      </c>
+      <c r="H645" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I645" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J645" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K645" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L645" s="6">
+        <v>75</v>
+      </c>
+      <c r="M645" s="7">
+        <v>28552.06</v>
+      </c>
+      <c r="N645" s="6">
+        <v>1</v>
+      </c>
+      <c r="O645" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P645" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q645" s="6">
+        <v>0</v>
+      </c>
+      <c r="R645" s="7">
+        <v>0</v>
+      </c>
+      <c r="S645" s="9">
+        <v>0</v>
+      </c>
+      <c r="T645" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U645" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V645" s="11">
+        <v>11</v>
+      </c>
+      <c r="W645" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X645" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y645" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z645" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA645" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB645" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC645" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD645" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE645" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF645" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG645" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH645" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI645" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ645" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK645" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL645" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM645" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN645" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO645" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP645" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ645" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR645" s="3" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="646" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A646" s="1">
+        <v>1</v>
+      </c>
+      <c r="B646" s="2">
+        <v>2</v>
+      </c>
+      <c r="C646" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D646" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E646" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F646" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G646" s="5">
+        <v>8</v>
+      </c>
+      <c r="H646" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I646" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J646" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K646" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L646" s="6">
+        <v>76</v>
+      </c>
+      <c r="M646" s="7">
+        <v>28932.75</v>
+      </c>
+      <c r="N646" s="6">
+        <v>1</v>
+      </c>
+      <c r="O646" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P646" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q646" s="6">
+        <v>0</v>
+      </c>
+      <c r="R646" s="7">
+        <v>0</v>
+      </c>
+      <c r="S646" s="9">
+        <v>0</v>
+      </c>
+      <c r="T646" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U646" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V646" s="11">
+        <v>11</v>
+      </c>
+      <c r="W646" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X646" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y646" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z646" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA646" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB646" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC646" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD646" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE646" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF646" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG646" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH646" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI646" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ646" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK646" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL646" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM646" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN646" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO646" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP646" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ646" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR646" s="3" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="647" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A647" s="1">
+        <v>1</v>
+      </c>
+      <c r="B647" s="2">
+        <v>2</v>
+      </c>
+      <c r="C647" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D647" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E647" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F647" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G647" s="5">
+        <v>9</v>
+      </c>
+      <c r="H647" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I647" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J647" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K647" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L647" s="6">
+        <v>77</v>
+      </c>
+      <c r="M647" s="7">
+        <v>29313.45</v>
+      </c>
+      <c r="N647" s="6">
+        <v>1</v>
+      </c>
+      <c r="O647" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P647" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q647" s="6">
+        <v>0</v>
+      </c>
+      <c r="R647" s="7">
+        <v>0</v>
+      </c>
+      <c r="S647" s="9">
+        <v>0</v>
+      </c>
+      <c r="T647" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U647" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V647" s="11">
+        <v>11</v>
+      </c>
+      <c r="W647" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X647" s="12">
+        <v>0.33888889999999999</v>
+      </c>
+      <c r="Y647" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z647" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA647" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB647" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC647" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD647" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE647" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF647" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG647" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH647" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI647" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ647" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK647" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL647" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM647" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN647" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO647" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP647" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ647" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR647" s="3" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="648" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A648" s="1">
+        <v>1</v>
+      </c>
+      <c r="B648" s="2">
+        <v>2</v>
+      </c>
+      <c r="C648" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D648" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E648" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F648" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G648" s="5">
+        <v>10</v>
+      </c>
+      <c r="H648" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I648" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J648" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K648" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L648" s="6">
+        <v>78</v>
+      </c>
+      <c r="M648" s="7">
+        <v>29694.14</v>
+      </c>
+      <c r="N648" s="6">
+        <v>1</v>
+      </c>
+      <c r="O648" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P648" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q648" s="6">
+        <v>0</v>
+      </c>
+      <c r="R648" s="7">
+        <v>0</v>
+      </c>
+      <c r="S648" s="9">
+        <v>0</v>
+      </c>
+      <c r="T648" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U648" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V648" s="11">
+        <v>11</v>
+      </c>
+      <c r="W648" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X648" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y648" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z648" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA648" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB648" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC648" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD648" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE648" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF648" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG648" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH648" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI648" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ648" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK648" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL648" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM648" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN648" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO648" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP648" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ648" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR648" s="3" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="649" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A649" s="1">
+        <v>1</v>
+      </c>
+      <c r="B649" s="2">
+        <v>2</v>
+      </c>
+      <c r="C649" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D649" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E649" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F649" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G649" s="5">
+        <v>11</v>
+      </c>
+      <c r="H649" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I649" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J649" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K649" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L649" s="6">
+        <v>79</v>
+      </c>
+      <c r="M649" s="7">
+        <v>30074.83</v>
+      </c>
+      <c r="N649" s="6">
+        <v>1</v>
+      </c>
+      <c r="O649" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P649" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q649" s="6">
+        <v>0</v>
+      </c>
+      <c r="R649" s="7">
+        <v>0</v>
+      </c>
+      <c r="S649" s="9">
+        <v>0</v>
+      </c>
+      <c r="T649" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U649" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V649" s="11">
+        <v>11</v>
+      </c>
+      <c r="W649" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X649" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y649" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z649" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA649" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB649" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC649" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD649" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE649" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF649" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG649" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH649" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI649" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ649" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK649" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL649" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM649" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN649" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO649" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP649" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ649" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR649" s="3" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="650" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A650" s="1">
+        <v>1</v>
+      </c>
+      <c r="B650" s="2">
+        <v>2</v>
+      </c>
+      <c r="C650" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="D650" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E650" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F650" s="4">
+        <v>46156</v>
+      </c>
+      <c r="G650" s="5">
+        <v>12</v>
+      </c>
+      <c r="H650" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I650" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J650" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K650" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L650" s="6">
+        <v>80</v>
+      </c>
+      <c r="M650" s="7">
+        <v>30455.53</v>
+      </c>
+      <c r="N650" s="6">
+        <v>1</v>
+      </c>
+      <c r="O650" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="P650" s="8">
+        <v>380.69</v>
+      </c>
+      <c r="Q650" s="6">
+        <v>0</v>
+      </c>
+      <c r="R650" s="7">
+        <v>0</v>
+      </c>
+      <c r="S650" s="9">
+        <v>0</v>
+      </c>
+      <c r="T650" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U650" s="10">
+        <v>64287</v>
+      </c>
+      <c r="V650" s="11">
+        <v>11</v>
+      </c>
+      <c r="W650" s="4">
+        <v>46156</v>
+      </c>
+      <c r="X650" s="12">
+        <v>0.35972219999999999</v>
+      </c>
+      <c r="Y650" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z650" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA650" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB650" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC650" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD650" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE650" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF650" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG650" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH650" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI650" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="AJ650" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK650" s="14">
+        <v>0</v>